<commit_message>
redo winter full flex with the lower flowrate penalty
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF0A6E1-B90F-40B0-9AC7-61A42977BB0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B41DF8E0-5A08-4535-BD00-BF0AAE01F630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -36,13 +36,11 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}</author>
-    <author>tc={815F3FDC-C725-4656-9AA0-DDB81C7546AD}</author>
     <author>tc={DFECE21F-32E0-4210-824A-1E57B1730184}</author>
-    <author>tc={D42C0CEC-223C-40FD-88E7-B5BC8DDF118E}</author>
     <author>tc={82EE7A36-D8EE-4051-AEAE-B403E815DFF2}</author>
+    <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
     <author>tc={F9308CF0-AB74-4ABB-91B6-7382ECEADD39}</author>
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
-    <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
     <author>tc={7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}</author>
     <author>tc={86E634AB-9E52-4A6D-BE85-5D191C9227C6}</author>
   </authors>
@@ -55,15 +53,7 @@
     This should be the same as the baseline</t>
       </text>
     </comment>
-    <comment ref="A22" authorId="1" shapeId="0" xr:uid="{815F3FDC-C725-4656-9AA0-DDB81C7546AD}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Have to rerun if I want to get the correct Flexibility metrics</t>
-      </text>
-    </comment>
-    <comment ref="A25" authorId="2" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
+    <comment ref="A25" authorId="1" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -71,15 +61,7 @@
     Curious if solver would eventually find same solution as the 4 flex trains</t>
       </text>
     </comment>
-    <comment ref="A28" authorId="3" shapeId="0" xr:uid="{D42C0CEC-223C-40FD-88E7-B5BC8DDF118E}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Need to rerun to confirm shutdowns are not optimal</t>
-      </text>
-    </comment>
-    <comment ref="A30" authorId="4" shapeId="0" xr:uid="{82EE7A36-D8EE-4051-AEAE-B403E815DFF2}">
+    <comment ref="A30" authorId="2" shapeId="0" xr:uid="{82EE7A36-D8EE-4051-AEAE-B403E815DFF2}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -87,7 +69,15 @@
     With a lower flow change penalty, this might become possible</t>
       </text>
     </comment>
-    <comment ref="A34" authorId="5" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A34" authorId="3" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Winter is low winter weekdays + low weekends</t>
+      </text>
+    </comment>
+    <comment ref="A35" authorId="4" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -95,7 +85,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T34" authorId="6" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T35" authorId="5" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -105,15 +95,7 @@
     The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A35" authorId="7" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Winter is low winter weekdays + low weekends</t>
-      </text>
-    </comment>
-    <comment ref="A41" authorId="8" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A41" authorId="6" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -121,7 +103,7 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="T67" authorId="9" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T66" authorId="7" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -134,7 +116,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="35">
   <si>
     <t>Season</t>
   </si>
@@ -232,9 +214,6 @@
     <t>TOU 8</t>
   </si>
   <si>
-    <t>Link to result: https://github.com/jakechurchi/watertap/blob/77b0fd3a12650b35dc7419a8ee835ba61fcc1512/tutorials/flex_ro/wrd_pricetaker_summary_results_20260529_155321.csv</t>
-  </si>
-  <si>
     <t>Simplified Rate Structures</t>
   </si>
   <si>
@@ -248,7 +227,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -402,12 +381,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -766,7 +739,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1151,34 +1124,28 @@
   <threadedComment ref="A16" dT="2026-07-01T17:37:32.24" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
     <text>This should be the same as the baseline</text>
   </threadedComment>
-  <threadedComment ref="A22" dT="2026-07-01T17:39:57.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{815F3FDC-C725-4656-9AA0-DDB81C7546AD}">
-    <text>Have to rerun if I want to get the correct Flexibility metrics</text>
-  </threadedComment>
   <threadedComment ref="A25" dT="2026-06-11T20:38:07.96" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{DFECE21F-32E0-4210-824A-1E57B1730184}">
     <text>Curious if solver would eventually find same solution as the 4 flex trains</text>
-  </threadedComment>
-  <threadedComment ref="A28" dT="2026-07-01T18:06:46.80" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{D42C0CEC-223C-40FD-88E7-B5BC8DDF118E}">
-    <text>Need to rerun to confirm shutdowns are not optimal</text>
   </threadedComment>
   <threadedComment ref="A30" dT="2026-07-01T19:38:50.85" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{82EE7A36-D8EE-4051-AEAE-B403E815DFF2}">
     <text>With a lower flow change penalty, this might become possible</text>
   </threadedComment>
-  <threadedComment ref="A34" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+  <threadedComment ref="A34" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <text>Winter is low winter weekdays + low weekends</text>
+  </threadedComment>
+  <threadedComment ref="A35" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
     <text>Summer week = hot summer weekdays + high weekends</text>
   </threadedComment>
-  <threadedComment ref="T34" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T35" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure</text>
   </threadedComment>
-  <threadedComment ref="T34" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T35" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>The baseline costs have to be updated in accordance with the demand structure type</text>
-  </threadedComment>
-  <threadedComment ref="A35" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
-    <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
   <threadedComment ref="A41" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
     <text>Result from the fast solve</text>
   </threadedComment>
-  <threadedComment ref="T67" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="T66" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1186,7 +1153,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:U70"/>
+  <dimension ref="A1:T69"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="9.61328125" customWidth="1"/>
@@ -1892,10 +1859,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1957,7 +1924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2019,11 +1986,11 @@
         <v>9.6260597723556093E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2034,42 +2001,72 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="3">
         <v>2</v>
       </c>
-      <c r="G22" s="4">
-        <v>20277.993676447401</v>
+      <c r="D22">
+        <v>118061.356447413</v>
+      </c>
+      <c r="E22">
+        <v>282179.67123275797</v>
+      </c>
+      <c r="F22">
+        <v>0.84915166967023703</v>
+      </c>
+      <c r="G22">
+        <v>20001.758947398499</v>
       </c>
       <c r="H22">
-        <v>6534.5593757614897</v>
+        <v>6545.6854256406996</v>
       </c>
       <c r="I22">
-        <v>5996.9333902952303</v>
+        <v>6069.3991958142597</v>
       </c>
       <c r="J22">
-        <v>32809.486442504203</v>
+        <v>32616.843568853401</v>
+      </c>
+      <c r="K22">
+        <v>50843.1840052314</v>
       </c>
       <c r="L22">
-        <v>15303.798385783</v>
+        <v>15303.7983840124</v>
+      </c>
+      <c r="M22">
+        <v>19297.530489315999</v>
+      </c>
+      <c r="N22">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O22">
+        <v>0</v>
       </c>
       <c r="P22">
-        <v>239805.98185054099</v>
-      </c>
-      <c r="U22" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.4">
+        <v>239613.33897429501</v>
+      </c>
+      <c r="Q22">
+        <v>1462.4682301396899</v>
+      </c>
+      <c r="R22">
+        <v>17686.324085333301</v>
+      </c>
+      <c r="S22">
+        <v>149.88410241807901</v>
+      </c>
+      <c r="T22">
+        <v>0.116169937532689</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2131,11 +2128,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A25" s="6" t="s">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C25">
@@ -2193,36 +2190,132 @@
         <v>1.20740363486328</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A27" s="2" t="s">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C27">
         <v>4</v>
       </c>
-    </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A28" s="2" t="s">
+      <c r="D27">
+        <v>111742.37918817</v>
+      </c>
+      <c r="E27">
+        <v>282179.67125500599</v>
+      </c>
+      <c r="F27">
+        <v>0.82675821641390801</v>
+      </c>
+      <c r="G27">
+        <v>18666.456843152599</v>
+      </c>
+      <c r="H27">
+        <v>4964.4646341457201</v>
+      </c>
+      <c r="I27">
+        <v>2666.9448136542001</v>
+      </c>
+      <c r="J27">
+        <v>26297.866290952599</v>
+      </c>
+      <c r="K27">
+        <v>50843.184012316902</v>
+      </c>
+      <c r="L27">
+        <v>15303.7983934401</v>
+      </c>
+      <c r="M27">
+        <v>19297.530491460901</v>
+      </c>
+      <c r="N27">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O27">
+        <v>0</v>
+      </c>
+      <c r="P27">
+        <v>233294.36171505199</v>
+      </c>
+      <c r="Q27">
+        <v>1127.27501819133</v>
+      </c>
+      <c r="R27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A28" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C28">
         <v>4</v>
       </c>
-    </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="D28">
+        <v>118002.301696422</v>
+      </c>
+      <c r="E28">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F28">
+        <v>0.84894238899869401</v>
+      </c>
+      <c r="G28">
+        <v>20022.627559674602</v>
+      </c>
+      <c r="H28">
+        <v>6537.0412109993104</v>
+      </c>
+      <c r="I28">
+        <v>5998.0824175879798</v>
+      </c>
+      <c r="J28">
+        <v>32557.7511882619</v>
+      </c>
+      <c r="K28">
+        <v>50843.193666259001</v>
+      </c>
+      <c r="L28">
+        <v>15303.8243479339</v>
+      </c>
+      <c r="M28">
+        <v>19297.532493967901</v>
+      </c>
+      <c r="N28">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O28">
+        <v>0</v>
+      </c>
+      <c r="P28">
+        <v>239554.28422330401</v>
+      </c>
+      <c r="Q28">
+        <v>1460.5368984148499</v>
+      </c>
+      <c r="R28">
+        <v>20030.045592225699</v>
+      </c>
+      <c r="S28">
+        <v>178.83969278772901</v>
+      </c>
+      <c r="T28">
+        <v>0.105527046108572</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2284,7 +2377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -2353,8 +2446,8 @@
       <c r="G33" s="4"/>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A34" t="s">
-        <v>22</v>
+      <c r="A34" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="B34" t="s">
         <v>23</v>
@@ -2363,34 +2456,34 @@
         <v>0</v>
       </c>
       <c r="D34">
-        <v>187020.456722612</v>
+        <v>247948.64160389101</v>
       </c>
       <c r="E34">
-        <v>282179.67123287602</v>
+        <v>374203.2</v>
       </c>
       <c r="F34">
-        <v>1.09353178385</v>
-      </c>
-      <c r="G34">
-        <v>89520.694507565597</v>
+        <v>0.98743309552342695</v>
+      </c>
+      <c r="G34" s="4">
+        <v>118659.96685142</v>
       </c>
       <c r="H34">
-        <v>6971.3813103080802</v>
+        <v>9240.5882208594503</v>
       </c>
       <c r="I34">
-        <v>5083.8680235841202</v>
+        <v>6738.6833231561404</v>
       </c>
       <c r="J34">
-        <v>101575.943841457</v>
+        <v>134639.23839543501</v>
       </c>
       <c r="K34">
-        <v>50843.184005923598</v>
+        <v>67424.000002171</v>
       </c>
       <c r="L34">
-        <v>15303.798385783</v>
+        <v>20294.624005833801</v>
       </c>
       <c r="M34">
-        <v>19297.5304894482</v>
+        <v>25590.779200450401</v>
       </c>
       <c r="N34">
         <v>992.31070788530405</v>
@@ -2399,24 +2492,24 @@
         <v>0</v>
       </c>
       <c r="P34">
-        <v>308572.439249494</v>
+        <v>369500.62413077202</v>
       </c>
       <c r="Q34">
-        <v>1106.4527933521999</v>
+        <v>1466.60671595592</v>
       </c>
       <c r="R34">
-        <v>3451.9307168288801</v>
+        <v>0</v>
       </c>
       <c r="S34">
-        <v>20.547206647791</v>
+        <v>0</v>
       </c>
       <c r="T34">
-        <v>-14.696886263168601</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A35" s="3" t="s">
-        <v>20</v>
+      <c r="A35" t="s">
+        <v>22</v>
       </c>
       <c r="B35" t="s">
         <v>23</v>
@@ -2425,34 +2518,34 @@
         <v>0</v>
       </c>
       <c r="D35">
-        <v>247948.64160389101</v>
+        <v>187020.456722612</v>
       </c>
       <c r="E35">
-        <v>374203.2</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F35">
-        <v>0.98743309552342695</v>
-      </c>
-      <c r="G35" s="4">
-        <v>118659.96685142</v>
+        <v>1.09353178385</v>
+      </c>
+      <c r="G35">
+        <v>89520.694507565597</v>
       </c>
       <c r="H35">
-        <v>9240.5882208594503</v>
+        <v>6971.3813103080802</v>
       </c>
       <c r="I35">
-        <v>6738.6833231561404</v>
+        <v>5083.8680235841202</v>
       </c>
       <c r="J35">
-        <v>134639.23839543501</v>
+        <v>101575.943841457</v>
       </c>
       <c r="K35">
-        <v>67424.000002171</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L35">
-        <v>20294.624005833801</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M35">
-        <v>25590.779200450401</v>
+        <v>19297.5304894482</v>
       </c>
       <c r="N35">
         <v>992.31070788530405</v>
@@ -2461,19 +2554,19 @@
         <v>0</v>
       </c>
       <c r="P35">
-        <v>369500.62413077202</v>
+        <v>308572.439249494</v>
       </c>
       <c r="Q35">
-        <v>1466.60671595592</v>
+        <v>1106.4527933521999</v>
       </c>
       <c r="R35">
-        <v>0</v>
+        <v>3451.9307168288801</v>
       </c>
       <c r="S35">
-        <v>0</v>
+        <v>20.547206647791</v>
       </c>
       <c r="T35">
-        <v>0</v>
+        <v>-14.696886263168601</v>
       </c>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.4">
@@ -2482,7 +2575,7 @@
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B37" t="s">
         <v>21</v>
@@ -2491,34 +2584,34 @@
         <v>0</v>
       </c>
       <c r="D37">
-        <v>171564.02128394699</v>
+        <v>117032.41959359701</v>
       </c>
       <c r="E37">
-        <v>282179.67123287701</v>
+        <v>282179.67123286898</v>
       </c>
       <c r="F37">
-        <v>1.03875662810921</v>
-      </c>
-      <c r="G37">
-        <v>73514.1870928641</v>
+        <v>0.845505280653571</v>
+      </c>
+      <c r="G37" s="4">
+        <v>23683.129427060001</v>
       </c>
       <c r="H37">
-        <v>7482.8438362204697</v>
+        <v>6986.3695969997798</v>
       </c>
       <c r="I37">
-        <v>4044.9309872213798</v>
+        <v>918.40768838365295</v>
       </c>
       <c r="J37">
-        <v>85041.961916305998</v>
+        <v>31587.906712443499</v>
       </c>
       <c r="K37">
-        <v>51119.832654572398</v>
+        <v>50843.1840059237</v>
       </c>
       <c r="L37">
-        <v>16047.2916290263</v>
+        <v>15303.7983857823</v>
       </c>
       <c r="M37">
-        <v>19354.9350840429</v>
+        <v>19297.530489448101</v>
       </c>
       <c r="N37">
         <v>992.31070788530405</v>
@@ -2527,24 +2620,24 @@
         <v>0</v>
       </c>
       <c r="P37">
-        <v>293116.00381082902</v>
+        <v>238584.402120479</v>
       </c>
       <c r="Q37">
-        <v>1187.62883512946</v>
+        <v>1108.83163779344</v>
       </c>
       <c r="R37">
-        <v>9393.8913494494009</v>
+        <v>0</v>
       </c>
       <c r="S37">
-        <v>260.94142637359403</v>
+        <v>230512.59606633501</v>
       </c>
       <c r="T37">
-        <v>-3.6405201993767098</v>
+        <v>1103.3673370121001</v>
       </c>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B38" t="s">
         <v>21</v>
@@ -2553,34 +2646,34 @@
         <v>0</v>
       </c>
       <c r="D38">
-        <v>117032.41959359701</v>
+        <v>171564.02128394699</v>
       </c>
       <c r="E38">
-        <v>282179.67123286898</v>
+        <v>282179.67123287701</v>
       </c>
       <c r="F38">
-        <v>0.845505280653571</v>
-      </c>
-      <c r="G38" s="4">
-        <v>23683.129427060001</v>
+        <v>1.03875662810921</v>
+      </c>
+      <c r="G38">
+        <v>73514.1870928641</v>
       </c>
       <c r="H38">
-        <v>6986.3695969997798</v>
+        <v>7482.8438362204697</v>
       </c>
       <c r="I38">
-        <v>918.40768838365295</v>
+        <v>4044.9309872213798</v>
       </c>
       <c r="J38">
-        <v>31587.906712443499</v>
+        <v>85041.961916305998</v>
       </c>
       <c r="K38">
-        <v>50843.1840059237</v>
+        <v>51119.832654572398</v>
       </c>
       <c r="L38">
-        <v>15303.7983857823</v>
+        <v>16047.2916290263</v>
       </c>
       <c r="M38">
-        <v>19297.530489448101</v>
+        <v>19354.9350840429</v>
       </c>
       <c r="N38">
         <v>992.31070788530405</v>
@@ -2589,19 +2682,19 @@
         <v>0</v>
       </c>
       <c r="P38">
-        <v>238584.402120479</v>
+        <v>293116.00381082902</v>
       </c>
       <c r="Q38">
-        <v>1108.83163779344</v>
+        <v>1187.62883512946</v>
       </c>
       <c r="R38">
-        <v>0</v>
+        <v>9393.8913494494009</v>
       </c>
       <c r="S38">
-        <v>230512.59606633501</v>
+        <v>260.94142637359403</v>
       </c>
       <c r="T38">
-        <v>1103.3673370121001</v>
+        <v>-3.6405201993767098</v>
       </c>
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.4">
@@ -2867,36 +2960,191 @@
       </c>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A48" s="1"/>
+      <c r="A48" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C48">
+        <v>0</v>
+      </c>
+      <c r="D48">
+        <v>115030.978322179</v>
+      </c>
+      <c r="E48">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F48">
+        <v>0.83841249022441</v>
+      </c>
+      <c r="G48">
+        <v>20114.092712805999</v>
+      </c>
+      <c r="H48">
+        <v>6942.2846600808298</v>
+      </c>
+      <c r="I48">
+        <v>2530.0880681377598</v>
+      </c>
+      <c r="J48">
+        <v>29586.4654410246</v>
+      </c>
+      <c r="K48">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L48">
+        <v>15303.798385783</v>
+      </c>
+      <c r="M48">
+        <v>19297.5304894482</v>
+      </c>
+      <c r="N48">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O48">
+        <v>0</v>
+      </c>
+      <c r="P48">
+        <v>236582.960849061</v>
+      </c>
+      <c r="Q48">
+        <v>1101.8347602124099</v>
+      </c>
+      <c r="R48">
+        <v>0</v>
+      </c>
+      <c r="S48">
+        <v>0</v>
+      </c>
+      <c r="T48">
+        <v>0</v>
+      </c>
     </row>
     <row r="49" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A49" s="2" t="s">
+      <c r="A49" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C49">
+        <v>0</v>
+      </c>
+      <c r="D49">
+        <v>124771.246709449</v>
+      </c>
+      <c r="E49">
+        <v>282179.67125180899</v>
+      </c>
+      <c r="F49">
+        <v>0.87293045648394496</v>
+      </c>
+      <c r="G49">
+        <v>22626.697961956499</v>
+      </c>
+      <c r="H49">
+        <v>7102.5767129513297</v>
+      </c>
+      <c r="I49">
+        <v>9597.4591384874802</v>
+      </c>
+      <c r="J49">
+        <v>39326.733813395302</v>
+      </c>
+      <c r="K49">
+        <v>50843.184011688398</v>
+      </c>
+      <c r="L49">
+        <v>15303.798393134501</v>
+      </c>
+      <c r="M49">
+        <v>19297.530491231599</v>
+      </c>
+      <c r="N49">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O49">
+        <v>0</v>
+      </c>
+      <c r="P49">
+        <v>246323.22923633101</v>
+      </c>
+      <c r="Q49">
+        <v>1127.27501714903</v>
+      </c>
+      <c r="R49">
+        <v>0</v>
+      </c>
+      <c r="S49">
+        <v>0</v>
+      </c>
+      <c r="T49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A50" s="1"/>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A51" t="s">
         <v>20</v>
       </c>
-      <c r="B49" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C49">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A50" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C50">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A51" s="1"/>
+      <c r="B51" t="s">
+        <v>21</v>
+      </c>
+      <c r="C51">
+        <v>2</v>
+      </c>
+      <c r="D51">
+        <v>115714.10508262301</v>
+      </c>
+      <c r="E51">
+        <v>282179.67125387199</v>
+      </c>
+      <c r="F51">
+        <v>0.840833383054163</v>
+      </c>
+      <c r="G51" s="4">
+        <v>20578.507216446698</v>
+      </c>
+      <c r="H51">
+        <v>7102.57515066207</v>
+      </c>
+      <c r="I51">
+        <v>2588.5052959285099</v>
+      </c>
+      <c r="J51">
+        <v>30269.587663037299</v>
+      </c>
+      <c r="K51">
+        <v>50843.185173268597</v>
+      </c>
+      <c r="L51">
+        <v>15303.8015139941</v>
+      </c>
+      <c r="M51">
+        <v>19297.530732323401</v>
+      </c>
+      <c r="N51">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O51">
+        <v>0</v>
+      </c>
+      <c r="P51">
+        <v>237266.08760950499</v>
+      </c>
+      <c r="Q51">
+        <v>1127.2750356983099</v>
+      </c>
+      <c r="R51">
+        <v>0</v>
+      </c>
     </row>
     <row r="52" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B52" t="s">
         <v>21</v>
@@ -2905,116 +3153,116 @@
         <v>2</v>
       </c>
       <c r="D52">
-        <v>115714.10508262301</v>
+        <v>120628.41082793</v>
       </c>
       <c r="E52">
-        <v>282179.67125387199</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F52">
-        <v>0.840833383054163</v>
+        <v>0.85824890324911396</v>
       </c>
       <c r="G52" s="4">
-        <v>20578.507216446698</v>
+        <v>20824.7129679639</v>
       </c>
       <c r="H52">
-        <v>7102.57515066207</v>
+        <v>7456.39074483072</v>
       </c>
       <c r="I52">
-        <v>2588.5052959285099</v>
+        <v>5114.4587365303096</v>
       </c>
       <c r="J52">
-        <v>30269.587663037299</v>
+        <v>33395.562449324898</v>
       </c>
       <c r="K52">
-        <v>50843.185173268597</v>
+        <v>51302.320205525801</v>
       </c>
       <c r="L52">
-        <v>15303.8015139941</v>
+        <v>16537.7269222135</v>
       </c>
       <c r="M52">
-        <v>19297.530732323401</v>
+        <v>19392.801250865799</v>
       </c>
       <c r="N52">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O52">
+        <v>0</v>
+      </c>
+      <c r="P52">
+        <v>242180.39335481101</v>
+      </c>
+      <c r="Q52">
+        <v>1183.4303612998101</v>
+      </c>
+      <c r="R52">
+        <v>15931.1957490451</v>
+      </c>
+      <c r="S52">
+        <v>346.33034237054602</v>
+      </c>
+      <c r="T52">
+        <v>1.0959871186973</v>
+      </c>
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A54" t="s">
+        <v>20</v>
+      </c>
+      <c r="B54" t="s">
+        <v>21</v>
+      </c>
+      <c r="C54">
+        <v>4</v>
+      </c>
+      <c r="D54">
+        <v>115714.10508261999</v>
+      </c>
+      <c r="E54">
+        <v>282179.671253876</v>
+      </c>
+      <c r="F54">
+        <v>0.84083338305413902</v>
+      </c>
+      <c r="G54" s="4">
+        <v>20578.5072164468</v>
+      </c>
+      <c r="H54">
+        <v>7102.5751506616798</v>
+      </c>
+      <c r="I54">
+        <v>2588.50529592865</v>
+      </c>
+      <c r="J54">
+        <v>30269.587663037099</v>
+      </c>
+      <c r="K54">
+        <v>50843.185173268197</v>
+      </c>
+      <c r="L54">
+        <v>15303.8015139912</v>
+      </c>
+      <c r="M54">
+        <v>19297.530732323299</v>
+      </c>
+      <c r="N54">
         <v>992.31070788530405</v>
       </c>
-      <c r="O52">
-        <v>0</v>
-      </c>
-      <c r="P52">
-        <v>237266.08760950499</v>
-      </c>
-      <c r="Q52">
-        <v>1127.2750356983099</v>
-      </c>
-      <c r="R52">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A53" t="s">
-        <v>22</v>
-      </c>
-      <c r="B53" t="s">
-        <v>21</v>
-      </c>
-      <c r="C53">
-        <v>2</v>
-      </c>
-      <c r="D53">
-        <v>120628.41082793</v>
-      </c>
-      <c r="E53">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F53">
-        <v>0.85824890324911396</v>
-      </c>
-      <c r="G53" s="4">
-        <v>20824.7129679639</v>
-      </c>
-      <c r="H53">
-        <v>7456.39074483072</v>
-      </c>
-      <c r="I53">
-        <v>5114.4587365303096</v>
-      </c>
-      <c r="J53">
-        <v>33395.562449324898</v>
-      </c>
-      <c r="K53">
-        <v>51302.320205525801</v>
-      </c>
-      <c r="L53">
-        <v>16537.7269222135</v>
-      </c>
-      <c r="M53">
-        <v>19392.801250865799</v>
-      </c>
-      <c r="N53">
-        <v>1004.9477757237401</v>
-      </c>
-      <c r="O53">
-        <v>0</v>
-      </c>
-      <c r="P53">
-        <v>242180.39335481101</v>
-      </c>
-      <c r="Q53">
-        <v>1183.4303612998101</v>
-      </c>
-      <c r="R53">
-        <v>15931.1957490451</v>
-      </c>
-      <c r="S53">
-        <v>346.33034237054602</v>
-      </c>
-      <c r="T53">
-        <v>1.0959871186973</v>
+      <c r="O54">
+        <v>0</v>
+      </c>
+      <c r="P54">
+        <v>237266.087609501</v>
+      </c>
+      <c r="Q54">
+        <v>1127.2750356983499</v>
+      </c>
+      <c r="R54">
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B55" t="s">
         <v>21</v>
@@ -3023,275 +3271,281 @@
         <v>4</v>
       </c>
       <c r="D55">
-        <v>115714.10508261999</v>
+        <v>120375.156660901</v>
       </c>
       <c r="E55">
-        <v>282179.671253876</v>
+        <v>282179.671232878</v>
       </c>
       <c r="F55">
-        <v>0.84083338305413902</v>
+        <v>0.857351410648304</v>
       </c>
       <c r="G55" s="4">
-        <v>20578.5072164468</v>
+        <v>21285.1004075495</v>
       </c>
       <c r="H55">
-        <v>7102.5751506616798</v>
+        <v>7426.32532798384</v>
       </c>
       <c r="I55">
-        <v>2588.50529592865</v>
+        <v>5046.79446201879</v>
       </c>
       <c r="J55">
-        <v>30269.587663037099</v>
+        <v>33758.220197552102</v>
       </c>
       <c r="K55">
-        <v>50843.185173268197</v>
+        <v>51144.191344099498</v>
       </c>
       <c r="L55">
-        <v>15303.8015139912</v>
+        <v>16112.7556071296</v>
       </c>
       <c r="M55">
-        <v>19297.530732323299</v>
+        <v>19359.989512119799</v>
       </c>
       <c r="N55">
-        <v>992.31070788530405</v>
+        <v>1006.77939378399</v>
       </c>
       <c r="O55">
         <v>0</v>
       </c>
       <c r="P55">
-        <v>237266.087609501</v>
+        <v>241927.13918778201</v>
       </c>
       <c r="Q55">
-        <v>1127.2750356983499</v>
+        <v>1178.65858109644</v>
       </c>
       <c r="R55">
-        <v>0</v>
+        <v>12586.325853030899</v>
+      </c>
+      <c r="S55">
+        <v>466.16021677892502</v>
+      </c>
+      <c r="T55">
+        <v>1.3585822738026401</v>
       </c>
     </row>
     <row r="56" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A56" t="s">
-        <v>22</v>
-      </c>
-      <c r="B56" t="s">
+      <c r="G56" s="4"/>
+    </row>
+    <row r="57" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A57" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G57" s="4"/>
+      <c r="P57" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>16</v>
+      </c>
+      <c r="R57" t="s">
+        <v>17</v>
+      </c>
+      <c r="S57" t="s">
+        <v>18</v>
+      </c>
+      <c r="T57" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="58" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A58" t="s">
+        <v>0</v>
+      </c>
+      <c r="B58" t="s">
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
+        <v>2</v>
+      </c>
+      <c r="D58" t="s">
+        <v>3</v>
+      </c>
+      <c r="E58" t="s">
+        <v>4</v>
+      </c>
+      <c r="F58" t="s">
+        <v>5</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H58" t="s">
+        <v>7</v>
+      </c>
+      <c r="I58" t="s">
+        <v>8</v>
+      </c>
+      <c r="J58" t="s">
+        <v>9</v>
+      </c>
+      <c r="K58" t="s">
+        <v>10</v>
+      </c>
+      <c r="L58" t="s">
+        <v>11</v>
+      </c>
+      <c r="M58" t="s">
+        <v>12</v>
+      </c>
+      <c r="N58" t="s">
+        <v>13</v>
+      </c>
+      <c r="O58" t="s">
+        <v>14</v>
+      </c>
+      <c r="P58">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q58">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R58">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S58">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T58">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="59" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A59" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B59" t="s">
         <v>21</v>
       </c>
-      <c r="C56">
+      <c r="C59">
         <v>4</v>
       </c>
-      <c r="D56">
-        <v>120375.156660901</v>
-      </c>
-      <c r="E56">
-        <v>282179.671232878</v>
-      </c>
-      <c r="F56">
-        <v>0.857351410648304</v>
-      </c>
-      <c r="G56" s="4">
-        <v>21285.1004075495</v>
-      </c>
-      <c r="H56">
-        <v>7426.32532798384</v>
-      </c>
-      <c r="I56">
-        <v>5046.79446201879</v>
-      </c>
-      <c r="J56">
-        <v>33758.220197552102</v>
-      </c>
-      <c r="K56">
-        <v>51144.191344099498</v>
-      </c>
-      <c r="L56">
-        <v>16112.7556071296</v>
-      </c>
-      <c r="M56">
-        <v>19359.989512119799</v>
-      </c>
-      <c r="N56">
-        <v>1006.77939378399</v>
-      </c>
-      <c r="O56">
-        <v>0</v>
-      </c>
-      <c r="P56">
-        <v>241927.13918778201</v>
-      </c>
-      <c r="Q56">
-        <v>1178.65858109644</v>
-      </c>
-      <c r="R56">
-        <v>12586.325853030899</v>
-      </c>
-      <c r="S56">
-        <v>466.16021677892502</v>
-      </c>
-      <c r="T56">
-        <v>1.3585822738026401</v>
-      </c>
-    </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="G57" s="4"/>
-    </row>
-    <row r="58" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A58" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G58" s="4"/>
-      <c r="P58" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q58" t="s">
-        <v>16</v>
-      </c>
-      <c r="R58" t="s">
-        <v>17</v>
-      </c>
-      <c r="S58" t="s">
-        <v>18</v>
-      </c>
-      <c r="T58" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="59" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A59" t="s">
-        <v>0</v>
-      </c>
-      <c r="B59" t="s">
-        <v>1</v>
-      </c>
-      <c r="C59" t="s">
+      <c r="D59">
+        <v>29525.427309999999</v>
+      </c>
+      <c r="E59">
+        <v>80391.755990000005</v>
+      </c>
+      <c r="F59">
+        <v>0.79280104200000001</v>
+      </c>
+      <c r="G59" s="4">
+        <v>5050.6365619999997</v>
+      </c>
+      <c r="H59">
+        <v>4678.3390820000004</v>
+      </c>
+      <c r="I59">
+        <v>2508.6600360000002</v>
+      </c>
+      <c r="J59">
+        <v>12237.635679999999</v>
+      </c>
+      <c r="K59">
+        <v>13920</v>
+      </c>
+      <c r="L59">
+        <v>2841.544922</v>
+      </c>
+      <c r="M59">
+        <v>5380.5444360000001</v>
+      </c>
+      <c r="N59">
+        <v>279.27307350000001</v>
+      </c>
+      <c r="O59">
+        <v>0</v>
+      </c>
+      <c r="P59">
+        <v>64865.028310000002</v>
+      </c>
+      <c r="Q59">
+        <v>1191.7509680000001</v>
+      </c>
+      <c r="R59">
+        <v>7243.7162129999997</v>
+      </c>
+      <c r="S59">
+        <v>452.7322633</v>
+      </c>
+      <c r="T59">
+        <v>5.8154128590000003</v>
+      </c>
+    </row>
+    <row r="60" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A60" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="62" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A62" t="s">
+        <v>33</v>
+      </c>
+      <c r="B62" t="s">
+        <v>34</v>
+      </c>
+      <c r="C62" t="s">
         <v>2</v>
       </c>
-      <c r="D59" t="s">
-        <v>3</v>
-      </c>
-      <c r="E59" t="s">
-        <v>4</v>
-      </c>
-      <c r="F59" t="s">
-        <v>5</v>
-      </c>
-      <c r="G59" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H59" t="s">
-        <v>7</v>
-      </c>
-      <c r="I59" t="s">
-        <v>8</v>
-      </c>
-      <c r="J59" t="s">
-        <v>9</v>
-      </c>
-      <c r="K59" t="s">
-        <v>10</v>
-      </c>
-      <c r="L59" t="s">
-        <v>11</v>
-      </c>
-      <c r="M59" t="s">
-        <v>12</v>
-      </c>
-      <c r="N59" t="s">
-        <v>13</v>
-      </c>
-      <c r="O59" t="s">
-        <v>14</v>
-      </c>
-      <c r="P59">
-        <v>63734.6679</v>
-      </c>
-      <c r="Q59">
-        <v>1078.4492829999999</v>
-      </c>
-      <c r="R59">
-        <v>624.70352849999995</v>
-      </c>
-      <c r="S59">
-        <v>13.014656840000001</v>
-      </c>
-      <c r="T59">
-        <v>27.514184579999998</v>
-      </c>
-    </row>
-    <row r="60" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A60" s="2" t="s">
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A63">
         <v>20</v>
       </c>
-      <c r="B60" t="s">
-        <v>21</v>
-      </c>
-      <c r="C60">
-        <v>4</v>
-      </c>
-      <c r="D60">
-        <v>29525.427309999999</v>
-      </c>
-      <c r="E60">
-        <v>80391.755990000005</v>
-      </c>
-      <c r="F60">
-        <v>0.79280104200000001</v>
-      </c>
-      <c r="G60" s="4">
-        <v>5050.6365619999997</v>
-      </c>
-      <c r="H60">
-        <v>4678.3390820000004</v>
-      </c>
-      <c r="I60">
-        <v>2508.6600360000002</v>
-      </c>
-      <c r="J60">
-        <v>12237.635679999999</v>
-      </c>
-      <c r="K60">
-        <v>13920</v>
-      </c>
-      <c r="L60">
-        <v>2841.544922</v>
-      </c>
-      <c r="M60">
-        <v>5380.5444360000001</v>
-      </c>
-      <c r="N60">
-        <v>279.27307350000001</v>
-      </c>
-      <c r="O60">
-        <v>0</v>
-      </c>
-      <c r="P60">
-        <v>64865.028310000002</v>
-      </c>
-      <c r="Q60">
-        <v>1191.7509680000001</v>
-      </c>
-      <c r="R60">
-        <v>7243.7162129999997</v>
-      </c>
-      <c r="S60">
-        <v>452.7322633</v>
-      </c>
-      <c r="T60">
-        <v>5.8154128590000003</v>
-      </c>
-    </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A61" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A63" t="s">
-        <v>34</v>
-      </c>
-      <c r="B63" t="s">
-        <v>35</v>
-      </c>
-      <c r="C63" t="s">
+      <c r="B63">
+        <v>60</v>
+      </c>
+      <c r="C63">
         <v>2</v>
+      </c>
+      <c r="D63">
+        <v>119696.652328767</v>
+      </c>
+      <c r="E63">
+        <v>282179.67123285501</v>
+      </c>
+      <c r="F63">
+        <v>0.854946898908852</v>
+      </c>
+      <c r="G63">
+        <v>18681.222424938602</v>
+      </c>
+      <c r="H63">
+        <v>5354.6114985546601</v>
+      </c>
+      <c r="I63">
+        <v>8156.08309050551</v>
+      </c>
+      <c r="J63">
+        <v>32191.917013998798</v>
+      </c>
+      <c r="K63">
+        <v>51372.124296964801</v>
+      </c>
+      <c r="L63">
+        <v>16725.325417965501</v>
+      </c>
+      <c r="M63">
+        <v>19407.285599838699</v>
+      </c>
+      <c r="N63">
+        <v>1016.03855436447</v>
+      </c>
+      <c r="O63">
+        <v>0</v>
+      </c>
+      <c r="P63">
+        <v>241248.634855649</v>
+      </c>
+      <c r="Q63">
+        <v>1192.7637589594799</v>
+      </c>
+      <c r="R63">
+        <v>19736.206339365101</v>
+      </c>
+      <c r="S63">
+        <v>481.37088632597801</v>
+      </c>
+      <c r="T63" s="6">
+        <v>0.12591688076390301</v>
       </c>
     </row>
     <row r="64" spans="1:20" x14ac:dyDescent="0.4">
@@ -3299,61 +3553,61 @@
         <v>20</v>
       </c>
       <c r="B64">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C64">
         <v>2</v>
       </c>
       <c r="D64">
-        <v>119696.652328767</v>
+        <v>118381.960809661</v>
       </c>
       <c r="E64">
-        <v>282179.67123285501</v>
+        <v>282254.81855225202</v>
       </c>
       <c r="F64">
-        <v>0.854946898908852</v>
+        <v>0.85006146065890897</v>
       </c>
       <c r="G64">
-        <v>18681.222424938602</v>
+        <v>19407.840072768398</v>
       </c>
       <c r="H64">
-        <v>5354.6114985546601</v>
+        <v>5891.8301217549197</v>
       </c>
       <c r="I64">
-        <v>8156.08309050551</v>
+        <v>6659.4942697455399</v>
       </c>
       <c r="J64">
-        <v>32191.917013998798</v>
+        <v>31959.164464268899</v>
       </c>
       <c r="K64">
-        <v>51372.124296964801</v>
+        <v>51102.045942938203</v>
       </c>
       <c r="L64">
-        <v>16725.325417965501</v>
+        <v>15967.176494174801</v>
       </c>
       <c r="M64">
-        <v>19407.285599838699</v>
+        <v>19353.573908279199</v>
       </c>
       <c r="N64">
-        <v>1016.03855436447</v>
+        <v>1010.46273302954</v>
       </c>
       <c r="O64">
         <v>0</v>
       </c>
       <c r="P64">
-        <v>241248.634855649</v>
+        <v>239933.943336542</v>
       </c>
       <c r="Q64">
-        <v>1192.7637589594799</v>
+        <v>1312.43161993582</v>
       </c>
       <c r="R64">
-        <v>19736.206339365101</v>
+        <v>18377.616631847999</v>
       </c>
       <c r="S64">
-        <v>481.37088632597801</v>
+        <v>459.4404157962</v>
       </c>
       <c r="T64" s="6">
-        <v>0.12591688076390301</v>
+        <v>0.14758705239613301</v>
       </c>
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.4">
@@ -3361,40 +3615,40 @@
         <v>20</v>
       </c>
       <c r="B65">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C65">
         <v>2</v>
       </c>
       <c r="D65">
-        <v>118381.960809661</v>
+        <v>116766.56672038</v>
       </c>
       <c r="E65">
-        <v>282254.81855225202</v>
+        <v>282179.67123287299</v>
       </c>
       <c r="F65">
-        <v>0.85006146065890897</v>
+        <v>0.84456314023622803</v>
       </c>
       <c r="G65">
-        <v>19407.840072768398</v>
+        <v>19298.245593088301</v>
       </c>
       <c r="H65">
-        <v>5891.8301217549197</v>
+        <v>5682.0016560700296</v>
       </c>
       <c r="I65">
-        <v>6659.4942697455399</v>
+        <v>5350.3346939491703</v>
       </c>
       <c r="J65">
-        <v>31959.164464268899</v>
+        <v>30330.5819431075</v>
       </c>
       <c r="K65">
-        <v>51102.045942938203</v>
+        <v>51097.733915068202</v>
       </c>
       <c r="L65">
-        <v>15967.176494174801</v>
+        <v>15987.901266609</v>
       </c>
       <c r="M65">
-        <v>19353.573908279199</v>
+        <v>19350.349595595701</v>
       </c>
       <c r="N65">
         <v>1010.46273302954</v>
@@ -3403,19 +3657,19 @@
         <v>0</v>
       </c>
       <c r="P65">
-        <v>239933.943336542</v>
+        <v>238318.54924726201</v>
       </c>
       <c r="Q65">
-        <v>1312.43161993582</v>
+        <v>1265.6913868611</v>
       </c>
       <c r="R65">
-        <v>18377.616631847999</v>
+        <v>17746.163883660702</v>
       </c>
       <c r="S65">
-        <v>459.4404157962</v>
+        <v>507.03325381887902</v>
       </c>
       <c r="T65" s="6">
-        <v>0.14758705239613301</v>
+        <v>-0.25983751983286502</v>
       </c>
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.4">
@@ -3423,102 +3677,102 @@
         <v>20</v>
       </c>
       <c r="B66">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C66">
         <v>2</v>
       </c>
       <c r="D66">
-        <v>116766.56672038</v>
+        <v>115610.996393592</v>
       </c>
       <c r="E66">
-        <v>282179.67123287299</v>
+        <v>282182.50548365602</v>
       </c>
       <c r="F66">
-        <v>0.84456314023622803</v>
+        <v>0.84045954058697003</v>
       </c>
       <c r="G66">
-        <v>19298.245593088301</v>
+        <v>19302.752565837702</v>
       </c>
       <c r="H66">
-        <v>5682.0016560700296</v>
+        <v>6226.5181629292701</v>
       </c>
       <c r="I66">
-        <v>5350.3346939491703</v>
+        <v>3974.5318253822402</v>
       </c>
       <c r="J66">
-        <v>30330.5819431075</v>
+        <v>29503.802554149199</v>
       </c>
       <c r="K66">
-        <v>51097.733915068202</v>
+        <v>51013.610661725899</v>
       </c>
       <c r="L66">
-        <v>15987.901266609</v>
+        <v>15760.601295416</v>
       </c>
       <c r="M66">
-        <v>19350.349595595701</v>
+        <v>19332.981882301501</v>
       </c>
       <c r="N66">
-        <v>1010.46273302954</v>
+        <v>1014.17312250211</v>
       </c>
       <c r="O66">
         <v>0</v>
       </c>
       <c r="P66">
-        <v>238318.54924726201</v>
+        <v>237162.97892047401</v>
       </c>
       <c r="Q66">
-        <v>1265.6913868611</v>
+        <v>1386.9848841974899</v>
       </c>
       <c r="R66">
-        <v>17746.163883660702</v>
+        <v>18436.445202769701</v>
       </c>
       <c r="S66">
-        <v>507.03325381887902</v>
+        <v>209.50505912238299</v>
       </c>
       <c r="T66" s="6">
-        <v>-0.25983751983286502</v>
+        <v>0.28049716262959101</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A67">
+      <c r="A67" s="3">
         <v>20</v>
       </c>
-      <c r="B67">
-        <v>30</v>
-      </c>
-      <c r="C67">
+      <c r="B67" s="3">
+        <v>20</v>
+      </c>
+      <c r="C67" s="3">
         <v>2</v>
       </c>
       <c r="D67">
-        <v>115610.996393592</v>
+        <v>114184.286860504</v>
       </c>
       <c r="E67">
-        <v>282182.50548365602</v>
+        <v>282179.67123297497</v>
       </c>
       <c r="F67">
-        <v>0.84045954058697003</v>
+        <v>0.83541194997266699</v>
       </c>
       <c r="G67">
-        <v>19302.752565837702</v>
+        <v>19351.2255529412</v>
       </c>
       <c r="H67">
-        <v>6226.5181629292701</v>
+        <v>6002.0469674603501</v>
       </c>
       <c r="I67">
-        <v>3974.5318253822402</v>
+        <v>2645.4376652921501</v>
       </c>
       <c r="J67">
-        <v>29503.802554149199</v>
+        <v>27998.710185693701</v>
       </c>
       <c r="K67">
-        <v>51013.610661725899</v>
+        <v>51033.4442867088</v>
       </c>
       <c r="L67">
-        <v>15760.601295416</v>
+        <v>15815.1228903871</v>
       </c>
       <c r="M67">
-        <v>19332.981882301501</v>
+        <v>19337.009497714302</v>
       </c>
       <c r="N67">
         <v>1014.17312250211</v>
@@ -3527,81 +3781,81 @@
         <v>0</v>
       </c>
       <c r="P67">
-        <v>237162.97892047401</v>
+        <v>235736.26938738499</v>
       </c>
       <c r="Q67">
-        <v>1386.9848841974899</v>
+        <v>1336.98290493166</v>
       </c>
       <c r="R67">
-        <v>18436.445202769701</v>
+        <v>18577.307877855899</v>
       </c>
       <c r="S67">
-        <v>209.50505912238299</v>
+        <v>432.030415764091</v>
       </c>
       <c r="T67" s="6">
-        <v>0.28049716262959101</v>
+        <v>-0.122490141098651</v>
       </c>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A68" s="3">
+      <c r="A68">
         <v>20</v>
       </c>
-      <c r="B68" s="3">
-        <v>20</v>
-      </c>
-      <c r="C68" s="3">
+      <c r="B68">
+        <v>15</v>
+      </c>
+      <c r="C68">
         <v>2</v>
       </c>
       <c r="D68">
-        <v>114184.286860504</v>
+        <v>113440.79599059001</v>
       </c>
       <c r="E68">
-        <v>282179.67123297497</v>
+        <v>282179.67123267101</v>
       </c>
       <c r="F68">
-        <v>0.83541194997266699</v>
+        <v>0.83277713625127903</v>
       </c>
       <c r="G68">
-        <v>19351.2255529412</v>
+        <v>19390.977969205</v>
       </c>
       <c r="H68">
-        <v>6002.0469674603501</v>
+        <v>5599.5405456203798</v>
       </c>
       <c r="I68">
-        <v>2645.4376652921501</v>
+        <v>2128.1287863747102</v>
       </c>
       <c r="J68">
-        <v>27998.710185693701</v>
+        <v>27118.647301200101</v>
       </c>
       <c r="K68">
-        <v>51033.4442867088</v>
+        <v>51068.507704320902</v>
       </c>
       <c r="L68">
-        <v>15815.1228903871</v>
+        <v>15909.3558282099</v>
       </c>
       <c r="M68">
-        <v>19337.009497714302</v>
+        <v>19344.285156859401</v>
       </c>
       <c r="N68">
-        <v>1014.17312250211</v>
+        <v>1010.46273302954</v>
       </c>
       <c r="O68">
         <v>0</v>
       </c>
       <c r="P68">
-        <v>235736.26938738499</v>
+        <v>234992.778517472</v>
       </c>
       <c r="Q68">
-        <v>1336.98290493166</v>
+        <v>1247.3228025527501</v>
       </c>
       <c r="R68">
-        <v>18577.307877855899</v>
+        <v>16417.502561416801</v>
       </c>
       <c r="S68">
-        <v>432.030415764091</v>
+        <v>469.07150175476602</v>
       </c>
       <c r="T68" s="6">
-        <v>-0.122490141098651</v>
+        <v>0.46004655114715598</v>
       </c>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.4">
@@ -3609,122 +3863,60 @@
         <v>20</v>
       </c>
       <c r="B69">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C69">
         <v>2</v>
       </c>
       <c r="D69">
-        <v>113440.79599059001</v>
+        <v>113795.448700252</v>
       </c>
       <c r="E69">
-        <v>282179.67123267101</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F69">
-        <v>0.83277713625127903</v>
+        <v>0.83403396920434802</v>
       </c>
       <c r="G69">
-        <v>19390.977969205</v>
+        <v>20436.472361711199</v>
       </c>
       <c r="H69">
-        <v>5599.5405456203798</v>
+        <v>4946.5396722567002</v>
       </c>
       <c r="I69">
-        <v>2128.1287863747102</v>
+        <v>2967.9237851293901</v>
       </c>
       <c r="J69">
-        <v>27118.647301200101</v>
+        <v>28350.9358190973</v>
       </c>
       <c r="K69">
-        <v>51068.507704320902</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L69">
-        <v>15909.3558282099</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M69">
-        <v>19344.285156859401</v>
+        <v>19297.530489448302</v>
       </c>
       <c r="N69">
-        <v>1010.46273302954</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O69">
         <v>0</v>
       </c>
       <c r="P69">
-        <v>234992.778517472</v>
+        <v>235347.43122713399</v>
       </c>
       <c r="Q69">
-        <v>1247.3228025527501</v>
+        <v>1101.8639118583401</v>
       </c>
       <c r="R69">
-        <v>16417.502561416801</v>
+        <v>13.380488321454299</v>
       </c>
       <c r="S69">
-        <v>469.07150175476602</v>
+        <v>2.67609766429086</v>
       </c>
       <c r="T69" s="6">
-        <v>0.46004655114715598</v>
-      </c>
-    </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A70">
-        <v>20</v>
-      </c>
-      <c r="B70">
-        <v>12</v>
-      </c>
-      <c r="C70">
-        <v>2</v>
-      </c>
-      <c r="D70">
-        <v>113795.448700252</v>
-      </c>
-      <c r="E70">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F70">
-        <v>0.83403396920434802</v>
-      </c>
-      <c r="G70">
-        <v>20436.472361711199</v>
-      </c>
-      <c r="H70">
-        <v>4946.5396722567002</v>
-      </c>
-      <c r="I70">
-        <v>2967.9237851293901</v>
-      </c>
-      <c r="J70">
-        <v>28350.9358190973</v>
-      </c>
-      <c r="K70">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L70">
-        <v>15303.798385783</v>
-      </c>
-      <c r="M70">
-        <v>19297.530489448302</v>
-      </c>
-      <c r="N70">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O70">
-        <v>0</v>
-      </c>
-      <c r="P70">
-        <v>235347.43122713399</v>
-      </c>
-      <c r="Q70">
-        <v>1101.8639118583401</v>
-      </c>
-      <c r="R70">
-        <v>13.380488321454299</v>
-      </c>
-      <c r="S70">
-        <v>2.67609766429086</v>
-      </c>
-      <c r="T70" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Redo-ing RTP baseline winter
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50825790-D006-4B37-8C89-7D5CA4787D57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0E7099-EC5D-4F93-8981-115085273E30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="440" windowWidth="19180" windowHeight="10060" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -227,7 +227,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -388,12 +388,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -2458,10 +2452,10 @@
       <c r="G33" s="4"/>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C34">
@@ -2470,7 +2464,7 @@
       <c r="D34">
         <v>247948.64160389101</v>
       </c>
-      <c r="E34">
+      <c r="E34" s="2">
         <v>374203.2</v>
       </c>
       <c r="F34">

</xml_diff>

<commit_message>
Moving a few files around
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0E7099-EC5D-4F93-8981-115085273E30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744A10FF-B0BC-44BA-A037-6FE019F0A0E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -38,6 +38,7 @@
     <author>tc={CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}</author>
     <author>tc={DFECE21F-32E0-4210-824A-1E57B1730184}</author>
     <author>tc={7128E1A1-FC03-4EA4-B47C-4E0569E512E5}</author>
+    <author>tc={D0DA4FB1-575F-4F90-BA19-F05AA3C8FBCE}</author>
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
     <author>tc={F9308CF0-AB74-4ABB-91B6-7382ECEADD39}</author>
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
@@ -69,7 +70,15 @@
     This is higher than the baseline because the solution is not optimal. It fails to optimize the UF pumps </t>
       </text>
     </comment>
-    <comment ref="A34" authorId="3" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A28" authorId="3" shapeId="0" xr:uid="{D0DA4FB1-575F-4F90-BA19-F05AA3C8FBCE}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    The operational plot is incorrect for this one</t>
+      </text>
+    </comment>
+    <comment ref="A34" authorId="4" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -77,7 +86,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="A35" authorId="4" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A35" authorId="5" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -85,7 +94,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T35" authorId="5" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T35" authorId="6" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -95,7 +104,7 @@
     The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A41" authorId="6" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A41" authorId="7" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -103,7 +112,7 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="T66" authorId="7" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T66" authorId="8" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -227,7 +236,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -388,6 +397,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -731,7 +746,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -740,6 +755,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1130,6 +1146,9 @@
   <threadedComment ref="Q27" dT="2026-07-02T17:46:58.68" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7128E1A1-FC03-4EA4-B47C-4E0569E512E5}">
     <text xml:space="preserve">This is higher than the baseline because the solution is not optimal. It fails to optimize the UF pumps </text>
   </threadedComment>
+  <threadedComment ref="A28" dT="2026-07-09T22:59:24.93" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{D0DA4FB1-575F-4F90-BA19-F05AA3C8FBCE}">
+    <text>The operational plot is incorrect for this one</text>
+  </threadedComment>
   <threadedComment ref="A34" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
@@ -2257,10 +2276,10 @@
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C28">
@@ -2452,44 +2471,44 @@
       <c r="G33" s="4"/>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="8" t="s">
         <v>23</v>
       </c>
       <c r="C34">
         <v>0</v>
       </c>
       <c r="D34">
-        <v>247948.64160389101</v>
-      </c>
-      <c r="E34" s="2">
-        <v>374203.2</v>
+        <v>116861.67991782499</v>
+      </c>
+      <c r="E34">
+        <v>282179.67123287602</v>
       </c>
       <c r="F34">
-        <v>0.98743309552342695</v>
-      </c>
-      <c r="G34" s="4">
-        <v>118659.96685142</v>
+        <v>0.84490020632262297</v>
+      </c>
+      <c r="G34">
+        <v>23556.420831705898</v>
       </c>
       <c r="H34">
-        <v>9240.5882208594503</v>
+        <v>6947.4542183048998</v>
       </c>
       <c r="I34">
-        <v>6738.6833231561404</v>
+        <v>913.29198665996</v>
       </c>
       <c r="J34">
-        <v>134639.23839543501</v>
+        <v>31417.167036670799</v>
       </c>
       <c r="K34">
-        <v>67424.000002171</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L34">
-        <v>20294.624005833801</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M34">
-        <v>25590.779200450401</v>
+        <v>19297.5304894482</v>
       </c>
       <c r="N34">
         <v>992.31070788530405</v>
@@ -2498,10 +2517,10 @@
         <v>0</v>
       </c>
       <c r="P34">
-        <v>369500.62413077202</v>
+        <v>238413.66244470701</v>
       </c>
       <c r="Q34">
-        <v>1466.60671595592</v>
+        <v>1102.6552392369899</v>
       </c>
       <c r="R34">
         <v>0</v>
@@ -2514,10 +2533,10 @@
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A35" t="s">
+      <c r="A35" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="8" t="s">
         <v>23</v>
       </c>
       <c r="C35">

</xml_diff>

<commit_message>
Adding plot function that reads operational data from plant data
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744A10FF-B0BC-44BA-A037-6FE019F0A0E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA4F3F07-B4D1-4F9F-B174-9FD48C489CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -43,6 +43,7 @@
     <author>tc={F9308CF0-AB74-4ABB-91B6-7382ECEADD39}</author>
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
     <author>tc={7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}</author>
+    <author>tc={9FF6B967-6104-43AC-8EED-15C48C9ACCA9}</author>
     <author>tc={86E634AB-9E52-4A6D-BE85-5D191C9227C6}</author>
   </authors>
   <commentList>
@@ -112,7 +113,15 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="T66" authorId="8" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="A58" authorId="8" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
+      </text>
+    </comment>
+    <comment ref="T70" authorId="9" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -125,7 +134,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="38">
   <si>
     <t>Season</t>
   </si>
@@ -230,6 +239,15 @@
   </si>
   <si>
     <t>On-Peak Demand Charge</t>
+  </si>
+  <si>
+    <t>Higher Water Target, TOU 3</t>
+  </si>
+  <si>
+    <t>real data</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -746,7 +764,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -755,7 +773,6 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1164,7 +1181,10 @@
   <threadedComment ref="A41" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
     <text>Result from the fast solve</text>
   </threadedComment>
-  <threadedComment ref="T66" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="A58" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
+  </threadedComment>
+  <threadedComment ref="T70" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1172,7 +1192,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:T69"/>
+  <dimension ref="A1:T73"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="9.61328125" customWidth="1"/>
@@ -2471,10 +2491,10 @@
       <c r="G33" s="4"/>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C34">
@@ -2533,10 +2553,10 @@
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C35">
@@ -3350,475 +3370,339 @@
     <row r="56" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G56" s="4"/>
     </row>
-    <row r="57" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A57" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G57" s="4"/>
+    </row>
+    <row r="58" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A58" t="s">
+        <v>22</v>
+      </c>
+      <c r="B58" t="s">
+        <v>21</v>
+      </c>
+      <c r="C58">
+        <v>4</v>
+      </c>
+      <c r="D58">
+        <v>146108.01933512901</v>
+      </c>
+      <c r="E58">
+        <v>355610.364944759</v>
+      </c>
+      <c r="F58">
+        <v>0.75267772890587503</v>
+      </c>
+      <c r="G58">
+        <v>25765.651662743599</v>
+      </c>
+      <c r="H58">
+        <v>7150.9042815892099</v>
+      </c>
+      <c r="I58">
+        <v>5144.3184852884797</v>
+      </c>
+      <c r="J58">
+        <v>38060.874429621297</v>
+      </c>
+      <c r="K58">
+        <v>64168.339029134899</v>
+      </c>
+      <c r="L58">
+        <v>19539.954214541001</v>
+      </c>
+      <c r="M58">
+        <v>24338.851661831999</v>
+      </c>
+      <c r="N58">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O58">
+        <v>0</v>
+      </c>
+      <c r="P58">
+        <v>267660.00186201098</v>
+      </c>
+      <c r="Q58">
+        <v>1597.68911089628</v>
+      </c>
+      <c r="R58">
+        <v>13084.0423994256</v>
+      </c>
+      <c r="S58">
+        <v>467.28722855091399</v>
+      </c>
+      <c r="T58">
+        <v>-0.25904927491985202</v>
+      </c>
+    </row>
+    <row r="59" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A59" t="s">
+        <v>22</v>
+      </c>
+      <c r="B59" t="s">
+        <v>36</v>
+      </c>
+      <c r="C59" t="s">
+        <v>36</v>
+      </c>
+      <c r="D59" t="s">
+        <v>37</v>
+      </c>
+      <c r="E59" t="s">
+        <v>37</v>
+      </c>
+      <c r="F59" t="s">
+        <v>37</v>
+      </c>
+      <c r="G59" s="4">
+        <v>28838</v>
+      </c>
+      <c r="H59">
+        <v>7567.5</v>
+      </c>
+      <c r="I59">
+        <v>13764.1</v>
+      </c>
+      <c r="J59">
+        <v>50169.7</v>
+      </c>
+      <c r="K59" t="s">
+        <v>37</v>
+      </c>
+      <c r="L59" t="s">
+        <v>37</v>
+      </c>
+      <c r="M59" t="s">
+        <v>37</v>
+      </c>
+      <c r="N59" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="61" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A61" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G57" s="4"/>
-      <c r="P57" t="s">
+      <c r="G61" s="4"/>
+      <c r="P61" t="s">
         <v>15</v>
       </c>
-      <c r="Q57" t="s">
+      <c r="Q61" t="s">
         <v>16</v>
       </c>
-      <c r="R57" t="s">
+      <c r="R61" t="s">
         <v>17</v>
       </c>
-      <c r="S57" t="s">
+      <c r="S61" t="s">
         <v>18</v>
       </c>
-      <c r="T57" t="s">
+      <c r="T61" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="58" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A58" t="s">
-        <v>0</v>
-      </c>
-      <c r="B58" t="s">
+    <row r="62" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B62" t="s">
         <v>1</v>
-      </c>
-      <c r="C58" t="s">
-        <v>2</v>
-      </c>
-      <c r="D58" t="s">
-        <v>3</v>
-      </c>
-      <c r="E58" t="s">
-        <v>4</v>
-      </c>
-      <c r="F58" t="s">
-        <v>5</v>
-      </c>
-      <c r="G58" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H58" t="s">
-        <v>7</v>
-      </c>
-      <c r="I58" t="s">
-        <v>8</v>
-      </c>
-      <c r="J58" t="s">
-        <v>9</v>
-      </c>
-      <c r="K58" t="s">
-        <v>10</v>
-      </c>
-      <c r="L58" t="s">
-        <v>11</v>
-      </c>
-      <c r="M58" t="s">
-        <v>12</v>
-      </c>
-      <c r="N58" t="s">
-        <v>13</v>
-      </c>
-      <c r="O58" t="s">
-        <v>14</v>
-      </c>
-      <c r="P58">
-        <v>63734.6679</v>
-      </c>
-      <c r="Q58">
-        <v>1078.4492829999999</v>
-      </c>
-      <c r="R58">
-        <v>624.70352849999995</v>
-      </c>
-      <c r="S58">
-        <v>13.014656840000001</v>
-      </c>
-      <c r="T58">
-        <v>27.514184579999998</v>
-      </c>
-    </row>
-    <row r="59" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A59" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B59" t="s">
-        <v>21</v>
-      </c>
-      <c r="C59">
-        <v>4</v>
-      </c>
-      <c r="D59">
-        <v>29525.427309999999</v>
-      </c>
-      <c r="E59">
-        <v>80391.755990000005</v>
-      </c>
-      <c r="F59">
-        <v>0.79280104200000001</v>
-      </c>
-      <c r="G59" s="4">
-        <v>5050.6365619999997</v>
-      </c>
-      <c r="H59">
-        <v>4678.3390820000004</v>
-      </c>
-      <c r="I59">
-        <v>2508.6600360000002</v>
-      </c>
-      <c r="J59">
-        <v>12237.635679999999</v>
-      </c>
-      <c r="K59">
-        <v>13920</v>
-      </c>
-      <c r="L59">
-        <v>2841.544922</v>
-      </c>
-      <c r="M59">
-        <v>5380.5444360000001</v>
-      </c>
-      <c r="N59">
-        <v>279.27307350000001</v>
-      </c>
-      <c r="O59">
-        <v>0</v>
-      </c>
-      <c r="P59">
-        <v>64865.028310000002</v>
-      </c>
-      <c r="Q59">
-        <v>1191.7509680000001</v>
-      </c>
-      <c r="R59">
-        <v>7243.7162129999997</v>
-      </c>
-      <c r="S59">
-        <v>452.7322633</v>
-      </c>
-      <c r="T59">
-        <v>5.8154128590000003</v>
-      </c>
-    </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A60" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A62" t="s">
-        <v>33</v>
-      </c>
-      <c r="B62" t="s">
-        <v>34</v>
       </c>
       <c r="C62" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A63">
+      <c r="D62" t="s">
+        <v>3</v>
+      </c>
+      <c r="E62" t="s">
+        <v>4</v>
+      </c>
+      <c r="F62" t="s">
+        <v>5</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H62" t="s">
+        <v>7</v>
+      </c>
+      <c r="I62" t="s">
+        <v>8</v>
+      </c>
+      <c r="J62" t="s">
+        <v>9</v>
+      </c>
+      <c r="K62" t="s">
+        <v>10</v>
+      </c>
+      <c r="L62" t="s">
+        <v>11</v>
+      </c>
+      <c r="M62" t="s">
+        <v>12</v>
+      </c>
+      <c r="N62" t="s">
+        <v>13</v>
+      </c>
+      <c r="O62" t="s">
+        <v>14</v>
+      </c>
+      <c r="P62">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q62">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R62">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S62">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T62">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="63" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A63" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B63">
+      <c r="B63" t="s">
+        <v>21</v>
+      </c>
+      <c r="C63">
+        <v>4</v>
+      </c>
+      <c r="D63">
+        <v>29525.427309999999</v>
+      </c>
+      <c r="E63">
+        <v>80391.755990000005</v>
+      </c>
+      <c r="F63">
+        <v>0.79280104200000001</v>
+      </c>
+      <c r="G63" s="4">
+        <v>5050.6365619999997</v>
+      </c>
+      <c r="H63">
+        <v>4678.3390820000004</v>
+      </c>
+      <c r="I63">
+        <v>2508.6600360000002</v>
+      </c>
+      <c r="J63">
+        <v>12237.635679999999</v>
+      </c>
+      <c r="K63">
+        <v>13920</v>
+      </c>
+      <c r="L63">
+        <v>2841.544922</v>
+      </c>
+      <c r="M63">
+        <v>5380.5444360000001</v>
+      </c>
+      <c r="N63">
+        <v>279.27307350000001</v>
+      </c>
+      <c r="O63">
+        <v>0</v>
+      </c>
+      <c r="P63">
+        <v>64865.028310000002</v>
+      </c>
+      <c r="Q63">
+        <v>1191.7509680000001</v>
+      </c>
+      <c r="R63">
+        <v>7243.7162129999997</v>
+      </c>
+      <c r="S63">
+        <v>452.7322633</v>
+      </c>
+      <c r="T63">
+        <v>5.8154128590000003</v>
+      </c>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A64" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="66" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A66" t="s">
+        <v>33</v>
+      </c>
+      <c r="B66" t="s">
+        <v>34</v>
+      </c>
+      <c r="C66" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A67">
+        <v>20</v>
+      </c>
+      <c r="B67">
         <v>60</v>
       </c>
-      <c r="C63">
+      <c r="C67">
         <v>2</v>
       </c>
-      <c r="D63">
+      <c r="D67">
         <v>119696.652328767</v>
       </c>
-      <c r="E63">
+      <c r="E67">
         <v>282179.67123285501</v>
       </c>
-      <c r="F63">
+      <c r="F67">
         <v>0.854946898908852</v>
       </c>
-      <c r="G63">
+      <c r="G67">
         <v>18681.222424938602</v>
       </c>
-      <c r="H63">
+      <c r="H67">
         <v>5354.6114985546601</v>
       </c>
-      <c r="I63">
+      <c r="I67">
         <v>8156.08309050551</v>
       </c>
-      <c r="J63">
+      <c r="J67">
         <v>32191.917013998798</v>
       </c>
-      <c r="K63">
+      <c r="K67">
         <v>51372.124296964801</v>
       </c>
-      <c r="L63">
+      <c r="L67">
         <v>16725.325417965501</v>
       </c>
-      <c r="M63">
+      <c r="M67">
         <v>19407.285599838699</v>
       </c>
-      <c r="N63">
+      <c r="N67">
         <v>1016.03855436447</v>
       </c>
-      <c r="O63">
-        <v>0</v>
-      </c>
-      <c r="P63">
+      <c r="O67">
+        <v>0</v>
+      </c>
+      <c r="P67">
         <v>241248.634855649</v>
       </c>
-      <c r="Q63">
+      <c r="Q67">
         <v>1192.7637589594799</v>
       </c>
-      <c r="R63">
+      <c r="R67">
         <v>19736.206339365101</v>
       </c>
-      <c r="S63">
+      <c r="S67">
         <v>481.37088632597801</v>
       </c>
-      <c r="T63" s="6">
+      <c r="T67" s="6">
         <v>0.12591688076390301</v>
-      </c>
-    </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A64">
-        <v>20</v>
-      </c>
-      <c r="B64">
-        <v>50</v>
-      </c>
-      <c r="C64">
-        <v>2</v>
-      </c>
-      <c r="D64">
-        <v>118381.960809661</v>
-      </c>
-      <c r="E64">
-        <v>282254.81855225202</v>
-      </c>
-      <c r="F64">
-        <v>0.85006146065890897</v>
-      </c>
-      <c r="G64">
-        <v>19407.840072768398</v>
-      </c>
-      <c r="H64">
-        <v>5891.8301217549197</v>
-      </c>
-      <c r="I64">
-        <v>6659.4942697455399</v>
-      </c>
-      <c r="J64">
-        <v>31959.164464268899</v>
-      </c>
-      <c r="K64">
-        <v>51102.045942938203</v>
-      </c>
-      <c r="L64">
-        <v>15967.176494174801</v>
-      </c>
-      <c r="M64">
-        <v>19353.573908279199</v>
-      </c>
-      <c r="N64">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O64">
-        <v>0</v>
-      </c>
-      <c r="P64">
-        <v>239933.943336542</v>
-      </c>
-      <c r="Q64">
-        <v>1312.43161993582</v>
-      </c>
-      <c r="R64">
-        <v>18377.616631847999</v>
-      </c>
-      <c r="S64">
-        <v>459.4404157962</v>
-      </c>
-      <c r="T64" s="6">
-        <v>0.14758705239613301</v>
-      </c>
-    </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A65">
-        <v>20</v>
-      </c>
-      <c r="B65">
-        <v>40</v>
-      </c>
-      <c r="C65">
-        <v>2</v>
-      </c>
-      <c r="D65">
-        <v>116766.56672038</v>
-      </c>
-      <c r="E65">
-        <v>282179.67123287299</v>
-      </c>
-      <c r="F65">
-        <v>0.84456314023622803</v>
-      </c>
-      <c r="G65">
-        <v>19298.245593088301</v>
-      </c>
-      <c r="H65">
-        <v>5682.0016560700296</v>
-      </c>
-      <c r="I65">
-        <v>5350.3346939491703</v>
-      </c>
-      <c r="J65">
-        <v>30330.5819431075</v>
-      </c>
-      <c r="K65">
-        <v>51097.733915068202</v>
-      </c>
-      <c r="L65">
-        <v>15987.901266609</v>
-      </c>
-      <c r="M65">
-        <v>19350.349595595701</v>
-      </c>
-      <c r="N65">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O65">
-        <v>0</v>
-      </c>
-      <c r="P65">
-        <v>238318.54924726201</v>
-      </c>
-      <c r="Q65">
-        <v>1265.6913868611</v>
-      </c>
-      <c r="R65">
-        <v>17746.163883660702</v>
-      </c>
-      <c r="S65">
-        <v>507.03325381887902</v>
-      </c>
-      <c r="T65" s="6">
-        <v>-0.25983751983286502</v>
-      </c>
-    </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A66">
-        <v>20</v>
-      </c>
-      <c r="B66">
-        <v>30</v>
-      </c>
-      <c r="C66">
-        <v>2</v>
-      </c>
-      <c r="D66">
-        <v>115610.996393592</v>
-      </c>
-      <c r="E66">
-        <v>282182.50548365602</v>
-      </c>
-      <c r="F66">
-        <v>0.84045954058697003</v>
-      </c>
-      <c r="G66">
-        <v>19302.752565837702</v>
-      </c>
-      <c r="H66">
-        <v>6226.5181629292701</v>
-      </c>
-      <c r="I66">
-        <v>3974.5318253822402</v>
-      </c>
-      <c r="J66">
-        <v>29503.802554149199</v>
-      </c>
-      <c r="K66">
-        <v>51013.610661725899</v>
-      </c>
-      <c r="L66">
-        <v>15760.601295416</v>
-      </c>
-      <c r="M66">
-        <v>19332.981882301501</v>
-      </c>
-      <c r="N66">
-        <v>1014.17312250211</v>
-      </c>
-      <c r="O66">
-        <v>0</v>
-      </c>
-      <c r="P66">
-        <v>237162.97892047401</v>
-      </c>
-      <c r="Q66">
-        <v>1386.9848841974899</v>
-      </c>
-      <c r="R66">
-        <v>18436.445202769701</v>
-      </c>
-      <c r="S66">
-        <v>209.50505912238299</v>
-      </c>
-      <c r="T66" s="6">
-        <v>0.28049716262959101</v>
-      </c>
-    </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A67" s="3">
-        <v>20</v>
-      </c>
-      <c r="B67" s="3">
-        <v>20</v>
-      </c>
-      <c r="C67" s="3">
-        <v>2</v>
-      </c>
-      <c r="D67">
-        <v>114184.286860504</v>
-      </c>
-      <c r="E67">
-        <v>282179.67123297497</v>
-      </c>
-      <c r="F67">
-        <v>0.83541194997266699</v>
-      </c>
-      <c r="G67">
-        <v>19351.2255529412</v>
-      </c>
-      <c r="H67">
-        <v>6002.0469674603501</v>
-      </c>
-      <c r="I67">
-        <v>2645.4376652921501</v>
-      </c>
-      <c r="J67">
-        <v>27998.710185693701</v>
-      </c>
-      <c r="K67">
-        <v>51033.4442867088</v>
-      </c>
-      <c r="L67">
-        <v>15815.1228903871</v>
-      </c>
-      <c r="M67">
-        <v>19337.009497714302</v>
-      </c>
-      <c r="N67">
-        <v>1014.17312250211</v>
-      </c>
-      <c r="O67">
-        <v>0</v>
-      </c>
-      <c r="P67">
-        <v>235736.26938738499</v>
-      </c>
-      <c r="Q67">
-        <v>1336.98290493166</v>
-      </c>
-      <c r="R67">
-        <v>18577.307877855899</v>
-      </c>
-      <c r="S67">
-        <v>432.030415764091</v>
-      </c>
-      <c r="T67" s="6">
-        <v>-0.122490141098651</v>
       </c>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.4">
@@ -3826,40 +3710,40 @@
         <v>20</v>
       </c>
       <c r="B68">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C68">
         <v>2</v>
       </c>
       <c r="D68">
-        <v>113440.79599059001</v>
+        <v>118381.960809661</v>
       </c>
       <c r="E68">
-        <v>282179.67123267101</v>
+        <v>282254.81855225202</v>
       </c>
       <c r="F68">
-        <v>0.83277713625127903</v>
+        <v>0.85006146065890897</v>
       </c>
       <c r="G68">
-        <v>19390.977969205</v>
+        <v>19407.840072768398</v>
       </c>
       <c r="H68">
-        <v>5599.5405456203798</v>
+        <v>5891.8301217549197</v>
       </c>
       <c r="I68">
-        <v>2128.1287863747102</v>
+        <v>6659.4942697455399</v>
       </c>
       <c r="J68">
-        <v>27118.647301200101</v>
+        <v>31959.164464268899</v>
       </c>
       <c r="K68">
-        <v>51068.507704320902</v>
+        <v>51102.045942938203</v>
       </c>
       <c r="L68">
-        <v>15909.3558282099</v>
+        <v>15967.176494174801</v>
       </c>
       <c r="M68">
-        <v>19344.285156859401</v>
+        <v>19353.573908279199</v>
       </c>
       <c r="N68">
         <v>1010.46273302954</v>
@@ -3868,19 +3752,19 @@
         <v>0</v>
       </c>
       <c r="P68">
-        <v>234992.778517472</v>
+        <v>239933.943336542</v>
       </c>
       <c r="Q68">
-        <v>1247.3228025527501</v>
+        <v>1312.43161993582</v>
       </c>
       <c r="R68">
-        <v>16417.502561416801</v>
+        <v>18377.616631847999</v>
       </c>
       <c r="S68">
-        <v>469.07150175476602</v>
+        <v>459.4404157962</v>
       </c>
       <c r="T68" s="6">
-        <v>0.46004655114715598</v>
+        <v>0.14758705239613301</v>
       </c>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.4">
@@ -3888,60 +3772,308 @@
         <v>20</v>
       </c>
       <c r="B69">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C69">
         <v>2</v>
       </c>
       <c r="D69">
+        <v>116766.56672038</v>
+      </c>
+      <c r="E69">
+        <v>282179.67123287299</v>
+      </c>
+      <c r="F69">
+        <v>0.84456314023622803</v>
+      </c>
+      <c r="G69">
+        <v>19298.245593088301</v>
+      </c>
+      <c r="H69">
+        <v>5682.0016560700296</v>
+      </c>
+      <c r="I69">
+        <v>5350.3346939491703</v>
+      </c>
+      <c r="J69">
+        <v>30330.5819431075</v>
+      </c>
+      <c r="K69">
+        <v>51097.733915068202</v>
+      </c>
+      <c r="L69">
+        <v>15987.901266609</v>
+      </c>
+      <c r="M69">
+        <v>19350.349595595701</v>
+      </c>
+      <c r="N69">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O69">
+        <v>0</v>
+      </c>
+      <c r="P69">
+        <v>238318.54924726201</v>
+      </c>
+      <c r="Q69">
+        <v>1265.6913868611</v>
+      </c>
+      <c r="R69">
+        <v>17746.163883660702</v>
+      </c>
+      <c r="S69">
+        <v>507.03325381887902</v>
+      </c>
+      <c r="T69" s="6">
+        <v>-0.25983751983286502</v>
+      </c>
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A70">
+        <v>20</v>
+      </c>
+      <c r="B70">
+        <v>30</v>
+      </c>
+      <c r="C70">
+        <v>2</v>
+      </c>
+      <c r="D70">
+        <v>115610.996393592</v>
+      </c>
+      <c r="E70">
+        <v>282182.50548365602</v>
+      </c>
+      <c r="F70">
+        <v>0.84045954058697003</v>
+      </c>
+      <c r="G70">
+        <v>19302.752565837702</v>
+      </c>
+      <c r="H70">
+        <v>6226.5181629292701</v>
+      </c>
+      <c r="I70">
+        <v>3974.5318253822402</v>
+      </c>
+      <c r="J70">
+        <v>29503.802554149199</v>
+      </c>
+      <c r="K70">
+        <v>51013.610661725899</v>
+      </c>
+      <c r="L70">
+        <v>15760.601295416</v>
+      </c>
+      <c r="M70">
+        <v>19332.981882301501</v>
+      </c>
+      <c r="N70">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O70">
+        <v>0</v>
+      </c>
+      <c r="P70">
+        <v>237162.97892047401</v>
+      </c>
+      <c r="Q70">
+        <v>1386.9848841974899</v>
+      </c>
+      <c r="R70">
+        <v>18436.445202769701</v>
+      </c>
+      <c r="S70">
+        <v>209.50505912238299</v>
+      </c>
+      <c r="T70" s="6">
+        <v>0.28049716262959101</v>
+      </c>
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A71" s="3">
+        <v>20</v>
+      </c>
+      <c r="B71" s="3">
+        <v>20</v>
+      </c>
+      <c r="C71" s="3">
+        <v>2</v>
+      </c>
+      <c r="D71">
+        <v>114184.286860504</v>
+      </c>
+      <c r="E71">
+        <v>282179.67123297497</v>
+      </c>
+      <c r="F71">
+        <v>0.83541194997266699</v>
+      </c>
+      <c r="G71">
+        <v>19351.2255529412</v>
+      </c>
+      <c r="H71">
+        <v>6002.0469674603501</v>
+      </c>
+      <c r="I71">
+        <v>2645.4376652921501</v>
+      </c>
+      <c r="J71">
+        <v>27998.710185693701</v>
+      </c>
+      <c r="K71">
+        <v>51033.4442867088</v>
+      </c>
+      <c r="L71">
+        <v>15815.1228903871</v>
+      </c>
+      <c r="M71">
+        <v>19337.009497714302</v>
+      </c>
+      <c r="N71">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O71">
+        <v>0</v>
+      </c>
+      <c r="P71">
+        <v>235736.26938738499</v>
+      </c>
+      <c r="Q71">
+        <v>1336.98290493166</v>
+      </c>
+      <c r="R71">
+        <v>18577.307877855899</v>
+      </c>
+      <c r="S71">
+        <v>432.030415764091</v>
+      </c>
+      <c r="T71" s="6">
+        <v>-0.122490141098651</v>
+      </c>
+    </row>
+    <row r="72" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A72">
+        <v>20</v>
+      </c>
+      <c r="B72">
+        <v>15</v>
+      </c>
+      <c r="C72">
+        <v>2</v>
+      </c>
+      <c r="D72">
+        <v>113440.79599059001</v>
+      </c>
+      <c r="E72">
+        <v>282179.67123267101</v>
+      </c>
+      <c r="F72">
+        <v>0.83277713625127903</v>
+      </c>
+      <c r="G72">
+        <v>19390.977969205</v>
+      </c>
+      <c r="H72">
+        <v>5599.5405456203798</v>
+      </c>
+      <c r="I72">
+        <v>2128.1287863747102</v>
+      </c>
+      <c r="J72">
+        <v>27118.647301200101</v>
+      </c>
+      <c r="K72">
+        <v>51068.507704320902</v>
+      </c>
+      <c r="L72">
+        <v>15909.3558282099</v>
+      </c>
+      <c r="M72">
+        <v>19344.285156859401</v>
+      </c>
+      <c r="N72">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O72">
+        <v>0</v>
+      </c>
+      <c r="P72">
+        <v>234992.778517472</v>
+      </c>
+      <c r="Q72">
+        <v>1247.3228025527501</v>
+      </c>
+      <c r="R72">
+        <v>16417.502561416801</v>
+      </c>
+      <c r="S72">
+        <v>469.07150175476602</v>
+      </c>
+      <c r="T72" s="6">
+        <v>0.46004655114715598</v>
+      </c>
+    </row>
+    <row r="73" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A73">
+        <v>20</v>
+      </c>
+      <c r="B73">
+        <v>12</v>
+      </c>
+      <c r="C73">
+        <v>2</v>
+      </c>
+      <c r="D73">
         <v>113795.448700252</v>
       </c>
-      <c r="E69">
+      <c r="E73">
         <v>282179.67123287602</v>
       </c>
-      <c r="F69">
+      <c r="F73">
         <v>0.83403396920434802</v>
       </c>
-      <c r="G69">
+      <c r="G73">
         <v>20436.472361711199</v>
       </c>
-      <c r="H69">
+      <c r="H73">
         <v>4946.5396722567002</v>
       </c>
-      <c r="I69">
+      <c r="I73">
         <v>2967.9237851293901</v>
       </c>
-      <c r="J69">
+      <c r="J73">
         <v>28350.9358190973</v>
       </c>
-      <c r="K69">
+      <c r="K73">
         <v>50843.184005923598</v>
       </c>
-      <c r="L69">
+      <c r="L73">
         <v>15303.798385783</v>
       </c>
-      <c r="M69">
+      <c r="M73">
         <v>19297.530489448302</v>
       </c>
-      <c r="N69">
+      <c r="N73">
         <v>992.31070788530405</v>
       </c>
-      <c r="O69">
-        <v>0</v>
-      </c>
-      <c r="P69">
+      <c r="O73">
+        <v>0</v>
+      </c>
+      <c r="P73">
         <v>235347.43122713399</v>
       </c>
-      <c r="Q69">
+      <c r="Q73">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R69">
+      <c r="R73">
         <v>13.380488321454299</v>
       </c>
-      <c r="S69">
+      <c r="S73">
         <v>2.67609766429086</v>
       </c>
-      <c r="T69" s="6">
+      <c r="T73" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>

</xml_diff>

<commit_message>
rerunning this case because plot is messed up
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA4F3F07-B4D1-4F9F-B174-9FD48C489CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -254,7 +254,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -415,12 +415,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">

</xml_diff>

<commit_message>
Copying over some csvs to make plots
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E492B944-4B4E-4BB0-866E-1AE18DD8C0CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F53ED5E-622A-433B-A196-2934A1CA2B2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -35,9 +35,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={CF8F1CCE-34DF-4D83-A6E8-651B12C72B40}</author>
     <author>tc={CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}</author>
     <author>tc={DFECE21F-32E0-4210-824A-1E57B1730184}</author>
     <author>tc={7128E1A1-FC03-4EA4-B47C-4E0569E512E5}</author>
+    <author>tc={FA39747C-8399-4DE8-BFC3-16508DD92F20}</author>
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
     <author>tc={F9308CF0-AB74-4ABB-91B6-7382ECEADD39}</author>
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
@@ -46,7 +48,15 @@
     <author>tc={86E634AB-9E52-4A6D-BE85-5D191C9227C6}</author>
   </authors>
   <commentList>
-    <comment ref="A16" authorId="0" shapeId="0" xr:uid="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
+    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{CF8F1CCE-34DF-4D83-A6E8-651B12C72B40}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This one is surprising to me… like shouldn’t it decrease the flowrate during peak hours a bit and increase slightly during off peak hours??</t>
+      </text>
+    </comment>
+    <comment ref="A16" authorId="1" shapeId="0" xr:uid="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -54,7 +64,7 @@
     This should be the same as the baseline</t>
       </text>
     </comment>
-    <comment ref="A25" authorId="1" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
+    <comment ref="A25" authorId="2" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -62,7 +72,7 @@
     Curious if solver would eventually find same solution as the 4 flex trains</t>
       </text>
     </comment>
-    <comment ref="Q27" authorId="2" shapeId="0" xr:uid="{7128E1A1-FC03-4EA4-B47C-4E0569E512E5}">
+    <comment ref="Q27" authorId="3" shapeId="0" xr:uid="{7128E1A1-FC03-4EA4-B47C-4E0569E512E5}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -70,7 +80,15 @@
     This is higher than the baseline because the solution is not optimal. It fails to optimize the UF pumps </t>
       </text>
     </comment>
-    <comment ref="A34" authorId="3" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A28" authorId="4" shapeId="0" xr:uid="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</t>
+      </text>
+    </comment>
+    <comment ref="A34" authorId="5" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -78,7 +96,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="A35" authorId="4" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A35" authorId="6" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -86,7 +104,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T35" authorId="5" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T35" authorId="7" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -96,7 +114,7 @@
     The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A41" authorId="6" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A41" authorId="8" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -104,7 +122,7 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="A58" authorId="7" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A58" authorId="9" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -112,7 +130,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T70" authorId="8" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T70" authorId="10" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -223,9 +241,6 @@
     <t>TOU 8</t>
   </si>
   <si>
-    <t>Simplified Rate Structures</t>
-  </si>
-  <si>
     <t>Off-Peak Demand Charge</t>
   </si>
   <si>
@@ -240,12 +255,15 @@
   <si>
     <t>N/A</t>
   </si>
+  <si>
+    <t>Simplified Rate Structure</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -406,6 +424,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1139,6 +1163,9 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A13" dT="2026-07-15T17:46:07.17" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{CF8F1CCE-34DF-4D83-A6E8-651B12C72B40}">
+    <text>This one is surprising to me… like shouldn’t it decrease the flowrate during peak hours a bit and increase slightly during off peak hours??</text>
+  </threadedComment>
   <threadedComment ref="A16" dT="2026-07-01T17:37:32.24" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
     <text>This should be the same as the baseline</text>
   </threadedComment>
@@ -1147,6 +1174,9 @@
   </threadedComment>
   <threadedComment ref="Q27" dT="2026-07-02T17:46:58.68" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7128E1A1-FC03-4EA4-B47C-4E0569E512E5}">
     <text xml:space="preserve">This is higher than the baseline because the solution is not optimal. It fails to optimize the UF pumps </text>
+  </threadedComment>
+  <threadedComment ref="A28" dT="2026-07-15T17:22:40.80" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
+    <text>This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</text>
   </threadedComment>
   <threadedComment ref="A34" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
@@ -1956,55 +1986,55 @@
         <v>2</v>
       </c>
       <c r="D19">
-        <v>118409.31653290401</v>
+        <v>117965.918152322</v>
       </c>
       <c r="E19">
         <v>282179.67123287602</v>
       </c>
       <c r="F19">
-        <v>0.85038478502496795</v>
+        <v>0.84881345148898202</v>
       </c>
       <c r="G19">
-        <v>20330.773698750199</v>
+        <v>19987.387727355999</v>
       </c>
       <c r="H19">
-        <v>6573.3255592595497</v>
+        <v>6536.1025167957996</v>
       </c>
       <c r="I19">
-        <v>6060.70439374338</v>
+        <v>5997.9150270156997</v>
       </c>
       <c r="J19">
-        <v>32964.803651753202</v>
+        <v>32521.405271167499</v>
       </c>
       <c r="K19">
-        <v>50843.184005922703</v>
+        <v>50843.1840059237</v>
       </c>
       <c r="L19">
-        <v>15303.798385780299</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M19">
-        <v>19297.5304894482</v>
+        <v>19297.530489448302</v>
       </c>
       <c r="N19">
-        <v>999.49269129581296</v>
+        <v>1010.46273302954</v>
       </c>
       <c r="O19">
         <v>0</v>
       </c>
       <c r="P19">
-        <v>239961.29905978599</v>
+        <v>239517.900679204</v>
       </c>
       <c r="Q19">
-        <v>1468.64372040951</v>
+        <v>1460.3271566616399</v>
       </c>
       <c r="R19">
-        <v>17615.608874695899</v>
+        <v>17682.539594118301</v>
       </c>
       <c r="S19">
-        <v>266.90316476812001</v>
+        <v>148.59276969847301</v>
       </c>
       <c r="T19">
-        <v>9.6260597723556093E-2</v>
+        <v>0.12159211918729</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.4">
@@ -2278,7 +2308,7 @@
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A28" t="s">
+      <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B28" t="s">
@@ -3354,7 +3384,7 @@
     </row>
     <row r="57" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A57" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G57" s="4"/>
     </row>
@@ -3425,19 +3455,19 @@
         <v>22</v>
       </c>
       <c r="B59" t="s">
+        <v>35</v>
+      </c>
+      <c r="C59" t="s">
+        <v>35</v>
+      </c>
+      <c r="D59" t="s">
         <v>36</v>
       </c>
-      <c r="C59" t="s">
+      <c r="E59" t="s">
         <v>36</v>
       </c>
-      <c r="D59" t="s">
-        <v>37</v>
-      </c>
-      <c r="E59" t="s">
-        <v>37</v>
-      </c>
       <c r="F59" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G59" s="4">
         <v>28838</v>
@@ -3452,16 +3482,16 @@
         <v>50169.7</v>
       </c>
       <c r="K59" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L59" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M59" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N59" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="61" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
@@ -3611,15 +3641,15 @@
     </row>
     <row r="64" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A64" s="7" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A66" t="s">
+        <v>32</v>
+      </c>
+      <c r="B66" t="s">
         <v>33</v>
-      </c>
-      <c r="B66" t="s">
-        <v>34</v>
       </c>
       <c r="C66" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
new replacement cost calculation
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F53ED5E-622A-433B-A196-2934A1CA2B2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E9F0CA-90CC-48E7-8DB8-22AAA1487469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-69" yWindow="-69" windowWidth="33052" windowHeight="17932" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -35,6 +35,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={BBF7D234-FE30-40AB-877C-48487A60B475}</author>
     <author>tc={CF8F1CCE-34DF-4D83-A6E8-651B12C72B40}</author>
     <author>tc={CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}</author>
     <author>tc={DFECE21F-32E0-4210-824A-1E57B1730184}</author>
@@ -48,7 +49,15 @@
     <author>tc={86E634AB-9E52-4A6D-BE85-5D191C9227C6}</author>
   </authors>
   <commentList>
-    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{CF8F1CCE-34DF-4D83-A6E8-651B12C72B40}">
+    <comment ref="N2" authorId="0" shapeId="0" xr:uid="{BBF7D234-FE30-40AB-877C-48487A60B475}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Will need to update with new numbers</t>
+      </text>
+    </comment>
+    <comment ref="A13" authorId="1" shapeId="0" xr:uid="{CF8F1CCE-34DF-4D83-A6E8-651B12C72B40}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -56,7 +65,7 @@
     This one is surprising to me… like shouldn’t it decrease the flowrate during peak hours a bit and increase slightly during off peak hours??</t>
       </text>
     </comment>
-    <comment ref="A16" authorId="1" shapeId="0" xr:uid="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
+    <comment ref="A16" authorId="2" shapeId="0" xr:uid="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -64,7 +73,7 @@
     This should be the same as the baseline</t>
       </text>
     </comment>
-    <comment ref="A25" authorId="2" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
+    <comment ref="A25" authorId="3" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -72,7 +81,7 @@
     Curious if solver would eventually find same solution as the 4 flex trains</t>
       </text>
     </comment>
-    <comment ref="Q27" authorId="3" shapeId="0" xr:uid="{7128E1A1-FC03-4EA4-B47C-4E0569E512E5}">
+    <comment ref="Q27" authorId="4" shapeId="0" xr:uid="{7128E1A1-FC03-4EA4-B47C-4E0569E512E5}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -80,7 +89,7 @@
     This is higher than the baseline because the solution is not optimal. It fails to optimize the UF pumps </t>
       </text>
     </comment>
-    <comment ref="A28" authorId="4" shapeId="0" xr:uid="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
+    <comment ref="A28" authorId="5" shapeId="0" xr:uid="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -88,7 +97,7 @@
     This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</t>
       </text>
     </comment>
-    <comment ref="A34" authorId="5" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A34" authorId="6" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -96,7 +105,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="A35" authorId="6" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A35" authorId="7" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -104,7 +113,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T35" authorId="7" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T35" authorId="8" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -114,7 +123,7 @@
     The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A41" authorId="8" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A41" authorId="9" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -122,7 +131,7 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="A58" authorId="9" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A58" authorId="10" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -130,7 +139,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T70" authorId="10" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T70" authorId="11" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1163,6 +1172,9 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="N2" dT="2026-07-15T21:03:49.32" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{BBF7D234-FE30-40AB-877C-48487A60B475}">
+    <text>Will need to update with new numbers</text>
+  </threadedComment>
   <threadedComment ref="A13" dT="2026-07-15T17:46:07.17" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{CF8F1CCE-34DF-4D83-A6E8-651B12C72B40}">
     <text>This one is surprising to me… like shouldn’t it decrease the flowrate during peak hours a bit and increase slightly during off peak hours??</text>
   </threadedComment>
@@ -1262,7 +1274,7 @@
       <c r="M2" t="s">
         <v>12</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" s="2" t="s">
         <v>13</v>
       </c>
       <c r="O2" t="s">

</xml_diff>

<commit_message>
Double checking these results with much tighter mip gap
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E9F0CA-90CC-48E7-8DB8-22AAA1487469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F186C33-9DAD-4F63-A920-DC829DCFDC58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-69" yWindow="-69" windowWidth="33052" windowHeight="17932" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={BBF7D234-FE30-40AB-877C-48487A60B475}</author>
-    <author>tc={CF8F1CCE-34DF-4D83-A6E8-651B12C72B40}</author>
+    <author>tc={73C7F34A-BCA8-44F2-A992-5B81BCD419CF}</author>
     <author>tc={CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}</author>
     <author>tc={DFECE21F-32E0-4210-824A-1E57B1730184}</author>
     <author>tc={7128E1A1-FC03-4EA4-B47C-4E0569E512E5}</author>
@@ -57,12 +57,12 @@
     Will need to update with new numbers</t>
       </text>
     </comment>
-    <comment ref="A13" authorId="1" shapeId="0" xr:uid="{CF8F1CCE-34DF-4D83-A6E8-651B12C72B40}">
+    <comment ref="A12" authorId="1" shapeId="0" xr:uid="{73C7F34A-BCA8-44F2-A992-5B81BCD419CF}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    This one is surprising to me… like shouldn’t it decrease the flowrate during peak hours a bit and increase slightly during off peak hours??</t>
+    Not sure I trust this results anymore</t>
       </text>
     </comment>
     <comment ref="A16" authorId="2" shapeId="0" xr:uid="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
@@ -438,7 +438,7 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1175,8 +1175,8 @@
   <threadedComment ref="N2" dT="2026-07-15T21:03:49.32" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{BBF7D234-FE30-40AB-877C-48487A60B475}">
     <text>Will need to update with new numbers</text>
   </threadedComment>
-  <threadedComment ref="A13" dT="2026-07-15T17:46:07.17" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{CF8F1CCE-34DF-4D83-A6E8-651B12C72B40}">
-    <text>This one is surprising to me… like shouldn’t it decrease the flowrate during peak hours a bit and increase slightly during off peak hours??</text>
+  <threadedComment ref="A12" dT="2026-07-15T22:24:25.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{73C7F34A-BCA8-44F2-A992-5B81BCD419CF}">
+    <text>Not sure I trust this results anymore</text>
   </threadedComment>
   <threadedComment ref="A16" dT="2026-07-01T17:37:32.24" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
     <text>This should be the same as the baseline</text>
@@ -1486,10 +1486,10 @@
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C7">
@@ -1613,10 +1613,10 @@
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C10">
@@ -1750,34 +1750,34 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <v>120105.62640119799</v>
+        <v>118611.04844584499</v>
       </c>
       <c r="E13">
-        <v>282179.67123287602</v>
+        <v>282179.67177163501</v>
       </c>
       <c r="F13">
-        <v>0.85639623815652299</v>
-      </c>
-      <c r="G13" s="4">
-        <v>20632.008189972999</v>
+        <v>0.85109968930394098</v>
+      </c>
+      <c r="G13">
+        <v>20424.331721278701</v>
       </c>
       <c r="H13">
-        <v>4931.94871395263</v>
+        <v>5117.5665325995597</v>
       </c>
       <c r="I13">
-        <v>9097.1451203198394</v>
+        <v>7308.5385824584</v>
       </c>
       <c r="J13">
-        <v>34661.102024245498</v>
+        <v>32850.436836336601</v>
       </c>
       <c r="K13">
-        <v>50843.186957348102</v>
+        <v>50924.339061968501</v>
       </c>
       <c r="L13">
-        <v>15303.8063177357</v>
+        <v>15521.9023672608</v>
       </c>
       <c r="M13">
-        <v>19297.531101868899</v>
+        <v>19314.3701802791</v>
       </c>
       <c r="N13">
         <v>992.31070788530405</v>
@@ -1786,19 +1786,19 @@
         <v>0</v>
       </c>
       <c r="P13">
-        <v>241657.60892808001</v>
+        <v>240163.03097272699</v>
       </c>
       <c r="Q13">
-        <v>1101.9194839550801</v>
+        <v>1143.3910977538401</v>
       </c>
       <c r="R13">
-        <v>0</v>
+        <v>5393.7865087666896</v>
       </c>
       <c r="S13">
-        <v>0</v>
+        <v>215.751460350667</v>
       </c>
       <c r="T13">
-        <v>0</v>
+        <v>0.33425013552507798</v>
       </c>
     </row>
     <row r="14" spans="1:20" hidden="1" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
LVOF included flow related costs. testing output
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F186C33-9DAD-4F63-A920-DC829DCFDC58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EDCB346-0E45-45BB-A8E9-788E32D18483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -36,6 +36,8 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={BBF7D234-FE30-40AB-877C-48487A60B475}</author>
+    <author>tc={508D361C-2D0C-49BA-974D-6C72FE37C504}</author>
+    <author>tc={F27CC18C-9CF0-4B96-A7C0-3CA554F9A587}</author>
     <author>tc={73C7F34A-BCA8-44F2-A992-5B81BCD419CF}</author>
     <author>tc={CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}</author>
     <author>tc={DFECE21F-32E0-4210-824A-1E57B1730184}</author>
@@ -57,7 +59,23 @@
     Will need to update with new numbers</t>
       </text>
     </comment>
-    <comment ref="A12" authorId="1" shapeId="0" xr:uid="{73C7F34A-BCA8-44F2-A992-5B81BCD419CF}">
+    <comment ref="S2" authorId="1" shapeId="0" xr:uid="{508D361C-2D0C-49BA-974D-6C72FE37C504}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This isn’t being calculated correctly...</t>
+      </text>
+    </comment>
+    <comment ref="A7" authorId="2" shapeId="0" xr:uid="{F27CC18C-9CF0-4B96-A7C0-3CA554F9A587}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This will of course give the baseline because it is already at the maximum recovery- there is no potential for charging capacity</t>
+      </text>
+    </comment>
+    <comment ref="A12" authorId="3" shapeId="0" xr:uid="{73C7F34A-BCA8-44F2-A992-5B81BCD419CF}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -65,7 +83,7 @@
     Not sure I trust this results anymore</t>
       </text>
     </comment>
-    <comment ref="A16" authorId="2" shapeId="0" xr:uid="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
+    <comment ref="A16" authorId="4" shapeId="0" xr:uid="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -73,7 +91,7 @@
     This should be the same as the baseline</t>
       </text>
     </comment>
-    <comment ref="A25" authorId="3" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
+    <comment ref="A25" authorId="5" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -81,7 +99,7 @@
     Curious if solver would eventually find same solution as the 4 flex trains</t>
       </text>
     </comment>
-    <comment ref="Q27" authorId="4" shapeId="0" xr:uid="{7128E1A1-FC03-4EA4-B47C-4E0569E512E5}">
+    <comment ref="Q27" authorId="6" shapeId="0" xr:uid="{7128E1A1-FC03-4EA4-B47C-4E0569E512E5}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -89,7 +107,7 @@
     This is higher than the baseline because the solution is not optimal. It fails to optimize the UF pumps </t>
       </text>
     </comment>
-    <comment ref="A28" authorId="5" shapeId="0" xr:uid="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
+    <comment ref="A28" authorId="7" shapeId="0" xr:uid="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -97,7 +115,7 @@
     This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</t>
       </text>
     </comment>
-    <comment ref="A34" authorId="6" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A34" authorId="8" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -105,7 +123,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="A35" authorId="7" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A35" authorId="9" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -113,7 +131,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T35" authorId="8" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T35" authorId="10" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -123,7 +141,7 @@
     The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A41" authorId="9" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A41" authorId="11" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -131,7 +149,7 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="A58" authorId="10" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A58" authorId="12" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -139,7 +157,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T70" authorId="11" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T70" authorId="13" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -438,7 +456,7 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1175,6 +1193,12 @@
   <threadedComment ref="N2" dT="2026-07-15T21:03:49.32" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{BBF7D234-FE30-40AB-877C-48487A60B475}">
     <text>Will need to update with new numbers</text>
   </threadedComment>
+  <threadedComment ref="S2" dT="2026-07-15T22:57:33.93" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{508D361C-2D0C-49BA-974D-6C72FE37C504}">
+    <text>This isn’t being calculated correctly...</text>
+  </threadedComment>
+  <threadedComment ref="A7" dT="2026-07-15T23:37:51.28" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F27CC18C-9CF0-4B96-A7C0-3CA554F9A587}">
+    <text>This will of course give the baseline because it is already at the maximum recovery- there is no potential for charging capacity</text>
+  </threadedComment>
   <threadedComment ref="A12" dT="2026-07-15T22:24:25.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{73C7F34A-BCA8-44F2-A992-5B81BCD419CF}">
     <text>Not sure I trust this results anymore</text>
   </threadedComment>
@@ -1289,7 +1313,7 @@
       <c r="R2" t="s">
         <v>17</v>
       </c>
-      <c r="S2" t="s">
+      <c r="S2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="T2" t="s">
@@ -1486,10 +1510,10 @@
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C7">
@@ -1613,10 +1637,10 @@
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C10">
@@ -1740,10 +1764,10 @@
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C13">
@@ -1794,7 +1818,7 @@
       <c r="R13">
         <v>5393.7865087666896</v>
       </c>
-      <c r="S13">
+      <c r="S13" s="5">
         <v>215.751460350667</v>
       </c>
       <c r="T13">
@@ -2042,7 +2066,7 @@
       <c r="R19">
         <v>17682.539594118301</v>
       </c>
-      <c r="S19">
+      <c r="S19" s="2">
         <v>148.59276969847301</v>
       </c>
       <c r="T19">
@@ -2052,6 +2076,7 @@
     <row r="20" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
+      <c r="S20" s="2"/>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
@@ -2119,7 +2144,7 @@
       <c r="R22">
         <v>17686.324085333301</v>
       </c>
-      <c r="S22">
+      <c r="S22" s="2">
         <v>149.88410241807901</v>
       </c>
       <c r="T22">
@@ -2246,7 +2271,7 @@
       <c r="R25">
         <v>15990.3109099755</v>
       </c>
-      <c r="S25">
+      <c r="S25" s="2">
         <v>135.51110940657199</v>
       </c>
       <c r="T25">
@@ -2374,7 +2399,7 @@
       <c r="R28">
         <v>20030.045592225699</v>
       </c>
-      <c r="S28">
+      <c r="S28" s="2">
         <v>178.83969278772901</v>
       </c>
       <c r="T28">
@@ -2447,10 +2472,10 @@
       </c>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C31">
@@ -2501,7 +2526,7 @@
       <c r="R31">
         <v>13651.1458247473</v>
       </c>
-      <c r="S31">
+      <c r="S31" s="2">
         <v>115.68767648091</v>
       </c>
       <c r="T31">

</xml_diff>

<commit_message>
Running basic full flex again with small mip gap
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EDCB346-0E45-45BB-A8E9-788E32D18483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E839DB60-1000-4C22-9DFC-074DBBECDA4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -80,7 +80,7 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Not sure I trust this results anymore</t>
+    This result still make sense because: the recovery change would cause an extra cost that outweighs the tiny electricity savings.</t>
       </text>
     </comment>
     <comment ref="A16" authorId="4" shapeId="0" xr:uid="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
@@ -290,7 +290,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -451,12 +451,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1200,7 +1194,7 @@
     <text>This will of course give the baseline because it is already at the maximum recovery- there is no potential for charging capacity</text>
   </threadedComment>
   <threadedComment ref="A12" dT="2026-07-15T22:24:25.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{73C7F34A-BCA8-44F2-A992-5B81BCD419CF}">
-    <text>Not sure I trust this results anymore</text>
+    <text>This result still make sense because: the recovery change would cause an extra cost that outweighs the tiny electricity savings.</text>
   </threadedComment>
   <threadedComment ref="A16" dT="2026-07-01T17:37:32.24" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
     <text>This should be the same as the baseline</text>

</xml_diff>

<commit_message>
Adding other rate structures
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E839DB60-1000-4C22-9DFC-074DBBECDA4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B249FF1E-39FC-45D1-8F1C-BAD1C73129A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="11730" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,9 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Curious if solver would eventually find same solution as the 4 flex trains</t>
+    So IMO the definition of “flexible trains is strange here. Shouldn’t the first two trains have operations totally fixed? Currently, this just prevents trains one and two from turning off
+Reply:
+    Which yields (somewhat obviously) the same result as 4 flexible trains</t>
       </text>
     </comment>
     <comment ref="Q27" authorId="6" shapeId="0" xr:uid="{7128E1A1-FC03-4EA4-B47C-4E0569E512E5}">
@@ -115,7 +117,7 @@
     This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</t>
       </text>
     </comment>
-    <comment ref="A34" authorId="8" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A38" authorId="8" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -123,7 +125,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="A35" authorId="9" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A39" authorId="9" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -131,7 +133,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T35" authorId="10" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T39" authorId="10" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -141,7 +143,7 @@
     The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A41" authorId="11" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A45" authorId="11" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -149,7 +151,7 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="A58" authorId="12" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A62" authorId="12" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -157,7 +159,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T70" authorId="13" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T74" authorId="13" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -170,7 +172,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="41">
   <si>
     <t>Season</t>
   </si>
@@ -284,6 +286,15 @@
   </si>
   <si>
     <t>Simplified Rate Structure</t>
+  </si>
+  <si>
+    <t>TOU 3 2026</t>
+  </si>
+  <si>
+    <t>Charge Energy Capacity</t>
+  </si>
+  <si>
+    <t>Charge Power Capacity</t>
   </si>
 </sst>
 </file>
@@ -1200,7 +1211,10 @@
     <text>This should be the same as the baseline</text>
   </threadedComment>
   <threadedComment ref="A25" dT="2026-06-11T20:38:07.96" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{DFECE21F-32E0-4210-824A-1E57B1730184}">
-    <text>Curious if solver would eventually find same solution as the 4 flex trains</text>
+    <text>So IMO the definition of “flexible trains is strange here. Shouldn’t the first two trains have operations totally fixed? Currently, this just prevents trains one and two from turning off</text>
+  </threadedComment>
+  <threadedComment ref="A25" dT="2026-07-17T16:31:03.99" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{668DBC5A-3C1B-4BF9-8368-F26E80CE9B35}" parentId="{DFECE21F-32E0-4210-824A-1E57B1730184}">
+    <text>Which yields (somewhat obviously) the same result as 4 flexible trains</text>
   </threadedComment>
   <threadedComment ref="Q27" dT="2026-07-02T17:46:58.68" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7128E1A1-FC03-4EA4-B47C-4E0569E512E5}">
     <text xml:space="preserve">This is higher than the baseline because the solution is not optimal. It fails to optimize the UF pumps </text>
@@ -1208,25 +1222,25 @@
   <threadedComment ref="A28" dT="2026-07-15T17:22:40.80" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
     <text>This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</text>
   </threadedComment>
-  <threadedComment ref="A34" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+  <threadedComment ref="A38" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
-  <threadedComment ref="A35" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+  <threadedComment ref="A39" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
     <text>Summer week = hot summer weekdays + high weekends</text>
   </threadedComment>
-  <threadedComment ref="T35" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T39" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure</text>
   </threadedComment>
-  <threadedComment ref="T35" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T39" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>The baseline costs have to be updated in accordance with the demand structure type</text>
   </threadedComment>
-  <threadedComment ref="A41" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+  <threadedComment ref="A45" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
     <text>Result from the fast solve</text>
   </threadedComment>
-  <threadedComment ref="A58" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+  <threadedComment ref="A62" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
     <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
   </threadedComment>
-  <threadedComment ref="T70" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="T74" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1234,25 +1248,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:T73"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:V77"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.61328125" customWidth="1"/>
-    <col min="3" max="3" width="11.4609375" customWidth="1"/>
-    <col min="5" max="5" width="10.23046875" customWidth="1"/>
-    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.69140625" customWidth="1"/>
-    <col min="9" max="9" width="9.07421875" customWidth="1"/>
-    <col min="15" max="15" width="9.53515625" customWidth="1"/>
-    <col min="20" max="20" width="7.84375" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" customWidth="1"/>
+    <col min="3" max="3" width="11.453125" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="15" max="15" width="9.54296875" customWidth="1"/>
+    <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1313,8 +1327,14 @@
       <c r="T2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="U2" t="s">
+        <v>39</v>
+      </c>
+      <c r="V2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1376,7 +1396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1438,10 +1458,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1503,7 +1523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -1565,10 +1585,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1630,7 +1650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -1692,10 +1712,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -1757,7 +1777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -1819,10 +1839,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1884,7 +1904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -1940,10 +1960,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2005,7 +2025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2067,12 +2087,12 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2083,7 +2103,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2145,10 +2165,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2210,7 +2230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2221,62 +2241,68 @@
         <v>2</v>
       </c>
       <c r="D25">
-        <v>117590.90519865</v>
+        <v>116354.41551491299</v>
       </c>
       <c r="E25">
-        <v>282179.671232878</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F25">
-        <v>0.84748446505974995</v>
+        <v>0.84310254173290999</v>
       </c>
       <c r="G25">
-        <v>19872.5530246782</v>
+        <v>19840.537050750401</v>
       </c>
       <c r="H25">
-        <v>5801.3546413486602</v>
+        <v>5280.6330826172398</v>
       </c>
       <c r="I25">
-        <v>5871.6372791994399</v>
+        <v>4877.4899493259099</v>
       </c>
       <c r="J25">
-        <v>31545.544945226298</v>
+        <v>29998.660082693601</v>
       </c>
       <c r="K25">
-        <v>50997.445205479402</v>
+        <v>51077.135880394701</v>
       </c>
       <c r="L25">
-        <v>15718.375359588401</v>
+        <v>15932.544048423801</v>
       </c>
       <c r="M25">
-        <v>19329.539688356101</v>
+        <v>19346.075503401102</v>
       </c>
       <c r="N25">
-        <v>1001.30446052474</v>
+        <v>1427.7916964369099</v>
       </c>
       <c r="O25">
         <v>0</v>
       </c>
       <c r="P25">
-        <v>239142.887725532</v>
+        <v>237906.39804179501</v>
       </c>
       <c r="Q25">
-        <v>1296.16628121386</v>
+        <v>1179.82420335646</v>
       </c>
       <c r="R25">
-        <v>15990.3109099755</v>
-      </c>
-      <c r="S25" s="2">
-        <v>135.51110940657199</v>
+        <v>12780.012944633199</v>
+      </c>
+      <c r="S25">
+        <v>511.20051778532797</v>
       </c>
       <c r="T25">
-        <v>1.20740363486328</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.4">
+        <v>0.18120426001776399</v>
+      </c>
+      <c r="U25">
+        <v>11081.318719635499</v>
+      </c>
+      <c r="V25">
+        <v>77.491739298150407</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2338,7 +2364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2400,10 +2426,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>20</v>
       </c>
@@ -2465,303 +2491,145 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A31" s="2" t="s">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C31">
         <v>4</v>
       </c>
       <c r="D31">
-        <v>117493.882010934</v>
+        <v>116354.41551491299</v>
       </c>
       <c r="E31">
-        <v>282179.67123284901</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F31">
-        <v>0.84714063027084496</v>
+        <v>0.84310254173290999</v>
       </c>
       <c r="G31">
-        <v>19869.854426770002</v>
+        <v>19840.537050750401</v>
       </c>
       <c r="H31">
-        <v>5589.63461833969</v>
+        <v>5280.6330826172398</v>
       </c>
       <c r="I31">
-        <v>5989.0327102104202</v>
+        <v>4877.4899493259099</v>
       </c>
       <c r="J31">
-        <v>31448.5217553201</v>
+        <v>29998.660082693601</v>
       </c>
       <c r="K31">
-        <v>50997.445205592398</v>
+        <v>51077.135880394701</v>
       </c>
       <c r="L31">
-        <v>15718.3753616421</v>
+        <v>15932.544048423801</v>
       </c>
       <c r="M31">
-        <v>19329.5396883797</v>
+        <v>19346.075503401102</v>
       </c>
       <c r="N31">
-        <v>1001.30446052474</v>
+        <v>1427.7916964369099</v>
       </c>
       <c r="O31">
         <v>0</v>
       </c>
       <c r="P31">
-        <v>239045.864537816</v>
+        <v>237906.39804179501</v>
       </c>
       <c r="Q31">
-        <v>1248.8628027930299</v>
+        <v>1179.82420335646</v>
       </c>
       <c r="R31">
-        <v>13651.1458247473</v>
-      </c>
-      <c r="S31" s="2">
-        <v>115.68767648091</v>
+        <v>12780.012944633199</v>
+      </c>
+      <c r="S31">
+        <v>511.20051778532797</v>
       </c>
       <c r="T31">
-        <v>1.42140322536358</v>
-      </c>
-    </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A33" s="1" t="s">
+        <v>0.18120426001776399</v>
+      </c>
+      <c r="U31">
+        <v>11081.318719635499</v>
+      </c>
+      <c r="V31">
+        <v>77.491739298150407</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="S32" s="2"/>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A33" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="S33" s="2"/>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A34" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" s="2"/>
+      <c r="S34" s="2"/>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A35" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B35" s="2"/>
+      <c r="S35" s="2"/>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G33" s="4"/>
-    </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A34" s="5" t="s">
+      <c r="G37" s="4"/>
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A38" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B38" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C34">
-        <v>0</v>
-      </c>
-      <c r="D34">
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38">
         <v>116861.67991782499</v>
       </c>
-      <c r="E34">
+      <c r="E38">
         <v>282179.67123287602</v>
       </c>
-      <c r="F34">
+      <c r="F38">
         <v>0.84490020632262297</v>
       </c>
-      <c r="G34">
+      <c r="G38">
         <v>23556.420831705898</v>
       </c>
-      <c r="H34">
+      <c r="H38">
         <v>6947.4542183048998</v>
       </c>
-      <c r="I34">
+      <c r="I38">
         <v>913.29198665996</v>
       </c>
-      <c r="J34">
+      <c r="J38">
         <v>31417.167036670799</v>
       </c>
-      <c r="K34">
+      <c r="K38">
         <v>50843.184005923598</v>
       </c>
-      <c r="L34">
+      <c r="L38">
         <v>15303.798385783</v>
       </c>
-      <c r="M34">
+      <c r="M38">
         <v>19297.5304894482</v>
-      </c>
-      <c r="N34">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O34">
-        <v>0</v>
-      </c>
-      <c r="P34">
-        <v>238413.66244470701</v>
-      </c>
-      <c r="Q34">
-        <v>1102.6552392369899</v>
-      </c>
-      <c r="R34">
-        <v>0</v>
-      </c>
-      <c r="S34">
-        <v>0</v>
-      </c>
-      <c r="T34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A35" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
-      <c r="D35">
-        <v>187020.456722612</v>
-      </c>
-      <c r="E35">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F35">
-        <v>1.09353178385</v>
-      </c>
-      <c r="G35">
-        <v>89520.694507565597</v>
-      </c>
-      <c r="H35">
-        <v>6971.3813103080802</v>
-      </c>
-      <c r="I35">
-        <v>5083.8680235841202</v>
-      </c>
-      <c r="J35">
-        <v>101575.943841457</v>
-      </c>
-      <c r="K35">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L35">
-        <v>15303.798385783</v>
-      </c>
-      <c r="M35">
-        <v>19297.5304894482</v>
-      </c>
-      <c r="N35">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O35">
-        <v>0</v>
-      </c>
-      <c r="P35">
-        <v>308572.439249494</v>
-      </c>
-      <c r="Q35">
-        <v>1106.4527933521999</v>
-      </c>
-      <c r="R35">
-        <v>3451.9307168288801</v>
-      </c>
-      <c r="S35">
-        <v>20.547206647791</v>
-      </c>
-      <c r="T35">
-        <v>-14.696886263168601</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A36" s="3"/>
-      <c r="G36" s="4"/>
-    </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A37" t="s">
-        <v>20</v>
-      </c>
-      <c r="B37" t="s">
-        <v>21</v>
-      </c>
-      <c r="C37">
-        <v>0</v>
-      </c>
-      <c r="D37">
-        <v>117032.41959359701</v>
-      </c>
-      <c r="E37">
-        <v>282179.67123286898</v>
-      </c>
-      <c r="F37">
-        <v>0.845505280653571</v>
-      </c>
-      <c r="G37" s="4">
-        <v>23683.129427060001</v>
-      </c>
-      <c r="H37">
-        <v>6986.3695969997798</v>
-      </c>
-      <c r="I37">
-        <v>918.40768838365295</v>
-      </c>
-      <c r="J37">
-        <v>31587.906712443499</v>
-      </c>
-      <c r="K37">
-        <v>50843.1840059237</v>
-      </c>
-      <c r="L37">
-        <v>15303.7983857823</v>
-      </c>
-      <c r="M37">
-        <v>19297.530489448101</v>
-      </c>
-      <c r="N37">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O37">
-        <v>0</v>
-      </c>
-      <c r="P37">
-        <v>238584.402120479</v>
-      </c>
-      <c r="Q37">
-        <v>1108.83163779344</v>
-      </c>
-      <c r="R37">
-        <v>0</v>
-      </c>
-      <c r="S37">
-        <v>230512.59606633501</v>
-      </c>
-      <c r="T37">
-        <v>1103.3673370121001</v>
-      </c>
-    </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A38" t="s">
-        <v>22</v>
-      </c>
-      <c r="B38" t="s">
-        <v>21</v>
-      </c>
-      <c r="C38">
-        <v>0</v>
-      </c>
-      <c r="D38">
-        <v>171564.02128394699</v>
-      </c>
-      <c r="E38">
-        <v>282179.67123287701</v>
-      </c>
-      <c r="F38">
-        <v>1.03875662810921</v>
-      </c>
-      <c r="G38">
-        <v>73514.1870928641</v>
-      </c>
-      <c r="H38">
-        <v>7482.8438362204697</v>
-      </c>
-      <c r="I38">
-        <v>4044.9309872213798</v>
-      </c>
-      <c r="J38">
-        <v>85041.961916305998</v>
-      </c>
-      <c r="K38">
-        <v>51119.832654572398</v>
-      </c>
-      <c r="L38">
-        <v>16047.2916290263</v>
-      </c>
-      <c r="M38">
-        <v>19354.9350840429</v>
       </c>
       <c r="N38">
         <v>992.31070788530405</v>
@@ -2770,658 +2638,721 @@
         <v>0</v>
       </c>
       <c r="P38">
-        <v>293116.00381082902</v>
+        <v>238413.66244470701</v>
       </c>
       <c r="Q38">
-        <v>1187.62883512946</v>
+        <v>1102.6552392369899</v>
       </c>
       <c r="R38">
-        <v>9393.8913494494009</v>
+        <v>0</v>
       </c>
       <c r="S38">
-        <v>260.94142637359403</v>
+        <v>0</v>
       </c>
       <c r="T38">
-        <v>-3.6405201993767098</v>
-      </c>
-    </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="G39" s="4"/>
-    </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A40" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A39" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C39">
+        <v>0</v>
+      </c>
+      <c r="D39">
+        <v>187020.456722612</v>
+      </c>
+      <c r="E39">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F39">
+        <v>1.09353178385</v>
+      </c>
+      <c r="G39">
+        <v>89520.694507565597</v>
+      </c>
+      <c r="H39">
+        <v>6971.3813103080802</v>
+      </c>
+      <c r="I39">
+        <v>5083.8680235841202</v>
+      </c>
+      <c r="J39">
+        <v>101575.943841457</v>
+      </c>
+      <c r="K39">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L39">
+        <v>15303.798385783</v>
+      </c>
+      <c r="M39">
+        <v>19297.5304894482</v>
+      </c>
+      <c r="N39">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O39">
+        <v>0</v>
+      </c>
+      <c r="P39">
+        <v>308572.439249494</v>
+      </c>
+      <c r="Q39">
+        <v>1106.4527933521999</v>
+      </c>
+      <c r="R39">
+        <v>3451.9307168288801</v>
+      </c>
+      <c r="S39">
+        <v>20.547206647791</v>
+      </c>
+      <c r="T39">
+        <v>-14.696886263168601</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A40" s="3"/>
+      <c r="G40" s="4"/>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>20</v>
-      </c>
-      <c r="B40" t="s">
-        <v>21</v>
-      </c>
-      <c r="C40">
-        <v>4</v>
-      </c>
-      <c r="D40">
-        <v>116833.749486644</v>
-      </c>
-      <c r="E40">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F40">
-        <v>0.84480122530439805</v>
-      </c>
-      <c r="G40" s="4">
-        <v>23535.478746437901</v>
-      </c>
-      <c r="H40">
-        <v>6941.2778055266899</v>
-      </c>
-      <c r="I40">
-        <v>912.48005352310201</v>
-      </c>
-      <c r="J40">
-        <v>31389.236605487698</v>
-      </c>
-      <c r="K40">
-        <v>50843.184005923998</v>
-      </c>
-      <c r="L40">
-        <v>15303.798385784499</v>
-      </c>
-      <c r="M40">
-        <v>19297.5304894484</v>
-      </c>
-      <c r="N40">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O40">
-        <v>0</v>
-      </c>
-      <c r="P40">
-        <v>0</v>
-      </c>
-      <c r="Q40">
-        <v>0</v>
-      </c>
-      <c r="R40">
-        <v>0</v>
-      </c>
-      <c r="S40">
-        <v>0</v>
-      </c>
-      <c r="T40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A41" t="s">
-        <v>22</v>
       </c>
       <c r="B41" t="s">
         <v>21</v>
       </c>
       <c r="C41">
+        <v>0</v>
+      </c>
+      <c r="D41">
+        <v>117032.41959359701</v>
+      </c>
+      <c r="E41">
+        <v>282179.67123286898</v>
+      </c>
+      <c r="F41">
+        <v>0.845505280653571</v>
+      </c>
+      <c r="G41" s="4">
+        <v>23683.129427060001</v>
+      </c>
+      <c r="H41">
+        <v>6986.3695969997798</v>
+      </c>
+      <c r="I41">
+        <v>918.40768838365295</v>
+      </c>
+      <c r="J41">
+        <v>31587.906712443499</v>
+      </c>
+      <c r="K41">
+        <v>50843.1840059237</v>
+      </c>
+      <c r="L41">
+        <v>15303.7983857823</v>
+      </c>
+      <c r="M41">
+        <v>19297.530489448101</v>
+      </c>
+      <c r="N41">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O41">
+        <v>0</v>
+      </c>
+      <c r="P41">
+        <v>238584.402120479</v>
+      </c>
+      <c r="Q41">
+        <v>1108.83163779344</v>
+      </c>
+      <c r="R41">
+        <v>0</v>
+      </c>
+      <c r="S41">
+        <v>230512.59606633501</v>
+      </c>
+      <c r="T41">
+        <v>1103.3673370121001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>22</v>
+      </c>
+      <c r="B42" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>171564.02128394699</v>
+      </c>
+      <c r="E42">
+        <v>282179.67123287701</v>
+      </c>
+      <c r="F42">
+        <v>1.03875662810921</v>
+      </c>
+      <c r="G42">
+        <v>73514.1870928641</v>
+      </c>
+      <c r="H42">
+        <v>7482.8438362204697</v>
+      </c>
+      <c r="I42">
+        <v>4044.9309872213798</v>
+      </c>
+      <c r="J42">
+        <v>85041.961916305998</v>
+      </c>
+      <c r="K42">
+        <v>51119.832654572398</v>
+      </c>
+      <c r="L42">
+        <v>16047.2916290263</v>
+      </c>
+      <c r="M42">
+        <v>19354.9350840429</v>
+      </c>
+      <c r="N42">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O42">
+        <v>0</v>
+      </c>
+      <c r="P42">
+        <v>293116.00381082902</v>
+      </c>
+      <c r="Q42">
+        <v>1187.62883512946</v>
+      </c>
+      <c r="R42">
+        <v>9393.8913494494009</v>
+      </c>
+      <c r="S42">
+        <v>260.94142637359403</v>
+      </c>
+      <c r="T42">
+        <v>-3.6405201993767098</v>
+      </c>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="G43" s="4"/>
+    </row>
+    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A44" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B44" t="s">
+        <v>21</v>
+      </c>
+      <c r="C44">
         <v>4</v>
       </c>
-      <c r="D41">
-        <v>124393.533174422</v>
-      </c>
-      <c r="E41">
-        <v>282179.67123444699</v>
-      </c>
-      <c r="F41">
-        <v>0.87159189967643702</v>
-      </c>
-      <c r="G41" s="4">
-        <v>21072.189860718699</v>
-      </c>
-      <c r="H41">
-        <v>9188.7245080883695</v>
-      </c>
-      <c r="I41">
-        <v>2618.8827210474601</v>
-      </c>
-      <c r="J41">
-        <v>32879.797089854597</v>
-      </c>
-      <c r="K41">
-        <v>50904.118537438801</v>
-      </c>
-      <c r="L41">
-        <v>20591.7266090095</v>
-      </c>
-      <c r="M41">
-        <v>20017.890938119701</v>
-      </c>
-      <c r="N41">
-        <v>1040.9289460857101</v>
-      </c>
-      <c r="O41">
-        <v>0</v>
-      </c>
-      <c r="P41">
-        <v>245945.51570130399</v>
-      </c>
-      <c r="Q41">
-        <v>1458.3752411216699</v>
-      </c>
-      <c r="R41">
-        <v>35012.612233571497</v>
-      </c>
-      <c r="S41">
-        <v>875.31530583928895</v>
-      </c>
-      <c r="T41">
-        <v>0.51444695802960605</v>
-      </c>
-    </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A43" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G43" s="4"/>
-    </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A44" t="s">
-        <v>22</v>
-      </c>
-      <c r="B44" t="s">
-        <v>25</v>
-      </c>
-      <c r="C44">
-        <v>2</v>
-      </c>
       <c r="D44">
-        <v>115472.147206908</v>
+        <v>116833.749486644</v>
       </c>
       <c r="E44">
-        <v>282495</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F44">
-        <v>0.83903831831993503</v>
+        <v>0.84480122530439805</v>
       </c>
       <c r="G44" s="4">
-        <v>20221.889710343999</v>
+        <v>23535.478746437901</v>
       </c>
       <c r="H44">
-        <v>6553.7440767980397</v>
+        <v>6941.2778055266899</v>
       </c>
       <c r="I44">
-        <v>6160.4249909476703</v>
+        <v>912.48005352310201</v>
       </c>
       <c r="J44">
-        <v>32936.058778089697</v>
+        <v>31389.236605487698</v>
       </c>
       <c r="K44">
-        <v>50939.5611113743</v>
+        <v>50843.184005923998</v>
       </c>
       <c r="L44">
-        <v>15427.2204868183</v>
+        <v>15303.798385784499</v>
       </c>
       <c r="M44">
-        <v>19327.3039306102</v>
+        <v>19297.5304894484</v>
       </c>
       <c r="N44">
-        <v>1004.9477757237401</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O44">
-        <v>3157.9970999842499</v>
+        <v>0</v>
       </c>
       <c r="P44">
-        <v>237024.12973379</v>
+        <v>0</v>
       </c>
       <c r="Q44">
-        <v>1464.2687322859999</v>
+        <v>0</v>
       </c>
       <c r="R44">
-        <v>8672.9882445954008</v>
+        <v>0</v>
       </c>
       <c r="S44">
-        <v>346.91952978381602</v>
+        <v>0</v>
       </c>
       <c r="T44">
-        <v>2.4302910949698302</v>
-      </c>
-    </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>22</v>
       </c>
       <c r="B45" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C45">
         <v>4</v>
       </c>
       <c r="D45">
+        <v>124393.533174422</v>
+      </c>
+      <c r="E45">
+        <v>282179.67123444699</v>
+      </c>
+      <c r="F45">
+        <v>0.87159189967643702</v>
+      </c>
+      <c r="G45" s="4">
+        <v>21072.189860718699</v>
+      </c>
+      <c r="H45">
+        <v>9188.7245080883695</v>
+      </c>
+      <c r="I45">
+        <v>2618.8827210474601</v>
+      </c>
+      <c r="J45">
+        <v>32879.797089854597</v>
+      </c>
+      <c r="K45">
+        <v>50904.118537438801</v>
+      </c>
+      <c r="L45">
+        <v>20591.7266090095</v>
+      </c>
+      <c r="M45">
+        <v>20017.890938119701</v>
+      </c>
+      <c r="N45">
+        <v>1040.9289460857101</v>
+      </c>
+      <c r="O45">
+        <v>0</v>
+      </c>
+      <c r="P45">
+        <v>245945.51570130399</v>
+      </c>
+      <c r="Q45">
+        <v>1458.3752411216699</v>
+      </c>
+      <c r="R45">
+        <v>35012.612233571497</v>
+      </c>
+      <c r="S45">
+        <v>875.31530583928895</v>
+      </c>
+      <c r="T45">
+        <v>0.51444695802960605</v>
+      </c>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A47" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G47" s="4"/>
+    </row>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>22</v>
+      </c>
+      <c r="B48" t="s">
+        <v>25</v>
+      </c>
+      <c r="C48">
+        <v>2</v>
+      </c>
+      <c r="D48">
+        <v>115472.147206908</v>
+      </c>
+      <c r="E48">
+        <v>282495</v>
+      </c>
+      <c r="F48">
+        <v>0.83903831831993503</v>
+      </c>
+      <c r="G48" s="4">
+        <v>20221.889710343999</v>
+      </c>
+      <c r="H48">
+        <v>6553.7440767980397</v>
+      </c>
+      <c r="I48">
+        <v>6160.4249909476703</v>
+      </c>
+      <c r="J48">
+        <v>32936.058778089697</v>
+      </c>
+      <c r="K48">
+        <v>50939.5611113743</v>
+      </c>
+      <c r="L48">
+        <v>15427.2204868183</v>
+      </c>
+      <c r="M48">
+        <v>19327.3039306102</v>
+      </c>
+      <c r="N48">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O48">
+        <v>3157.9970999842499</v>
+      </c>
+      <c r="P48">
+        <v>237024.12973379</v>
+      </c>
+      <c r="Q48">
+        <v>1464.2687322859999</v>
+      </c>
+      <c r="R48">
+        <v>8672.9882445954008</v>
+      </c>
+      <c r="S48">
+        <v>346.91952978381602</v>
+      </c>
+      <c r="T48">
+        <v>2.4302910949698302</v>
+      </c>
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>22</v>
+      </c>
+      <c r="B49" t="s">
+        <v>25</v>
+      </c>
+      <c r="C49">
+        <v>4</v>
+      </c>
+      <c r="D49">
         <v>108958.027502652</v>
       </c>
-      <c r="E45">
+      <c r="E49">
         <v>282179.67123287602</v>
       </c>
-      <c r="F45">
+      <c r="F49">
         <v>0.81689091571482797</v>
       </c>
-      <c r="G45" s="4">
+      <c r="G49" s="4">
         <v>20285.098342207999</v>
       </c>
-      <c r="H45">
+      <c r="H49">
         <v>6552.6722224723899</v>
       </c>
-      <c r="I45">
+      <c r="I49">
         <v>6068.9240568166097</v>
       </c>
-      <c r="J45">
+      <c r="J49">
         <v>32906.694621497001</v>
       </c>
-      <c r="K45">
+      <c r="K49">
         <v>50843.184005923598</v>
       </c>
-      <c r="L45">
+      <c r="L49">
         <v>16378.7983857829</v>
       </c>
-      <c r="M45">
+      <c r="M49">
         <v>19449.350489448301</v>
       </c>
-      <c r="N45">
+      <c r="N49">
         <v>1004.9477757237401</v>
       </c>
-      <c r="O45">
+      <c r="O49">
         <v>10620</v>
       </c>
-      <c r="P45">
+      <c r="P49">
         <v>230510.010029533</v>
       </c>
-      <c r="Q45">
+      <c r="Q49">
         <v>1464.02925348484</v>
       </c>
-      <c r="R45">
+      <c r="R49">
         <v>26064.489084194902</v>
       </c>
-      <c r="S45">
+      <c r="S49">
         <v>407.257641940545</v>
       </c>
-      <c r="T45">
+      <c r="T49">
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A47" s="1" t="s">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A51" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A48" s="3" t="s">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A52" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="B52" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C48">
-        <v>0</v>
-      </c>
-      <c r="D48">
+      <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52">
         <v>115030.978322179</v>
-      </c>
-      <c r="E48">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F48">
-        <v>0.83841249022441</v>
-      </c>
-      <c r="G48">
-        <v>20114.092712805999</v>
-      </c>
-      <c r="H48">
-        <v>6942.2846600808298</v>
-      </c>
-      <c r="I48">
-        <v>2530.0880681377598</v>
-      </c>
-      <c r="J48">
-        <v>29586.4654410246</v>
-      </c>
-      <c r="K48">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L48">
-        <v>15303.798385783</v>
-      </c>
-      <c r="M48">
-        <v>19297.5304894482</v>
-      </c>
-      <c r="N48">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O48">
-        <v>0</v>
-      </c>
-      <c r="P48">
-        <v>236582.960849061</v>
-      </c>
-      <c r="Q48">
-        <v>1101.8347602124099</v>
-      </c>
-      <c r="R48">
-        <v>0</v>
-      </c>
-      <c r="S48">
-        <v>0</v>
-      </c>
-      <c r="T48">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A49" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C49">
-        <v>0</v>
-      </c>
-      <c r="D49">
-        <v>124771.246709449</v>
-      </c>
-      <c r="E49">
-        <v>282179.67125180899</v>
-      </c>
-      <c r="F49">
-        <v>0.87293045648394496</v>
-      </c>
-      <c r="G49">
-        <v>22626.697961956499</v>
-      </c>
-      <c r="H49">
-        <v>7102.5767129513297</v>
-      </c>
-      <c r="I49">
-        <v>9597.4591384874802</v>
-      </c>
-      <c r="J49">
-        <v>39326.733813395302</v>
-      </c>
-      <c r="K49">
-        <v>50843.184011688398</v>
-      </c>
-      <c r="L49">
-        <v>15303.798393134501</v>
-      </c>
-      <c r="M49">
-        <v>19297.530491231599</v>
-      </c>
-      <c r="N49">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O49">
-        <v>0</v>
-      </c>
-      <c r="P49">
-        <v>246323.22923633101</v>
-      </c>
-      <c r="Q49">
-        <v>1127.27501714903</v>
-      </c>
-      <c r="R49">
-        <v>0</v>
-      </c>
-      <c r="S49">
-        <v>0</v>
-      </c>
-      <c r="T49">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A50" s="1"/>
-    </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A51" t="s">
-        <v>20</v>
-      </c>
-      <c r="B51" t="s">
-        <v>21</v>
-      </c>
-      <c r="C51">
-        <v>2</v>
-      </c>
-      <c r="D51">
-        <v>115714.10508262301</v>
-      </c>
-      <c r="E51">
-        <v>282179.67125387199</v>
-      </c>
-      <c r="F51">
-        <v>0.840833383054163</v>
-      </c>
-      <c r="G51" s="4">
-        <v>20578.507216446698</v>
-      </c>
-      <c r="H51">
-        <v>7102.57515066207</v>
-      </c>
-      <c r="I51">
-        <v>2588.5052959285099</v>
-      </c>
-      <c r="J51">
-        <v>30269.587663037299</v>
-      </c>
-      <c r="K51">
-        <v>50843.185173268597</v>
-      </c>
-      <c r="L51">
-        <v>15303.8015139941</v>
-      </c>
-      <c r="M51">
-        <v>19297.530732323401</v>
-      </c>
-      <c r="N51">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O51">
-        <v>0</v>
-      </c>
-      <c r="P51">
-        <v>237266.08760950499</v>
-      </c>
-      <c r="Q51">
-        <v>1127.2750356983099</v>
-      </c>
-      <c r="R51">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A52" t="s">
-        <v>22</v>
-      </c>
-      <c r="B52" t="s">
-        <v>21</v>
-      </c>
-      <c r="C52">
-        <v>2</v>
-      </c>
-      <c r="D52">
-        <v>120628.41082793</v>
       </c>
       <c r="E52">
         <v>282179.67123287602</v>
       </c>
       <c r="F52">
-        <v>0.85824890324911396</v>
-      </c>
-      <c r="G52" s="4">
-        <v>20824.7129679639</v>
+        <v>0.83841249022441</v>
+      </c>
+      <c r="G52">
+        <v>20114.092712805999</v>
       </c>
       <c r="H52">
-        <v>7456.39074483072</v>
+        <v>6942.2846600808298</v>
       </c>
       <c r="I52">
-        <v>5114.4587365303096</v>
+        <v>2530.0880681377598</v>
       </c>
       <c r="J52">
-        <v>33395.562449324898</v>
+        <v>29586.4654410246</v>
       </c>
       <c r="K52">
-        <v>51302.320205525801</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L52">
-        <v>16537.7269222135</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M52">
-        <v>19392.801250865799</v>
+        <v>19297.5304894482</v>
       </c>
       <c r="N52">
-        <v>1004.9477757237401</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O52">
         <v>0</v>
       </c>
       <c r="P52">
-        <v>242180.39335481101</v>
+        <v>236582.960849061</v>
       </c>
       <c r="Q52">
-        <v>1183.4303612998101</v>
+        <v>1101.8347602124099</v>
       </c>
       <c r="R52">
-        <v>15931.1957490451</v>
+        <v>0</v>
       </c>
       <c r="S52">
-        <v>346.33034237054602</v>
+        <v>0</v>
       </c>
       <c r="T52">
-        <v>1.0959871186973</v>
-      </c>
-    </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A54" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A53" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C53">
+        <v>0</v>
+      </c>
+      <c r="D53">
+        <v>124771.246709449</v>
+      </c>
+      <c r="E53">
+        <v>282179.67125180899</v>
+      </c>
+      <c r="F53">
+        <v>0.87293045648394496</v>
+      </c>
+      <c r="G53">
+        <v>22626.697961956499</v>
+      </c>
+      <c r="H53">
+        <v>7102.5767129513297</v>
+      </c>
+      <c r="I53">
+        <v>9597.4591384874802</v>
+      </c>
+      <c r="J53">
+        <v>39326.733813395302</v>
+      </c>
+      <c r="K53">
+        <v>50843.184011688398</v>
+      </c>
+      <c r="L53">
+        <v>15303.798393134501</v>
+      </c>
+      <c r="M53">
+        <v>19297.530491231599</v>
+      </c>
+      <c r="N53">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O53">
+        <v>0</v>
+      </c>
+      <c r="P53">
+        <v>246323.22923633101</v>
+      </c>
+      <c r="Q53">
+        <v>1127.27501714903</v>
+      </c>
+      <c r="R53">
+        <v>0</v>
+      </c>
+      <c r="S53">
+        <v>0</v>
+      </c>
+      <c r="T53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A54" s="1"/>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>20</v>
-      </c>
-      <c r="B54" t="s">
-        <v>21</v>
-      </c>
-      <c r="C54">
-        <v>4</v>
-      </c>
-      <c r="D54">
-        <v>115714.10508261999</v>
-      </c>
-      <c r="E54">
-        <v>282179.671253876</v>
-      </c>
-      <c r="F54">
-        <v>0.84083338305413902</v>
-      </c>
-      <c r="G54" s="4">
-        <v>20578.5072164468</v>
-      </c>
-      <c r="H54">
-        <v>7102.5751506616798</v>
-      </c>
-      <c r="I54">
-        <v>2588.50529592865</v>
-      </c>
-      <c r="J54">
-        <v>30269.587663037099</v>
-      </c>
-      <c r="K54">
-        <v>50843.185173268197</v>
-      </c>
-      <c r="L54">
-        <v>15303.8015139912</v>
-      </c>
-      <c r="M54">
-        <v>19297.530732323299</v>
-      </c>
-      <c r="N54">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O54">
-        <v>0</v>
-      </c>
-      <c r="P54">
-        <v>237266.087609501</v>
-      </c>
-      <c r="Q54">
-        <v>1127.2750356983499</v>
-      </c>
-      <c r="R54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A55" t="s">
-        <v>22</v>
       </c>
       <c r="B55" t="s">
         <v>21</v>
       </c>
       <c r="C55">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D55">
-        <v>120375.156660901</v>
+        <v>115714.10508262301</v>
       </c>
       <c r="E55">
-        <v>282179.671232878</v>
+        <v>282179.67125387199</v>
       </c>
       <c r="F55">
-        <v>0.857351410648304</v>
+        <v>0.840833383054163</v>
       </c>
       <c r="G55" s="4">
-        <v>21285.1004075495</v>
+        <v>20578.507216446698</v>
       </c>
       <c r="H55">
-        <v>7426.32532798384</v>
+        <v>7102.57515066207</v>
       </c>
       <c r="I55">
-        <v>5046.79446201879</v>
+        <v>2588.5052959285099</v>
       </c>
       <c r="J55">
-        <v>33758.220197552102</v>
+        <v>30269.587663037299</v>
       </c>
       <c r="K55">
-        <v>51144.191344099498</v>
+        <v>50843.185173268597</v>
       </c>
       <c r="L55">
-        <v>16112.7556071296</v>
+        <v>15303.8015139941</v>
       </c>
       <c r="M55">
-        <v>19359.989512119799</v>
+        <v>19297.530732323401</v>
       </c>
       <c r="N55">
-        <v>1006.77939378399</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O55">
         <v>0</v>
       </c>
       <c r="P55">
-        <v>241927.13918778201</v>
+        <v>237266.08760950499</v>
       </c>
       <c r="Q55">
-        <v>1178.65858109644</v>
+        <v>1127.2750356983099</v>
       </c>
       <c r="R55">
-        <v>12586.325853030899</v>
-      </c>
-      <c r="S55">
-        <v>466.16021677892502</v>
-      </c>
-      <c r="T55">
-        <v>1.3585822738026401</v>
-      </c>
-    </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="G56" s="4"/>
-    </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A57" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G57" s="4"/>
-    </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>22</v>
+      </c>
+      <c r="B56" t="s">
+        <v>21</v>
+      </c>
+      <c r="C56">
+        <v>2</v>
+      </c>
+      <c r="D56">
+        <v>120628.41082793</v>
+      </c>
+      <c r="E56">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F56">
+        <v>0.85824890324911396</v>
+      </c>
+      <c r="G56" s="4">
+        <v>20824.7129679639</v>
+      </c>
+      <c r="H56">
+        <v>7456.39074483072</v>
+      </c>
+      <c r="I56">
+        <v>5114.4587365303096</v>
+      </c>
+      <c r="J56">
+        <v>33395.562449324898</v>
+      </c>
+      <c r="K56">
+        <v>51302.320205525801</v>
+      </c>
+      <c r="L56">
+        <v>16537.7269222135</v>
+      </c>
+      <c r="M56">
+        <v>19392.801250865799</v>
+      </c>
+      <c r="N56">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O56">
+        <v>0</v>
+      </c>
+      <c r="P56">
+        <v>242180.39335481101</v>
+      </c>
+      <c r="Q56">
+        <v>1183.4303612998101</v>
+      </c>
+      <c r="R56">
+        <v>15931.1957490451</v>
+      </c>
+      <c r="S56">
+        <v>346.33034237054602</v>
+      </c>
+      <c r="T56">
+        <v>1.0959871186973</v>
+      </c>
+    </row>
+    <row r="58" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B58" t="s">
         <v>21</v>
@@ -3430,611 +3361,490 @@
         <v>4</v>
       </c>
       <c r="D58">
-        <v>146108.01933512901</v>
+        <v>115714.10508261999</v>
       </c>
       <c r="E58">
-        <v>355610.364944759</v>
+        <v>282179.671253876</v>
       </c>
       <c r="F58">
-        <v>0.75267772890587503</v>
-      </c>
-      <c r="G58">
-        <v>25765.651662743599</v>
+        <v>0.84083338305413902</v>
+      </c>
+      <c r="G58" s="4">
+        <v>20578.5072164468</v>
       </c>
       <c r="H58">
-        <v>7150.9042815892099</v>
+        <v>7102.5751506616798</v>
       </c>
       <c r="I58">
-        <v>5144.3184852884797</v>
+        <v>2588.50529592865</v>
       </c>
       <c r="J58">
-        <v>38060.874429621297</v>
+        <v>30269.587663037099</v>
       </c>
       <c r="K58">
-        <v>64168.339029134899</v>
+        <v>50843.185173268197</v>
       </c>
       <c r="L58">
-        <v>19539.954214541001</v>
+        <v>15303.8015139912</v>
       </c>
       <c r="M58">
-        <v>24338.851661831999</v>
+        <v>19297.530732323299</v>
       </c>
       <c r="N58">
-        <v>1010.46273302954</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O58">
         <v>0</v>
       </c>
       <c r="P58">
-        <v>267660.00186201098</v>
+        <v>237266.087609501</v>
       </c>
       <c r="Q58">
-        <v>1597.68911089628</v>
+        <v>1127.2750356983499</v>
       </c>
       <c r="R58">
-        <v>13084.0423994256</v>
-      </c>
-      <c r="S58">
-        <v>467.28722855091399</v>
-      </c>
-      <c r="T58">
-        <v>-0.25904927491985202</v>
-      </c>
-    </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>22</v>
       </c>
       <c r="B59" t="s">
+        <v>21</v>
+      </c>
+      <c r="C59">
+        <v>4</v>
+      </c>
+      <c r="D59">
+        <v>120375.156660901</v>
+      </c>
+      <c r="E59">
+        <v>282179.671232878</v>
+      </c>
+      <c r="F59">
+        <v>0.857351410648304</v>
+      </c>
+      <c r="G59" s="4">
+        <v>21285.1004075495</v>
+      </c>
+      <c r="H59">
+        <v>7426.32532798384</v>
+      </c>
+      <c r="I59">
+        <v>5046.79446201879</v>
+      </c>
+      <c r="J59">
+        <v>33758.220197552102</v>
+      </c>
+      <c r="K59">
+        <v>51144.191344099498</v>
+      </c>
+      <c r="L59">
+        <v>16112.7556071296</v>
+      </c>
+      <c r="M59">
+        <v>19359.989512119799</v>
+      </c>
+      <c r="N59">
+        <v>1006.77939378399</v>
+      </c>
+      <c r="O59">
+        <v>0</v>
+      </c>
+      <c r="P59">
+        <v>241927.13918778201</v>
+      </c>
+      <c r="Q59">
+        <v>1178.65858109644</v>
+      </c>
+      <c r="R59">
+        <v>12586.325853030899</v>
+      </c>
+      <c r="S59">
+        <v>466.16021677892502</v>
+      </c>
+      <c r="T59">
+        <v>1.3585822738026401</v>
+      </c>
+    </row>
+    <row r="60" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="G60" s="4"/>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A61" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G61" s="4"/>
+    </row>
+    <row r="62" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>22</v>
+      </c>
+      <c r="B62" t="s">
+        <v>21</v>
+      </c>
+      <c r="C62">
+        <v>4</v>
+      </c>
+      <c r="D62">
+        <v>146108.01933512901</v>
+      </c>
+      <c r="E62">
+        <v>355610.364944759</v>
+      </c>
+      <c r="F62">
+        <v>0.75267772890587503</v>
+      </c>
+      <c r="G62">
+        <v>25765.651662743599</v>
+      </c>
+      <c r="H62">
+        <v>7150.9042815892099</v>
+      </c>
+      <c r="I62">
+        <v>5144.3184852884797</v>
+      </c>
+      <c r="J62">
+        <v>38060.874429621297</v>
+      </c>
+      <c r="K62">
+        <v>64168.339029134899</v>
+      </c>
+      <c r="L62">
+        <v>19539.954214541001</v>
+      </c>
+      <c r="M62">
+        <v>24338.851661831999</v>
+      </c>
+      <c r="N62">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O62">
+        <v>0</v>
+      </c>
+      <c r="P62">
+        <v>267660.00186201098</v>
+      </c>
+      <c r="Q62">
+        <v>1597.68911089628</v>
+      </c>
+      <c r="R62">
+        <v>13084.0423994256</v>
+      </c>
+      <c r="S62">
+        <v>467.28722855091399</v>
+      </c>
+      <c r="T62">
+        <v>-0.25904927491985202</v>
+      </c>
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>22</v>
+      </c>
+      <c r="B63" t="s">
         <v>35</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C63" t="s">
         <v>35</v>
       </c>
-      <c r="D59" t="s">
+      <c r="D63" t="s">
         <v>36</v>
       </c>
-      <c r="E59" t="s">
+      <c r="E63" t="s">
         <v>36</v>
       </c>
-      <c r="F59" t="s">
+      <c r="F63" t="s">
         <v>36</v>
       </c>
-      <c r="G59" s="4">
+      <c r="G63" s="4">
         <v>28838</v>
       </c>
-      <c r="H59">
+      <c r="H63">
         <v>7567.5</v>
       </c>
-      <c r="I59">
+      <c r="I63">
         <v>13764.1</v>
       </c>
-      <c r="J59">
+      <c r="J63">
         <v>50169.7</v>
       </c>
-      <c r="K59" t="s">
+      <c r="K63" t="s">
         <v>36</v>
       </c>
-      <c r="L59" t="s">
+      <c r="L63" t="s">
         <v>36</v>
       </c>
-      <c r="M59" t="s">
+      <c r="M63" t="s">
         <v>36</v>
       </c>
-      <c r="N59" t="s">
+      <c r="N63" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="61" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A61" s="1" t="s">
+    <row r="65" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A65" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G61" s="4"/>
-      <c r="P61" t="s">
+      <c r="G65" s="4"/>
+      <c r="P65" t="s">
         <v>15</v>
       </c>
-      <c r="Q61" t="s">
+      <c r="Q65" t="s">
         <v>16</v>
       </c>
-      <c r="R61" t="s">
+      <c r="R65" t="s">
         <v>17</v>
       </c>
-      <c r="S61" t="s">
+      <c r="S65" t="s">
         <v>18</v>
       </c>
-      <c r="T61" t="s">
+      <c r="T65" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B62" t="s">
+    <row r="66" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" t="s">
         <v>1</v>
-      </c>
-      <c r="C62" t="s">
-        <v>2</v>
-      </c>
-      <c r="D62" t="s">
-        <v>3</v>
-      </c>
-      <c r="E62" t="s">
-        <v>4</v>
-      </c>
-      <c r="F62" t="s">
-        <v>5</v>
-      </c>
-      <c r="G62" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H62" t="s">
-        <v>7</v>
-      </c>
-      <c r="I62" t="s">
-        <v>8</v>
-      </c>
-      <c r="J62" t="s">
-        <v>9</v>
-      </c>
-      <c r="K62" t="s">
-        <v>10</v>
-      </c>
-      <c r="L62" t="s">
-        <v>11</v>
-      </c>
-      <c r="M62" t="s">
-        <v>12</v>
-      </c>
-      <c r="N62" t="s">
-        <v>13</v>
-      </c>
-      <c r="O62" t="s">
-        <v>14</v>
-      </c>
-      <c r="P62">
-        <v>63734.6679</v>
-      </c>
-      <c r="Q62">
-        <v>1078.4492829999999</v>
-      </c>
-      <c r="R62">
-        <v>624.70352849999995</v>
-      </c>
-      <c r="S62">
-        <v>13.014656840000001</v>
-      </c>
-      <c r="T62">
-        <v>27.514184579999998</v>
-      </c>
-    </row>
-    <row r="63" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A63" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B63" t="s">
-        <v>21</v>
-      </c>
-      <c r="C63">
-        <v>4</v>
-      </c>
-      <c r="D63">
-        <v>29525.427309999999</v>
-      </c>
-      <c r="E63">
-        <v>80391.755990000005</v>
-      </c>
-      <c r="F63">
-        <v>0.79280104200000001</v>
-      </c>
-      <c r="G63" s="4">
-        <v>5050.6365619999997</v>
-      </c>
-      <c r="H63">
-        <v>4678.3390820000004</v>
-      </c>
-      <c r="I63">
-        <v>2508.6600360000002</v>
-      </c>
-      <c r="J63">
-        <v>12237.635679999999</v>
-      </c>
-      <c r="K63">
-        <v>13920</v>
-      </c>
-      <c r="L63">
-        <v>2841.544922</v>
-      </c>
-      <c r="M63">
-        <v>5380.5444360000001</v>
-      </c>
-      <c r="N63">
-        <v>279.27307350000001</v>
-      </c>
-      <c r="O63">
-        <v>0</v>
-      </c>
-      <c r="P63">
-        <v>64865.028310000002</v>
-      </c>
-      <c r="Q63">
-        <v>1191.7509680000001</v>
-      </c>
-      <c r="R63">
-        <v>7243.7162129999997</v>
-      </c>
-      <c r="S63">
-        <v>452.7322633</v>
-      </c>
-      <c r="T63">
-        <v>5.8154128590000003</v>
-      </c>
-    </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A64" s="7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A66" t="s">
-        <v>32</v>
-      </c>
-      <c r="B66" t="s">
-        <v>33</v>
       </c>
       <c r="C66" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A67">
+      <c r="D66" t="s">
+        <v>3</v>
+      </c>
+      <c r="E66" t="s">
+        <v>4</v>
+      </c>
+      <c r="F66" t="s">
+        <v>5</v>
+      </c>
+      <c r="G66" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H66" t="s">
+        <v>7</v>
+      </c>
+      <c r="I66" t="s">
+        <v>8</v>
+      </c>
+      <c r="J66" t="s">
+        <v>9</v>
+      </c>
+      <c r="K66" t="s">
+        <v>10</v>
+      </c>
+      <c r="L66" t="s">
+        <v>11</v>
+      </c>
+      <c r="M66" t="s">
+        <v>12</v>
+      </c>
+      <c r="N66" t="s">
+        <v>13</v>
+      </c>
+      <c r="O66" t="s">
+        <v>14</v>
+      </c>
+      <c r="P66">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q66">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R66">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S66">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T66">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="67" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A67" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B67">
+      <c r="B67" t="s">
+        <v>21</v>
+      </c>
+      <c r="C67">
+        <v>4</v>
+      </c>
+      <c r="D67">
+        <v>29525.427309999999</v>
+      </c>
+      <c r="E67">
+        <v>80391.755990000005</v>
+      </c>
+      <c r="F67">
+        <v>0.79280104200000001</v>
+      </c>
+      <c r="G67" s="4">
+        <v>5050.6365619999997</v>
+      </c>
+      <c r="H67">
+        <v>4678.3390820000004</v>
+      </c>
+      <c r="I67">
+        <v>2508.6600360000002</v>
+      </c>
+      <c r="J67">
+        <v>12237.635679999999</v>
+      </c>
+      <c r="K67">
+        <v>13920</v>
+      </c>
+      <c r="L67">
+        <v>2841.544922</v>
+      </c>
+      <c r="M67">
+        <v>5380.5444360000001</v>
+      </c>
+      <c r="N67">
+        <v>279.27307350000001</v>
+      </c>
+      <c r="O67">
+        <v>0</v>
+      </c>
+      <c r="P67">
+        <v>64865.028310000002</v>
+      </c>
+      <c r="Q67">
+        <v>1191.7509680000001</v>
+      </c>
+      <c r="R67">
+        <v>7243.7162129999997</v>
+      </c>
+      <c r="S67">
+        <v>452.7322633</v>
+      </c>
+      <c r="T67">
+        <v>5.8154128590000003</v>
+      </c>
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A68" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>32</v>
+      </c>
+      <c r="B70" t="s">
+        <v>33</v>
+      </c>
+      <c r="C70" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A71">
+        <v>20</v>
+      </c>
+      <c r="B71">
         <v>60</v>
       </c>
-      <c r="C67">
+      <c r="C71">
         <v>2</v>
       </c>
-      <c r="D67">
+      <c r="D71">
         <v>119696.652328767</v>
       </c>
-      <c r="E67">
+      <c r="E71">
         <v>282179.67123285501</v>
       </c>
-      <c r="F67">
+      <c r="F71">
         <v>0.854946898908852</v>
       </c>
-      <c r="G67">
+      <c r="G71">
         <v>18681.222424938602</v>
       </c>
-      <c r="H67">
+      <c r="H71">
         <v>5354.6114985546601</v>
       </c>
-      <c r="I67">
+      <c r="I71">
         <v>8156.08309050551</v>
       </c>
-      <c r="J67">
+      <c r="J71">
         <v>32191.917013998798</v>
       </c>
-      <c r="K67">
+      <c r="K71">
         <v>51372.124296964801</v>
       </c>
-      <c r="L67">
+      <c r="L71">
         <v>16725.325417965501</v>
       </c>
-      <c r="M67">
+      <c r="M71">
         <v>19407.285599838699</v>
       </c>
-      <c r="N67">
+      <c r="N71">
         <v>1016.03855436447</v>
       </c>
-      <c r="O67">
-        <v>0</v>
-      </c>
-      <c r="P67">
+      <c r="O71">
+        <v>0</v>
+      </c>
+      <c r="P71">
         <v>241248.634855649</v>
       </c>
-      <c r="Q67">
+      <c r="Q71">
         <v>1192.7637589594799</v>
       </c>
-      <c r="R67">
+      <c r="R71">
         <v>19736.206339365101</v>
       </c>
-      <c r="S67">
+      <c r="S71">
         <v>481.37088632597801</v>
       </c>
-      <c r="T67" s="6">
+      <c r="T71" s="6">
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A68">
-        <v>20</v>
-      </c>
-      <c r="B68">
-        <v>50</v>
-      </c>
-      <c r="C68">
-        <v>2</v>
-      </c>
-      <c r="D68">
-        <v>118381.960809661</v>
-      </c>
-      <c r="E68">
-        <v>282254.81855225202</v>
-      </c>
-      <c r="F68">
-        <v>0.85006146065890897</v>
-      </c>
-      <c r="G68">
-        <v>19407.840072768398</v>
-      </c>
-      <c r="H68">
-        <v>5891.8301217549197</v>
-      </c>
-      <c r="I68">
-        <v>6659.4942697455399</v>
-      </c>
-      <c r="J68">
-        <v>31959.164464268899</v>
-      </c>
-      <c r="K68">
-        <v>51102.045942938203</v>
-      </c>
-      <c r="L68">
-        <v>15967.176494174801</v>
-      </c>
-      <c r="M68">
-        <v>19353.573908279199</v>
-      </c>
-      <c r="N68">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O68">
-        <v>0</v>
-      </c>
-      <c r="P68">
-        <v>239933.943336542</v>
-      </c>
-      <c r="Q68">
-        <v>1312.43161993582</v>
-      </c>
-      <c r="R68">
-        <v>18377.616631847999</v>
-      </c>
-      <c r="S68">
-        <v>459.4404157962</v>
-      </c>
-      <c r="T68" s="6">
-        <v>0.14758705239613301</v>
-      </c>
-    </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A69">
-        <v>20</v>
-      </c>
-      <c r="B69">
-        <v>40</v>
-      </c>
-      <c r="C69">
-        <v>2</v>
-      </c>
-      <c r="D69">
-        <v>116766.56672038</v>
-      </c>
-      <c r="E69">
-        <v>282179.67123287299</v>
-      </c>
-      <c r="F69">
-        <v>0.84456314023622803</v>
-      </c>
-      <c r="G69">
-        <v>19298.245593088301</v>
-      </c>
-      <c r="H69">
-        <v>5682.0016560700296</v>
-      </c>
-      <c r="I69">
-        <v>5350.3346939491703</v>
-      </c>
-      <c r="J69">
-        <v>30330.5819431075</v>
-      </c>
-      <c r="K69">
-        <v>51097.733915068202</v>
-      </c>
-      <c r="L69">
-        <v>15987.901266609</v>
-      </c>
-      <c r="M69">
-        <v>19350.349595595701</v>
-      </c>
-      <c r="N69">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O69">
-        <v>0</v>
-      </c>
-      <c r="P69">
-        <v>238318.54924726201</v>
-      </c>
-      <c r="Q69">
-        <v>1265.6913868611</v>
-      </c>
-      <c r="R69">
-        <v>17746.163883660702</v>
-      </c>
-      <c r="S69">
-        <v>507.03325381887902</v>
-      </c>
-      <c r="T69" s="6">
-        <v>-0.25983751983286502</v>
-      </c>
-    </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A70">
-        <v>20</v>
-      </c>
-      <c r="B70">
-        <v>30</v>
-      </c>
-      <c r="C70">
-        <v>2</v>
-      </c>
-      <c r="D70">
-        <v>115610.996393592</v>
-      </c>
-      <c r="E70">
-        <v>282182.50548365602</v>
-      </c>
-      <c r="F70">
-        <v>0.84045954058697003</v>
-      </c>
-      <c r="G70">
-        <v>19302.752565837702</v>
-      </c>
-      <c r="H70">
-        <v>6226.5181629292701</v>
-      </c>
-      <c r="I70">
-        <v>3974.5318253822402</v>
-      </c>
-      <c r="J70">
-        <v>29503.802554149199</v>
-      </c>
-      <c r="K70">
-        <v>51013.610661725899</v>
-      </c>
-      <c r="L70">
-        <v>15760.601295416</v>
-      </c>
-      <c r="M70">
-        <v>19332.981882301501</v>
-      </c>
-      <c r="N70">
-        <v>1014.17312250211</v>
-      </c>
-      <c r="O70">
-        <v>0</v>
-      </c>
-      <c r="P70">
-        <v>237162.97892047401</v>
-      </c>
-      <c r="Q70">
-        <v>1386.9848841974899</v>
-      </c>
-      <c r="R70">
-        <v>18436.445202769701</v>
-      </c>
-      <c r="S70">
-        <v>209.50505912238299</v>
-      </c>
-      <c r="T70" s="6">
-        <v>0.28049716262959101</v>
-      </c>
-    </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A71" s="3">
-        <v>20</v>
-      </c>
-      <c r="B71" s="3">
-        <v>20</v>
-      </c>
-      <c r="C71" s="3">
-        <v>2</v>
-      </c>
-      <c r="D71">
-        <v>114184.286860504</v>
-      </c>
-      <c r="E71">
-        <v>282179.67123297497</v>
-      </c>
-      <c r="F71">
-        <v>0.83541194997266699</v>
-      </c>
-      <c r="G71">
-        <v>19351.2255529412</v>
-      </c>
-      <c r="H71">
-        <v>6002.0469674603501</v>
-      </c>
-      <c r="I71">
-        <v>2645.4376652921501</v>
-      </c>
-      <c r="J71">
-        <v>27998.710185693701</v>
-      </c>
-      <c r="K71">
-        <v>51033.4442867088</v>
-      </c>
-      <c r="L71">
-        <v>15815.1228903871</v>
-      </c>
-      <c r="M71">
-        <v>19337.009497714302</v>
-      </c>
-      <c r="N71">
-        <v>1014.17312250211</v>
-      </c>
-      <c r="O71">
-        <v>0</v>
-      </c>
-      <c r="P71">
-        <v>235736.26938738499</v>
-      </c>
-      <c r="Q71">
-        <v>1336.98290493166</v>
-      </c>
-      <c r="R71">
-        <v>18577.307877855899</v>
-      </c>
-      <c r="S71">
-        <v>432.030415764091</v>
-      </c>
-      <c r="T71" s="6">
-        <v>-0.122490141098651</v>
-      </c>
-    </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>20</v>
       </c>
       <c r="B72">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C72">
         <v>2</v>
       </c>
       <c r="D72">
-        <v>113440.79599059001</v>
+        <v>118381.960809661</v>
       </c>
       <c r="E72">
-        <v>282179.67123267101</v>
+        <v>282254.81855225202</v>
       </c>
       <c r="F72">
-        <v>0.83277713625127903</v>
+        <v>0.85006146065890897</v>
       </c>
       <c r="G72">
-        <v>19390.977969205</v>
+        <v>19407.840072768398</v>
       </c>
       <c r="H72">
-        <v>5599.5405456203798</v>
+        <v>5891.8301217549197</v>
       </c>
       <c r="I72">
-        <v>2128.1287863747102</v>
+        <v>6659.4942697455399</v>
       </c>
       <c r="J72">
-        <v>27118.647301200101</v>
+        <v>31959.164464268899</v>
       </c>
       <c r="K72">
-        <v>51068.507704320902</v>
+        <v>51102.045942938203</v>
       </c>
       <c r="L72">
-        <v>15909.3558282099</v>
+        <v>15967.176494174801</v>
       </c>
       <c r="M72">
-        <v>19344.285156859401</v>
+        <v>19353.573908279199</v>
       </c>
       <c r="N72">
         <v>1010.46273302954</v>
@@ -4043,80 +3853,328 @@
         <v>0</v>
       </c>
       <c r="P72">
-        <v>234992.778517472</v>
+        <v>239933.943336542</v>
       </c>
       <c r="Q72">
-        <v>1247.3228025527501</v>
+        <v>1312.43161993582</v>
       </c>
       <c r="R72">
-        <v>16417.502561416801</v>
+        <v>18377.616631847999</v>
       </c>
       <c r="S72">
-        <v>469.07150175476602</v>
+        <v>459.4404157962</v>
       </c>
       <c r="T72" s="6">
-        <v>0.46004655114715598</v>
-      </c>
-    </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.4">
+        <v>0.14758705239613301</v>
+      </c>
+    </row>
+    <row r="73" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>20</v>
       </c>
       <c r="B73">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C73">
         <v>2</v>
       </c>
       <c r="D73">
+        <v>116766.56672038</v>
+      </c>
+      <c r="E73">
+        <v>282179.67123287299</v>
+      </c>
+      <c r="F73">
+        <v>0.84456314023622803</v>
+      </c>
+      <c r="G73">
+        <v>19298.245593088301</v>
+      </c>
+      <c r="H73">
+        <v>5682.0016560700296</v>
+      </c>
+      <c r="I73">
+        <v>5350.3346939491703</v>
+      </c>
+      <c r="J73">
+        <v>30330.5819431075</v>
+      </c>
+      <c r="K73">
+        <v>51097.733915068202</v>
+      </c>
+      <c r="L73">
+        <v>15987.901266609</v>
+      </c>
+      <c r="M73">
+        <v>19350.349595595701</v>
+      </c>
+      <c r="N73">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O73">
+        <v>0</v>
+      </c>
+      <c r="P73">
+        <v>238318.54924726201</v>
+      </c>
+      <c r="Q73">
+        <v>1265.6913868611</v>
+      </c>
+      <c r="R73">
+        <v>17746.163883660702</v>
+      </c>
+      <c r="S73">
+        <v>507.03325381887902</v>
+      </c>
+      <c r="T73" s="6">
+        <v>-0.25983751983286502</v>
+      </c>
+    </row>
+    <row r="74" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A74">
+        <v>20</v>
+      </c>
+      <c r="B74">
+        <v>30</v>
+      </c>
+      <c r="C74">
+        <v>2</v>
+      </c>
+      <c r="D74">
+        <v>115610.996393592</v>
+      </c>
+      <c r="E74">
+        <v>282182.50548365602</v>
+      </c>
+      <c r="F74">
+        <v>0.84045954058697003</v>
+      </c>
+      <c r="G74">
+        <v>19302.752565837702</v>
+      </c>
+      <c r="H74">
+        <v>6226.5181629292701</v>
+      </c>
+      <c r="I74">
+        <v>3974.5318253822402</v>
+      </c>
+      <c r="J74">
+        <v>29503.802554149199</v>
+      </c>
+      <c r="K74">
+        <v>51013.610661725899</v>
+      </c>
+      <c r="L74">
+        <v>15760.601295416</v>
+      </c>
+      <c r="M74">
+        <v>19332.981882301501</v>
+      </c>
+      <c r="N74">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O74">
+        <v>0</v>
+      </c>
+      <c r="P74">
+        <v>237162.97892047401</v>
+      </c>
+      <c r="Q74">
+        <v>1386.9848841974899</v>
+      </c>
+      <c r="R74">
+        <v>18436.445202769701</v>
+      </c>
+      <c r="S74">
+        <v>209.50505912238299</v>
+      </c>
+      <c r="T74" s="6">
+        <v>0.28049716262959101</v>
+      </c>
+    </row>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A75" s="3">
+        <v>20</v>
+      </c>
+      <c r="B75" s="3">
+        <v>20</v>
+      </c>
+      <c r="C75" s="3">
+        <v>2</v>
+      </c>
+      <c r="D75">
+        <v>114184.286860504</v>
+      </c>
+      <c r="E75">
+        <v>282179.67123297497</v>
+      </c>
+      <c r="F75">
+        <v>0.83541194997266699</v>
+      </c>
+      <c r="G75">
+        <v>19351.2255529412</v>
+      </c>
+      <c r="H75">
+        <v>6002.0469674603501</v>
+      </c>
+      <c r="I75">
+        <v>2645.4376652921501</v>
+      </c>
+      <c r="J75">
+        <v>27998.710185693701</v>
+      </c>
+      <c r="K75">
+        <v>51033.4442867088</v>
+      </c>
+      <c r="L75">
+        <v>15815.1228903871</v>
+      </c>
+      <c r="M75">
+        <v>19337.009497714302</v>
+      </c>
+      <c r="N75">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O75">
+        <v>0</v>
+      </c>
+      <c r="P75">
+        <v>235736.26938738499</v>
+      </c>
+      <c r="Q75">
+        <v>1336.98290493166</v>
+      </c>
+      <c r="R75">
+        <v>18577.307877855899</v>
+      </c>
+      <c r="S75">
+        <v>432.030415764091</v>
+      </c>
+      <c r="T75" s="6">
+        <v>-0.122490141098651</v>
+      </c>
+    </row>
+    <row r="76" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A76">
+        <v>20</v>
+      </c>
+      <c r="B76">
+        <v>15</v>
+      </c>
+      <c r="C76">
+        <v>2</v>
+      </c>
+      <c r="D76">
+        <v>113440.79599059001</v>
+      </c>
+      <c r="E76">
+        <v>282179.67123267101</v>
+      </c>
+      <c r="F76">
+        <v>0.83277713625127903</v>
+      </c>
+      <c r="G76">
+        <v>19390.977969205</v>
+      </c>
+      <c r="H76">
+        <v>5599.5405456203798</v>
+      </c>
+      <c r="I76">
+        <v>2128.1287863747102</v>
+      </c>
+      <c r="J76">
+        <v>27118.647301200101</v>
+      </c>
+      <c r="K76">
+        <v>51068.507704320902</v>
+      </c>
+      <c r="L76">
+        <v>15909.3558282099</v>
+      </c>
+      <c r="M76">
+        <v>19344.285156859401</v>
+      </c>
+      <c r="N76">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O76">
+        <v>0</v>
+      </c>
+      <c r="P76">
+        <v>234992.778517472</v>
+      </c>
+      <c r="Q76">
+        <v>1247.3228025527501</v>
+      </c>
+      <c r="R76">
+        <v>16417.502561416801</v>
+      </c>
+      <c r="S76">
+        <v>469.07150175476602</v>
+      </c>
+      <c r="T76" s="6">
+        <v>0.46004655114715598</v>
+      </c>
+    </row>
+    <row r="77" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A77">
+        <v>20</v>
+      </c>
+      <c r="B77">
+        <v>12</v>
+      </c>
+      <c r="C77">
+        <v>2</v>
+      </c>
+      <c r="D77">
         <v>113795.448700252</v>
       </c>
-      <c r="E73">
+      <c r="E77">
         <v>282179.67123287602</v>
       </c>
-      <c r="F73">
+      <c r="F77">
         <v>0.83403396920434802</v>
       </c>
-      <c r="G73">
+      <c r="G77">
         <v>20436.472361711199</v>
       </c>
-      <c r="H73">
+      <c r="H77">
         <v>4946.5396722567002</v>
       </c>
-      <c r="I73">
+      <c r="I77">
         <v>2967.9237851293901</v>
       </c>
-      <c r="J73">
+      <c r="J77">
         <v>28350.9358190973</v>
       </c>
-      <c r="K73">
+      <c r="K77">
         <v>50843.184005923598</v>
       </c>
-      <c r="L73">
+      <c r="L77">
         <v>15303.798385783</v>
       </c>
-      <c r="M73">
+      <c r="M77">
         <v>19297.530489448302</v>
       </c>
-      <c r="N73">
+      <c r="N77">
         <v>992.31070788530405</v>
       </c>
-      <c r="O73">
-        <v>0</v>
-      </c>
-      <c r="P73">
+      <c r="O77">
+        <v>0</v>
+      </c>
+      <c r="P77">
         <v>235347.43122713399</v>
       </c>
-      <c r="Q73">
+      <c r="Q77">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R73">
+      <c r="R77">
         <v>13.380488321454299</v>
       </c>
-      <c r="S73">
+      <c r="S77">
         <v>2.67609766429086</v>
       </c>
-      <c r="T73" s="6">
+      <c r="T77" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>

</xml_diff>

<commit_message>
getting baseline for 2026
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B249FF1E-39FC-45D1-8F1C-BAD1C73129A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A7A9567-2B89-4C2B-B980-28520FD85CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="11730" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="10170" yWindow="0" windowWidth="9120" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -117,7 +117,7 @@
     This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</t>
       </text>
     </comment>
-    <comment ref="A38" authorId="8" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A42" authorId="8" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -125,7 +125,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="A39" authorId="9" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A43" authorId="9" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -133,7 +133,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T39" authorId="10" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T43" authorId="10" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -143,7 +143,7 @@
     The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A45" authorId="11" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A49" authorId="11" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -151,7 +151,7 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="A62" authorId="12" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A66" authorId="12" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -159,7 +159,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T74" authorId="13" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T78" authorId="13" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -172,7 +172,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="42">
   <si>
     <t>Season</t>
   </si>
@@ -295,6 +295,9 @@
   </si>
   <si>
     <t>Charge Power Capacity</t>
+  </si>
+  <si>
+    <t>no flex</t>
   </si>
 </sst>
 </file>
@@ -1222,25 +1225,25 @@
   <threadedComment ref="A28" dT="2026-07-15T17:22:40.80" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
     <text>This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</text>
   </threadedComment>
-  <threadedComment ref="A38" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+  <threadedComment ref="A42" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
-  <threadedComment ref="A39" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+  <threadedComment ref="A43" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
     <text>Summer week = hot summer weekdays + high weekends</text>
   </threadedComment>
-  <threadedComment ref="T39" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T43" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure</text>
   </threadedComment>
-  <threadedComment ref="T39" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T43" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>The baseline costs have to be updated in accordance with the demand structure type</text>
   </threadedComment>
-  <threadedComment ref="A45" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+  <threadedComment ref="A49" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
     <text>Result from the fast solve</text>
   </threadedComment>
-  <threadedComment ref="A62" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+  <threadedComment ref="A66" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
     <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
   </threadedComment>
-  <threadedComment ref="T74" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="T78" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1248,7 +1251,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:V77"/>
+  <dimension ref="A1:V81"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.6328125" customWidth="1"/>
@@ -2564,262 +2567,218 @@
       <c r="B32" s="2"/>
       <c r="S32" s="2"/>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B33" s="2"/>
       <c r="S33" s="2"/>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A34" s="3" t="s">
-        <v>20</v>
-      </c>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A34" s="7"/>
       <c r="B34" s="2"/>
       <c r="S34" s="2"/>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A35" s="3" t="s">
-        <v>22</v>
-      </c>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A35" s="7"/>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A37" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="G37" s="4"/>
-    </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A38" s="5" t="s">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A36" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="S36" s="2"/>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A37" s="7"/>
+      <c r="B37" s="2"/>
+      <c r="S37" s="2"/>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A38" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B38" s="5" t="s">
-        <v>23</v>
+      <c r="B38" t="s">
+        <v>21</v>
       </c>
       <c r="C38">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D38">
-        <v>116861.67991782499</v>
+        <v>115568.67725355701</v>
       </c>
       <c r="E38">
-        <v>282179.67123287602</v>
+        <v>282179.671254922</v>
       </c>
       <c r="F38">
-        <v>0.84490020632262297</v>
+        <v>0.84031800989031202</v>
       </c>
       <c r="G38">
-        <v>23556.420831705898</v>
+        <v>21174.931050348201</v>
       </c>
       <c r="H38">
-        <v>6947.4542183048998</v>
+        <v>6483.8014286718599</v>
       </c>
       <c r="I38">
-        <v>913.29198665996</v>
+        <v>2465.4271592782502</v>
       </c>
       <c r="J38">
-        <v>31417.167036670799</v>
+        <v>30124.159638298399</v>
       </c>
       <c r="K38">
-        <v>50843.184005923598</v>
+        <v>50843.185222512198</v>
       </c>
       <c r="L38">
-        <v>15303.798385783</v>
+        <v>15303.8016501727</v>
       </c>
       <c r="M38">
-        <v>19297.5304894482</v>
+        <v>19297.530742573799</v>
       </c>
       <c r="N38">
-        <v>992.31070788530405</v>
+        <v>1409.83742959549</v>
       </c>
       <c r="O38">
         <v>0</v>
       </c>
       <c r="P38">
-        <v>238413.66244470701</v>
+        <v>237120.659780438</v>
       </c>
       <c r="Q38">
-        <v>1102.6552392369899</v>
+        <v>1101.67497109485</v>
       </c>
       <c r="R38">
-        <v>0</v>
+        <v>54.604983409531002</v>
       </c>
       <c r="S38">
-        <v>0</v>
+        <v>0.32502966315197002</v>
       </c>
       <c r="T38">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A39" s="5" t="s">
+        <v>-106.83117764915301</v>
+      </c>
+      <c r="U38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A39" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B39" s="5" t="s">
-        <v>23</v>
+      <c r="B39" t="s">
+        <v>21</v>
       </c>
       <c r="C39">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D39">
-        <v>187020.456722612</v>
+        <v>120779.539344445</v>
       </c>
       <c r="E39">
         <v>282179.67123287602</v>
       </c>
       <c r="F39">
-        <v>1.09353178385</v>
+        <v>0.858784478742043</v>
       </c>
       <c r="G39">
-        <v>89520.694507565597</v>
+        <v>22232.9956437156</v>
       </c>
       <c r="H39">
-        <v>6971.3813103080802</v>
+        <v>6892.28291987389</v>
       </c>
       <c r="I39">
-        <v>5083.8680235841202</v>
+        <v>5063.3926573547897</v>
       </c>
       <c r="J39">
-        <v>101575.943841457</v>
+        <v>34188.671220944299</v>
       </c>
       <c r="K39">
+        <v>51137.498573919998</v>
+      </c>
+      <c r="L39">
+        <v>16094.7687872735</v>
+      </c>
+      <c r="M39">
+        <v>19358.6007623076</v>
+      </c>
+      <c r="N39">
+        <v>1430.39398992981</v>
+      </c>
+      <c r="O39">
+        <v>0</v>
+      </c>
+      <c r="P39">
+        <v>242331.52187132699</v>
+      </c>
+      <c r="Q39">
+        <v>1171.0808202107701</v>
+      </c>
+      <c r="R39">
+        <v>13170.183258303599</v>
+      </c>
+      <c r="S39">
+        <v>487.784565122358</v>
+      </c>
+      <c r="T39">
+        <v>-0.16035717141929801</v>
+      </c>
+      <c r="U39">
+        <v>9733.9102750884304</v>
+      </c>
+      <c r="V39">
+        <v>69.034824646017199</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A41" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G41" s="4"/>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A42" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>116861.67991782499</v>
+      </c>
+      <c r="E42">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F42">
+        <v>0.84490020632262297</v>
+      </c>
+      <c r="G42">
+        <v>23556.420831705898</v>
+      </c>
+      <c r="H42">
+        <v>6947.4542183048998</v>
+      </c>
+      <c r="I42">
+        <v>913.29198665996</v>
+      </c>
+      <c r="J42">
+        <v>31417.167036670799</v>
+      </c>
+      <c r="K42">
         <v>50843.184005923598</v>
       </c>
-      <c r="L39">
+      <c r="L42">
         <v>15303.798385783</v>
       </c>
-      <c r="M39">
+      <c r="M42">
         <v>19297.5304894482</v>
-      </c>
-      <c r="N39">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O39">
-        <v>0</v>
-      </c>
-      <c r="P39">
-        <v>308572.439249494</v>
-      </c>
-      <c r="Q39">
-        <v>1106.4527933521999</v>
-      </c>
-      <c r="R39">
-        <v>3451.9307168288801</v>
-      </c>
-      <c r="S39">
-        <v>20.547206647791</v>
-      </c>
-      <c r="T39">
-        <v>-14.696886263168601</v>
-      </c>
-    </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A40" s="3"/>
-      <c r="G40" s="4"/>
-    </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>20</v>
-      </c>
-      <c r="B41" t="s">
-        <v>21</v>
-      </c>
-      <c r="C41">
-        <v>0</v>
-      </c>
-      <c r="D41">
-        <v>117032.41959359701</v>
-      </c>
-      <c r="E41">
-        <v>282179.67123286898</v>
-      </c>
-      <c r="F41">
-        <v>0.845505280653571</v>
-      </c>
-      <c r="G41" s="4">
-        <v>23683.129427060001</v>
-      </c>
-      <c r="H41">
-        <v>6986.3695969997798</v>
-      </c>
-      <c r="I41">
-        <v>918.40768838365295</v>
-      </c>
-      <c r="J41">
-        <v>31587.906712443499</v>
-      </c>
-      <c r="K41">
-        <v>50843.1840059237</v>
-      </c>
-      <c r="L41">
-        <v>15303.7983857823</v>
-      </c>
-      <c r="M41">
-        <v>19297.530489448101</v>
-      </c>
-      <c r="N41">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O41">
-        <v>0</v>
-      </c>
-      <c r="P41">
-        <v>238584.402120479</v>
-      </c>
-      <c r="Q41">
-        <v>1108.83163779344</v>
-      </c>
-      <c r="R41">
-        <v>0</v>
-      </c>
-      <c r="S41">
-        <v>230512.59606633501</v>
-      </c>
-      <c r="T41">
-        <v>1103.3673370121001</v>
-      </c>
-    </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>22</v>
-      </c>
-      <c r="B42" t="s">
-        <v>21</v>
-      </c>
-      <c r="C42">
-        <v>0</v>
-      </c>
-      <c r="D42">
-        <v>171564.02128394699</v>
-      </c>
-      <c r="E42">
-        <v>282179.67123287701</v>
-      </c>
-      <c r="F42">
-        <v>1.03875662810921</v>
-      </c>
-      <c r="G42">
-        <v>73514.1870928641</v>
-      </c>
-      <c r="H42">
-        <v>7482.8438362204697</v>
-      </c>
-      <c r="I42">
-        <v>4044.9309872213798</v>
-      </c>
-      <c r="J42">
-        <v>85041.961916305998</v>
-      </c>
-      <c r="K42">
-        <v>51119.832654572398</v>
-      </c>
-      <c r="L42">
-        <v>16047.2916290263</v>
-      </c>
-      <c r="M42">
-        <v>19354.9350840429</v>
       </c>
       <c r="N42">
         <v>992.31070788530405</v>
@@ -2828,214 +2787,274 @@
         <v>0</v>
       </c>
       <c r="P42">
-        <v>293116.00381082902</v>
+        <v>238413.66244470701</v>
       </c>
       <c r="Q42">
-        <v>1187.62883512946</v>
+        <v>1102.6552392369899</v>
       </c>
       <c r="R42">
-        <v>9393.8913494494009</v>
+        <v>0</v>
       </c>
       <c r="S42">
-        <v>260.94142637359403</v>
+        <v>0</v>
       </c>
       <c r="T42">
-        <v>-3.6405201993767098</v>
-      </c>
-    </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="G43" s="4"/>
-    </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A44" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A43" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+      <c r="D43">
+        <v>187020.456722612</v>
+      </c>
+      <c r="E43">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F43">
+        <v>1.09353178385</v>
+      </c>
+      <c r="G43">
+        <v>89520.694507565597</v>
+      </c>
+      <c r="H43">
+        <v>6971.3813103080802</v>
+      </c>
+      <c r="I43">
+        <v>5083.8680235841202</v>
+      </c>
+      <c r="J43">
+        <v>101575.943841457</v>
+      </c>
+      <c r="K43">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L43">
+        <v>15303.798385783</v>
+      </c>
+      <c r="M43">
+        <v>19297.5304894482</v>
+      </c>
+      <c r="N43">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O43">
+        <v>0</v>
+      </c>
+      <c r="P43">
+        <v>308572.439249494</v>
+      </c>
+      <c r="Q43">
+        <v>1106.4527933521999</v>
+      </c>
+      <c r="R43">
+        <v>3451.9307168288801</v>
+      </c>
+      <c r="S43">
+        <v>20.547206647791</v>
+      </c>
+      <c r="T43">
+        <v>-14.696886263168601</v>
+      </c>
+    </row>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A44" s="3"/>
+      <c r="G44" s="4"/>
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
         <v>20</v>
-      </c>
-      <c r="B44" t="s">
-        <v>21</v>
-      </c>
-      <c r="C44">
-        <v>4</v>
-      </c>
-      <c r="D44">
-        <v>116833.749486644</v>
-      </c>
-      <c r="E44">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F44">
-        <v>0.84480122530439805</v>
-      </c>
-      <c r="G44" s="4">
-        <v>23535.478746437901</v>
-      </c>
-      <c r="H44">
-        <v>6941.2778055266899</v>
-      </c>
-      <c r="I44">
-        <v>912.48005352310201</v>
-      </c>
-      <c r="J44">
-        <v>31389.236605487698</v>
-      </c>
-      <c r="K44">
-        <v>50843.184005923998</v>
-      </c>
-      <c r="L44">
-        <v>15303.798385784499</v>
-      </c>
-      <c r="M44">
-        <v>19297.5304894484</v>
-      </c>
-      <c r="N44">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O44">
-        <v>0</v>
-      </c>
-      <c r="P44">
-        <v>0</v>
-      </c>
-      <c r="Q44">
-        <v>0</v>
-      </c>
-      <c r="R44">
-        <v>0</v>
-      </c>
-      <c r="S44">
-        <v>0</v>
-      </c>
-      <c r="T44">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>22</v>
       </c>
       <c r="B45" t="s">
         <v>21</v>
       </c>
       <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>117032.41959359701</v>
+      </c>
+      <c r="E45">
+        <v>282179.67123286898</v>
+      </c>
+      <c r="F45">
+        <v>0.845505280653571</v>
+      </c>
+      <c r="G45" s="4">
+        <v>23683.129427060001</v>
+      </c>
+      <c r="H45">
+        <v>6986.3695969997798</v>
+      </c>
+      <c r="I45">
+        <v>918.40768838365295</v>
+      </c>
+      <c r="J45">
+        <v>31587.906712443499</v>
+      </c>
+      <c r="K45">
+        <v>50843.1840059237</v>
+      </c>
+      <c r="L45">
+        <v>15303.7983857823</v>
+      </c>
+      <c r="M45">
+        <v>19297.530489448101</v>
+      </c>
+      <c r="N45">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O45">
+        <v>0</v>
+      </c>
+      <c r="P45">
+        <v>238584.402120479</v>
+      </c>
+      <c r="Q45">
+        <v>1108.83163779344</v>
+      </c>
+      <c r="R45">
+        <v>0</v>
+      </c>
+      <c r="S45">
+        <v>230512.59606633501</v>
+      </c>
+      <c r="T45">
+        <v>1103.3673370121001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>22</v>
+      </c>
+      <c r="B46" t="s">
+        <v>21</v>
+      </c>
+      <c r="C46">
+        <v>0</v>
+      </c>
+      <c r="D46">
+        <v>171564.02128394699</v>
+      </c>
+      <c r="E46">
+        <v>282179.67123287701</v>
+      </c>
+      <c r="F46">
+        <v>1.03875662810921</v>
+      </c>
+      <c r="G46">
+        <v>73514.1870928641</v>
+      </c>
+      <c r="H46">
+        <v>7482.8438362204697</v>
+      </c>
+      <c r="I46">
+        <v>4044.9309872213798</v>
+      </c>
+      <c r="J46">
+        <v>85041.961916305998</v>
+      </c>
+      <c r="K46">
+        <v>51119.832654572398</v>
+      </c>
+      <c r="L46">
+        <v>16047.2916290263</v>
+      </c>
+      <c r="M46">
+        <v>19354.9350840429</v>
+      </c>
+      <c r="N46">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O46">
+        <v>0</v>
+      </c>
+      <c r="P46">
+        <v>293116.00381082902</v>
+      </c>
+      <c r="Q46">
+        <v>1187.62883512946</v>
+      </c>
+      <c r="R46">
+        <v>9393.8913494494009</v>
+      </c>
+      <c r="S46">
+        <v>260.94142637359403</v>
+      </c>
+      <c r="T46">
+        <v>-3.6405201993767098</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="G47" s="4"/>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A48" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B48" t="s">
+        <v>21</v>
+      </c>
+      <c r="C48">
         <v>4</v>
       </c>
-      <c r="D45">
-        <v>124393.533174422</v>
-      </c>
-      <c r="E45">
-        <v>282179.67123444699</v>
-      </c>
-      <c r="F45">
-        <v>0.87159189967643702</v>
-      </c>
-      <c r="G45" s="4">
-        <v>21072.189860718699</v>
-      </c>
-      <c r="H45">
-        <v>9188.7245080883695</v>
-      </c>
-      <c r="I45">
-        <v>2618.8827210474601</v>
-      </c>
-      <c r="J45">
-        <v>32879.797089854597</v>
-      </c>
-      <c r="K45">
-        <v>50904.118537438801</v>
-      </c>
-      <c r="L45">
-        <v>20591.7266090095</v>
-      </c>
-      <c r="M45">
-        <v>20017.890938119701</v>
-      </c>
-      <c r="N45">
-        <v>1040.9289460857101</v>
-      </c>
-      <c r="O45">
-        <v>0</v>
-      </c>
-      <c r="P45">
-        <v>245945.51570130399</v>
-      </c>
-      <c r="Q45">
-        <v>1458.3752411216699</v>
-      </c>
-      <c r="R45">
-        <v>35012.612233571497</v>
-      </c>
-      <c r="S45">
-        <v>875.31530583928895</v>
-      </c>
-      <c r="T45">
-        <v>0.51444695802960605</v>
-      </c>
-    </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A47" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G47" s="4"/>
-    </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>22</v>
-      </c>
-      <c r="B48" t="s">
-        <v>25</v>
-      </c>
-      <c r="C48">
-        <v>2</v>
-      </c>
       <c r="D48">
-        <v>115472.147206908</v>
+        <v>116833.749486644</v>
       </c>
       <c r="E48">
-        <v>282495</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F48">
-        <v>0.83903831831993503</v>
+        <v>0.84480122530439805</v>
       </c>
       <c r="G48" s="4">
-        <v>20221.889710343999</v>
+        <v>23535.478746437901</v>
       </c>
       <c r="H48">
-        <v>6553.7440767980397</v>
+        <v>6941.2778055266899</v>
       </c>
       <c r="I48">
-        <v>6160.4249909476703</v>
+        <v>912.48005352310201</v>
       </c>
       <c r="J48">
-        <v>32936.058778089697</v>
+        <v>31389.236605487698</v>
       </c>
       <c r="K48">
-        <v>50939.5611113743</v>
+        <v>50843.184005923998</v>
       </c>
       <c r="L48">
-        <v>15427.2204868183</v>
+        <v>15303.798385784499</v>
       </c>
       <c r="M48">
-        <v>19327.3039306102</v>
+        <v>19297.5304894484</v>
       </c>
       <c r="N48">
-        <v>1004.9477757237401</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O48">
-        <v>3157.9970999842499</v>
+        <v>0</v>
       </c>
       <c r="P48">
-        <v>237024.12973379</v>
+        <v>0</v>
       </c>
       <c r="Q48">
-        <v>1464.2687322859999</v>
+        <v>0</v>
       </c>
       <c r="R48">
-        <v>8672.9882445954008</v>
+        <v>0</v>
       </c>
       <c r="S48">
-        <v>346.91952978381602</v>
+        <v>0</v>
       </c>
       <c r="T48">
-        <v>2.4302910949698302</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:20" x14ac:dyDescent="0.35">
@@ -3043,443 +3062,446 @@
         <v>22</v>
       </c>
       <c r="B49" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C49">
         <v>4</v>
       </c>
       <c r="D49">
-        <v>108958.027502652</v>
+        <v>124393.533174422</v>
       </c>
       <c r="E49">
-        <v>282179.67123287602</v>
+        <v>282179.67123444699</v>
       </c>
       <c r="F49">
-        <v>0.81689091571482797</v>
+        <v>0.87159189967643702</v>
       </c>
       <c r="G49" s="4">
-        <v>20285.098342207999</v>
+        <v>21072.189860718699</v>
       </c>
       <c r="H49">
-        <v>6552.6722224723899</v>
+        <v>9188.7245080883695</v>
       </c>
       <c r="I49">
-        <v>6068.9240568166097</v>
+        <v>2618.8827210474601</v>
       </c>
       <c r="J49">
-        <v>32906.694621497001</v>
+        <v>32879.797089854597</v>
       </c>
       <c r="K49">
-        <v>50843.184005923598</v>
+        <v>50904.118537438801</v>
       </c>
       <c r="L49">
-        <v>16378.7983857829</v>
+        <v>20591.7266090095</v>
       </c>
       <c r="M49">
-        <v>19449.350489448301</v>
+        <v>20017.890938119701</v>
       </c>
       <c r="N49">
-        <v>1004.9477757237401</v>
+        <v>1040.9289460857101</v>
       </c>
       <c r="O49">
-        <v>10620</v>
+        <v>0</v>
       </c>
       <c r="P49">
-        <v>230510.010029533</v>
+        <v>245945.51570130399</v>
       </c>
       <c r="Q49">
-        <v>1464.02925348484</v>
+        <v>1458.3752411216699</v>
       </c>
       <c r="R49">
-        <v>26064.489084194902</v>
+        <v>35012.612233571497</v>
       </c>
       <c r="S49">
-        <v>407.257641940545</v>
+        <v>875.31530583928895</v>
       </c>
       <c r="T49">
-        <v>1.09609872121186</v>
+        <v>0.51444695802960605</v>
       </c>
     </row>
     <row r="51" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G51" s="4"/>
+    </row>
+    <row r="52" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>22</v>
+      </c>
+      <c r="B52" t="s">
+        <v>25</v>
+      </c>
+      <c r="C52">
+        <v>2</v>
+      </c>
+      <c r="D52">
+        <v>115472.147206908</v>
+      </c>
+      <c r="E52">
+        <v>282495</v>
+      </c>
+      <c r="F52">
+        <v>0.83903831831993503</v>
+      </c>
+      <c r="G52" s="4">
+        <v>20221.889710343999</v>
+      </c>
+      <c r="H52">
+        <v>6553.7440767980397</v>
+      </c>
+      <c r="I52">
+        <v>6160.4249909476703</v>
+      </c>
+      <c r="J52">
+        <v>32936.058778089697</v>
+      </c>
+      <c r="K52">
+        <v>50939.5611113743</v>
+      </c>
+      <c r="L52">
+        <v>15427.2204868183</v>
+      </c>
+      <c r="M52">
+        <v>19327.3039306102</v>
+      </c>
+      <c r="N52">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O52">
+        <v>3157.9970999842499</v>
+      </c>
+      <c r="P52">
+        <v>237024.12973379</v>
+      </c>
+      <c r="Q52">
+        <v>1464.2687322859999</v>
+      </c>
+      <c r="R52">
+        <v>8672.9882445954008</v>
+      </c>
+      <c r="S52">
+        <v>346.91952978381602</v>
+      </c>
+      <c r="T52">
+        <v>2.4302910949698302</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>22</v>
+      </c>
+      <c r="B53" t="s">
+        <v>25</v>
+      </c>
+      <c r="C53">
+        <v>4</v>
+      </c>
+      <c r="D53">
+        <v>108958.027502652</v>
+      </c>
+      <c r="E53">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F53">
+        <v>0.81689091571482797</v>
+      </c>
+      <c r="G53" s="4">
+        <v>20285.098342207999</v>
+      </c>
+      <c r="H53">
+        <v>6552.6722224723899</v>
+      </c>
+      <c r="I53">
+        <v>6068.9240568166097</v>
+      </c>
+      <c r="J53">
+        <v>32906.694621497001</v>
+      </c>
+      <c r="K53">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L53">
+        <v>16378.7983857829</v>
+      </c>
+      <c r="M53">
+        <v>19449.350489448301</v>
+      </c>
+      <c r="N53">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O53">
+        <v>10620</v>
+      </c>
+      <c r="P53">
+        <v>230510.010029533</v>
+      </c>
+      <c r="Q53">
+        <v>1464.02925348484</v>
+      </c>
+      <c r="R53">
+        <v>26064.489084194902</v>
+      </c>
+      <c r="S53">
+        <v>407.257641940545</v>
+      </c>
+      <c r="T53">
+        <v>1.09609872121186</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A55" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A52" s="3" t="s">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="B56" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C52">
-        <v>0</v>
-      </c>
-      <c r="D52">
+      <c r="C56">
+        <v>0</v>
+      </c>
+      <c r="D56">
         <v>115030.978322179</v>
-      </c>
-      <c r="E52">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F52">
-        <v>0.83841249022441</v>
-      </c>
-      <c r="G52">
-        <v>20114.092712805999</v>
-      </c>
-      <c r="H52">
-        <v>6942.2846600808298</v>
-      </c>
-      <c r="I52">
-        <v>2530.0880681377598</v>
-      </c>
-      <c r="J52">
-        <v>29586.4654410246</v>
-      </c>
-      <c r="K52">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L52">
-        <v>15303.798385783</v>
-      </c>
-      <c r="M52">
-        <v>19297.5304894482</v>
-      </c>
-      <c r="N52">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O52">
-        <v>0</v>
-      </c>
-      <c r="P52">
-        <v>236582.960849061</v>
-      </c>
-      <c r="Q52">
-        <v>1101.8347602124099</v>
-      </c>
-      <c r="R52">
-        <v>0</v>
-      </c>
-      <c r="S52">
-        <v>0</v>
-      </c>
-      <c r="T52">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A53" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C53">
-        <v>0</v>
-      </c>
-      <c r="D53">
-        <v>124771.246709449</v>
-      </c>
-      <c r="E53">
-        <v>282179.67125180899</v>
-      </c>
-      <c r="F53">
-        <v>0.87293045648394496</v>
-      </c>
-      <c r="G53">
-        <v>22626.697961956499</v>
-      </c>
-      <c r="H53">
-        <v>7102.5767129513297</v>
-      </c>
-      <c r="I53">
-        <v>9597.4591384874802</v>
-      </c>
-      <c r="J53">
-        <v>39326.733813395302</v>
-      </c>
-      <c r="K53">
-        <v>50843.184011688398</v>
-      </c>
-      <c r="L53">
-        <v>15303.798393134501</v>
-      </c>
-      <c r="M53">
-        <v>19297.530491231599</v>
-      </c>
-      <c r="N53">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O53">
-        <v>0</v>
-      </c>
-      <c r="P53">
-        <v>246323.22923633101</v>
-      </c>
-      <c r="Q53">
-        <v>1127.27501714903</v>
-      </c>
-      <c r="R53">
-        <v>0</v>
-      </c>
-      <c r="S53">
-        <v>0</v>
-      </c>
-      <c r="T53">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A54" s="1"/>
-    </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>20</v>
-      </c>
-      <c r="B55" t="s">
-        <v>21</v>
-      </c>
-      <c r="C55">
-        <v>2</v>
-      </c>
-      <c r="D55">
-        <v>115714.10508262301</v>
-      </c>
-      <c r="E55">
-        <v>282179.67125387199</v>
-      </c>
-      <c r="F55">
-        <v>0.840833383054163</v>
-      </c>
-      <c r="G55" s="4">
-        <v>20578.507216446698</v>
-      </c>
-      <c r="H55">
-        <v>7102.57515066207</v>
-      </c>
-      <c r="I55">
-        <v>2588.5052959285099</v>
-      </c>
-      <c r="J55">
-        <v>30269.587663037299</v>
-      </c>
-      <c r="K55">
-        <v>50843.185173268597</v>
-      </c>
-      <c r="L55">
-        <v>15303.8015139941</v>
-      </c>
-      <c r="M55">
-        <v>19297.530732323401</v>
-      </c>
-      <c r="N55">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O55">
-        <v>0</v>
-      </c>
-      <c r="P55">
-        <v>237266.08760950499</v>
-      </c>
-      <c r="Q55">
-        <v>1127.2750356983099</v>
-      </c>
-      <c r="R55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>22</v>
-      </c>
-      <c r="B56" t="s">
-        <v>21</v>
-      </c>
-      <c r="C56">
-        <v>2</v>
-      </c>
-      <c r="D56">
-        <v>120628.41082793</v>
       </c>
       <c r="E56">
         <v>282179.67123287602</v>
       </c>
       <c r="F56">
-        <v>0.85824890324911396</v>
-      </c>
-      <c r="G56" s="4">
-        <v>20824.7129679639</v>
+        <v>0.83841249022441</v>
+      </c>
+      <c r="G56">
+        <v>20114.092712805999</v>
       </c>
       <c r="H56">
-        <v>7456.39074483072</v>
+        <v>6942.2846600808298</v>
       </c>
       <c r="I56">
-        <v>5114.4587365303096</v>
+        <v>2530.0880681377598</v>
       </c>
       <c r="J56">
-        <v>33395.562449324898</v>
+        <v>29586.4654410246</v>
       </c>
       <c r="K56">
-        <v>51302.320205525801</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L56">
-        <v>16537.7269222135</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M56">
-        <v>19392.801250865799</v>
+        <v>19297.5304894482</v>
       </c>
       <c r="N56">
-        <v>1004.9477757237401</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O56">
         <v>0</v>
       </c>
       <c r="P56">
-        <v>242180.39335481101</v>
+        <v>236582.960849061</v>
       </c>
       <c r="Q56">
-        <v>1183.4303612998101</v>
+        <v>1101.8347602124099</v>
       </c>
       <c r="R56">
-        <v>15931.1957490451</v>
+        <v>0</v>
       </c>
       <c r="S56">
-        <v>346.33034237054602</v>
+        <v>0</v>
       </c>
       <c r="T56">
-        <v>1.0959871186973</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A57" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C57">
+        <v>0</v>
+      </c>
+      <c r="D57">
+        <v>124771.246709449</v>
+      </c>
+      <c r="E57">
+        <v>282179.67125180899</v>
+      </c>
+      <c r="F57">
+        <v>0.87293045648394496</v>
+      </c>
+      <c r="G57">
+        <v>22626.697961956499</v>
+      </c>
+      <c r="H57">
+        <v>7102.5767129513297</v>
+      </c>
+      <c r="I57">
+        <v>9597.4591384874802</v>
+      </c>
+      <c r="J57">
+        <v>39326.733813395302</v>
+      </c>
+      <c r="K57">
+        <v>50843.184011688398</v>
+      </c>
+      <c r="L57">
+        <v>15303.798393134501</v>
+      </c>
+      <c r="M57">
+        <v>19297.530491231599</v>
+      </c>
+      <c r="N57">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O57">
+        <v>0</v>
+      </c>
+      <c r="P57">
+        <v>246323.22923633101</v>
+      </c>
+      <c r="Q57">
+        <v>1127.27501714903</v>
+      </c>
+      <c r="R57">
+        <v>0</v>
+      </c>
+      <c r="S57">
+        <v>0</v>
+      </c>
+      <c r="T57">
+        <v>0</v>
       </c>
     </row>
     <row r="58" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>20</v>
-      </c>
-      <c r="B58" t="s">
-        <v>21</v>
-      </c>
-      <c r="C58">
-        <v>4</v>
-      </c>
-      <c r="D58">
-        <v>115714.10508261999</v>
-      </c>
-      <c r="E58">
-        <v>282179.671253876</v>
-      </c>
-      <c r="F58">
-        <v>0.84083338305413902</v>
-      </c>
-      <c r="G58" s="4">
-        <v>20578.5072164468</v>
-      </c>
-      <c r="H58">
-        <v>7102.5751506616798</v>
-      </c>
-      <c r="I58">
-        <v>2588.50529592865</v>
-      </c>
-      <c r="J58">
-        <v>30269.587663037099</v>
-      </c>
-      <c r="K58">
-        <v>50843.185173268197</v>
-      </c>
-      <c r="L58">
-        <v>15303.8015139912</v>
-      </c>
-      <c r="M58">
-        <v>19297.530732323299</v>
-      </c>
-      <c r="N58">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O58">
-        <v>0</v>
-      </c>
-      <c r="P58">
-        <v>237266.087609501</v>
-      </c>
-      <c r="Q58">
-        <v>1127.2750356983499</v>
-      </c>
-      <c r="R58">
-        <v>0</v>
-      </c>
+      <c r="A58" s="1"/>
     </row>
     <row r="59" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B59" t="s">
         <v>21</v>
       </c>
       <c r="C59">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D59">
-        <v>120375.156660901</v>
+        <v>115714.10508262301</v>
       </c>
       <c r="E59">
-        <v>282179.671232878</v>
+        <v>282179.67125387199</v>
       </c>
       <c r="F59">
-        <v>0.857351410648304</v>
+        <v>0.840833383054163</v>
       </c>
       <c r="G59" s="4">
-        <v>21285.1004075495</v>
+        <v>20578.507216446698</v>
       </c>
       <c r="H59">
-        <v>7426.32532798384</v>
+        <v>7102.57515066207</v>
       </c>
       <c r="I59">
-        <v>5046.79446201879</v>
+        <v>2588.5052959285099</v>
       </c>
       <c r="J59">
-        <v>33758.220197552102</v>
+        <v>30269.587663037299</v>
       </c>
       <c r="K59">
-        <v>51144.191344099498</v>
+        <v>50843.185173268597</v>
       </c>
       <c r="L59">
-        <v>16112.7556071296</v>
+        <v>15303.8015139941</v>
       </c>
       <c r="M59">
-        <v>19359.989512119799</v>
+        <v>19297.530732323401</v>
       </c>
       <c r="N59">
-        <v>1006.77939378399</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O59">
         <v>0</v>
       </c>
       <c r="P59">
-        <v>241927.13918778201</v>
+        <v>237266.08760950499</v>
       </c>
       <c r="Q59">
-        <v>1178.65858109644</v>
+        <v>1127.2750356983099</v>
       </c>
       <c r="R59">
-        <v>12586.325853030899</v>
-      </c>
-      <c r="S59">
-        <v>466.16021677892502</v>
-      </c>
-      <c r="T59">
-        <v>1.3585822738026401</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="G60" s="4"/>
-    </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A61" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G61" s="4"/>
+      <c r="A60" t="s">
+        <v>22</v>
+      </c>
+      <c r="B60" t="s">
+        <v>21</v>
+      </c>
+      <c r="C60">
+        <v>2</v>
+      </c>
+      <c r="D60">
+        <v>120628.41082793</v>
+      </c>
+      <c r="E60">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F60">
+        <v>0.85824890324911396</v>
+      </c>
+      <c r="G60" s="4">
+        <v>20824.7129679639</v>
+      </c>
+      <c r="H60">
+        <v>7456.39074483072</v>
+      </c>
+      <c r="I60">
+        <v>5114.4587365303096</v>
+      </c>
+      <c r="J60">
+        <v>33395.562449324898</v>
+      </c>
+      <c r="K60">
+        <v>51302.320205525801</v>
+      </c>
+      <c r="L60">
+        <v>16537.7269222135</v>
+      </c>
+      <c r="M60">
+        <v>19392.801250865799</v>
+      </c>
+      <c r="N60">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O60">
+        <v>0</v>
+      </c>
+      <c r="P60">
+        <v>242180.39335481101</v>
+      </c>
+      <c r="Q60">
+        <v>1183.4303612998101</v>
+      </c>
+      <c r="R60">
+        <v>15931.1957490451</v>
+      </c>
+      <c r="S60">
+        <v>346.33034237054602</v>
+      </c>
+      <c r="T60">
+        <v>1.0959871186973</v>
+      </c>
     </row>
     <row r="62" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B62" t="s">
         <v>21</v>
@@ -3488,55 +3510,49 @@
         <v>4</v>
       </c>
       <c r="D62">
-        <v>146108.01933512901</v>
+        <v>115714.10508261999</v>
       </c>
       <c r="E62">
-        <v>355610.364944759</v>
+        <v>282179.671253876</v>
       </c>
       <c r="F62">
-        <v>0.75267772890587503</v>
-      </c>
-      <c r="G62">
-        <v>25765.651662743599</v>
+        <v>0.84083338305413902</v>
+      </c>
+      <c r="G62" s="4">
+        <v>20578.5072164468</v>
       </c>
       <c r="H62">
-        <v>7150.9042815892099</v>
+        <v>7102.5751506616798</v>
       </c>
       <c r="I62">
-        <v>5144.3184852884797</v>
+        <v>2588.50529592865</v>
       </c>
       <c r="J62">
-        <v>38060.874429621297</v>
+        <v>30269.587663037099</v>
       </c>
       <c r="K62">
-        <v>64168.339029134899</v>
+        <v>50843.185173268197</v>
       </c>
       <c r="L62">
-        <v>19539.954214541001</v>
+        <v>15303.8015139912</v>
       </c>
       <c r="M62">
-        <v>24338.851661831999</v>
+        <v>19297.530732323299</v>
       </c>
       <c r="N62">
-        <v>1010.46273302954</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O62">
         <v>0</v>
       </c>
       <c r="P62">
-        <v>267660.00186201098</v>
+        <v>237266.087609501</v>
       </c>
       <c r="Q62">
-        <v>1597.68911089628</v>
+        <v>1127.2750356983499</v>
       </c>
       <c r="R62">
-        <v>13084.0423994256</v>
-      </c>
-      <c r="S62">
-        <v>467.28722855091399</v>
-      </c>
-      <c r="T62">
-        <v>-0.25904927491985202</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:20" x14ac:dyDescent="0.35">
@@ -3544,514 +3560,399 @@
         <v>22</v>
       </c>
       <c r="B63" t="s">
+        <v>21</v>
+      </c>
+      <c r="C63">
+        <v>4</v>
+      </c>
+      <c r="D63">
+        <v>120375.156660901</v>
+      </c>
+      <c r="E63">
+        <v>282179.671232878</v>
+      </c>
+      <c r="F63">
+        <v>0.857351410648304</v>
+      </c>
+      <c r="G63" s="4">
+        <v>21285.1004075495</v>
+      </c>
+      <c r="H63">
+        <v>7426.32532798384</v>
+      </c>
+      <c r="I63">
+        <v>5046.79446201879</v>
+      </c>
+      <c r="J63">
+        <v>33758.220197552102</v>
+      </c>
+      <c r="K63">
+        <v>51144.191344099498</v>
+      </c>
+      <c r="L63">
+        <v>16112.7556071296</v>
+      </c>
+      <c r="M63">
+        <v>19359.989512119799</v>
+      </c>
+      <c r="N63">
+        <v>1006.77939378399</v>
+      </c>
+      <c r="O63">
+        <v>0</v>
+      </c>
+      <c r="P63">
+        <v>241927.13918778201</v>
+      </c>
+      <c r="Q63">
+        <v>1178.65858109644</v>
+      </c>
+      <c r="R63">
+        <v>12586.325853030899</v>
+      </c>
+      <c r="S63">
+        <v>466.16021677892502</v>
+      </c>
+      <c r="T63">
+        <v>1.3585822738026401</v>
+      </c>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="G64" s="4"/>
+    </row>
+    <row r="65" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A65" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G65" s="4"/>
+    </row>
+    <row r="66" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>22</v>
+      </c>
+      <c r="B66" t="s">
+        <v>21</v>
+      </c>
+      <c r="C66">
+        <v>4</v>
+      </c>
+      <c r="D66">
+        <v>146108.01933512901</v>
+      </c>
+      <c r="E66">
+        <v>355610.364944759</v>
+      </c>
+      <c r="F66">
+        <v>0.75267772890587503</v>
+      </c>
+      <c r="G66">
+        <v>25765.651662743599</v>
+      </c>
+      <c r="H66">
+        <v>7150.9042815892099</v>
+      </c>
+      <c r="I66">
+        <v>5144.3184852884797</v>
+      </c>
+      <c r="J66">
+        <v>38060.874429621297</v>
+      </c>
+      <c r="K66">
+        <v>64168.339029134899</v>
+      </c>
+      <c r="L66">
+        <v>19539.954214541001</v>
+      </c>
+      <c r="M66">
+        <v>24338.851661831999</v>
+      </c>
+      <c r="N66">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O66">
+        <v>0</v>
+      </c>
+      <c r="P66">
+        <v>267660.00186201098</v>
+      </c>
+      <c r="Q66">
+        <v>1597.68911089628</v>
+      </c>
+      <c r="R66">
+        <v>13084.0423994256</v>
+      </c>
+      <c r="S66">
+        <v>467.28722855091399</v>
+      </c>
+      <c r="T66">
+        <v>-0.25904927491985202</v>
+      </c>
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>22</v>
+      </c>
+      <c r="B67" t="s">
         <v>35</v>
       </c>
-      <c r="C63" t="s">
+      <c r="C67" t="s">
         <v>35</v>
       </c>
-      <c r="D63" t="s">
+      <c r="D67" t="s">
         <v>36</v>
       </c>
-      <c r="E63" t="s">
+      <c r="E67" t="s">
         <v>36</v>
       </c>
-      <c r="F63" t="s">
+      <c r="F67" t="s">
         <v>36</v>
       </c>
-      <c r="G63" s="4">
+      <c r="G67" s="4">
         <v>28838</v>
       </c>
-      <c r="H63">
+      <c r="H67">
         <v>7567.5</v>
       </c>
-      <c r="I63">
+      <c r="I67">
         <v>13764.1</v>
       </c>
-      <c r="J63">
+      <c r="J67">
         <v>50169.7</v>
       </c>
-      <c r="K63" t="s">
+      <c r="K67" t="s">
         <v>36</v>
       </c>
-      <c r="L63" t="s">
+      <c r="L67" t="s">
         <v>36</v>
       </c>
-      <c r="M63" t="s">
+      <c r="M67" t="s">
         <v>36</v>
       </c>
-      <c r="N63" t="s">
+      <c r="N67" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="65" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="1" t="s">
+    <row r="69" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G65" s="4"/>
-      <c r="P65" t="s">
+      <c r="G69" s="4"/>
+      <c r="P69" t="s">
         <v>15</v>
       </c>
-      <c r="Q65" t="s">
+      <c r="Q69" t="s">
         <v>16</v>
       </c>
-      <c r="R65" t="s">
+      <c r="R69" t="s">
         <v>17</v>
       </c>
-      <c r="S65" t="s">
+      <c r="S69" t="s">
         <v>18</v>
       </c>
-      <c r="T65" t="s">
+      <c r="T69" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="66" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
-        <v>0</v>
-      </c>
-      <c r="B66" t="s">
+    <row r="70" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>0</v>
+      </c>
+      <c r="B70" t="s">
         <v>1</v>
-      </c>
-      <c r="C66" t="s">
-        <v>2</v>
-      </c>
-      <c r="D66" t="s">
-        <v>3</v>
-      </c>
-      <c r="E66" t="s">
-        <v>4</v>
-      </c>
-      <c r="F66" t="s">
-        <v>5</v>
-      </c>
-      <c r="G66" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H66" t="s">
-        <v>7</v>
-      </c>
-      <c r="I66" t="s">
-        <v>8</v>
-      </c>
-      <c r="J66" t="s">
-        <v>9</v>
-      </c>
-      <c r="K66" t="s">
-        <v>10</v>
-      </c>
-      <c r="L66" t="s">
-        <v>11</v>
-      </c>
-      <c r="M66" t="s">
-        <v>12</v>
-      </c>
-      <c r="N66" t="s">
-        <v>13</v>
-      </c>
-      <c r="O66" t="s">
-        <v>14</v>
-      </c>
-      <c r="P66">
-        <v>63734.6679</v>
-      </c>
-      <c r="Q66">
-        <v>1078.4492829999999</v>
-      </c>
-      <c r="R66">
-        <v>624.70352849999995</v>
-      </c>
-      <c r="S66">
-        <v>13.014656840000001</v>
-      </c>
-      <c r="T66">
-        <v>27.514184579999998</v>
-      </c>
-    </row>
-    <row r="67" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B67" t="s">
-        <v>21</v>
-      </c>
-      <c r="C67">
-        <v>4</v>
-      </c>
-      <c r="D67">
-        <v>29525.427309999999</v>
-      </c>
-      <c r="E67">
-        <v>80391.755990000005</v>
-      </c>
-      <c r="F67">
-        <v>0.79280104200000001</v>
-      </c>
-      <c r="G67" s="4">
-        <v>5050.6365619999997</v>
-      </c>
-      <c r="H67">
-        <v>4678.3390820000004</v>
-      </c>
-      <c r="I67">
-        <v>2508.6600360000002</v>
-      </c>
-      <c r="J67">
-        <v>12237.635679999999</v>
-      </c>
-      <c r="K67">
-        <v>13920</v>
-      </c>
-      <c r="L67">
-        <v>2841.544922</v>
-      </c>
-      <c r="M67">
-        <v>5380.5444360000001</v>
-      </c>
-      <c r="N67">
-        <v>279.27307350000001</v>
-      </c>
-      <c r="O67">
-        <v>0</v>
-      </c>
-      <c r="P67">
-        <v>64865.028310000002</v>
-      </c>
-      <c r="Q67">
-        <v>1191.7509680000001</v>
-      </c>
-      <c r="R67">
-        <v>7243.7162129999997</v>
-      </c>
-      <c r="S67">
-        <v>452.7322633</v>
-      </c>
-      <c r="T67">
-        <v>5.8154128590000003</v>
-      </c>
-    </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A68" s="7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
-        <v>32</v>
-      </c>
-      <c r="B70" t="s">
-        <v>33</v>
       </c>
       <c r="C70" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A71">
+      <c r="D70" t="s">
+        <v>3</v>
+      </c>
+      <c r="E70" t="s">
+        <v>4</v>
+      </c>
+      <c r="F70" t="s">
+        <v>5</v>
+      </c>
+      <c r="G70" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H70" t="s">
+        <v>7</v>
+      </c>
+      <c r="I70" t="s">
+        <v>8</v>
+      </c>
+      <c r="J70" t="s">
+        <v>9</v>
+      </c>
+      <c r="K70" t="s">
+        <v>10</v>
+      </c>
+      <c r="L70" t="s">
+        <v>11</v>
+      </c>
+      <c r="M70" t="s">
+        <v>12</v>
+      </c>
+      <c r="N70" t="s">
+        <v>13</v>
+      </c>
+      <c r="O70" t="s">
+        <v>14</v>
+      </c>
+      <c r="P70">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q70">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R70">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S70">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T70">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="71" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B71">
+      <c r="B71" t="s">
+        <v>21</v>
+      </c>
+      <c r="C71">
+        <v>4</v>
+      </c>
+      <c r="D71">
+        <v>29525.427309999999</v>
+      </c>
+      <c r="E71">
+        <v>80391.755990000005</v>
+      </c>
+      <c r="F71">
+        <v>0.79280104200000001</v>
+      </c>
+      <c r="G71" s="4">
+        <v>5050.6365619999997</v>
+      </c>
+      <c r="H71">
+        <v>4678.3390820000004</v>
+      </c>
+      <c r="I71">
+        <v>2508.6600360000002</v>
+      </c>
+      <c r="J71">
+        <v>12237.635679999999</v>
+      </c>
+      <c r="K71">
+        <v>13920</v>
+      </c>
+      <c r="L71">
+        <v>2841.544922</v>
+      </c>
+      <c r="M71">
+        <v>5380.5444360000001</v>
+      </c>
+      <c r="N71">
+        <v>279.27307350000001</v>
+      </c>
+      <c r="O71">
+        <v>0</v>
+      </c>
+      <c r="P71">
+        <v>64865.028310000002</v>
+      </c>
+      <c r="Q71">
+        <v>1191.7509680000001</v>
+      </c>
+      <c r="R71">
+        <v>7243.7162129999997</v>
+      </c>
+      <c r="S71">
+        <v>452.7322633</v>
+      </c>
+      <c r="T71">
+        <v>5.8154128590000003</v>
+      </c>
+    </row>
+    <row r="72" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A72" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="74" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>32</v>
+      </c>
+      <c r="B74" t="s">
+        <v>33</v>
+      </c>
+      <c r="C74" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A75">
+        <v>20</v>
+      </c>
+      <c r="B75">
         <v>60</v>
       </c>
-      <c r="C71">
+      <c r="C75">
         <v>2</v>
       </c>
-      <c r="D71">
+      <c r="D75">
         <v>119696.652328767</v>
       </c>
-      <c r="E71">
+      <c r="E75">
         <v>282179.67123285501</v>
       </c>
-      <c r="F71">
+      <c r="F75">
         <v>0.854946898908852</v>
       </c>
-      <c r="G71">
+      <c r="G75">
         <v>18681.222424938602</v>
       </c>
-      <c r="H71">
+      <c r="H75">
         <v>5354.6114985546601</v>
       </c>
-      <c r="I71">
+      <c r="I75">
         <v>8156.08309050551</v>
       </c>
-      <c r="J71">
+      <c r="J75">
         <v>32191.917013998798</v>
       </c>
-      <c r="K71">
+      <c r="K75">
         <v>51372.124296964801</v>
       </c>
-      <c r="L71">
+      <c r="L75">
         <v>16725.325417965501</v>
       </c>
-      <c r="M71">
+      <c r="M75">
         <v>19407.285599838699</v>
       </c>
-      <c r="N71">
+      <c r="N75">
         <v>1016.03855436447</v>
       </c>
-      <c r="O71">
-        <v>0</v>
-      </c>
-      <c r="P71">
+      <c r="O75">
+        <v>0</v>
+      </c>
+      <c r="P75">
         <v>241248.634855649</v>
       </c>
-      <c r="Q71">
+      <c r="Q75">
         <v>1192.7637589594799</v>
       </c>
-      <c r="R71">
+      <c r="R75">
         <v>19736.206339365101</v>
       </c>
-      <c r="S71">
+      <c r="S75">
         <v>481.37088632597801</v>
       </c>
-      <c r="T71" s="6">
+      <c r="T75" s="6">
         <v>0.12591688076390301</v>
-      </c>
-    </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A72">
-        <v>20</v>
-      </c>
-      <c r="B72">
-        <v>50</v>
-      </c>
-      <c r="C72">
-        <v>2</v>
-      </c>
-      <c r="D72">
-        <v>118381.960809661</v>
-      </c>
-      <c r="E72">
-        <v>282254.81855225202</v>
-      </c>
-      <c r="F72">
-        <v>0.85006146065890897</v>
-      </c>
-      <c r="G72">
-        <v>19407.840072768398</v>
-      </c>
-      <c r="H72">
-        <v>5891.8301217549197</v>
-      </c>
-      <c r="I72">
-        <v>6659.4942697455399</v>
-      </c>
-      <c r="J72">
-        <v>31959.164464268899</v>
-      </c>
-      <c r="K72">
-        <v>51102.045942938203</v>
-      </c>
-      <c r="L72">
-        <v>15967.176494174801</v>
-      </c>
-      <c r="M72">
-        <v>19353.573908279199</v>
-      </c>
-      <c r="N72">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O72">
-        <v>0</v>
-      </c>
-      <c r="P72">
-        <v>239933.943336542</v>
-      </c>
-      <c r="Q72">
-        <v>1312.43161993582</v>
-      </c>
-      <c r="R72">
-        <v>18377.616631847999</v>
-      </c>
-      <c r="S72">
-        <v>459.4404157962</v>
-      </c>
-      <c r="T72" s="6">
-        <v>0.14758705239613301</v>
-      </c>
-    </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A73">
-        <v>20</v>
-      </c>
-      <c r="B73">
-        <v>40</v>
-      </c>
-      <c r="C73">
-        <v>2</v>
-      </c>
-      <c r="D73">
-        <v>116766.56672038</v>
-      </c>
-      <c r="E73">
-        <v>282179.67123287299</v>
-      </c>
-      <c r="F73">
-        <v>0.84456314023622803</v>
-      </c>
-      <c r="G73">
-        <v>19298.245593088301</v>
-      </c>
-      <c r="H73">
-        <v>5682.0016560700296</v>
-      </c>
-      <c r="I73">
-        <v>5350.3346939491703</v>
-      </c>
-      <c r="J73">
-        <v>30330.5819431075</v>
-      </c>
-      <c r="K73">
-        <v>51097.733915068202</v>
-      </c>
-      <c r="L73">
-        <v>15987.901266609</v>
-      </c>
-      <c r="M73">
-        <v>19350.349595595701</v>
-      </c>
-      <c r="N73">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O73">
-        <v>0</v>
-      </c>
-      <c r="P73">
-        <v>238318.54924726201</v>
-      </c>
-      <c r="Q73">
-        <v>1265.6913868611</v>
-      </c>
-      <c r="R73">
-        <v>17746.163883660702</v>
-      </c>
-      <c r="S73">
-        <v>507.03325381887902</v>
-      </c>
-      <c r="T73" s="6">
-        <v>-0.25983751983286502</v>
-      </c>
-    </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A74">
-        <v>20</v>
-      </c>
-      <c r="B74">
-        <v>30</v>
-      </c>
-      <c r="C74">
-        <v>2</v>
-      </c>
-      <c r="D74">
-        <v>115610.996393592</v>
-      </c>
-      <c r="E74">
-        <v>282182.50548365602</v>
-      </c>
-      <c r="F74">
-        <v>0.84045954058697003</v>
-      </c>
-      <c r="G74">
-        <v>19302.752565837702</v>
-      </c>
-      <c r="H74">
-        <v>6226.5181629292701</v>
-      </c>
-      <c r="I74">
-        <v>3974.5318253822402</v>
-      </c>
-      <c r="J74">
-        <v>29503.802554149199</v>
-      </c>
-      <c r="K74">
-        <v>51013.610661725899</v>
-      </c>
-      <c r="L74">
-        <v>15760.601295416</v>
-      </c>
-      <c r="M74">
-        <v>19332.981882301501</v>
-      </c>
-      <c r="N74">
-        <v>1014.17312250211</v>
-      </c>
-      <c r="O74">
-        <v>0</v>
-      </c>
-      <c r="P74">
-        <v>237162.97892047401</v>
-      </c>
-      <c r="Q74">
-        <v>1386.9848841974899</v>
-      </c>
-      <c r="R74">
-        <v>18436.445202769701</v>
-      </c>
-      <c r="S74">
-        <v>209.50505912238299</v>
-      </c>
-      <c r="T74" s="6">
-        <v>0.28049716262959101</v>
-      </c>
-    </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A75" s="3">
-        <v>20</v>
-      </c>
-      <c r="B75" s="3">
-        <v>20</v>
-      </c>
-      <c r="C75" s="3">
-        <v>2</v>
-      </c>
-      <c r="D75">
-        <v>114184.286860504</v>
-      </c>
-      <c r="E75">
-        <v>282179.67123297497</v>
-      </c>
-      <c r="F75">
-        <v>0.83541194997266699</v>
-      </c>
-      <c r="G75">
-        <v>19351.2255529412</v>
-      </c>
-      <c r="H75">
-        <v>6002.0469674603501</v>
-      </c>
-      <c r="I75">
-        <v>2645.4376652921501</v>
-      </c>
-      <c r="J75">
-        <v>27998.710185693701</v>
-      </c>
-      <c r="K75">
-        <v>51033.4442867088</v>
-      </c>
-      <c r="L75">
-        <v>15815.1228903871</v>
-      </c>
-      <c r="M75">
-        <v>19337.009497714302</v>
-      </c>
-      <c r="N75">
-        <v>1014.17312250211</v>
-      </c>
-      <c r="O75">
-        <v>0</v>
-      </c>
-      <c r="P75">
-        <v>235736.26938738499</v>
-      </c>
-      <c r="Q75">
-        <v>1336.98290493166</v>
-      </c>
-      <c r="R75">
-        <v>18577.307877855899</v>
-      </c>
-      <c r="S75">
-        <v>432.030415764091</v>
-      </c>
-      <c r="T75" s="6">
-        <v>-0.122490141098651</v>
       </c>
     </row>
     <row r="76" spans="1:20" x14ac:dyDescent="0.35">
@@ -4059,40 +3960,40 @@
         <v>20</v>
       </c>
       <c r="B76">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C76">
         <v>2</v>
       </c>
       <c r="D76">
-        <v>113440.79599059001</v>
+        <v>118381.960809661</v>
       </c>
       <c r="E76">
-        <v>282179.67123267101</v>
+        <v>282254.81855225202</v>
       </c>
       <c r="F76">
-        <v>0.83277713625127903</v>
+        <v>0.85006146065890897</v>
       </c>
       <c r="G76">
-        <v>19390.977969205</v>
+        <v>19407.840072768398</v>
       </c>
       <c r="H76">
-        <v>5599.5405456203798</v>
+        <v>5891.8301217549197</v>
       </c>
       <c r="I76">
-        <v>2128.1287863747102</v>
+        <v>6659.4942697455399</v>
       </c>
       <c r="J76">
-        <v>27118.647301200101</v>
+        <v>31959.164464268899</v>
       </c>
       <c r="K76">
-        <v>51068.507704320902</v>
+        <v>51102.045942938203</v>
       </c>
       <c r="L76">
-        <v>15909.3558282099</v>
+        <v>15967.176494174801</v>
       </c>
       <c r="M76">
-        <v>19344.285156859401</v>
+        <v>19353.573908279199</v>
       </c>
       <c r="N76">
         <v>1010.46273302954</v>
@@ -4101,19 +4002,19 @@
         <v>0</v>
       </c>
       <c r="P76">
-        <v>234992.778517472</v>
+        <v>239933.943336542</v>
       </c>
       <c r="Q76">
-        <v>1247.3228025527501</v>
+        <v>1312.43161993582</v>
       </c>
       <c r="R76">
-        <v>16417.502561416801</v>
+        <v>18377.616631847999</v>
       </c>
       <c r="S76">
-        <v>469.07150175476602</v>
+        <v>459.4404157962</v>
       </c>
       <c r="T76" s="6">
-        <v>0.46004655114715598</v>
+        <v>0.14758705239613301</v>
       </c>
     </row>
     <row r="77" spans="1:20" x14ac:dyDescent="0.35">
@@ -4121,60 +4022,308 @@
         <v>20</v>
       </c>
       <c r="B77">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C77">
         <v>2</v>
       </c>
       <c r="D77">
+        <v>116766.56672038</v>
+      </c>
+      <c r="E77">
+        <v>282179.67123287299</v>
+      </c>
+      <c r="F77">
+        <v>0.84456314023622803</v>
+      </c>
+      <c r="G77">
+        <v>19298.245593088301</v>
+      </c>
+      <c r="H77">
+        <v>5682.0016560700296</v>
+      </c>
+      <c r="I77">
+        <v>5350.3346939491703</v>
+      </c>
+      <c r="J77">
+        <v>30330.5819431075</v>
+      </c>
+      <c r="K77">
+        <v>51097.733915068202</v>
+      </c>
+      <c r="L77">
+        <v>15987.901266609</v>
+      </c>
+      <c r="M77">
+        <v>19350.349595595701</v>
+      </c>
+      <c r="N77">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O77">
+        <v>0</v>
+      </c>
+      <c r="P77">
+        <v>238318.54924726201</v>
+      </c>
+      <c r="Q77">
+        <v>1265.6913868611</v>
+      </c>
+      <c r="R77">
+        <v>17746.163883660702</v>
+      </c>
+      <c r="S77">
+        <v>507.03325381887902</v>
+      </c>
+      <c r="T77" s="6">
+        <v>-0.25983751983286502</v>
+      </c>
+    </row>
+    <row r="78" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A78">
+        <v>20</v>
+      </c>
+      <c r="B78">
+        <v>30</v>
+      </c>
+      <c r="C78">
+        <v>2</v>
+      </c>
+      <c r="D78">
+        <v>115610.996393592</v>
+      </c>
+      <c r="E78">
+        <v>282182.50548365602</v>
+      </c>
+      <c r="F78">
+        <v>0.84045954058697003</v>
+      </c>
+      <c r="G78">
+        <v>19302.752565837702</v>
+      </c>
+      <c r="H78">
+        <v>6226.5181629292701</v>
+      </c>
+      <c r="I78">
+        <v>3974.5318253822402</v>
+      </c>
+      <c r="J78">
+        <v>29503.802554149199</v>
+      </c>
+      <c r="K78">
+        <v>51013.610661725899</v>
+      </c>
+      <c r="L78">
+        <v>15760.601295416</v>
+      </c>
+      <c r="M78">
+        <v>19332.981882301501</v>
+      </c>
+      <c r="N78">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O78">
+        <v>0</v>
+      </c>
+      <c r="P78">
+        <v>237162.97892047401</v>
+      </c>
+      <c r="Q78">
+        <v>1386.9848841974899</v>
+      </c>
+      <c r="R78">
+        <v>18436.445202769701</v>
+      </c>
+      <c r="S78">
+        <v>209.50505912238299</v>
+      </c>
+      <c r="T78" s="6">
+        <v>0.28049716262959101</v>
+      </c>
+    </row>
+    <row r="79" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A79" s="3">
+        <v>20</v>
+      </c>
+      <c r="B79" s="3">
+        <v>20</v>
+      </c>
+      <c r="C79" s="3">
+        <v>2</v>
+      </c>
+      <c r="D79">
+        <v>114184.286860504</v>
+      </c>
+      <c r="E79">
+        <v>282179.67123297497</v>
+      </c>
+      <c r="F79">
+        <v>0.83541194997266699</v>
+      </c>
+      <c r="G79">
+        <v>19351.2255529412</v>
+      </c>
+      <c r="H79">
+        <v>6002.0469674603501</v>
+      </c>
+      <c r="I79">
+        <v>2645.4376652921501</v>
+      </c>
+      <c r="J79">
+        <v>27998.710185693701</v>
+      </c>
+      <c r="K79">
+        <v>51033.4442867088</v>
+      </c>
+      <c r="L79">
+        <v>15815.1228903871</v>
+      </c>
+      <c r="M79">
+        <v>19337.009497714302</v>
+      </c>
+      <c r="N79">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O79">
+        <v>0</v>
+      </c>
+      <c r="P79">
+        <v>235736.26938738499</v>
+      </c>
+      <c r="Q79">
+        <v>1336.98290493166</v>
+      </c>
+      <c r="R79">
+        <v>18577.307877855899</v>
+      </c>
+      <c r="S79">
+        <v>432.030415764091</v>
+      </c>
+      <c r="T79" s="6">
+        <v>-0.122490141098651</v>
+      </c>
+    </row>
+    <row r="80" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A80">
+        <v>20</v>
+      </c>
+      <c r="B80">
+        <v>15</v>
+      </c>
+      <c r="C80">
+        <v>2</v>
+      </c>
+      <c r="D80">
+        <v>113440.79599059001</v>
+      </c>
+      <c r="E80">
+        <v>282179.67123267101</v>
+      </c>
+      <c r="F80">
+        <v>0.83277713625127903</v>
+      </c>
+      <c r="G80">
+        <v>19390.977969205</v>
+      </c>
+      <c r="H80">
+        <v>5599.5405456203798</v>
+      </c>
+      <c r="I80">
+        <v>2128.1287863747102</v>
+      </c>
+      <c r="J80">
+        <v>27118.647301200101</v>
+      </c>
+      <c r="K80">
+        <v>51068.507704320902</v>
+      </c>
+      <c r="L80">
+        <v>15909.3558282099</v>
+      </c>
+      <c r="M80">
+        <v>19344.285156859401</v>
+      </c>
+      <c r="N80">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O80">
+        <v>0</v>
+      </c>
+      <c r="P80">
+        <v>234992.778517472</v>
+      </c>
+      <c r="Q80">
+        <v>1247.3228025527501</v>
+      </c>
+      <c r="R80">
+        <v>16417.502561416801</v>
+      </c>
+      <c r="S80">
+        <v>469.07150175476602</v>
+      </c>
+      <c r="T80" s="6">
+        <v>0.46004655114715598</v>
+      </c>
+    </row>
+    <row r="81" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A81">
+        <v>20</v>
+      </c>
+      <c r="B81">
+        <v>12</v>
+      </c>
+      <c r="C81">
+        <v>2</v>
+      </c>
+      <c r="D81">
         <v>113795.448700252</v>
       </c>
-      <c r="E77">
+      <c r="E81">
         <v>282179.67123287602</v>
       </c>
-      <c r="F77">
+      <c r="F81">
         <v>0.83403396920434802</v>
       </c>
-      <c r="G77">
+      <c r="G81">
         <v>20436.472361711199</v>
       </c>
-      <c r="H77">
+      <c r="H81">
         <v>4946.5396722567002</v>
       </c>
-      <c r="I77">
+      <c r="I81">
         <v>2967.9237851293901</v>
       </c>
-      <c r="J77">
+      <c r="J81">
         <v>28350.9358190973</v>
       </c>
-      <c r="K77">
+      <c r="K81">
         <v>50843.184005923598</v>
       </c>
-      <c r="L77">
+      <c r="L81">
         <v>15303.798385783</v>
       </c>
-      <c r="M77">
+      <c r="M81">
         <v>19297.530489448302</v>
       </c>
-      <c r="N77">
+      <c r="N81">
         <v>992.31070788530405</v>
       </c>
-      <c r="O77">
-        <v>0</v>
-      </c>
-      <c r="P77">
+      <c r="O81">
+        <v>0</v>
+      </c>
+      <c r="P81">
         <v>235347.43122713399</v>
       </c>
-      <c r="Q77">
+      <c r="Q81">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R77">
+      <c r="R81">
         <v>13.380488321454299</v>
       </c>
-      <c r="S77">
+      <c r="S81">
         <v>2.67609766429086</v>
       </c>
-      <c r="T77" s="6">
+      <c r="T81" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update to find basline with new num_flex_trains constraint
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A7A9567-2B89-4C2B-B980-28520FD85CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{830F13C9-BBB4-42FC-9D89-F410E2378D29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10170" yWindow="0" windowWidth="9120" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -117,7 +117,7 @@
     This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</t>
       </text>
     </comment>
-    <comment ref="A42" authorId="8" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A41" authorId="8" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -125,7 +125,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="A43" authorId="9" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A42" authorId="9" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -133,7 +133,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T43" authorId="10" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T42" authorId="10" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -143,7 +143,7 @@
     The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A49" authorId="11" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A48" authorId="11" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -151,7 +151,7 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="A66" authorId="12" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A65" authorId="12" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -159,7 +159,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T78" authorId="13" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T77" authorId="13" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -172,7 +172,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="41">
   <si>
     <t>Season</t>
   </si>
@@ -295,9 +295,6 @@
   </si>
   <si>
     <t>Charge Power Capacity</t>
-  </si>
-  <si>
-    <t>no flex</t>
   </si>
 </sst>
 </file>
@@ -1225,25 +1222,25 @@
   <threadedComment ref="A28" dT="2026-07-15T17:22:40.80" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
     <text>This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</text>
   </threadedComment>
-  <threadedComment ref="A42" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+  <threadedComment ref="A41" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
-  <threadedComment ref="A43" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+  <threadedComment ref="A42" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
     <text>Summer week = hot summer weekdays + high weekends</text>
   </threadedComment>
-  <threadedComment ref="T43" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T42" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure</text>
   </threadedComment>
-  <threadedComment ref="T43" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T42" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>The baseline costs have to be updated in accordance with the demand structure type</text>
   </threadedComment>
-  <threadedComment ref="A49" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+  <threadedComment ref="A48" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
     <text>Result from the fast solve</text>
   </threadedComment>
-  <threadedComment ref="A66" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+  <threadedComment ref="A65" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
     <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
   </threadedComment>
-  <threadedComment ref="T78" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="T77" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1251,7 +1248,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:V81"/>
+  <dimension ref="A1:V80"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.6328125" customWidth="1"/>
@@ -2575,35 +2572,202 @@
       <c r="S33" s="2"/>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" s="7"/>
-      <c r="B34" s="2"/>
-      <c r="S34" s="2"/>
+      <c r="A34" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+      <c r="D34">
+        <v>153412.243053051</v>
+      </c>
+      <c r="E34">
+        <v>374203.2</v>
+      </c>
+      <c r="F34">
+        <v>0.73479923629710397</v>
+      </c>
+      <c r="G34">
+        <v>28189.163715008799</v>
+      </c>
+      <c r="H34">
+        <v>8631.5718994758809</v>
+      </c>
+      <c r="I34">
+        <v>3282.10418908369</v>
+      </c>
+      <c r="J34">
+        <v>40102.8398035684</v>
+      </c>
+      <c r="K34">
+        <v>67424.000035550795</v>
+      </c>
+      <c r="L34">
+        <v>20294.624006555201</v>
+      </c>
+      <c r="M34">
+        <v>25590.779207376701</v>
+      </c>
+      <c r="N34">
+        <v>1409.83742959549</v>
+      </c>
+      <c r="O34">
+        <v>0</v>
+      </c>
+      <c r="P34">
+        <v>274964.22557993297</v>
+      </c>
+      <c r="Q34">
+        <v>1466.6067163636201</v>
+      </c>
+      <c r="R34">
+        <v>0</v>
+      </c>
+      <c r="U34">
+        <v>61253.928349088899</v>
+      </c>
+      <c r="V34">
+        <v>364.606716363624</v>
+      </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" s="7"/>
-      <c r="B35" s="2"/>
-      <c r="S35" s="2"/>
+      <c r="A35" t="s">
+        <v>22</v>
+      </c>
+      <c r="B35" t="s">
+        <v>23</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>165265.875469322</v>
+      </c>
+      <c r="E35">
+        <v>374203.2</v>
+      </c>
+      <c r="F35">
+        <v>0.76647623001674903</v>
+      </c>
+      <c r="G35">
+        <v>30792.331969512299</v>
+      </c>
+      <c r="H35">
+        <v>8631.5718986985103</v>
+      </c>
+      <c r="I35">
+        <v>12532.568351771601</v>
+      </c>
+      <c r="J35">
+        <v>51956.472219982403</v>
+      </c>
+      <c r="K35">
+        <v>67424.000035514298</v>
+      </c>
+      <c r="L35">
+        <v>20294.624006456401</v>
+      </c>
+      <c r="M35">
+        <v>25590.7792073692</v>
+      </c>
+      <c r="N35">
+        <v>1409.83742959549</v>
+      </c>
+      <c r="O35">
+        <v>0</v>
+      </c>
+      <c r="P35">
+        <v>286817.85799620399</v>
+      </c>
+      <c r="Q35">
+        <v>1466.6067162315301</v>
+      </c>
+      <c r="R35">
+        <v>0</v>
+      </c>
+      <c r="U35">
+        <v>61253.928326898502</v>
+      </c>
+      <c r="V35">
+        <v>364.606716231539</v>
+      </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C36">
-        <v>0</v>
-      </c>
+      <c r="A36" s="7"/>
+      <c r="B36" s="2"/>
       <c r="S36" s="2"/>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="7"/>
-      <c r="B37" s="2"/>
-      <c r="S37" s="2"/>
+      <c r="A37" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B37" t="s">
+        <v>21</v>
+      </c>
+      <c r="C37">
+        <v>4</v>
+      </c>
+      <c r="D37">
+        <v>115568.67725355701</v>
+      </c>
+      <c r="E37">
+        <v>282179.671254922</v>
+      </c>
+      <c r="F37">
+        <v>0.84031800989031202</v>
+      </c>
+      <c r="G37">
+        <v>21174.931050348201</v>
+      </c>
+      <c r="H37">
+        <v>6483.8014286718599</v>
+      </c>
+      <c r="I37">
+        <v>2465.4271592782502</v>
+      </c>
+      <c r="J37">
+        <v>30124.159638298399</v>
+      </c>
+      <c r="K37">
+        <v>50843.185222512198</v>
+      </c>
+      <c r="L37">
+        <v>15303.8016501727</v>
+      </c>
+      <c r="M37">
+        <v>19297.530742573799</v>
+      </c>
+      <c r="N37">
+        <v>1409.83742959549</v>
+      </c>
+      <c r="O37">
+        <v>0</v>
+      </c>
+      <c r="P37">
+        <v>237120.659780438</v>
+      </c>
+      <c r="Q37">
+        <v>1101.67497109485</v>
+      </c>
+      <c r="R37">
+        <v>54.604983409531002</v>
+      </c>
+      <c r="S37">
+        <v>0.32502966315197002</v>
+      </c>
+      <c r="T37">
+        <v>-106.83117764915301</v>
+      </c>
+      <c r="U37">
+        <v>0</v>
+      </c>
     </row>
     <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B38" t="s">
         <v>21</v>
@@ -2612,137 +2776,134 @@
         <v>4</v>
       </c>
       <c r="D38">
-        <v>115568.67725355701</v>
+        <v>120779.539344445</v>
       </c>
       <c r="E38">
-        <v>282179.671254922</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F38">
-        <v>0.84031800989031202</v>
+        <v>0.858784478742043</v>
       </c>
       <c r="G38">
-        <v>21174.931050348201</v>
+        <v>22232.9956437156</v>
       </c>
       <c r="H38">
-        <v>6483.8014286718599</v>
+        <v>6892.28291987389</v>
       </c>
       <c r="I38">
-        <v>2465.4271592782502</v>
+        <v>5063.3926573547897</v>
       </c>
       <c r="J38">
-        <v>30124.159638298399</v>
+        <v>34188.671220944299</v>
       </c>
       <c r="K38">
-        <v>50843.185222512198</v>
+        <v>51137.498573919998</v>
       </c>
       <c r="L38">
-        <v>15303.8016501727</v>
+        <v>16094.7687872735</v>
       </c>
       <c r="M38">
-        <v>19297.530742573799</v>
+        <v>19358.6007623076</v>
       </c>
       <c r="N38">
-        <v>1409.83742959549</v>
+        <v>1430.39398992981</v>
       </c>
       <c r="O38">
         <v>0</v>
       </c>
       <c r="P38">
-        <v>237120.659780438</v>
+        <v>242331.52187132699</v>
       </c>
       <c r="Q38">
-        <v>1101.67497109485</v>
+        <v>1171.0808202107701</v>
       </c>
       <c r="R38">
-        <v>54.604983409531002</v>
+        <v>13170.183258303599</v>
       </c>
       <c r="S38">
-        <v>0.32502966315197002</v>
+        <v>487.784565122358</v>
       </c>
       <c r="T38">
-        <v>-106.83117764915301</v>
+        <v>-0.16035717141929801</v>
       </c>
       <c r="U38">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A39" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B39" t="s">
-        <v>21</v>
-      </c>
-      <c r="C39">
-        <v>4</v>
-      </c>
-      <c r="D39">
-        <v>120779.539344445</v>
-      </c>
-      <c r="E39">
+        <v>9733.9102750884304</v>
+      </c>
+      <c r="V38">
+        <v>69.034824646017199</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A40" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G40" s="4"/>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A41" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C41">
+        <v>0</v>
+      </c>
+      <c r="D41">
+        <v>116861.67991782499</v>
+      </c>
+      <c r="E41">
         <v>282179.67123287602</v>
       </c>
-      <c r="F39">
-        <v>0.858784478742043</v>
-      </c>
-      <c r="G39">
-        <v>22232.9956437156</v>
-      </c>
-      <c r="H39">
-        <v>6892.28291987389</v>
-      </c>
-      <c r="I39">
-        <v>5063.3926573547897</v>
-      </c>
-      <c r="J39">
-        <v>34188.671220944299</v>
-      </c>
-      <c r="K39">
-        <v>51137.498573919998</v>
-      </c>
-      <c r="L39">
-        <v>16094.7687872735</v>
-      </c>
-      <c r="M39">
-        <v>19358.6007623076</v>
-      </c>
-      <c r="N39">
-        <v>1430.39398992981</v>
-      </c>
-      <c r="O39">
-        <v>0</v>
-      </c>
-      <c r="P39">
-        <v>242331.52187132699</v>
-      </c>
-      <c r="Q39">
-        <v>1171.0808202107701</v>
-      </c>
-      <c r="R39">
-        <v>13170.183258303599</v>
-      </c>
-      <c r="S39">
-        <v>487.784565122358</v>
-      </c>
-      <c r="T39">
-        <v>-0.16035717141929801</v>
-      </c>
-      <c r="U39">
-        <v>9733.9102750884304</v>
-      </c>
-      <c r="V39">
-        <v>69.034824646017199</v>
-      </c>
-    </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A41" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="G41" s="4"/>
+      <c r="F41">
+        <v>0.84490020632262297</v>
+      </c>
+      <c r="G41">
+        <v>23556.420831705898</v>
+      </c>
+      <c r="H41">
+        <v>6947.4542183048998</v>
+      </c>
+      <c r="I41">
+        <v>913.29198665996</v>
+      </c>
+      <c r="J41">
+        <v>31417.167036670799</v>
+      </c>
+      <c r="K41">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L41">
+        <v>15303.798385783</v>
+      </c>
+      <c r="M41">
+        <v>19297.5304894482</v>
+      </c>
+      <c r="N41">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O41">
+        <v>0</v>
+      </c>
+      <c r="P41">
+        <v>238413.66244470701</v>
+      </c>
+      <c r="Q41">
+        <v>1102.6552392369899</v>
+      </c>
+      <c r="R41">
+        <v>0</v>
+      </c>
+      <c r="S41">
+        <v>0</v>
+      </c>
+      <c r="T41">
+        <v>0</v>
+      </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>23</v>
@@ -2751,25 +2912,25 @@
         <v>0</v>
       </c>
       <c r="D42">
-        <v>116861.67991782499</v>
+        <v>187020.456722612</v>
       </c>
       <c r="E42">
         <v>282179.67123287602</v>
       </c>
       <c r="F42">
-        <v>0.84490020632262297</v>
+        <v>1.09353178385</v>
       </c>
       <c r="G42">
-        <v>23556.420831705898</v>
+        <v>89520.694507565597</v>
       </c>
       <c r="H42">
-        <v>6947.4542183048998</v>
+        <v>6971.3813103080802</v>
       </c>
       <c r="I42">
-        <v>913.29198665996</v>
+        <v>5083.8680235841202</v>
       </c>
       <c r="J42">
-        <v>31417.167036670799</v>
+        <v>101575.943841457</v>
       </c>
       <c r="K42">
         <v>50843.184005923598</v>
@@ -2787,90 +2948,90 @@
         <v>0</v>
       </c>
       <c r="P42">
-        <v>238413.66244470701</v>
+        <v>308572.439249494</v>
       </c>
       <c r="Q42">
-        <v>1102.6552392369899</v>
+        <v>1106.4527933521999</v>
       </c>
       <c r="R42">
-        <v>0</v>
+        <v>3451.9307168288801</v>
       </c>
       <c r="S42">
-        <v>0</v>
+        <v>20.547206647791</v>
       </c>
       <c r="T42">
-        <v>0</v>
+        <v>-14.696886263168601</v>
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C43">
-        <v>0</v>
-      </c>
-      <c r="D43">
-        <v>187020.456722612</v>
-      </c>
-      <c r="E43">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F43">
-        <v>1.09353178385</v>
-      </c>
-      <c r="G43">
-        <v>89520.694507565597</v>
-      </c>
-      <c r="H43">
-        <v>6971.3813103080802</v>
-      </c>
-      <c r="I43">
-        <v>5083.8680235841202</v>
-      </c>
-      <c r="J43">
-        <v>101575.943841457</v>
-      </c>
-      <c r="K43">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L43">
-        <v>15303.798385783</v>
-      </c>
-      <c r="M43">
-        <v>19297.5304894482</v>
-      </c>
-      <c r="N43">
+      <c r="A43" s="3"/>
+      <c r="G43" s="4"/>
+    </row>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>20</v>
+      </c>
+      <c r="B44" t="s">
+        <v>21</v>
+      </c>
+      <c r="C44">
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <v>117032.41959359701</v>
+      </c>
+      <c r="E44">
+        <v>282179.67123286898</v>
+      </c>
+      <c r="F44">
+        <v>0.845505280653571</v>
+      </c>
+      <c r="G44" s="4">
+        <v>23683.129427060001</v>
+      </c>
+      <c r="H44">
+        <v>6986.3695969997798</v>
+      </c>
+      <c r="I44">
+        <v>918.40768838365295</v>
+      </c>
+      <c r="J44">
+        <v>31587.906712443499</v>
+      </c>
+      <c r="K44">
+        <v>50843.1840059237</v>
+      </c>
+      <c r="L44">
+        <v>15303.7983857823</v>
+      </c>
+      <c r="M44">
+        <v>19297.530489448101</v>
+      </c>
+      <c r="N44">
         <v>992.31070788530405</v>
       </c>
-      <c r="O43">
-        <v>0</v>
-      </c>
-      <c r="P43">
-        <v>308572.439249494</v>
-      </c>
-      <c r="Q43">
-        <v>1106.4527933521999</v>
-      </c>
-      <c r="R43">
-        <v>3451.9307168288801</v>
-      </c>
-      <c r="S43">
-        <v>20.547206647791</v>
-      </c>
-      <c r="T43">
-        <v>-14.696886263168601</v>
-      </c>
-    </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="3"/>
-      <c r="G44" s="4"/>
+      <c r="O44">
+        <v>0</v>
+      </c>
+      <c r="P44">
+        <v>238584.402120479</v>
+      </c>
+      <c r="Q44">
+        <v>1108.83163779344</v>
+      </c>
+      <c r="R44">
+        <v>0</v>
+      </c>
+      <c r="S44">
+        <v>230512.59606633501</v>
+      </c>
+      <c r="T44">
+        <v>1103.3673370121001</v>
+      </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B45" t="s">
         <v>21</v>
@@ -2879,34 +3040,34 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>117032.41959359701</v>
+        <v>171564.02128394699</v>
       </c>
       <c r="E45">
-        <v>282179.67123286898</v>
+        <v>282179.67123287701</v>
       </c>
       <c r="F45">
-        <v>0.845505280653571</v>
-      </c>
-      <c r="G45" s="4">
-        <v>23683.129427060001</v>
+        <v>1.03875662810921</v>
+      </c>
+      <c r="G45">
+        <v>73514.1870928641</v>
       </c>
       <c r="H45">
-        <v>6986.3695969997798</v>
+        <v>7482.8438362204697</v>
       </c>
       <c r="I45">
-        <v>918.40768838365295</v>
+        <v>4044.9309872213798</v>
       </c>
       <c r="J45">
-        <v>31587.906712443499</v>
+        <v>85041.961916305998</v>
       </c>
       <c r="K45">
-        <v>50843.1840059237</v>
+        <v>51119.832654572398</v>
       </c>
       <c r="L45">
-        <v>15303.7983857823</v>
+        <v>16047.2916290263</v>
       </c>
       <c r="M45">
-        <v>19297.530489448101</v>
+        <v>19354.9350840429</v>
       </c>
       <c r="N45">
         <v>992.31070788530405</v>
@@ -2915,89 +3076,89 @@
         <v>0</v>
       </c>
       <c r="P45">
-        <v>238584.402120479</v>
+        <v>293116.00381082902</v>
       </c>
       <c r="Q45">
-        <v>1108.83163779344</v>
+        <v>1187.62883512946</v>
       </c>
       <c r="R45">
-        <v>0</v>
+        <v>9393.8913494494009</v>
       </c>
       <c r="S45">
-        <v>230512.59606633501</v>
+        <v>260.94142637359403</v>
       </c>
       <c r="T45">
-        <v>1103.3673370121001</v>
+        <v>-3.6405201993767098</v>
       </c>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+      <c r="G46" s="4"/>
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A47" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B47" t="s">
+        <v>21</v>
+      </c>
+      <c r="C47">
+        <v>4</v>
+      </c>
+      <c r="D47">
+        <v>116833.749486644</v>
+      </c>
+      <c r="E47">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F47">
+        <v>0.84480122530439805</v>
+      </c>
+      <c r="G47" s="4">
+        <v>23535.478746437901</v>
+      </c>
+      <c r="H47">
+        <v>6941.2778055266899</v>
+      </c>
+      <c r="I47">
+        <v>912.48005352310201</v>
+      </c>
+      <c r="J47">
+        <v>31389.236605487698</v>
+      </c>
+      <c r="K47">
+        <v>50843.184005923998</v>
+      </c>
+      <c r="L47">
+        <v>15303.798385784499</v>
+      </c>
+      <c r="M47">
+        <v>19297.5304894484</v>
+      </c>
+      <c r="N47">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O47">
+        <v>0</v>
+      </c>
+      <c r="P47">
+        <v>0</v>
+      </c>
+      <c r="Q47">
+        <v>0</v>
+      </c>
+      <c r="R47">
+        <v>0</v>
+      </c>
+      <c r="S47">
+        <v>0</v>
+      </c>
+      <c r="T47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
         <v>22</v>
-      </c>
-      <c r="B46" t="s">
-        <v>21</v>
-      </c>
-      <c r="C46">
-        <v>0</v>
-      </c>
-      <c r="D46">
-        <v>171564.02128394699</v>
-      </c>
-      <c r="E46">
-        <v>282179.67123287701</v>
-      </c>
-      <c r="F46">
-        <v>1.03875662810921</v>
-      </c>
-      <c r="G46">
-        <v>73514.1870928641</v>
-      </c>
-      <c r="H46">
-        <v>7482.8438362204697</v>
-      </c>
-      <c r="I46">
-        <v>4044.9309872213798</v>
-      </c>
-      <c r="J46">
-        <v>85041.961916305998</v>
-      </c>
-      <c r="K46">
-        <v>51119.832654572398</v>
-      </c>
-      <c r="L46">
-        <v>16047.2916290263</v>
-      </c>
-      <c r="M46">
-        <v>19354.9350840429</v>
-      </c>
-      <c r="N46">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O46">
-        <v>0</v>
-      </c>
-      <c r="P46">
-        <v>293116.00381082902</v>
-      </c>
-      <c r="Q46">
-        <v>1187.62883512946</v>
-      </c>
-      <c r="R46">
-        <v>9393.8913494494009</v>
-      </c>
-      <c r="S46">
-        <v>260.94142637359403</v>
-      </c>
-      <c r="T46">
-        <v>-3.6405201993767098</v>
-      </c>
-    </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="G47" s="4"/>
-    </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="3" t="s">
-        <v>20</v>
       </c>
       <c r="B48" t="s">
         <v>21</v>
@@ -3006,124 +3167,124 @@
         <v>4</v>
       </c>
       <c r="D48">
-        <v>116833.749486644</v>
+        <v>124393.533174422</v>
       </c>
       <c r="E48">
-        <v>282179.67123287602</v>
+        <v>282179.67123444699</v>
       </c>
       <c r="F48">
-        <v>0.84480122530439805</v>
+        <v>0.87159189967643702</v>
       </c>
       <c r="G48" s="4">
-        <v>23535.478746437901</v>
+        <v>21072.189860718699</v>
       </c>
       <c r="H48">
-        <v>6941.2778055266899</v>
+        <v>9188.7245080883695</v>
       </c>
       <c r="I48">
-        <v>912.48005352310201</v>
+        <v>2618.8827210474601</v>
       </c>
       <c r="J48">
-        <v>31389.236605487698</v>
+        <v>32879.797089854597</v>
       </c>
       <c r="K48">
-        <v>50843.184005923998</v>
+        <v>50904.118537438801</v>
       </c>
       <c r="L48">
-        <v>15303.798385784499</v>
+        <v>20591.7266090095</v>
       </c>
       <c r="M48">
-        <v>19297.5304894484</v>
+        <v>20017.890938119701</v>
       </c>
       <c r="N48">
-        <v>992.31070788530405</v>
+        <v>1040.9289460857101</v>
       </c>
       <c r="O48">
         <v>0</v>
       </c>
       <c r="P48">
-        <v>0</v>
+        <v>245945.51570130399</v>
       </c>
       <c r="Q48">
-        <v>0</v>
+        <v>1458.3752411216699</v>
       </c>
       <c r="R48">
-        <v>0</v>
+        <v>35012.612233571497</v>
       </c>
       <c r="S48">
-        <v>0</v>
+        <v>875.31530583928895</v>
       </c>
       <c r="T48">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+        <v>0.51444695802960605</v>
+      </c>
+    </row>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A50" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G50" s="4"/>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>22</v>
       </c>
-      <c r="B49" t="s">
-        <v>21</v>
-      </c>
-      <c r="C49">
-        <v>4</v>
-      </c>
-      <c r="D49">
-        <v>124393.533174422</v>
-      </c>
-      <c r="E49">
-        <v>282179.67123444699</v>
-      </c>
-      <c r="F49">
-        <v>0.87159189967643702</v>
-      </c>
-      <c r="G49" s="4">
-        <v>21072.189860718699</v>
-      </c>
-      <c r="H49">
-        <v>9188.7245080883695</v>
-      </c>
-      <c r="I49">
-        <v>2618.8827210474601</v>
-      </c>
-      <c r="J49">
-        <v>32879.797089854597</v>
-      </c>
-      <c r="K49">
-        <v>50904.118537438801</v>
-      </c>
-      <c r="L49">
-        <v>20591.7266090095</v>
-      </c>
-      <c r="M49">
-        <v>20017.890938119701</v>
-      </c>
-      <c r="N49">
-        <v>1040.9289460857101</v>
-      </c>
-      <c r="O49">
-        <v>0</v>
-      </c>
-      <c r="P49">
-        <v>245945.51570130399</v>
-      </c>
-      <c r="Q49">
-        <v>1458.3752411216699</v>
-      </c>
-      <c r="R49">
-        <v>35012.612233571497</v>
-      </c>
-      <c r="S49">
-        <v>875.31530583928895</v>
-      </c>
-      <c r="T49">
-        <v>0.51444695802960605</v>
-      </c>
-    </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A51" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G51" s="4"/>
+      <c r="B51" t="s">
+        <v>25</v>
+      </c>
+      <c r="C51">
+        <v>2</v>
+      </c>
+      <c r="D51">
+        <v>115472.147206908</v>
+      </c>
+      <c r="E51">
+        <v>282495</v>
+      </c>
+      <c r="F51">
+        <v>0.83903831831993503</v>
+      </c>
+      <c r="G51" s="4">
+        <v>20221.889710343999</v>
+      </c>
+      <c r="H51">
+        <v>6553.7440767980397</v>
+      </c>
+      <c r="I51">
+        <v>6160.4249909476703</v>
+      </c>
+      <c r="J51">
+        <v>32936.058778089697</v>
+      </c>
+      <c r="K51">
+        <v>50939.5611113743</v>
+      </c>
+      <c r="L51">
+        <v>15427.2204868183</v>
+      </c>
+      <c r="M51">
+        <v>19327.3039306102</v>
+      </c>
+      <c r="N51">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O51">
+        <v>3157.9970999842499</v>
+      </c>
+      <c r="P51">
+        <v>237024.12973379</v>
+      </c>
+      <c r="Q51">
+        <v>1464.2687322859999</v>
+      </c>
+      <c r="R51">
+        <v>8672.9882445954008</v>
+      </c>
+      <c r="S51">
+        <v>346.91952978381602</v>
+      </c>
+      <c r="T51">
+        <v>2.4302910949698302</v>
+      </c>
     </row>
     <row r="52" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
@@ -3133,130 +3294,130 @@
         <v>25</v>
       </c>
       <c r="C52">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D52">
-        <v>115472.147206908</v>
+        <v>108958.027502652</v>
       </c>
       <c r="E52">
-        <v>282495</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F52">
-        <v>0.83903831831993503</v>
+        <v>0.81689091571482797</v>
       </c>
       <c r="G52" s="4">
-        <v>20221.889710343999</v>
+        <v>20285.098342207999</v>
       </c>
       <c r="H52">
-        <v>6553.7440767980397</v>
+        <v>6552.6722224723899</v>
       </c>
       <c r="I52">
-        <v>6160.4249909476703</v>
+        <v>6068.9240568166097</v>
       </c>
       <c r="J52">
-        <v>32936.058778089697</v>
+        <v>32906.694621497001</v>
       </c>
       <c r="K52">
-        <v>50939.5611113743</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L52">
-        <v>15427.2204868183</v>
+        <v>16378.7983857829</v>
       </c>
       <c r="M52">
-        <v>19327.3039306102</v>
+        <v>19449.350489448301</v>
       </c>
       <c r="N52">
         <v>1004.9477757237401</v>
       </c>
       <c r="O52">
-        <v>3157.9970999842499</v>
+        <v>10620</v>
       </c>
       <c r="P52">
-        <v>237024.12973379</v>
+        <v>230510.010029533</v>
       </c>
       <c r="Q52">
-        <v>1464.2687322859999</v>
+        <v>1464.02925348484</v>
       </c>
       <c r="R52">
-        <v>8672.9882445954008</v>
+        <v>26064.489084194902</v>
       </c>
       <c r="S52">
-        <v>346.91952978381602</v>
+        <v>407.257641940545</v>
       </c>
       <c r="T52">
-        <v>2.4302910949698302</v>
-      </c>
-    </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>22</v>
-      </c>
-      <c r="B53" t="s">
-        <v>25</v>
-      </c>
-      <c r="C53">
-        <v>4</v>
-      </c>
-      <c r="D53">
-        <v>108958.027502652</v>
-      </c>
-      <c r="E53">
+        <v>1.09609872121186</v>
+      </c>
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A54" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A55" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C55">
+        <v>0</v>
+      </c>
+      <c r="D55">
+        <v>115030.978322179</v>
+      </c>
+      <c r="E55">
         <v>282179.67123287602</v>
       </c>
-      <c r="F53">
-        <v>0.81689091571482797</v>
-      </c>
-      <c r="G53" s="4">
-        <v>20285.098342207999</v>
-      </c>
-      <c r="H53">
-        <v>6552.6722224723899</v>
-      </c>
-      <c r="I53">
-        <v>6068.9240568166097</v>
-      </c>
-      <c r="J53">
-        <v>32906.694621497001</v>
-      </c>
-      <c r="K53">
+      <c r="F55">
+        <v>0.83841249022441</v>
+      </c>
+      <c r="G55">
+        <v>20114.092712805999</v>
+      </c>
+      <c r="H55">
+        <v>6942.2846600808298</v>
+      </c>
+      <c r="I55">
+        <v>2530.0880681377598</v>
+      </c>
+      <c r="J55">
+        <v>29586.4654410246</v>
+      </c>
+      <c r="K55">
         <v>50843.184005923598</v>
       </c>
-      <c r="L53">
-        <v>16378.7983857829</v>
-      </c>
-      <c r="M53">
-        <v>19449.350489448301</v>
-      </c>
-      <c r="N53">
-        <v>1004.9477757237401</v>
-      </c>
-      <c r="O53">
-        <v>10620</v>
-      </c>
-      <c r="P53">
-        <v>230510.010029533</v>
-      </c>
-      <c r="Q53">
-        <v>1464.02925348484</v>
-      </c>
-      <c r="R53">
-        <v>26064.489084194902</v>
-      </c>
-      <c r="S53">
-        <v>407.257641940545</v>
-      </c>
-      <c r="T53">
-        <v>1.09609872121186</v>
-      </c>
-    </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A55" s="1" t="s">
-        <v>31</v>
+      <c r="L55">
+        <v>15303.798385783</v>
+      </c>
+      <c r="M55">
+        <v>19297.5304894482</v>
+      </c>
+      <c r="N55">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O55">
+        <v>0</v>
+      </c>
+      <c r="P55">
+        <v>236582.960849061</v>
+      </c>
+      <c r="Q55">
+        <v>1101.8347602124099</v>
+      </c>
+      <c r="R55">
+        <v>0</v>
+      </c>
+      <c r="S55">
+        <v>0</v>
+      </c>
+      <c r="T55">
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>23</v>
@@ -3265,34 +3426,34 @@
         <v>0</v>
       </c>
       <c r="D56">
-        <v>115030.978322179</v>
+        <v>124771.246709449</v>
       </c>
       <c r="E56">
-        <v>282179.67123287602</v>
+        <v>282179.67125180899</v>
       </c>
       <c r="F56">
-        <v>0.83841249022441</v>
+        <v>0.87293045648394496</v>
       </c>
       <c r="G56">
-        <v>20114.092712805999</v>
+        <v>22626.697961956499</v>
       </c>
       <c r="H56">
-        <v>6942.2846600808298</v>
+        <v>7102.5767129513297</v>
       </c>
       <c r="I56">
-        <v>2530.0880681377598</v>
+        <v>9597.4591384874802</v>
       </c>
       <c r="J56">
-        <v>29586.4654410246</v>
+        <v>39326.733813395302</v>
       </c>
       <c r="K56">
-        <v>50843.184005923598</v>
+        <v>50843.184011688398</v>
       </c>
       <c r="L56">
-        <v>15303.798385783</v>
+        <v>15303.798393134501</v>
       </c>
       <c r="M56">
-        <v>19297.5304894482</v>
+        <v>19297.530491231599</v>
       </c>
       <c r="N56">
         <v>992.31070788530405</v>
@@ -3301,10 +3462,10 @@
         <v>0</v>
       </c>
       <c r="P56">
-        <v>236582.960849061</v>
+        <v>246323.22923633101</v>
       </c>
       <c r="Q56">
-        <v>1101.8347602124099</v>
+        <v>1127.27501714903</v>
       </c>
       <c r="R56">
         <v>0</v>
@@ -3317,73 +3478,67 @@
       </c>
     </row>
     <row r="57" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A57" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C57">
-        <v>0</v>
-      </c>
-      <c r="D57">
-        <v>124771.246709449</v>
-      </c>
-      <c r="E57">
-        <v>282179.67125180899</v>
-      </c>
-      <c r="F57">
-        <v>0.87293045648394496</v>
-      </c>
-      <c r="G57">
-        <v>22626.697961956499</v>
-      </c>
-      <c r="H57">
-        <v>7102.5767129513297</v>
-      </c>
-      <c r="I57">
-        <v>9597.4591384874802</v>
-      </c>
-      <c r="J57">
-        <v>39326.733813395302</v>
-      </c>
-      <c r="K57">
-        <v>50843.184011688398</v>
-      </c>
-      <c r="L57">
-        <v>15303.798393134501</v>
-      </c>
-      <c r="M57">
-        <v>19297.530491231599</v>
-      </c>
-      <c r="N57">
+      <c r="A57" s="1"/>
+    </row>
+    <row r="58" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>20</v>
+      </c>
+      <c r="B58" t="s">
+        <v>21</v>
+      </c>
+      <c r="C58">
+        <v>2</v>
+      </c>
+      <c r="D58">
+        <v>115714.10508262301</v>
+      </c>
+      <c r="E58">
+        <v>282179.67125387199</v>
+      </c>
+      <c r="F58">
+        <v>0.840833383054163</v>
+      </c>
+      <c r="G58" s="4">
+        <v>20578.507216446698</v>
+      </c>
+      <c r="H58">
+        <v>7102.57515066207</v>
+      </c>
+      <c r="I58">
+        <v>2588.5052959285099</v>
+      </c>
+      <c r="J58">
+        <v>30269.587663037299</v>
+      </c>
+      <c r="K58">
+        <v>50843.185173268597</v>
+      </c>
+      <c r="L58">
+        <v>15303.8015139941</v>
+      </c>
+      <c r="M58">
+        <v>19297.530732323401</v>
+      </c>
+      <c r="N58">
         <v>992.31070788530405</v>
       </c>
-      <c r="O57">
-        <v>0</v>
-      </c>
-      <c r="P57">
-        <v>246323.22923633101</v>
-      </c>
-      <c r="Q57">
-        <v>1127.27501714903</v>
-      </c>
-      <c r="R57">
-        <v>0</v>
-      </c>
-      <c r="S57">
-        <v>0</v>
-      </c>
-      <c r="T57">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A58" s="1"/>
+      <c r="O58">
+        <v>0</v>
+      </c>
+      <c r="P58">
+        <v>237266.08760950499</v>
+      </c>
+      <c r="Q58">
+        <v>1127.2750356983099</v>
+      </c>
+      <c r="R58">
+        <v>0</v>
+      </c>
     </row>
     <row r="59" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B59" t="s">
         <v>21</v>
@@ -3392,116 +3547,116 @@
         <v>2</v>
       </c>
       <c r="D59">
-        <v>115714.10508262301</v>
+        <v>120628.41082793</v>
       </c>
       <c r="E59">
-        <v>282179.67125387199</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F59">
-        <v>0.840833383054163</v>
+        <v>0.85824890324911396</v>
       </c>
       <c r="G59" s="4">
-        <v>20578.507216446698</v>
+        <v>20824.7129679639</v>
       </c>
       <c r="H59">
-        <v>7102.57515066207</v>
+        <v>7456.39074483072</v>
       </c>
       <c r="I59">
-        <v>2588.5052959285099</v>
+        <v>5114.4587365303096</v>
       </c>
       <c r="J59">
-        <v>30269.587663037299</v>
+        <v>33395.562449324898</v>
       </c>
       <c r="K59">
-        <v>50843.185173268597</v>
+        <v>51302.320205525801</v>
       </c>
       <c r="L59">
-        <v>15303.8015139941</v>
+        <v>16537.7269222135</v>
       </c>
       <c r="M59">
-        <v>19297.530732323401</v>
+        <v>19392.801250865799</v>
       </c>
       <c r="N59">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O59">
+        <v>0</v>
+      </c>
+      <c r="P59">
+        <v>242180.39335481101</v>
+      </c>
+      <c r="Q59">
+        <v>1183.4303612998101</v>
+      </c>
+      <c r="R59">
+        <v>15931.1957490451</v>
+      </c>
+      <c r="S59">
+        <v>346.33034237054602</v>
+      </c>
+      <c r="T59">
+        <v>1.0959871186973</v>
+      </c>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>20</v>
+      </c>
+      <c r="B61" t="s">
+        <v>21</v>
+      </c>
+      <c r="C61">
+        <v>4</v>
+      </c>
+      <c r="D61">
+        <v>115714.10508261999</v>
+      </c>
+      <c r="E61">
+        <v>282179.671253876</v>
+      </c>
+      <c r="F61">
+        <v>0.84083338305413902</v>
+      </c>
+      <c r="G61" s="4">
+        <v>20578.5072164468</v>
+      </c>
+      <c r="H61">
+        <v>7102.5751506616798</v>
+      </c>
+      <c r="I61">
+        <v>2588.50529592865</v>
+      </c>
+      <c r="J61">
+        <v>30269.587663037099</v>
+      </c>
+      <c r="K61">
+        <v>50843.185173268197</v>
+      </c>
+      <c r="L61">
+        <v>15303.8015139912</v>
+      </c>
+      <c r="M61">
+        <v>19297.530732323299</v>
+      </c>
+      <c r="N61">
         <v>992.31070788530405</v>
       </c>
-      <c r="O59">
-        <v>0</v>
-      </c>
-      <c r="P59">
-        <v>237266.08760950499</v>
-      </c>
-      <c r="Q59">
-        <v>1127.2750356983099</v>
-      </c>
-      <c r="R59">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
-        <v>22</v>
-      </c>
-      <c r="B60" t="s">
-        <v>21</v>
-      </c>
-      <c r="C60">
-        <v>2</v>
-      </c>
-      <c r="D60">
-        <v>120628.41082793</v>
-      </c>
-      <c r="E60">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F60">
-        <v>0.85824890324911396</v>
-      </c>
-      <c r="G60" s="4">
-        <v>20824.7129679639</v>
-      </c>
-      <c r="H60">
-        <v>7456.39074483072</v>
-      </c>
-      <c r="I60">
-        <v>5114.4587365303096</v>
-      </c>
-      <c r="J60">
-        <v>33395.562449324898</v>
-      </c>
-      <c r="K60">
-        <v>51302.320205525801</v>
-      </c>
-      <c r="L60">
-        <v>16537.7269222135</v>
-      </c>
-      <c r="M60">
-        <v>19392.801250865799</v>
-      </c>
-      <c r="N60">
-        <v>1004.9477757237401</v>
-      </c>
-      <c r="O60">
-        <v>0</v>
-      </c>
-      <c r="P60">
-        <v>242180.39335481101</v>
-      </c>
-      <c r="Q60">
-        <v>1183.4303612998101</v>
-      </c>
-      <c r="R60">
-        <v>15931.1957490451</v>
-      </c>
-      <c r="S60">
-        <v>346.33034237054602</v>
-      </c>
-      <c r="T60">
-        <v>1.0959871186973</v>
+      <c r="O61">
+        <v>0</v>
+      </c>
+      <c r="P61">
+        <v>237266.087609501</v>
+      </c>
+      <c r="Q61">
+        <v>1127.2750356983499</v>
+      </c>
+      <c r="R61">
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B62" t="s">
         <v>21</v>
@@ -3510,387 +3665,393 @@
         <v>4</v>
       </c>
       <c r="D62">
-        <v>115714.10508261999</v>
+        <v>120375.156660901</v>
       </c>
       <c r="E62">
-        <v>282179.671253876</v>
+        <v>282179.671232878</v>
       </c>
       <c r="F62">
-        <v>0.84083338305413902</v>
+        <v>0.857351410648304</v>
       </c>
       <c r="G62" s="4">
-        <v>20578.5072164468</v>
+        <v>21285.1004075495</v>
       </c>
       <c r="H62">
-        <v>7102.5751506616798</v>
+        <v>7426.32532798384</v>
       </c>
       <c r="I62">
-        <v>2588.50529592865</v>
+        <v>5046.79446201879</v>
       </c>
       <c r="J62">
-        <v>30269.587663037099</v>
+        <v>33758.220197552102</v>
       </c>
       <c r="K62">
-        <v>50843.185173268197</v>
+        <v>51144.191344099498</v>
       </c>
       <c r="L62">
-        <v>15303.8015139912</v>
+        <v>16112.7556071296</v>
       </c>
       <c r="M62">
-        <v>19297.530732323299</v>
+        <v>19359.989512119799</v>
       </c>
       <c r="N62">
-        <v>992.31070788530405</v>
+        <v>1006.77939378399</v>
       </c>
       <c r="O62">
         <v>0</v>
       </c>
       <c r="P62">
-        <v>237266.087609501</v>
+        <v>241927.13918778201</v>
       </c>
       <c r="Q62">
-        <v>1127.2750356983499</v>
+        <v>1178.65858109644</v>
       </c>
       <c r="R62">
-        <v>0</v>
+        <v>12586.325853030899</v>
+      </c>
+      <c r="S62">
+        <v>466.16021677892502</v>
+      </c>
+      <c r="T62">
+        <v>1.3585822738026401</v>
       </c>
     </row>
     <row r="63" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
+      <c r="G63" s="4"/>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A64" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G64" s="4"/>
+    </row>
+    <row r="65" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>22</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B65" t="s">
         <v>21</v>
       </c>
-      <c r="C63">
+      <c r="C65">
         <v>4</v>
       </c>
-      <c r="D63">
-        <v>120375.156660901</v>
-      </c>
-      <c r="E63">
-        <v>282179.671232878</v>
-      </c>
-      <c r="F63">
-        <v>0.857351410648304</v>
-      </c>
-      <c r="G63" s="4">
-        <v>21285.1004075495</v>
-      </c>
-      <c r="H63">
-        <v>7426.32532798384</v>
-      </c>
-      <c r="I63">
-        <v>5046.79446201879</v>
-      </c>
-      <c r="J63">
-        <v>33758.220197552102</v>
-      </c>
-      <c r="K63">
-        <v>51144.191344099498</v>
-      </c>
-      <c r="L63">
-        <v>16112.7556071296</v>
-      </c>
-      <c r="M63">
-        <v>19359.989512119799</v>
-      </c>
-      <c r="N63">
-        <v>1006.77939378399</v>
-      </c>
-      <c r="O63">
-        <v>0</v>
-      </c>
-      <c r="P63">
-        <v>241927.13918778201</v>
-      </c>
-      <c r="Q63">
-        <v>1178.65858109644</v>
-      </c>
-      <c r="R63">
-        <v>12586.325853030899</v>
-      </c>
-      <c r="S63">
-        <v>466.16021677892502</v>
-      </c>
-      <c r="T63">
-        <v>1.3585822738026401</v>
-      </c>
-    </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="G64" s="4"/>
-    </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A65" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G65" s="4"/>
+      <c r="D65">
+        <v>146108.01933512901</v>
+      </c>
+      <c r="E65">
+        <v>355610.364944759</v>
+      </c>
+      <c r="F65">
+        <v>0.75267772890587503</v>
+      </c>
+      <c r="G65">
+        <v>25765.651662743599</v>
+      </c>
+      <c r="H65">
+        <v>7150.9042815892099</v>
+      </c>
+      <c r="I65">
+        <v>5144.3184852884797</v>
+      </c>
+      <c r="J65">
+        <v>38060.874429621297</v>
+      </c>
+      <c r="K65">
+        <v>64168.339029134899</v>
+      </c>
+      <c r="L65">
+        <v>19539.954214541001</v>
+      </c>
+      <c r="M65">
+        <v>24338.851661831999</v>
+      </c>
+      <c r="N65">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O65">
+        <v>0</v>
+      </c>
+      <c r="P65">
+        <v>267660.00186201098</v>
+      </c>
+      <c r="Q65">
+        <v>1597.68911089628</v>
+      </c>
+      <c r="R65">
+        <v>13084.0423994256</v>
+      </c>
+      <c r="S65">
+        <v>467.28722855091399</v>
+      </c>
+      <c r="T65">
+        <v>-0.25904927491985202</v>
+      </c>
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>22</v>
       </c>
       <c r="B66" t="s">
+        <v>35</v>
+      </c>
+      <c r="C66" t="s">
+        <v>35</v>
+      </c>
+      <c r="D66" t="s">
+        <v>36</v>
+      </c>
+      <c r="E66" t="s">
+        <v>36</v>
+      </c>
+      <c r="F66" t="s">
+        <v>36</v>
+      </c>
+      <c r="G66" s="4">
+        <v>28838</v>
+      </c>
+      <c r="H66">
+        <v>7567.5</v>
+      </c>
+      <c r="I66">
+        <v>13764.1</v>
+      </c>
+      <c r="J66">
+        <v>50169.7</v>
+      </c>
+      <c r="K66" t="s">
+        <v>36</v>
+      </c>
+      <c r="L66" t="s">
+        <v>36</v>
+      </c>
+      <c r="M66" t="s">
+        <v>36</v>
+      </c>
+      <c r="N66" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="68" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A68" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G68" s="4"/>
+      <c r="P68" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>16</v>
+      </c>
+      <c r="R68" t="s">
+        <v>17</v>
+      </c>
+      <c r="S68" t="s">
+        <v>18</v>
+      </c>
+      <c r="T68" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="69" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B69" t="s">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>2</v>
+      </c>
+      <c r="D69" t="s">
+        <v>3</v>
+      </c>
+      <c r="E69" t="s">
+        <v>4</v>
+      </c>
+      <c r="F69" t="s">
+        <v>5</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H69" t="s">
+        <v>7</v>
+      </c>
+      <c r="I69" t="s">
+        <v>8</v>
+      </c>
+      <c r="J69" t="s">
+        <v>9</v>
+      </c>
+      <c r="K69" t="s">
+        <v>10</v>
+      </c>
+      <c r="L69" t="s">
+        <v>11</v>
+      </c>
+      <c r="M69" t="s">
+        <v>12</v>
+      </c>
+      <c r="N69" t="s">
+        <v>13</v>
+      </c>
+      <c r="O69" t="s">
+        <v>14</v>
+      </c>
+      <c r="P69">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q69">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R69">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S69">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T69">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="70" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A70" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B70" t="s">
         <v>21</v>
       </c>
-      <c r="C66">
+      <c r="C70">
         <v>4</v>
       </c>
-      <c r="D66">
-        <v>146108.01933512901</v>
-      </c>
-      <c r="E66">
-        <v>355610.364944759</v>
-      </c>
-      <c r="F66">
-        <v>0.75267772890587503</v>
-      </c>
-      <c r="G66">
-        <v>25765.651662743599</v>
-      </c>
-      <c r="H66">
-        <v>7150.9042815892099</v>
-      </c>
-      <c r="I66">
-        <v>5144.3184852884797</v>
-      </c>
-      <c r="J66">
-        <v>38060.874429621297</v>
-      </c>
-      <c r="K66">
-        <v>64168.339029134899</v>
-      </c>
-      <c r="L66">
-        <v>19539.954214541001</v>
-      </c>
-      <c r="M66">
-        <v>24338.851661831999</v>
-      </c>
-      <c r="N66">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O66">
-        <v>0</v>
-      </c>
-      <c r="P66">
-        <v>267660.00186201098</v>
-      </c>
-      <c r="Q66">
-        <v>1597.68911089628</v>
-      </c>
-      <c r="R66">
-        <v>13084.0423994256</v>
-      </c>
-      <c r="S66">
-        <v>467.28722855091399</v>
-      </c>
-      <c r="T66">
-        <v>-0.25904927491985202</v>
-      </c>
-    </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
-        <v>22</v>
-      </c>
-      <c r="B67" t="s">
-        <v>35</v>
-      </c>
-      <c r="C67" t="s">
-        <v>35</v>
-      </c>
-      <c r="D67" t="s">
-        <v>36</v>
-      </c>
-      <c r="E67" t="s">
-        <v>36</v>
-      </c>
-      <c r="F67" t="s">
-        <v>36</v>
-      </c>
-      <c r="G67" s="4">
-        <v>28838</v>
-      </c>
-      <c r="H67">
-        <v>7567.5</v>
-      </c>
-      <c r="I67">
-        <v>13764.1</v>
-      </c>
-      <c r="J67">
-        <v>50169.7</v>
-      </c>
-      <c r="K67" t="s">
-        <v>36</v>
-      </c>
-      <c r="L67" t="s">
-        <v>36</v>
-      </c>
-      <c r="M67" t="s">
-        <v>36</v>
-      </c>
-      <c r="N67" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="69" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G69" s="4"/>
-      <c r="P69" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q69" t="s">
-        <v>16</v>
-      </c>
-      <c r="R69" t="s">
-        <v>17</v>
-      </c>
-      <c r="S69" t="s">
-        <v>18</v>
-      </c>
-      <c r="T69" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="70" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
-        <v>0</v>
-      </c>
-      <c r="B70" t="s">
-        <v>1</v>
-      </c>
-      <c r="C70" t="s">
+      <c r="D70">
+        <v>29525.427309999999</v>
+      </c>
+      <c r="E70">
+        <v>80391.755990000005</v>
+      </c>
+      <c r="F70">
+        <v>0.79280104200000001</v>
+      </c>
+      <c r="G70" s="4">
+        <v>5050.6365619999997</v>
+      </c>
+      <c r="H70">
+        <v>4678.3390820000004</v>
+      </c>
+      <c r="I70">
+        <v>2508.6600360000002</v>
+      </c>
+      <c r="J70">
+        <v>12237.635679999999</v>
+      </c>
+      <c r="K70">
+        <v>13920</v>
+      </c>
+      <c r="L70">
+        <v>2841.544922</v>
+      </c>
+      <c r="M70">
+        <v>5380.5444360000001</v>
+      </c>
+      <c r="N70">
+        <v>279.27307350000001</v>
+      </c>
+      <c r="O70">
+        <v>0</v>
+      </c>
+      <c r="P70">
+        <v>64865.028310000002</v>
+      </c>
+      <c r="Q70">
+        <v>1191.7509680000001</v>
+      </c>
+      <c r="R70">
+        <v>7243.7162129999997</v>
+      </c>
+      <c r="S70">
+        <v>452.7322633</v>
+      </c>
+      <c r="T70">
+        <v>5.8154128590000003</v>
+      </c>
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A71" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="73" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>32</v>
+      </c>
+      <c r="B73" t="s">
+        <v>33</v>
+      </c>
+      <c r="C73" t="s">
         <v>2</v>
       </c>
-      <c r="D70" t="s">
-        <v>3</v>
-      </c>
-      <c r="E70" t="s">
-        <v>4</v>
-      </c>
-      <c r="F70" t="s">
-        <v>5</v>
-      </c>
-      <c r="G70" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H70" t="s">
-        <v>7</v>
-      </c>
-      <c r="I70" t="s">
-        <v>8</v>
-      </c>
-      <c r="J70" t="s">
-        <v>9</v>
-      </c>
-      <c r="K70" t="s">
-        <v>10</v>
-      </c>
-      <c r="L70" t="s">
-        <v>11</v>
-      </c>
-      <c r="M70" t="s">
-        <v>12</v>
-      </c>
-      <c r="N70" t="s">
-        <v>13</v>
-      </c>
-      <c r="O70" t="s">
-        <v>14</v>
-      </c>
-      <c r="P70">
-        <v>63734.6679</v>
-      </c>
-      <c r="Q70">
-        <v>1078.4492829999999</v>
-      </c>
-      <c r="R70">
-        <v>624.70352849999995</v>
-      </c>
-      <c r="S70">
-        <v>13.014656840000001</v>
-      </c>
-      <c r="T70">
-        <v>27.514184579999998</v>
-      </c>
-    </row>
-    <row r="71" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="2" t="s">
+    </row>
+    <row r="74" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A74">
         <v>20</v>
       </c>
-      <c r="B71" t="s">
-        <v>21</v>
-      </c>
-      <c r="C71">
-        <v>4</v>
-      </c>
-      <c r="D71">
-        <v>29525.427309999999</v>
-      </c>
-      <c r="E71">
-        <v>80391.755990000005</v>
-      </c>
-      <c r="F71">
-        <v>0.79280104200000001</v>
-      </c>
-      <c r="G71" s="4">
-        <v>5050.6365619999997</v>
-      </c>
-      <c r="H71">
-        <v>4678.3390820000004</v>
-      </c>
-      <c r="I71">
-        <v>2508.6600360000002</v>
-      </c>
-      <c r="J71">
-        <v>12237.635679999999</v>
-      </c>
-      <c r="K71">
-        <v>13920</v>
-      </c>
-      <c r="L71">
-        <v>2841.544922</v>
-      </c>
-      <c r="M71">
-        <v>5380.5444360000001</v>
-      </c>
-      <c r="N71">
-        <v>279.27307350000001</v>
-      </c>
-      <c r="O71">
-        <v>0</v>
-      </c>
-      <c r="P71">
-        <v>64865.028310000002</v>
-      </c>
-      <c r="Q71">
-        <v>1191.7509680000001</v>
-      </c>
-      <c r="R71">
-        <v>7243.7162129999997</v>
-      </c>
-      <c r="S71">
-        <v>452.7322633</v>
-      </c>
-      <c r="T71">
-        <v>5.8154128590000003</v>
-      </c>
-    </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A72" s="7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
-        <v>32</v>
-      </c>
-      <c r="B74" t="s">
-        <v>33</v>
-      </c>
-      <c r="C74" t="s">
+      <c r="B74">
+        <v>60</v>
+      </c>
+      <c r="C74">
         <v>2</v>
+      </c>
+      <c r="D74">
+        <v>119696.652328767</v>
+      </c>
+      <c r="E74">
+        <v>282179.67123285501</v>
+      </c>
+      <c r="F74">
+        <v>0.854946898908852</v>
+      </c>
+      <c r="G74">
+        <v>18681.222424938602</v>
+      </c>
+      <c r="H74">
+        <v>5354.6114985546601</v>
+      </c>
+      <c r="I74">
+        <v>8156.08309050551</v>
+      </c>
+      <c r="J74">
+        <v>32191.917013998798</v>
+      </c>
+      <c r="K74">
+        <v>51372.124296964801</v>
+      </c>
+      <c r="L74">
+        <v>16725.325417965501</v>
+      </c>
+      <c r="M74">
+        <v>19407.285599838699</v>
+      </c>
+      <c r="N74">
+        <v>1016.03855436447</v>
+      </c>
+      <c r="O74">
+        <v>0</v>
+      </c>
+      <c r="P74">
+        <v>241248.634855649</v>
+      </c>
+      <c r="Q74">
+        <v>1192.7637589594799</v>
+      </c>
+      <c r="R74">
+        <v>19736.206339365101</v>
+      </c>
+      <c r="S74">
+        <v>481.37088632597801</v>
+      </c>
+      <c r="T74" s="6">
+        <v>0.12591688076390301</v>
       </c>
     </row>
     <row r="75" spans="1:20" x14ac:dyDescent="0.35">
@@ -3898,61 +4059,61 @@
         <v>20</v>
       </c>
       <c r="B75">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C75">
         <v>2</v>
       </c>
       <c r="D75">
-        <v>119696.652328767</v>
+        <v>118381.960809661</v>
       </c>
       <c r="E75">
-        <v>282179.67123285501</v>
+        <v>282254.81855225202</v>
       </c>
       <c r="F75">
-        <v>0.854946898908852</v>
+        <v>0.85006146065890897</v>
       </c>
       <c r="G75">
-        <v>18681.222424938602</v>
+        <v>19407.840072768398</v>
       </c>
       <c r="H75">
-        <v>5354.6114985546601</v>
+        <v>5891.8301217549197</v>
       </c>
       <c r="I75">
-        <v>8156.08309050551</v>
+        <v>6659.4942697455399</v>
       </c>
       <c r="J75">
-        <v>32191.917013998798</v>
+        <v>31959.164464268899</v>
       </c>
       <c r="K75">
-        <v>51372.124296964801</v>
+        <v>51102.045942938203</v>
       </c>
       <c r="L75">
-        <v>16725.325417965501</v>
+        <v>15967.176494174801</v>
       </c>
       <c r="M75">
-        <v>19407.285599838699</v>
+        <v>19353.573908279199</v>
       </c>
       <c r="N75">
-        <v>1016.03855436447</v>
+        <v>1010.46273302954</v>
       </c>
       <c r="O75">
         <v>0</v>
       </c>
       <c r="P75">
-        <v>241248.634855649</v>
+        <v>239933.943336542</v>
       </c>
       <c r="Q75">
-        <v>1192.7637589594799</v>
+        <v>1312.43161993582</v>
       </c>
       <c r="R75">
-        <v>19736.206339365101</v>
+        <v>18377.616631847999</v>
       </c>
       <c r="S75">
-        <v>481.37088632597801</v>
+        <v>459.4404157962</v>
       </c>
       <c r="T75" s="6">
-        <v>0.12591688076390301</v>
+        <v>0.14758705239613301</v>
       </c>
     </row>
     <row r="76" spans="1:20" x14ac:dyDescent="0.35">
@@ -3960,40 +4121,40 @@
         <v>20</v>
       </c>
       <c r="B76">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C76">
         <v>2</v>
       </c>
       <c r="D76">
-        <v>118381.960809661</v>
+        <v>116766.56672038</v>
       </c>
       <c r="E76">
-        <v>282254.81855225202</v>
+        <v>282179.67123287299</v>
       </c>
       <c r="F76">
-        <v>0.85006146065890897</v>
+        <v>0.84456314023622803</v>
       </c>
       <c r="G76">
-        <v>19407.840072768398</v>
+        <v>19298.245593088301</v>
       </c>
       <c r="H76">
-        <v>5891.8301217549197</v>
+        <v>5682.0016560700296</v>
       </c>
       <c r="I76">
-        <v>6659.4942697455399</v>
+        <v>5350.3346939491703</v>
       </c>
       <c r="J76">
-        <v>31959.164464268899</v>
+        <v>30330.5819431075</v>
       </c>
       <c r="K76">
-        <v>51102.045942938203</v>
+        <v>51097.733915068202</v>
       </c>
       <c r="L76">
-        <v>15967.176494174801</v>
+        <v>15987.901266609</v>
       </c>
       <c r="M76">
-        <v>19353.573908279199</v>
+        <v>19350.349595595701</v>
       </c>
       <c r="N76">
         <v>1010.46273302954</v>
@@ -4002,19 +4163,19 @@
         <v>0</v>
       </c>
       <c r="P76">
-        <v>239933.943336542</v>
+        <v>238318.54924726201</v>
       </c>
       <c r="Q76">
-        <v>1312.43161993582</v>
+        <v>1265.6913868611</v>
       </c>
       <c r="R76">
-        <v>18377.616631847999</v>
+        <v>17746.163883660702</v>
       </c>
       <c r="S76">
-        <v>459.4404157962</v>
+        <v>507.03325381887902</v>
       </c>
       <c r="T76" s="6">
-        <v>0.14758705239613301</v>
+        <v>-0.25983751983286502</v>
       </c>
     </row>
     <row r="77" spans="1:20" x14ac:dyDescent="0.35">
@@ -4022,102 +4183,102 @@
         <v>20</v>
       </c>
       <c r="B77">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C77">
         <v>2</v>
       </c>
       <c r="D77">
-        <v>116766.56672038</v>
+        <v>115610.996393592</v>
       </c>
       <c r="E77">
-        <v>282179.67123287299</v>
+        <v>282182.50548365602</v>
       </c>
       <c r="F77">
-        <v>0.84456314023622803</v>
+        <v>0.84045954058697003</v>
       </c>
       <c r="G77">
-        <v>19298.245593088301</v>
+        <v>19302.752565837702</v>
       </c>
       <c r="H77">
-        <v>5682.0016560700296</v>
+        <v>6226.5181629292701</v>
       </c>
       <c r="I77">
-        <v>5350.3346939491703</v>
+        <v>3974.5318253822402</v>
       </c>
       <c r="J77">
-        <v>30330.5819431075</v>
+        <v>29503.802554149199</v>
       </c>
       <c r="K77">
-        <v>51097.733915068202</v>
+        <v>51013.610661725899</v>
       </c>
       <c r="L77">
-        <v>15987.901266609</v>
+        <v>15760.601295416</v>
       </c>
       <c r="M77">
-        <v>19350.349595595701</v>
+        <v>19332.981882301501</v>
       </c>
       <c r="N77">
-        <v>1010.46273302954</v>
+        <v>1014.17312250211</v>
       </c>
       <c r="O77">
         <v>0</v>
       </c>
       <c r="P77">
-        <v>238318.54924726201</v>
+        <v>237162.97892047401</v>
       </c>
       <c r="Q77">
-        <v>1265.6913868611</v>
+        <v>1386.9848841974899</v>
       </c>
       <c r="R77">
-        <v>17746.163883660702</v>
+        <v>18436.445202769701</v>
       </c>
       <c r="S77">
-        <v>507.03325381887902</v>
+        <v>209.50505912238299</v>
       </c>
       <c r="T77" s="6">
-        <v>-0.25983751983286502</v>
+        <v>0.28049716262959101</v>
       </c>
     </row>
     <row r="78" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A78">
+      <c r="A78" s="3">
         <v>20</v>
       </c>
-      <c r="B78">
-        <v>30</v>
-      </c>
-      <c r="C78">
+      <c r="B78" s="3">
+        <v>20</v>
+      </c>
+      <c r="C78" s="3">
         <v>2</v>
       </c>
       <c r="D78">
-        <v>115610.996393592</v>
+        <v>114184.286860504</v>
       </c>
       <c r="E78">
-        <v>282182.50548365602</v>
+        <v>282179.67123297497</v>
       </c>
       <c r="F78">
-        <v>0.84045954058697003</v>
+        <v>0.83541194997266699</v>
       </c>
       <c r="G78">
-        <v>19302.752565837702</v>
+        <v>19351.2255529412</v>
       </c>
       <c r="H78">
-        <v>6226.5181629292701</v>
+        <v>6002.0469674603501</v>
       </c>
       <c r="I78">
-        <v>3974.5318253822402</v>
+        <v>2645.4376652921501</v>
       </c>
       <c r="J78">
-        <v>29503.802554149199</v>
+        <v>27998.710185693701</v>
       </c>
       <c r="K78">
-        <v>51013.610661725899</v>
+        <v>51033.4442867088</v>
       </c>
       <c r="L78">
-        <v>15760.601295416</v>
+        <v>15815.1228903871</v>
       </c>
       <c r="M78">
-        <v>19332.981882301501</v>
+        <v>19337.009497714302</v>
       </c>
       <c r="N78">
         <v>1014.17312250211</v>
@@ -4126,81 +4287,81 @@
         <v>0</v>
       </c>
       <c r="P78">
-        <v>237162.97892047401</v>
+        <v>235736.26938738499</v>
       </c>
       <c r="Q78">
-        <v>1386.9848841974899</v>
+        <v>1336.98290493166</v>
       </c>
       <c r="R78">
-        <v>18436.445202769701</v>
+        <v>18577.307877855899</v>
       </c>
       <c r="S78">
-        <v>209.50505912238299</v>
+        <v>432.030415764091</v>
       </c>
       <c r="T78" s="6">
-        <v>0.28049716262959101</v>
+        <v>-0.122490141098651</v>
       </c>
     </row>
     <row r="79" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A79" s="3">
+      <c r="A79">
         <v>20</v>
       </c>
-      <c r="B79" s="3">
-        <v>20</v>
-      </c>
-      <c r="C79" s="3">
+      <c r="B79">
+        <v>15</v>
+      </c>
+      <c r="C79">
         <v>2</v>
       </c>
       <c r="D79">
-        <v>114184.286860504</v>
+        <v>113440.79599059001</v>
       </c>
       <c r="E79">
-        <v>282179.67123297497</v>
+        <v>282179.67123267101</v>
       </c>
       <c r="F79">
-        <v>0.83541194997266699</v>
+        <v>0.83277713625127903</v>
       </c>
       <c r="G79">
-        <v>19351.2255529412</v>
+        <v>19390.977969205</v>
       </c>
       <c r="H79">
-        <v>6002.0469674603501</v>
+        <v>5599.5405456203798</v>
       </c>
       <c r="I79">
-        <v>2645.4376652921501</v>
+        <v>2128.1287863747102</v>
       </c>
       <c r="J79">
-        <v>27998.710185693701</v>
+        <v>27118.647301200101</v>
       </c>
       <c r="K79">
-        <v>51033.4442867088</v>
+        <v>51068.507704320902</v>
       </c>
       <c r="L79">
-        <v>15815.1228903871</v>
+        <v>15909.3558282099</v>
       </c>
       <c r="M79">
-        <v>19337.009497714302</v>
+        <v>19344.285156859401</v>
       </c>
       <c r="N79">
-        <v>1014.17312250211</v>
+        <v>1010.46273302954</v>
       </c>
       <c r="O79">
         <v>0</v>
       </c>
       <c r="P79">
-        <v>235736.26938738499</v>
+        <v>234992.778517472</v>
       </c>
       <c r="Q79">
-        <v>1336.98290493166</v>
+        <v>1247.3228025527501</v>
       </c>
       <c r="R79">
-        <v>18577.307877855899</v>
+        <v>16417.502561416801</v>
       </c>
       <c r="S79">
-        <v>432.030415764091</v>
+        <v>469.07150175476602</v>
       </c>
       <c r="T79" s="6">
-        <v>-0.122490141098651</v>
+        <v>0.46004655114715598</v>
       </c>
     </row>
     <row r="80" spans="1:20" x14ac:dyDescent="0.35">
@@ -4208,122 +4369,60 @@
         <v>20</v>
       </c>
       <c r="B80">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C80">
         <v>2</v>
       </c>
       <c r="D80">
-        <v>113440.79599059001</v>
+        <v>113795.448700252</v>
       </c>
       <c r="E80">
-        <v>282179.67123267101</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F80">
-        <v>0.83277713625127903</v>
+        <v>0.83403396920434802</v>
       </c>
       <c r="G80">
-        <v>19390.977969205</v>
+        <v>20436.472361711199</v>
       </c>
       <c r="H80">
-        <v>5599.5405456203798</v>
+        <v>4946.5396722567002</v>
       </c>
       <c r="I80">
-        <v>2128.1287863747102</v>
+        <v>2967.9237851293901</v>
       </c>
       <c r="J80">
-        <v>27118.647301200101</v>
+        <v>28350.9358190973</v>
       </c>
       <c r="K80">
-        <v>51068.507704320902</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L80">
-        <v>15909.3558282099</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M80">
-        <v>19344.285156859401</v>
+        <v>19297.530489448302</v>
       </c>
       <c r="N80">
-        <v>1010.46273302954</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O80">
         <v>0</v>
       </c>
       <c r="P80">
-        <v>234992.778517472</v>
+        <v>235347.43122713399</v>
       </c>
       <c r="Q80">
-        <v>1247.3228025527501</v>
+        <v>1101.8639118583401</v>
       </c>
       <c r="R80">
-        <v>16417.502561416801</v>
+        <v>13.380488321454299</v>
       </c>
       <c r="S80">
-        <v>469.07150175476602</v>
+        <v>2.67609766429086</v>
       </c>
       <c r="T80" s="6">
-        <v>0.46004655114715598</v>
-      </c>
-    </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A81">
-        <v>20</v>
-      </c>
-      <c r="B81">
-        <v>12</v>
-      </c>
-      <c r="C81">
-        <v>2</v>
-      </c>
-      <c r="D81">
-        <v>113795.448700252</v>
-      </c>
-      <c r="E81">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F81">
-        <v>0.83403396920434802</v>
-      </c>
-      <c r="G81">
-        <v>20436.472361711199</v>
-      </c>
-      <c r="H81">
-        <v>4946.5396722567002</v>
-      </c>
-      <c r="I81">
-        <v>2967.9237851293901</v>
-      </c>
-      <c r="J81">
-        <v>28350.9358190973</v>
-      </c>
-      <c r="K81">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L81">
-        <v>15303.798385783</v>
-      </c>
-      <c r="M81">
-        <v>19297.530489448302</v>
-      </c>
-      <c r="N81">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O81">
-        <v>0</v>
-      </c>
-      <c r="P81">
-        <v>235347.43122713399</v>
-      </c>
-      <c r="Q81">
-        <v>1101.8639118583401</v>
-      </c>
-      <c r="R81">
-        <v>13.380488321454299</v>
-      </c>
-      <c r="S81">
-        <v>2.67609766429086</v>
-      </c>
-      <c r="T81" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>

</xml_diff>

<commit_message>
baseline for split cost increase across all electricity bill components
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{830F13C9-BBB4-42FC-9D89-F410E2378D29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0879A5B2-96B0-4357-ADE0-41E51172CD4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -117,7 +117,7 @@
     This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</t>
       </text>
     </comment>
-    <comment ref="A41" authorId="8" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A48" authorId="8" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -125,7 +125,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="A42" authorId="9" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A49" authorId="9" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -133,7 +133,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T42" authorId="10" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T49" authorId="10" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -143,7 +143,7 @@
     The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A48" authorId="11" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A55" authorId="11" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -151,7 +151,7 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="A65" authorId="12" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A72" authorId="12" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -159,7 +159,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T77" authorId="13" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T84" authorId="13" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -172,7 +172,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="42">
   <si>
     <t>Season</t>
   </si>
@@ -295,6 +295,9 @@
   </si>
   <si>
     <t>Charge Power Capacity</t>
+  </si>
+  <si>
+    <t>Higher Rate Even Division</t>
   </si>
 </sst>
 </file>
@@ -1222,25 +1225,25 @@
   <threadedComment ref="A28" dT="2026-07-15T17:22:40.80" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
     <text>This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</text>
   </threadedComment>
-  <threadedComment ref="A41" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+  <threadedComment ref="A48" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
-  <threadedComment ref="A42" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+  <threadedComment ref="A49" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
     <text>Summer week = hot summer weekdays + high weekends</text>
   </threadedComment>
-  <threadedComment ref="T42" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T49" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure</text>
   </threadedComment>
-  <threadedComment ref="T42" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T49" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>The baseline costs have to be updated in accordance with the demand structure type</text>
   </threadedComment>
-  <threadedComment ref="A48" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+  <threadedComment ref="A55" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
     <text>Result from the fast solve</text>
   </threadedComment>
-  <threadedComment ref="A65" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+  <threadedComment ref="A72" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
     <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
   </threadedComment>
-  <threadedComment ref="T77" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="T84" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1248,7 +1251,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:V80"/>
+  <dimension ref="A1:V87"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.6328125" customWidth="1"/>
@@ -2582,34 +2585,34 @@
         <v>0</v>
       </c>
       <c r="D34">
-        <v>153412.243053051</v>
+        <v>115583.48181615899</v>
       </c>
       <c r="E34">
-        <v>374203.2</v>
+        <v>282190.859999999</v>
       </c>
       <c r="F34">
-        <v>0.73479923629710397</v>
+        <v>0.84033715458764902</v>
       </c>
       <c r="G34">
-        <v>28189.163715008799</v>
+        <v>21182.959346048301</v>
       </c>
       <c r="H34">
-        <v>8631.5718994758809</v>
+        <v>6486.2597020478397</v>
       </c>
       <c r="I34">
-        <v>3282.10418908369</v>
+        <v>2466.3619080631902</v>
       </c>
       <c r="J34">
-        <v>40102.8398035684</v>
+        <v>30135.5809561594</v>
       </c>
       <c r="K34">
-        <v>67424.000035550795</v>
+        <v>50845.200000000099</v>
       </c>
       <c r="L34">
-        <v>20294.624006555201</v>
+        <v>15304.405199999899</v>
       </c>
       <c r="M34">
-        <v>25590.779207376701</v>
+        <v>19298.29566</v>
       </c>
       <c r="N34">
         <v>1409.83742959549</v>
@@ -2618,19 +2621,19 @@
         <v>0</v>
       </c>
       <c r="P34">
-        <v>274964.22557993297</v>
+        <v>237135.46434304101</v>
       </c>
       <c r="Q34">
-        <v>1466.6067163636201</v>
+        <v>1102.0926609763501</v>
       </c>
       <c r="R34">
         <v>0</v>
       </c>
       <c r="U34">
-        <v>61253.928349088899</v>
+        <v>15.5670440273115</v>
       </c>
       <c r="V34">
-        <v>364.606716363624</v>
+        <v>9.2660976353045002E-2</v>
       </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.35">
@@ -2644,34 +2647,34 @@
         <v>0</v>
       </c>
       <c r="D35">
-        <v>165265.875469322</v>
+        <v>124490.983160207</v>
       </c>
       <c r="E35">
-        <v>374203.2</v>
+        <v>282190.859999999</v>
       </c>
       <c r="F35">
-        <v>0.76647623001674903</v>
+        <v>0.87190267497356</v>
       </c>
       <c r="G35">
-        <v>30792.331969512299</v>
+        <v>23139.129735574901</v>
       </c>
       <c r="H35">
-        <v>8631.5718986985103</v>
+        <v>6486.2597020478397</v>
       </c>
       <c r="I35">
-        <v>12532.568351771601</v>
+        <v>9417.6928625843393</v>
       </c>
       <c r="J35">
-        <v>51956.472219982403</v>
+        <v>39043.082300207097</v>
       </c>
       <c r="K35">
-        <v>67424.000035514298</v>
+        <v>50845.200000000099</v>
       </c>
       <c r="L35">
-        <v>20294.624006456401</v>
+        <v>15304.405199999899</v>
       </c>
       <c r="M35">
-        <v>25590.7792073692</v>
+        <v>19298.29566</v>
       </c>
       <c r="N35">
         <v>1409.83742959549</v>
@@ -2680,19 +2683,19 @@
         <v>0</v>
       </c>
       <c r="P35">
-        <v>286817.85799620399</v>
+        <v>246042.96568708899</v>
       </c>
       <c r="Q35">
-        <v>1466.6067162315301</v>
+        <v>1102.0926609763501</v>
       </c>
       <c r="R35">
         <v>0</v>
       </c>
       <c r="U35">
-        <v>61253.928326898502</v>
+        <v>15.5670440273115</v>
       </c>
       <c r="V35">
-        <v>364.606716231539</v>
+        <v>9.2660976353045002E-2</v>
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.35">
@@ -2833,457 +2836,231 @@
         <v>69.034824646017199</v>
       </c>
     </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A39" s="3"/>
+    </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A40" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="G40" s="4"/>
+      <c r="A40" s="7" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B41" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C41">
-        <v>0</v>
-      </c>
-      <c r="D41">
-        <v>116861.67991782499</v>
-      </c>
-      <c r="E41">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F41">
-        <v>0.84490020632262297</v>
-      </c>
-      <c r="G41">
-        <v>23556.420831705898</v>
-      </c>
-      <c r="H41">
-        <v>6947.4542183048998</v>
-      </c>
-      <c r="I41">
-        <v>913.29198665996</v>
-      </c>
-      <c r="J41">
-        <v>31417.167036670799</v>
-      </c>
-      <c r="K41">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L41">
-        <v>15303.798385783</v>
-      </c>
-      <c r="M41">
-        <v>19297.5304894482</v>
-      </c>
-      <c r="N41">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O41">
-        <v>0</v>
-      </c>
-      <c r="P41">
-        <v>238413.66244470701</v>
-      </c>
-      <c r="Q41">
-        <v>1102.6552392369899</v>
-      </c>
-      <c r="R41">
-        <v>0</v>
-      </c>
-      <c r="S41">
-        <v>0</v>
-      </c>
-      <c r="T41">
-        <v>0</v>
-      </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C42">
-        <v>0</v>
-      </c>
-      <c r="D42">
-        <v>187020.456722612</v>
-      </c>
-      <c r="E42">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F42">
-        <v>1.09353178385</v>
-      </c>
-      <c r="G42">
-        <v>89520.694507565597</v>
-      </c>
-      <c r="H42">
-        <v>6971.3813103080802</v>
-      </c>
-      <c r="I42">
-        <v>5083.8680235841202</v>
-      </c>
-      <c r="J42">
-        <v>101575.943841457</v>
-      </c>
-      <c r="K42">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L42">
-        <v>15303.798385783</v>
-      </c>
-      <c r="M42">
-        <v>19297.5304894482</v>
-      </c>
-      <c r="N42">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O42">
-        <v>0</v>
-      </c>
-      <c r="P42">
-        <v>308572.439249494</v>
-      </c>
-      <c r="Q42">
-        <v>1106.4527933521999</v>
-      </c>
-      <c r="R42">
-        <v>3451.9307168288801</v>
-      </c>
-      <c r="S42">
-        <v>20.547206647791</v>
-      </c>
-      <c r="T42">
-        <v>-14.696886263168601</v>
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43" s="3"/>
-      <c r="G43" s="4"/>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+      <c r="A44" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B44" t="s">
-        <v>21</v>
-      </c>
-      <c r="C44">
-        <v>0</v>
-      </c>
-      <c r="D44">
-        <v>117032.41959359701</v>
-      </c>
-      <c r="E44">
-        <v>282179.67123286898</v>
-      </c>
-      <c r="F44">
-        <v>0.845505280653571</v>
-      </c>
-      <c r="G44" s="4">
-        <v>23683.129427060001</v>
-      </c>
-      <c r="H44">
-        <v>6986.3695969997798</v>
-      </c>
-      <c r="I44">
-        <v>918.40768838365295</v>
-      </c>
-      <c r="J44">
-        <v>31587.906712443499</v>
-      </c>
-      <c r="K44">
-        <v>50843.1840059237</v>
-      </c>
-      <c r="L44">
-        <v>15303.7983857823</v>
-      </c>
-      <c r="M44">
-        <v>19297.530489448101</v>
-      </c>
-      <c r="N44">
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A45" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A47" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G47" s="4"/>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A48" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C48">
+        <v>0</v>
+      </c>
+      <c r="D48">
+        <v>116861.67991782499</v>
+      </c>
+      <c r="E48">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F48">
+        <v>0.84490020632262297</v>
+      </c>
+      <c r="G48">
+        <v>23556.420831705898</v>
+      </c>
+      <c r="H48">
+        <v>6947.4542183048998</v>
+      </c>
+      <c r="I48">
+        <v>913.29198665996</v>
+      </c>
+      <c r="J48">
+        <v>31417.167036670799</v>
+      </c>
+      <c r="K48">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L48">
+        <v>15303.798385783</v>
+      </c>
+      <c r="M48">
+        <v>19297.5304894482</v>
+      </c>
+      <c r="N48">
         <v>992.31070788530405</v>
       </c>
-      <c r="O44">
-        <v>0</v>
-      </c>
-      <c r="P44">
-        <v>238584.402120479</v>
-      </c>
-      <c r="Q44">
-        <v>1108.83163779344</v>
-      </c>
-      <c r="R44">
-        <v>0</v>
-      </c>
-      <c r="S44">
-        <v>230512.59606633501</v>
-      </c>
-      <c r="T44">
-        <v>1103.3673370121001</v>
-      </c>
-    </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+      <c r="O48">
+        <v>0</v>
+      </c>
+      <c r="P48">
+        <v>238413.66244470701</v>
+      </c>
+      <c r="Q48">
+        <v>1102.6552392369899</v>
+      </c>
+      <c r="R48">
+        <v>0</v>
+      </c>
+      <c r="S48">
+        <v>0</v>
+      </c>
+      <c r="T48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A49" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B45" t="s">
-        <v>21</v>
-      </c>
-      <c r="C45">
-        <v>0</v>
-      </c>
-      <c r="D45">
-        <v>171564.02128394699</v>
-      </c>
-      <c r="E45">
-        <v>282179.67123287701</v>
-      </c>
-      <c r="F45">
-        <v>1.03875662810921</v>
-      </c>
-      <c r="G45">
-        <v>73514.1870928641</v>
-      </c>
-      <c r="H45">
-        <v>7482.8438362204697</v>
-      </c>
-      <c r="I45">
-        <v>4044.9309872213798</v>
-      </c>
-      <c r="J45">
-        <v>85041.961916305998</v>
-      </c>
-      <c r="K45">
-        <v>51119.832654572398</v>
-      </c>
-      <c r="L45">
-        <v>16047.2916290263</v>
-      </c>
-      <c r="M45">
-        <v>19354.9350840429</v>
-      </c>
-      <c r="N45">
+      <c r="B49" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C49">
+        <v>0</v>
+      </c>
+      <c r="D49">
+        <v>187020.456722612</v>
+      </c>
+      <c r="E49">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F49">
+        <v>1.09353178385</v>
+      </c>
+      <c r="G49">
+        <v>89520.694507565597</v>
+      </c>
+      <c r="H49">
+        <v>6971.3813103080802</v>
+      </c>
+      <c r="I49">
+        <v>5083.8680235841202</v>
+      </c>
+      <c r="J49">
+        <v>101575.943841457</v>
+      </c>
+      <c r="K49">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L49">
+        <v>15303.798385783</v>
+      </c>
+      <c r="M49">
+        <v>19297.5304894482</v>
+      </c>
+      <c r="N49">
         <v>992.31070788530405</v>
       </c>
-      <c r="O45">
-        <v>0</v>
-      </c>
-      <c r="P45">
-        <v>293116.00381082902</v>
-      </c>
-      <c r="Q45">
-        <v>1187.62883512946</v>
-      </c>
-      <c r="R45">
-        <v>9393.8913494494009</v>
-      </c>
-      <c r="S45">
-        <v>260.94142637359403</v>
-      </c>
-      <c r="T45">
-        <v>-3.6405201993767098</v>
-      </c>
-    </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="G46" s="4"/>
-    </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B47" t="s">
-        <v>21</v>
-      </c>
-      <c r="C47">
-        <v>4</v>
-      </c>
-      <c r="D47">
-        <v>116833.749486644</v>
-      </c>
-      <c r="E47">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F47">
-        <v>0.84480122530439805</v>
-      </c>
-      <c r="G47" s="4">
-        <v>23535.478746437901</v>
-      </c>
-      <c r="H47">
-        <v>6941.2778055266899</v>
-      </c>
-      <c r="I47">
-        <v>912.48005352310201</v>
-      </c>
-      <c r="J47">
-        <v>31389.236605487698</v>
-      </c>
-      <c r="K47">
-        <v>50843.184005923998</v>
-      </c>
-      <c r="L47">
-        <v>15303.798385784499</v>
-      </c>
-      <c r="M47">
-        <v>19297.5304894484</v>
-      </c>
-      <c r="N47">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O47">
-        <v>0</v>
-      </c>
-      <c r="P47">
-        <v>0</v>
-      </c>
-      <c r="Q47">
-        <v>0</v>
-      </c>
-      <c r="R47">
-        <v>0</v>
-      </c>
-      <c r="S47">
-        <v>0</v>
-      </c>
-      <c r="T47">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>22</v>
-      </c>
-      <c r="B48" t="s">
-        <v>21</v>
-      </c>
-      <c r="C48">
-        <v>4</v>
-      </c>
-      <c r="D48">
-        <v>124393.533174422</v>
-      </c>
-      <c r="E48">
-        <v>282179.67123444699</v>
-      </c>
-      <c r="F48">
-        <v>0.87159189967643702</v>
-      </c>
-      <c r="G48" s="4">
-        <v>21072.189860718699</v>
-      </c>
-      <c r="H48">
-        <v>9188.7245080883695</v>
-      </c>
-      <c r="I48">
-        <v>2618.8827210474601</v>
-      </c>
-      <c r="J48">
-        <v>32879.797089854597</v>
-      </c>
-      <c r="K48">
-        <v>50904.118537438801</v>
-      </c>
-      <c r="L48">
-        <v>20591.7266090095</v>
-      </c>
-      <c r="M48">
-        <v>20017.890938119701</v>
-      </c>
-      <c r="N48">
-        <v>1040.9289460857101</v>
-      </c>
-      <c r="O48">
-        <v>0</v>
-      </c>
-      <c r="P48">
-        <v>245945.51570130399</v>
-      </c>
-      <c r="Q48">
-        <v>1458.3752411216699</v>
-      </c>
-      <c r="R48">
-        <v>35012.612233571497</v>
-      </c>
-      <c r="S48">
-        <v>875.31530583928895</v>
-      </c>
-      <c r="T48">
-        <v>0.51444695802960605</v>
+      <c r="O49">
+        <v>0</v>
+      </c>
+      <c r="P49">
+        <v>308572.439249494</v>
+      </c>
+      <c r="Q49">
+        <v>1106.4527933521999</v>
+      </c>
+      <c r="R49">
+        <v>3451.9307168288801</v>
+      </c>
+      <c r="S49">
+        <v>20.547206647791</v>
+      </c>
+      <c r="T49">
+        <v>-14.696886263168601</v>
       </c>
     </row>
     <row r="50" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A50" s="1" t="s">
-        <v>30</v>
-      </c>
+      <c r="A50" s="3"/>
       <c r="G50" s="4"/>
     </row>
     <row r="51" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B51" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C51">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D51">
-        <v>115472.147206908</v>
+        <v>117032.41959359701</v>
       </c>
       <c r="E51">
-        <v>282495</v>
+        <v>282179.67123286898</v>
       </c>
       <c r="F51">
-        <v>0.83903831831993503</v>
+        <v>0.845505280653571</v>
       </c>
       <c r="G51" s="4">
-        <v>20221.889710343999</v>
+        <v>23683.129427060001</v>
       </c>
       <c r="H51">
-        <v>6553.7440767980397</v>
+        <v>6986.3695969997798</v>
       </c>
       <c r="I51">
-        <v>6160.4249909476703</v>
+        <v>918.40768838365295</v>
       </c>
       <c r="J51">
-        <v>32936.058778089697</v>
+        <v>31587.906712443499</v>
       </c>
       <c r="K51">
-        <v>50939.5611113743</v>
+        <v>50843.1840059237</v>
       </c>
       <c r="L51">
-        <v>15427.2204868183</v>
+        <v>15303.7983857823</v>
       </c>
       <c r="M51">
-        <v>19327.3039306102</v>
+        <v>19297.530489448101</v>
       </c>
       <c r="N51">
-        <v>1004.9477757237401</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O51">
-        <v>3157.9970999842499</v>
+        <v>0</v>
       </c>
       <c r="P51">
-        <v>237024.12973379</v>
+        <v>238584.402120479</v>
       </c>
       <c r="Q51">
-        <v>1464.2687322859999</v>
+        <v>1108.83163779344</v>
       </c>
       <c r="R51">
-        <v>8672.9882445954008</v>
+        <v>0</v>
       </c>
       <c r="S51">
-        <v>346.91952978381602</v>
+        <v>230512.59606633501</v>
       </c>
       <c r="T51">
-        <v>2.4302910949698302</v>
+        <v>1103.3673370121001</v>
       </c>
     </row>
     <row r="52" spans="1:20" x14ac:dyDescent="0.35">
@@ -3291,249 +3068,256 @@
         <v>22</v>
       </c>
       <c r="B52" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52">
+        <v>171564.02128394699</v>
+      </c>
+      <c r="E52">
+        <v>282179.67123287701</v>
+      </c>
+      <c r="F52">
+        <v>1.03875662810921</v>
+      </c>
+      <c r="G52">
+        <v>73514.1870928641</v>
+      </c>
+      <c r="H52">
+        <v>7482.8438362204697</v>
+      </c>
+      <c r="I52">
+        <v>4044.9309872213798</v>
+      </c>
+      <c r="J52">
+        <v>85041.961916305998</v>
+      </c>
+      <c r="K52">
+        <v>51119.832654572398</v>
+      </c>
+      <c r="L52">
+        <v>16047.2916290263</v>
+      </c>
+      <c r="M52">
+        <v>19354.9350840429</v>
+      </c>
+      <c r="N52">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O52">
+        <v>0</v>
+      </c>
+      <c r="P52">
+        <v>293116.00381082902</v>
+      </c>
+      <c r="Q52">
+        <v>1187.62883512946</v>
+      </c>
+      <c r="R52">
+        <v>9393.8913494494009</v>
+      </c>
+      <c r="S52">
+        <v>260.94142637359403</v>
+      </c>
+      <c r="T52">
+        <v>-3.6405201993767098</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="G53" s="4"/>
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A54" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B54" t="s">
+        <v>21</v>
+      </c>
+      <c r="C54">
         <v>4</v>
       </c>
-      <c r="D52">
-        <v>108958.027502652</v>
-      </c>
-      <c r="E52">
+      <c r="D54">
+        <v>116833.749486644</v>
+      </c>
+      <c r="E54">
         <v>282179.67123287602</v>
       </c>
-      <c r="F52">
-        <v>0.81689091571482797</v>
-      </c>
-      <c r="G52" s="4">
-        <v>20285.098342207999</v>
-      </c>
-      <c r="H52">
-        <v>6552.6722224723899</v>
-      </c>
-      <c r="I52">
-        <v>6068.9240568166097</v>
-      </c>
-      <c r="J52">
-        <v>32906.694621497001</v>
-      </c>
-      <c r="K52">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L52">
-        <v>16378.7983857829</v>
-      </c>
-      <c r="M52">
-        <v>19449.350489448301</v>
-      </c>
-      <c r="N52">
-        <v>1004.9477757237401</v>
-      </c>
-      <c r="O52">
-        <v>10620</v>
-      </c>
-      <c r="P52">
-        <v>230510.010029533</v>
-      </c>
-      <c r="Q52">
-        <v>1464.02925348484</v>
-      </c>
-      <c r="R52">
-        <v>26064.489084194902</v>
-      </c>
-      <c r="S52">
-        <v>407.257641940545</v>
-      </c>
-      <c r="T52">
-        <v>1.09609872121186</v>
-      </c>
-    </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A54" s="1" t="s">
-        <v>31</v>
+      <c r="F54">
+        <v>0.84480122530439805</v>
+      </c>
+      <c r="G54" s="4">
+        <v>23535.478746437901</v>
+      </c>
+      <c r="H54">
+        <v>6941.2778055266899</v>
+      </c>
+      <c r="I54">
+        <v>912.48005352310201</v>
+      </c>
+      <c r="J54">
+        <v>31389.236605487698</v>
+      </c>
+      <c r="K54">
+        <v>50843.184005923998</v>
+      </c>
+      <c r="L54">
+        <v>15303.798385784499</v>
+      </c>
+      <c r="M54">
+        <v>19297.5304894484</v>
+      </c>
+      <c r="N54">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O54">
+        <v>0</v>
+      </c>
+      <c r="P54">
+        <v>0</v>
+      </c>
+      <c r="Q54">
+        <v>0</v>
+      </c>
+      <c r="R54">
+        <v>0</v>
+      </c>
+      <c r="S54">
+        <v>0</v>
+      </c>
+      <c r="T54">
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A55" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>23</v>
+      <c r="A55" t="s">
+        <v>22</v>
+      </c>
+      <c r="B55" t="s">
+        <v>21</v>
       </c>
       <c r="C55">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D55">
-        <v>115030.978322179</v>
+        <v>124393.533174422</v>
       </c>
       <c r="E55">
-        <v>282179.67123287602</v>
+        <v>282179.67123444699</v>
       </c>
       <c r="F55">
-        <v>0.83841249022441</v>
-      </c>
-      <c r="G55">
-        <v>20114.092712805999</v>
+        <v>0.87159189967643702</v>
+      </c>
+      <c r="G55" s="4">
+        <v>21072.189860718699</v>
       </c>
       <c r="H55">
-        <v>6942.2846600808298</v>
+        <v>9188.7245080883695</v>
       </c>
       <c r="I55">
-        <v>2530.0880681377598</v>
+        <v>2618.8827210474601</v>
       </c>
       <c r="J55">
-        <v>29586.4654410246</v>
+        <v>32879.797089854597</v>
       </c>
       <c r="K55">
-        <v>50843.184005923598</v>
+        <v>50904.118537438801</v>
       </c>
       <c r="L55">
-        <v>15303.798385783</v>
+        <v>20591.7266090095</v>
       </c>
       <c r="M55">
-        <v>19297.5304894482</v>
+        <v>20017.890938119701</v>
       </c>
       <c r="N55">
-        <v>992.31070788530405</v>
+        <v>1040.9289460857101</v>
       </c>
       <c r="O55">
         <v>0</v>
       </c>
       <c r="P55">
-        <v>236582.960849061</v>
+        <v>245945.51570130399</v>
       </c>
       <c r="Q55">
-        <v>1101.8347602124099</v>
+        <v>1458.3752411216699</v>
       </c>
       <c r="R55">
-        <v>0</v>
+        <v>35012.612233571497</v>
       </c>
       <c r="S55">
-        <v>0</v>
+        <v>875.31530583928895</v>
       </c>
       <c r="T55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A56" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C56">
-        <v>0</v>
-      </c>
-      <c r="D56">
-        <v>124771.246709449</v>
-      </c>
-      <c r="E56">
-        <v>282179.67125180899</v>
-      </c>
-      <c r="F56">
-        <v>0.87293045648394496</v>
-      </c>
-      <c r="G56">
-        <v>22626.697961956499</v>
-      </c>
-      <c r="H56">
-        <v>7102.5767129513297</v>
-      </c>
-      <c r="I56">
-        <v>9597.4591384874802</v>
-      </c>
-      <c r="J56">
-        <v>39326.733813395302</v>
-      </c>
-      <c r="K56">
-        <v>50843.184011688398</v>
-      </c>
-      <c r="L56">
-        <v>15303.798393134501</v>
-      </c>
-      <c r="M56">
-        <v>19297.530491231599</v>
-      </c>
-      <c r="N56">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O56">
-        <v>0</v>
-      </c>
-      <c r="P56">
-        <v>246323.22923633101</v>
-      </c>
-      <c r="Q56">
-        <v>1127.27501714903</v>
-      </c>
-      <c r="R56">
-        <v>0</v>
-      </c>
-      <c r="S56">
-        <v>0</v>
-      </c>
-      <c r="T56">
-        <v>0</v>
+        <v>0.51444695802960605</v>
       </c>
     </row>
     <row r="57" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A57" s="1"/>
+      <c r="A57" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G57" s="4"/>
     </row>
     <row r="58" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B58" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C58">
         <v>2</v>
       </c>
       <c r="D58">
-        <v>115714.10508262301</v>
+        <v>115472.147206908</v>
       </c>
       <c r="E58">
-        <v>282179.67125387199</v>
+        <v>282495</v>
       </c>
       <c r="F58">
-        <v>0.840833383054163</v>
+        <v>0.83903831831993503</v>
       </c>
       <c r="G58" s="4">
-        <v>20578.507216446698</v>
+        <v>20221.889710343999</v>
       </c>
       <c r="H58">
-        <v>7102.57515066207</v>
+        <v>6553.7440767980397</v>
       </c>
       <c r="I58">
-        <v>2588.5052959285099</v>
+        <v>6160.4249909476703</v>
       </c>
       <c r="J58">
-        <v>30269.587663037299</v>
+        <v>32936.058778089697</v>
       </c>
       <c r="K58">
-        <v>50843.185173268597</v>
+        <v>50939.5611113743</v>
       </c>
       <c r="L58">
-        <v>15303.8015139941</v>
+        <v>15427.2204868183</v>
       </c>
       <c r="M58">
-        <v>19297.530732323401</v>
+        <v>19327.3039306102</v>
       </c>
       <c r="N58">
-        <v>992.31070788530405</v>
+        <v>1004.9477757237401</v>
       </c>
       <c r="O58">
-        <v>0</v>
+        <v>3157.9970999842499</v>
       </c>
       <c r="P58">
-        <v>237266.08760950499</v>
+        <v>237024.12973379</v>
       </c>
       <c r="Q58">
-        <v>1127.2750356983099</v>
+        <v>1464.2687322859999</v>
       </c>
       <c r="R58">
-        <v>0</v>
+        <v>8672.9882445954008</v>
+      </c>
+      <c r="S58">
+        <v>346.91952978381602</v>
+      </c>
+      <c r="T58">
+        <v>2.4302910949698302</v>
       </c>
     </row>
     <row r="59" spans="1:20" x14ac:dyDescent="0.35">
@@ -3541,250 +3325,249 @@
         <v>22</v>
       </c>
       <c r="B59" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C59">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D59">
-        <v>120628.41082793</v>
+        <v>108958.027502652</v>
       </c>
       <c r="E59">
         <v>282179.67123287602</v>
       </c>
       <c r="F59">
-        <v>0.85824890324911396</v>
+        <v>0.81689091571482797</v>
       </c>
       <c r="G59" s="4">
-        <v>20824.7129679639</v>
+        <v>20285.098342207999</v>
       </c>
       <c r="H59">
-        <v>7456.39074483072</v>
+        <v>6552.6722224723899</v>
       </c>
       <c r="I59">
-        <v>5114.4587365303096</v>
+        <v>6068.9240568166097</v>
       </c>
       <c r="J59">
-        <v>33395.562449324898</v>
+        <v>32906.694621497001</v>
       </c>
       <c r="K59">
-        <v>51302.320205525801</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L59">
-        <v>16537.7269222135</v>
+        <v>16378.7983857829</v>
       </c>
       <c r="M59">
-        <v>19392.801250865799</v>
+        <v>19449.350489448301</v>
       </c>
       <c r="N59">
         <v>1004.9477757237401</v>
       </c>
       <c r="O59">
-        <v>0</v>
+        <v>10620</v>
       </c>
       <c r="P59">
-        <v>242180.39335481101</v>
+        <v>230510.010029533</v>
       </c>
       <c r="Q59">
-        <v>1183.4303612998101</v>
+        <v>1464.02925348484</v>
       </c>
       <c r="R59">
-        <v>15931.1957490451</v>
+        <v>26064.489084194902</v>
       </c>
       <c r="S59">
-        <v>346.33034237054602</v>
+        <v>407.257641940545</v>
       </c>
       <c r="T59">
-        <v>1.0959871186973</v>
+        <v>1.09609872121186</v>
       </c>
     </row>
     <row r="61" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
+      <c r="A61" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="62" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A62" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B61" t="s">
-        <v>21</v>
-      </c>
-      <c r="C61">
-        <v>4</v>
-      </c>
-      <c r="D61">
-        <v>115714.10508261999</v>
-      </c>
-      <c r="E61">
-        <v>282179.671253876</v>
-      </c>
-      <c r="F61">
-        <v>0.84083338305413902</v>
-      </c>
-      <c r="G61" s="4">
-        <v>20578.5072164468</v>
-      </c>
-      <c r="H61">
-        <v>7102.5751506616798</v>
-      </c>
-      <c r="I61">
-        <v>2588.50529592865</v>
-      </c>
-      <c r="J61">
-        <v>30269.587663037099</v>
-      </c>
-      <c r="K61">
-        <v>50843.185173268197</v>
-      </c>
-      <c r="L61">
-        <v>15303.8015139912</v>
-      </c>
-      <c r="M61">
-        <v>19297.530732323299</v>
-      </c>
-      <c r="N61">
+      <c r="B62" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C62">
+        <v>0</v>
+      </c>
+      <c r="D62">
+        <v>115030.978322179</v>
+      </c>
+      <c r="E62">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F62">
+        <v>0.83841249022441</v>
+      </c>
+      <c r="G62">
+        <v>20114.092712805999</v>
+      </c>
+      <c r="H62">
+        <v>6942.2846600808298</v>
+      </c>
+      <c r="I62">
+        <v>2530.0880681377598</v>
+      </c>
+      <c r="J62">
+        <v>29586.4654410246</v>
+      </c>
+      <c r="K62">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L62">
+        <v>15303.798385783</v>
+      </c>
+      <c r="M62">
+        <v>19297.5304894482</v>
+      </c>
+      <c r="N62">
         <v>992.31070788530405</v>
       </c>
-      <c r="O61">
-        <v>0</v>
-      </c>
-      <c r="P61">
-        <v>237266.087609501</v>
-      </c>
-      <c r="Q61">
-        <v>1127.2750356983499</v>
-      </c>
-      <c r="R61">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
+      <c r="O62">
+        <v>0</v>
+      </c>
+      <c r="P62">
+        <v>236582.960849061</v>
+      </c>
+      <c r="Q62">
+        <v>1101.8347602124099</v>
+      </c>
+      <c r="R62">
+        <v>0</v>
+      </c>
+      <c r="S62">
+        <v>0</v>
+      </c>
+      <c r="T62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A63" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B62" t="s">
-        <v>21</v>
-      </c>
-      <c r="C62">
-        <v>4</v>
-      </c>
-      <c r="D62">
-        <v>120375.156660901</v>
-      </c>
-      <c r="E62">
-        <v>282179.671232878</v>
-      </c>
-      <c r="F62">
-        <v>0.857351410648304</v>
-      </c>
-      <c r="G62" s="4">
-        <v>21285.1004075495</v>
-      </c>
-      <c r="H62">
-        <v>7426.32532798384</v>
-      </c>
-      <c r="I62">
-        <v>5046.79446201879</v>
-      </c>
-      <c r="J62">
-        <v>33758.220197552102</v>
-      </c>
-      <c r="K62">
-        <v>51144.191344099498</v>
-      </c>
-      <c r="L62">
-        <v>16112.7556071296</v>
-      </c>
-      <c r="M62">
-        <v>19359.989512119799</v>
-      </c>
-      <c r="N62">
-        <v>1006.77939378399</v>
-      </c>
-      <c r="O62">
-        <v>0</v>
-      </c>
-      <c r="P62">
-        <v>241927.13918778201</v>
-      </c>
-      <c r="Q62">
-        <v>1178.65858109644</v>
-      </c>
-      <c r="R62">
-        <v>12586.325853030899</v>
-      </c>
-      <c r="S62">
-        <v>466.16021677892502</v>
-      </c>
-      <c r="T62">
-        <v>1.3585822738026401</v>
-      </c>
-    </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="G63" s="4"/>
+      <c r="B63" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C63">
+        <v>0</v>
+      </c>
+      <c r="D63">
+        <v>124771.246709449</v>
+      </c>
+      <c r="E63">
+        <v>282179.67125180899</v>
+      </c>
+      <c r="F63">
+        <v>0.87293045648394496</v>
+      </c>
+      <c r="G63">
+        <v>22626.697961956499</v>
+      </c>
+      <c r="H63">
+        <v>7102.5767129513297</v>
+      </c>
+      <c r="I63">
+        <v>9597.4591384874802</v>
+      </c>
+      <c r="J63">
+        <v>39326.733813395302</v>
+      </c>
+      <c r="K63">
+        <v>50843.184011688398</v>
+      </c>
+      <c r="L63">
+        <v>15303.798393134501</v>
+      </c>
+      <c r="M63">
+        <v>19297.530491231599</v>
+      </c>
+      <c r="N63">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O63">
+        <v>0</v>
+      </c>
+      <c r="P63">
+        <v>246323.22923633101</v>
+      </c>
+      <c r="Q63">
+        <v>1127.27501714903</v>
+      </c>
+      <c r="R63">
+        <v>0</v>
+      </c>
+      <c r="S63">
+        <v>0</v>
+      </c>
+      <c r="T63">
+        <v>0</v>
+      </c>
     </row>
     <row r="64" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A64" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G64" s="4"/>
+      <c r="A64" s="1"/>
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B65" t="s">
         <v>21</v>
       </c>
       <c r="C65">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D65">
-        <v>146108.01933512901</v>
+        <v>115714.10508262301</v>
       </c>
       <c r="E65">
-        <v>355610.364944759</v>
+        <v>282179.67125387199</v>
       </c>
       <c r="F65">
-        <v>0.75267772890587503</v>
-      </c>
-      <c r="G65">
-        <v>25765.651662743599</v>
+        <v>0.840833383054163</v>
+      </c>
+      <c r="G65" s="4">
+        <v>20578.507216446698</v>
       </c>
       <c r="H65">
-        <v>7150.9042815892099</v>
+        <v>7102.57515066207</v>
       </c>
       <c r="I65">
-        <v>5144.3184852884797</v>
+        <v>2588.5052959285099</v>
       </c>
       <c r="J65">
-        <v>38060.874429621297</v>
+        <v>30269.587663037299</v>
       </c>
       <c r="K65">
-        <v>64168.339029134899</v>
+        <v>50843.185173268597</v>
       </c>
       <c r="L65">
-        <v>19539.954214541001</v>
+        <v>15303.8015139941</v>
       </c>
       <c r="M65">
-        <v>24338.851661831999</v>
+        <v>19297.530732323401</v>
       </c>
       <c r="N65">
-        <v>1010.46273302954</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O65">
         <v>0</v>
       </c>
       <c r="P65">
-        <v>267660.00186201098</v>
+        <v>237266.08760950499</v>
       </c>
       <c r="Q65">
-        <v>1597.68911089628</v>
+        <v>1127.2750356983099</v>
       </c>
       <c r="R65">
-        <v>13084.0423994256</v>
-      </c>
-      <c r="S65">
-        <v>467.28722855091399</v>
-      </c>
-      <c r="T65">
-        <v>-0.25904927491985202</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.35">
@@ -3792,637 +3575,888 @@
         <v>22</v>
       </c>
       <c r="B66" t="s">
-        <v>35</v>
-      </c>
-      <c r="C66" t="s">
-        <v>35</v>
-      </c>
-      <c r="D66" t="s">
-        <v>36</v>
-      </c>
-      <c r="E66" t="s">
-        <v>36</v>
-      </c>
-      <c r="F66" t="s">
-        <v>36</v>
+        <v>21</v>
+      </c>
+      <c r="C66">
+        <v>2</v>
+      </c>
+      <c r="D66">
+        <v>120628.41082793</v>
+      </c>
+      <c r="E66">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F66">
+        <v>0.85824890324911396</v>
       </c>
       <c r="G66" s="4">
-        <v>28838</v>
+        <v>20824.7129679639</v>
       </c>
       <c r="H66">
-        <v>7567.5</v>
+        <v>7456.39074483072</v>
       </c>
       <c r="I66">
-        <v>13764.1</v>
+        <v>5114.4587365303096</v>
       </c>
       <c r="J66">
-        <v>50169.7</v>
-      </c>
-      <c r="K66" t="s">
-        <v>36</v>
-      </c>
-      <c r="L66" t="s">
-        <v>36</v>
-      </c>
-      <c r="M66" t="s">
-        <v>36</v>
-      </c>
-      <c r="N66" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="68" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G68" s="4"/>
-      <c r="P68" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q68" t="s">
-        <v>16</v>
-      </c>
-      <c r="R68" t="s">
-        <v>17</v>
-      </c>
-      <c r="S68" t="s">
-        <v>18</v>
-      </c>
-      <c r="T68" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="69" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+        <v>33395.562449324898</v>
+      </c>
+      <c r="K66">
+        <v>51302.320205525801</v>
+      </c>
+      <c r="L66">
+        <v>16537.7269222135</v>
+      </c>
+      <c r="M66">
+        <v>19392.801250865799</v>
+      </c>
+      <c r="N66">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O66">
+        <v>0</v>
+      </c>
+      <c r="P66">
+        <v>242180.39335481101</v>
+      </c>
+      <c r="Q66">
+        <v>1183.4303612998101</v>
+      </c>
+      <c r="R66">
+        <v>15931.1957490451</v>
+      </c>
+      <c r="S66">
+        <v>346.33034237054602</v>
+      </c>
+      <c r="T66">
+        <v>1.0959871186973</v>
+      </c>
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>20</v>
+      </c>
+      <c r="B68" t="s">
+        <v>21</v>
+      </c>
+      <c r="C68">
+        <v>4</v>
+      </c>
+      <c r="D68">
+        <v>115714.10508261999</v>
+      </c>
+      <c r="E68">
+        <v>282179.671253876</v>
+      </c>
+      <c r="F68">
+        <v>0.84083338305413902</v>
+      </c>
+      <c r="G68" s="4">
+        <v>20578.5072164468</v>
+      </c>
+      <c r="H68">
+        <v>7102.5751506616798</v>
+      </c>
+      <c r="I68">
+        <v>2588.50529592865</v>
+      </c>
+      <c r="J68">
+        <v>30269.587663037099</v>
+      </c>
+      <c r="K68">
+        <v>50843.185173268197</v>
+      </c>
+      <c r="L68">
+        <v>15303.8015139912</v>
+      </c>
+      <c r="M68">
+        <v>19297.530732323299</v>
+      </c>
+      <c r="N68">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O68">
+        <v>0</v>
+      </c>
+      <c r="P68">
+        <v>237266.087609501</v>
+      </c>
+      <c r="Q68">
+        <v>1127.2750356983499</v>
+      </c>
+      <c r="R68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="B69" t="s">
-        <v>1</v>
-      </c>
-      <c r="C69" t="s">
-        <v>2</v>
-      </c>
-      <c r="D69" t="s">
-        <v>3</v>
-      </c>
-      <c r="E69" t="s">
+        <v>21</v>
+      </c>
+      <c r="C69">
         <v>4</v>
       </c>
-      <c r="F69" t="s">
-        <v>5</v>
-      </c>
-      <c r="G69" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H69" t="s">
-        <v>7</v>
-      </c>
-      <c r="I69" t="s">
-        <v>8</v>
-      </c>
-      <c r="J69" t="s">
-        <v>9</v>
-      </c>
-      <c r="K69" t="s">
-        <v>10</v>
-      </c>
-      <c r="L69" t="s">
-        <v>11</v>
-      </c>
-      <c r="M69" t="s">
-        <v>12</v>
-      </c>
-      <c r="N69" t="s">
-        <v>13</v>
-      </c>
-      <c r="O69" t="s">
-        <v>14</v>
+      <c r="D69">
+        <v>120375.156660901</v>
+      </c>
+      <c r="E69">
+        <v>282179.671232878</v>
+      </c>
+      <c r="F69">
+        <v>0.857351410648304</v>
+      </c>
+      <c r="G69" s="4">
+        <v>21285.1004075495</v>
+      </c>
+      <c r="H69">
+        <v>7426.32532798384</v>
+      </c>
+      <c r="I69">
+        <v>5046.79446201879</v>
+      </c>
+      <c r="J69">
+        <v>33758.220197552102</v>
+      </c>
+      <c r="K69">
+        <v>51144.191344099498</v>
+      </c>
+      <c r="L69">
+        <v>16112.7556071296</v>
+      </c>
+      <c r="M69">
+        <v>19359.989512119799</v>
+      </c>
+      <c r="N69">
+        <v>1006.77939378399</v>
+      </c>
+      <c r="O69">
+        <v>0</v>
       </c>
       <c r="P69">
-        <v>63734.6679</v>
+        <v>241927.13918778201</v>
       </c>
       <c r="Q69">
-        <v>1078.4492829999999</v>
+        <v>1178.65858109644</v>
       </c>
       <c r="R69">
-        <v>624.70352849999995</v>
+        <v>12586.325853030899</v>
       </c>
       <c r="S69">
-        <v>13.014656840000001</v>
+        <v>466.16021677892502</v>
       </c>
       <c r="T69">
-        <v>27.514184579999998</v>
-      </c>
-    </row>
-    <row r="70" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B70" t="s">
+        <v>1.3585822738026401</v>
+      </c>
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="G70" s="4"/>
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A71" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G71" s="4"/>
+    </row>
+    <row r="72" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>22</v>
+      </c>
+      <c r="B72" t="s">
         <v>21</v>
       </c>
-      <c r="C70">
+      <c r="C72">
         <v>4</v>
       </c>
-      <c r="D70">
-        <v>29525.427309999999</v>
-      </c>
-      <c r="E70">
-        <v>80391.755990000005</v>
-      </c>
-      <c r="F70">
-        <v>0.79280104200000001</v>
-      </c>
-      <c r="G70" s="4">
-        <v>5050.6365619999997</v>
-      </c>
-      <c r="H70">
-        <v>4678.3390820000004</v>
-      </c>
-      <c r="I70">
-        <v>2508.6600360000002</v>
-      </c>
-      <c r="J70">
-        <v>12237.635679999999</v>
-      </c>
-      <c r="K70">
-        <v>13920</v>
-      </c>
-      <c r="L70">
-        <v>2841.544922</v>
-      </c>
-      <c r="M70">
-        <v>5380.5444360000001</v>
-      </c>
-      <c r="N70">
-        <v>279.27307350000001</v>
-      </c>
-      <c r="O70">
-        <v>0</v>
-      </c>
-      <c r="P70">
-        <v>64865.028310000002</v>
-      </c>
-      <c r="Q70">
-        <v>1191.7509680000001</v>
-      </c>
-      <c r="R70">
-        <v>7243.7162129999997</v>
-      </c>
-      <c r="S70">
-        <v>452.7322633</v>
-      </c>
-      <c r="T70">
-        <v>5.8154128590000003</v>
-      </c>
-    </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A71" s="7" t="s">
-        <v>37</v>
+      <c r="D72">
+        <v>146108.01933512901</v>
+      </c>
+      <c r="E72">
+        <v>355610.364944759</v>
+      </c>
+      <c r="F72">
+        <v>0.75267772890587503</v>
+      </c>
+      <c r="G72">
+        <v>25765.651662743599</v>
+      </c>
+      <c r="H72">
+        <v>7150.9042815892099</v>
+      </c>
+      <c r="I72">
+        <v>5144.3184852884797</v>
+      </c>
+      <c r="J72">
+        <v>38060.874429621297</v>
+      </c>
+      <c r="K72">
+        <v>64168.339029134899</v>
+      </c>
+      <c r="L72">
+        <v>19539.954214541001</v>
+      </c>
+      <c r="M72">
+        <v>24338.851661831999</v>
+      </c>
+      <c r="N72">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O72">
+        <v>0</v>
+      </c>
+      <c r="P72">
+        <v>267660.00186201098</v>
+      </c>
+      <c r="Q72">
+        <v>1597.68911089628</v>
+      </c>
+      <c r="R72">
+        <v>13084.0423994256</v>
+      </c>
+      <c r="S72">
+        <v>467.28722855091399</v>
+      </c>
+      <c r="T72">
+        <v>-0.25904927491985202</v>
       </c>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
+        <v>22</v>
+      </c>
+      <c r="B73" t="s">
+        <v>35</v>
+      </c>
+      <c r="C73" t="s">
+        <v>35</v>
+      </c>
+      <c r="D73" t="s">
+        <v>36</v>
+      </c>
+      <c r="E73" t="s">
+        <v>36</v>
+      </c>
+      <c r="F73" t="s">
+        <v>36</v>
+      </c>
+      <c r="G73" s="4">
+        <v>28838</v>
+      </c>
+      <c r="H73">
+        <v>7567.5</v>
+      </c>
+      <c r="I73">
+        <v>13764.1</v>
+      </c>
+      <c r="J73">
+        <v>50169.7</v>
+      </c>
+      <c r="K73" t="s">
+        <v>36</v>
+      </c>
+      <c r="L73" t="s">
+        <v>36</v>
+      </c>
+      <c r="M73" t="s">
+        <v>36</v>
+      </c>
+      <c r="N73" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="75" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A75" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G75" s="4"/>
+      <c r="P75" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q75" t="s">
+        <v>16</v>
+      </c>
+      <c r="R75" t="s">
+        <v>17</v>
+      </c>
+      <c r="S75" t="s">
+        <v>18</v>
+      </c>
+      <c r="T75" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="76" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>0</v>
+      </c>
+      <c r="B76" t="s">
+        <v>1</v>
+      </c>
+      <c r="C76" t="s">
+        <v>2</v>
+      </c>
+      <c r="D76" t="s">
+        <v>3</v>
+      </c>
+      <c r="E76" t="s">
+        <v>4</v>
+      </c>
+      <c r="F76" t="s">
+        <v>5</v>
+      </c>
+      <c r="G76" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H76" t="s">
+        <v>7</v>
+      </c>
+      <c r="I76" t="s">
+        <v>8</v>
+      </c>
+      <c r="J76" t="s">
+        <v>9</v>
+      </c>
+      <c r="K76" t="s">
+        <v>10</v>
+      </c>
+      <c r="L76" t="s">
+        <v>11</v>
+      </c>
+      <c r="M76" t="s">
+        <v>12</v>
+      </c>
+      <c r="N76" t="s">
+        <v>13</v>
+      </c>
+      <c r="O76" t="s">
+        <v>14</v>
+      </c>
+      <c r="P76">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q76">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R76">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S76">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T76">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="77" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B77" t="s">
+        <v>21</v>
+      </c>
+      <c r="C77">
+        <v>4</v>
+      </c>
+      <c r="D77">
+        <v>29525.427309999999</v>
+      </c>
+      <c r="E77">
+        <v>80391.755990000005</v>
+      </c>
+      <c r="F77">
+        <v>0.79280104200000001</v>
+      </c>
+      <c r="G77" s="4">
+        <v>5050.6365619999997</v>
+      </c>
+      <c r="H77">
+        <v>4678.3390820000004</v>
+      </c>
+      <c r="I77">
+        <v>2508.6600360000002</v>
+      </c>
+      <c r="J77">
+        <v>12237.635679999999</v>
+      </c>
+      <c r="K77">
+        <v>13920</v>
+      </c>
+      <c r="L77">
+        <v>2841.544922</v>
+      </c>
+      <c r="M77">
+        <v>5380.5444360000001</v>
+      </c>
+      <c r="N77">
+        <v>279.27307350000001</v>
+      </c>
+      <c r="O77">
+        <v>0</v>
+      </c>
+      <c r="P77">
+        <v>64865.028310000002</v>
+      </c>
+      <c r="Q77">
+        <v>1191.7509680000001</v>
+      </c>
+      <c r="R77">
+        <v>7243.7162129999997</v>
+      </c>
+      <c r="S77">
+        <v>452.7322633</v>
+      </c>
+      <c r="T77">
+        <v>5.8154128590000003</v>
+      </c>
+    </row>
+    <row r="78" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A78" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="80" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
         <v>32</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B80" t="s">
         <v>33</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C80" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A74">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A81">
         <v>20</v>
       </c>
-      <c r="B74">
+      <c r="B81">
         <v>60</v>
       </c>
-      <c r="C74">
+      <c r="C81">
         <v>2</v>
       </c>
-      <c r="D74">
+      <c r="D81">
         <v>119696.652328767</v>
       </c>
-      <c r="E74">
+      <c r="E81">
         <v>282179.67123285501</v>
       </c>
-      <c r="F74">
+      <c r="F81">
         <v>0.854946898908852</v>
       </c>
-      <c r="G74">
+      <c r="G81">
         <v>18681.222424938602</v>
       </c>
-      <c r="H74">
+      <c r="H81">
         <v>5354.6114985546601</v>
       </c>
-      <c r="I74">
+      <c r="I81">
         <v>8156.08309050551</v>
       </c>
-      <c r="J74">
+      <c r="J81">
         <v>32191.917013998798</v>
       </c>
-      <c r="K74">
+      <c r="K81">
         <v>51372.124296964801</v>
       </c>
-      <c r="L74">
+      <c r="L81">
         <v>16725.325417965501</v>
       </c>
-      <c r="M74">
+      <c r="M81">
         <v>19407.285599838699</v>
       </c>
-      <c r="N74">
+      <c r="N81">
         <v>1016.03855436447</v>
       </c>
-      <c r="O74">
-        <v>0</v>
-      </c>
-      <c r="P74">
+      <c r="O81">
+        <v>0</v>
+      </c>
+      <c r="P81">
         <v>241248.634855649</v>
       </c>
-      <c r="Q74">
+      <c r="Q81">
         <v>1192.7637589594799</v>
       </c>
-      <c r="R74">
+      <c r="R81">
         <v>19736.206339365101</v>
       </c>
-      <c r="S74">
+      <c r="S81">
         <v>481.37088632597801</v>
       </c>
-      <c r="T74" s="6">
+      <c r="T81" s="6">
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A75">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A82">
         <v>20</v>
       </c>
-      <c r="B75">
+      <c r="B82">
         <v>50</v>
       </c>
-      <c r="C75">
+      <c r="C82">
         <v>2</v>
       </c>
-      <c r="D75">
+      <c r="D82">
         <v>118381.960809661</v>
       </c>
-      <c r="E75">
+      <c r="E82">
         <v>282254.81855225202</v>
       </c>
-      <c r="F75">
+      <c r="F82">
         <v>0.85006146065890897</v>
       </c>
-      <c r="G75">
+      <c r="G82">
         <v>19407.840072768398</v>
       </c>
-      <c r="H75">
+      <c r="H82">
         <v>5891.8301217549197</v>
       </c>
-      <c r="I75">
+      <c r="I82">
         <v>6659.4942697455399</v>
       </c>
-      <c r="J75">
+      <c r="J82">
         <v>31959.164464268899</v>
       </c>
-      <c r="K75">
+      <c r="K82">
         <v>51102.045942938203</v>
       </c>
-      <c r="L75">
+      <c r="L82">
         <v>15967.176494174801</v>
       </c>
-      <c r="M75">
+      <c r="M82">
         <v>19353.573908279199</v>
       </c>
-      <c r="N75">
+      <c r="N82">
         <v>1010.46273302954</v>
       </c>
-      <c r="O75">
-        <v>0</v>
-      </c>
-      <c r="P75">
+      <c r="O82">
+        <v>0</v>
+      </c>
+      <c r="P82">
         <v>239933.943336542</v>
       </c>
-      <c r="Q75">
+      <c r="Q82">
         <v>1312.43161993582</v>
       </c>
-      <c r="R75">
+      <c r="R82">
         <v>18377.616631847999</v>
       </c>
-      <c r="S75">
+      <c r="S82">
         <v>459.4404157962</v>
       </c>
-      <c r="T75" s="6">
+      <c r="T82" s="6">
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A76">
+    <row r="83" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A83">
         <v>20</v>
       </c>
-      <c r="B76">
+      <c r="B83">
         <v>40</v>
       </c>
-      <c r="C76">
+      <c r="C83">
         <v>2</v>
       </c>
-      <c r="D76">
+      <c r="D83">
         <v>116766.56672038</v>
       </c>
-      <c r="E76">
+      <c r="E83">
         <v>282179.67123287299</v>
       </c>
-      <c r="F76">
+      <c r="F83">
         <v>0.84456314023622803</v>
       </c>
-      <c r="G76">
+      <c r="G83">
         <v>19298.245593088301</v>
       </c>
-      <c r="H76">
+      <c r="H83">
         <v>5682.0016560700296</v>
       </c>
-      <c r="I76">
+      <c r="I83">
         <v>5350.3346939491703</v>
       </c>
-      <c r="J76">
+      <c r="J83">
         <v>30330.5819431075</v>
       </c>
-      <c r="K76">
+      <c r="K83">
         <v>51097.733915068202</v>
       </c>
-      <c r="L76">
+      <c r="L83">
         <v>15987.901266609</v>
       </c>
-      <c r="M76">
+      <c r="M83">
         <v>19350.349595595701</v>
       </c>
-      <c r="N76">
+      <c r="N83">
         <v>1010.46273302954</v>
       </c>
-      <c r="O76">
-        <v>0</v>
-      </c>
-      <c r="P76">
+      <c r="O83">
+        <v>0</v>
+      </c>
+      <c r="P83">
         <v>238318.54924726201</v>
       </c>
-      <c r="Q76">
+      <c r="Q83">
         <v>1265.6913868611</v>
       </c>
-      <c r="R76">
+      <c r="R83">
         <v>17746.163883660702</v>
       </c>
-      <c r="S76">
+      <c r="S83">
         <v>507.03325381887902</v>
       </c>
-      <c r="T76" s="6">
+      <c r="T83" s="6">
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A77">
+    <row r="84" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A84">
         <v>20</v>
       </c>
-      <c r="B77">
+      <c r="B84">
         <v>30</v>
       </c>
-      <c r="C77">
+      <c r="C84">
         <v>2</v>
       </c>
-      <c r="D77">
+      <c r="D84">
         <v>115610.996393592</v>
       </c>
-      <c r="E77">
+      <c r="E84">
         <v>282182.50548365602</v>
       </c>
-      <c r="F77">
+      <c r="F84">
         <v>0.84045954058697003</v>
       </c>
-      <c r="G77">
+      <c r="G84">
         <v>19302.752565837702</v>
       </c>
-      <c r="H77">
+      <c r="H84">
         <v>6226.5181629292701</v>
       </c>
-      <c r="I77">
+      <c r="I84">
         <v>3974.5318253822402</v>
       </c>
-      <c r="J77">
+      <c r="J84">
         <v>29503.802554149199</v>
       </c>
-      <c r="K77">
+      <c r="K84">
         <v>51013.610661725899</v>
       </c>
-      <c r="L77">
+      <c r="L84">
         <v>15760.601295416</v>
       </c>
-      <c r="M77">
+      <c r="M84">
         <v>19332.981882301501</v>
       </c>
-      <c r="N77">
+      <c r="N84">
         <v>1014.17312250211</v>
       </c>
-      <c r="O77">
-        <v>0</v>
-      </c>
-      <c r="P77">
+      <c r="O84">
+        <v>0</v>
+      </c>
+      <c r="P84">
         <v>237162.97892047401</v>
       </c>
-      <c r="Q77">
+      <c r="Q84">
         <v>1386.9848841974899</v>
       </c>
-      <c r="R77">
+      <c r="R84">
         <v>18436.445202769701</v>
       </c>
-      <c r="S77">
+      <c r="S84">
         <v>209.50505912238299</v>
       </c>
-      <c r="T77" s="6">
+      <c r="T84" s="6">
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A78" s="3">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A85" s="3">
         <v>20</v>
       </c>
-      <c r="B78" s="3">
+      <c r="B85" s="3">
         <v>20</v>
       </c>
-      <c r="C78" s="3">
+      <c r="C85" s="3">
         <v>2</v>
       </c>
-      <c r="D78">
+      <c r="D85">
         <v>114184.286860504</v>
       </c>
-      <c r="E78">
+      <c r="E85">
         <v>282179.67123297497</v>
       </c>
-      <c r="F78">
+      <c r="F85">
         <v>0.83541194997266699</v>
       </c>
-      <c r="G78">
+      <c r="G85">
         <v>19351.2255529412</v>
       </c>
-      <c r="H78">
+      <c r="H85">
         <v>6002.0469674603501</v>
       </c>
-      <c r="I78">
+      <c r="I85">
         <v>2645.4376652921501</v>
       </c>
-      <c r="J78">
+      <c r="J85">
         <v>27998.710185693701</v>
       </c>
-      <c r="K78">
+      <c r="K85">
         <v>51033.4442867088</v>
       </c>
-      <c r="L78">
+      <c r="L85">
         <v>15815.1228903871</v>
       </c>
-      <c r="M78">
+      <c r="M85">
         <v>19337.009497714302</v>
       </c>
-      <c r="N78">
+      <c r="N85">
         <v>1014.17312250211</v>
       </c>
-      <c r="O78">
-        <v>0</v>
-      </c>
-      <c r="P78">
+      <c r="O85">
+        <v>0</v>
+      </c>
+      <c r="P85">
         <v>235736.26938738499</v>
       </c>
-      <c r="Q78">
+      <c r="Q85">
         <v>1336.98290493166</v>
       </c>
-      <c r="R78">
+      <c r="R85">
         <v>18577.307877855899</v>
       </c>
-      <c r="S78">
+      <c r="S85">
         <v>432.030415764091</v>
       </c>
-      <c r="T78" s="6">
+      <c r="T85" s="6">
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A79">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A86">
         <v>20</v>
       </c>
-      <c r="B79">
+      <c r="B86">
         <v>15</v>
       </c>
-      <c r="C79">
+      <c r="C86">
         <v>2</v>
       </c>
-      <c r="D79">
+      <c r="D86">
         <v>113440.79599059001</v>
       </c>
-      <c r="E79">
+      <c r="E86">
         <v>282179.67123267101</v>
       </c>
-      <c r="F79">
+      <c r="F86">
         <v>0.83277713625127903</v>
       </c>
-      <c r="G79">
+      <c r="G86">
         <v>19390.977969205</v>
       </c>
-      <c r="H79">
+      <c r="H86">
         <v>5599.5405456203798</v>
       </c>
-      <c r="I79">
+      <c r="I86">
         <v>2128.1287863747102</v>
       </c>
-      <c r="J79">
+      <c r="J86">
         <v>27118.647301200101</v>
       </c>
-      <c r="K79">
+      <c r="K86">
         <v>51068.507704320902</v>
       </c>
-      <c r="L79">
+      <c r="L86">
         <v>15909.3558282099</v>
       </c>
-      <c r="M79">
+      <c r="M86">
         <v>19344.285156859401</v>
       </c>
-      <c r="N79">
+      <c r="N86">
         <v>1010.46273302954</v>
       </c>
-      <c r="O79">
-        <v>0</v>
-      </c>
-      <c r="P79">
+      <c r="O86">
+        <v>0</v>
+      </c>
+      <c r="P86">
         <v>234992.778517472</v>
       </c>
-      <c r="Q79">
+      <c r="Q86">
         <v>1247.3228025527501</v>
       </c>
-      <c r="R79">
+      <c r="R86">
         <v>16417.502561416801</v>
       </c>
-      <c r="S79">
+      <c r="S86">
         <v>469.07150175476602</v>
       </c>
-      <c r="T79" s="6">
+      <c r="T86" s="6">
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A80">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A87">
         <v>20</v>
       </c>
-      <c r="B80">
+      <c r="B87">
         <v>12</v>
       </c>
-      <c r="C80">
+      <c r="C87">
         <v>2</v>
       </c>
-      <c r="D80">
+      <c r="D87">
         <v>113795.448700252</v>
       </c>
-      <c r="E80">
+      <c r="E87">
         <v>282179.67123287602</v>
       </c>
-      <c r="F80">
+      <c r="F87">
         <v>0.83403396920434802</v>
       </c>
-      <c r="G80">
+      <c r="G87">
         <v>20436.472361711199</v>
       </c>
-      <c r="H80">
+      <c r="H87">
         <v>4946.5396722567002</v>
       </c>
-      <c r="I80">
+      <c r="I87">
         <v>2967.9237851293901</v>
       </c>
-      <c r="J80">
+      <c r="J87">
         <v>28350.9358190973</v>
       </c>
-      <c r="K80">
+      <c r="K87">
         <v>50843.184005923598</v>
       </c>
-      <c r="L80">
+      <c r="L87">
         <v>15303.798385783</v>
       </c>
-      <c r="M80">
+      <c r="M87">
         <v>19297.530489448302</v>
       </c>
-      <c r="N80">
+      <c r="N87">
         <v>992.31070788530405</v>
       </c>
-      <c r="O80">
-        <v>0</v>
-      </c>
-      <c r="P80">
+      <c r="O87">
+        <v>0</v>
+      </c>
+      <c r="P87">
         <v>235347.43122713399</v>
       </c>
-      <c r="Q80">
+      <c r="Q87">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R80">
+      <c r="R87">
         <v>13.380488321454299</v>
       </c>
-      <c r="S80">
+      <c r="S87">
         <v>2.67609766429086</v>
       </c>
-      <c r="T80" s="6">
+      <c r="T87" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>

</xml_diff>

<commit_message>
full flex with higher rate even
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0879A5B2-96B0-4357-ADE0-41E51172CD4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{101267D2-0F0A-4C65-9924-082E41E79838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -172,7 +172,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="42">
   <si>
     <t>Season</t>
   </si>
@@ -2850,8 +2850,65 @@
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" s="3" t="s">
+      <c r="A42" t="s">
         <v>22</v>
+      </c>
+      <c r="B42" t="s">
+        <v>23</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>124517.10383110899</v>
+      </c>
+      <c r="E42">
+        <v>282190.859999999</v>
+      </c>
+      <c r="F42">
+        <v>0.87199523881812102</v>
+      </c>
+      <c r="G42">
+        <v>23255.929405575898</v>
+      </c>
+      <c r="H42">
+        <v>5559.1797407744398</v>
+      </c>
+      <c r="I42">
+        <v>10254.0938247584</v>
+      </c>
+      <c r="J42">
+        <v>39069.202971108898</v>
+      </c>
+      <c r="K42">
+        <v>50845.200000000099</v>
+      </c>
+      <c r="L42">
+        <v>15304.405199999899</v>
+      </c>
+      <c r="M42">
+        <v>19298.29566</v>
+      </c>
+      <c r="N42">
+        <v>1409.83742959549</v>
+      </c>
+      <c r="O42">
+        <v>0</v>
+      </c>
+      <c r="P42">
+        <v>246069.08635798999</v>
+      </c>
+      <c r="Q42">
+        <v>1102.0926609763501</v>
+      </c>
+      <c r="R42">
+        <v>0</v>
+      </c>
+      <c r="U42">
+        <v>15.5670440273115</v>
+      </c>
+      <c r="V42">
+        <v>9.2660976353045002E-2</v>
       </c>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Double Checking TOU 8 results
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{101267D2-0F0A-4C65-9924-082E41E79838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C902FE-5850-432C-9AF2-47800AC054F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -3807,9 +3807,6 @@
         <v>1.3585822738026401</v>
       </c>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="G70" s="4"/>
-    </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
Finding the break-even lifetime degradation for replacement costs
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47A470BD-4B9C-4D4E-A528-2C589223ED97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26D042F5-3620-43D0-A03E-0A02C08BEB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-69" yWindow="-69" windowWidth="33052" windowHeight="17932" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -35,6 +35,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={0A68C4F8-DD37-4E19-A8B1-830AE9F7EA20}</author>
     <author>tc={BBF7D234-FE30-40AB-877C-48487A60B475}</author>
     <author>tc={508D361C-2D0C-49BA-974D-6C72FE37C504}</author>
     <author>tc={F27CC18C-9CF0-4B96-A7C0-3CA554F9A587}</author>
@@ -51,7 +52,15 @@
     <author>tc={86E634AB-9E52-4A6D-BE85-5D191C9227C6}</author>
   </authors>
   <commentList>
-    <comment ref="N2" authorId="0" shapeId="0" xr:uid="{BBF7D234-FE30-40AB-877C-48487A60B475}">
+    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{0A68C4F8-DD37-4E19-A8B1-830AE9F7EA20}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This should be a formula</t>
+      </text>
+    </comment>
+    <comment ref="N2" authorId="1" shapeId="0" xr:uid="{BBF7D234-FE30-40AB-877C-48487A60B475}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -59,7 +68,7 @@
     Will need to update with new numbers</t>
       </text>
     </comment>
-    <comment ref="S2" authorId="1" shapeId="0" xr:uid="{508D361C-2D0C-49BA-974D-6C72FE37C504}">
+    <comment ref="S2" authorId="2" shapeId="0" xr:uid="{508D361C-2D0C-49BA-974D-6C72FE37C504}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -67,7 +76,7 @@
     This isn’t being calculated correctly...</t>
       </text>
     </comment>
-    <comment ref="A7" authorId="2" shapeId="0" xr:uid="{F27CC18C-9CF0-4B96-A7C0-3CA554F9A587}">
+    <comment ref="A7" authorId="3" shapeId="0" xr:uid="{F27CC18C-9CF0-4B96-A7C0-3CA554F9A587}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -75,7 +84,7 @@
     This will of course give the baseline because it is already at the maximum recovery- there is no potential for charging capacity</t>
       </text>
     </comment>
-    <comment ref="A12" authorId="3" shapeId="0" xr:uid="{73C7F34A-BCA8-44F2-A992-5B81BCD419CF}">
+    <comment ref="A12" authorId="4" shapeId="0" xr:uid="{73C7F34A-BCA8-44F2-A992-5B81BCD419CF}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -83,7 +92,7 @@
     This result still make sense because: the recovery change would cause an extra cost that outweighs the tiny electricity savings.</t>
       </text>
     </comment>
-    <comment ref="A16" authorId="4" shapeId="0" xr:uid="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
+    <comment ref="A16" authorId="5" shapeId="0" xr:uid="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -91,7 +100,7 @@
     This should be the same as the baseline</t>
       </text>
     </comment>
-    <comment ref="A25" authorId="5" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
+    <comment ref="A25" authorId="6" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -101,7 +110,7 @@
     Which yields (somewhat obviously) the same result as 4 flexible trains</t>
       </text>
     </comment>
-    <comment ref="Q27" authorId="6" shapeId="0" xr:uid="{7128E1A1-FC03-4EA4-B47C-4E0569E512E5}">
+    <comment ref="Q27" authorId="7" shapeId="0" xr:uid="{7128E1A1-FC03-4EA4-B47C-4E0569E512E5}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -109,7 +118,7 @@
     This is higher than the baseline because the solution is not optimal. It fails to optimize the UF pumps </t>
       </text>
     </comment>
-    <comment ref="A28" authorId="7" shapeId="0" xr:uid="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
+    <comment ref="A28" authorId="8" shapeId="0" xr:uid="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -117,7 +126,7 @@
     This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</t>
       </text>
     </comment>
-    <comment ref="A48" authorId="8" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A48" authorId="9" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -125,7 +134,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="A49" authorId="9" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A49" authorId="10" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -133,7 +142,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T49" authorId="10" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T49" authorId="11" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -143,7 +152,7 @@
     The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A55" authorId="11" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A55" authorId="12" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -151,7 +160,7 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="A79" authorId="12" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A79" authorId="13" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -159,7 +168,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T91" authorId="13" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T91" authorId="14" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -172,7 +181,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="44">
   <si>
     <t>Season</t>
   </si>
@@ -302,12 +311,15 @@
   <si>
     <t>CPP DR Program</t>
   </si>
+  <si>
+    <t>CAPEX =&gt;</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -468,6 +480,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1201,6 +1219,9 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="D2" dT="2026-07-20T22:02:04.36" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{0A68C4F8-DD37-4E19-A8B1-830AE9F7EA20}">
+    <text>This should be a formula</text>
+  </threadedComment>
   <threadedComment ref="N2" dT="2026-07-15T21:03:49.32" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{BBF7D234-FE30-40AB-877C-48487A60B475}">
     <text>Will need to update with new numbers</text>
   </threadedComment>
@@ -1264,6 +1285,7 @@
     <col min="7" max="7" width="10.7265625" customWidth="1"/>
     <col min="9" max="9" width="9.08984375" customWidth="1"/>
     <col min="15" max="15" width="9.54296875" customWidth="1"/>
+    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1271,6 +1293,12 @@
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
+      <c r="O1" t="s">
+        <v>43</v>
+      </c>
+      <c r="P1">
+        <v>120559.67181899652</v>
+      </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -1282,7 +1310,7 @@
       <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E2" t="s">
@@ -1351,7 +1379,8 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>111145.161086081</v>
+        <f>J3+K3+L3+M3+N3</f>
+        <v>112555.1610860814</v>
       </c>
       <c r="E3">
         <v>282179.67123287602</v>
@@ -1380,14 +1409,15 @@
       <c r="M3">
         <v>19297.5304894482</v>
       </c>
-      <c r="N3">
-        <v>992.31070788530405</v>
+      <c r="N3" s="5">
+        <v>1410</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>232697.143612963</v>
+        <f>D3+$P$1</f>
+        <v>233114.8329050779</v>
       </c>
       <c r="Q3">
         <v>1101.6748792595399</v>
@@ -1413,7 +1443,8 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>120097.924543835</v>
+        <f>J4+K4+L4+M4+N4</f>
+        <v>121507.92454383519</v>
       </c>
       <c r="E4">
         <v>282179.67123287602</v>
@@ -1442,14 +1473,15 @@
       <c r="M4">
         <v>19297.5304894482</v>
       </c>
-      <c r="N4">
-        <v>992.31070788530405</v>
+      <c r="N4" s="5">
+        <v>1410</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>241649.90707071699</v>
+        <f>D4+$P$1</f>
+        <v>242067.59636283171</v>
       </c>
       <c r="Q4">
         <v>1101.6749453094101</v>
@@ -1478,7 +1510,8 @@
         <v>0</v>
       </c>
       <c r="D6">
-        <v>111142.758477303</v>
+        <f>J6+K6+L6+M6+N6</f>
+        <v>112135.0691851889</v>
       </c>
       <c r="E6">
         <v>282179.67123287602</v>
@@ -1514,7 +1547,8 @@
         <v>0</v>
       </c>
       <c r="P6">
-        <v>232694.74100418499</v>
+        <f t="shared" ref="P6:P13" si="0">D6+$P$1</f>
+        <v>232694.7410041854</v>
       </c>
       <c r="Q6">
         <v>1101.5718970651201</v>
@@ -1540,7 +1574,8 @@
         <v>0</v>
       </c>
       <c r="D7">
-        <v>120105.62640119799</v>
+        <f>J7+K7+L7+M7+N7</f>
+        <v>121097.93710908349</v>
       </c>
       <c r="E7">
         <v>282179.67123287602</v>
@@ -1576,6 +1611,7 @@
         <v>0</v>
       </c>
       <c r="P7">
+        <f t="shared" si="0"/>
         <v>241657.60892808001</v>
       </c>
       <c r="Q7">
@@ -1605,7 +1641,8 @@
         <v>0</v>
       </c>
       <c r="D9">
-        <v>111179.352715972</v>
+        <f>J9+K9+L9+M9+N9</f>
+        <v>112171.66342385749</v>
       </c>
       <c r="E9">
         <v>282179.67123287602</v>
@@ -1641,7 +1678,8 @@
         <v>0</v>
       </c>
       <c r="P9">
-        <v>232731.33524285399</v>
+        <f t="shared" si="0"/>
+        <v>232731.33524285402</v>
       </c>
       <c r="Q9">
         <v>1103.1405255510299</v>
@@ -1667,7 +1705,8 @@
         <v>0</v>
       </c>
       <c r="D10">
-        <v>120133.22940371701</v>
+        <f>J10+K10+L10+M10+N10</f>
+        <v>121125.54011160239</v>
       </c>
       <c r="E10">
         <v>282181.81222384499</v>
@@ -1703,7 +1742,8 @@
         <v>0</v>
       </c>
       <c r="P10">
-        <v>241685.21193059901</v>
+        <f t="shared" si="0"/>
+        <v>241685.21193059889</v>
       </c>
       <c r="Q10">
         <v>1102.72373433861</v>
@@ -1732,7 +1772,8 @@
         <v>0</v>
       </c>
       <c r="D12">
-        <v>111142.758477303</v>
+        <f>J12+K12+L12+M12+N12</f>
+        <v>112135.0691851889</v>
       </c>
       <c r="E12">
         <v>282179.67123287602</v>
@@ -1768,7 +1809,8 @@
         <v>0</v>
       </c>
       <c r="P12">
-        <v>232694.74100418499</v>
+        <f t="shared" si="0"/>
+        <v>232694.7410041854</v>
       </c>
       <c r="Q12">
         <v>1101.5718970651201</v>
@@ -1794,7 +1836,8 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <v>118611.04844584499</v>
+        <f>J13+K13+L13+M13+N13</f>
+        <v>119603.35915373031</v>
       </c>
       <c r="E13">
         <v>282179.67177163501</v>
@@ -1830,7 +1873,8 @@
         <v>0</v>
       </c>
       <c r="P13">
-        <v>240163.03097272699</v>
+        <f t="shared" si="0"/>
+        <v>240163.03097272682</v>
       </c>
       <c r="Q13">
         <v>1143.3910977538401</v>
@@ -1980,7 +2024,8 @@
         <v>2</v>
       </c>
       <c r="D18">
-        <v>111737.917851103</v>
+        <f>J18+K18+L18+M18+N18</f>
+        <v>112730.2285589885</v>
       </c>
       <c r="E18">
         <v>282179.67125484499</v>
@@ -2016,7 +2061,8 @@
         <v>0</v>
       </c>
       <c r="P18">
-        <v>233289.900377985</v>
+        <f t="shared" ref="P18:P19" si="1">D18+$P$1</f>
+        <v>233289.90037798503</v>
       </c>
       <c r="Q18">
         <v>1127.0837800240299</v>
@@ -2042,7 +2088,8 @@
         <v>2</v>
       </c>
       <c r="D19">
-        <v>117965.918152322</v>
+        <f>J19+K19+L19+M19+N19</f>
+        <v>118976.38088535203</v>
       </c>
       <c r="E19">
         <v>282179.67123287602</v>
@@ -2078,7 +2125,8 @@
         <v>0</v>
       </c>
       <c r="P19">
-        <v>239517.900679204</v>
+        <f t="shared" si="1"/>
+        <v>239536.05270434855</v>
       </c>
       <c r="Q19">
         <v>1460.3271566616399</v>
@@ -2120,7 +2168,8 @@
         <v>2</v>
       </c>
       <c r="D22">
-        <v>118061.356447413</v>
+        <f>J22+K22+L22+M22+N22</f>
+        <v>119071.81918044275</v>
       </c>
       <c r="E22">
         <v>282179.67123275797</v>
@@ -2156,7 +2205,8 @@
         <v>0</v>
       </c>
       <c r="P22">
-        <v>239613.33897429501</v>
+        <f t="shared" ref="P22:P23" si="2">D22+$P$1</f>
+        <v>239631.49099943927</v>
       </c>
       <c r="Q22">
         <v>1462.4682301396899</v>
@@ -2185,7 +2235,8 @@
         <v>2</v>
       </c>
       <c r="D24">
-        <v>111737.92287843001</v>
+        <f>J24+K24+L24+M24+N24</f>
+        <v>112730.23358631571</v>
       </c>
       <c r="E24">
         <v>282179.67125484499</v>
@@ -2221,7 +2272,8 @@
         <v>0</v>
       </c>
       <c r="P24">
-        <v>233289.90540531199</v>
+        <f t="shared" ref="P24:P25" si="3">D24+$P$1</f>
+        <v>233289.90540531222</v>
       </c>
       <c r="Q24">
         <v>1127.08379747136</v>
@@ -2247,7 +2299,8 @@
         <v>2</v>
       </c>
       <c r="D25">
-        <v>116354.41551491299</v>
+        <f>J25+K25+L25+M25+N25</f>
+        <v>117782.20721135012</v>
       </c>
       <c r="E25">
         <v>282179.67123287602</v>
@@ -2283,7 +2336,8 @@
         <v>0</v>
       </c>
       <c r="P25">
-        <v>237906.39804179501</v>
+        <f t="shared" si="3"/>
+        <v>238341.87903034664</v>
       </c>
       <c r="Q25">
         <v>1179.82420335646</v>
@@ -2319,7 +2373,8 @@
         <v>4</v>
       </c>
       <c r="D27">
-        <v>111742.37918817</v>
+        <f>J27+K27+L27+M27+N27</f>
+        <v>112734.6898960558</v>
       </c>
       <c r="E27">
         <v>282179.67125500599</v>
@@ -2355,7 +2410,8 @@
         <v>0</v>
       </c>
       <c r="P27">
-        <v>233294.36171505199</v>
+        <f t="shared" ref="P27:P28" si="4">D27+$P$1</f>
+        <v>233294.36171505234</v>
       </c>
       <c r="Q27">
         <v>1127.27501819133</v>
@@ -2381,7 +2437,8 @@
         <v>4</v>
       </c>
       <c r="D28">
-        <v>118002.301696422</v>
+        <f>J28+K28+L28+M28+N28</f>
+        <v>119012.76442945223</v>
       </c>
       <c r="E28">
         <v>282179.67123287602</v>
@@ -2417,7 +2474,8 @@
         <v>0</v>
       </c>
       <c r="P28">
-        <v>239554.28422330401</v>
+        <f t="shared" si="4"/>
+        <v>239572.43624844874</v>
       </c>
       <c r="Q28">
         <v>1460.5368984148499</v>
@@ -2436,17 +2494,18 @@
       <c r="G29" s="4"/>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C30">
         <v>4</v>
       </c>
       <c r="D30">
-        <v>111742.37432318801</v>
+        <f>J30+K30+L30+M30+N30</f>
+        <v>113152.3743231883</v>
       </c>
       <c r="E30">
         <v>282179.67123264802</v>
@@ -2475,14 +2534,15 @@
       <c r="M30">
         <v>19297.530511697802</v>
       </c>
-      <c r="N30">
-        <v>992.31070788530405</v>
+      <c r="N30" s="5">
+        <v>1410</v>
       </c>
       <c r="O30">
         <v>0</v>
       </c>
       <c r="P30">
-        <v>233294.35685007001</v>
+        <f t="shared" ref="P30:P31" si="5">D30+$P$1</f>
+        <v>233712.04614218482</v>
       </c>
       <c r="Q30">
         <v>1127.27479036512</v>
@@ -2508,7 +2568,8 @@
         <v>4</v>
       </c>
       <c r="D31">
-        <v>116354.41551491299</v>
+        <f>J31+K31+L31+M31+N31</f>
+        <v>117790.41551491321</v>
       </c>
       <c r="E31">
         <v>282179.67123287602</v>
@@ -2537,14 +2598,15 @@
       <c r="M31">
         <v>19346.075503401102</v>
       </c>
-      <c r="N31">
-        <v>1427.7916964369099</v>
+      <c r="N31" s="5">
+        <v>1436</v>
       </c>
       <c r="O31">
         <v>0</v>
       </c>
       <c r="P31">
-        <v>237906.39804179501</v>
+        <f t="shared" si="5"/>
+        <v>238350.08733390973</v>
       </c>
       <c r="Q31">
         <v>1179.82420335646</v>
@@ -2588,7 +2650,8 @@
         <v>0</v>
       </c>
       <c r="D34">
-        <v>115583.48181615899</v>
+        <f>J34+K34+L34+M34+N34</f>
+        <v>116993.31924575487</v>
       </c>
       <c r="E34">
         <v>282190.859999999</v>
@@ -2624,7 +2687,8 @@
         <v>0</v>
       </c>
       <c r="P34">
-        <v>237135.46434304101</v>
+        <f t="shared" ref="P34:P35" si="6">D34+$P$1</f>
+        <v>237552.9910647514</v>
       </c>
       <c r="Q34">
         <v>1102.0926609763501</v>
@@ -2650,7 +2714,8 @@
         <v>0</v>
       </c>
       <c r="D35">
-        <v>124490.983160207</v>
+        <f>J35+K35+L35+M35+N35</f>
+        <v>125900.82058980259</v>
       </c>
       <c r="E35">
         <v>282190.859999999</v>
@@ -2686,7 +2751,8 @@
         <v>0</v>
       </c>
       <c r="P35">
-        <v>246042.96568708899</v>
+        <f t="shared" si="6"/>
+        <v>246460.49240879912</v>
       </c>
       <c r="Q35">
         <v>1102.0926609763501</v>
@@ -2717,7 +2783,8 @@
         <v>4</v>
       </c>
       <c r="D37">
-        <v>115568.67725355701</v>
+        <f>J37+K37+L37+M37+N37</f>
+        <v>116978.51468315258</v>
       </c>
       <c r="E37">
         <v>282179.671254922</v>
@@ -2753,7 +2820,8 @@
         <v>0</v>
       </c>
       <c r="P37">
-        <v>237120.659780438</v>
+        <f t="shared" ref="P37:P39" si="7">D37+$P$1</f>
+        <v>237538.1865021491</v>
       </c>
       <c r="Q37">
         <v>1101.67497109485</v>
@@ -2782,7 +2850,8 @@
         <v>4</v>
       </c>
       <c r="D38">
-        <v>120779.539344445</v>
+        <f>J38+K38+L38+M38+N38</f>
+        <v>122209.93333437521</v>
       </c>
       <c r="E38">
         <v>282179.67123287602</v>
@@ -2818,7 +2887,8 @@
         <v>0</v>
       </c>
       <c r="P38">
-        <v>242331.52187132699</v>
+        <f t="shared" si="7"/>
+        <v>242769.60515337173</v>
       </c>
       <c r="Q38">
         <v>1171.0808202107701</v>
@@ -2841,6 +2911,54 @@
     </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="3"/>
+      <c r="D39">
+        <f>D38-D35</f>
+        <v>-3690.8872554273839</v>
+      </c>
+      <c r="E39">
+        <f t="shared" ref="E39:N39" si="8">E38-E35</f>
+        <v>-11.188767122977879</v>
+      </c>
+      <c r="F39">
+        <f t="shared" si="8"/>
+        <v>-1.3118196231516999E-2</v>
+      </c>
+      <c r="G39">
+        <f t="shared" si="8"/>
+        <v>-906.13409185930141</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="8"/>
+        <v>406.02321782605031</v>
+      </c>
+      <c r="I39">
+        <f t="shared" si="8"/>
+        <v>-4354.3002052295496</v>
+      </c>
+      <c r="J39">
+        <f t="shared" si="8"/>
+        <v>-4854.411079262798</v>
+      </c>
+      <c r="K39">
+        <f t="shared" si="8"/>
+        <v>292.29857391989935</v>
+      </c>
+      <c r="L39">
+        <f t="shared" si="8"/>
+        <v>790.3635872736013</v>
+      </c>
+      <c r="M39">
+        <f t="shared" si="8"/>
+        <v>60.305102307600464</v>
+      </c>
+      <c r="N39">
+        <f t="shared" si="8"/>
+        <v>20.556560334320011</v>
+      </c>
+      <c r="P39">
+        <f t="shared" si="7"/>
+        <v>116868.78456356913</v>
+      </c>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A40" s="7" t="s">
@@ -2863,7 +2981,8 @@
         <v>0</v>
       </c>
       <c r="D42">
-        <v>124517.10383110899</v>
+        <f>J42+K42+L42+M42+N42</f>
+        <v>125926.94126070438</v>
       </c>
       <c r="E42">
         <v>282190.859999999</v>
@@ -2899,7 +3018,8 @@
         <v>0</v>
       </c>
       <c r="P42">
-        <v>246069.08635798999</v>
+        <f t="shared" ref="P42" si="9">D42+$P$1</f>
+        <v>246486.61307970091</v>
       </c>
       <c r="Q42">
         <v>1102.0926609763501</v>
@@ -2923,8 +3043,73 @@
       </c>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" s="3" t="s">
+      <c r="A45" t="s">
         <v>22</v>
+      </c>
+      <c r="B45" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45">
+        <v>4</v>
+      </c>
+      <c r="D45">
+        <f>J45+K45+L45+M45+N45</f>
+        <v>121548.56732352625</v>
+      </c>
+      <c r="E45">
+        <v>282179.67171295901</v>
+      </c>
+      <c r="F45">
+        <v>0.85645911177426404</v>
+      </c>
+      <c r="G45">
+        <v>21922.670949606902</v>
+      </c>
+      <c r="H45">
+        <v>5892.0772301955703</v>
+      </c>
+      <c r="I45">
+        <v>5494.1642193806101</v>
+      </c>
+      <c r="J45">
+        <v>33308.9123991831</v>
+      </c>
+      <c r="K45">
+        <v>51194.9024604468</v>
+      </c>
+      <c r="L45">
+        <v>16249.0415258787</v>
+      </c>
+      <c r="M45">
+        <v>19370.512083644498</v>
+      </c>
+      <c r="N45">
+        <v>1425.19885437316</v>
+      </c>
+      <c r="O45">
+        <v>0</v>
+      </c>
+      <c r="P45">
+        <f t="shared" ref="P45" si="10">D45+$P$1</f>
+        <v>242108.23914252277</v>
+      </c>
+      <c r="Q45">
+        <v>1168.0887035395799</v>
+      </c>
+      <c r="R45">
+        <v>12792.663740961099</v>
+      </c>
+      <c r="S45">
+        <v>511.70654963844697</v>
+      </c>
+      <c r="T45">
+        <v>-0.11339056141074599</v>
+      </c>
+      <c r="U45">
+        <v>7320.3796501147199</v>
+      </c>
+      <c r="V45">
+        <v>51.1914660847183</v>
       </c>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.35">
@@ -2944,7 +3129,8 @@
         <v>0</v>
       </c>
       <c r="D48">
-        <v>116861.67991782499</v>
+        <f>J48+K48+L48+M48+N48</f>
+        <v>117853.9906257109</v>
       </c>
       <c r="E48">
         <v>282179.67123287602</v>
@@ -2980,7 +3166,8 @@
         <v>0</v>
       </c>
       <c r="P48">
-        <v>238413.66244470701</v>
+        <f t="shared" ref="P48:P55" si="11">D48+$P$1</f>
+        <v>238413.66244470741</v>
       </c>
       <c r="Q48">
         <v>1102.6552392369899</v>
@@ -3006,7 +3193,8 @@
         <v>0</v>
       </c>
       <c r="D49">
-        <v>187020.456722612</v>
+        <f>J49+K49+L49+M49+N49</f>
+        <v>188012.7674304971</v>
       </c>
       <c r="E49">
         <v>282179.67123287602</v>
@@ -3042,7 +3230,8 @@
         <v>0</v>
       </c>
       <c r="P49">
-        <v>308572.439249494</v>
+        <f t="shared" si="11"/>
+        <v>308572.43924949365</v>
       </c>
       <c r="Q49">
         <v>1106.4527933521999</v>
@@ -3072,7 +3261,8 @@
         <v>0</v>
       </c>
       <c r="D51">
-        <v>117032.41959359701</v>
+        <f>J51+K51+L51+M51+N51</f>
+        <v>118024.73030148289</v>
       </c>
       <c r="E51">
         <v>282179.67123286898</v>
@@ -3108,7 +3298,8 @@
         <v>0</v>
       </c>
       <c r="P51">
-        <v>238584.402120479</v>
+        <f t="shared" si="11"/>
+        <v>238584.40212047941</v>
       </c>
       <c r="Q51">
         <v>1108.83163779344</v>
@@ -3134,7 +3325,8 @@
         <v>0</v>
       </c>
       <c r="D52">
-        <v>171564.02128394699</v>
+        <f>J52+K52+L52+M52+N52</f>
+        <v>172556.33199183288</v>
       </c>
       <c r="E52">
         <v>282179.67123287701</v>
@@ -3170,7 +3362,8 @@
         <v>0</v>
       </c>
       <c r="P52">
-        <v>293116.00381082902</v>
+        <f t="shared" si="11"/>
+        <v>293116.00381082937</v>
       </c>
       <c r="Q52">
         <v>1187.62883512946</v>
@@ -3199,7 +3392,8 @@
         <v>4</v>
       </c>
       <c r="D54">
-        <v>116833.749486644</v>
+        <f>J54+K54+L54+M54+N54</f>
+        <v>117826.0601945299</v>
       </c>
       <c r="E54">
         <v>282179.67123287602</v>
@@ -3235,7 +3429,8 @@
         <v>0</v>
       </c>
       <c r="P54">
-        <v>0</v>
+        <f t="shared" si="11"/>
+        <v>238385.73201352643</v>
       </c>
       <c r="Q54">
         <v>0</v>
@@ -3261,7 +3456,8 @@
         <v>4</v>
       </c>
       <c r="D55">
-        <v>124393.533174422</v>
+        <f>J55+K55+L55+M55+N55</f>
+        <v>125434.46212050831</v>
       </c>
       <c r="E55">
         <v>282179.67123444699</v>
@@ -3297,7 +3493,8 @@
         <v>0</v>
       </c>
       <c r="P55">
-        <v>245945.51570130399</v>
+        <f t="shared" si="11"/>
+        <v>245994.13393950483</v>
       </c>
       <c r="Q55">
         <v>1458.3752411216699</v>
@@ -3329,7 +3526,8 @@
         <v>2</v>
       </c>
       <c r="D58">
-        <v>115472.147206908</v>
+        <f>J58+K58+L58+M58+N58</f>
+        <v>119635.09208261623</v>
       </c>
       <c r="E58">
         <v>282495</v>
@@ -3365,7 +3563,8 @@
         <v>3157.9970999842499</v>
       </c>
       <c r="P58">
-        <v>237024.12973379</v>
+        <f t="shared" ref="P58:P59" si="12">D58+$P$1</f>
+        <v>240194.76390161275</v>
       </c>
       <c r="Q58">
         <v>1464.2687322859999</v>
@@ -3391,7 +3590,8 @@
         <v>4</v>
       </c>
       <c r="D59">
-        <v>108958.027502652</v>
+        <f>J59+K59+L59+M59+N59</f>
+        <v>120582.97527837555</v>
       </c>
       <c r="E59">
         <v>282179.67123287602</v>
@@ -3427,7 +3627,8 @@
         <v>10620</v>
       </c>
       <c r="P59">
-        <v>230510.010029533</v>
+        <f t="shared" si="12"/>
+        <v>241142.64709737207</v>
       </c>
       <c r="Q59">
         <v>1464.02925348484</v>
@@ -3524,7 +3725,8 @@
         <v>0</v>
       </c>
       <c r="D69">
-        <v>115030.978322179</v>
+        <f>J69+K69+L69+M69+N69</f>
+        <v>116023.2890300647</v>
       </c>
       <c r="E69">
         <v>282179.67123287602</v>
@@ -3560,7 +3762,8 @@
         <v>0</v>
       </c>
       <c r="P69">
-        <v>236582.960849061</v>
+        <f t="shared" ref="P69:P70" si="13">D69+$P$1</f>
+        <v>236582.9608490612</v>
       </c>
       <c r="Q69">
         <v>1101.8347602124099</v>
@@ -3586,7 +3789,8 @@
         <v>0</v>
       </c>
       <c r="D70">
-        <v>124771.246709449</v>
+        <f>J70+K70+L70+M70+N70</f>
+        <v>125763.55741733511</v>
       </c>
       <c r="E70">
         <v>282179.67125180899</v>
@@ -3622,7 +3826,8 @@
         <v>0</v>
       </c>
       <c r="P70">
-        <v>246323.22923633101</v>
+        <f t="shared" si="13"/>
+        <v>246323.22923633162</v>
       </c>
       <c r="Q70">
         <v>1127.27501714903</v>
@@ -3651,7 +3856,8 @@
         <v>2</v>
       </c>
       <c r="D72">
-        <v>115714.10508262301</v>
+        <f>J72+K72+L72+M72+N72</f>
+        <v>116706.4157905087</v>
       </c>
       <c r="E72">
         <v>282179.67125387199</v>
@@ -3687,7 +3893,8 @@
         <v>0</v>
       </c>
       <c r="P72">
-        <v>237266.08760950499</v>
+        <f t="shared" ref="P72:P73" si="14">D72+$P$1</f>
+        <v>237266.08760950522</v>
       </c>
       <c r="Q72">
         <v>1127.2750356983099</v>
@@ -3707,7 +3914,8 @@
         <v>2</v>
       </c>
       <c r="D73">
-        <v>120628.41082793</v>
+        <f>J73+K73+L73+M73+N73</f>
+        <v>121633.35860365373</v>
       </c>
       <c r="E73">
         <v>282179.67123287602</v>
@@ -3743,7 +3951,8 @@
         <v>0</v>
       </c>
       <c r="P73">
-        <v>242180.39335481101</v>
+        <f t="shared" si="14"/>
+        <v>242193.03042265025</v>
       </c>
       <c r="Q73">
         <v>1183.4303612998101</v>
@@ -3769,7 +3978,8 @@
         <v>4</v>
       </c>
       <c r="D75">
-        <v>115714.10508261999</v>
+        <f>J75+K75+L75+M75+N75</f>
+        <v>116706.4157905051</v>
       </c>
       <c r="E75">
         <v>282179.671253876</v>
@@ -3805,7 +4015,8 @@
         <v>0</v>
       </c>
       <c r="P75">
-        <v>237266.087609501</v>
+        <f t="shared" ref="P75:P76" si="15">D75+$P$1</f>
+        <v>237266.08760950161</v>
       </c>
       <c r="Q75">
         <v>1127.2750356983499</v>
@@ -3825,7 +4036,8 @@
         <v>4</v>
       </c>
       <c r="D76">
-        <v>120375.156660901</v>
+        <f>J76+K76+L76+M76+N76</f>
+        <v>121381.93605468499</v>
       </c>
       <c r="E76">
         <v>282179.671232878</v>
@@ -3861,7 +4073,8 @@
         <v>0</v>
       </c>
       <c r="P76">
-        <v>241927.13918778201</v>
+        <f t="shared" si="15"/>
+        <v>241941.60787368153</v>
       </c>
       <c r="Q76">
         <v>1178.65858109644</v>
@@ -3893,7 +4106,8 @@
         <v>4</v>
       </c>
       <c r="D79">
-        <v>146108.01933512901</v>
+        <f>J79+K79+L79+M79+N79</f>
+        <v>147118.48206815872</v>
       </c>
       <c r="E79">
         <v>355610.364944759</v>
@@ -3929,7 +4143,8 @@
         <v>0</v>
       </c>
       <c r="P79">
-        <v>267660.00186201098</v>
+        <f t="shared" ref="P79:P80" si="16">D79+$P$1</f>
+        <v>267678.15388715523</v>
       </c>
       <c r="Q79">
         <v>1597.68911089628</v>
@@ -4160,7 +4375,8 @@
         <v>2</v>
       </c>
       <c r="D88">
-        <v>119696.652328767</v>
+        <f t="shared" ref="D88:D94" si="17">J88+K88+L88+M88+N88</f>
+        <v>120712.69088313227</v>
       </c>
       <c r="E88">
         <v>282179.67123285501</v>
@@ -4196,7 +4412,8 @@
         <v>0</v>
       </c>
       <c r="P88">
-        <v>241248.634855649</v>
+        <f t="shared" ref="P88:P95" si="18">D88+$P$1</f>
+        <v>241272.36270212877</v>
       </c>
       <c r="Q88">
         <v>1192.7637589594799</v>
@@ -4222,7 +4439,8 @@
         <v>2</v>
       </c>
       <c r="D89">
-        <v>118381.960809661</v>
+        <f t="shared" si="17"/>
+        <v>119392.42354269064</v>
       </c>
       <c r="E89">
         <v>282254.81855225202</v>
@@ -4258,7 +4476,8 @@
         <v>0</v>
       </c>
       <c r="P89">
-        <v>239933.943336542</v>
+        <f t="shared" si="18"/>
+        <v>239952.09536168716</v>
       </c>
       <c r="Q89">
         <v>1312.43161993582</v>
@@ -4284,7 +4503,8 @@
         <v>2</v>
       </c>
       <c r="D90">
-        <v>116766.56672038</v>
+        <f t="shared" si="17"/>
+        <v>117777.02945340994</v>
       </c>
       <c r="E90">
         <v>282179.67123287299</v>
@@ -4320,7 +4540,8 @@
         <v>0</v>
       </c>
       <c r="P90">
-        <v>238318.54924726201</v>
+        <f t="shared" si="18"/>
+        <v>238336.70127240644</v>
       </c>
       <c r="Q90">
         <v>1265.6913868611</v>
@@ -4346,7 +4567,8 @@
         <v>2</v>
       </c>
       <c r="D91">
-        <v>115610.996393592</v>
+        <f t="shared" si="17"/>
+        <v>116625.1695160947</v>
       </c>
       <c r="E91">
         <v>282182.50548365602</v>
@@ -4382,7 +4604,8 @@
         <v>0</v>
       </c>
       <c r="P91">
-        <v>237162.97892047401</v>
+        <f t="shared" si="18"/>
+        <v>237184.84133509122</v>
       </c>
       <c r="Q91">
         <v>1386.9848841974899</v>
@@ -4408,7 +4631,8 @@
         <v>2</v>
       </c>
       <c r="D92">
-        <v>114184.286860504</v>
+        <f t="shared" si="17"/>
+        <v>115198.459983006</v>
       </c>
       <c r="E92">
         <v>282179.67123297497</v>
@@ -4444,7 +4668,8 @@
         <v>0</v>
       </c>
       <c r="P92">
-        <v>235736.26938738499</v>
+        <f t="shared" si="18"/>
+        <v>235758.13180200252</v>
       </c>
       <c r="Q92">
         <v>1336.98290493166</v>
@@ -4470,7 +4695,8 @@
         <v>2</v>
       </c>
       <c r="D93">
-        <v>113440.79599059001</v>
+        <f t="shared" si="17"/>
+        <v>114451.25872361983</v>
       </c>
       <c r="E93">
         <v>282179.67123267101</v>
@@ -4506,7 +4732,8 @@
         <v>0</v>
       </c>
       <c r="P93">
-        <v>234992.778517472</v>
+        <f t="shared" si="18"/>
+        <v>235010.93054261635</v>
       </c>
       <c r="Q93">
         <v>1247.3228025527501</v>
@@ -4532,7 +4759,8 @@
         <v>2</v>
       </c>
       <c r="D94">
-        <v>113795.448700252</v>
+        <f t="shared" si="17"/>
+        <v>114787.7594081375</v>
       </c>
       <c r="E94">
         <v>282179.67123287602</v>
@@ -4568,7 +4796,8 @@
         <v>0</v>
       </c>
       <c r="P94">
-        <v>235347.43122713399</v>
+        <f t="shared" si="18"/>
+        <v>235347.43122713402</v>
       </c>
       <c r="Q94">
         <v>1101.8639118583401</v>

</xml_diff>

<commit_message>
baseline for CPP rate
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26D042F5-3620-43D0-A03E-0A02C08BEB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A0584AE-2B19-4DEC-8544-012E51EE8479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-69" yWindow="-69" windowWidth="33052" windowHeight="17932" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -48,6 +48,7 @@
     <author>tc={F9308CF0-AB74-4ABB-91B6-7382ECEADD39}</author>
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
     <author>tc={7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}</author>
+    <author>tc={4644E393-F522-4E79-88BA-041770B595A7}</author>
     <author>tc={9FF6B967-6104-43AC-8EED-15C48C9ACCA9}</author>
     <author>tc={86E634AB-9E52-4A6D-BE85-5D191C9227C6}</author>
   </authors>
@@ -160,7 +161,15 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="A79" authorId="13" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A73" authorId="13" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Pretty sure this solution is wrong, but I don’t think I need this case for the paper</t>
+      </text>
+    </comment>
+    <comment ref="A79" authorId="14" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -168,7 +177,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T91" authorId="14" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T91" authorId="15" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1264,6 +1273,9 @@
   <threadedComment ref="A55" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
     <text>Result from the fast solve</text>
   </threadedComment>
+  <threadedComment ref="A73" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
+    <text>Pretty sure this solution is wrong, but I don’t think I need this case for the paper</text>
+  </threadedComment>
   <threadedComment ref="A79" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
     <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
   </threadedComment>
@@ -1276,20 +1288,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:V94"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" customWidth="1"/>
-    <col min="3" max="3" width="11.453125" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" customWidth="1"/>
-    <col min="15" max="15" width="9.54296875" customWidth="1"/>
-    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.81640625" customWidth="1"/>
+    <col min="1" max="1" width="9.61328125" customWidth="1"/>
+    <col min="3" max="3" width="11.4609375" customWidth="1"/>
+    <col min="5" max="5" width="10.23046875" customWidth="1"/>
+    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.69140625" customWidth="1"/>
+    <col min="9" max="9" width="9.07421875" customWidth="1"/>
+    <col min="15" max="15" width="9.53515625" customWidth="1"/>
+    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1300,7 +1312,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1368,7 +1380,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1432,7 +1444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1496,10 +1508,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1563,7 +1575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -1627,10 +1639,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1694,7 +1706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -1758,10 +1770,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -1825,7 +1837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -1889,10 +1901,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1954,7 +1966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2010,10 +2022,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2077,7 +2089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2141,12 +2153,12 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2157,7 +2169,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2205,7 +2217,7 @@
         <v>0</v>
       </c>
       <c r="P22">
-        <f t="shared" ref="P22:P23" si="2">D22+$P$1</f>
+        <f t="shared" ref="P22" si="2">D22+$P$1</f>
         <v>239631.49099943927</v>
       </c>
       <c r="Q22">
@@ -2221,10 +2233,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2288,7 +2300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2358,11 +2370,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2426,7 +2438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2490,10 +2502,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2557,7 +2569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -2627,19 +2639,19 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="S32" s="2"/>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A33" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B33" s="2"/>
       <c r="S33" s="2"/>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>20</v>
       </c>
@@ -2703,7 +2715,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>22</v>
       </c>
@@ -2767,12 +2779,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A36" s="7"/>
       <c r="B36" s="2"/>
       <c r="S36" s="2"/>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A37" s="3" t="s">
         <v>20</v>
       </c>
@@ -2839,7 +2851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A38" s="3" t="s">
         <v>22</v>
       </c>
@@ -2909,68 +2921,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A39" s="3"/>
-      <c r="D39">
-        <f>D38-D35</f>
-        <v>-3690.8872554273839</v>
-      </c>
-      <c r="E39">
-        <f t="shared" ref="E39:N39" si="8">E38-E35</f>
-        <v>-11.188767122977879</v>
-      </c>
-      <c r="F39">
-        <f t="shared" si="8"/>
-        <v>-1.3118196231516999E-2</v>
-      </c>
-      <c r="G39">
-        <f t="shared" si="8"/>
-        <v>-906.13409185930141</v>
-      </c>
-      <c r="H39">
-        <f t="shared" si="8"/>
-        <v>406.02321782605031</v>
-      </c>
-      <c r="I39">
-        <f t="shared" si="8"/>
-        <v>-4354.3002052295496</v>
-      </c>
-      <c r="J39">
-        <f t="shared" si="8"/>
-        <v>-4854.411079262798</v>
-      </c>
-      <c r="K39">
-        <f t="shared" si="8"/>
-        <v>292.29857391989935</v>
-      </c>
-      <c r="L39">
-        <f t="shared" si="8"/>
-        <v>790.3635872736013</v>
-      </c>
-      <c r="M39">
-        <f t="shared" si="8"/>
-        <v>60.305102307600464</v>
-      </c>
-      <c r="N39">
-        <f t="shared" si="8"/>
-        <v>20.556560334320011</v>
-      </c>
-      <c r="P39">
-        <f t="shared" si="7"/>
-        <v>116868.78456356913</v>
-      </c>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A40" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A41" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>22</v>
       </c>
@@ -3018,7 +2982,7 @@
         <v>0</v>
       </c>
       <c r="P42">
-        <f t="shared" ref="P42" si="9">D42+$P$1</f>
+        <f t="shared" ref="P42" si="8">D42+$P$1</f>
         <v>246486.61307970091</v>
       </c>
       <c r="Q42">
@@ -3034,15 +2998,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A43" s="3"/>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A44" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>22</v>
       </c>
@@ -3090,7 +3054,7 @@
         <v>0</v>
       </c>
       <c r="P45">
-        <f t="shared" ref="P45" si="10">D45+$P$1</f>
+        <f>D45+$P$1</f>
         <v>242108.23914252277</v>
       </c>
       <c r="Q45">
@@ -3112,13 +3076,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A47" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G47" s="4"/>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A48" s="5" t="s">
         <v>20</v>
       </c>
@@ -3166,7 +3130,7 @@
         <v>0</v>
       </c>
       <c r="P48">
-        <f t="shared" ref="P48:P55" si="11">D48+$P$1</f>
+        <f t="shared" ref="P48:P55" si="9">D48+$P$1</f>
         <v>238413.66244470741</v>
       </c>
       <c r="Q48">
@@ -3182,7 +3146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A49" s="5" t="s">
         <v>22</v>
       </c>
@@ -3230,7 +3194,7 @@
         <v>0</v>
       </c>
       <c r="P49">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>308572.43924949365</v>
       </c>
       <c r="Q49">
@@ -3246,11 +3210,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A50" s="3"/>
       <c r="G50" s="4"/>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>20</v>
       </c>
@@ -3298,7 +3262,7 @@
         <v>0</v>
       </c>
       <c r="P51">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>238584.40212047941</v>
       </c>
       <c r="Q51">
@@ -3314,7 +3278,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>22</v>
       </c>
@@ -3362,7 +3326,7 @@
         <v>0</v>
       </c>
       <c r="P52">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>293116.00381082937</v>
       </c>
       <c r="Q52">
@@ -3378,10 +3342,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G53" s="4"/>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A54" s="3" t="s">
         <v>20</v>
       </c>
@@ -3429,7 +3393,7 @@
         <v>0</v>
       </c>
       <c r="P54">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>238385.73201352643</v>
       </c>
       <c r="Q54">
@@ -3445,7 +3409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>22</v>
       </c>
@@ -3493,7 +3457,7 @@
         <v>0</v>
       </c>
       <c r="P55">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>245994.13393950483</v>
       </c>
       <c r="Q55">
@@ -3509,13 +3473,13 @@
         <v>0.51444695802960605</v>
       </c>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A57" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G57" s="4"/>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
         <v>22</v>
       </c>
@@ -3563,7 +3527,7 @@
         <v>3157.9970999842499</v>
       </c>
       <c r="P58">
-        <f t="shared" ref="P58:P59" si="12">D58+$P$1</f>
+        <f t="shared" ref="P58:P59" si="10">D58+$P$1</f>
         <v>240194.76390161275</v>
       </c>
       <c r="Q58">
@@ -3579,7 +3543,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
         <v>22</v>
       </c>
@@ -3627,7 +3591,7 @@
         <v>10620</v>
       </c>
       <c r="P59">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>241142.64709737207</v>
       </c>
       <c r="Q59">
@@ -3643,16 +3607,16 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G60" s="4"/>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A61" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G61" s="4"/>
     </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A62" s="3" t="s">
         <v>20</v>
       </c>
@@ -3664,7 +3628,7 @@
       </c>
       <c r="G62" s="4"/>
     </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A63" s="3" t="s">
         <v>22</v>
       </c>
@@ -3676,13 +3640,13 @@
       </c>
       <c r="G63" s="4"/>
     </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
       <c r="G64" s="4"/>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A65" s="3" t="s">
         <v>20</v>
       </c>
@@ -3694,7 +3658,7 @@
       </c>
       <c r="G65" s="4"/>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A66" s="3" t="s">
         <v>22</v>
       </c>
@@ -3705,16 +3669,16 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A67" s="5"/>
       <c r="B67" s="5"/>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A68" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A69" s="3" t="s">
         <v>20</v>
       </c>
@@ -3762,7 +3726,7 @@
         <v>0</v>
       </c>
       <c r="P69">
-        <f t="shared" ref="P69:P70" si="13">D69+$P$1</f>
+        <f t="shared" ref="P69:P70" si="11">D69+$P$1</f>
         <v>236582.9608490612</v>
       </c>
       <c r="Q69">
@@ -3778,7 +3742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A70" s="3" t="s">
         <v>22</v>
       </c>
@@ -3826,7 +3790,7 @@
         <v>0</v>
       </c>
       <c r="P70">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>246323.22923633162</v>
       </c>
       <c r="Q70">
@@ -3842,10 +3806,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A71" s="1"/>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A72" t="s">
         <v>20</v>
       </c>
@@ -3893,7 +3857,7 @@
         <v>0</v>
       </c>
       <c r="P72">
-        <f t="shared" ref="P72:P73" si="14">D72+$P$1</f>
+        <f t="shared" ref="P72:P73" si="12">D72+$P$1</f>
         <v>237266.08760950522</v>
       </c>
       <c r="Q72">
@@ -3903,11 +3867,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A73" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C73">
@@ -3951,7 +3915,7 @@
         <v>0</v>
       </c>
       <c r="P73">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>242193.03042265025</v>
       </c>
       <c r="Q73">
@@ -3967,7 +3931,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A75" t="s">
         <v>20</v>
       </c>
@@ -4015,7 +3979,7 @@
         <v>0</v>
       </c>
       <c r="P75">
-        <f t="shared" ref="P75:P76" si="15">D75+$P$1</f>
+        <f t="shared" ref="P75:P76" si="13">D75+$P$1</f>
         <v>237266.08760950161</v>
       </c>
       <c r="Q75">
@@ -4025,7 +3989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -4037,65 +4001,71 @@
       </c>
       <c r="D76">
         <f>J76+K76+L76+M76+N76</f>
-        <v>121381.93605468499</v>
+        <v>121744.79706913032</v>
       </c>
       <c r="E76">
-        <v>282179.671232878</v>
+        <v>282179.88376308198</v>
       </c>
       <c r="F76">
-        <v>0.857351410648304</v>
-      </c>
-      <c r="G76" s="4">
-        <v>21285.1004075495</v>
+        <v>0.85713546401894802</v>
+      </c>
+      <c r="G76">
+        <v>21291.5607898614</v>
       </c>
       <c r="H76">
-        <v>7426.32532798384</v>
+        <v>7432.3603175362596</v>
       </c>
       <c r="I76">
-        <v>5046.79446201879</v>
+        <v>5035.2758648834497</v>
       </c>
       <c r="J76">
-        <v>33758.220197552102</v>
+        <v>33759.196972281097</v>
       </c>
       <c r="K76">
-        <v>51144.191344099498</v>
+        <v>51128.3645002267</v>
       </c>
       <c r="L76">
-        <v>16112.7556071296</v>
+        <v>16070.129576240101</v>
       </c>
       <c r="M76">
-        <v>19359.989512119799</v>
+        <v>19356.7120304526</v>
       </c>
       <c r="N76">
-        <v>1006.77939378399</v>
+        <v>1430.39398992981</v>
       </c>
       <c r="O76">
         <v>0</v>
       </c>
       <c r="P76">
-        <f t="shared" si="15"/>
-        <v>241941.60787368153</v>
+        <f t="shared" si="13"/>
+        <v>242304.46888812684</v>
       </c>
       <c r="Q76">
-        <v>1178.65858109644</v>
+        <v>1179.61640190856</v>
       </c>
       <c r="R76">
-        <v>12586.325853030899</v>
+        <v>13411.4010346792</v>
       </c>
       <c r="S76">
-        <v>466.16021677892502</v>
+        <v>478.97860838140201</v>
       </c>
       <c r="T76">
-        <v>1.3585822738026401</v>
-      </c>
-    </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.35">
+        <v>0.22564405635506199</v>
+      </c>
+      <c r="U76">
+        <v>10550.3210016294</v>
+      </c>
+      <c r="V76">
+        <v>75.359435725924598</v>
+      </c>
+    </row>
+    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A78" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G78" s="4"/>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A79" t="s">
         <v>22</v>
       </c>
@@ -4143,7 +4113,7 @@
         <v>0</v>
       </c>
       <c r="P79">
-        <f t="shared" ref="P79:P80" si="16">D79+$P$1</f>
+        <f t="shared" ref="P79" si="14">D79+$P$1</f>
         <v>267678.15388715523</v>
       </c>
       <c r="Q79">
@@ -4159,7 +4129,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A80" t="s">
         <v>22</v>
       </c>
@@ -4203,7 +4173,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="82" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="A82" s="1" t="s">
         <v>26</v>
       </c>
@@ -4224,7 +4194,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="83" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="A83" t="s">
         <v>0</v>
       </c>
@@ -4286,7 +4256,7 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="A84" s="2" t="s">
         <v>20</v>
       </c>
@@ -4348,12 +4318,12 @@
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A85" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A87" t="s">
         <v>32</v>
       </c>
@@ -4364,7 +4334,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A88">
         <v>20</v>
       </c>
@@ -4375,7 +4345,7 @@
         <v>2</v>
       </c>
       <c r="D88">
-        <f t="shared" ref="D88:D94" si="17">J88+K88+L88+M88+N88</f>
+        <f t="shared" ref="D88:D94" si="15">J88+K88+L88+M88+N88</f>
         <v>120712.69088313227</v>
       </c>
       <c r="E88">
@@ -4412,7 +4382,7 @@
         <v>0</v>
       </c>
       <c r="P88">
-        <f t="shared" ref="P88:P95" si="18">D88+$P$1</f>
+        <f t="shared" ref="P88:P94" si="16">D88+$P$1</f>
         <v>241272.36270212877</v>
       </c>
       <c r="Q88">
@@ -4428,7 +4398,7 @@
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A89">
         <v>20</v>
       </c>
@@ -4439,7 +4409,7 @@
         <v>2</v>
       </c>
       <c r="D89">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>119392.42354269064</v>
       </c>
       <c r="E89">
@@ -4476,7 +4446,7 @@
         <v>0</v>
       </c>
       <c r="P89">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>239952.09536168716</v>
       </c>
       <c r="Q89">
@@ -4492,7 +4462,7 @@
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A90">
         <v>20</v>
       </c>
@@ -4503,7 +4473,7 @@
         <v>2</v>
       </c>
       <c r="D90">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>117777.02945340994</v>
       </c>
       <c r="E90">
@@ -4540,7 +4510,7 @@
         <v>0</v>
       </c>
       <c r="P90">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>238336.70127240644</v>
       </c>
       <c r="Q90">
@@ -4556,7 +4526,7 @@
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A91">
         <v>20</v>
       </c>
@@ -4567,7 +4537,7 @@
         <v>2</v>
       </c>
       <c r="D91">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>116625.1695160947</v>
       </c>
       <c r="E91">
@@ -4604,7 +4574,7 @@
         <v>0</v>
       </c>
       <c r="P91">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>237184.84133509122</v>
       </c>
       <c r="Q91">
@@ -4620,7 +4590,7 @@
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A92" s="3">
         <v>20</v>
       </c>
@@ -4631,7 +4601,7 @@
         <v>2</v>
       </c>
       <c r="D92">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>115198.459983006</v>
       </c>
       <c r="E92">
@@ -4668,7 +4638,7 @@
         <v>0</v>
       </c>
       <c r="P92">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>235758.13180200252</v>
       </c>
       <c r="Q92">
@@ -4684,7 +4654,7 @@
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A93">
         <v>20</v>
       </c>
@@ -4695,7 +4665,7 @@
         <v>2</v>
       </c>
       <c r="D93">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>114451.25872361983</v>
       </c>
       <c r="E93">
@@ -4732,7 +4702,7 @@
         <v>0</v>
       </c>
       <c r="P93">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>235010.93054261635</v>
       </c>
       <c r="Q93">
@@ -4748,7 +4718,7 @@
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A94">
         <v>20</v>
       </c>
@@ -4759,7 +4729,7 @@
         <v>2</v>
       </c>
       <c r="D94">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>114787.7594081375</v>
       </c>
       <c r="E94">
@@ -4796,7 +4766,7 @@
         <v>0</v>
       </c>
       <c r="P94">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>235347.43122713402</v>
       </c>
       <c r="Q94">

</xml_diff>

<commit_message>
Update to demand response revenue baseline power calculation
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A0584AE-2B19-4DEC-8544-012E51EE8479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{375D47A7-1E45-478A-AACA-52386B27996A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -48,6 +48,8 @@
     <author>tc={F9308CF0-AB74-4ABB-91B6-7382ECEADD39}</author>
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
     <author>tc={7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}</author>
+    <author>tc={B12FED98-6BE9-4BE2-A887-4CF314FA442B}</author>
+    <author>tc={667E4A37-89FC-4B6E-B3D1-92EA6BC08C00}</author>
     <author>tc={4644E393-F522-4E79-88BA-041770B595A7}</author>
     <author>tc={9FF6B967-6104-43AC-8EED-15C48C9ACCA9}</author>
     <author>tc={86E634AB-9E52-4A6D-BE85-5D191C9227C6}</author>
@@ -161,7 +163,23 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="A73" authorId="13" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
+    <comment ref="A58" authorId="13" shapeId="0" xr:uid="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Wrong baseline power was used</t>
+      </text>
+    </comment>
+    <comment ref="A59" authorId="14" shapeId="0" xr:uid="{667E4A37-89FC-4B6E-B3D1-92EA6BC08C00}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Wrong baseline power used</t>
+      </text>
+    </comment>
+    <comment ref="A73" authorId="15" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -169,7 +187,7 @@
     Pretty sure this solution is wrong, but I don’t think I need this case for the paper</t>
       </text>
     </comment>
-    <comment ref="A79" authorId="14" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A79" authorId="16" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -177,7 +195,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T91" authorId="15" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T91" authorId="17" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1273,6 +1291,12 @@
   <threadedComment ref="A55" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
     <text>Result from the fast solve</text>
   </threadedComment>
+  <threadedComment ref="A58" dT="2026-07-21T19:50:00.59" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
+    <text>Wrong baseline power was used</text>
+  </threadedComment>
+  <threadedComment ref="A59" dT="2026-07-21T19:50:19.49" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{667E4A37-89FC-4B6E-B3D1-92EA6BC08C00}">
+    <text>Wrong baseline power used</text>
+  </threadedComment>
   <threadedComment ref="A73" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
     <text>Pretty sure this solution is wrong, but I don’t think I need this case for the paper</text>
   </threadedComment>
@@ -2832,7 +2856,7 @@
         <v>0</v>
       </c>
       <c r="P37">
-        <f t="shared" ref="P37:P39" si="7">D37+$P$1</f>
+        <f t="shared" ref="P37:P38" si="7">D37+$P$1</f>
         <v>237538.1865021491</v>
       </c>
       <c r="Q37">
@@ -3146,7 +3170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A49" s="5" t="s">
         <v>22</v>
       </c>
@@ -3210,11 +3234,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A50" s="3"/>
       <c r="G50" s="4"/>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>20</v>
       </c>
@@ -3278,7 +3302,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>22</v>
       </c>
@@ -3342,10 +3366,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G53" s="4"/>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A54" s="3" t="s">
         <v>20</v>
       </c>
@@ -3409,7 +3433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>22</v>
       </c>
@@ -3473,17 +3497,17 @@
         <v>0.51444695802960605</v>
       </c>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A57" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G57" s="4"/>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A58" t="s">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A58" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C58">
@@ -3543,11 +3567,11 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A59" t="s">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A59" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C59">
@@ -3607,16 +3631,16 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G60" s="4"/>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A61" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G61" s="4"/>
     </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A62" s="3" t="s">
         <v>20</v>
       </c>
@@ -3628,19 +3652,71 @@
       </c>
       <c r="G62" s="4"/>
     </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A63" s="3" t="s">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A63" t="s">
         <v>22</v>
       </c>
-      <c r="B63" s="3" t="s">
+      <c r="B63" t="s">
         <v>23</v>
       </c>
-      <c r="C63" s="3">
-        <v>0</v>
-      </c>
-      <c r="G63" s="4"/>
-    </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="C63">
+        <v>0</v>
+      </c>
+      <c r="D63">
+        <f>J63+K63+L63+M63+N63</f>
+        <v>125092.66169779528</v>
+      </c>
+      <c r="E63">
+        <v>282190.859999999</v>
+      </c>
+      <c r="F63">
+        <v>0.87440267535043703</v>
+      </c>
+      <c r="G63">
+        <v>24203.5781618162</v>
+      </c>
+      <c r="H63">
+        <v>4932.7402012145303</v>
+      </c>
+      <c r="I63">
+        <v>9098.6050451690407</v>
+      </c>
+      <c r="J63">
+        <v>38234.9234081998</v>
+      </c>
+      <c r="K63">
+        <v>50845.200000000099</v>
+      </c>
+      <c r="L63">
+        <v>15304.405199999899</v>
+      </c>
+      <c r="M63">
+        <v>19298.29566</v>
+      </c>
+      <c r="N63">
+        <v>1409.83742959549</v>
+      </c>
+      <c r="O63">
+        <v>-1513.63614835872</v>
+      </c>
+      <c r="P63">
+        <f t="shared" ref="P63" si="11">D63+$P$1</f>
+        <v>245652.33351679181</v>
+      </c>
+      <c r="Q63">
+        <v>1102.09632181082</v>
+      </c>
+      <c r="R63">
+        <v>0</v>
+      </c>
+      <c r="U63">
+        <v>16.182064218907001</v>
+      </c>
+      <c r="V63">
+        <v>9.63218108268276E-2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
@@ -3726,7 +3802,7 @@
         <v>0</v>
       </c>
       <c r="P69">
-        <f t="shared" ref="P69:P70" si="11">D69+$P$1</f>
+        <f t="shared" ref="P69:P70" si="12">D69+$P$1</f>
         <v>236582.9608490612</v>
       </c>
       <c r="Q69">
@@ -3790,7 +3866,7 @@
         <v>0</v>
       </c>
       <c r="P70">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>246323.22923633162</v>
       </c>
       <c r="Q70">
@@ -3857,7 +3933,7 @@
         <v>0</v>
       </c>
       <c r="P72">
-        <f t="shared" ref="P72:P73" si="12">D72+$P$1</f>
+        <f t="shared" ref="P72:P73" si="13">D72+$P$1</f>
         <v>237266.08760950522</v>
       </c>
       <c r="Q72">
@@ -3915,7 +3991,7 @@
         <v>0</v>
       </c>
       <c r="P73">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>242193.03042265025</v>
       </c>
       <c r="Q73">
@@ -3979,7 +4055,7 @@
         <v>0</v>
       </c>
       <c r="P75">
-        <f t="shared" ref="P75:P76" si="13">D75+$P$1</f>
+        <f t="shared" ref="P75:P76" si="14">D75+$P$1</f>
         <v>237266.08760950161</v>
       </c>
       <c r="Q75">
@@ -4037,7 +4113,7 @@
         <v>0</v>
       </c>
       <c r="P76">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>242304.46888812684</v>
       </c>
       <c r="Q76">
@@ -4113,7 +4189,7 @@
         <v>0</v>
       </c>
       <c r="P79">
-        <f t="shared" ref="P79" si="14">D79+$P$1</f>
+        <f t="shared" ref="P79" si="15">D79+$P$1</f>
         <v>267678.15388715523</v>
       </c>
       <c r="Q79">
@@ -4345,7 +4421,7 @@
         <v>2</v>
       </c>
       <c r="D88">
-        <f t="shared" ref="D88:D94" si="15">J88+K88+L88+M88+N88</f>
+        <f t="shared" ref="D88:D94" si="16">J88+K88+L88+M88+N88</f>
         <v>120712.69088313227</v>
       </c>
       <c r="E88">
@@ -4382,7 +4458,7 @@
         <v>0</v>
       </c>
       <c r="P88">
-        <f t="shared" ref="P88:P94" si="16">D88+$P$1</f>
+        <f t="shared" ref="P88:P94" si="17">D88+$P$1</f>
         <v>241272.36270212877</v>
       </c>
       <c r="Q88">
@@ -4409,7 +4485,7 @@
         <v>2</v>
       </c>
       <c r="D89">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>119392.42354269064</v>
       </c>
       <c r="E89">
@@ -4446,7 +4522,7 @@
         <v>0</v>
       </c>
       <c r="P89">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>239952.09536168716</v>
       </c>
       <c r="Q89">
@@ -4473,7 +4549,7 @@
         <v>2</v>
       </c>
       <c r="D90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>117777.02945340994</v>
       </c>
       <c r="E90">
@@ -4510,7 +4586,7 @@
         <v>0</v>
       </c>
       <c r="P90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>238336.70127240644</v>
       </c>
       <c r="Q90">
@@ -4537,7 +4613,7 @@
         <v>2</v>
       </c>
       <c r="D91">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>116625.1695160947</v>
       </c>
       <c r="E91">
@@ -4574,7 +4650,7 @@
         <v>0</v>
       </c>
       <c r="P91">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>237184.84133509122</v>
       </c>
       <c r="Q91">
@@ -4601,7 +4677,7 @@
         <v>2</v>
       </c>
       <c r="D92">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>115198.459983006</v>
       </c>
       <c r="E92">
@@ -4638,7 +4714,7 @@
         <v>0</v>
       </c>
       <c r="P92">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>235758.13180200252</v>
       </c>
       <c r="Q92">
@@ -4665,7 +4741,7 @@
         <v>2</v>
       </c>
       <c r="D93">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>114451.25872361983</v>
       </c>
       <c r="E93">
@@ -4702,7 +4778,7 @@
         <v>0</v>
       </c>
       <c r="P93">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>235010.93054261635</v>
       </c>
       <c r="Q93">
@@ -4729,7 +4805,7 @@
         <v>2</v>
       </c>
       <c r="D94">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>114787.7594081375</v>
       </c>
       <c r="E94">
@@ -4766,7 +4842,7 @@
         <v>0</v>
       </c>
       <c r="P94">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>235347.43122713402</v>
       </c>
       <c r="Q94">

</xml_diff>

<commit_message>
Redoing DR result with smaller MIP gap to comare against the CPP
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF67E9D6-57CD-4841-9F45-FE6F6A9FCBF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{123C8684-B9A9-4BCE-AFA6-D698B791E854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -49,6 +49,7 @@
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
     <author>tc={7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}</author>
     <author>tc={B12FED98-6BE9-4BE2-A887-4CF314FA442B}</author>
+    <author>tc={FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}</author>
     <author>tc={4644E393-F522-4E79-88BA-041770B595A7}</author>
     <author>tc={9FF6B967-6104-43AC-8EED-15C48C9ACCA9}</author>
     <author>tc={86E634AB-9E52-4A6D-BE85-5D191C9227C6}</author>
@@ -170,7 +171,16 @@
     Wrong baseline power was used</t>
       </text>
     </comment>
-    <comment ref="A73" authorId="14" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
+    <comment ref="A66" authorId="14" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Why is this so different from the other DR solution? I would assume they would be the same…
+</t>
+      </text>
+    </comment>
+    <comment ref="A73" authorId="15" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -178,7 +188,7 @@
     Pretty sure this solution is wrong, but I don’t think I need this case for the paper</t>
       </text>
     </comment>
-    <comment ref="A79" authorId="15" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A79" authorId="16" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -186,7 +196,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T91" authorId="16" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T91" authorId="17" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -337,7 +347,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -498,6 +508,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -841,7 +857,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -850,6 +866,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1279,6 +1296,10 @@
   <threadedComment ref="A58" dT="2026-07-21T19:50:00.59" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
     <text>Wrong baseline power was used</text>
   </threadedComment>
+  <threadedComment ref="A66" dT="2026-07-22T16:56:30.58" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+    <text xml:space="preserve">Why is this so different from the other DR solution? I would assume they would be the same…
+</text>
+  </threadedComment>
   <threadedComment ref="A73" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
     <text>Pretty sure this solution is wrong, but I don’t think I need this case for the paper</text>
   </threadedComment>
@@ -3615,7 +3636,74 @@
       </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="G60" s="4"/>
+      <c r="D60">
+        <f>D59-D4</f>
+        <v>-11944.94926545964</v>
+      </c>
+      <c r="E60">
+        <f t="shared" ref="E60:T60" si="11">E59-E4</f>
+        <v>0</v>
+      </c>
+      <c r="F60">
+        <f t="shared" si="11"/>
+        <v>-3.947802828074698E-2</v>
+      </c>
+      <c r="G60">
+        <f t="shared" si="11"/>
+        <v>-342.33283128200128</v>
+      </c>
+      <c r="H60">
+        <f t="shared" si="11"/>
+        <v>1621.8180095940897</v>
+      </c>
+      <c r="I60">
+        <f t="shared" si="11"/>
+        <v>-3026.2022194955298</v>
+      </c>
+      <c r="J60">
+        <f t="shared" si="11"/>
+        <v>-1746.7170411834013</v>
+      </c>
+      <c r="K60">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="L60">
+        <f t="shared" si="11"/>
+        <v>1074.9999999999</v>
+      </c>
+      <c r="M60">
+        <f t="shared" si="11"/>
+        <v>151.82000000010157</v>
+      </c>
+      <c r="N60">
+        <f t="shared" si="11"/>
+        <v>-405.05222427625995</v>
+      </c>
+      <c r="O60">
+        <f t="shared" si="11"/>
+        <v>11020</v>
+      </c>
+      <c r="P60">
+        <f t="shared" si="11"/>
+        <v>-11944.94926545964</v>
+      </c>
+      <c r="Q60">
+        <f t="shared" si="11"/>
+        <v>362.35430817542988</v>
+      </c>
+      <c r="R60">
+        <f t="shared" si="11"/>
+        <v>26064.489084194902</v>
+      </c>
+      <c r="S60">
+        <f t="shared" si="11"/>
+        <v>407.257641940545</v>
+      </c>
+      <c r="T60">
+        <f t="shared" si="11"/>
+        <v>1.09609872121186</v>
+      </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A61" s="1" t="s">
@@ -3718,19 +3806,152 @@
       <c r="G65" s="4"/>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A66" s="3" t="s">
+      <c r="A66" t="s">
         <v>22</v>
       </c>
-      <c r="B66" s="3" t="s">
+      <c r="B66" t="s">
         <v>21</v>
       </c>
-      <c r="C66" s="3">
+      <c r="C66">
         <v>4</v>
+      </c>
+      <c r="D66">
+        <v>108832.74020782999</v>
+      </c>
+      <c r="E66">
+        <v>282179.67123306898</v>
+      </c>
+      <c r="F66">
+        <v>0.81644691741250097</v>
+      </c>
+      <c r="G66">
+        <v>19728.523245555101</v>
+      </c>
+      <c r="H66">
+        <v>6281.7321988746498</v>
+      </c>
+      <c r="I66" s="8">
+        <v>9.8877442286147301E-6</v>
+      </c>
+      <c r="J66">
+        <v>26010.255454317499</v>
+      </c>
+      <c r="K66">
+        <v>50944.9452054754</v>
+      </c>
+      <c r="L66">
+        <v>20235.614943009699</v>
+      </c>
+      <c r="M66">
+        <v>19962.024605027898</v>
+      </c>
+      <c r="N66">
+        <v>1462.3779549220301</v>
+      </c>
+      <c r="O66">
+        <v>8320.1</v>
+      </c>
+      <c r="P66">
+        <v>230384.72273471201</v>
+      </c>
+      <c r="Q66">
+        <v>1403.49453592792</v>
+      </c>
+      <c r="R66">
+        <v>34518.506961381201</v>
+      </c>
+      <c r="S66">
+        <v>841.91480393612801</v>
+      </c>
+      <c r="T66">
+        <v>0.38784649209264499</v>
+      </c>
+      <c r="U66">
+        <v>38264.627438579002</v>
+      </c>
+      <c r="V66">
+        <v>301.29627904392902</v>
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A67" s="5"/>
       <c r="B67" s="5"/>
+      <c r="D67">
+        <f>D66-D63</f>
+        <v>-16260.494075352748</v>
+      </c>
+      <c r="E67">
+        <f t="shared" ref="E67:V67" si="12">E66-E63</f>
+        <v>-11.188766930019483</v>
+      </c>
+      <c r="F67">
+        <f t="shared" si="12"/>
+        <v>-5.2593913252494073E-2</v>
+      </c>
+      <c r="G67">
+        <f t="shared" si="12"/>
+        <v>-4474.9745192109003</v>
+      </c>
+      <c r="H67">
+        <f t="shared" si="12"/>
+        <v>1349.0083827482595</v>
+      </c>
+      <c r="I67">
+        <f t="shared" si="12"/>
+        <v>-9098.574812435656</v>
+      </c>
+      <c r="J67">
+        <f t="shared" si="12"/>
+        <v>-12224.540948898299</v>
+      </c>
+      <c r="K67">
+        <f t="shared" si="12"/>
+        <v>99.745205475301191</v>
+      </c>
+      <c r="L67">
+        <f t="shared" si="12"/>
+        <v>4931.2097430098001</v>
+      </c>
+      <c r="M67">
+        <f t="shared" si="12"/>
+        <v>663.72894502789859</v>
+      </c>
+      <c r="N67">
+        <f t="shared" si="12"/>
+        <v>52.540525326540092</v>
+      </c>
+      <c r="O67">
+        <f t="shared" si="12"/>
+        <v>8320.7995903714655</v>
+      </c>
+      <c r="P67">
+        <f t="shared" si="12"/>
+        <v>-15268.183367467253</v>
+      </c>
+      <c r="Q67">
+        <f t="shared" si="12"/>
+        <v>301.40187495156988</v>
+      </c>
+      <c r="R67">
+        <f t="shared" si="12"/>
+        <v>34518.506961381201</v>
+      </c>
+      <c r="S67">
+        <f t="shared" si="12"/>
+        <v>841.91480393612801</v>
+      </c>
+      <c r="T67">
+        <f t="shared" si="12"/>
+        <v>0.38784649209264499</v>
+      </c>
+      <c r="U67">
+        <f t="shared" si="12"/>
+        <v>38249.060394551692</v>
+      </c>
+      <c r="V67">
+        <f t="shared" si="12"/>
+        <v>301.20361806757597</v>
+      </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A68" s="1" t="s">
@@ -3785,7 +4006,7 @@
         <v>0</v>
       </c>
       <c r="P69">
-        <f t="shared" ref="P69:P70" si="11">D69+$P$1</f>
+        <f t="shared" ref="P69:P70" si="13">D69+$P$1</f>
         <v>236582.9608490612</v>
       </c>
       <c r="Q69">
@@ -3849,7 +4070,7 @@
         <v>0</v>
       </c>
       <c r="P70">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>246323.22923633162</v>
       </c>
       <c r="Q70">
@@ -3916,7 +4137,7 @@
         <v>0</v>
       </c>
       <c r="P72">
-        <f t="shared" ref="P72:P73" si="12">D72+$P$1</f>
+        <f t="shared" ref="P72:P73" si="14">D72+$P$1</f>
         <v>237266.08760950522</v>
       </c>
       <c r="Q72">
@@ -3974,7 +4195,7 @@
         <v>0</v>
       </c>
       <c r="P73">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>242193.03042265025</v>
       </c>
       <c r="Q73">
@@ -4038,7 +4259,7 @@
         <v>0</v>
       </c>
       <c r="P75">
-        <f t="shared" ref="P75:P76" si="13">D75+$P$1</f>
+        <f t="shared" ref="P75:P77" si="15">D75+$P$1</f>
         <v>237266.08760950161</v>
       </c>
       <c r="Q75">
@@ -4096,7 +4317,7 @@
         <v>0</v>
       </c>
       <c r="P76">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>242304.46888812684</v>
       </c>
       <c r="Q76">
@@ -4116,6 +4337,56 @@
       </c>
       <c r="V76">
         <v>75.359435725924598</v>
+      </c>
+    </row>
+    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="D77">
+        <f>D76-D70</f>
+        <v>-4018.7603482047853</v>
+      </c>
+      <c r="E77">
+        <f t="shared" ref="E77:N77" si="16">E76-E70</f>
+        <v>0.21251127298455685</v>
+      </c>
+      <c r="F77">
+        <f t="shared" si="16"/>
+        <v>-1.5794992464996938E-2</v>
+      </c>
+      <c r="G77">
+        <f t="shared" si="16"/>
+        <v>-1335.1371720950992</v>
+      </c>
+      <c r="H77">
+        <f t="shared" si="16"/>
+        <v>329.78360458492989</v>
+      </c>
+      <c r="I77">
+        <f t="shared" si="16"/>
+        <v>-4562.1832736040305</v>
+      </c>
+      <c r="J77">
+        <f t="shared" si="16"/>
+        <v>-5567.5368411142044</v>
+      </c>
+      <c r="K77">
+        <f t="shared" si="16"/>
+        <v>285.1804885383026</v>
+      </c>
+      <c r="L77">
+        <f t="shared" si="16"/>
+        <v>766.33118310559985</v>
+      </c>
+      <c r="M77">
+        <f t="shared" si="16"/>
+        <v>59.181539221001003</v>
+      </c>
+      <c r="N77">
+        <f t="shared" si="16"/>
+        <v>438.08328204450595</v>
+      </c>
+      <c r="P77">
+        <f t="shared" si="15"/>
+        <v>116540.91147079173</v>
       </c>
     </row>
     <row r="78" spans="1:22" x14ac:dyDescent="0.4">
@@ -4172,7 +4443,7 @@
         <v>0</v>
       </c>
       <c r="P79">
-        <f t="shared" ref="P79" si="14">D79+$P$1</f>
+        <f t="shared" ref="P79" si="17">D79+$P$1</f>
         <v>267678.15388715523</v>
       </c>
       <c r="Q79">
@@ -4404,7 +4675,7 @@
         <v>2</v>
       </c>
       <c r="D88">
-        <f t="shared" ref="D88:D94" si="15">J88+K88+L88+M88+N88</f>
+        <f t="shared" ref="D88:D94" si="18">J88+K88+L88+M88+N88</f>
         <v>120712.69088313227</v>
       </c>
       <c r="E88">
@@ -4441,7 +4712,7 @@
         <v>0</v>
       </c>
       <c r="P88">
-        <f t="shared" ref="P88:P94" si="16">D88+$P$1</f>
+        <f t="shared" ref="P88:P94" si="19">D88+$P$1</f>
         <v>241272.36270212877</v>
       </c>
       <c r="Q88">
@@ -4468,7 +4739,7 @@
         <v>2</v>
       </c>
       <c r="D89">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>119392.42354269064</v>
       </c>
       <c r="E89">
@@ -4505,7 +4776,7 @@
         <v>0</v>
       </c>
       <c r="P89">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>239952.09536168716</v>
       </c>
       <c r="Q89">
@@ -4532,7 +4803,7 @@
         <v>2</v>
       </c>
       <c r="D90">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>117777.02945340994</v>
       </c>
       <c r="E90">
@@ -4569,7 +4840,7 @@
         <v>0</v>
       </c>
       <c r="P90">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>238336.70127240644</v>
       </c>
       <c r="Q90">
@@ -4596,7 +4867,7 @@
         <v>2</v>
       </c>
       <c r="D91">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>116625.1695160947</v>
       </c>
       <c r="E91">
@@ -4633,7 +4904,7 @@
         <v>0</v>
       </c>
       <c r="P91">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>237184.84133509122</v>
       </c>
       <c r="Q91">
@@ -4660,7 +4931,7 @@
         <v>2</v>
       </c>
       <c r="D92">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>115198.459983006</v>
       </c>
       <c r="E92">
@@ -4697,7 +4968,7 @@
         <v>0</v>
       </c>
       <c r="P92">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>235758.13180200252</v>
       </c>
       <c r="Q92">
@@ -4724,7 +4995,7 @@
         <v>2</v>
       </c>
       <c r="D93">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>114451.25872361983</v>
       </c>
       <c r="E93">
@@ -4761,7 +5032,7 @@
         <v>0</v>
       </c>
       <c r="P93">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>235010.93054261635</v>
       </c>
       <c r="Q93">
@@ -4788,7 +5059,7 @@
         <v>2</v>
       </c>
       <c r="D94">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>114787.7594081375</v>
       </c>
       <c r="E94">
@@ -4825,7 +5096,7 @@
         <v>0</v>
       </c>
       <c r="P94">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>235347.43122713402</v>
       </c>
       <c r="Q94">

</xml_diff>

<commit_message>
Testing a DR scenario with one plant shutdown
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{123C8684-B9A9-4BCE-AFA6-D698B791E854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A5B651-2BB1-42D9-89F9-4DDB7DF3E311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -49,6 +49,8 @@
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
     <author>tc={7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}</author>
     <author>tc={B12FED98-6BE9-4BE2-A887-4CF314FA442B}</author>
+    <author>tc={7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}</author>
+    <author>tc={B7EDEAAD-67C9-4693-A0FC-570282E02182}</author>
     <author>tc={FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}</author>
     <author>tc={4644E393-F522-4E79-88BA-041770B595A7}</author>
     <author>tc={9FF6B967-6104-43AC-8EED-15C48C9ACCA9}</author>
@@ -171,7 +173,25 @@
     Wrong baseline power was used</t>
       </text>
     </comment>
-    <comment ref="A66" authorId="14" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+    <comment ref="A59" authorId="14" shapeId="0" xr:uid="{7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Old solution where there is only one plant shutdown.</t>
+      </text>
+    </comment>
+    <comment ref="A60" authorId="15" shapeId="0" xr:uid="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Solution where there is a shutdown for all peak hours
+Reply:
+    I’d like to see numbers for only one shutdown</t>
+      </text>
+    </comment>
+    <comment ref="A67" authorId="16" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -180,7 +200,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="A73" authorId="15" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
+    <comment ref="A74" authorId="17" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -188,7 +208,7 @@
     Pretty sure this solution is wrong, but I don’t think I need this case for the paper</t>
       </text>
     </comment>
-    <comment ref="A79" authorId="16" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A80" authorId="18" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -196,7 +216,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T91" authorId="17" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T92" authorId="19" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -209,7 +229,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="44">
   <si>
     <t>Season</t>
   </si>
@@ -1296,17 +1316,26 @@
   <threadedComment ref="A58" dT="2026-07-21T19:50:00.59" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
     <text>Wrong baseline power was used</text>
   </threadedComment>
-  <threadedComment ref="A66" dT="2026-07-22T16:56:30.58" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+  <threadedComment ref="A59" dT="2026-07-22T19:28:49.80" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}">
+    <text>Old solution where there is only one plant shutdown.</text>
+  </threadedComment>
+  <threadedComment ref="A60" dT="2026-07-22T19:29:10.19" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
+    <text>Solution where there is a shutdown for all peak hours</text>
+  </threadedComment>
+  <threadedComment ref="A60" dT="2026-07-22T19:37:51.21" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{DB15DF8F-6887-4CDD-9A38-5D318EAEEFFF}" parentId="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
+    <text>I’d like to see numbers for only one shutdown</text>
+  </threadedComment>
+  <threadedComment ref="A67" dT="2026-07-22T16:56:30.58" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
     <text xml:space="preserve">Why is this so different from the other DR solution? I would assume they would be the same…
 </text>
   </threadedComment>
-  <threadedComment ref="A73" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
+  <threadedComment ref="A74" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
     <text>Pretty sure this solution is wrong, but I don’t think I need this case for the paper</text>
   </threadedComment>
-  <threadedComment ref="A79" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+  <threadedComment ref="A80" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
     <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
   </threadedComment>
-  <threadedComment ref="T91" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="T92" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1314,21 +1343,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:V94"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:V95"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.61328125" customWidth="1"/>
-    <col min="3" max="3" width="11.4609375" customWidth="1"/>
-    <col min="5" max="5" width="10.23046875" customWidth="1"/>
-    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.69140625" customWidth="1"/>
-    <col min="9" max="9" width="9.07421875" customWidth="1"/>
-    <col min="15" max="15" width="9.53515625" customWidth="1"/>
-    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.84375" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" customWidth="1"/>
+    <col min="3" max="3" width="11.453125" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="15" max="15" width="9.54296875" customWidth="1"/>
+    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1339,7 +1368,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1407,7 +1436,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1471,7 +1500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1535,10 +1564,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1602,7 +1631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -1666,10 +1695,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1733,7 +1762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -1797,10 +1826,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -1864,7 +1893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -1928,10 +1957,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1993,7 +2022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2049,10 +2078,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2116,7 +2145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2180,12 +2209,12 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2196,7 +2225,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2260,10 +2289,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2327,7 +2356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2397,11 +2426,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2465,7 +2494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2529,10 +2558,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2596,7 +2625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -2666,19 +2695,19 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="S32" s="2"/>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B33" s="2"/>
       <c r="S33" s="2"/>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>20</v>
       </c>
@@ -2742,7 +2771,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>22</v>
       </c>
@@ -2806,12 +2835,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A36" s="7"/>
       <c r="B36" s="2"/>
       <c r="S36" s="2"/>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>20</v>
       </c>
@@ -2878,7 +2907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>22</v>
       </c>
@@ -2948,20 +2977,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="3"/>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A40" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>22</v>
       </c>
@@ -3025,15 +3054,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43" s="3"/>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>22</v>
       </c>
@@ -3103,13 +3132,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G47" s="4"/>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
         <v>20</v>
       </c>
@@ -3173,7 +3202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
         <v>22</v>
       </c>
@@ -3237,11 +3266,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A50" s="3"/>
       <c r="G50" s="4"/>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>20</v>
       </c>
@@ -3305,7 +3334,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>22</v>
       </c>
@@ -3369,10 +3398,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G53" s="4"/>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
         <v>20</v>
       </c>
@@ -3436,7 +3465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>22</v>
       </c>
@@ -3500,13 +3529,13 @@
         <v>0.51444695802960605</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G57" s="4"/>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>22</v>
       </c>
@@ -3570,7 +3599,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
         <v>22</v>
       </c>
@@ -3635,396 +3664,410 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A60" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C60">
+        <v>4</v>
+      </c>
       <c r="D60">
-        <f>D59-D4</f>
-        <v>-11944.94926545964</v>
+        <v>106092.92029140001</v>
       </c>
       <c r="E60">
-        <f t="shared" ref="E60:T60" si="11">E59-E4</f>
-        <v>0</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F60">
+        <v>0.80673743017586796</v>
+      </c>
+      <c r="G60">
+        <v>19617.269555424798</v>
+      </c>
+      <c r="H60">
+        <v>6177.79087142139</v>
+      </c>
+      <c r="I60" s="8">
+        <v>1.4897343661976701E-5</v>
+      </c>
+      <c r="J60">
+        <v>25795.060441743601</v>
+      </c>
+      <c r="K60">
+        <v>50989.945229661498</v>
+      </c>
+      <c r="L60">
+        <v>20356.552509954701</v>
+      </c>
+      <c r="M60">
+        <v>19971.3621100407</v>
+      </c>
+      <c r="N60">
+        <v>1462.3779549220301</v>
+      </c>
+      <c r="O60">
+        <v>11020</v>
+      </c>
+      <c r="P60">
+        <v>227644.90281828199</v>
+      </c>
+      <c r="Q60">
+        <v>1380.27146414547</v>
+      </c>
+      <c r="R60">
+        <v>33980.634383525299</v>
+      </c>
+      <c r="S60">
+        <v>943.906510653483</v>
+      </c>
+      <c r="T60">
+        <v>0.36911323114551098</v>
+      </c>
+      <c r="U60">
+        <v>36719.7300995962</v>
+      </c>
+      <c r="V60">
+        <v>278.17977348178903</v>
+      </c>
+    </row>
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A61" s="3"/>
+      <c r="B61" s="3"/>
+      <c r="D61">
+        <f>D60-D59</f>
+        <v>-3470.0549869755487</v>
+      </c>
+      <c r="E61">
+        <f t="shared" ref="E61:V61" si="11">E60-E59</f>
+        <v>0</v>
+      </c>
+      <c r="F61">
         <f t="shared" si="11"/>
-        <v>-3.947802828074698E-2</v>
-      </c>
-      <c r="G60">
+        <v>-1.0153485538960005E-2</v>
+      </c>
+      <c r="G61">
         <f t="shared" si="11"/>
-        <v>-342.33283128200128</v>
-      </c>
-      <c r="H60">
+        <v>-667.82878678320048</v>
+      </c>
+      <c r="H61">
         <f t="shared" si="11"/>
-        <v>1621.8180095940897</v>
-      </c>
-      <c r="I60">
+        <v>-374.88135105099991</v>
+      </c>
+      <c r="I61">
         <f t="shared" si="11"/>
-        <v>-3026.2022194955298</v>
-      </c>
-      <c r="J60">
+        <v>-6068.9240419192656</v>
+      </c>
+      <c r="J61">
         <f t="shared" si="11"/>
-        <v>-1746.7170411834013</v>
-      </c>
-      <c r="K60">
+        <v>-7111.6341797534005</v>
+      </c>
+      <c r="K61">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="L60">
+        <v>146.76122373789985</v>
+      </c>
+      <c r="L61">
         <f t="shared" si="11"/>
-        <v>1074.9999999999</v>
-      </c>
-      <c r="M60">
+        <v>3977.7541241718009</v>
+      </c>
+      <c r="M61">
         <f t="shared" si="11"/>
-        <v>151.82000000010157</v>
-      </c>
-      <c r="N60">
+        <v>522.01162059239869</v>
+      </c>
+      <c r="N61">
         <f t="shared" si="11"/>
-        <v>-405.05222427625995</v>
-      </c>
-      <c r="O60">
+        <v>457.43017919829003</v>
+      </c>
+      <c r="O61">
         <f t="shared" si="11"/>
-        <v>11020</v>
-      </c>
-      <c r="P60">
+        <v>0</v>
+      </c>
+      <c r="P61">
         <f t="shared" si="11"/>
-        <v>-11944.94926545964</v>
-      </c>
-      <c r="Q60">
+        <v>-2477.7442790900823</v>
+      </c>
+      <c r="Q61">
         <f t="shared" si="11"/>
-        <v>362.35430817542988</v>
-      </c>
-      <c r="R60">
+        <v>-83.757789339369992</v>
+      </c>
+      <c r="R61">
         <f t="shared" si="11"/>
-        <v>26064.489084194902</v>
-      </c>
-      <c r="S60">
+        <v>7916.1452993303974</v>
+      </c>
+      <c r="S61">
         <f t="shared" si="11"/>
-        <v>407.257641940545</v>
-      </c>
-      <c r="T60">
+        <v>536.648868712938</v>
+      </c>
+      <c r="T61">
         <f t="shared" si="11"/>
-        <v>1.09609872121186</v>
-      </c>
-    </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A61" s="1" t="s">
+        <v>-0.72698549006634905</v>
+      </c>
+      <c r="U61">
+        <f t="shared" si="11"/>
+        <v>36719.7300995962</v>
+      </c>
+      <c r="V61">
+        <f t="shared" si="11"/>
+        <v>278.17977348178903</v>
+      </c>
+    </row>
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A62" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G61" s="4"/>
-    </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A62" s="3" t="s">
+      <c r="G62" s="4"/>
+    </row>
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A63" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B62" s="3" t="s">
+      <c r="B63" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C62" s="3">
-        <v>0</v>
-      </c>
-      <c r="G62" s="4"/>
-    </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A63" t="s">
+      <c r="C63" s="3">
+        <v>0</v>
+      </c>
+      <c r="G63" s="4"/>
+    </row>
+    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
         <v>22</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B64" t="s">
         <v>23</v>
       </c>
-      <c r="C63">
-        <v>0</v>
-      </c>
-      <c r="D63">
-        <f>J63+K63+L63+M63+N63-O63</f>
+      <c r="C64">
+        <v>0</v>
+      </c>
+      <c r="D64">
+        <f>J64+K64+L64+M64+N64-O64</f>
         <v>125093.23428318274</v>
       </c>
-      <c r="E63">
+      <c r="E64">
         <v>282190.859999999</v>
       </c>
-      <c r="F63">
+      <c r="F64">
         <v>0.86904083066499505</v>
       </c>
-      <c r="G63">
+      <c r="G64">
         <v>24203.497764766002</v>
       </c>
-      <c r="H63">
+      <c r="H64">
         <v>4932.7238161263904</v>
       </c>
-      <c r="I63">
+      <c r="I64">
         <v>9098.5748223234004</v>
       </c>
-      <c r="J63">
+      <c r="J64">
         <v>38234.796403215798</v>
       </c>
-      <c r="K63">
+      <c r="K64">
         <v>50845.200000000099</v>
       </c>
-      <c r="L63">
+      <c r="L64">
         <v>15304.405199999899</v>
       </c>
-      <c r="M63">
+      <c r="M64">
         <v>19298.29566</v>
       </c>
-      <c r="N63">
+      <c r="N64">
         <v>1409.83742959549</v>
       </c>
-      <c r="O63">
+      <c r="O64">
         <v>-0.69959037146548997</v>
       </c>
-      <c r="P63">
-        <f>D63+$P$1</f>
+      <c r="P64">
+        <f>D64+$P$1</f>
         <v>245652.90610217926</v>
       </c>
-      <c r="Q63">
+      <c r="Q64">
         <v>1102.0926609763501</v>
       </c>
-      <c r="R63">
-        <v>0</v>
-      </c>
-      <c r="U63">
+      <c r="R64">
+        <v>0</v>
+      </c>
+      <c r="U64">
         <v>15.5670440273115</v>
       </c>
-      <c r="V63">
+      <c r="V64">
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A64" s="3"/>
-      <c r="B64" s="3"/>
-      <c r="C64" s="3"/>
-      <c r="G64" s="4"/>
-    </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A65" s="3" t="s">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A65" s="3"/>
+      <c r="B65" s="3"/>
+      <c r="C65" s="3"/>
+      <c r="G65" s="4"/>
+    </row>
+    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A66" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B65" s="3" t="s">
+      <c r="B66" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C65" s="3">
+      <c r="C66" s="3">
         <v>4</v>
       </c>
-      <c r="G65" s="4"/>
-    </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A66" t="s">
+      <c r="G66" s="4"/>
+    </row>
+    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>22</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B67" t="s">
         <v>21</v>
       </c>
-      <c r="C66">
+      <c r="C67">
         <v>4</v>
       </c>
-      <c r="D66">
+      <c r="D67">
         <v>108832.74020782999</v>
       </c>
-      <c r="E66">
+      <c r="E67">
         <v>282179.67123306898</v>
       </c>
-      <c r="F66">
+      <c r="F67">
         <v>0.81644691741250097</v>
       </c>
-      <c r="G66">
+      <c r="G67">
         <v>19728.523245555101</v>
       </c>
-      <c r="H66">
+      <c r="H67">
         <v>6281.7321988746498</v>
       </c>
-      <c r="I66" s="8">
+      <c r="I67" s="8">
         <v>9.8877442286147301E-6</v>
       </c>
-      <c r="J66">
+      <c r="J67">
         <v>26010.255454317499</v>
       </c>
-      <c r="K66">
+      <c r="K67">
         <v>50944.9452054754</v>
       </c>
-      <c r="L66">
+      <c r="L67">
         <v>20235.614943009699</v>
       </c>
-      <c r="M66">
+      <c r="M67">
         <v>19962.024605027898</v>
       </c>
-      <c r="N66">
+      <c r="N67">
         <v>1462.3779549220301</v>
       </c>
-      <c r="O66">
+      <c r="O67">
         <v>8320.1</v>
       </c>
-      <c r="P66">
+      <c r="P67">
         <v>230384.72273471201</v>
       </c>
-      <c r="Q66">
+      <c r="Q67">
         <v>1403.49453592792</v>
       </c>
-      <c r="R66">
+      <c r="R67">
         <v>34518.506961381201</v>
       </c>
-      <c r="S66">
+      <c r="S67">
         <v>841.91480393612801</v>
       </c>
-      <c r="T66">
+      <c r="T67">
         <v>0.38784649209264499</v>
       </c>
-      <c r="U66">
+      <c r="U67">
         <v>38264.627438579002</v>
       </c>
-      <c r="V66">
+      <c r="V67">
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A67" s="5"/>
-      <c r="B67" s="5"/>
-      <c r="D67">
-        <f>D66-D63</f>
+    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A68" s="5"/>
+      <c r="B68" s="5"/>
+      <c r="D68">
+        <f>D67-D64</f>
         <v>-16260.494075352748</v>
       </c>
-      <c r="E67">
-        <f t="shared" ref="E67:V67" si="12">E66-E63</f>
+      <c r="E68">
+        <f t="shared" ref="E68:V68" si="12">E67-E64</f>
         <v>-11.188766930019483</v>
       </c>
-      <c r="F67">
+      <c r="F68">
         <f t="shared" si="12"/>
         <v>-5.2593913252494073E-2</v>
       </c>
-      <c r="G67">
+      <c r="G68">
         <f t="shared" si="12"/>
         <v>-4474.9745192109003</v>
       </c>
-      <c r="H67">
+      <c r="H68">
         <f t="shared" si="12"/>
         <v>1349.0083827482595</v>
       </c>
-      <c r="I67">
+      <c r="I68">
         <f t="shared" si="12"/>
         <v>-9098.574812435656</v>
       </c>
-      <c r="J67">
+      <c r="J68">
         <f t="shared" si="12"/>
         <v>-12224.540948898299</v>
       </c>
-      <c r="K67">
+      <c r="K68">
         <f t="shared" si="12"/>
         <v>99.745205475301191</v>
       </c>
-      <c r="L67">
+      <c r="L68">
         <f t="shared" si="12"/>
         <v>4931.2097430098001</v>
       </c>
-      <c r="M67">
+      <c r="M68">
         <f t="shared" si="12"/>
         <v>663.72894502789859</v>
       </c>
-      <c r="N67">
+      <c r="N68">
         <f t="shared" si="12"/>
         <v>52.540525326540092</v>
       </c>
-      <c r="O67">
+      <c r="O68">
         <f t="shared" si="12"/>
         <v>8320.7995903714655</v>
       </c>
-      <c r="P67">
+      <c r="P68">
         <f t="shared" si="12"/>
         <v>-15268.183367467253</v>
       </c>
-      <c r="Q67">
+      <c r="Q68">
         <f t="shared" si="12"/>
         <v>301.40187495156988</v>
       </c>
-      <c r="R67">
+      <c r="R68">
         <f t="shared" si="12"/>
         <v>34518.506961381201</v>
       </c>
-      <c r="S67">
+      <c r="S68">
         <f t="shared" si="12"/>
         <v>841.91480393612801</v>
       </c>
-      <c r="T67">
+      <c r="T68">
         <f t="shared" si="12"/>
         <v>0.38784649209264499</v>
       </c>
-      <c r="U67">
+      <c r="U68">
         <f t="shared" si="12"/>
         <v>38249.060394551692</v>
       </c>
-      <c r="V67">
+      <c r="V68">
         <f t="shared" si="12"/>
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A68" s="1" t="s">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A69" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A69" s="3" t="s">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A70" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C69">
-        <v>0</v>
-      </c>
-      <c r="D69">
-        <f>J69+K69+L69+M69+N69</f>
-        <v>116023.2890300647</v>
-      </c>
-      <c r="E69">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F69">
-        <v>0.83841249022441</v>
-      </c>
-      <c r="G69">
-        <v>20114.092712805999</v>
-      </c>
-      <c r="H69">
-        <v>6942.2846600808298</v>
-      </c>
-      <c r="I69">
-        <v>2530.0880681377598</v>
-      </c>
-      <c r="J69">
-        <v>29586.4654410246</v>
-      </c>
-      <c r="K69">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L69">
-        <v>15303.798385783</v>
-      </c>
-      <c r="M69">
-        <v>19297.5304894482</v>
-      </c>
-      <c r="N69">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O69">
-        <v>0</v>
-      </c>
-      <c r="P69">
-        <f t="shared" ref="P69:P70" si="13">D69+$P$1</f>
-        <v>236582.9608490612</v>
-      </c>
-      <c r="Q69">
-        <v>1101.8347602124099</v>
-      </c>
-      <c r="R69">
-        <v>0</v>
-      </c>
-      <c r="S69">
-        <v>0</v>
-      </c>
-      <c r="T69">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A70" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>23</v>
@@ -4034,34 +4077,34 @@
       </c>
       <c r="D70">
         <f>J70+K70+L70+M70+N70</f>
-        <v>125763.55741733511</v>
+        <v>116023.2890300647</v>
       </c>
       <c r="E70">
-        <v>282179.67125180899</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F70">
-        <v>0.87293045648394496</v>
+        <v>0.83841249022441</v>
       </c>
       <c r="G70">
-        <v>22626.697961956499</v>
+        <v>20114.092712805999</v>
       </c>
       <c r="H70">
-        <v>7102.5767129513297</v>
+        <v>6942.2846600808298</v>
       </c>
       <c r="I70">
-        <v>9597.4591384874802</v>
+        <v>2530.0880681377598</v>
       </c>
       <c r="J70">
-        <v>39326.733813395302</v>
+        <v>29586.4654410246</v>
       </c>
       <c r="K70">
-        <v>50843.184011688398</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L70">
-        <v>15303.798393134501</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M70">
-        <v>19297.530491231599</v>
+        <v>19297.5304894482</v>
       </c>
       <c r="N70">
         <v>992.31070788530405</v>
@@ -4070,88 +4113,94 @@
         <v>0</v>
       </c>
       <c r="P70">
+        <f t="shared" ref="P70:P71" si="13">D70+$P$1</f>
+        <v>236582.9608490612</v>
+      </c>
+      <c r="Q70">
+        <v>1101.8347602124099</v>
+      </c>
+      <c r="R70">
+        <v>0</v>
+      </c>
+      <c r="S70">
+        <v>0</v>
+      </c>
+      <c r="T70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A71" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C71">
+        <v>0</v>
+      </c>
+      <c r="D71">
+        <f>J71+K71+L71+M71+N71</f>
+        <v>125763.55741733511</v>
+      </c>
+      <c r="E71">
+        <v>282179.67125180899</v>
+      </c>
+      <c r="F71">
+        <v>0.87293045648394496</v>
+      </c>
+      <c r="G71">
+        <v>22626.697961956499</v>
+      </c>
+      <c r="H71">
+        <v>7102.5767129513297</v>
+      </c>
+      <c r="I71">
+        <v>9597.4591384874802</v>
+      </c>
+      <c r="J71">
+        <v>39326.733813395302</v>
+      </c>
+      <c r="K71">
+        <v>50843.184011688398</v>
+      </c>
+      <c r="L71">
+        <v>15303.798393134501</v>
+      </c>
+      <c r="M71">
+        <v>19297.530491231599</v>
+      </c>
+      <c r="N71">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O71">
+        <v>0</v>
+      </c>
+      <c r="P71">
         <f t="shared" si="13"/>
         <v>246323.22923633162</v>
       </c>
-      <c r="Q70">
+      <c r="Q71">
         <v>1127.27501714903</v>
       </c>
-      <c r="R70">
-        <v>0</v>
-      </c>
-      <c r="S70">
-        <v>0</v>
-      </c>
-      <c r="T70">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A71" s="1"/>
-    </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A72" t="s">
+      <c r="R71">
+        <v>0</v>
+      </c>
+      <c r="S71">
+        <v>0</v>
+      </c>
+      <c r="T71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A72" s="1"/>
+    </row>
+    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>20</v>
       </c>
-      <c r="B72" t="s">
-        <v>21</v>
-      </c>
-      <c r="C72">
-        <v>2</v>
-      </c>
-      <c r="D72">
-        <f>J72+K72+L72+M72+N72</f>
-        <v>116706.4157905087</v>
-      </c>
-      <c r="E72">
-        <v>282179.67125387199</v>
-      </c>
-      <c r="F72">
-        <v>0.840833383054163</v>
-      </c>
-      <c r="G72" s="4">
-        <v>20578.507216446698</v>
-      </c>
-      <c r="H72">
-        <v>7102.57515066207</v>
-      </c>
-      <c r="I72">
-        <v>2588.5052959285099</v>
-      </c>
-      <c r="J72">
-        <v>30269.587663037299</v>
-      </c>
-      <c r="K72">
-        <v>50843.185173268597</v>
-      </c>
-      <c r="L72">
-        <v>15303.8015139941</v>
-      </c>
-      <c r="M72">
-        <v>19297.530732323401</v>
-      </c>
-      <c r="N72">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O72">
-        <v>0</v>
-      </c>
-      <c r="P72">
-        <f t="shared" ref="P72:P73" si="14">D72+$P$1</f>
-        <v>237266.08760950522</v>
-      </c>
-      <c r="Q72">
-        <v>1127.2750356983099</v>
-      </c>
-      <c r="R72">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A73" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" t="s">
         <v>21</v>
       </c>
       <c r="C73">
@@ -4159,119 +4208,119 @@
       </c>
       <c r="D73">
         <f>J73+K73+L73+M73+N73</f>
+        <v>116706.4157905087</v>
+      </c>
+      <c r="E73">
+        <v>282179.67125387199</v>
+      </c>
+      <c r="F73">
+        <v>0.840833383054163</v>
+      </c>
+      <c r="G73" s="4">
+        <v>20578.507216446698</v>
+      </c>
+      <c r="H73">
+        <v>7102.57515066207</v>
+      </c>
+      <c r="I73">
+        <v>2588.5052959285099</v>
+      </c>
+      <c r="J73">
+        <v>30269.587663037299</v>
+      </c>
+      <c r="K73">
+        <v>50843.185173268597</v>
+      </c>
+      <c r="L73">
+        <v>15303.8015139941</v>
+      </c>
+      <c r="M73">
+        <v>19297.530732323401</v>
+      </c>
+      <c r="N73">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O73">
+        <v>0</v>
+      </c>
+      <c r="P73">
+        <f t="shared" ref="P73:P74" si="14">D73+$P$1</f>
+        <v>237266.08760950522</v>
+      </c>
+      <c r="Q73">
+        <v>1127.2750356983099</v>
+      </c>
+      <c r="R73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A74" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C74">
+        <v>2</v>
+      </c>
+      <c r="D74">
+        <f>J74+K74+L74+M74+N74</f>
         <v>121633.35860365373</v>
       </c>
-      <c r="E73">
+      <c r="E74">
         <v>282179.67123287602</v>
       </c>
-      <c r="F73">
+      <c r="F74">
         <v>0.85824890324911396</v>
       </c>
-      <c r="G73" s="4">
+      <c r="G74" s="4">
         <v>20824.7129679639</v>
       </c>
-      <c r="H73">
+      <c r="H74">
         <v>7456.39074483072</v>
       </c>
-      <c r="I73">
+      <c r="I74">
         <v>5114.4587365303096</v>
       </c>
-      <c r="J73">
+      <c r="J74">
         <v>33395.562449324898</v>
       </c>
-      <c r="K73">
+      <c r="K74">
         <v>51302.320205525801</v>
       </c>
-      <c r="L73">
+      <c r="L74">
         <v>16537.7269222135</v>
       </c>
-      <c r="M73">
+      <c r="M74">
         <v>19392.801250865799</v>
       </c>
-      <c r="N73">
+      <c r="N74">
         <v>1004.9477757237401</v>
       </c>
-      <c r="O73">
-        <v>0</v>
-      </c>
-      <c r="P73">
+      <c r="O74">
+        <v>0</v>
+      </c>
+      <c r="P74">
         <f t="shared" si="14"/>
         <v>242193.03042265025</v>
       </c>
-      <c r="Q73">
+      <c r="Q74">
         <v>1183.4303612998101</v>
       </c>
-      <c r="R73">
+      <c r="R74">
         <v>15931.1957490451</v>
       </c>
-      <c r="S73">
+      <c r="S74">
         <v>346.33034237054602</v>
       </c>
-      <c r="T73">
+      <c r="T74">
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A75" t="s">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
         <v>20</v>
-      </c>
-      <c r="B75" t="s">
-        <v>21</v>
-      </c>
-      <c r="C75">
-        <v>4</v>
-      </c>
-      <c r="D75">
-        <f>J75+K75+L75+M75+N75</f>
-        <v>116706.4157905051</v>
-      </c>
-      <c r="E75">
-        <v>282179.671253876</v>
-      </c>
-      <c r="F75">
-        <v>0.84083338305413902</v>
-      </c>
-      <c r="G75" s="4">
-        <v>20578.5072164468</v>
-      </c>
-      <c r="H75">
-        <v>7102.5751506616798</v>
-      </c>
-      <c r="I75">
-        <v>2588.50529592865</v>
-      </c>
-      <c r="J75">
-        <v>30269.587663037099</v>
-      </c>
-      <c r="K75">
-        <v>50843.185173268197</v>
-      </c>
-      <c r="L75">
-        <v>15303.8015139912</v>
-      </c>
-      <c r="M75">
-        <v>19297.530732323299</v>
-      </c>
-      <c r="N75">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O75">
-        <v>0</v>
-      </c>
-      <c r="P75">
-        <f t="shared" ref="P75:P77" si="15">D75+$P$1</f>
-        <v>237266.08760950161</v>
-      </c>
-      <c r="Q75">
-        <v>1127.2750356983499</v>
-      </c>
-      <c r="R75">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A76" t="s">
-        <v>22</v>
       </c>
       <c r="B76" t="s">
         <v>21</v>
@@ -4281,834 +4330,892 @@
       </c>
       <c r="D76">
         <f>J76+K76+L76+M76+N76</f>
+        <v>116706.4157905051</v>
+      </c>
+      <c r="E76">
+        <v>282179.671253876</v>
+      </c>
+      <c r="F76">
+        <v>0.84083338305413902</v>
+      </c>
+      <c r="G76" s="4">
+        <v>20578.5072164468</v>
+      </c>
+      <c r="H76">
+        <v>7102.5751506616798</v>
+      </c>
+      <c r="I76">
+        <v>2588.50529592865</v>
+      </c>
+      <c r="J76">
+        <v>30269.587663037099</v>
+      </c>
+      <c r="K76">
+        <v>50843.185173268197</v>
+      </c>
+      <c r="L76">
+        <v>15303.8015139912</v>
+      </c>
+      <c r="M76">
+        <v>19297.530732323299</v>
+      </c>
+      <c r="N76">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O76">
+        <v>0</v>
+      </c>
+      <c r="P76">
+        <f t="shared" ref="P76:P78" si="15">D76+$P$1</f>
+        <v>237266.08760950161</v>
+      </c>
+      <c r="Q76">
+        <v>1127.2750356983499</v>
+      </c>
+      <c r="R76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>22</v>
+      </c>
+      <c r="B77" t="s">
+        <v>21</v>
+      </c>
+      <c r="C77">
+        <v>4</v>
+      </c>
+      <c r="D77">
+        <f>J77+K77+L77+M77+N77</f>
         <v>121744.79706913032</v>
       </c>
-      <c r="E76">
+      <c r="E77">
         <v>282179.88376308198</v>
       </c>
-      <c r="F76">
+      <c r="F77">
         <v>0.85713546401894802</v>
       </c>
-      <c r="G76">
+      <c r="G77">
         <v>21291.5607898614</v>
       </c>
-      <c r="H76">
+      <c r="H77">
         <v>7432.3603175362596</v>
       </c>
-      <c r="I76">
+      <c r="I77">
         <v>5035.2758648834497</v>
       </c>
-      <c r="J76">
+      <c r="J77">
         <v>33759.196972281097</v>
       </c>
-      <c r="K76">
+      <c r="K77">
         <v>51128.3645002267</v>
       </c>
-      <c r="L76">
+      <c r="L77">
         <v>16070.129576240101</v>
       </c>
-      <c r="M76">
+      <c r="M77">
         <v>19356.7120304526</v>
       </c>
-      <c r="N76">
+      <c r="N77">
         <v>1430.39398992981</v>
       </c>
-      <c r="O76">
-        <v>0</v>
-      </c>
-      <c r="P76">
+      <c r="O77">
+        <v>0</v>
+      </c>
+      <c r="P77">
         <f t="shared" si="15"/>
         <v>242304.46888812684</v>
       </c>
-      <c r="Q76">
+      <c r="Q77">
         <v>1179.61640190856</v>
       </c>
-      <c r="R76">
+      <c r="R77">
         <v>13411.4010346792</v>
       </c>
-      <c r="S76">
+      <c r="S77">
         <v>478.97860838140201</v>
       </c>
-      <c r="T76">
+      <c r="T77">
         <v>0.22564405635506199</v>
       </c>
-      <c r="U76">
+      <c r="U77">
         <v>10550.3210016294</v>
       </c>
-      <c r="V76">
+      <c r="V77">
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="D77">
-        <f>D76-D70</f>
+    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="D78">
+        <f>D77-D71</f>
         <v>-4018.7603482047853</v>
       </c>
-      <c r="E77">
-        <f t="shared" ref="E77:N77" si="16">E76-E70</f>
+      <c r="E78">
+        <f t="shared" ref="E78:N78" si="16">E77-E71</f>
         <v>0.21251127298455685</v>
       </c>
-      <c r="F77">
+      <c r="F78">
         <f t="shared" si="16"/>
         <v>-1.5794992464996938E-2</v>
       </c>
-      <c r="G77">
+      <c r="G78">
         <f t="shared" si="16"/>
         <v>-1335.1371720950992</v>
       </c>
-      <c r="H77">
+      <c r="H78">
         <f t="shared" si="16"/>
         <v>329.78360458492989</v>
       </c>
-      <c r="I77">
+      <c r="I78">
         <f t="shared" si="16"/>
         <v>-4562.1832736040305</v>
       </c>
-      <c r="J77">
+      <c r="J78">
         <f t="shared" si="16"/>
         <v>-5567.5368411142044</v>
       </c>
-      <c r="K77">
+      <c r="K78">
         <f t="shared" si="16"/>
         <v>285.1804885383026</v>
       </c>
-      <c r="L77">
+      <c r="L78">
         <f t="shared" si="16"/>
         <v>766.33118310559985</v>
       </c>
-      <c r="M77">
+      <c r="M78">
         <f t="shared" si="16"/>
         <v>59.181539221001003</v>
       </c>
-      <c r="N77">
+      <c r="N78">
         <f t="shared" si="16"/>
         <v>438.08328204450595</v>
       </c>
-      <c r="P77">
+      <c r="P78">
         <f t="shared" si="15"/>
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A78" s="1" t="s">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A79" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G78" s="4"/>
-    </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A79" t="s">
-        <v>22</v>
-      </c>
-      <c r="B79" t="s">
-        <v>21</v>
-      </c>
-      <c r="C79">
-        <v>4</v>
-      </c>
-      <c r="D79">
-        <f>J79+K79+L79+M79+N79</f>
-        <v>147118.48206815872</v>
-      </c>
-      <c r="E79">
-        <v>355610.364944759</v>
-      </c>
-      <c r="F79">
-        <v>0.75267772890587503</v>
-      </c>
-      <c r="G79">
-        <v>25765.651662743599</v>
-      </c>
-      <c r="H79">
-        <v>7150.9042815892099</v>
-      </c>
-      <c r="I79">
-        <v>5144.3184852884797</v>
-      </c>
-      <c r="J79">
-        <v>38060.874429621297</v>
-      </c>
-      <c r="K79">
-        <v>64168.339029134899</v>
-      </c>
-      <c r="L79">
-        <v>19539.954214541001</v>
-      </c>
-      <c r="M79">
-        <v>24338.851661831999</v>
-      </c>
-      <c r="N79">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O79">
-        <v>0</v>
-      </c>
-      <c r="P79">
-        <f t="shared" ref="P79" si="17">D79+$P$1</f>
-        <v>267678.15388715523</v>
-      </c>
-      <c r="Q79">
-        <v>1597.68911089628</v>
-      </c>
-      <c r="R79">
-        <v>13084.0423994256</v>
-      </c>
-      <c r="S79">
-        <v>467.28722855091399</v>
-      </c>
-      <c r="T79">
-        <v>-0.25904927491985202</v>
-      </c>
-    </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="G79" s="4"/>
+    </row>
+    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>22</v>
       </c>
       <c r="B80" t="s">
+        <v>21</v>
+      </c>
+      <c r="C80">
+        <v>4</v>
+      </c>
+      <c r="D80">
+        <f>J80+K80+L80+M80+N80</f>
+        <v>147118.48206815872</v>
+      </c>
+      <c r="E80">
+        <v>355610.364944759</v>
+      </c>
+      <c r="F80">
+        <v>0.75267772890587503</v>
+      </c>
+      <c r="G80">
+        <v>25765.651662743599</v>
+      </c>
+      <c r="H80">
+        <v>7150.9042815892099</v>
+      </c>
+      <c r="I80">
+        <v>5144.3184852884797</v>
+      </c>
+      <c r="J80">
+        <v>38060.874429621297</v>
+      </c>
+      <c r="K80">
+        <v>64168.339029134899</v>
+      </c>
+      <c r="L80">
+        <v>19539.954214541001</v>
+      </c>
+      <c r="M80">
+        <v>24338.851661831999</v>
+      </c>
+      <c r="N80">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O80">
+        <v>0</v>
+      </c>
+      <c r="P80">
+        <f t="shared" ref="P80" si="17">D80+$P$1</f>
+        <v>267678.15388715523</v>
+      </c>
+      <c r="Q80">
+        <v>1597.68911089628</v>
+      </c>
+      <c r="R80">
+        <v>13084.0423994256</v>
+      </c>
+      <c r="S80">
+        <v>467.28722855091399</v>
+      </c>
+      <c r="T80">
+        <v>-0.25904927491985202</v>
+      </c>
+    </row>
+    <row r="81" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>22</v>
+      </c>
+      <c r="B81" t="s">
         <v>35</v>
       </c>
-      <c r="C80" t="s">
+      <c r="C81" t="s">
         <v>35</v>
       </c>
-      <c r="D80" t="s">
+      <c r="D81" t="s">
         <v>36</v>
       </c>
-      <c r="E80" t="s">
+      <c r="E81" t="s">
         <v>36</v>
       </c>
-      <c r="F80" t="s">
+      <c r="F81" t="s">
         <v>36</v>
       </c>
-      <c r="G80" s="4">
+      <c r="G81" s="4">
         <v>28838</v>
       </c>
-      <c r="H80">
+      <c r="H81">
         <v>7567.5</v>
       </c>
-      <c r="I80">
+      <c r="I81">
         <v>13764.1</v>
       </c>
-      <c r="J80">
+      <c r="J81">
         <v>50169.7</v>
       </c>
-      <c r="K80" t="s">
+      <c r="K81" t="s">
         <v>36</v>
       </c>
-      <c r="L80" t="s">
+      <c r="L81" t="s">
         <v>36</v>
       </c>
-      <c r="M80" t="s">
+      <c r="M81" t="s">
         <v>36</v>
       </c>
-      <c r="N80" t="s">
+      <c r="N81" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="82" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A82" s="1" t="s">
+    <row r="83" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A83" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G82" s="4"/>
-      <c r="P82" t="s">
+      <c r="G83" s="4"/>
+      <c r="P83" t="s">
         <v>15</v>
       </c>
-      <c r="Q82" t="s">
+      <c r="Q83" t="s">
         <v>16</v>
       </c>
-      <c r="R82" t="s">
+      <c r="R83" t="s">
         <v>17</v>
       </c>
-      <c r="S82" t="s">
+      <c r="S83" t="s">
         <v>18</v>
       </c>
-      <c r="T82" t="s">
+      <c r="T83" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="83" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B83" t="s">
+    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>0</v>
+      </c>
+      <c r="B84" t="s">
         <v>1</v>
       </c>
-      <c r="C83" t="s">
+      <c r="C84" t="s">
         <v>2</v>
       </c>
-      <c r="D83" t="s">
+      <c r="D84" t="s">
         <v>3</v>
       </c>
-      <c r="E83" t="s">
+      <c r="E84" t="s">
         <v>4</v>
       </c>
-      <c r="F83" t="s">
+      <c r="F84" t="s">
         <v>5</v>
       </c>
-      <c r="G83" s="4" t="s">
+      <c r="G84" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H83" t="s">
+      <c r="H84" t="s">
         <v>7</v>
       </c>
-      <c r="I83" t="s">
+      <c r="I84" t="s">
         <v>8</v>
       </c>
-      <c r="J83" t="s">
+      <c r="J84" t="s">
         <v>9</v>
       </c>
-      <c r="K83" t="s">
+      <c r="K84" t="s">
         <v>10</v>
       </c>
-      <c r="L83" t="s">
+      <c r="L84" t="s">
         <v>11</v>
       </c>
-      <c r="M83" t="s">
+      <c r="M84" t="s">
         <v>12</v>
       </c>
-      <c r="N83" t="s">
+      <c r="N84" t="s">
         <v>13</v>
       </c>
-      <c r="O83" t="s">
+      <c r="O84" t="s">
         <v>14</v>
       </c>
-      <c r="P83">
+      <c r="P84">
         <v>63734.6679</v>
       </c>
-      <c r="Q83">
+      <c r="Q84">
         <v>1078.4492829999999</v>
       </c>
-      <c r="R83">
+      <c r="R84">
         <v>624.70352849999995</v>
       </c>
-      <c r="S83">
+      <c r="S84">
         <v>13.014656840000001</v>
       </c>
-      <c r="T83">
+      <c r="T84">
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A84" s="2" t="s">
+    <row r="85" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A85" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B85" t="s">
         <v>21</v>
       </c>
-      <c r="C84">
+      <c r="C85">
         <v>4</v>
       </c>
-      <c r="D84">
+      <c r="D85">
         <v>29525.427309999999</v>
       </c>
-      <c r="E84">
+      <c r="E85">
         <v>80391.755990000005</v>
       </c>
-      <c r="F84">
+      <c r="F85">
         <v>0.79280104200000001</v>
       </c>
-      <c r="G84" s="4">
+      <c r="G85" s="4">
         <v>5050.6365619999997</v>
       </c>
-      <c r="H84">
+      <c r="H85">
         <v>4678.3390820000004</v>
       </c>
-      <c r="I84">
+      <c r="I85">
         <v>2508.6600360000002</v>
       </c>
-      <c r="J84">
+      <c r="J85">
         <v>12237.635679999999</v>
       </c>
-      <c r="K84">
+      <c r="K85">
         <v>13920</v>
       </c>
-      <c r="L84">
+      <c r="L85">
         <v>2841.544922</v>
       </c>
-      <c r="M84">
+      <c r="M85">
         <v>5380.5444360000001</v>
       </c>
-      <c r="N84">
+      <c r="N85">
         <v>279.27307350000001</v>
       </c>
-      <c r="O84">
-        <v>0</v>
-      </c>
-      <c r="P84">
+      <c r="O85">
+        <v>0</v>
+      </c>
+      <c r="P85">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q84">
+      <c r="Q85">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R84">
+      <c r="R85">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S84">
+      <c r="S85">
         <v>452.7322633</v>
       </c>
-      <c r="T84">
+      <c r="T85">
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A85" s="7" t="s">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A86" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A87" t="s">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
         <v>32</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B88" t="s">
         <v>33</v>
       </c>
-      <c r="C87" t="s">
+      <c r="C88" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A88">
-        <v>20</v>
-      </c>
-      <c r="B88">
-        <v>60</v>
-      </c>
-      <c r="C88">
-        <v>2</v>
-      </c>
-      <c r="D88">
-        <f t="shared" ref="D88:D94" si="18">J88+K88+L88+M88+N88</f>
-        <v>120712.69088313227</v>
-      </c>
-      <c r="E88">
-        <v>282179.67123285501</v>
-      </c>
-      <c r="F88">
-        <v>0.854946898908852</v>
-      </c>
-      <c r="G88">
-        <v>18681.222424938602</v>
-      </c>
-      <c r="H88">
-        <v>5354.6114985546601</v>
-      </c>
-      <c r="I88">
-        <v>8156.08309050551</v>
-      </c>
-      <c r="J88">
-        <v>32191.917013998798</v>
-      </c>
-      <c r="K88">
-        <v>51372.124296964801</v>
-      </c>
-      <c r="L88">
-        <v>16725.325417965501</v>
-      </c>
-      <c r="M88">
-        <v>19407.285599838699</v>
-      </c>
-      <c r="N88">
-        <v>1016.03855436447</v>
-      </c>
-      <c r="O88">
-        <v>0</v>
-      </c>
-      <c r="P88">
-        <f t="shared" ref="P88:P94" si="19">D88+$P$1</f>
-        <v>241272.36270212877</v>
-      </c>
-      <c r="Q88">
-        <v>1192.7637589594799</v>
-      </c>
-      <c r="R88">
-        <v>19736.206339365101</v>
-      </c>
-      <c r="S88">
-        <v>481.37088632597801</v>
-      </c>
-      <c r="T88" s="6">
-        <v>0.12591688076390301</v>
-      </c>
-    </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>20</v>
       </c>
       <c r="B89">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C89">
         <v>2</v>
       </c>
       <c r="D89">
+        <f t="shared" ref="D89:D95" si="18">J89+K89+L89+M89+N89</f>
+        <v>120712.69088313227</v>
+      </c>
+      <c r="E89">
+        <v>282179.67123285501</v>
+      </c>
+      <c r="F89">
+        <v>0.854946898908852</v>
+      </c>
+      <c r="G89">
+        <v>18681.222424938602</v>
+      </c>
+      <c r="H89">
+        <v>5354.6114985546601</v>
+      </c>
+      <c r="I89">
+        <v>8156.08309050551</v>
+      </c>
+      <c r="J89">
+        <v>32191.917013998798</v>
+      </c>
+      <c r="K89">
+        <v>51372.124296964801</v>
+      </c>
+      <c r="L89">
+        <v>16725.325417965501</v>
+      </c>
+      <c r="M89">
+        <v>19407.285599838699</v>
+      </c>
+      <c r="N89">
+        <v>1016.03855436447</v>
+      </c>
+      <c r="O89">
+        <v>0</v>
+      </c>
+      <c r="P89">
+        <f t="shared" ref="P89:P95" si="19">D89+$P$1</f>
+        <v>241272.36270212877</v>
+      </c>
+      <c r="Q89">
+        <v>1192.7637589594799</v>
+      </c>
+      <c r="R89">
+        <v>19736.206339365101</v>
+      </c>
+      <c r="S89">
+        <v>481.37088632597801</v>
+      </c>
+      <c r="T89" s="6">
+        <v>0.12591688076390301</v>
+      </c>
+    </row>
+    <row r="90" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A90">
+        <v>20</v>
+      </c>
+      <c r="B90">
+        <v>50</v>
+      </c>
+      <c r="C90">
+        <v>2</v>
+      </c>
+      <c r="D90">
         <f t="shared" si="18"/>
         <v>119392.42354269064</v>
       </c>
-      <c r="E89">
+      <c r="E90">
         <v>282254.81855225202</v>
       </c>
-      <c r="F89">
+      <c r="F90">
         <v>0.85006146065890897</v>
       </c>
-      <c r="G89">
+      <c r="G90">
         <v>19407.840072768398</v>
       </c>
-      <c r="H89">
+      <c r="H90">
         <v>5891.8301217549197</v>
       </c>
-      <c r="I89">
+      <c r="I90">
         <v>6659.4942697455399</v>
       </c>
-      <c r="J89">
+      <c r="J90">
         <v>31959.164464268899</v>
       </c>
-      <c r="K89">
+      <c r="K90">
         <v>51102.045942938203</v>
       </c>
-      <c r="L89">
+      <c r="L90">
         <v>15967.176494174801</v>
       </c>
-      <c r="M89">
+      <c r="M90">
         <v>19353.573908279199</v>
       </c>
-      <c r="N89">
+      <c r="N90">
         <v>1010.46273302954</v>
       </c>
-      <c r="O89">
-        <v>0</v>
-      </c>
-      <c r="P89">
+      <c r="O90">
+        <v>0</v>
+      </c>
+      <c r="P90">
         <f t="shared" si="19"/>
         <v>239952.09536168716</v>
       </c>
-      <c r="Q89">
+      <c r="Q90">
         <v>1312.43161993582</v>
       </c>
-      <c r="R89">
+      <c r="R90">
         <v>18377.616631847999</v>
       </c>
-      <c r="S89">
+      <c r="S90">
         <v>459.4404157962</v>
       </c>
-      <c r="T89" s="6">
+      <c r="T90" s="6">
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A90">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A91">
         <v>20</v>
       </c>
-      <c r="B90">
+      <c r="B91">
         <v>40</v>
       </c>
-      <c r="C90">
+      <c r="C91">
         <v>2</v>
       </c>
-      <c r="D90">
+      <c r="D91">
         <f t="shared" si="18"/>
         <v>117777.02945340994</v>
       </c>
-      <c r="E90">
+      <c r="E91">
         <v>282179.67123287299</v>
       </c>
-      <c r="F90">
+      <c r="F91">
         <v>0.84456314023622803</v>
       </c>
-      <c r="G90">
+      <c r="G91">
         <v>19298.245593088301</v>
       </c>
-      <c r="H90">
+      <c r="H91">
         <v>5682.0016560700296</v>
       </c>
-      <c r="I90">
+      <c r="I91">
         <v>5350.3346939491703</v>
       </c>
-      <c r="J90">
+      <c r="J91">
         <v>30330.5819431075</v>
       </c>
-      <c r="K90">
+      <c r="K91">
         <v>51097.733915068202</v>
       </c>
-      <c r="L90">
+      <c r="L91">
         <v>15987.901266609</v>
       </c>
-      <c r="M90">
+      <c r="M91">
         <v>19350.349595595701</v>
       </c>
-      <c r="N90">
+      <c r="N91">
         <v>1010.46273302954</v>
       </c>
-      <c r="O90">
-        <v>0</v>
-      </c>
-      <c r="P90">
+      <c r="O91">
+        <v>0</v>
+      </c>
+      <c r="P91">
         <f t="shared" si="19"/>
         <v>238336.70127240644</v>
       </c>
-      <c r="Q90">
+      <c r="Q91">
         <v>1265.6913868611</v>
       </c>
-      <c r="R90">
+      <c r="R91">
         <v>17746.163883660702</v>
       </c>
-      <c r="S90">
+      <c r="S91">
         <v>507.03325381887902</v>
       </c>
-      <c r="T90" s="6">
+      <c r="T91" s="6">
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A91">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A92">
         <v>20</v>
       </c>
-      <c r="B91">
+      <c r="B92">
         <v>30</v>
       </c>
-      <c r="C91">
+      <c r="C92">
         <v>2</v>
       </c>
-      <c r="D91">
+      <c r="D92">
         <f t="shared" si="18"/>
         <v>116625.1695160947</v>
       </c>
-      <c r="E91">
+      <c r="E92">
         <v>282182.50548365602</v>
       </c>
-      <c r="F91">
+      <c r="F92">
         <v>0.84045954058697003</v>
       </c>
-      <c r="G91">
+      <c r="G92">
         <v>19302.752565837702</v>
       </c>
-      <c r="H91">
+      <c r="H92">
         <v>6226.5181629292701</v>
       </c>
-      <c r="I91">
+      <c r="I92">
         <v>3974.5318253822402</v>
       </c>
-      <c r="J91">
+      <c r="J92">
         <v>29503.802554149199</v>
       </c>
-      <c r="K91">
+      <c r="K92">
         <v>51013.610661725899</v>
       </c>
-      <c r="L91">
+      <c r="L92">
         <v>15760.601295416</v>
       </c>
-      <c r="M91">
+      <c r="M92">
         <v>19332.981882301501</v>
       </c>
-      <c r="N91">
+      <c r="N92">
         <v>1014.17312250211</v>
       </c>
-      <c r="O91">
-        <v>0</v>
-      </c>
-      <c r="P91">
+      <c r="O92">
+        <v>0</v>
+      </c>
+      <c r="P92">
         <f t="shared" si="19"/>
         <v>237184.84133509122</v>
       </c>
-      <c r="Q91">
+      <c r="Q92">
         <v>1386.9848841974899</v>
       </c>
-      <c r="R91">
+      <c r="R92">
         <v>18436.445202769701</v>
       </c>
-      <c r="S91">
+      <c r="S92">
         <v>209.50505912238299</v>
       </c>
-      <c r="T91" s="6">
+      <c r="T92" s="6">
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A92" s="3">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A93" s="3">
         <v>20</v>
       </c>
-      <c r="B92" s="3">
+      <c r="B93" s="3">
         <v>20</v>
       </c>
-      <c r="C92" s="3">
+      <c r="C93" s="3">
         <v>2</v>
       </c>
-      <c r="D92">
+      <c r="D93">
         <f t="shared" si="18"/>
         <v>115198.459983006</v>
       </c>
-      <c r="E92">
+      <c r="E93">
         <v>282179.67123297497</v>
       </c>
-      <c r="F92">
+      <c r="F93">
         <v>0.83541194997266699</v>
       </c>
-      <c r="G92">
+      <c r="G93">
         <v>19351.2255529412</v>
       </c>
-      <c r="H92">
+      <c r="H93">
         <v>6002.0469674603501</v>
       </c>
-      <c r="I92">
+      <c r="I93">
         <v>2645.4376652921501</v>
       </c>
-      <c r="J92">
+      <c r="J93">
         <v>27998.710185693701</v>
       </c>
-      <c r="K92">
+      <c r="K93">
         <v>51033.4442867088</v>
       </c>
-      <c r="L92">
+      <c r="L93">
         <v>15815.1228903871</v>
       </c>
-      <c r="M92">
+      <c r="M93">
         <v>19337.009497714302</v>
       </c>
-      <c r="N92">
+      <c r="N93">
         <v>1014.17312250211</v>
       </c>
-      <c r="O92">
-        <v>0</v>
-      </c>
-      <c r="P92">
+      <c r="O93">
+        <v>0</v>
+      </c>
+      <c r="P93">
         <f t="shared" si="19"/>
         <v>235758.13180200252</v>
       </c>
-      <c r="Q92">
+      <c r="Q93">
         <v>1336.98290493166</v>
       </c>
-      <c r="R92">
+      <c r="R93">
         <v>18577.307877855899</v>
       </c>
-      <c r="S92">
+      <c r="S93">
         <v>432.030415764091</v>
       </c>
-      <c r="T92" s="6">
+      <c r="T93" s="6">
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A93">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A94">
         <v>20</v>
       </c>
-      <c r="B93">
+      <c r="B94">
         <v>15</v>
       </c>
-      <c r="C93">
+      <c r="C94">
         <v>2</v>
       </c>
-      <c r="D93">
+      <c r="D94">
         <f t="shared" si="18"/>
         <v>114451.25872361983</v>
       </c>
-      <c r="E93">
+      <c r="E94">
         <v>282179.67123267101</v>
       </c>
-      <c r="F93">
+      <c r="F94">
         <v>0.83277713625127903</v>
       </c>
-      <c r="G93">
+      <c r="G94">
         <v>19390.977969205</v>
       </c>
-      <c r="H93">
+      <c r="H94">
         <v>5599.5405456203798</v>
       </c>
-      <c r="I93">
+      <c r="I94">
         <v>2128.1287863747102</v>
       </c>
-      <c r="J93">
+      <c r="J94">
         <v>27118.647301200101</v>
       </c>
-      <c r="K93">
+      <c r="K94">
         <v>51068.507704320902</v>
       </c>
-      <c r="L93">
+      <c r="L94">
         <v>15909.3558282099</v>
       </c>
-      <c r="M93">
+      <c r="M94">
         <v>19344.285156859401</v>
       </c>
-      <c r="N93">
+      <c r="N94">
         <v>1010.46273302954</v>
       </c>
-      <c r="O93">
-        <v>0</v>
-      </c>
-      <c r="P93">
+      <c r="O94">
+        <v>0</v>
+      </c>
+      <c r="P94">
         <f t="shared" si="19"/>
         <v>235010.93054261635</v>
       </c>
-      <c r="Q93">
+      <c r="Q94">
         <v>1247.3228025527501</v>
       </c>
-      <c r="R93">
+      <c r="R94">
         <v>16417.502561416801</v>
       </c>
-      <c r="S93">
+      <c r="S94">
         <v>469.07150175476602</v>
       </c>
-      <c r="T93" s="6">
+      <c r="T94" s="6">
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A94">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A95">
         <v>20</v>
       </c>
-      <c r="B94">
+      <c r="B95">
         <v>12</v>
       </c>
-      <c r="C94">
+      <c r="C95">
         <v>2</v>
       </c>
-      <c r="D94">
+      <c r="D95">
         <f t="shared" si="18"/>
         <v>114787.7594081375</v>
       </c>
-      <c r="E94">
+      <c r="E95">
         <v>282179.67123287602</v>
       </c>
-      <c r="F94">
+      <c r="F95">
         <v>0.83403396920434802</v>
       </c>
-      <c r="G94">
+      <c r="G95">
         <v>20436.472361711199</v>
       </c>
-      <c r="H94">
+      <c r="H95">
         <v>4946.5396722567002</v>
       </c>
-      <c r="I94">
+      <c r="I95">
         <v>2967.9237851293901</v>
       </c>
-      <c r="J94">
+      <c r="J95">
         <v>28350.9358190973</v>
       </c>
-      <c r="K94">
+      <c r="K95">
         <v>50843.184005923598</v>
       </c>
-      <c r="L94">
+      <c r="L95">
         <v>15303.798385783</v>
       </c>
-      <c r="M94">
+      <c r="M95">
         <v>19297.530489448302</v>
       </c>
-      <c r="N94">
+      <c r="N95">
         <v>992.31070788530405</v>
       </c>
-      <c r="O94">
-        <v>0</v>
-      </c>
-      <c r="P94">
+      <c r="O95">
+        <v>0</v>
+      </c>
+      <c r="P95">
         <f t="shared" si="19"/>
         <v>235347.43122713402</v>
       </c>
-      <c r="Q94">
+      <c r="Q95">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R94">
+      <c r="R95">
         <v>13.380488321454299</v>
       </c>
-      <c r="S94">
+      <c r="S95">
         <v>2.67609766429086</v>
       </c>
-      <c r="T94" s="6">
+      <c r="T95" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>

</xml_diff>

<commit_message>
testing 5 shutdowns with the TOU 3 summer week
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A5B651-2BB1-42D9-89F9-4DDB7DF3E311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8070B048-2D18-40B1-BE2F-8718C4D8BA85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -51,6 +51,7 @@
     <author>tc={B12FED98-6BE9-4BE2-A887-4CF314FA442B}</author>
     <author>tc={7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}</author>
     <author>tc={B7EDEAAD-67C9-4693-A0FC-570282E02182}</author>
+    <author>tc={0EBBD83F-AB64-4248-87E6-B99F88EE5F88}</author>
     <author>tc={FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}</author>
     <author>tc={4644E393-F522-4E79-88BA-041770B595A7}</author>
     <author>tc={9FF6B967-6104-43AC-8EED-15C48C9ACCA9}</author>
@@ -191,7 +192,15 @@
     I’d like to see numbers for only one shutdown</t>
       </text>
     </comment>
-    <comment ref="A67" authorId="16" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+    <comment ref="A61" authorId="16" shapeId="0" xr:uid="{0EBBD83F-AB64-4248-87E6-B99F88EE5F88}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Only one plant shutdown allowed</t>
+      </text>
+    </comment>
+    <comment ref="A68" authorId="17" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -200,7 +209,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="A74" authorId="17" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
+    <comment ref="A75" authorId="18" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -208,7 +217,7 @@
     Pretty sure this solution is wrong, but I don’t think I need this case for the paper</t>
       </text>
     </comment>
-    <comment ref="A80" authorId="18" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A81" authorId="19" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -216,7 +225,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T92" authorId="19" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T93" authorId="20" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -229,7 +238,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="44">
   <si>
     <t>Season</t>
   </si>
@@ -1325,17 +1334,20 @@
   <threadedComment ref="A60" dT="2026-07-22T19:37:51.21" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{DB15DF8F-6887-4CDD-9A38-5D318EAEEFFF}" parentId="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
     <text>I’d like to see numbers for only one shutdown</text>
   </threadedComment>
-  <threadedComment ref="A67" dT="2026-07-22T16:56:30.58" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+  <threadedComment ref="A61" dT="2026-07-22T21:09:49.14" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{0EBBD83F-AB64-4248-87E6-B99F88EE5F88}">
+    <text>Only one plant shutdown allowed</text>
+  </threadedComment>
+  <threadedComment ref="A68" dT="2026-07-22T16:56:30.58" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
     <text xml:space="preserve">Why is this so different from the other DR solution? I would assume they would be the same…
 </text>
   </threadedComment>
-  <threadedComment ref="A74" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
+  <threadedComment ref="A75" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
     <text>Pretty sure this solution is wrong, but I don’t think I need this case for the paper</text>
   </threadedComment>
-  <threadedComment ref="A80" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+  <threadedComment ref="A81" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
     <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
   </threadedComment>
-  <threadedComment ref="T92" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="T93" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1343,7 +1355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:V95"/>
+  <dimension ref="A1:V96"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.6328125" customWidth="1"/>
@@ -3733,405 +3745,409 @@
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" s="3"/>
-      <c r="B61" s="3"/>
+      <c r="A61" t="s">
+        <v>22</v>
+      </c>
+      <c r="B61" t="s">
+        <v>21</v>
+      </c>
+      <c r="C61">
+        <v>4</v>
+      </c>
       <c r="D61">
-        <f>D60-D59</f>
-        <v>-3470.0549869755487</v>
+        <v>106606.33139463799</v>
       </c>
       <c r="E61">
-        <f t="shared" ref="E61:V61" si="11">E60-E59</f>
-        <v>0</v>
+        <v>282179.67123277002</v>
       </c>
       <c r="F61">
+        <v>0.80855687769694595</v>
+      </c>
+      <c r="G61">
+        <v>19403.054157778199</v>
+      </c>
+      <c r="H61">
+        <v>5553.2925107720503</v>
+      </c>
+      <c r="I61">
+        <v>4877.88612389215</v>
+      </c>
+      <c r="J61">
+        <v>29834.232792442399</v>
+      </c>
+      <c r="K61">
+        <v>51173.670096007401</v>
+      </c>
+      <c r="L61">
+        <v>17123.646419717399</v>
+      </c>
+      <c r="M61">
+        <v>19494.782086470699</v>
+      </c>
+      <c r="N61">
+        <v>1435.62713867346</v>
+      </c>
+      <c r="O61">
+        <v>11020</v>
+      </c>
+      <c r="P61">
+        <v>228158.313921519</v>
+      </c>
+      <c r="Q61">
+        <v>1240.7430631340701</v>
+      </c>
+      <c r="R61">
+        <v>17914.482434871101</v>
+      </c>
+      <c r="S61">
+        <v>398.09960966380203</v>
+      </c>
+      <c r="T61">
+        <v>0.67297738075987301</v>
+      </c>
+      <c r="U61">
+        <v>13163.232180323101</v>
+      </c>
+      <c r="V61">
+        <v>107.018147807505</v>
+      </c>
+    </row>
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A62" s="3"/>
+      <c r="B62" s="3"/>
+      <c r="D62">
+        <f>D61-D60</f>
+        <v>513.41110323798785</v>
+      </c>
+      <c r="E62">
+        <f t="shared" ref="E62:V62" si="11">E61-E60</f>
+        <v>-1.0599615052342415E-7</v>
+      </c>
+      <c r="F62">
         <f t="shared" si="11"/>
-        <v>-1.0153485538960005E-2</v>
-      </c>
-      <c r="G61">
+        <v>1.8194475210779881E-3</v>
+      </c>
+      <c r="G62">
         <f t="shared" si="11"/>
-        <v>-667.82878678320048</v>
-      </c>
-      <c r="H61">
+        <v>-214.21539764659974</v>
+      </c>
+      <c r="H62">
         <f t="shared" si="11"/>
-        <v>-374.88135105099991</v>
-      </c>
-      <c r="I61">
+        <v>-624.4983606493397</v>
+      </c>
+      <c r="I62">
         <f t="shared" si="11"/>
-        <v>-6068.9240419192656</v>
-      </c>
-      <c r="J61">
+        <v>4877.8861089948059</v>
+      </c>
+      <c r="J62">
         <f t="shared" si="11"/>
-        <v>-7111.6341797534005</v>
-      </c>
-      <c r="K61">
+        <v>4039.1723506987983</v>
+      </c>
+      <c r="K62">
         <f t="shared" si="11"/>
-        <v>146.76122373789985</v>
-      </c>
-      <c r="L61">
+        <v>183.72486634590314</v>
+      </c>
+      <c r="L62">
         <f t="shared" si="11"/>
-        <v>3977.7541241718009</v>
-      </c>
-      <c r="M61">
+        <v>-3232.9060902373021</v>
+      </c>
+      <c r="M62">
         <f t="shared" si="11"/>
-        <v>522.01162059239869</v>
-      </c>
-      <c r="N61">
+        <v>-476.58002357000078</v>
+      </c>
+      <c r="N62">
         <f t="shared" si="11"/>
-        <v>457.43017919829003</v>
-      </c>
-      <c r="O61">
+        <v>-26.750816248570118</v>
+      </c>
+      <c r="O62">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="P61">
+      <c r="P62">
         <f t="shared" si="11"/>
-        <v>-2477.7442790900823</v>
-      </c>
-      <c r="Q61">
+        <v>513.41110323701287</v>
+      </c>
+      <c r="Q62">
         <f t="shared" si="11"/>
-        <v>-83.757789339369992</v>
-      </c>
-      <c r="R61">
+        <v>-139.52840101139986</v>
+      </c>
+      <c r="R62">
         <f t="shared" si="11"/>
-        <v>7916.1452993303974</v>
-      </c>
-      <c r="S61">
+        <v>-16066.151948654198</v>
+      </c>
+      <c r="S62">
         <f t="shared" si="11"/>
-        <v>536.648868712938</v>
-      </c>
-      <c r="T61">
+        <v>-545.80690098968103</v>
+      </c>
+      <c r="T62">
         <f t="shared" si="11"/>
-        <v>-0.72698549006634905</v>
-      </c>
-      <c r="U61">
+        <v>0.30386414961436203</v>
+      </c>
+      <c r="U62">
         <f t="shared" si="11"/>
-        <v>36719.7300995962</v>
-      </c>
-      <c r="V61">
+        <v>-23556.497919273097</v>
+      </c>
+      <c r="V62">
         <f t="shared" si="11"/>
-        <v>278.17977348178903</v>
-      </c>
-    </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A62" s="1" t="s">
+        <v>-171.16162567428404</v>
+      </c>
+    </row>
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A63" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G62" s="4"/>
-    </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A63" s="3" t="s">
+      <c r="G63" s="4"/>
+    </row>
+    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A64" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B63" s="3" t="s">
+      <c r="B64" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C63" s="3">
-        <v>0</v>
-      </c>
-      <c r="G63" s="4"/>
-    </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
+      <c r="C64" s="3">
+        <v>0</v>
+      </c>
+      <c r="G64" s="4"/>
+    </row>
+    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>22</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B65" t="s">
         <v>23</v>
       </c>
-      <c r="C64">
-        <v>0</v>
-      </c>
-      <c r="D64">
-        <f>J64+K64+L64+M64+N64-O64</f>
+      <c r="C65">
+        <v>0</v>
+      </c>
+      <c r="D65">
+        <f>J65+K65+L65+M65+N65-O65</f>
         <v>125093.23428318274</v>
       </c>
-      <c r="E64">
+      <c r="E65">
         <v>282190.859999999</v>
       </c>
-      <c r="F64">
+      <c r="F65">
         <v>0.86904083066499505</v>
       </c>
-      <c r="G64">
+      <c r="G65">
         <v>24203.497764766002</v>
       </c>
-      <c r="H64">
+      <c r="H65">
         <v>4932.7238161263904</v>
       </c>
-      <c r="I64">
+      <c r="I65">
         <v>9098.5748223234004</v>
       </c>
-      <c r="J64">
+      <c r="J65">
         <v>38234.796403215798</v>
       </c>
-      <c r="K64">
+      <c r="K65">
         <v>50845.200000000099</v>
       </c>
-      <c r="L64">
+      <c r="L65">
         <v>15304.405199999899</v>
       </c>
-      <c r="M64">
+      <c r="M65">
         <v>19298.29566</v>
       </c>
-      <c r="N64">
+      <c r="N65">
         <v>1409.83742959549</v>
       </c>
-      <c r="O64">
+      <c r="O65">
         <v>-0.69959037146548997</v>
       </c>
-      <c r="P64">
-        <f>D64+$P$1</f>
+      <c r="P65">
+        <f>D65+$P$1</f>
         <v>245652.90610217926</v>
       </c>
-      <c r="Q64">
+      <c r="Q65">
         <v>1102.0926609763501</v>
       </c>
-      <c r="R64">
-        <v>0</v>
-      </c>
-      <c r="U64">
+      <c r="R65">
+        <v>0</v>
+      </c>
+      <c r="U65">
         <v>15.5670440273115</v>
       </c>
-      <c r="V64">
+      <c r="V65">
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A65" s="3"/>
-      <c r="B65" s="3"/>
-      <c r="C65" s="3"/>
-      <c r="G65" s="4"/>
-    </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="3" t="s">
+      <c r="A66" s="3"/>
+      <c r="B66" s="3"/>
+      <c r="C66" s="3"/>
+      <c r="G66" s="4"/>
+    </row>
+    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A67" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B66" s="3" t="s">
+      <c r="B67" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C66" s="3">
+      <c r="C67" s="3">
         <v>4</v>
       </c>
-      <c r="G66" s="4"/>
-    </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
+      <c r="G67" s="4"/>
+    </row>
+    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>22</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B68" t="s">
         <v>21</v>
       </c>
-      <c r="C67">
+      <c r="C68">
         <v>4</v>
       </c>
-      <c r="D67">
+      <c r="D68">
         <v>108832.74020782999</v>
       </c>
-      <c r="E67">
+      <c r="E68">
         <v>282179.67123306898</v>
       </c>
-      <c r="F67">
+      <c r="F68">
         <v>0.81644691741250097</v>
       </c>
-      <c r="G67">
+      <c r="G68">
         <v>19728.523245555101</v>
       </c>
-      <c r="H67">
+      <c r="H68">
         <v>6281.7321988746498</v>
       </c>
-      <c r="I67" s="8">
+      <c r="I68" s="8">
         <v>9.8877442286147301E-6</v>
       </c>
-      <c r="J67">
+      <c r="J68">
         <v>26010.255454317499</v>
       </c>
-      <c r="K67">
+      <c r="K68">
         <v>50944.9452054754</v>
       </c>
-      <c r="L67">
+      <c r="L68">
         <v>20235.614943009699</v>
       </c>
-      <c r="M67">
+      <c r="M68">
         <v>19962.024605027898</v>
       </c>
-      <c r="N67">
+      <c r="N68">
         <v>1462.3779549220301</v>
       </c>
-      <c r="O67">
+      <c r="O68">
         <v>8320.1</v>
       </c>
-      <c r="P67">
+      <c r="P68">
         <v>230384.72273471201</v>
       </c>
-      <c r="Q67">
+      <c r="Q68">
         <v>1403.49453592792</v>
       </c>
-      <c r="R67">
+      <c r="R68">
         <v>34518.506961381201</v>
       </c>
-      <c r="S67">
+      <c r="S68">
         <v>841.91480393612801</v>
       </c>
-      <c r="T67">
+      <c r="T68">
         <v>0.38784649209264499</v>
       </c>
-      <c r="U67">
+      <c r="U68">
         <v>38264.627438579002</v>
       </c>
-      <c r="V67">
+      <c r="V68">
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" s="5"/>
-      <c r="B68" s="5"/>
-      <c r="D68">
-        <f>D67-D64</f>
+    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A69" s="5"/>
+      <c r="B69" s="5"/>
+      <c r="D69">
+        <f>D68-D65</f>
         <v>-16260.494075352748</v>
       </c>
-      <c r="E68">
-        <f t="shared" ref="E68:V68" si="12">E67-E64</f>
+      <c r="E69">
+        <f t="shared" ref="E69:V69" si="12">E68-E65</f>
         <v>-11.188766930019483</v>
       </c>
-      <c r="F68">
+      <c r="F69">
         <f t="shared" si="12"/>
         <v>-5.2593913252494073E-2</v>
       </c>
-      <c r="G68">
+      <c r="G69">
         <f t="shared" si="12"/>
         <v>-4474.9745192109003</v>
       </c>
-      <c r="H68">
+      <c r="H69">
         <f t="shared" si="12"/>
         <v>1349.0083827482595</v>
       </c>
-      <c r="I68">
+      <c r="I69">
         <f t="shared" si="12"/>
         <v>-9098.574812435656</v>
       </c>
-      <c r="J68">
+      <c r="J69">
         <f t="shared" si="12"/>
         <v>-12224.540948898299</v>
       </c>
-      <c r="K68">
+      <c r="K69">
         <f t="shared" si="12"/>
         <v>99.745205475301191</v>
       </c>
-      <c r="L68">
+      <c r="L69">
         <f t="shared" si="12"/>
         <v>4931.2097430098001</v>
       </c>
-      <c r="M68">
+      <c r="M69">
         <f t="shared" si="12"/>
         <v>663.72894502789859</v>
       </c>
-      <c r="N68">
+      <c r="N69">
         <f t="shared" si="12"/>
         <v>52.540525326540092</v>
       </c>
-      <c r="O68">
+      <c r="O69">
         <f t="shared" si="12"/>
         <v>8320.7995903714655</v>
       </c>
-      <c r="P68">
+      <c r="P69">
         <f t="shared" si="12"/>
         <v>-15268.183367467253</v>
       </c>
-      <c r="Q68">
+      <c r="Q69">
         <f t="shared" si="12"/>
         <v>301.40187495156988</v>
       </c>
-      <c r="R68">
+      <c r="R69">
         <f t="shared" si="12"/>
         <v>34518.506961381201</v>
       </c>
-      <c r="S68">
+      <c r="S69">
         <f t="shared" si="12"/>
         <v>841.91480393612801</v>
       </c>
-      <c r="T68">
+      <c r="T69">
         <f t="shared" si="12"/>
         <v>0.38784649209264499</v>
       </c>
-      <c r="U68">
+      <c r="U69">
         <f t="shared" si="12"/>
         <v>38249.060394551692</v>
       </c>
-      <c r="V68">
+      <c r="V69">
         <f t="shared" si="12"/>
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="1" t="s">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A70" s="1" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C70">
-        <v>0</v>
-      </c>
-      <c r="D70">
-        <f>J70+K70+L70+M70+N70</f>
-        <v>116023.2890300647</v>
-      </c>
-      <c r="E70">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F70">
-        <v>0.83841249022441</v>
-      </c>
-      <c r="G70">
-        <v>20114.092712805999</v>
-      </c>
-      <c r="H70">
-        <v>6942.2846600808298</v>
-      </c>
-      <c r="I70">
-        <v>2530.0880681377598</v>
-      </c>
-      <c r="J70">
-        <v>29586.4654410246</v>
-      </c>
-      <c r="K70">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L70">
-        <v>15303.798385783</v>
-      </c>
-      <c r="M70">
-        <v>19297.5304894482</v>
-      </c>
-      <c r="N70">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O70">
-        <v>0</v>
-      </c>
-      <c r="P70">
-        <f t="shared" ref="P70:P71" si="13">D70+$P$1</f>
-        <v>236582.9608490612</v>
-      </c>
-      <c r="Q70">
-        <v>1101.8347602124099</v>
-      </c>
-      <c r="R70">
-        <v>0</v>
-      </c>
-      <c r="S70">
-        <v>0</v>
-      </c>
-      <c r="T70">
-        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A71" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>23</v>
@@ -4141,34 +4157,34 @@
       </c>
       <c r="D71">
         <f>J71+K71+L71+M71+N71</f>
-        <v>125763.55741733511</v>
+        <v>116023.2890300647</v>
       </c>
       <c r="E71">
-        <v>282179.67125180899</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F71">
-        <v>0.87293045648394496</v>
+        <v>0.83841249022441</v>
       </c>
       <c r="G71">
-        <v>22626.697961956499</v>
+        <v>20114.092712805999</v>
       </c>
       <c r="H71">
-        <v>7102.5767129513297</v>
+        <v>6942.2846600808298</v>
       </c>
       <c r="I71">
-        <v>9597.4591384874802</v>
+        <v>2530.0880681377598</v>
       </c>
       <c r="J71">
-        <v>39326.733813395302</v>
+        <v>29586.4654410246</v>
       </c>
       <c r="K71">
-        <v>50843.184011688398</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L71">
-        <v>15303.798393134501</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M71">
-        <v>19297.530491231599</v>
+        <v>19297.5304894482</v>
       </c>
       <c r="N71">
         <v>992.31070788530405</v>
@@ -4177,88 +4193,94 @@
         <v>0</v>
       </c>
       <c r="P71">
+        <f t="shared" ref="P71:P72" si="13">D71+$P$1</f>
+        <v>236582.9608490612</v>
+      </c>
+      <c r="Q71">
+        <v>1101.8347602124099</v>
+      </c>
+      <c r="R71">
+        <v>0</v>
+      </c>
+      <c r="S71">
+        <v>0</v>
+      </c>
+      <c r="T71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A72" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C72">
+        <v>0</v>
+      </c>
+      <c r="D72">
+        <f>J72+K72+L72+M72+N72</f>
+        <v>125763.55741733511</v>
+      </c>
+      <c r="E72">
+        <v>282179.67125180899</v>
+      </c>
+      <c r="F72">
+        <v>0.87293045648394496</v>
+      </c>
+      <c r="G72">
+        <v>22626.697961956499</v>
+      </c>
+      <c r="H72">
+        <v>7102.5767129513297</v>
+      </c>
+      <c r="I72">
+        <v>9597.4591384874802</v>
+      </c>
+      <c r="J72">
+        <v>39326.733813395302</v>
+      </c>
+      <c r="K72">
+        <v>50843.184011688398</v>
+      </c>
+      <c r="L72">
+        <v>15303.798393134501</v>
+      </c>
+      <c r="M72">
+        <v>19297.530491231599</v>
+      </c>
+      <c r="N72">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O72">
+        <v>0</v>
+      </c>
+      <c r="P72">
         <f t="shared" si="13"/>
         <v>246323.22923633162</v>
       </c>
-      <c r="Q71">
+      <c r="Q72">
         <v>1127.27501714903</v>
       </c>
-      <c r="R71">
-        <v>0</v>
-      </c>
-      <c r="S71">
-        <v>0</v>
-      </c>
-      <c r="T71">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="1"/>
+      <c r="R72">
+        <v>0</v>
+      </c>
+      <c r="S72">
+        <v>0</v>
+      </c>
+      <c r="T72">
+        <v>0</v>
+      </c>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
+      <c r="A73" s="1"/>
+    </row>
+    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>20</v>
       </c>
-      <c r="B73" t="s">
-        <v>21</v>
-      </c>
-      <c r="C73">
-        <v>2</v>
-      </c>
-      <c r="D73">
-        <f>J73+K73+L73+M73+N73</f>
-        <v>116706.4157905087</v>
-      </c>
-      <c r="E73">
-        <v>282179.67125387199</v>
-      </c>
-      <c r="F73">
-        <v>0.840833383054163</v>
-      </c>
-      <c r="G73" s="4">
-        <v>20578.507216446698</v>
-      </c>
-      <c r="H73">
-        <v>7102.57515066207</v>
-      </c>
-      <c r="I73">
-        <v>2588.5052959285099</v>
-      </c>
-      <c r="J73">
-        <v>30269.587663037299</v>
-      </c>
-      <c r="K73">
-        <v>50843.185173268597</v>
-      </c>
-      <c r="L73">
-        <v>15303.8015139941</v>
-      </c>
-      <c r="M73">
-        <v>19297.530732323401</v>
-      </c>
-      <c r="N73">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O73">
-        <v>0</v>
-      </c>
-      <c r="P73">
-        <f t="shared" ref="P73:P74" si="14">D73+$P$1</f>
-        <v>237266.08760950522</v>
-      </c>
-      <c r="Q73">
-        <v>1127.2750356983099</v>
-      </c>
-      <c r="R73">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A74" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" t="s">
         <v>21</v>
       </c>
       <c r="C74">
@@ -4266,119 +4288,119 @@
       </c>
       <c r="D74">
         <f>J74+K74+L74+M74+N74</f>
+        <v>116706.4157905087</v>
+      </c>
+      <c r="E74">
+        <v>282179.67125387199</v>
+      </c>
+      <c r="F74">
+        <v>0.840833383054163</v>
+      </c>
+      <c r="G74" s="4">
+        <v>20578.507216446698</v>
+      </c>
+      <c r="H74">
+        <v>7102.57515066207</v>
+      </c>
+      <c r="I74">
+        <v>2588.5052959285099</v>
+      </c>
+      <c r="J74">
+        <v>30269.587663037299</v>
+      </c>
+      <c r="K74">
+        <v>50843.185173268597</v>
+      </c>
+      <c r="L74">
+        <v>15303.8015139941</v>
+      </c>
+      <c r="M74">
+        <v>19297.530732323401</v>
+      </c>
+      <c r="N74">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O74">
+        <v>0</v>
+      </c>
+      <c r="P74">
+        <f t="shared" ref="P74:P75" si="14">D74+$P$1</f>
+        <v>237266.08760950522</v>
+      </c>
+      <c r="Q74">
+        <v>1127.2750356983099</v>
+      </c>
+      <c r="R74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A75" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C75">
+        <v>2</v>
+      </c>
+      <c r="D75">
+        <f>J75+K75+L75+M75+N75</f>
         <v>121633.35860365373</v>
       </c>
-      <c r="E74">
+      <c r="E75">
         <v>282179.67123287602</v>
       </c>
-      <c r="F74">
+      <c r="F75">
         <v>0.85824890324911396</v>
       </c>
-      <c r="G74" s="4">
+      <c r="G75" s="4">
         <v>20824.7129679639</v>
       </c>
-      <c r="H74">
+      <c r="H75">
         <v>7456.39074483072</v>
       </c>
-      <c r="I74">
+      <c r="I75">
         <v>5114.4587365303096</v>
       </c>
-      <c r="J74">
+      <c r="J75">
         <v>33395.562449324898</v>
       </c>
-      <c r="K74">
+      <c r="K75">
         <v>51302.320205525801</v>
       </c>
-      <c r="L74">
+      <c r="L75">
         <v>16537.7269222135</v>
       </c>
-      <c r="M74">
+      <c r="M75">
         <v>19392.801250865799</v>
       </c>
-      <c r="N74">
+      <c r="N75">
         <v>1004.9477757237401</v>
       </c>
-      <c r="O74">
-        <v>0</v>
-      </c>
-      <c r="P74">
+      <c r="O75">
+        <v>0</v>
+      </c>
+      <c r="P75">
         <f t="shared" si="14"/>
         <v>242193.03042265025</v>
       </c>
-      <c r="Q74">
+      <c r="Q75">
         <v>1183.4303612998101</v>
       </c>
-      <c r="R74">
+      <c r="R75">
         <v>15931.1957490451</v>
       </c>
-      <c r="S74">
+      <c r="S75">
         <v>346.33034237054602</v>
       </c>
-      <c r="T74">
+      <c r="T75">
         <v>1.0959871186973</v>
-      </c>
-    </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
-        <v>20</v>
-      </c>
-      <c r="B76" t="s">
-        <v>21</v>
-      </c>
-      <c r="C76">
-        <v>4</v>
-      </c>
-      <c r="D76">
-        <f>J76+K76+L76+M76+N76</f>
-        <v>116706.4157905051</v>
-      </c>
-      <c r="E76">
-        <v>282179.671253876</v>
-      </c>
-      <c r="F76">
-        <v>0.84083338305413902</v>
-      </c>
-      <c r="G76" s="4">
-        <v>20578.5072164468</v>
-      </c>
-      <c r="H76">
-        <v>7102.5751506616798</v>
-      </c>
-      <c r="I76">
-        <v>2588.50529592865</v>
-      </c>
-      <c r="J76">
-        <v>30269.587663037099</v>
-      </c>
-      <c r="K76">
-        <v>50843.185173268197</v>
-      </c>
-      <c r="L76">
-        <v>15303.8015139912</v>
-      </c>
-      <c r="M76">
-        <v>19297.530732323299</v>
-      </c>
-      <c r="N76">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O76">
-        <v>0</v>
-      </c>
-      <c r="P76">
-        <f t="shared" ref="P76:P78" si="15">D76+$P$1</f>
-        <v>237266.08760950161</v>
-      </c>
-      <c r="Q76">
-        <v>1127.2750356983499</v>
-      </c>
-      <c r="R76">
-        <v>0</v>
       </c>
     </row>
     <row r="77" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B77" t="s">
         <v>21</v>
@@ -4388,451 +4410,445 @@
       </c>
       <c r="D77">
         <f>J77+K77+L77+M77+N77</f>
+        <v>116706.4157905051</v>
+      </c>
+      <c r="E77">
+        <v>282179.671253876</v>
+      </c>
+      <c r="F77">
+        <v>0.84083338305413902</v>
+      </c>
+      <c r="G77" s="4">
+        <v>20578.5072164468</v>
+      </c>
+      <c r="H77">
+        <v>7102.5751506616798</v>
+      </c>
+      <c r="I77">
+        <v>2588.50529592865</v>
+      </c>
+      <c r="J77">
+        <v>30269.587663037099</v>
+      </c>
+      <c r="K77">
+        <v>50843.185173268197</v>
+      </c>
+      <c r="L77">
+        <v>15303.8015139912</v>
+      </c>
+      <c r="M77">
+        <v>19297.530732323299</v>
+      </c>
+      <c r="N77">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O77">
+        <v>0</v>
+      </c>
+      <c r="P77">
+        <f t="shared" ref="P77:P79" si="15">D77+$P$1</f>
+        <v>237266.08760950161</v>
+      </c>
+      <c r="Q77">
+        <v>1127.2750356983499</v>
+      </c>
+      <c r="R77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>22</v>
+      </c>
+      <c r="B78" t="s">
+        <v>21</v>
+      </c>
+      <c r="C78">
+        <v>4</v>
+      </c>
+      <c r="D78">
+        <f>J78+K78+L78+M78+N78</f>
         <v>121744.79706913032</v>
       </c>
-      <c r="E77">
+      <c r="E78">
         <v>282179.88376308198</v>
       </c>
-      <c r="F77">
+      <c r="F78">
         <v>0.85713546401894802</v>
       </c>
-      <c r="G77">
+      <c r="G78">
         <v>21291.5607898614</v>
       </c>
-      <c r="H77">
+      <c r="H78">
         <v>7432.3603175362596</v>
       </c>
-      <c r="I77">
+      <c r="I78">
         <v>5035.2758648834497</v>
       </c>
-      <c r="J77">
+      <c r="J78">
         <v>33759.196972281097</v>
       </c>
-      <c r="K77">
+      <c r="K78">
         <v>51128.3645002267</v>
       </c>
-      <c r="L77">
+      <c r="L78">
         <v>16070.129576240101</v>
       </c>
-      <c r="M77">
+      <c r="M78">
         <v>19356.7120304526</v>
       </c>
-      <c r="N77">
+      <c r="N78">
         <v>1430.39398992981</v>
       </c>
-      <c r="O77">
-        <v>0</v>
-      </c>
-      <c r="P77">
+      <c r="O78">
+        <v>0</v>
+      </c>
+      <c r="P78">
         <f t="shared" si="15"/>
         <v>242304.46888812684</v>
       </c>
-      <c r="Q77">
+      <c r="Q78">
         <v>1179.61640190856</v>
       </c>
-      <c r="R77">
+      <c r="R78">
         <v>13411.4010346792</v>
       </c>
-      <c r="S77">
+      <c r="S78">
         <v>478.97860838140201</v>
       </c>
-      <c r="T77">
+      <c r="T78">
         <v>0.22564405635506199</v>
       </c>
-      <c r="U77">
+      <c r="U78">
         <v>10550.3210016294</v>
       </c>
-      <c r="V77">
+      <c r="V78">
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="D78">
-        <f>D77-D71</f>
+    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="D79">
+        <f>D78-D72</f>
         <v>-4018.7603482047853</v>
       </c>
-      <c r="E78">
-        <f t="shared" ref="E78:N78" si="16">E77-E71</f>
+      <c r="E79">
+        <f t="shared" ref="E79:N79" si="16">E78-E72</f>
         <v>0.21251127298455685</v>
       </c>
-      <c r="F78">
+      <c r="F79">
         <f t="shared" si="16"/>
         <v>-1.5794992464996938E-2</v>
       </c>
-      <c r="G78">
+      <c r="G79">
         <f t="shared" si="16"/>
         <v>-1335.1371720950992</v>
       </c>
-      <c r="H78">
+      <c r="H79">
         <f t="shared" si="16"/>
         <v>329.78360458492989</v>
       </c>
-      <c r="I78">
+      <c r="I79">
         <f t="shared" si="16"/>
         <v>-4562.1832736040305</v>
       </c>
-      <c r="J78">
+      <c r="J79">
         <f t="shared" si="16"/>
         <v>-5567.5368411142044</v>
       </c>
-      <c r="K78">
+      <c r="K79">
         <f t="shared" si="16"/>
         <v>285.1804885383026</v>
       </c>
-      <c r="L78">
+      <c r="L79">
         <f t="shared" si="16"/>
         <v>766.33118310559985</v>
       </c>
-      <c r="M78">
+      <c r="M79">
         <f t="shared" si="16"/>
         <v>59.181539221001003</v>
       </c>
-      <c r="N78">
+      <c r="N79">
         <f t="shared" si="16"/>
         <v>438.08328204450595</v>
       </c>
-      <c r="P78">
+      <c r="P79">
         <f t="shared" si="15"/>
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A79" s="1" t="s">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A80" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G79" s="4"/>
-    </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
-        <v>22</v>
-      </c>
-      <c r="B80" t="s">
-        <v>21</v>
-      </c>
-      <c r="C80">
-        <v>4</v>
-      </c>
-      <c r="D80">
-        <f>J80+K80+L80+M80+N80</f>
-        <v>147118.48206815872</v>
-      </c>
-      <c r="E80">
-        <v>355610.364944759</v>
-      </c>
-      <c r="F80">
-        <v>0.75267772890587503</v>
-      </c>
-      <c r="G80">
-        <v>25765.651662743599</v>
-      </c>
-      <c r="H80">
-        <v>7150.9042815892099</v>
-      </c>
-      <c r="I80">
-        <v>5144.3184852884797</v>
-      </c>
-      <c r="J80">
-        <v>38060.874429621297</v>
-      </c>
-      <c r="K80">
-        <v>64168.339029134899</v>
-      </c>
-      <c r="L80">
-        <v>19539.954214541001</v>
-      </c>
-      <c r="M80">
-        <v>24338.851661831999</v>
-      </c>
-      <c r="N80">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O80">
-        <v>0</v>
-      </c>
-      <c r="P80">
-        <f t="shared" ref="P80" si="17">D80+$P$1</f>
-        <v>267678.15388715523</v>
-      </c>
-      <c r="Q80">
-        <v>1597.68911089628</v>
-      </c>
-      <c r="R80">
-        <v>13084.0423994256</v>
-      </c>
-      <c r="S80">
-        <v>467.28722855091399</v>
-      </c>
-      <c r="T80">
-        <v>-0.25904927491985202</v>
-      </c>
+      <c r="G80" s="4"/>
     </row>
     <row r="81" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>22</v>
       </c>
       <c r="B81" t="s">
+        <v>21</v>
+      </c>
+      <c r="C81">
+        <v>4</v>
+      </c>
+      <c r="D81">
+        <f>J81+K81+L81+M81+N81</f>
+        <v>147118.48206815872</v>
+      </c>
+      <c r="E81">
+        <v>355610.364944759</v>
+      </c>
+      <c r="F81">
+        <v>0.75267772890587503</v>
+      </c>
+      <c r="G81">
+        <v>25765.651662743599</v>
+      </c>
+      <c r="H81">
+        <v>7150.9042815892099</v>
+      </c>
+      <c r="I81">
+        <v>5144.3184852884797</v>
+      </c>
+      <c r="J81">
+        <v>38060.874429621297</v>
+      </c>
+      <c r="K81">
+        <v>64168.339029134899</v>
+      </c>
+      <c r="L81">
+        <v>19539.954214541001</v>
+      </c>
+      <c r="M81">
+        <v>24338.851661831999</v>
+      </c>
+      <c r="N81">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O81">
+        <v>0</v>
+      </c>
+      <c r="P81">
+        <f t="shared" ref="P81" si="17">D81+$P$1</f>
+        <v>267678.15388715523</v>
+      </c>
+      <c r="Q81">
+        <v>1597.68911089628</v>
+      </c>
+      <c r="R81">
+        <v>13084.0423994256</v>
+      </c>
+      <c r="S81">
+        <v>467.28722855091399</v>
+      </c>
+      <c r="T81">
+        <v>-0.25904927491985202</v>
+      </c>
+    </row>
+    <row r="82" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>22</v>
+      </c>
+      <c r="B82" t="s">
         <v>35</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C82" t="s">
         <v>35</v>
       </c>
-      <c r="D81" t="s">
+      <c r="D82" t="s">
         <v>36</v>
       </c>
-      <c r="E81" t="s">
+      <c r="E82" t="s">
         <v>36</v>
       </c>
-      <c r="F81" t="s">
+      <c r="F82" t="s">
         <v>36</v>
       </c>
-      <c r="G81" s="4">
+      <c r="G82" s="4">
         <v>28838</v>
       </c>
-      <c r="H81">
+      <c r="H82">
         <v>7567.5</v>
       </c>
-      <c r="I81">
+      <c r="I82">
         <v>13764.1</v>
       </c>
-      <c r="J81">
+      <c r="J82">
         <v>50169.7</v>
       </c>
-      <c r="K81" t="s">
+      <c r="K82" t="s">
         <v>36</v>
       </c>
-      <c r="L81" t="s">
+      <c r="L82" t="s">
         <v>36</v>
       </c>
-      <c r="M81" t="s">
+      <c r="M82" t="s">
         <v>36</v>
       </c>
-      <c r="N81" t="s">
+      <c r="N82" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="83" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A83" s="1" t="s">
+    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A84" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G83" s="4"/>
-      <c r="P83" t="s">
+      <c r="G84" s="4"/>
+      <c r="P84" t="s">
         <v>15</v>
       </c>
-      <c r="Q83" t="s">
+      <c r="Q84" t="s">
         <v>16</v>
       </c>
-      <c r="R83" t="s">
+      <c r="R84" t="s">
         <v>17</v>
       </c>
-      <c r="S83" t="s">
+      <c r="S84" t="s">
         <v>18</v>
       </c>
-      <c r="T83" t="s">
+      <c r="T84" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
-        <v>0</v>
-      </c>
-      <c r="B84" t="s">
+    <row r="85" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>0</v>
+      </c>
+      <c r="B85" t="s">
         <v>1</v>
       </c>
-      <c r="C84" t="s">
+      <c r="C85" t="s">
         <v>2</v>
       </c>
-      <c r="D84" t="s">
+      <c r="D85" t="s">
         <v>3</v>
       </c>
-      <c r="E84" t="s">
+      <c r="E85" t="s">
         <v>4</v>
       </c>
-      <c r="F84" t="s">
+      <c r="F85" t="s">
         <v>5</v>
       </c>
-      <c r="G84" s="4" t="s">
+      <c r="G85" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H84" t="s">
+      <c r="H85" t="s">
         <v>7</v>
       </c>
-      <c r="I84" t="s">
+      <c r="I85" t="s">
         <v>8</v>
       </c>
-      <c r="J84" t="s">
+      <c r="J85" t="s">
         <v>9</v>
       </c>
-      <c r="K84" t="s">
+      <c r="K85" t="s">
         <v>10</v>
       </c>
-      <c r="L84" t="s">
+      <c r="L85" t="s">
         <v>11</v>
       </c>
-      <c r="M84" t="s">
+      <c r="M85" t="s">
         <v>12</v>
       </c>
-      <c r="N84" t="s">
+      <c r="N85" t="s">
         <v>13</v>
       </c>
-      <c r="O84" t="s">
+      <c r="O85" t="s">
         <v>14</v>
       </c>
-      <c r="P84">
+      <c r="P85">
         <v>63734.6679</v>
       </c>
-      <c r="Q84">
+      <c r="Q85">
         <v>1078.4492829999999</v>
       </c>
-      <c r="R84">
+      <c r="R85">
         <v>624.70352849999995</v>
       </c>
-      <c r="S84">
+      <c r="S85">
         <v>13.014656840000001</v>
       </c>
-      <c r="T84">
+      <c r="T85">
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="85" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A85" s="2" t="s">
+    <row r="86" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A86" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B86" t="s">
         <v>21</v>
       </c>
-      <c r="C85">
+      <c r="C86">
         <v>4</v>
       </c>
-      <c r="D85">
+      <c r="D86">
         <v>29525.427309999999</v>
       </c>
-      <c r="E85">
+      <c r="E86">
         <v>80391.755990000005</v>
       </c>
-      <c r="F85">
+      <c r="F86">
         <v>0.79280104200000001</v>
       </c>
-      <c r="G85" s="4">
+      <c r="G86" s="4">
         <v>5050.6365619999997</v>
       </c>
-      <c r="H85">
+      <c r="H86">
         <v>4678.3390820000004</v>
       </c>
-      <c r="I85">
+      <c r="I86">
         <v>2508.6600360000002</v>
       </c>
-      <c r="J85">
+      <c r="J86">
         <v>12237.635679999999</v>
       </c>
-      <c r="K85">
+      <c r="K86">
         <v>13920</v>
       </c>
-      <c r="L85">
+      <c r="L86">
         <v>2841.544922</v>
       </c>
-      <c r="M85">
+      <c r="M86">
         <v>5380.5444360000001</v>
       </c>
-      <c r="N85">
+      <c r="N86">
         <v>279.27307350000001</v>
       </c>
-      <c r="O85">
-        <v>0</v>
-      </c>
-      <c r="P85">
+      <c r="O86">
+        <v>0</v>
+      </c>
+      <c r="P86">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q85">
+      <c r="Q86">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R85">
+      <c r="R86">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S85">
+      <c r="S86">
         <v>452.7322633</v>
       </c>
-      <c r="T85">
+      <c r="T86">
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A86" s="7" t="s">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A87" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
         <v>32</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B89" t="s">
         <v>33</v>
       </c>
-      <c r="C88" t="s">
+      <c r="C89" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A89">
-        <v>20</v>
-      </c>
-      <c r="B89">
-        <v>60</v>
-      </c>
-      <c r="C89">
-        <v>2</v>
-      </c>
-      <c r="D89">
-        <f t="shared" ref="D89:D95" si="18">J89+K89+L89+M89+N89</f>
-        <v>120712.69088313227</v>
-      </c>
-      <c r="E89">
-        <v>282179.67123285501</v>
-      </c>
-      <c r="F89">
-        <v>0.854946898908852</v>
-      </c>
-      <c r="G89">
-        <v>18681.222424938602</v>
-      </c>
-      <c r="H89">
-        <v>5354.6114985546601</v>
-      </c>
-      <c r="I89">
-        <v>8156.08309050551</v>
-      </c>
-      <c r="J89">
-        <v>32191.917013998798</v>
-      </c>
-      <c r="K89">
-        <v>51372.124296964801</v>
-      </c>
-      <c r="L89">
-        <v>16725.325417965501</v>
-      </c>
-      <c r="M89">
-        <v>19407.285599838699</v>
-      </c>
-      <c r="N89">
-        <v>1016.03855436447</v>
-      </c>
-      <c r="O89">
-        <v>0</v>
-      </c>
-      <c r="P89">
-        <f t="shared" ref="P89:P95" si="19">D89+$P$1</f>
-        <v>241272.36270212877</v>
-      </c>
-      <c r="Q89">
-        <v>1192.7637589594799</v>
-      </c>
-      <c r="R89">
-        <v>19736.206339365101</v>
-      </c>
-      <c r="S89">
-        <v>481.37088632597801</v>
-      </c>
-      <c r="T89" s="6">
-        <v>0.12591688076390301</v>
       </c>
     </row>
     <row r="90" spans="1:20" x14ac:dyDescent="0.35">
@@ -4840,63 +4856,63 @@
         <v>20</v>
       </c>
       <c r="B90">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C90">
         <v>2</v>
       </c>
       <c r="D90">
-        <f t="shared" si="18"/>
-        <v>119392.42354269064</v>
+        <f t="shared" ref="D90:D96" si="18">J90+K90+L90+M90+N90</f>
+        <v>120712.69088313227</v>
       </c>
       <c r="E90">
-        <v>282254.81855225202</v>
+        <v>282179.67123285501</v>
       </c>
       <c r="F90">
-        <v>0.85006146065890897</v>
+        <v>0.854946898908852</v>
       </c>
       <c r="G90">
-        <v>19407.840072768398</v>
+        <v>18681.222424938602</v>
       </c>
       <c r="H90">
-        <v>5891.8301217549197</v>
+        <v>5354.6114985546601</v>
       </c>
       <c r="I90">
-        <v>6659.4942697455399</v>
+        <v>8156.08309050551</v>
       </c>
       <c r="J90">
-        <v>31959.164464268899</v>
+        <v>32191.917013998798</v>
       </c>
       <c r="K90">
-        <v>51102.045942938203</v>
+        <v>51372.124296964801</v>
       </c>
       <c r="L90">
-        <v>15967.176494174801</v>
+        <v>16725.325417965501</v>
       </c>
       <c r="M90">
-        <v>19353.573908279199</v>
+        <v>19407.285599838699</v>
       </c>
       <c r="N90">
-        <v>1010.46273302954</v>
+        <v>1016.03855436447</v>
       </c>
       <c r="O90">
         <v>0</v>
       </c>
       <c r="P90">
-        <f t="shared" si="19"/>
-        <v>239952.09536168716</v>
+        <f t="shared" ref="P90:P96" si="19">D90+$P$1</f>
+        <v>241272.36270212877</v>
       </c>
       <c r="Q90">
-        <v>1312.43161993582</v>
+        <v>1192.7637589594799</v>
       </c>
       <c r="R90">
-        <v>18377.616631847999</v>
+        <v>19736.206339365101</v>
       </c>
       <c r="S90">
-        <v>459.4404157962</v>
+        <v>481.37088632597801</v>
       </c>
       <c r="T90" s="6">
-        <v>0.14758705239613301</v>
+        <v>0.12591688076390301</v>
       </c>
     </row>
     <row r="91" spans="1:20" x14ac:dyDescent="0.35">
@@ -4904,41 +4920,41 @@
         <v>20</v>
       </c>
       <c r="B91">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C91">
         <v>2</v>
       </c>
       <c r="D91">
         <f t="shared" si="18"/>
-        <v>117777.02945340994</v>
+        <v>119392.42354269064</v>
       </c>
       <c r="E91">
-        <v>282179.67123287299</v>
+        <v>282254.81855225202</v>
       </c>
       <c r="F91">
-        <v>0.84456314023622803</v>
+        <v>0.85006146065890897</v>
       </c>
       <c r="G91">
-        <v>19298.245593088301</v>
+        <v>19407.840072768398</v>
       </c>
       <c r="H91">
-        <v>5682.0016560700296</v>
+        <v>5891.8301217549197</v>
       </c>
       <c r="I91">
-        <v>5350.3346939491703</v>
+        <v>6659.4942697455399</v>
       </c>
       <c r="J91">
-        <v>30330.5819431075</v>
+        <v>31959.164464268899</v>
       </c>
       <c r="K91">
-        <v>51097.733915068202</v>
+        <v>51102.045942938203</v>
       </c>
       <c r="L91">
-        <v>15987.901266609</v>
+        <v>15967.176494174801</v>
       </c>
       <c r="M91">
-        <v>19350.349595595701</v>
+        <v>19353.573908279199</v>
       </c>
       <c r="N91">
         <v>1010.46273302954</v>
@@ -4948,19 +4964,19 @@
       </c>
       <c r="P91">
         <f t="shared" si="19"/>
-        <v>238336.70127240644</v>
+        <v>239952.09536168716</v>
       </c>
       <c r="Q91">
-        <v>1265.6913868611</v>
+        <v>1312.43161993582</v>
       </c>
       <c r="R91">
-        <v>17746.163883660702</v>
+        <v>18377.616631847999</v>
       </c>
       <c r="S91">
-        <v>507.03325381887902</v>
+        <v>459.4404157962</v>
       </c>
       <c r="T91" s="6">
-        <v>-0.25983751983286502</v>
+        <v>0.14758705239613301</v>
       </c>
     </row>
     <row r="92" spans="1:20" x14ac:dyDescent="0.35">
@@ -4968,105 +4984,105 @@
         <v>20</v>
       </c>
       <c r="B92">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C92">
         <v>2</v>
       </c>
       <c r="D92">
         <f t="shared" si="18"/>
-        <v>116625.1695160947</v>
+        <v>117777.02945340994</v>
       </c>
       <c r="E92">
-        <v>282182.50548365602</v>
+        <v>282179.67123287299</v>
       </c>
       <c r="F92">
-        <v>0.84045954058697003</v>
+        <v>0.84456314023622803</v>
       </c>
       <c r="G92">
-        <v>19302.752565837702</v>
+        <v>19298.245593088301</v>
       </c>
       <c r="H92">
-        <v>6226.5181629292701</v>
+        <v>5682.0016560700296</v>
       </c>
       <c r="I92">
-        <v>3974.5318253822402</v>
+        <v>5350.3346939491703</v>
       </c>
       <c r="J92">
-        <v>29503.802554149199</v>
+        <v>30330.5819431075</v>
       </c>
       <c r="K92">
-        <v>51013.610661725899</v>
+        <v>51097.733915068202</v>
       </c>
       <c r="L92">
-        <v>15760.601295416</v>
+        <v>15987.901266609</v>
       </c>
       <c r="M92">
-        <v>19332.981882301501</v>
+        <v>19350.349595595701</v>
       </c>
       <c r="N92">
-        <v>1014.17312250211</v>
+        <v>1010.46273302954</v>
       </c>
       <c r="O92">
         <v>0</v>
       </c>
       <c r="P92">
         <f t="shared" si="19"/>
-        <v>237184.84133509122</v>
+        <v>238336.70127240644</v>
       </c>
       <c r="Q92">
-        <v>1386.9848841974899</v>
+        <v>1265.6913868611</v>
       </c>
       <c r="R92">
-        <v>18436.445202769701</v>
+        <v>17746.163883660702</v>
       </c>
       <c r="S92">
-        <v>209.50505912238299</v>
+        <v>507.03325381887902</v>
       </c>
       <c r="T92" s="6">
-        <v>0.28049716262959101</v>
+        <v>-0.25983751983286502</v>
       </c>
     </row>
     <row r="93" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A93" s="3">
+      <c r="A93">
         <v>20</v>
       </c>
-      <c r="B93" s="3">
-        <v>20</v>
-      </c>
-      <c r="C93" s="3">
+      <c r="B93">
+        <v>30</v>
+      </c>
+      <c r="C93">
         <v>2</v>
       </c>
       <c r="D93">
         <f t="shared" si="18"/>
-        <v>115198.459983006</v>
+        <v>116625.1695160947</v>
       </c>
       <c r="E93">
-        <v>282179.67123297497</v>
+        <v>282182.50548365602</v>
       </c>
       <c r="F93">
-        <v>0.83541194997266699</v>
+        <v>0.84045954058697003</v>
       </c>
       <c r="G93">
-        <v>19351.2255529412</v>
+        <v>19302.752565837702</v>
       </c>
       <c r="H93">
-        <v>6002.0469674603501</v>
+        <v>6226.5181629292701</v>
       </c>
       <c r="I93">
-        <v>2645.4376652921501</v>
+        <v>3974.5318253822402</v>
       </c>
       <c r="J93">
-        <v>27998.710185693701</v>
+        <v>29503.802554149199</v>
       </c>
       <c r="K93">
-        <v>51033.4442867088</v>
+        <v>51013.610661725899</v>
       </c>
       <c r="L93">
-        <v>15815.1228903871</v>
+        <v>15760.601295416</v>
       </c>
       <c r="M93">
-        <v>19337.009497714302</v>
+        <v>19332.981882301501</v>
       </c>
       <c r="N93">
         <v>1014.17312250211</v>
@@ -5076,83 +5092,83 @@
       </c>
       <c r="P93">
         <f t="shared" si="19"/>
-        <v>235758.13180200252</v>
+        <v>237184.84133509122</v>
       </c>
       <c r="Q93">
-        <v>1336.98290493166</v>
+        <v>1386.9848841974899</v>
       </c>
       <c r="R93">
-        <v>18577.307877855899</v>
+        <v>18436.445202769701</v>
       </c>
       <c r="S93">
-        <v>432.030415764091</v>
+        <v>209.50505912238299</v>
       </c>
       <c r="T93" s="6">
-        <v>-0.122490141098651</v>
+        <v>0.28049716262959101</v>
       </c>
     </row>
     <row r="94" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A94">
+      <c r="A94" s="3">
         <v>20</v>
       </c>
-      <c r="B94">
-        <v>15</v>
-      </c>
-      <c r="C94">
+      <c r="B94" s="3">
+        <v>20</v>
+      </c>
+      <c r="C94" s="3">
         <v>2</v>
       </c>
       <c r="D94">
         <f t="shared" si="18"/>
-        <v>114451.25872361983</v>
+        <v>115198.459983006</v>
       </c>
       <c r="E94">
-        <v>282179.67123267101</v>
+        <v>282179.67123297497</v>
       </c>
       <c r="F94">
-        <v>0.83277713625127903</v>
+        <v>0.83541194997266699</v>
       </c>
       <c r="G94">
-        <v>19390.977969205</v>
+        <v>19351.2255529412</v>
       </c>
       <c r="H94">
-        <v>5599.5405456203798</v>
+        <v>6002.0469674603501</v>
       </c>
       <c r="I94">
-        <v>2128.1287863747102</v>
+        <v>2645.4376652921501</v>
       </c>
       <c r="J94">
-        <v>27118.647301200101</v>
+        <v>27998.710185693701</v>
       </c>
       <c r="K94">
-        <v>51068.507704320902</v>
+        <v>51033.4442867088</v>
       </c>
       <c r="L94">
-        <v>15909.3558282099</v>
+        <v>15815.1228903871</v>
       </c>
       <c r="M94">
-        <v>19344.285156859401</v>
+        <v>19337.009497714302</v>
       </c>
       <c r="N94">
-        <v>1010.46273302954</v>
+        <v>1014.17312250211</v>
       </c>
       <c r="O94">
         <v>0</v>
       </c>
       <c r="P94">
         <f t="shared" si="19"/>
-        <v>235010.93054261635</v>
+        <v>235758.13180200252</v>
       </c>
       <c r="Q94">
-        <v>1247.3228025527501</v>
+        <v>1336.98290493166</v>
       </c>
       <c r="R94">
-        <v>16417.502561416801</v>
+        <v>18577.307877855899</v>
       </c>
       <c r="S94">
-        <v>469.07150175476602</v>
+        <v>432.030415764091</v>
       </c>
       <c r="T94" s="6">
-        <v>0.46004655114715598</v>
+        <v>-0.122490141098651</v>
       </c>
     </row>
     <row r="95" spans="1:20" x14ac:dyDescent="0.35">
@@ -5160,62 +5176,126 @@
         <v>20</v>
       </c>
       <c r="B95">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C95">
         <v>2</v>
       </c>
       <c r="D95">
         <f t="shared" si="18"/>
-        <v>114787.7594081375</v>
+        <v>114451.25872361983</v>
       </c>
       <c r="E95">
-        <v>282179.67123287602</v>
+        <v>282179.67123267101</v>
       </c>
       <c r="F95">
-        <v>0.83403396920434802</v>
+        <v>0.83277713625127903</v>
       </c>
       <c r="G95">
-        <v>20436.472361711199</v>
+        <v>19390.977969205</v>
       </c>
       <c r="H95">
-        <v>4946.5396722567002</v>
+        <v>5599.5405456203798</v>
       </c>
       <c r="I95">
-        <v>2967.9237851293901</v>
+        <v>2128.1287863747102</v>
       </c>
       <c r="J95">
-        <v>28350.9358190973</v>
+        <v>27118.647301200101</v>
       </c>
       <c r="K95">
-        <v>50843.184005923598</v>
+        <v>51068.507704320902</v>
       </c>
       <c r="L95">
-        <v>15303.798385783</v>
+        <v>15909.3558282099</v>
       </c>
       <c r="M95">
-        <v>19297.530489448302</v>
+        <v>19344.285156859401</v>
       </c>
       <c r="N95">
-        <v>992.31070788530405</v>
+        <v>1010.46273302954</v>
       </c>
       <c r="O95">
         <v>0</v>
       </c>
       <c r="P95">
         <f t="shared" si="19"/>
+        <v>235010.93054261635</v>
+      </c>
+      <c r="Q95">
+        <v>1247.3228025527501</v>
+      </c>
+      <c r="R95">
+        <v>16417.502561416801</v>
+      </c>
+      <c r="S95">
+        <v>469.07150175476602</v>
+      </c>
+      <c r="T95" s="6">
+        <v>0.46004655114715598</v>
+      </c>
+    </row>
+    <row r="96" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A96">
+        <v>20</v>
+      </c>
+      <c r="B96">
+        <v>12</v>
+      </c>
+      <c r="C96">
+        <v>2</v>
+      </c>
+      <c r="D96">
+        <f t="shared" si="18"/>
+        <v>114787.7594081375</v>
+      </c>
+      <c r="E96">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F96">
+        <v>0.83403396920434802</v>
+      </c>
+      <c r="G96">
+        <v>20436.472361711199</v>
+      </c>
+      <c r="H96">
+        <v>4946.5396722567002</v>
+      </c>
+      <c r="I96">
+        <v>2967.9237851293901</v>
+      </c>
+      <c r="J96">
+        <v>28350.9358190973</v>
+      </c>
+      <c r="K96">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L96">
+        <v>15303.798385783</v>
+      </c>
+      <c r="M96">
+        <v>19297.530489448302</v>
+      </c>
+      <c r="N96">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O96">
+        <v>0</v>
+      </c>
+      <c r="P96">
+        <f t="shared" si="19"/>
         <v>235347.43122713402</v>
       </c>
-      <c r="Q95">
+      <c r="Q96">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R95">
+      <c r="R96">
         <v>13.380488321454299</v>
       </c>
-      <c r="S95">
+      <c r="S96">
         <v>2.67609766429086</v>
       </c>
-      <c r="T95" s="6">
+      <c r="T96" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improving the analytical equations for cost savings. Work remains.
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8070B048-2D18-40B1-BE2F-8718C4D8BA85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09720A58-31D4-4647-97B7-598DF1A895E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -44,6 +44,7 @@
     <author>tc={DFECE21F-32E0-4210-824A-1E57B1730184}</author>
     <author>tc={7128E1A1-FC03-4EA4-B47C-4E0569E512E5}</author>
     <author>tc={FA39747C-8399-4DE8-BFC3-16508DD92F20}</author>
+    <author>tc={0CE66D44-40D7-4762-8700-23B9C4E639CE}</author>
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
     <author>tc={F9308CF0-AB74-4ABB-91B6-7382ECEADD39}</author>
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
@@ -132,7 +133,15 @@
     This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</t>
       </text>
     </comment>
-    <comment ref="A48" authorId="9" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A32" authorId="9" shapeId="0" xr:uid="{0CE66D44-40D7-4762-8700-23B9C4E639CE}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Forced Five shutdowns</t>
+      </text>
+    </comment>
+    <comment ref="A50" authorId="10" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -140,7 +149,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="A49" authorId="10" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A51" authorId="11" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -148,7 +157,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T49" authorId="11" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T51" authorId="12" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -158,7 +167,7 @@
     The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A55" authorId="12" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A57" authorId="13" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -166,7 +175,7 @@
     Result from the fast solve</t>
       </text>
     </comment>
-    <comment ref="A58" authorId="13" shapeId="0" xr:uid="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
+    <comment ref="A60" authorId="14" shapeId="0" xr:uid="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -174,7 +183,7 @@
     Wrong baseline power was used</t>
       </text>
     </comment>
-    <comment ref="A59" authorId="14" shapeId="0" xr:uid="{7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}">
+    <comment ref="A61" authorId="15" shapeId="0" xr:uid="{7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -182,7 +191,7 @@
     Old solution where there is only one plant shutdown.</t>
       </text>
     </comment>
-    <comment ref="A60" authorId="15" shapeId="0" xr:uid="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
+    <comment ref="A62" authorId="16" shapeId="0" xr:uid="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -192,7 +201,7 @@
     I’d like to see numbers for only one shutdown</t>
       </text>
     </comment>
-    <comment ref="A61" authorId="16" shapeId="0" xr:uid="{0EBBD83F-AB64-4248-87E6-B99F88EE5F88}">
+    <comment ref="A63" authorId="17" shapeId="0" xr:uid="{0EBBD83F-AB64-4248-87E6-B99F88EE5F88}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -200,7 +209,7 @@
     Only one plant shutdown allowed</t>
       </text>
     </comment>
-    <comment ref="A68" authorId="17" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+    <comment ref="A70" authorId="18" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -209,7 +218,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="A75" authorId="18" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
+    <comment ref="A77" authorId="19" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -217,7 +226,7 @@
     Pretty sure this solution is wrong, but I don’t think I need this case for the paper</t>
       </text>
     </comment>
-    <comment ref="A81" authorId="19" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A83" authorId="20" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -225,7 +234,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T93" authorId="20" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T95" authorId="21" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -238,7 +247,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="44">
   <si>
     <t>Season</t>
   </si>
@@ -1307,47 +1316,50 @@
   <threadedComment ref="A28" dT="2026-07-15T17:22:40.80" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FA39747C-8399-4DE8-BFC3-16508DD92F20}">
     <text>This cannot be higher than the two flex trains case, so I think it’s fair to use the same solution for both.</text>
   </threadedComment>
-  <threadedComment ref="A48" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+  <threadedComment ref="A32" dT="2026-07-23T21:50:18.94" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{0CE66D44-40D7-4762-8700-23B9C4E639CE}">
+    <text>Forced Five shutdowns</text>
+  </threadedComment>
+  <threadedComment ref="A50" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
-  <threadedComment ref="A49" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+  <threadedComment ref="A51" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
     <text>Summer week = hot summer weekdays + high weekends</text>
   </threadedComment>
-  <threadedComment ref="T49" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T51" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure</text>
   </threadedComment>
-  <threadedComment ref="T49" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T51" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>The baseline costs have to be updated in accordance with the demand structure type</text>
   </threadedComment>
-  <threadedComment ref="A55" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+  <threadedComment ref="A57" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
     <text>Result from the fast solve</text>
   </threadedComment>
-  <threadedComment ref="A58" dT="2026-07-21T19:50:00.59" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
+  <threadedComment ref="A60" dT="2026-07-21T19:50:00.59" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
     <text>Wrong baseline power was used</text>
   </threadedComment>
-  <threadedComment ref="A59" dT="2026-07-22T19:28:49.80" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}">
+  <threadedComment ref="A61" dT="2026-07-22T19:28:49.80" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}">
     <text>Old solution where there is only one plant shutdown.</text>
   </threadedComment>
-  <threadedComment ref="A60" dT="2026-07-22T19:29:10.19" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
+  <threadedComment ref="A62" dT="2026-07-22T19:29:10.19" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
     <text>Solution where there is a shutdown for all peak hours</text>
   </threadedComment>
-  <threadedComment ref="A60" dT="2026-07-22T19:37:51.21" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{DB15DF8F-6887-4CDD-9A38-5D318EAEEFFF}" parentId="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
+  <threadedComment ref="A62" dT="2026-07-22T19:37:51.21" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{DB15DF8F-6887-4CDD-9A38-5D318EAEEFFF}" parentId="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
     <text>I’d like to see numbers for only one shutdown</text>
   </threadedComment>
-  <threadedComment ref="A61" dT="2026-07-22T21:09:49.14" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{0EBBD83F-AB64-4248-87E6-B99F88EE5F88}">
+  <threadedComment ref="A63" dT="2026-07-22T21:09:49.14" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{0EBBD83F-AB64-4248-87E6-B99F88EE5F88}">
     <text>Only one plant shutdown allowed</text>
   </threadedComment>
-  <threadedComment ref="A68" dT="2026-07-22T16:56:30.58" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+  <threadedComment ref="A70" dT="2026-07-22T16:56:30.58" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
     <text xml:space="preserve">Why is this so different from the other DR solution? I would assume they would be the same…
 </text>
   </threadedComment>
-  <threadedComment ref="A75" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
+  <threadedComment ref="A77" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
     <text>Pretty sure this solution is wrong, but I don’t think I need this case for the paper</text>
   </threadedComment>
-  <threadedComment ref="A81" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+  <threadedComment ref="A83" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
     <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
   </threadedComment>
-  <threadedComment ref="T93" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="T95" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1355,21 +1367,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:V96"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:V98"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" customWidth="1"/>
-    <col min="3" max="3" width="11.453125" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" customWidth="1"/>
-    <col min="15" max="15" width="9.54296875" customWidth="1"/>
-    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.81640625" customWidth="1"/>
+    <col min="1" max="1" width="9.61328125" customWidth="1"/>
+    <col min="3" max="3" width="11.4609375" customWidth="1"/>
+    <col min="5" max="5" width="10.23046875" customWidth="1"/>
+    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.69140625" customWidth="1"/>
+    <col min="9" max="9" width="9.07421875" customWidth="1"/>
+    <col min="15" max="15" width="9.53515625" customWidth="1"/>
+    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1380,7 +1392,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1448,7 +1460,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1512,7 +1524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1576,10 +1588,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1643,7 +1655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -1707,10 +1719,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1774,7 +1786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -1838,10 +1850,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -1905,7 +1917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -1969,10 +1981,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2034,7 +2046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2090,10 +2102,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2157,7 +2169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2221,12 +2233,12 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2237,7 +2249,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2301,10 +2313,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2368,7 +2380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2438,11 +2450,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2506,7 +2518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2570,10 +2582,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2621,7 +2633,7 @@
         <v>0</v>
       </c>
       <c r="P30">
-        <f t="shared" ref="P30:P31" si="5">D30+$P$1</f>
+        <f t="shared" ref="P30:P32" si="5">D30+$P$1</f>
         <v>233712.04614218482</v>
       </c>
       <c r="Q30">
@@ -2637,7 +2649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -2707,2595 +2719,2744 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="S32" s="2"/>
-    </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="7" t="s">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A32" t="s">
+        <v>22</v>
+      </c>
+      <c r="B32" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32">
+        <v>4</v>
+      </c>
+      <c r="D32">
+        <f>J32+K32+L32+M32+N32</f>
+        <v>118576.07841019254</v>
+      </c>
+      <c r="E32">
+        <v>282179.67123290099</v>
+      </c>
+      <c r="F32">
+        <v>0.84579332713576405</v>
+      </c>
+      <c r="G32">
+        <v>19619.107842410202</v>
+      </c>
+      <c r="H32">
+        <v>6176.7328450860596</v>
+      </c>
+      <c r="I32" s="8">
+        <v>1.43619850991576E-5</v>
+      </c>
+      <c r="J32">
+        <v>25795.8407018582</v>
+      </c>
+      <c r="K32">
+        <v>50989.945205476797</v>
+      </c>
+      <c r="L32">
+        <v>20356.5524429125</v>
+      </c>
+      <c r="M32">
+        <v>19971.362105022999</v>
+      </c>
+      <c r="N32">
+        <v>1462.3779549220301</v>
+      </c>
+      <c r="O32">
+        <v>0</v>
+      </c>
+      <c r="P32">
+        <f t="shared" si="5"/>
+        <v>239135.75022918906</v>
+      </c>
+      <c r="Q32">
+        <v>1380.03506977654</v>
+      </c>
+      <c r="R32">
+        <v>33615.943500043497</v>
+      </c>
+      <c r="S32">
+        <v>908.53901351469096</v>
+      </c>
+      <c r="T32">
+        <v>4.5273802587315601E-2</v>
+      </c>
+      <c r="U32">
+        <v>36375.165695697498</v>
+      </c>
+      <c r="V32">
+        <v>277.67302057784298</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="D33">
+        <f>D32-D31</f>
+        <v>785.66289527932531</v>
+      </c>
+      <c r="E33">
+        <f>E32-E31</f>
+        <v>2.4971086531877518E-8</v>
+      </c>
+      <c r="F33">
+        <f>F32-F31</f>
+        <v>2.6907854028540568E-3</v>
+      </c>
+      <c r="G33">
+        <f>G32-G31</f>
+        <v>-221.42920834019969</v>
+      </c>
+      <c r="H33">
+        <f>H32-H31</f>
+        <v>896.09976246881979</v>
+      </c>
+      <c r="I33">
+        <f>I32-I31</f>
+        <v>-4877.4899349639245</v>
+      </c>
+      <c r="J33">
+        <f>J32-J31</f>
+        <v>-4202.8193808354008</v>
+      </c>
+      <c r="K33">
+        <f>K32-K31</f>
+        <v>-87.19067491790338</v>
+      </c>
+      <c r="L33">
+        <f>L32-L31</f>
+        <v>4424.0083944886992</v>
+      </c>
+      <c r="M33">
+        <f>M32-M31</f>
+        <v>625.28660162189772</v>
+      </c>
+      <c r="N33">
+        <f>N32-N31</f>
+        <v>26.377954922030085</v>
+      </c>
+      <c r="O33">
+        <f>O32-O31</f>
+        <v>0</v>
+      </c>
+      <c r="P33">
+        <f>P32-P31</f>
+        <v>785.66289527932531</v>
+      </c>
+      <c r="Q33">
+        <f>Q32-Q31</f>
+        <v>200.21086642008004</v>
+      </c>
+      <c r="R33">
+        <f>R32-R31</f>
+        <v>20835.930555410298</v>
+      </c>
+      <c r="S33">
+        <f>S32-S31</f>
+        <v>397.33849572936299</v>
+      </c>
+      <c r="T33">
+        <f>T32-T31</f>
+        <v>-0.1359304574304484</v>
+      </c>
+      <c r="U33">
+        <f>U32-U31</f>
+        <v>25293.846976061999</v>
+      </c>
+      <c r="V33">
+        <f>V32-V31</f>
+        <v>200.18128127969257</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B33" s="2"/>
-      <c r="S33" s="2"/>
-    </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+      <c r="B35" s="2"/>
+      <c r="S35" s="2"/>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A36" t="s">
         <v>20</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B36" t="s">
         <v>23</v>
       </c>
-      <c r="C34">
-        <v>0</v>
-      </c>
-      <c r="D34">
-        <f>J34+K34+L34+M34+N34</f>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <f>J36+K36+L36+M36+N36</f>
         <v>116993.31924575487</v>
       </c>
-      <c r="E34">
+      <c r="E36">
         <v>282190.859999999</v>
       </c>
-      <c r="F34">
+      <c r="F36">
         <v>0.84033715458764902</v>
       </c>
-      <c r="G34">
+      <c r="G36">
         <v>21182.959346048301</v>
       </c>
-      <c r="H34">
+      <c r="H36">
         <v>6486.2597020478397</v>
       </c>
-      <c r="I34">
+      <c r="I36">
         <v>2466.3619080631902</v>
       </c>
-      <c r="J34">
+      <c r="J36">
         <v>30135.5809561594</v>
       </c>
-      <c r="K34">
+      <c r="K36">
         <v>50845.200000000099</v>
       </c>
-      <c r="L34">
+      <c r="L36">
         <v>15304.405199999899</v>
       </c>
-      <c r="M34">
+      <c r="M36">
         <v>19298.29566</v>
       </c>
-      <c r="N34">
+      <c r="N36">
         <v>1409.83742959549</v>
       </c>
-      <c r="O34">
-        <v>0</v>
-      </c>
-      <c r="P34">
-        <f t="shared" ref="P34:P35" si="6">D34+$P$1</f>
+      <c r="O36">
+        <v>0</v>
+      </c>
+      <c r="P36">
+        <f t="shared" ref="P36:P37" si="6">D36+$P$1</f>
         <v>237552.9910647514</v>
       </c>
-      <c r="Q34">
+      <c r="Q36">
         <v>1102.0926609763501</v>
       </c>
-      <c r="R34">
-        <v>0</v>
-      </c>
-      <c r="U34">
+      <c r="R36">
+        <v>0</v>
+      </c>
+      <c r="U36">
         <v>15.5670440273115</v>
       </c>
-      <c r="V34">
+      <c r="V36">
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A37" t="s">
         <v>22</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B37" t="s">
         <v>23</v>
       </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
-      <c r="D35">
-        <f>J35+K35+L35+M35+N35</f>
+      <c r="C37">
+        <v>0</v>
+      </c>
+      <c r="D37">
+        <f>J37+K37+L37+M37+N37</f>
         <v>125900.82058980259</v>
       </c>
-      <c r="E35">
+      <c r="E37">
         <v>282190.859999999</v>
       </c>
-      <c r="F35">
+      <c r="F37">
         <v>0.87190267497356</v>
       </c>
-      <c r="G35">
+      <c r="G37">
         <v>23139.129735574901</v>
       </c>
-      <c r="H35">
+      <c r="H37">
         <v>6486.2597020478397</v>
       </c>
-      <c r="I35">
+      <c r="I37">
         <v>9417.6928625843393</v>
       </c>
-      <c r="J35">
+      <c r="J37">
         <v>39043.082300207097</v>
       </c>
-      <c r="K35">
+      <c r="K37">
         <v>50845.200000000099</v>
       </c>
-      <c r="L35">
+      <c r="L37">
         <v>15304.405199999899</v>
       </c>
-      <c r="M35">
+      <c r="M37">
         <v>19298.29566</v>
       </c>
-      <c r="N35">
+      <c r="N37">
         <v>1409.83742959549</v>
       </c>
-      <c r="O35">
-        <v>0</v>
-      </c>
-      <c r="P35">
+      <c r="O37">
+        <v>0</v>
+      </c>
+      <c r="P37">
         <f t="shared" si="6"/>
         <v>246460.49240879912</v>
       </c>
-      <c r="Q35">
+      <c r="Q37">
         <v>1102.0926609763501</v>
       </c>
-      <c r="R35">
-        <v>0</v>
-      </c>
-      <c r="U35">
+      <c r="R37">
+        <v>0</v>
+      </c>
+      <c r="U37">
         <v>15.5670440273115</v>
       </c>
-      <c r="V35">
+      <c r="V37">
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A36" s="7"/>
-      <c r="B36" s="2"/>
-      <c r="S36" s="2"/>
-    </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A37" s="3" t="s">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A38" s="7"/>
+      <c r="B38" s="2"/>
+      <c r="S38" s="2"/>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B39" t="s">
         <v>21</v>
       </c>
-      <c r="C37">
+      <c r="C39">
         <v>4</v>
       </c>
-      <c r="D37">
-        <f>J37+K37+L37+M37+N37</f>
+      <c r="D39">
+        <f>J39+K39+L39+M39+N39</f>
         <v>116978.51468315258</v>
       </c>
-      <c r="E37">
+      <c r="E39">
         <v>282179.671254922</v>
       </c>
-      <c r="F37">
+      <c r="F39">
         <v>0.84031800989031202</v>
       </c>
-      <c r="G37">
+      <c r="G39">
         <v>21174.931050348201</v>
       </c>
-      <c r="H37">
+      <c r="H39">
         <v>6483.8014286718599</v>
       </c>
-      <c r="I37">
+      <c r="I39">
         <v>2465.4271592782502</v>
       </c>
-      <c r="J37">
+      <c r="J39">
         <v>30124.159638298399</v>
       </c>
-      <c r="K37">
+      <c r="K39">
         <v>50843.185222512198</v>
       </c>
-      <c r="L37">
+      <c r="L39">
         <v>15303.8016501727</v>
       </c>
-      <c r="M37">
+      <c r="M39">
         <v>19297.530742573799</v>
       </c>
-      <c r="N37">
+      <c r="N39">
         <v>1409.83742959549</v>
       </c>
-      <c r="O37">
-        <v>0</v>
-      </c>
-      <c r="P37">
-        <f t="shared" ref="P37:P38" si="7">D37+$P$1</f>
+      <c r="O39">
+        <v>0</v>
+      </c>
+      <c r="P39">
+        <f t="shared" ref="P39:P40" si="7">D39+$P$1</f>
         <v>237538.1865021491</v>
       </c>
-      <c r="Q37">
+      <c r="Q39">
         <v>1101.67497109485</v>
       </c>
-      <c r="R37">
+      <c r="R39">
         <v>54.604983409531002</v>
       </c>
-      <c r="S37">
+      <c r="S39">
         <v>0.32502966315197002</v>
       </c>
-      <c r="T37">
+      <c r="T39">
         <v>-106.83117764915301</v>
       </c>
-      <c r="U37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A38" s="3" t="s">
+      <c r="U39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B40" t="s">
         <v>21</v>
       </c>
-      <c r="C38">
+      <c r="C40">
         <v>4</v>
       </c>
-      <c r="D38">
-        <f>J38+K38+L38+M38+N38</f>
+      <c r="D40">
+        <f>J40+K40+L40+M40+N40</f>
         <v>122209.93333437521</v>
       </c>
-      <c r="E38">
+      <c r="E40">
         <v>282179.67123287602</v>
       </c>
-      <c r="F38">
+      <c r="F40">
         <v>0.858784478742043</v>
       </c>
-      <c r="G38">
+      <c r="G40">
         <v>22232.9956437156</v>
       </c>
-      <c r="H38">
+      <c r="H40">
         <v>6892.28291987389</v>
       </c>
-      <c r="I38">
+      <c r="I40">
         <v>5063.3926573547897</v>
       </c>
-      <c r="J38">
+      <c r="J40">
         <v>34188.671220944299</v>
       </c>
-      <c r="K38">
+      <c r="K40">
         <v>51137.498573919998</v>
       </c>
-      <c r="L38">
+      <c r="L40">
         <v>16094.7687872735</v>
       </c>
-      <c r="M38">
+      <c r="M40">
         <v>19358.6007623076</v>
       </c>
-      <c r="N38">
+      <c r="N40">
         <v>1430.39398992981</v>
       </c>
-      <c r="O38">
-        <v>0</v>
-      </c>
-      <c r="P38">
+      <c r="O40">
+        <v>0</v>
+      </c>
+      <c r="P40">
         <f t="shared" si="7"/>
         <v>242769.60515337173</v>
       </c>
-      <c r="Q38">
+      <c r="Q40">
         <v>1171.0808202107701</v>
       </c>
-      <c r="R38">
+      <c r="R40">
         <v>13170.183258303599</v>
       </c>
-      <c r="S38">
+      <c r="S40">
         <v>487.784565122358</v>
       </c>
-      <c r="T38">
+      <c r="T40">
         <v>-0.16035717141929801</v>
       </c>
-      <c r="U38">
+      <c r="U40">
         <v>9733.9102750884304</v>
       </c>
-      <c r="V38">
+      <c r="V40">
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A39" s="3"/>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A40" s="7" t="s">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A41" s="3" t="s">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A44" t="s">
         <v>22</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B44" t="s">
         <v>23</v>
       </c>
-      <c r="C42">
-        <v>0</v>
-      </c>
-      <c r="D42">
-        <f>J42+K42+L42+M42+N42</f>
+      <c r="C44">
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <f>J44+K44+L44+M44+N44</f>
         <v>125926.94126070438</v>
       </c>
-      <c r="E42">
+      <c r="E44">
         <v>282190.859999999</v>
       </c>
-      <c r="F42">
+      <c r="F44">
         <v>0.87199523881812102</v>
       </c>
-      <c r="G42">
+      <c r="G44">
         <v>23255.929405575898</v>
       </c>
-      <c r="H42">
+      <c r="H44">
         <v>5559.1797407744398</v>
       </c>
-      <c r="I42">
+      <c r="I44">
         <v>10254.0938247584</v>
       </c>
-      <c r="J42">
+      <c r="J44">
         <v>39069.202971108898</v>
       </c>
-      <c r="K42">
+      <c r="K44">
         <v>50845.200000000099</v>
       </c>
-      <c r="L42">
+      <c r="L44">
         <v>15304.405199999899</v>
       </c>
-      <c r="M42">
+      <c r="M44">
         <v>19298.29566</v>
       </c>
-      <c r="N42">
+      <c r="N44">
         <v>1409.83742959549</v>
       </c>
-      <c r="O42">
-        <v>0</v>
-      </c>
-      <c r="P42">
-        <f t="shared" ref="P42" si="8">D42+$P$1</f>
+      <c r="O44">
+        <v>0</v>
+      </c>
+      <c r="P44">
+        <f t="shared" ref="P44" si="8">D44+$P$1</f>
         <v>246486.61307970091</v>
       </c>
-      <c r="Q42">
+      <c r="Q44">
         <v>1102.0926609763501</v>
       </c>
-      <c r="R42">
-        <v>0</v>
-      </c>
-      <c r="U42">
+      <c r="R44">
+        <v>0</v>
+      </c>
+      <c r="U44">
         <v>15.5670440273115</v>
       </c>
-      <c r="V42">
+      <c r="V44">
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A43" s="3"/>
-    </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A44" s="3" t="s">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A45" s="3"/>
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A47" t="s">
         <v>22</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B47" t="s">
         <v>21</v>
       </c>
-      <c r="C45">
+      <c r="C47">
         <v>4</v>
       </c>
-      <c r="D45">
-        <f>J45+K45+L45+M45+N45</f>
+      <c r="D47">
+        <f>J47+K47+L47+M47+N47</f>
         <v>121548.56732352625</v>
       </c>
-      <c r="E45">
+      <c r="E47">
         <v>282179.67171295901</v>
       </c>
-      <c r="F45">
+      <c r="F47">
         <v>0.85645911177426404</v>
       </c>
-      <c r="G45">
+      <c r="G47">
         <v>21922.670949606902</v>
       </c>
-      <c r="H45">
+      <c r="H47">
         <v>5892.0772301955703</v>
       </c>
-      <c r="I45">
+      <c r="I47">
         <v>5494.1642193806101</v>
       </c>
-      <c r="J45">
+      <c r="J47">
         <v>33308.9123991831</v>
       </c>
-      <c r="K45">
+      <c r="K47">
         <v>51194.9024604468</v>
       </c>
-      <c r="L45">
+      <c r="L47">
         <v>16249.0415258787</v>
       </c>
-      <c r="M45">
+      <c r="M47">
         <v>19370.512083644498</v>
       </c>
-      <c r="N45">
+      <c r="N47">
         <v>1425.19885437316</v>
       </c>
-      <c r="O45">
-        <v>0</v>
-      </c>
-      <c r="P45">
-        <f>D45+$P$1</f>
+      <c r="O47">
+        <v>0</v>
+      </c>
+      <c r="P47">
+        <f>D47+$P$1</f>
         <v>242108.23914252277</v>
       </c>
-      <c r="Q45">
+      <c r="Q47">
         <v>1168.0887035395799</v>
       </c>
-      <c r="R45">
+      <c r="R47">
         <v>12792.663740961099</v>
       </c>
-      <c r="S45">
+      <c r="S47">
         <v>511.70654963844697</v>
       </c>
-      <c r="T45">
+      <c r="T47">
         <v>-0.11339056141074599</v>
       </c>
-      <c r="U45">
+      <c r="U47">
         <v>7320.3796501147199</v>
       </c>
-      <c r="V45">
+      <c r="V47">
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A47" s="1" t="s">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G47" s="4"/>
-    </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A48" s="5" t="s">
+      <c r="G49" s="4"/>
+    </row>
+    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="B50" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C48">
-        <v>0</v>
-      </c>
-      <c r="D48">
-        <f>J48+K48+L48+M48+N48</f>
+      <c r="C50">
+        <v>0</v>
+      </c>
+      <c r="D50">
+        <f>J50+K50+L50+M50+N50</f>
         <v>117853.9906257109</v>
       </c>
-      <c r="E48">
+      <c r="E50">
         <v>282179.67123287602</v>
       </c>
-      <c r="F48">
+      <c r="F50">
         <v>0.84490020632262297</v>
       </c>
-      <c r="G48">
+      <c r="G50">
         <v>23556.420831705898</v>
       </c>
-      <c r="H48">
+      <c r="H50">
         <v>6947.4542183048998</v>
       </c>
-      <c r="I48">
+      <c r="I50">
         <v>913.29198665996</v>
       </c>
-      <c r="J48">
+      <c r="J50">
         <v>31417.167036670799</v>
       </c>
-      <c r="K48">
+      <c r="K50">
         <v>50843.184005923598</v>
       </c>
-      <c r="L48">
+      <c r="L50">
         <v>15303.798385783</v>
       </c>
-      <c r="M48">
+      <c r="M50">
         <v>19297.5304894482</v>
       </c>
-      <c r="N48">
+      <c r="N50">
         <v>992.31070788530405</v>
       </c>
-      <c r="O48">
-        <v>0</v>
-      </c>
-      <c r="P48">
-        <f t="shared" ref="P48:P55" si="9">D48+$P$1</f>
+      <c r="O50">
+        <v>0</v>
+      </c>
+      <c r="P50">
+        <f t="shared" ref="P50:P57" si="9">D50+$P$1</f>
         <v>238413.66244470741</v>
       </c>
-      <c r="Q48">
+      <c r="Q50">
         <v>1102.6552392369899</v>
       </c>
-      <c r="R48">
-        <v>0</v>
-      </c>
-      <c r="S48">
-        <v>0</v>
-      </c>
-      <c r="T48">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A49" s="5" t="s">
+      <c r="R50">
+        <v>0</v>
+      </c>
+      <c r="S50">
+        <v>0</v>
+      </c>
+      <c r="T50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B51" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C49">
-        <v>0</v>
-      </c>
-      <c r="D49">
-        <f>J49+K49+L49+M49+N49</f>
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <f>J51+K51+L51+M51+N51</f>
         <v>188012.7674304971</v>
       </c>
-      <c r="E49">
+      <c r="E51">
         <v>282179.67123287602</v>
       </c>
-      <c r="F49">
+      <c r="F51">
         <v>1.09353178385</v>
       </c>
-      <c r="G49">
+      <c r="G51">
         <v>89520.694507565597</v>
       </c>
-      <c r="H49">
+      <c r="H51">
         <v>6971.3813103080802</v>
       </c>
-      <c r="I49">
+      <c r="I51">
         <v>5083.8680235841202</v>
       </c>
-      <c r="J49">
+      <c r="J51">
         <v>101575.943841457</v>
       </c>
-      <c r="K49">
+      <c r="K51">
         <v>50843.184005923598</v>
       </c>
-      <c r="L49">
+      <c r="L51">
         <v>15303.798385783</v>
       </c>
-      <c r="M49">
+      <c r="M51">
         <v>19297.5304894482</v>
       </c>
-      <c r="N49">
+      <c r="N51">
         <v>992.31070788530405</v>
       </c>
-      <c r="O49">
-        <v>0</v>
-      </c>
-      <c r="P49">
+      <c r="O51">
+        <v>0</v>
+      </c>
+      <c r="P51">
         <f t="shared" si="9"/>
         <v>308572.43924949365</v>
       </c>
-      <c r="Q49">
+      <c r="Q51">
         <v>1106.4527933521999</v>
       </c>
-      <c r="R49">
+      <c r="R51">
         <v>3451.9307168288801</v>
       </c>
-      <c r="S49">
+      <c r="S51">
         <v>20.547206647791</v>
       </c>
-      <c r="T49">
+      <c r="T51">
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A50" s="3"/>
-      <c r="G50" s="4"/>
-    </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A52" s="3"/>
+      <c r="G52" s="4"/>
+    </row>
+    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A53" t="s">
         <v>20</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B53" t="s">
         <v>21</v>
       </c>
-      <c r="C51">
-        <v>0</v>
-      </c>
-      <c r="D51">
-        <f>J51+K51+L51+M51+N51</f>
+      <c r="C53">
+        <v>0</v>
+      </c>
+      <c r="D53">
+        <f>J53+K53+L53+M53+N53</f>
         <v>118024.73030148289</v>
       </c>
-      <c r="E51">
+      <c r="E53">
         <v>282179.67123286898</v>
       </c>
-      <c r="F51">
+      <c r="F53">
         <v>0.845505280653571</v>
       </c>
-      <c r="G51" s="4">
+      <c r="G53" s="4">
         <v>23683.129427060001</v>
       </c>
-      <c r="H51">
+      <c r="H53">
         <v>6986.3695969997798</v>
       </c>
-      <c r="I51">
+      <c r="I53">
         <v>918.40768838365295</v>
       </c>
-      <c r="J51">
+      <c r="J53">
         <v>31587.906712443499</v>
       </c>
-      <c r="K51">
+      <c r="K53">
         <v>50843.1840059237</v>
       </c>
-      <c r="L51">
+      <c r="L53">
         <v>15303.7983857823</v>
       </c>
-      <c r="M51">
+      <c r="M53">
         <v>19297.530489448101</v>
       </c>
-      <c r="N51">
+      <c r="N53">
         <v>992.31070788530405</v>
       </c>
-      <c r="O51">
-        <v>0</v>
-      </c>
-      <c r="P51">
+      <c r="O53">
+        <v>0</v>
+      </c>
+      <c r="P53">
         <f t="shared" si="9"/>
         <v>238584.40212047941</v>
       </c>
-      <c r="Q51">
+      <c r="Q53">
         <v>1108.83163779344</v>
       </c>
-      <c r="R51">
-        <v>0</v>
-      </c>
-      <c r="S51">
+      <c r="R53">
+        <v>0</v>
+      </c>
+      <c r="S53">
         <v>230512.59606633501</v>
       </c>
-      <c r="T51">
+      <c r="T53">
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A54" t="s">
         <v>22</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B54" t="s">
         <v>21</v>
       </c>
-      <c r="C52">
-        <v>0</v>
-      </c>
-      <c r="D52">
-        <f>J52+K52+L52+M52+N52</f>
+      <c r="C54">
+        <v>0</v>
+      </c>
+      <c r="D54">
+        <f>J54+K54+L54+M54+N54</f>
         <v>172556.33199183288</v>
       </c>
-      <c r="E52">
+      <c r="E54">
         <v>282179.67123287701</v>
       </c>
-      <c r="F52">
+      <c r="F54">
         <v>1.03875662810921</v>
       </c>
-      <c r="G52">
+      <c r="G54">
         <v>73514.1870928641</v>
       </c>
-      <c r="H52">
+      <c r="H54">
         <v>7482.8438362204697</v>
       </c>
-      <c r="I52">
+      <c r="I54">
         <v>4044.9309872213798</v>
       </c>
-      <c r="J52">
+      <c r="J54">
         <v>85041.961916305998</v>
       </c>
-      <c r="K52">
+      <c r="K54">
         <v>51119.832654572398</v>
       </c>
-      <c r="L52">
+      <c r="L54">
         <v>16047.2916290263</v>
       </c>
-      <c r="M52">
+      <c r="M54">
         <v>19354.9350840429</v>
       </c>
-      <c r="N52">
+      <c r="N54">
         <v>992.31070788530405</v>
       </c>
-      <c r="O52">
-        <v>0</v>
-      </c>
-      <c r="P52">
+      <c r="O54">
+        <v>0</v>
+      </c>
+      <c r="P54">
         <f t="shared" si="9"/>
         <v>293116.00381082937</v>
       </c>
-      <c r="Q52">
+      <c r="Q54">
         <v>1187.62883512946</v>
       </c>
-      <c r="R52">
+      <c r="R54">
         <v>9393.8913494494009</v>
       </c>
-      <c r="S52">
+      <c r="S54">
         <v>260.94142637359403</v>
       </c>
-      <c r="T52">
+      <c r="T54">
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="G53" s="4"/>
-    </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A54" s="3" t="s">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="G55" s="4"/>
+    </row>
+    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B56" t="s">
         <v>21</v>
       </c>
-      <c r="C54">
+      <c r="C56">
         <v>4</v>
       </c>
-      <c r="D54">
-        <f>J54+K54+L54+M54+N54</f>
+      <c r="D56">
+        <f>J56+K56+L56+M56+N56</f>
         <v>117826.0601945299</v>
       </c>
-      <c r="E54">
+      <c r="E56">
         <v>282179.67123287602</v>
       </c>
-      <c r="F54">
+      <c r="F56">
         <v>0.84480122530439805</v>
       </c>
-      <c r="G54" s="4">
+      <c r="G56" s="4">
         <v>23535.478746437901</v>
       </c>
-      <c r="H54">
+      <c r="H56">
         <v>6941.2778055266899</v>
       </c>
-      <c r="I54">
+      <c r="I56">
         <v>912.48005352310201</v>
       </c>
-      <c r="J54">
+      <c r="J56">
         <v>31389.236605487698</v>
       </c>
-      <c r="K54">
+      <c r="K56">
         <v>50843.184005923998</v>
       </c>
-      <c r="L54">
+      <c r="L56">
         <v>15303.798385784499</v>
       </c>
-      <c r="M54">
+      <c r="M56">
         <v>19297.5304894484</v>
       </c>
-      <c r="N54">
+      <c r="N56">
         <v>992.31070788530405</v>
       </c>
-      <c r="O54">
-        <v>0</v>
-      </c>
-      <c r="P54">
+      <c r="O56">
+        <v>0</v>
+      </c>
+      <c r="P56">
         <f t="shared" si="9"/>
         <v>238385.73201352643</v>
       </c>
-      <c r="Q54">
-        <v>0</v>
-      </c>
-      <c r="R54">
-        <v>0</v>
-      </c>
-      <c r="S54">
-        <v>0</v>
-      </c>
-      <c r="T54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
+      <c r="Q56">
+        <v>0</v>
+      </c>
+      <c r="R56">
+        <v>0</v>
+      </c>
+      <c r="S56">
+        <v>0</v>
+      </c>
+      <c r="T56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A57" t="s">
         <v>22</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B57" t="s">
         <v>21</v>
       </c>
-      <c r="C55">
+      <c r="C57">
         <v>4</v>
       </c>
-      <c r="D55">
-        <f>J55+K55+L55+M55+N55</f>
+      <c r="D57">
+        <f>J57+K57+L57+M57+N57</f>
         <v>125434.46212050831</v>
       </c>
-      <c r="E55">
+      <c r="E57">
         <v>282179.67123444699</v>
       </c>
-      <c r="F55">
+      <c r="F57">
         <v>0.87159189967643702</v>
       </c>
-      <c r="G55" s="4">
+      <c r="G57" s="4">
         <v>21072.189860718699</v>
       </c>
-      <c r="H55">
+      <c r="H57">
         <v>9188.7245080883695</v>
       </c>
-      <c r="I55">
+      <c r="I57">
         <v>2618.8827210474601</v>
       </c>
-      <c r="J55">
+      <c r="J57">
         <v>32879.797089854597</v>
       </c>
-      <c r="K55">
+      <c r="K57">
         <v>50904.118537438801</v>
       </c>
-      <c r="L55">
+      <c r="L57">
         <v>20591.7266090095</v>
       </c>
-      <c r="M55">
+      <c r="M57">
         <v>20017.890938119701</v>
       </c>
-      <c r="N55">
+      <c r="N57">
         <v>1040.9289460857101</v>
       </c>
-      <c r="O55">
-        <v>0</v>
-      </c>
-      <c r="P55">
+      <c r="O57">
+        <v>0</v>
+      </c>
+      <c r="P57">
         <f t="shared" si="9"/>
         <v>245994.13393950483</v>
       </c>
-      <c r="Q55">
+      <c r="Q57">
         <v>1458.3752411216699</v>
       </c>
-      <c r="R55">
+      <c r="R57">
         <v>35012.612233571497</v>
       </c>
-      <c r="S55">
+      <c r="S57">
         <v>875.31530583928895</v>
       </c>
-      <c r="T55">
+      <c r="T57">
         <v>0.51444695802960605</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" s="1" t="s">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G57" s="4"/>
-    </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A58" s="2" t="s">
+      <c r="G59" s="4"/>
+    </row>
+    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B60" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C58">
+      <c r="C60">
         <v>2</v>
       </c>
-      <c r="D58">
-        <f>J58+K58+L58+M58+N58</f>
+      <c r="D60">
+        <f>J60+K60+L60+M60+N60</f>
         <v>119635.09208261623</v>
       </c>
-      <c r="E58">
+      <c r="E60">
         <v>282495</v>
       </c>
-      <c r="F58">
+      <c r="F60">
         <v>0.83903831831993503</v>
       </c>
-      <c r="G58" s="4">
+      <c r="G60" s="4">
         <v>20221.889710343999</v>
       </c>
-      <c r="H58">
+      <c r="H60">
         <v>6553.7440767980397</v>
       </c>
-      <c r="I58">
+      <c r="I60">
         <v>6160.4249909476703</v>
       </c>
-      <c r="J58">
+      <c r="J60">
         <v>32936.058778089697</v>
       </c>
-      <c r="K58">
+      <c r="K60">
         <v>50939.5611113743</v>
       </c>
-      <c r="L58">
+      <c r="L60">
         <v>15427.2204868183</v>
       </c>
-      <c r="M58">
+      <c r="M60">
         <v>19327.3039306102</v>
       </c>
-      <c r="N58">
+      <c r="N60">
         <v>1004.9477757237401</v>
       </c>
-      <c r="O58">
+      <c r="O60">
         <v>3157.9970999842499</v>
       </c>
-      <c r="P58">
-        <f t="shared" ref="P58" si="10">D58+$P$1</f>
+      <c r="P60">
+        <f t="shared" ref="P60" si="10">D60+$P$1</f>
         <v>240194.76390161275</v>
       </c>
-      <c r="Q58">
+      <c r="Q60">
         <v>1464.2687322859999</v>
       </c>
-      <c r="R58">
+      <c r="R60">
         <v>8672.9882445954008</v>
       </c>
-      <c r="S58">
+      <c r="S60">
         <v>346.91952978381602</v>
       </c>
-      <c r="T58">
+      <c r="T60">
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A59" s="3" t="s">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B59" s="3" t="s">
+      <c r="B61" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C59">
+      <c r="C61">
         <v>4</v>
       </c>
-      <c r="D59">
-        <f>J59+K59+L59+M59+N59-O59</f>
+      <c r="D61">
+        <f>J61+K61+L61+M61+N61-O61</f>
         <v>109562.97527837555</v>
       </c>
-      <c r="E59">
+      <c r="E61">
         <v>282179.67123287602</v>
       </c>
-      <c r="F59">
+      <c r="F61">
         <v>0.81689091571482797</v>
       </c>
-      <c r="G59" s="4">
+      <c r="G61" s="4">
         <v>20285.098342207999</v>
       </c>
-      <c r="H59">
+      <c r="H61">
         <v>6552.6722224723899</v>
       </c>
-      <c r="I59">
+      <c r="I61">
         <v>6068.9240568166097</v>
       </c>
-      <c r="J59">
+      <c r="J61">
         <v>32906.694621497001</v>
       </c>
-      <c r="K59">
+      <c r="K61">
         <v>50843.184005923598</v>
       </c>
-      <c r="L59">
+      <c r="L61">
         <v>16378.7983857829</v>
       </c>
-      <c r="M59">
+      <c r="M61">
         <v>19449.350489448301</v>
       </c>
-      <c r="N59">
+      <c r="N61">
         <v>1004.9477757237401</v>
       </c>
-      <c r="O59">
+      <c r="O61">
         <f>1102*5*2</f>
         <v>11020</v>
       </c>
-      <c r="P59">
-        <f>D59+$P$1</f>
+      <c r="P61">
+        <f>D61+$P$1</f>
         <v>230122.64709737207</v>
       </c>
-      <c r="Q59">
+      <c r="Q61">
         <v>1464.02925348484</v>
       </c>
-      <c r="R59">
+      <c r="R61">
         <v>26064.489084194902</v>
       </c>
-      <c r="S59">
+      <c r="S61">
         <v>407.257641940545</v>
       </c>
-      <c r="T59">
+      <c r="T61">
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A60" s="3" t="s">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A62" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B60" s="3" t="s">
+      <c r="B62" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C60">
+      <c r="C62">
         <v>4</v>
       </c>
-      <c r="D60">
+      <c r="D62">
         <v>106092.92029140001</v>
       </c>
-      <c r="E60">
+      <c r="E62">
         <v>282179.67123287602</v>
       </c>
-      <c r="F60">
+      <c r="F62">
         <v>0.80673743017586796</v>
       </c>
-      <c r="G60">
+      <c r="G62">
         <v>19617.269555424798</v>
       </c>
-      <c r="H60">
+      <c r="H62">
         <v>6177.79087142139</v>
       </c>
-      <c r="I60" s="8">
+      <c r="I62" s="8">
         <v>1.4897343661976701E-5</v>
       </c>
-      <c r="J60">
+      <c r="J62">
         <v>25795.060441743601</v>
       </c>
-      <c r="K60">
+      <c r="K62">
         <v>50989.945229661498</v>
       </c>
-      <c r="L60">
+      <c r="L62">
         <v>20356.552509954701</v>
       </c>
-      <c r="M60">
+      <c r="M62">
         <v>19971.3621100407</v>
       </c>
-      <c r="N60">
+      <c r="N62">
         <v>1462.3779549220301</v>
       </c>
-      <c r="O60">
+      <c r="O62">
         <v>11020</v>
       </c>
-      <c r="P60">
+      <c r="P62">
         <v>227644.90281828199</v>
       </c>
-      <c r="Q60">
+      <c r="Q62">
         <v>1380.27146414547</v>
       </c>
-      <c r="R60">
+      <c r="R62">
         <v>33980.634383525299</v>
       </c>
-      <c r="S60">
+      <c r="S62">
         <v>943.906510653483</v>
       </c>
-      <c r="T60">
+      <c r="T62">
         <v>0.36911323114551098</v>
       </c>
-      <c r="U60">
+      <c r="U62">
         <v>36719.7300995962</v>
       </c>
-      <c r="V60">
+      <c r="V62">
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A63" t="s">
         <v>22</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B63" t="s">
         <v>21</v>
       </c>
-      <c r="C61">
+      <c r="C63">
         <v>4</v>
       </c>
-      <c r="D61">
+      <c r="D63">
         <v>106606.33139463799</v>
       </c>
-      <c r="E61">
+      <c r="E63">
         <v>282179.67123277002</v>
       </c>
-      <c r="F61">
+      <c r="F63">
         <v>0.80855687769694595</v>
       </c>
-      <c r="G61">
+      <c r="G63">
         <v>19403.054157778199</v>
       </c>
-      <c r="H61">
+      <c r="H63">
         <v>5553.2925107720503</v>
       </c>
-      <c r="I61">
+      <c r="I63">
         <v>4877.88612389215</v>
       </c>
-      <c r="J61">
+      <c r="J63">
         <v>29834.232792442399</v>
       </c>
-      <c r="K61">
+      <c r="K63">
         <v>51173.670096007401</v>
       </c>
-      <c r="L61">
+      <c r="L63">
         <v>17123.646419717399</v>
       </c>
-      <c r="M61">
+      <c r="M63">
         <v>19494.782086470699</v>
       </c>
-      <c r="N61">
+      <c r="N63">
         <v>1435.62713867346</v>
       </c>
-      <c r="O61">
+      <c r="O63">
         <v>11020</v>
       </c>
-      <c r="P61">
+      <c r="P63">
         <v>228158.313921519</v>
       </c>
-      <c r="Q61">
+      <c r="Q63">
         <v>1240.7430631340701</v>
       </c>
-      <c r="R61">
+      <c r="R63">
         <v>17914.482434871101</v>
       </c>
-      <c r="S61">
+      <c r="S63">
         <v>398.09960966380203</v>
       </c>
-      <c r="T61">
+      <c r="T63">
         <v>0.67297738075987301</v>
       </c>
-      <c r="U61">
+      <c r="U63">
         <v>13163.232180323101</v>
       </c>
-      <c r="V61">
+      <c r="V63">
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A62" s="3"/>
-      <c r="B62" s="3"/>
-      <c r="D62">
-        <f>D61-D60</f>
+    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A64" s="3"/>
+      <c r="B64" s="3"/>
+      <c r="D64">
+        <f>D63-D62</f>
         <v>513.41110323798785</v>
       </c>
-      <c r="E62">
-        <f t="shared" ref="E62:V62" si="11">E61-E60</f>
+      <c r="E64">
+        <f t="shared" ref="E64:V64" si="11">E63-E62</f>
         <v>-1.0599615052342415E-7</v>
       </c>
-      <c r="F62">
+      <c r="F64">
         <f t="shared" si="11"/>
         <v>1.8194475210779881E-3</v>
       </c>
-      <c r="G62">
+      <c r="G64">
         <f t="shared" si="11"/>
         <v>-214.21539764659974</v>
       </c>
-      <c r="H62">
+      <c r="H64">
         <f t="shared" si="11"/>
         <v>-624.4983606493397</v>
       </c>
-      <c r="I62">
+      <c r="I64">
         <f t="shared" si="11"/>
         <v>4877.8861089948059</v>
       </c>
-      <c r="J62">
+      <c r="J64">
         <f t="shared" si="11"/>
         <v>4039.1723506987983</v>
       </c>
-      <c r="K62">
+      <c r="K64">
         <f t="shared" si="11"/>
         <v>183.72486634590314</v>
       </c>
-      <c r="L62">
+      <c r="L64">
         <f t="shared" si="11"/>
         <v>-3232.9060902373021</v>
       </c>
-      <c r="M62">
+      <c r="M64">
         <f t="shared" si="11"/>
         <v>-476.58002357000078</v>
       </c>
-      <c r="N62">
+      <c r="N64">
         <f t="shared" si="11"/>
         <v>-26.750816248570118</v>
       </c>
-      <c r="O62">
+      <c r="O64">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="P62">
+      <c r="P64">
         <f t="shared" si="11"/>
         <v>513.41110323701287</v>
       </c>
-      <c r="Q62">
+      <c r="Q64">
         <f t="shared" si="11"/>
         <v>-139.52840101139986</v>
       </c>
-      <c r="R62">
+      <c r="R64">
         <f t="shared" si="11"/>
         <v>-16066.151948654198</v>
       </c>
-      <c r="S62">
+      <c r="S64">
         <f t="shared" si="11"/>
         <v>-545.80690098968103</v>
       </c>
-      <c r="T62">
+      <c r="T64">
         <f t="shared" si="11"/>
         <v>0.30386414961436203</v>
       </c>
-      <c r="U62">
+      <c r="U64">
         <f t="shared" si="11"/>
         <v>-23556.497919273097</v>
       </c>
-      <c r="V62">
+      <c r="V64">
         <f t="shared" si="11"/>
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A63" s="1" t="s">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A65" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G63" s="4"/>
-    </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A64" s="3" t="s">
+      <c r="G65" s="4"/>
+    </row>
+    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A66" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B64" s="3" t="s">
+      <c r="B66" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C64" s="3">
-        <v>0</v>
-      </c>
-      <c r="G64" s="4"/>
-    </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
+      <c r="C66" s="3">
+        <v>0</v>
+      </c>
+      <c r="G66" s="4"/>
+    </row>
+    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A67" t="s">
         <v>22</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B67" t="s">
         <v>23</v>
       </c>
-      <c r="C65">
-        <v>0</v>
-      </c>
-      <c r="D65">
-        <f>J65+K65+L65+M65+N65-O65</f>
+      <c r="C67">
+        <v>0</v>
+      </c>
+      <c r="D67">
+        <f>J67+K67+L67+M67+N67-O67</f>
         <v>125093.23428318274</v>
       </c>
-      <c r="E65">
+      <c r="E67">
         <v>282190.859999999</v>
       </c>
-      <c r="F65">
+      <c r="F67">
         <v>0.86904083066499505</v>
       </c>
-      <c r="G65">
+      <c r="G67">
         <v>24203.497764766002</v>
       </c>
-      <c r="H65">
+      <c r="H67">
         <v>4932.7238161263904</v>
       </c>
-      <c r="I65">
+      <c r="I67">
         <v>9098.5748223234004</v>
       </c>
-      <c r="J65">
+      <c r="J67">
         <v>38234.796403215798</v>
       </c>
-      <c r="K65">
+      <c r="K67">
         <v>50845.200000000099</v>
       </c>
-      <c r="L65">
+      <c r="L67">
         <v>15304.405199999899</v>
       </c>
-      <c r="M65">
+      <c r="M67">
         <v>19298.29566</v>
       </c>
-      <c r="N65">
+      <c r="N67">
         <v>1409.83742959549</v>
       </c>
-      <c r="O65">
+      <c r="O67">
         <v>-0.69959037146548997</v>
       </c>
-      <c r="P65">
-        <f>D65+$P$1</f>
+      <c r="P67">
+        <f>D67+$P$1</f>
         <v>245652.90610217926</v>
       </c>
-      <c r="Q65">
+      <c r="Q67">
         <v>1102.0926609763501</v>
       </c>
-      <c r="R65">
-        <v>0</v>
-      </c>
-      <c r="U65">
+      <c r="R67">
+        <v>0</v>
+      </c>
+      <c r="U67">
         <v>15.5670440273115</v>
       </c>
-      <c r="V65">
+      <c r="V67">
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A66" s="3"/>
-      <c r="B66" s="3"/>
-      <c r="C66" s="3"/>
-      <c r="G66" s="4"/>
-    </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="3" t="s">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A68" s="3"/>
+      <c r="B68" s="3"/>
+      <c r="C68" s="3"/>
+      <c r="G68" s="4"/>
+    </row>
+    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A69" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B67" s="3" t="s">
+      <c r="B69" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C67" s="3">
+      <c r="C69" s="3">
         <v>4</v>
       </c>
-      <c r="G67" s="4"/>
-    </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
+      <c r="G69" s="4"/>
+    </row>
+    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A70" t="s">
         <v>22</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B70" t="s">
         <v>21</v>
       </c>
-      <c r="C68">
+      <c r="C70">
         <v>4</v>
       </c>
-      <c r="D68">
+      <c r="D70">
         <v>108832.74020782999</v>
       </c>
-      <c r="E68">
+      <c r="E70">
         <v>282179.67123306898</v>
       </c>
-      <c r="F68">
+      <c r="F70">
         <v>0.81644691741250097</v>
       </c>
-      <c r="G68">
+      <c r="G70">
         <v>19728.523245555101</v>
       </c>
-      <c r="H68">
+      <c r="H70">
         <v>6281.7321988746498</v>
       </c>
-      <c r="I68" s="8">
+      <c r="I70" s="8">
         <v>9.8877442286147301E-6</v>
       </c>
-      <c r="J68">
+      <c r="J70">
         <v>26010.255454317499</v>
       </c>
-      <c r="K68">
+      <c r="K70">
         <v>50944.9452054754</v>
       </c>
-      <c r="L68">
+      <c r="L70">
         <v>20235.614943009699</v>
       </c>
-      <c r="M68">
+      <c r="M70">
         <v>19962.024605027898</v>
       </c>
-      <c r="N68">
+      <c r="N70">
         <v>1462.3779549220301</v>
       </c>
-      <c r="O68">
+      <c r="O70">
         <v>8320.1</v>
       </c>
-      <c r="P68">
+      <c r="P70">
         <v>230384.72273471201</v>
       </c>
-      <c r="Q68">
+      <c r="Q70">
         <v>1403.49453592792</v>
       </c>
-      <c r="R68">
+      <c r="R70">
         <v>34518.506961381201</v>
       </c>
-      <c r="S68">
+      <c r="S70">
         <v>841.91480393612801</v>
       </c>
-      <c r="T68">
+      <c r="T70">
         <v>0.38784649209264499</v>
       </c>
-      <c r="U68">
+      <c r="U70">
         <v>38264.627438579002</v>
       </c>
-      <c r="V68">
+      <c r="V70">
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="5"/>
-      <c r="B69" s="5"/>
-      <c r="D69">
-        <f>D68-D65</f>
+    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A71" s="5"/>
+      <c r="B71" s="5"/>
+      <c r="D71">
+        <f>D70-D67</f>
         <v>-16260.494075352748</v>
       </c>
-      <c r="E69">
-        <f t="shared" ref="E69:V69" si="12">E68-E65</f>
+      <c r="E71">
+        <f t="shared" ref="E71:V71" si="12">E70-E67</f>
         <v>-11.188766930019483</v>
       </c>
-      <c r="F69">
+      <c r="F71">
         <f t="shared" si="12"/>
         <v>-5.2593913252494073E-2</v>
       </c>
-      <c r="G69">
+      <c r="G71">
         <f t="shared" si="12"/>
         <v>-4474.9745192109003</v>
       </c>
-      <c r="H69">
+      <c r="H71">
         <f t="shared" si="12"/>
         <v>1349.0083827482595</v>
       </c>
-      <c r="I69">
+      <c r="I71">
         <f t="shared" si="12"/>
         <v>-9098.574812435656</v>
       </c>
-      <c r="J69">
+      <c r="J71">
         <f t="shared" si="12"/>
         <v>-12224.540948898299</v>
       </c>
-      <c r="K69">
+      <c r="K71">
         <f t="shared" si="12"/>
         <v>99.745205475301191</v>
       </c>
-      <c r="L69">
+      <c r="L71">
         <f t="shared" si="12"/>
         <v>4931.2097430098001</v>
       </c>
-      <c r="M69">
+      <c r="M71">
         <f t="shared" si="12"/>
         <v>663.72894502789859</v>
       </c>
-      <c r="N69">
+      <c r="N71">
         <f t="shared" si="12"/>
         <v>52.540525326540092</v>
       </c>
-      <c r="O69">
+      <c r="O71">
         <f t="shared" si="12"/>
         <v>8320.7995903714655</v>
       </c>
-      <c r="P69">
+      <c r="P71">
         <f t="shared" si="12"/>
         <v>-15268.183367467253</v>
       </c>
-      <c r="Q69">
+      <c r="Q71">
         <f t="shared" si="12"/>
         <v>301.40187495156988</v>
       </c>
-      <c r="R69">
+      <c r="R71">
         <f t="shared" si="12"/>
         <v>34518.506961381201</v>
       </c>
-      <c r="S69">
+      <c r="S71">
         <f t="shared" si="12"/>
         <v>841.91480393612801</v>
       </c>
-      <c r="T69">
+      <c r="T71">
         <f t="shared" si="12"/>
         <v>0.38784649209264499</v>
       </c>
-      <c r="U69">
+      <c r="U71">
         <f t="shared" si="12"/>
         <v>38249.060394551692</v>
       </c>
-      <c r="V69">
+      <c r="V71">
         <f t="shared" si="12"/>
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A70" s="1" t="s">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A72" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A71" s="3" t="s">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A73" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B71" s="3" t="s">
+      <c r="B73" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C71">
-        <v>0</v>
-      </c>
-      <c r="D71">
-        <f>J71+K71+L71+M71+N71</f>
+      <c r="C73">
+        <v>0</v>
+      </c>
+      <c r="D73">
+        <f>J73+K73+L73+M73+N73</f>
         <v>116023.2890300647</v>
       </c>
-      <c r="E71">
+      <c r="E73">
         <v>282179.67123287602</v>
       </c>
-      <c r="F71">
+      <c r="F73">
         <v>0.83841249022441</v>
       </c>
-      <c r="G71">
+      <c r="G73">
         <v>20114.092712805999</v>
       </c>
-      <c r="H71">
+      <c r="H73">
         <v>6942.2846600808298</v>
       </c>
-      <c r="I71">
+      <c r="I73">
         <v>2530.0880681377598</v>
       </c>
-      <c r="J71">
+      <c r="J73">
         <v>29586.4654410246</v>
       </c>
-      <c r="K71">
+      <c r="K73">
         <v>50843.184005923598</v>
       </c>
-      <c r="L71">
+      <c r="L73">
         <v>15303.798385783</v>
       </c>
-      <c r="M71">
+      <c r="M73">
         <v>19297.5304894482</v>
       </c>
-      <c r="N71">
+      <c r="N73">
         <v>992.31070788530405</v>
       </c>
-      <c r="O71">
-        <v>0</v>
-      </c>
-      <c r="P71">
-        <f t="shared" ref="P71:P72" si="13">D71+$P$1</f>
+      <c r="O73">
+        <v>0</v>
+      </c>
+      <c r="P73">
+        <f t="shared" ref="P73:P74" si="13">D73+$P$1</f>
         <v>236582.9608490612</v>
       </c>
-      <c r="Q71">
+      <c r="Q73">
         <v>1101.8347602124099</v>
       </c>
-      <c r="R71">
-        <v>0</v>
-      </c>
-      <c r="S71">
-        <v>0</v>
-      </c>
-      <c r="T71">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A72" s="3" t="s">
+      <c r="R73">
+        <v>0</v>
+      </c>
+      <c r="S73">
+        <v>0</v>
+      </c>
+      <c r="T73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A74" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B72" s="3" t="s">
+      <c r="B74" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C72">
-        <v>0</v>
-      </c>
-      <c r="D72">
-        <f>J72+K72+L72+M72+N72</f>
+      <c r="C74">
+        <v>0</v>
+      </c>
+      <c r="D74">
+        <f>J74+K74+L74+M74+N74</f>
         <v>125763.55741733511</v>
       </c>
-      <c r="E72">
+      <c r="E74">
         <v>282179.67125180899</v>
       </c>
-      <c r="F72">
+      <c r="F74">
         <v>0.87293045648394496</v>
       </c>
-      <c r="G72">
+      <c r="G74">
         <v>22626.697961956499</v>
       </c>
-      <c r="H72">
+      <c r="H74">
         <v>7102.5767129513297</v>
       </c>
-      <c r="I72">
+      <c r="I74">
         <v>9597.4591384874802</v>
       </c>
-      <c r="J72">
+      <c r="J74">
         <v>39326.733813395302</v>
       </c>
-      <c r="K72">
+      <c r="K74">
         <v>50843.184011688398</v>
       </c>
-      <c r="L72">
+      <c r="L74">
         <v>15303.798393134501</v>
       </c>
-      <c r="M72">
+      <c r="M74">
         <v>19297.530491231599</v>
       </c>
-      <c r="N72">
+      <c r="N74">
         <v>992.31070788530405</v>
       </c>
-      <c r="O72">
-        <v>0</v>
-      </c>
-      <c r="P72">
+      <c r="O74">
+        <v>0</v>
+      </c>
+      <c r="P74">
         <f t="shared" si="13"/>
         <v>246323.22923633162</v>
       </c>
-      <c r="Q72">
+      <c r="Q74">
         <v>1127.27501714903</v>
       </c>
-      <c r="R72">
-        <v>0</v>
-      </c>
-      <c r="S72">
-        <v>0</v>
-      </c>
-      <c r="T72">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A73" s="1"/>
-    </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
+      <c r="R74">
+        <v>0</v>
+      </c>
+      <c r="S74">
+        <v>0</v>
+      </c>
+      <c r="T74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A75" s="1"/>
+    </row>
+    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A76" t="s">
         <v>20</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B76" t="s">
         <v>21</v>
       </c>
-      <c r="C74">
+      <c r="C76">
         <v>2</v>
       </c>
-      <c r="D74">
-        <f>J74+K74+L74+M74+N74</f>
+      <c r="D76">
+        <f>J76+K76+L76+M76+N76</f>
         <v>116706.4157905087</v>
       </c>
-      <c r="E74">
+      <c r="E76">
         <v>282179.67125387199</v>
       </c>
-      <c r="F74">
+      <c r="F76">
         <v>0.840833383054163</v>
       </c>
-      <c r="G74" s="4">
+      <c r="G76" s="4">
         <v>20578.507216446698</v>
       </c>
-      <c r="H74">
+      <c r="H76">
         <v>7102.57515066207</v>
       </c>
-      <c r="I74">
+      <c r="I76">
         <v>2588.5052959285099</v>
       </c>
-      <c r="J74">
+      <c r="J76">
         <v>30269.587663037299</v>
       </c>
-      <c r="K74">
+      <c r="K76">
         <v>50843.185173268597</v>
       </c>
-      <c r="L74">
+      <c r="L76">
         <v>15303.8015139941</v>
       </c>
-      <c r="M74">
+      <c r="M76">
         <v>19297.530732323401</v>
       </c>
-      <c r="N74">
+      <c r="N76">
         <v>992.31070788530405</v>
       </c>
-      <c r="O74">
-        <v>0</v>
-      </c>
-      <c r="P74">
-        <f t="shared" ref="P74:P75" si="14">D74+$P$1</f>
+      <c r="O76">
+        <v>0</v>
+      </c>
+      <c r="P76">
+        <f t="shared" ref="P76:P77" si="14">D76+$P$1</f>
         <v>237266.08760950522</v>
       </c>
-      <c r="Q74">
+      <c r="Q76">
         <v>1127.2750356983099</v>
       </c>
-      <c r="R74">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A75" s="2" t="s">
+      <c r="R76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A77" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B77" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C75">
+      <c r="C77">
         <v>2</v>
       </c>
-      <c r="D75">
-        <f>J75+K75+L75+M75+N75</f>
+      <c r="D77">
+        <f>J77+K77+L77+M77+N77</f>
         <v>121633.35860365373</v>
       </c>
-      <c r="E75">
+      <c r="E77">
         <v>282179.67123287602</v>
       </c>
-      <c r="F75">
+      <c r="F77">
         <v>0.85824890324911396</v>
       </c>
-      <c r="G75" s="4">
+      <c r="G77" s="4">
         <v>20824.7129679639</v>
       </c>
-      <c r="H75">
+      <c r="H77">
         <v>7456.39074483072</v>
       </c>
-      <c r="I75">
+      <c r="I77">
         <v>5114.4587365303096</v>
       </c>
-      <c r="J75">
+      <c r="J77">
         <v>33395.562449324898</v>
       </c>
-      <c r="K75">
+      <c r="K77">
         <v>51302.320205525801</v>
       </c>
-      <c r="L75">
+      <c r="L77">
         <v>16537.7269222135</v>
       </c>
-      <c r="M75">
+      <c r="M77">
         <v>19392.801250865799</v>
       </c>
-      <c r="N75">
+      <c r="N77">
         <v>1004.9477757237401</v>
       </c>
-      <c r="O75">
-        <v>0</v>
-      </c>
-      <c r="P75">
+      <c r="O77">
+        <v>0</v>
+      </c>
+      <c r="P77">
         <f t="shared" si="14"/>
         <v>242193.03042265025</v>
       </c>
-      <c r="Q75">
+      <c r="Q77">
         <v>1183.4303612998101</v>
       </c>
-      <c r="R75">
+      <c r="R77">
         <v>15931.1957490451</v>
       </c>
-      <c r="S75">
+      <c r="S77">
         <v>346.33034237054602</v>
       </c>
-      <c r="T75">
+      <c r="T77">
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A79" t="s">
         <v>20</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B79" t="s">
         <v>21</v>
       </c>
-      <c r="C77">
+      <c r="C79">
         <v>4</v>
       </c>
-      <c r="D77">
-        <f>J77+K77+L77+M77+N77</f>
+      <c r="D79">
+        <f>J79+K79+L79+M79+N79</f>
         <v>116706.4157905051</v>
       </c>
-      <c r="E77">
+      <c r="E79">
         <v>282179.671253876</v>
       </c>
-      <c r="F77">
+      <c r="F79">
         <v>0.84083338305413902</v>
       </c>
-      <c r="G77" s="4">
+      <c r="G79" s="4">
         <v>20578.5072164468</v>
       </c>
-      <c r="H77">
+      <c r="H79">
         <v>7102.5751506616798</v>
       </c>
-      <c r="I77">
+      <c r="I79">
         <v>2588.50529592865</v>
       </c>
-      <c r="J77">
+      <c r="J79">
         <v>30269.587663037099</v>
       </c>
-      <c r="K77">
+      <c r="K79">
         <v>50843.185173268197</v>
       </c>
-      <c r="L77">
+      <c r="L79">
         <v>15303.8015139912</v>
       </c>
-      <c r="M77">
+      <c r="M79">
         <v>19297.530732323299</v>
       </c>
-      <c r="N77">
+      <c r="N79">
         <v>992.31070788530405</v>
       </c>
-      <c r="O77">
-        <v>0</v>
-      </c>
-      <c r="P77">
-        <f t="shared" ref="P77:P79" si="15">D77+$P$1</f>
+      <c r="O79">
+        <v>0</v>
+      </c>
+      <c r="P79">
+        <f t="shared" ref="P79:P81" si="15">D79+$P$1</f>
         <v>237266.08760950161</v>
       </c>
-      <c r="Q77">
+      <c r="Q79">
         <v>1127.2750356983499</v>
       </c>
-      <c r="R77">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
+      <c r="R79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A80" t="s">
         <v>22</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B80" t="s">
         <v>21</v>
       </c>
-      <c r="C78">
+      <c r="C80">
         <v>4</v>
       </c>
-      <c r="D78">
-        <f>J78+K78+L78+M78+N78</f>
+      <c r="D80">
+        <f>J80+K80+L80+M80+N80</f>
         <v>121744.79706913032</v>
       </c>
-      <c r="E78">
+      <c r="E80">
         <v>282179.88376308198</v>
       </c>
-      <c r="F78">
+      <c r="F80">
         <v>0.85713546401894802</v>
       </c>
-      <c r="G78">
+      <c r="G80">
         <v>21291.5607898614</v>
       </c>
-      <c r="H78">
+      <c r="H80">
         <v>7432.3603175362596</v>
       </c>
-      <c r="I78">
+      <c r="I80">
         <v>5035.2758648834497</v>
       </c>
-      <c r="J78">
+      <c r="J80">
         <v>33759.196972281097</v>
       </c>
-      <c r="K78">
+      <c r="K80">
         <v>51128.3645002267</v>
       </c>
-      <c r="L78">
+      <c r="L80">
         <v>16070.129576240101</v>
       </c>
-      <c r="M78">
+      <c r="M80">
         <v>19356.7120304526</v>
       </c>
-      <c r="N78">
+      <c r="N80">
         <v>1430.39398992981</v>
       </c>
-      <c r="O78">
-        <v>0</v>
-      </c>
-      <c r="P78">
+      <c r="O80">
+        <v>0</v>
+      </c>
+      <c r="P80">
         <f t="shared" si="15"/>
         <v>242304.46888812684</v>
       </c>
-      <c r="Q78">
+      <c r="Q80">
         <v>1179.61640190856</v>
       </c>
-      <c r="R78">
+      <c r="R80">
         <v>13411.4010346792</v>
       </c>
-      <c r="S78">
+      <c r="S80">
         <v>478.97860838140201</v>
       </c>
-      <c r="T78">
+      <c r="T80">
         <v>0.22564405635506199</v>
       </c>
-      <c r="U78">
+      <c r="U80">
         <v>10550.3210016294</v>
       </c>
-      <c r="V78">
+      <c r="V80">
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="D79">
-        <f>D78-D72</f>
+    <row r="81" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="D81">
+        <f>D80-D74</f>
         <v>-4018.7603482047853</v>
       </c>
-      <c r="E79">
-        <f t="shared" ref="E79:N79" si="16">E78-E72</f>
+      <c r="E81">
+        <f t="shared" ref="E81:N81" si="16">E80-E74</f>
         <v>0.21251127298455685</v>
       </c>
-      <c r="F79">
+      <c r="F81">
         <f t="shared" si="16"/>
         <v>-1.5794992464996938E-2</v>
       </c>
-      <c r="G79">
+      <c r="G81">
         <f t="shared" si="16"/>
         <v>-1335.1371720950992</v>
       </c>
-      <c r="H79">
+      <c r="H81">
         <f t="shared" si="16"/>
         <v>329.78360458492989</v>
       </c>
-      <c r="I79">
+      <c r="I81">
         <f t="shared" si="16"/>
         <v>-4562.1832736040305</v>
       </c>
-      <c r="J79">
+      <c r="J81">
         <f t="shared" si="16"/>
         <v>-5567.5368411142044</v>
       </c>
-      <c r="K79">
+      <c r="K81">
         <f t="shared" si="16"/>
         <v>285.1804885383026</v>
       </c>
-      <c r="L79">
+      <c r="L81">
         <f t="shared" si="16"/>
         <v>766.33118310559985</v>
       </c>
-      <c r="M79">
+      <c r="M81">
         <f t="shared" si="16"/>
         <v>59.181539221001003</v>
       </c>
-      <c r="N79">
+      <c r="N81">
         <f t="shared" si="16"/>
         <v>438.08328204450595</v>
       </c>
-      <c r="P79">
+      <c r="P81">
         <f t="shared" si="15"/>
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A80" s="1" t="s">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A82" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G80" s="4"/>
-    </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
+      <c r="G82" s="4"/>
+    </row>
+    <row r="83" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A83" t="s">
         <v>22</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B83" t="s">
         <v>21</v>
       </c>
-      <c r="C81">
+      <c r="C83">
         <v>4</v>
       </c>
-      <c r="D81">
-        <f>J81+K81+L81+M81+N81</f>
+      <c r="D83">
+        <f>J83+K83+L83+M83+N83</f>
         <v>147118.48206815872</v>
       </c>
-      <c r="E81">
+      <c r="E83">
         <v>355610.364944759</v>
       </c>
-      <c r="F81">
+      <c r="F83">
         <v>0.75267772890587503</v>
       </c>
-      <c r="G81">
+      <c r="G83">
         <v>25765.651662743599</v>
       </c>
-      <c r="H81">
+      <c r="H83">
         <v>7150.9042815892099</v>
       </c>
-      <c r="I81">
+      <c r="I83">
         <v>5144.3184852884797</v>
       </c>
-      <c r="J81">
+      <c r="J83">
         <v>38060.874429621297</v>
       </c>
-      <c r="K81">
+      <c r="K83">
         <v>64168.339029134899</v>
       </c>
-      <c r="L81">
+      <c r="L83">
         <v>19539.954214541001</v>
       </c>
-      <c r="M81">
+      <c r="M83">
         <v>24338.851661831999</v>
       </c>
-      <c r="N81">
+      <c r="N83">
         <v>1010.46273302954</v>
       </c>
-      <c r="O81">
-        <v>0</v>
-      </c>
-      <c r="P81">
-        <f t="shared" ref="P81" si="17">D81+$P$1</f>
+      <c r="O83">
+        <v>0</v>
+      </c>
+      <c r="P83">
+        <f t="shared" ref="P83" si="17">D83+$P$1</f>
         <v>267678.15388715523</v>
       </c>
-      <c r="Q81">
+      <c r="Q83">
         <v>1597.68911089628</v>
       </c>
-      <c r="R81">
+      <c r="R83">
         <v>13084.0423994256</v>
       </c>
-      <c r="S81">
+      <c r="S83">
         <v>467.28722855091399</v>
       </c>
-      <c r="T81">
+      <c r="T83">
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
+    <row r="84" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A84" t="s">
         <v>22</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B84" t="s">
         <v>35</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C84" t="s">
         <v>35</v>
       </c>
-      <c r="D82" t="s">
+      <c r="D84" t="s">
         <v>36</v>
       </c>
-      <c r="E82" t="s">
+      <c r="E84" t="s">
         <v>36</v>
       </c>
-      <c r="F82" t="s">
+      <c r="F84" t="s">
         <v>36</v>
       </c>
-      <c r="G82" s="4">
+      <c r="G84" s="4">
         <v>28838</v>
       </c>
-      <c r="H82">
+      <c r="H84">
         <v>7567.5</v>
       </c>
-      <c r="I82">
+      <c r="I84">
         <v>13764.1</v>
       </c>
-      <c r="J82">
+      <c r="J84">
         <v>50169.7</v>
       </c>
-      <c r="K82" t="s">
+      <c r="K84" t="s">
         <v>36</v>
       </c>
-      <c r="L82" t="s">
+      <c r="L84" t="s">
         <v>36</v>
       </c>
-      <c r="M82" t="s">
+      <c r="M84" t="s">
         <v>36</v>
       </c>
-      <c r="N82" t="s">
+      <c r="N84" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A84" s="1" t="s">
+    <row r="86" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A86" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G84" s="4"/>
-      <c r="P84" t="s">
+      <c r="G86" s="4"/>
+      <c r="P86" t="s">
         <v>15</v>
       </c>
-      <c r="Q84" t="s">
+      <c r="Q86" t="s">
         <v>16</v>
       </c>
-      <c r="R84" t="s">
+      <c r="R86" t="s">
         <v>17</v>
       </c>
-      <c r="S84" t="s">
+      <c r="S86" t="s">
         <v>18</v>
       </c>
-      <c r="T84" t="s">
+      <c r="T86" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="85" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
-        <v>0</v>
-      </c>
-      <c r="B85" t="s">
+    <row r="87" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A87" t="s">
+        <v>0</v>
+      </c>
+      <c r="B87" t="s">
         <v>1</v>
       </c>
-      <c r="C85" t="s">
+      <c r="C87" t="s">
         <v>2</v>
       </c>
-      <c r="D85" t="s">
+      <c r="D87" t="s">
         <v>3</v>
       </c>
-      <c r="E85" t="s">
+      <c r="E87" t="s">
         <v>4</v>
       </c>
-      <c r="F85" t="s">
+      <c r="F87" t="s">
         <v>5</v>
       </c>
-      <c r="G85" s="4" t="s">
+      <c r="G87" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H85" t="s">
+      <c r="H87" t="s">
         <v>7</v>
       </c>
-      <c r="I85" t="s">
+      <c r="I87" t="s">
         <v>8</v>
       </c>
-      <c r="J85" t="s">
+      <c r="J87" t="s">
         <v>9</v>
       </c>
-      <c r="K85" t="s">
+      <c r="K87" t="s">
         <v>10</v>
       </c>
-      <c r="L85" t="s">
+      <c r="L87" t="s">
         <v>11</v>
       </c>
-      <c r="M85" t="s">
+      <c r="M87" t="s">
         <v>12</v>
       </c>
-      <c r="N85" t="s">
+      <c r="N87" t="s">
         <v>13</v>
       </c>
-      <c r="O85" t="s">
+      <c r="O87" t="s">
         <v>14</v>
       </c>
-      <c r="P85">
+      <c r="P87">
         <v>63734.6679</v>
       </c>
-      <c r="Q85">
+      <c r="Q87">
         <v>1078.4492829999999</v>
       </c>
-      <c r="R85">
+      <c r="R87">
         <v>624.70352849999995</v>
       </c>
-      <c r="S85">
+      <c r="S87">
         <v>13.014656840000001</v>
       </c>
-      <c r="T85">
+      <c r="T87">
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="86" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A86" s="2" t="s">
+    <row r="88" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A88" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B88" t="s">
         <v>21</v>
       </c>
-      <c r="C86">
+      <c r="C88">
         <v>4</v>
       </c>
-      <c r="D86">
+      <c r="D88">
         <v>29525.427309999999</v>
       </c>
-      <c r="E86">
+      <c r="E88">
         <v>80391.755990000005</v>
       </c>
-      <c r="F86">
+      <c r="F88">
         <v>0.79280104200000001</v>
       </c>
-      <c r="G86" s="4">
+      <c r="G88" s="4">
         <v>5050.6365619999997</v>
       </c>
-      <c r="H86">
+      <c r="H88">
         <v>4678.3390820000004</v>
       </c>
-      <c r="I86">
+      <c r="I88">
         <v>2508.6600360000002</v>
       </c>
-      <c r="J86">
+      <c r="J88">
         <v>12237.635679999999</v>
       </c>
-      <c r="K86">
+      <c r="K88">
         <v>13920</v>
       </c>
-      <c r="L86">
+      <c r="L88">
         <v>2841.544922</v>
       </c>
-      <c r="M86">
+      <c r="M88">
         <v>5380.5444360000001</v>
       </c>
-      <c r="N86">
+      <c r="N88">
         <v>279.27307350000001</v>
       </c>
-      <c r="O86">
-        <v>0</v>
-      </c>
-      <c r="P86">
+      <c r="O88">
+        <v>0</v>
+      </c>
+      <c r="P88">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q86">
+      <c r="Q88">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R86">
+      <c r="R88">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S86">
+      <c r="S88">
         <v>452.7322633</v>
       </c>
-      <c r="T86">
+      <c r="T88">
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A87" s="7" t="s">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A89" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A91" t="s">
         <v>32</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B91" t="s">
         <v>33</v>
       </c>
-      <c r="C89" t="s">
+      <c r="C91" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A90">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A92">
         <v>20</v>
       </c>
-      <c r="B90">
+      <c r="B92">
         <v>60</v>
       </c>
-      <c r="C90">
+      <c r="C92">
         <v>2</v>
       </c>
-      <c r="D90">
-        <f t="shared" ref="D90:D96" si="18">J90+K90+L90+M90+N90</f>
+      <c r="D92">
+        <f t="shared" ref="D92:D98" si="18">J92+K92+L92+M92+N92</f>
         <v>120712.69088313227</v>
       </c>
-      <c r="E90">
+      <c r="E92">
         <v>282179.67123285501</v>
       </c>
-      <c r="F90">
+      <c r="F92">
         <v>0.854946898908852</v>
       </c>
-      <c r="G90">
+      <c r="G92">
         <v>18681.222424938602</v>
       </c>
-      <c r="H90">
+      <c r="H92">
         <v>5354.6114985546601</v>
       </c>
-      <c r="I90">
+      <c r="I92">
         <v>8156.08309050551</v>
       </c>
-      <c r="J90">
+      <c r="J92">
         <v>32191.917013998798</v>
       </c>
-      <c r="K90">
+      <c r="K92">
         <v>51372.124296964801</v>
       </c>
-      <c r="L90">
+      <c r="L92">
         <v>16725.325417965501</v>
       </c>
-      <c r="M90">
+      <c r="M92">
         <v>19407.285599838699</v>
       </c>
-      <c r="N90">
+      <c r="N92">
         <v>1016.03855436447</v>
       </c>
-      <c r="O90">
-        <v>0</v>
-      </c>
-      <c r="P90">
-        <f t="shared" ref="P90:P96" si="19">D90+$P$1</f>
+      <c r="O92">
+        <v>0</v>
+      </c>
+      <c r="P92">
+        <f t="shared" ref="P92:P98" si="19">D92+$P$1</f>
         <v>241272.36270212877</v>
       </c>
-      <c r="Q90">
+      <c r="Q92">
         <v>1192.7637589594799</v>
       </c>
-      <c r="R90">
+      <c r="R92">
         <v>19736.206339365101</v>
       </c>
-      <c r="S90">
+      <c r="S92">
         <v>481.37088632597801</v>
       </c>
-      <c r="T90" s="6">
+      <c r="T92" s="6">
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A91">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A93">
         <v>20</v>
       </c>
-      <c r="B91">
+      <c r="B93">
         <v>50</v>
       </c>
-      <c r="C91">
+      <c r="C93">
         <v>2</v>
       </c>
-      <c r="D91">
+      <c r="D93">
         <f t="shared" si="18"/>
         <v>119392.42354269064</v>
       </c>
-      <c r="E91">
+      <c r="E93">
         <v>282254.81855225202</v>
       </c>
-      <c r="F91">
+      <c r="F93">
         <v>0.85006146065890897</v>
       </c>
-      <c r="G91">
+      <c r="G93">
         <v>19407.840072768398</v>
       </c>
-      <c r="H91">
+      <c r="H93">
         <v>5891.8301217549197</v>
       </c>
-      <c r="I91">
+      <c r="I93">
         <v>6659.4942697455399</v>
       </c>
-      <c r="J91">
+      <c r="J93">
         <v>31959.164464268899</v>
       </c>
-      <c r="K91">
+      <c r="K93">
         <v>51102.045942938203</v>
       </c>
-      <c r="L91">
+      <c r="L93">
         <v>15967.176494174801</v>
       </c>
-      <c r="M91">
+      <c r="M93">
         <v>19353.573908279199</v>
       </c>
-      <c r="N91">
+      <c r="N93">
         <v>1010.46273302954</v>
       </c>
-      <c r="O91">
-        <v>0</v>
-      </c>
-      <c r="P91">
+      <c r="O93">
+        <v>0</v>
+      </c>
+      <c r="P93">
         <f t="shared" si="19"/>
         <v>239952.09536168716</v>
       </c>
-      <c r="Q91">
+      <c r="Q93">
         <v>1312.43161993582</v>
       </c>
-      <c r="R91">
+      <c r="R93">
         <v>18377.616631847999</v>
       </c>
-      <c r="S91">
+      <c r="S93">
         <v>459.4404157962</v>
       </c>
-      <c r="T91" s="6">
+      <c r="T93" s="6">
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A92">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A94">
         <v>20</v>
       </c>
-      <c r="B92">
+      <c r="B94">
         <v>40</v>
       </c>
-      <c r="C92">
+      <c r="C94">
         <v>2</v>
       </c>
-      <c r="D92">
+      <c r="D94">
         <f t="shared" si="18"/>
         <v>117777.02945340994</v>
       </c>
-      <c r="E92">
+      <c r="E94">
         <v>282179.67123287299</v>
       </c>
-      <c r="F92">
+      <c r="F94">
         <v>0.84456314023622803</v>
       </c>
-      <c r="G92">
+      <c r="G94">
         <v>19298.245593088301</v>
       </c>
-      <c r="H92">
+      <c r="H94">
         <v>5682.0016560700296</v>
       </c>
-      <c r="I92">
+      <c r="I94">
         <v>5350.3346939491703</v>
       </c>
-      <c r="J92">
+      <c r="J94">
         <v>30330.5819431075</v>
       </c>
-      <c r="K92">
+      <c r="K94">
         <v>51097.733915068202</v>
       </c>
-      <c r="L92">
+      <c r="L94">
         <v>15987.901266609</v>
       </c>
-      <c r="M92">
+      <c r="M94">
         <v>19350.349595595701</v>
       </c>
-      <c r="N92">
+      <c r="N94">
         <v>1010.46273302954</v>
       </c>
-      <c r="O92">
-        <v>0</v>
-      </c>
-      <c r="P92">
+      <c r="O94">
+        <v>0</v>
+      </c>
+      <c r="P94">
         <f t="shared" si="19"/>
         <v>238336.70127240644</v>
       </c>
-      <c r="Q92">
+      <c r="Q94">
         <v>1265.6913868611</v>
       </c>
-      <c r="R92">
+      <c r="R94">
         <v>17746.163883660702</v>
       </c>
-      <c r="S92">
+      <c r="S94">
         <v>507.03325381887902</v>
       </c>
-      <c r="T92" s="6">
+      <c r="T94" s="6">
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A93">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A95">
         <v>20</v>
       </c>
-      <c r="B93">
+      <c r="B95">
         <v>30</v>
       </c>
-      <c r="C93">
+      <c r="C95">
         <v>2</v>
       </c>
-      <c r="D93">
+      <c r="D95">
         <f t="shared" si="18"/>
         <v>116625.1695160947</v>
       </c>
-      <c r="E93">
+      <c r="E95">
         <v>282182.50548365602</v>
       </c>
-      <c r="F93">
+      <c r="F95">
         <v>0.84045954058697003</v>
       </c>
-      <c r="G93">
+      <c r="G95">
         <v>19302.752565837702</v>
       </c>
-      <c r="H93">
+      <c r="H95">
         <v>6226.5181629292701</v>
       </c>
-      <c r="I93">
+      <c r="I95">
         <v>3974.5318253822402</v>
       </c>
-      <c r="J93">
+      <c r="J95">
         <v>29503.802554149199</v>
       </c>
-      <c r="K93">
+      <c r="K95">
         <v>51013.610661725899</v>
       </c>
-      <c r="L93">
+      <c r="L95">
         <v>15760.601295416</v>
       </c>
-      <c r="M93">
+      <c r="M95">
         <v>19332.981882301501</v>
       </c>
-      <c r="N93">
+      <c r="N95">
         <v>1014.17312250211</v>
       </c>
-      <c r="O93">
-        <v>0</v>
-      </c>
-      <c r="P93">
+      <c r="O95">
+        <v>0</v>
+      </c>
+      <c r="P95">
         <f t="shared" si="19"/>
         <v>237184.84133509122</v>
       </c>
-      <c r="Q93">
+      <c r="Q95">
         <v>1386.9848841974899</v>
       </c>
-      <c r="R93">
+      <c r="R95">
         <v>18436.445202769701</v>
       </c>
-      <c r="S93">
+      <c r="S95">
         <v>209.50505912238299</v>
       </c>
-      <c r="T93" s="6">
+      <c r="T95" s="6">
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A94" s="3">
+    <row r="96" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A96" s="3">
         <v>20</v>
       </c>
-      <c r="B94" s="3">
+      <c r="B96" s="3">
         <v>20</v>
       </c>
-      <c r="C94" s="3">
+      <c r="C96" s="3">
         <v>2</v>
       </c>
-      <c r="D94">
+      <c r="D96">
         <f t="shared" si="18"/>
         <v>115198.459983006</v>
       </c>
-      <c r="E94">
+      <c r="E96">
         <v>282179.67123297497</v>
       </c>
-      <c r="F94">
+      <c r="F96">
         <v>0.83541194997266699</v>
       </c>
-      <c r="G94">
+      <c r="G96">
         <v>19351.2255529412</v>
       </c>
-      <c r="H94">
+      <c r="H96">
         <v>6002.0469674603501</v>
       </c>
-      <c r="I94">
+      <c r="I96">
         <v>2645.4376652921501</v>
       </c>
-      <c r="J94">
+      <c r="J96">
         <v>27998.710185693701</v>
       </c>
-      <c r="K94">
+      <c r="K96">
         <v>51033.4442867088</v>
       </c>
-      <c r="L94">
+      <c r="L96">
         <v>15815.1228903871</v>
       </c>
-      <c r="M94">
+      <c r="M96">
         <v>19337.009497714302</v>
       </c>
-      <c r="N94">
+      <c r="N96">
         <v>1014.17312250211</v>
       </c>
-      <c r="O94">
-        <v>0</v>
-      </c>
-      <c r="P94">
+      <c r="O96">
+        <v>0</v>
+      </c>
+      <c r="P96">
         <f t="shared" si="19"/>
         <v>235758.13180200252</v>
       </c>
-      <c r="Q94">
+      <c r="Q96">
         <v>1336.98290493166</v>
       </c>
-      <c r="R94">
+      <c r="R96">
         <v>18577.307877855899</v>
       </c>
-      <c r="S94">
+      <c r="S96">
         <v>432.030415764091</v>
       </c>
-      <c r="T94" s="6">
+      <c r="T96" s="6">
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A95">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A97">
         <v>20</v>
       </c>
-      <c r="B95">
+      <c r="B97">
         <v>15</v>
       </c>
-      <c r="C95">
+      <c r="C97">
         <v>2</v>
       </c>
-      <c r="D95">
+      <c r="D97">
         <f t="shared" si="18"/>
         <v>114451.25872361983</v>
       </c>
-      <c r="E95">
+      <c r="E97">
         <v>282179.67123267101</v>
       </c>
-      <c r="F95">
+      <c r="F97">
         <v>0.83277713625127903</v>
       </c>
-      <c r="G95">
+      <c r="G97">
         <v>19390.977969205</v>
       </c>
-      <c r="H95">
+      <c r="H97">
         <v>5599.5405456203798</v>
       </c>
-      <c r="I95">
+      <c r="I97">
         <v>2128.1287863747102</v>
       </c>
-      <c r="J95">
+      <c r="J97">
         <v>27118.647301200101</v>
       </c>
-      <c r="K95">
+      <c r="K97">
         <v>51068.507704320902</v>
       </c>
-      <c r="L95">
+      <c r="L97">
         <v>15909.3558282099</v>
       </c>
-      <c r="M95">
+      <c r="M97">
         <v>19344.285156859401</v>
       </c>
-      <c r="N95">
+      <c r="N97">
         <v>1010.46273302954</v>
       </c>
-      <c r="O95">
-        <v>0</v>
-      </c>
-      <c r="P95">
+      <c r="O97">
+        <v>0</v>
+      </c>
+      <c r="P97">
         <f t="shared" si="19"/>
         <v>235010.93054261635</v>
       </c>
-      <c r="Q95">
+      <c r="Q97">
         <v>1247.3228025527501</v>
       </c>
-      <c r="R95">
+      <c r="R97">
         <v>16417.502561416801</v>
       </c>
-      <c r="S95">
+      <c r="S97">
         <v>469.07150175476602</v>
       </c>
-      <c r="T95" s="6">
+      <c r="T97" s="6">
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A96">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A98">
         <v>20</v>
       </c>
-      <c r="B96">
+      <c r="B98">
         <v>12</v>
       </c>
-      <c r="C96">
+      <c r="C98">
         <v>2</v>
       </c>
-      <c r="D96">
+      <c r="D98">
         <f t="shared" si="18"/>
         <v>114787.7594081375</v>
       </c>
-      <c r="E96">
+      <c r="E98">
         <v>282179.67123287602</v>
       </c>
-      <c r="F96">
+      <c r="F98">
         <v>0.83403396920434802</v>
       </c>
-      <c r="G96">
+      <c r="G98">
         <v>20436.472361711199</v>
       </c>
-      <c r="H96">
+      <c r="H98">
         <v>4946.5396722567002</v>
       </c>
-      <c r="I96">
+      <c r="I98">
         <v>2967.9237851293901</v>
       </c>
-      <c r="J96">
+      <c r="J98">
         <v>28350.9358190973</v>
       </c>
-      <c r="K96">
+      <c r="K98">
         <v>50843.184005923598</v>
       </c>
-      <c r="L96">
+      <c r="L98">
         <v>15303.798385783</v>
       </c>
-      <c r="M96">
+      <c r="M98">
         <v>19297.530489448302</v>
       </c>
-      <c r="N96">
+      <c r="N98">
         <v>992.31070788530405</v>
       </c>
-      <c r="O96">
-        <v>0</v>
-      </c>
-      <c r="P96">
+      <c r="O98">
+        <v>0</v>
+      </c>
+      <c r="P98">
         <f t="shared" si="19"/>
         <v>235347.43122713402</v>
       </c>
-      <c r="Q96">
+      <c r="Q98">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R96">
+      <c r="R98">
         <v>13.380488321454299</v>
       </c>
-      <c r="S96">
+      <c r="S98">
         <v>2.67609766429086</v>
       </c>
-      <c r="T96" s="6">
+      <c r="T98" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Further updates to the analytical equations. Not finished yet.
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09720A58-31D4-4647-97B7-598DF1A895E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A374B3F-32CF-40D3-B745-2118EAAFF94F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -385,7 +385,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -546,12 +546,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -2236,6 +2230,10 @@
     <row r="20" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
+      <c r="K20">
+        <f>K19+L19+M19</f>
+        <v>85444.512881154995</v>
+      </c>
       <c r="S20" s="2"/>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.4">
@@ -2453,6 +2451,10 @@
     <row r="26" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
+      <c r="K26">
+        <f>K25+L25+M25</f>
+        <v>86355.755432219594</v>
+      </c>
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
@@ -2793,85 +2795,89 @@
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="D33">
-        <f>D32-D31</f>
+        <f t="shared" ref="D33:V33" si="6">D32-D31</f>
         <v>785.66289527932531</v>
       </c>
       <c r="E33">
-        <f>E32-E31</f>
+        <f t="shared" si="6"/>
         <v>2.4971086531877518E-8</v>
       </c>
       <c r="F33">
-        <f>F32-F31</f>
+        <f t="shared" si="6"/>
         <v>2.6907854028540568E-3</v>
       </c>
       <c r="G33">
-        <f>G32-G31</f>
+        <f t="shared" si="6"/>
         <v>-221.42920834019969</v>
       </c>
       <c r="H33">
-        <f>H32-H31</f>
+        <f t="shared" si="6"/>
         <v>896.09976246881979</v>
       </c>
       <c r="I33">
-        <f>I32-I31</f>
+        <f t="shared" si="6"/>
         <v>-4877.4899349639245</v>
       </c>
       <c r="J33">
-        <f>J32-J31</f>
+        <f t="shared" si="6"/>
         <v>-4202.8193808354008</v>
       </c>
       <c r="K33">
-        <f>K32-K31</f>
+        <f t="shared" si="6"/>
         <v>-87.19067491790338</v>
       </c>
       <c r="L33">
-        <f>L32-L31</f>
+        <f t="shared" si="6"/>
         <v>4424.0083944886992</v>
       </c>
       <c r="M33">
-        <f>M32-M31</f>
+        <f t="shared" si="6"/>
         <v>625.28660162189772</v>
       </c>
       <c r="N33">
-        <f>N32-N31</f>
+        <f t="shared" si="6"/>
         <v>26.377954922030085</v>
       </c>
       <c r="O33">
-        <f>O32-O31</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="P33">
-        <f>P32-P31</f>
+        <f t="shared" si="6"/>
         <v>785.66289527932531</v>
       </c>
       <c r="Q33">
-        <f>Q32-Q31</f>
+        <f t="shared" si="6"/>
         <v>200.21086642008004</v>
       </c>
       <c r="R33">
-        <f>R32-R31</f>
+        <f t="shared" si="6"/>
         <v>20835.930555410298</v>
       </c>
       <c r="S33">
-        <f>S32-S31</f>
+        <f t="shared" si="6"/>
         <v>397.33849572936299</v>
       </c>
       <c r="T33">
-        <f>T32-T31</f>
+        <f t="shared" si="6"/>
         <v>-0.1359304574304484</v>
       </c>
       <c r="U33">
-        <f>U32-U31</f>
+        <f t="shared" si="6"/>
         <v>25293.846976061999</v>
       </c>
       <c r="V33">
-        <f>V32-V31</f>
+        <f t="shared" si="6"/>
         <v>200.18128127969257</v>
       </c>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
+      <c r="K34">
+        <f>K31+L31+M31</f>
+        <v>86355.755432219594</v>
+      </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A35" s="7" t="s">
@@ -2928,7 +2934,7 @@
         <v>0</v>
       </c>
       <c r="P36">
-        <f t="shared" ref="P36:P37" si="6">D36+$P$1</f>
+        <f t="shared" ref="P36:P37" si="7">D36+$P$1</f>
         <v>237552.9910647514</v>
       </c>
       <c r="Q36">
@@ -2992,7 +2998,7 @@
         <v>0</v>
       </c>
       <c r="P37">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>246460.49240879912</v>
       </c>
       <c r="Q37">
@@ -3061,7 +3067,7 @@
         <v>0</v>
       </c>
       <c r="P39">
-        <f t="shared" ref="P39:P40" si="7">D39+$P$1</f>
+        <f t="shared" ref="P39:P40" si="8">D39+$P$1</f>
         <v>237538.1865021491</v>
       </c>
       <c r="Q39">
@@ -3128,7 +3134,7 @@
         <v>0</v>
       </c>
       <c r="P40">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>242769.60515337173</v>
       </c>
       <c r="Q40">
@@ -3211,7 +3217,7 @@
         <v>0</v>
       </c>
       <c r="P44">
-        <f t="shared" ref="P44" si="8">D44+$P$1</f>
+        <f t="shared" ref="P44" si="9">D44+$P$1</f>
         <v>246486.61307970091</v>
       </c>
       <c r="Q44">
@@ -3359,7 +3365,7 @@
         <v>0</v>
       </c>
       <c r="P50">
-        <f t="shared" ref="P50:P57" si="9">D50+$P$1</f>
+        <f t="shared" ref="P50:P57" si="10">D50+$P$1</f>
         <v>238413.66244470741</v>
       </c>
       <c r="Q50">
@@ -3423,7 +3429,7 @@
         <v>0</v>
       </c>
       <c r="P51">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>308572.43924949365</v>
       </c>
       <c r="Q51">
@@ -3491,7 +3497,7 @@
         <v>0</v>
       </c>
       <c r="P53">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>238584.40212047941</v>
       </c>
       <c r="Q53">
@@ -3555,7 +3561,7 @@
         <v>0</v>
       </c>
       <c r="P54">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>293116.00381082937</v>
       </c>
       <c r="Q54">
@@ -3622,7 +3628,7 @@
         <v>0</v>
       </c>
       <c r="P56">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>238385.73201352643</v>
       </c>
       <c r="Q56">
@@ -3686,7 +3692,7 @@
         <v>0</v>
       </c>
       <c r="P57">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>245994.13393950483</v>
       </c>
       <c r="Q57">
@@ -3756,7 +3762,7 @@
         <v>3157.9970999842499</v>
       </c>
       <c r="P60">
-        <f t="shared" ref="P60" si="10">D60+$P$1</f>
+        <f t="shared" ref="P60" si="11">D60+$P$1</f>
         <v>240194.76390161275</v>
       </c>
       <c r="Q60">
@@ -3981,75 +3987,75 @@
         <v>513.41110323798785</v>
       </c>
       <c r="E64">
-        <f t="shared" ref="E64:V64" si="11">E63-E62</f>
+        <f t="shared" ref="E64:V64" si="12">E63-E62</f>
         <v>-1.0599615052342415E-7</v>
       </c>
       <c r="F64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>1.8194475210779881E-3</v>
       </c>
       <c r="G64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-214.21539764659974</v>
       </c>
       <c r="H64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-624.4983606493397</v>
       </c>
       <c r="I64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>4877.8861089948059</v>
       </c>
       <c r="J64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>4039.1723506987983</v>
       </c>
       <c r="K64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>183.72486634590314</v>
       </c>
       <c r="L64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-3232.9060902373021</v>
       </c>
       <c r="M64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-476.58002357000078</v>
       </c>
       <c r="N64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-26.750816248570118</v>
       </c>
       <c r="O64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="P64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>513.41110323701287</v>
       </c>
       <c r="Q64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-139.52840101139986</v>
       </c>
       <c r="R64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-16066.151948654198</v>
       </c>
       <c r="S64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-545.80690098968103</v>
       </c>
       <c r="T64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.30386414961436203</v>
       </c>
       <c r="U64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-23556.497919273097</v>
       </c>
       <c r="V64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-171.16162567428404</v>
       </c>
     </row>
@@ -4229,75 +4235,75 @@
         <v>-16260.494075352748</v>
       </c>
       <c r="E71">
-        <f t="shared" ref="E71:V71" si="12">E70-E67</f>
+        <f t="shared" ref="E71:V71" si="13">E70-E67</f>
         <v>-11.188766930019483</v>
       </c>
       <c r="F71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-5.2593913252494073E-2</v>
       </c>
       <c r="G71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-4474.9745192109003</v>
       </c>
       <c r="H71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1349.0083827482595</v>
       </c>
       <c r="I71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-9098.574812435656</v>
       </c>
       <c r="J71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-12224.540948898299</v>
       </c>
       <c r="K71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>99.745205475301191</v>
       </c>
       <c r="L71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>4931.2097430098001</v>
       </c>
       <c r="M71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>663.72894502789859</v>
       </c>
       <c r="N71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>52.540525326540092</v>
       </c>
       <c r="O71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>8320.7995903714655</v>
       </c>
       <c r="P71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-15268.183367467253</v>
       </c>
       <c r="Q71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>301.40187495156988</v>
       </c>
       <c r="R71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>34518.506961381201</v>
       </c>
       <c r="S71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>841.91480393612801</v>
       </c>
       <c r="T71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0.38784649209264499</v>
       </c>
       <c r="U71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>38249.060394551692</v>
       </c>
       <c r="V71">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>301.20361806757597</v>
       </c>
     </row>
@@ -4354,7 +4360,7 @@
         <v>0</v>
       </c>
       <c r="P73">
-        <f t="shared" ref="P73:P74" si="13">D73+$P$1</f>
+        <f t="shared" ref="P73:P74" si="14">D73+$P$1</f>
         <v>236582.9608490612</v>
       </c>
       <c r="Q73">
@@ -4418,7 +4424,7 @@
         <v>0</v>
       </c>
       <c r="P74">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>246323.22923633162</v>
       </c>
       <c r="Q74">
@@ -4485,7 +4491,7 @@
         <v>0</v>
       </c>
       <c r="P76">
-        <f t="shared" ref="P76:P77" si="14">D76+$P$1</f>
+        <f t="shared" ref="P76:P77" si="15">D76+$P$1</f>
         <v>237266.08760950522</v>
       </c>
       <c r="Q76">
@@ -4543,7 +4549,7 @@
         <v>0</v>
       </c>
       <c r="P77">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>242193.03042265025</v>
       </c>
       <c r="Q77">
@@ -4607,7 +4613,7 @@
         <v>0</v>
       </c>
       <c r="P79">
-        <f t="shared" ref="P79:P81" si="15">D79+$P$1</f>
+        <f t="shared" ref="P79:P81" si="16">D79+$P$1</f>
         <v>237266.08760950161</v>
       </c>
       <c r="Q79">
@@ -4665,7 +4671,7 @@
         <v>0</v>
       </c>
       <c r="P80">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>242304.46888812684</v>
       </c>
       <c r="Q80">
@@ -4693,47 +4699,47 @@
         <v>-4018.7603482047853</v>
       </c>
       <c r="E81">
-        <f t="shared" ref="E81:N81" si="16">E80-E74</f>
+        <f t="shared" ref="E81:N81" si="17">E80-E74</f>
         <v>0.21251127298455685</v>
       </c>
       <c r="F81">
+        <f t="shared" si="17"/>
+        <v>-1.5794992464996938E-2</v>
+      </c>
+      <c r="G81">
+        <f t="shared" si="17"/>
+        <v>-1335.1371720950992</v>
+      </c>
+      <c r="H81">
+        <f t="shared" si="17"/>
+        <v>329.78360458492989</v>
+      </c>
+      <c r="I81">
+        <f t="shared" si="17"/>
+        <v>-4562.1832736040305</v>
+      </c>
+      <c r="J81">
+        <f t="shared" si="17"/>
+        <v>-5567.5368411142044</v>
+      </c>
+      <c r="K81">
+        <f t="shared" si="17"/>
+        <v>285.1804885383026</v>
+      </c>
+      <c r="L81">
+        <f t="shared" si="17"/>
+        <v>766.33118310559985</v>
+      </c>
+      <c r="M81">
+        <f t="shared" si="17"/>
+        <v>59.181539221001003</v>
+      </c>
+      <c r="N81">
+        <f t="shared" si="17"/>
+        <v>438.08328204450595</v>
+      </c>
+      <c r="P81">
         <f t="shared" si="16"/>
-        <v>-1.5794992464996938E-2</v>
-      </c>
-      <c r="G81">
-        <f t="shared" si="16"/>
-        <v>-1335.1371720950992</v>
-      </c>
-      <c r="H81">
-        <f t="shared" si="16"/>
-        <v>329.78360458492989</v>
-      </c>
-      <c r="I81">
-        <f t="shared" si="16"/>
-        <v>-4562.1832736040305</v>
-      </c>
-      <c r="J81">
-        <f t="shared" si="16"/>
-        <v>-5567.5368411142044</v>
-      </c>
-      <c r="K81">
-        <f t="shared" si="16"/>
-        <v>285.1804885383026</v>
-      </c>
-      <c r="L81">
-        <f t="shared" si="16"/>
-        <v>766.33118310559985</v>
-      </c>
-      <c r="M81">
-        <f t="shared" si="16"/>
-        <v>59.181539221001003</v>
-      </c>
-      <c r="N81">
-        <f t="shared" si="16"/>
-        <v>438.08328204450595</v>
-      </c>
-      <c r="P81">
-        <f t="shared" si="15"/>
         <v>116540.91147079173</v>
       </c>
     </row>
@@ -4791,7 +4797,7 @@
         <v>0</v>
       </c>
       <c r="P83">
-        <f t="shared" ref="P83" si="17">D83+$P$1</f>
+        <f t="shared" ref="P83" si="18">D83+$P$1</f>
         <v>267678.15388715523</v>
       </c>
       <c r="Q83">
@@ -5023,7 +5029,7 @@
         <v>2</v>
       </c>
       <c r="D92">
-        <f t="shared" ref="D92:D98" si="18">J92+K92+L92+M92+N92</f>
+        <f t="shared" ref="D92:D98" si="19">J92+K92+L92+M92+N92</f>
         <v>120712.69088313227</v>
       </c>
       <c r="E92">
@@ -5060,7 +5066,7 @@
         <v>0</v>
       </c>
       <c r="P92">
-        <f t="shared" ref="P92:P98" si="19">D92+$P$1</f>
+        <f t="shared" ref="P92:P98" si="20">D92+$P$1</f>
         <v>241272.36270212877</v>
       </c>
       <c r="Q92">
@@ -5087,7 +5093,7 @@
         <v>2</v>
       </c>
       <c r="D93">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>119392.42354269064</v>
       </c>
       <c r="E93">
@@ -5124,7 +5130,7 @@
         <v>0</v>
       </c>
       <c r="P93">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>239952.09536168716</v>
       </c>
       <c r="Q93">
@@ -5151,7 +5157,7 @@
         <v>2</v>
       </c>
       <c r="D94">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>117777.02945340994</v>
       </c>
       <c r="E94">
@@ -5188,7 +5194,7 @@
         <v>0</v>
       </c>
       <c r="P94">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>238336.70127240644</v>
       </c>
       <c r="Q94">
@@ -5215,7 +5221,7 @@
         <v>2</v>
       </c>
       <c r="D95">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>116625.1695160947</v>
       </c>
       <c r="E95">
@@ -5252,7 +5258,7 @@
         <v>0</v>
       </c>
       <c r="P95">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>237184.84133509122</v>
       </c>
       <c r="Q95">
@@ -5279,7 +5285,7 @@
         <v>2</v>
       </c>
       <c r="D96">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>115198.459983006</v>
       </c>
       <c r="E96">
@@ -5316,7 +5322,7 @@
         <v>0</v>
       </c>
       <c r="P96">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>235758.13180200252</v>
       </c>
       <c r="Q96">
@@ -5343,7 +5349,7 @@
         <v>2</v>
       </c>
       <c r="D97">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>114451.25872361983</v>
       </c>
       <c r="E97">
@@ -5380,7 +5386,7 @@
         <v>0</v>
       </c>
       <c r="P97">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>235010.93054261635</v>
       </c>
       <c r="Q97">
@@ -5407,7 +5413,7 @@
         <v>2</v>
       </c>
       <c r="D98">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>114787.7594081375</v>
       </c>
       <c r="E98">
@@ -5444,7 +5450,7 @@
         <v>0</v>
       </c>
       <c r="P98">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>235347.43122713402</v>
       </c>
       <c r="Q98">

</xml_diff>

<commit_message>
trying DR with delayed shutdowns
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A374B3F-32CF-40D3-B745-2118EAAFF94F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95735DB1-404D-4A87-9D05-5A43B928C329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -247,7 +247,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="45">
   <si>
     <t>Season</t>
   </si>
@@ -379,6 +379,9 @@
   </si>
   <si>
     <t>CAPEX =&gt;</t>
+  </si>
+  <si>
+    <t>1 shutdown - 5 shutdowns =</t>
   </si>
 </sst>
 </file>
@@ -889,7 +892,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -899,6 +902,10 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3762,7 +3769,7 @@
         <v>3157.9970999842499</v>
       </c>
       <c r="P60">
-        <f t="shared" ref="P60" si="11">D60+$P$1</f>
+        <f t="shared" ref="P60:P64" si="11">D60+$P$1</f>
         <v>240194.76390161275</v>
       </c>
       <c r="Q60">
@@ -3827,7 +3834,7 @@
         <v>11020</v>
       </c>
       <c r="P61">
-        <f>D61+$P$1</f>
+        <f t="shared" si="11"/>
         <v>230122.64709737207</v>
       </c>
       <c r="Q61">
@@ -3853,8 +3860,9 @@
       <c r="C62">
         <v>4</v>
       </c>
-      <c r="D62">
-        <v>106092.92029140001</v>
+      <c r="D62" s="10">
+        <f>J62+K62+L62+M62+N62-O62</f>
+        <v>107555.29824632255</v>
       </c>
       <c r="E62">
         <v>282179.67123287602</v>
@@ -3890,7 +3898,8 @@
         <v>11020</v>
       </c>
       <c r="P62">
-        <v>227644.90281828199</v>
+        <f t="shared" si="11"/>
+        <v>228114.97006531907</v>
       </c>
       <c r="Q62">
         <v>1380.27146414547</v>
@@ -3922,7 +3931,8 @@
         <v>4</v>
       </c>
       <c r="D63">
-        <v>106606.33139463799</v>
+        <f>J63+K63+L63+M63+N63-O63</f>
+        <v>108041.95853331135</v>
       </c>
       <c r="E63">
         <v>282179.67123277002</v>
@@ -3958,7 +3968,8 @@
         <v>11020</v>
       </c>
       <c r="P63">
-        <v>228158.313921519</v>
+        <f t="shared" si="11"/>
+        <v>228601.63035230787</v>
       </c>
       <c r="Q63">
         <v>1240.7430631340701</v>
@@ -3980,11 +3991,14 @@
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A64" s="3"/>
-      <c r="B64" s="3"/>
-      <c r="D64">
+      <c r="A64" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B64" s="9"/>
+      <c r="C64" s="9"/>
+      <c r="D64" s="10">
         <f>D63-D62</f>
-        <v>513.41110323798785</v>
+        <v>486.66028698880109</v>
       </c>
       <c r="E64">
         <f t="shared" ref="E64:V64" si="12">E63-E62</f>
@@ -4032,7 +4046,7 @@
       </c>
       <c r="P64">
         <f t="shared" si="12"/>
-        <v>513.41110323701287</v>
+        <v>486.66028698880109</v>
       </c>
       <c r="Q64">
         <f t="shared" si="12"/>
@@ -5467,6 +5481,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A64:C64"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>

</xml_diff>

<commit_message>
Updates to analytical equations notebook
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95735DB1-404D-4A87-9D05-5A43B928C329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E100DDC-5ADE-4EE0-A35A-79A2F83459B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-19310" yWindow="10680" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -209,7 +209,7 @@
     Only one plant shutdown allowed</t>
       </text>
     </comment>
-    <comment ref="A70" authorId="18" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+    <comment ref="A71" authorId="18" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -218,7 +218,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="A77" authorId="19" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
+    <comment ref="A78" authorId="19" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -226,7 +226,7 @@
     Pretty sure this solution is wrong, but I don’t think I need this case for the paper</t>
       </text>
     </comment>
-    <comment ref="A83" authorId="20" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A84" authorId="20" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -234,7 +234,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T95" authorId="21" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T96" authorId="21" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -892,7 +892,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -906,6 +906,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1350,17 +1353,17 @@
   <threadedComment ref="A63" dT="2026-07-22T21:09:49.14" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{0EBBD83F-AB64-4248-87E6-B99F88EE5F88}">
     <text>Only one plant shutdown allowed</text>
   </threadedComment>
-  <threadedComment ref="A70" dT="2026-07-22T16:56:30.58" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+  <threadedComment ref="A71" dT="2026-07-22T16:56:30.58" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
     <text xml:space="preserve">Why is this so different from the other DR solution? I would assume they would be the same…
 </text>
   </threadedComment>
-  <threadedComment ref="A77" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
+  <threadedComment ref="A78" dT="2026-07-21T19:23:55.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{4644E393-F522-4E79-88BA-041770B595A7}">
     <text>Pretty sure this solution is wrong, but I don’t think I need this case for the paper</text>
   </threadedComment>
-  <threadedComment ref="A83" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+  <threadedComment ref="A84" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
     <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
   </threadedComment>
-  <threadedComment ref="T95" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="T96" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1368,21 +1371,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:V98"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:V99"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.61328125" customWidth="1"/>
-    <col min="3" max="3" width="11.4609375" customWidth="1"/>
-    <col min="5" max="5" width="10.23046875" customWidth="1"/>
-    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.69140625" customWidth="1"/>
-    <col min="9" max="9" width="9.07421875" customWidth="1"/>
-    <col min="15" max="15" width="9.53515625" customWidth="1"/>
-    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.84375" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" customWidth="1"/>
+    <col min="3" max="3" width="11.453125" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="15" max="15" width="9.54296875" customWidth="1"/>
+    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1393,7 +1396,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1461,7 +1464,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1525,7 +1528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1589,10 +1592,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1656,7 +1659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -1720,10 +1723,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1787,7 +1790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -1851,10 +1854,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -1918,7 +1921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -1982,10 +1985,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2047,7 +2050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2103,10 +2106,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2170,7 +2173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2234,7 +2237,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2243,7 +2246,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2254,7 +2257,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2318,10 +2321,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2385,7 +2388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2455,7 +2458,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="K26">
@@ -2463,7 +2466,7 @@
         <v>86355.755432219594</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2527,7 +2530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2591,10 +2594,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2658,7 +2661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -2728,7 +2731,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -2798,7 +2801,7 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="D33">
@@ -2878,7 +2881,7 @@
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="K34">
@@ -2886,14 +2889,14 @@
         <v>86355.755432219594</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -2957,7 +2960,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3021,12 +3024,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3093,7 +3096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3163,20 +3166,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3240,15 +3243,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3318,13 +3321,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
@@ -3388,7 +3391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
@@ -3452,11 +3455,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -3520,7 +3523,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -3584,10 +3587,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
@@ -3651,7 +3654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>22</v>
       </c>
@@ -3715,13 +3718,13 @@
         <v>0.51444695802960605</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -3732,8 +3735,8 @@
         <v>2</v>
       </c>
       <c r="D60">
-        <f>J60+K60+L60+M60+N60</f>
-        <v>119635.09208261623</v>
+        <f>J60+K60+L60+M60+N60-O60</f>
+        <v>116477.09498263198</v>
       </c>
       <c r="E60">
         <v>282495</v>
@@ -3769,8 +3772,8 @@
         <v>3157.9970999842499</v>
       </c>
       <c r="P60">
-        <f t="shared" ref="P60:P64" si="11">D60+$P$1</f>
-        <v>240194.76390161275</v>
+        <f t="shared" ref="P60:P63" si="11">D60+$P$1</f>
+        <v>237036.76680162852</v>
       </c>
       <c r="Q60">
         <v>1464.2687322859999</v>
@@ -3785,7 +3788,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -3850,7 +3853,7 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
         <v>22</v>
       </c>
@@ -3920,7 +3923,7 @@
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -3990,12 +3993,12 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A64" s="9" t="s">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A64" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B64" s="9"/>
-      <c r="C64" s="9"/>
+      <c r="B64" s="11"/>
+      <c r="C64" s="11"/>
       <c r="D64" s="10">
         <f>D63-D62</f>
         <v>486.66028698880109</v>
@@ -4073,326 +4076,268 @@
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A65" s="1" t="s">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A65" s="9"/>
+      <c r="B65" s="9"/>
+      <c r="C65" s="9"/>
+      <c r="D65" s="10"/>
+    </row>
+    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A66" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G65" s="4"/>
-    </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A66" s="3" t="s">
+      <c r="G66" s="4"/>
+    </row>
+    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A67" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B66" s="3" t="s">
+      <c r="B67" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C66" s="3">
-        <v>0</v>
-      </c>
-      <c r="G66" s="4"/>
-    </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A67" t="s">
+      <c r="C67" s="3">
+        <v>0</v>
+      </c>
+      <c r="G67" s="4"/>
+    </row>
+    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>22</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B68" t="s">
         <v>23</v>
       </c>
-      <c r="C67">
-        <v>0</v>
-      </c>
-      <c r="D67">
-        <f>J67+K67+L67+M67+N67-O67</f>
+      <c r="C68">
+        <v>0</v>
+      </c>
+      <c r="D68">
+        <f>J68+K68+L68+M68+N68-O68</f>
         <v>125093.23428318274</v>
       </c>
-      <c r="E67">
+      <c r="E68">
         <v>282190.859999999</v>
       </c>
-      <c r="F67">
+      <c r="F68">
         <v>0.86904083066499505</v>
       </c>
-      <c r="G67">
+      <c r="G68">
         <v>24203.497764766002</v>
       </c>
-      <c r="H67">
+      <c r="H68">
         <v>4932.7238161263904</v>
       </c>
-      <c r="I67">
+      <c r="I68">
         <v>9098.5748223234004</v>
       </c>
-      <c r="J67">
+      <c r="J68">
         <v>38234.796403215798</v>
       </c>
-      <c r="K67">
+      <c r="K68">
         <v>50845.200000000099</v>
       </c>
-      <c r="L67">
+      <c r="L68">
         <v>15304.405199999899</v>
       </c>
-      <c r="M67">
+      <c r="M68">
         <v>19298.29566</v>
       </c>
-      <c r="N67">
+      <c r="N68">
         <v>1409.83742959549</v>
       </c>
-      <c r="O67">
+      <c r="O68">
         <v>-0.69959037146548997</v>
       </c>
-      <c r="P67">
-        <f>D67+$P$1</f>
+      <c r="P68">
+        <f>D68+$P$1</f>
         <v>245652.90610217926</v>
       </c>
-      <c r="Q67">
+      <c r="Q68">
         <v>1102.0926609763501</v>
       </c>
-      <c r="R67">
-        <v>0</v>
-      </c>
-      <c r="U67">
+      <c r="R68">
+        <v>0</v>
+      </c>
+      <c r="U68">
         <v>15.5670440273115</v>
       </c>
-      <c r="V67">
+      <c r="V68">
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A68" s="3"/>
-      <c r="B68" s="3"/>
-      <c r="C68" s="3"/>
-      <c r="G68" s="4"/>
-    </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A69" s="3" t="s">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A69" s="3"/>
+      <c r="B69" s="3"/>
+      <c r="C69" s="3"/>
+      <c r="G69" s="4"/>
+    </row>
+    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A70" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B69" s="3" t="s">
+      <c r="B70" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C69" s="3">
+      <c r="C70" s="3">
         <v>4</v>
       </c>
-      <c r="G69" s="4"/>
-    </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A70" t="s">
+      <c r="G70" s="4"/>
+    </row>
+    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>22</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B71" t="s">
         <v>21</v>
       </c>
-      <c r="C70">
+      <c r="C71">
         <v>4</v>
       </c>
-      <c r="D70">
+      <c r="D71">
         <v>108832.74020782999</v>
       </c>
-      <c r="E70">
+      <c r="E71">
         <v>282179.67123306898</v>
       </c>
-      <c r="F70">
+      <c r="F71">
         <v>0.81644691741250097</v>
       </c>
-      <c r="G70">
+      <c r="G71">
         <v>19728.523245555101</v>
       </c>
-      <c r="H70">
+      <c r="H71">
         <v>6281.7321988746498</v>
       </c>
-      <c r="I70" s="8">
+      <c r="I71" s="8">
         <v>9.8877442286147301E-6</v>
       </c>
-      <c r="J70">
+      <c r="J71">
         <v>26010.255454317499</v>
       </c>
-      <c r="K70">
+      <c r="K71">
         <v>50944.9452054754</v>
       </c>
-      <c r="L70">
+      <c r="L71">
         <v>20235.614943009699</v>
       </c>
-      <c r="M70">
+      <c r="M71">
         <v>19962.024605027898</v>
       </c>
-      <c r="N70">
+      <c r="N71">
         <v>1462.3779549220301</v>
       </c>
-      <c r="O70">
+      <c r="O71">
         <v>8320.1</v>
       </c>
-      <c r="P70">
+      <c r="P71">
         <v>230384.72273471201</v>
       </c>
-      <c r="Q70">
+      <c r="Q71">
         <v>1403.49453592792</v>
       </c>
-      <c r="R70">
+      <c r="R71">
         <v>34518.506961381201</v>
       </c>
-      <c r="S70">
+      <c r="S71">
         <v>841.91480393612801</v>
       </c>
-      <c r="T70">
+      <c r="T71">
         <v>0.38784649209264499</v>
       </c>
-      <c r="U70">
+      <c r="U71">
         <v>38264.627438579002</v>
       </c>
-      <c r="V70">
+      <c r="V71">
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A71" s="5"/>
-      <c r="B71" s="5"/>
-      <c r="D71">
-        <f>D70-D67</f>
+    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A72" s="5"/>
+      <c r="B72" s="5"/>
+      <c r="D72">
+        <f>D71-D68</f>
         <v>-16260.494075352748</v>
       </c>
-      <c r="E71">
-        <f t="shared" ref="E71:V71" si="13">E70-E67</f>
+      <c r="E72">
+        <f t="shared" ref="E72:V72" si="13">E71-E68</f>
         <v>-11.188766930019483</v>
       </c>
-      <c r="F71">
+      <c r="F72">
         <f t="shared" si="13"/>
         <v>-5.2593913252494073E-2</v>
       </c>
-      <c r="G71">
+      <c r="G72">
         <f t="shared" si="13"/>
         <v>-4474.9745192109003</v>
       </c>
-      <c r="H71">
+      <c r="H72">
         <f t="shared" si="13"/>
         <v>1349.0083827482595</v>
       </c>
-      <c r="I71">
+      <c r="I72">
         <f t="shared" si="13"/>
         <v>-9098.574812435656</v>
       </c>
-      <c r="J71">
+      <c r="J72">
         <f t="shared" si="13"/>
         <v>-12224.540948898299</v>
       </c>
-      <c r="K71">
+      <c r="K72">
         <f t="shared" si="13"/>
         <v>99.745205475301191</v>
       </c>
-      <c r="L71">
+      <c r="L72">
         <f t="shared" si="13"/>
         <v>4931.2097430098001</v>
       </c>
-      <c r="M71">
+      <c r="M72">
         <f t="shared" si="13"/>
         <v>663.72894502789859</v>
       </c>
-      <c r="N71">
+      <c r="N72">
         <f t="shared" si="13"/>
         <v>52.540525326540092</v>
       </c>
-      <c r="O71">
+      <c r="O72">
         <f t="shared" si="13"/>
         <v>8320.7995903714655</v>
       </c>
-      <c r="P71">
+      <c r="P72">
         <f t="shared" si="13"/>
         <v>-15268.183367467253</v>
       </c>
-      <c r="Q71">
+      <c r="Q72">
         <f t="shared" si="13"/>
         <v>301.40187495156988</v>
       </c>
-      <c r="R71">
+      <c r="R72">
         <f t="shared" si="13"/>
         <v>34518.506961381201</v>
       </c>
-      <c r="S71">
+      <c r="S72">
         <f t="shared" si="13"/>
         <v>841.91480393612801</v>
       </c>
-      <c r="T71">
+      <c r="T72">
         <f t="shared" si="13"/>
         <v>0.38784649209264499</v>
       </c>
-      <c r="U71">
+      <c r="U72">
         <f t="shared" si="13"/>
         <v>38249.060394551692</v>
       </c>
-      <c r="V71">
+      <c r="V72">
         <f t="shared" si="13"/>
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A72" s="1" t="s">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A73" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A73" s="3" t="s">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A74" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C73">
-        <v>0</v>
-      </c>
-      <c r="D73">
-        <f>J73+K73+L73+M73+N73</f>
-        <v>116023.2890300647</v>
-      </c>
-      <c r="E73">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F73">
-        <v>0.83841249022441</v>
-      </c>
-      <c r="G73">
-        <v>20114.092712805999</v>
-      </c>
-      <c r="H73">
-        <v>6942.2846600808298</v>
-      </c>
-      <c r="I73">
-        <v>2530.0880681377598</v>
-      </c>
-      <c r="J73">
-        <v>29586.4654410246</v>
-      </c>
-      <c r="K73">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L73">
-        <v>15303.798385783</v>
-      </c>
-      <c r="M73">
-        <v>19297.5304894482</v>
-      </c>
-      <c r="N73">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O73">
-        <v>0</v>
-      </c>
-      <c r="P73">
-        <f t="shared" ref="P73:P74" si="14">D73+$P$1</f>
-        <v>236582.9608490612</v>
-      </c>
-      <c r="Q73">
-        <v>1101.8347602124099</v>
-      </c>
-      <c r="R73">
-        <v>0</v>
-      </c>
-      <c r="S73">
-        <v>0</v>
-      </c>
-      <c r="T73">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A74" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>23</v>
@@ -4402,34 +4347,34 @@
       </c>
       <c r="D74">
         <f>J74+K74+L74+M74+N74</f>
-        <v>125763.55741733511</v>
+        <v>116023.2890300647</v>
       </c>
       <c r="E74">
-        <v>282179.67125180899</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F74">
-        <v>0.87293045648394496</v>
+        <v>0.83841249022441</v>
       </c>
       <c r="G74">
-        <v>22626.697961956499</v>
+        <v>20114.092712805999</v>
       </c>
       <c r="H74">
-        <v>7102.5767129513297</v>
+        <v>6942.2846600808298</v>
       </c>
       <c r="I74">
-        <v>9597.4591384874802</v>
+        <v>2530.0880681377598</v>
       </c>
       <c r="J74">
-        <v>39326.733813395302</v>
+        <v>29586.4654410246</v>
       </c>
       <c r="K74">
-        <v>50843.184011688398</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L74">
-        <v>15303.798393134501</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M74">
-        <v>19297.530491231599</v>
+        <v>19297.5304894482</v>
       </c>
       <c r="N74">
         <v>992.31070788530405</v>
@@ -4438,88 +4383,94 @@
         <v>0</v>
       </c>
       <c r="P74">
+        <f t="shared" ref="P74:P75" si="14">D74+$P$1</f>
+        <v>236582.9608490612</v>
+      </c>
+      <c r="Q74">
+        <v>1101.8347602124099</v>
+      </c>
+      <c r="R74">
+        <v>0</v>
+      </c>
+      <c r="S74">
+        <v>0</v>
+      </c>
+      <c r="T74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A75" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C75">
+        <v>0</v>
+      </c>
+      <c r="D75">
+        <f>J75+K75+L75+M75+N75</f>
+        <v>125763.55741733511</v>
+      </c>
+      <c r="E75">
+        <v>282179.67125180899</v>
+      </c>
+      <c r="F75">
+        <v>0.87293045648394496</v>
+      </c>
+      <c r="G75">
+        <v>22626.697961956499</v>
+      </c>
+      <c r="H75">
+        <v>7102.5767129513297</v>
+      </c>
+      <c r="I75">
+        <v>9597.4591384874802</v>
+      </c>
+      <c r="J75">
+        <v>39326.733813395302</v>
+      </c>
+      <c r="K75">
+        <v>50843.184011688398</v>
+      </c>
+      <c r="L75">
+        <v>15303.798393134501</v>
+      </c>
+      <c r="M75">
+        <v>19297.530491231599</v>
+      </c>
+      <c r="N75">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O75">
+        <v>0</v>
+      </c>
+      <c r="P75">
         <f t="shared" si="14"/>
         <v>246323.22923633162</v>
       </c>
-      <c r="Q74">
+      <c r="Q75">
         <v>1127.27501714903</v>
       </c>
-      <c r="R74">
-        <v>0</v>
-      </c>
-      <c r="S74">
-        <v>0</v>
-      </c>
-      <c r="T74">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A75" s="1"/>
-    </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A76" t="s">
+      <c r="R75">
+        <v>0</v>
+      </c>
+      <c r="S75">
+        <v>0</v>
+      </c>
+      <c r="T75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A76" s="1"/>
+    </row>
+    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
         <v>20</v>
       </c>
-      <c r="B76" t="s">
-        <v>21</v>
-      </c>
-      <c r="C76">
-        <v>2</v>
-      </c>
-      <c r="D76">
-        <f>J76+K76+L76+M76+N76</f>
-        <v>116706.4157905087</v>
-      </c>
-      <c r="E76">
-        <v>282179.67125387199</v>
-      </c>
-      <c r="F76">
-        <v>0.840833383054163</v>
-      </c>
-      <c r="G76" s="4">
-        <v>20578.507216446698</v>
-      </c>
-      <c r="H76">
-        <v>7102.57515066207</v>
-      </c>
-      <c r="I76">
-        <v>2588.5052959285099</v>
-      </c>
-      <c r="J76">
-        <v>30269.587663037299</v>
-      </c>
-      <c r="K76">
-        <v>50843.185173268597</v>
-      </c>
-      <c r="L76">
-        <v>15303.8015139941</v>
-      </c>
-      <c r="M76">
-        <v>19297.530732323401</v>
-      </c>
-      <c r="N76">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O76">
-        <v>0</v>
-      </c>
-      <c r="P76">
-        <f t="shared" ref="P76:P77" si="15">D76+$P$1</f>
-        <v>237266.08760950522</v>
-      </c>
-      <c r="Q76">
-        <v>1127.2750356983099</v>
-      </c>
-      <c r="R76">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A77" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" t="s">
         <v>21</v>
       </c>
       <c r="C77">
@@ -4527,119 +4478,119 @@
       </c>
       <c r="D77">
         <f>J77+K77+L77+M77+N77</f>
+        <v>116706.4157905087</v>
+      </c>
+      <c r="E77">
+        <v>282179.67125387199</v>
+      </c>
+      <c r="F77">
+        <v>0.840833383054163</v>
+      </c>
+      <c r="G77" s="4">
+        <v>20578.507216446698</v>
+      </c>
+      <c r="H77">
+        <v>7102.57515066207</v>
+      </c>
+      <c r="I77">
+        <v>2588.5052959285099</v>
+      </c>
+      <c r="J77">
+        <v>30269.587663037299</v>
+      </c>
+      <c r="K77">
+        <v>50843.185173268597</v>
+      </c>
+      <c r="L77">
+        <v>15303.8015139941</v>
+      </c>
+      <c r="M77">
+        <v>19297.530732323401</v>
+      </c>
+      <c r="N77">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O77">
+        <v>0</v>
+      </c>
+      <c r="P77">
+        <f t="shared" ref="P77:P78" si="15">D77+$P$1</f>
+        <v>237266.08760950522</v>
+      </c>
+      <c r="Q77">
+        <v>1127.2750356983099</v>
+      </c>
+      <c r="R77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A78" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C78">
+        <v>2</v>
+      </c>
+      <c r="D78">
+        <f>J78+K78+L78+M78+N78</f>
         <v>121633.35860365373</v>
       </c>
-      <c r="E77">
+      <c r="E78">
         <v>282179.67123287602</v>
       </c>
-      <c r="F77">
+      <c r="F78">
         <v>0.85824890324911396</v>
       </c>
-      <c r="G77" s="4">
+      <c r="G78" s="4">
         <v>20824.7129679639</v>
       </c>
-      <c r="H77">
+      <c r="H78">
         <v>7456.39074483072</v>
       </c>
-      <c r="I77">
+      <c r="I78">
         <v>5114.4587365303096</v>
       </c>
-      <c r="J77">
+      <c r="J78">
         <v>33395.562449324898</v>
       </c>
-      <c r="K77">
+      <c r="K78">
         <v>51302.320205525801</v>
       </c>
-      <c r="L77">
+      <c r="L78">
         <v>16537.7269222135</v>
       </c>
-      <c r="M77">
+      <c r="M78">
         <v>19392.801250865799</v>
       </c>
-      <c r="N77">
+      <c r="N78">
         <v>1004.9477757237401</v>
       </c>
-      <c r="O77">
-        <v>0</v>
-      </c>
-      <c r="P77">
+      <c r="O78">
+        <v>0</v>
+      </c>
+      <c r="P78">
         <f t="shared" si="15"/>
         <v>242193.03042265025</v>
       </c>
-      <c r="Q77">
+      <c r="Q78">
         <v>1183.4303612998101</v>
       </c>
-      <c r="R77">
+      <c r="R78">
         <v>15931.1957490451</v>
       </c>
-      <c r="S77">
+      <c r="S78">
         <v>346.33034237054602</v>
       </c>
-      <c r="T77">
+      <c r="T78">
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A79" t="s">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
         <v>20</v>
-      </c>
-      <c r="B79" t="s">
-        <v>21</v>
-      </c>
-      <c r="C79">
-        <v>4</v>
-      </c>
-      <c r="D79">
-        <f>J79+K79+L79+M79+N79</f>
-        <v>116706.4157905051</v>
-      </c>
-      <c r="E79">
-        <v>282179.671253876</v>
-      </c>
-      <c r="F79">
-        <v>0.84083338305413902</v>
-      </c>
-      <c r="G79" s="4">
-        <v>20578.5072164468</v>
-      </c>
-      <c r="H79">
-        <v>7102.5751506616798</v>
-      </c>
-      <c r="I79">
-        <v>2588.50529592865</v>
-      </c>
-      <c r="J79">
-        <v>30269.587663037099</v>
-      </c>
-      <c r="K79">
-        <v>50843.185173268197</v>
-      </c>
-      <c r="L79">
-        <v>15303.8015139912</v>
-      </c>
-      <c r="M79">
-        <v>19297.530732323299</v>
-      </c>
-      <c r="N79">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O79">
-        <v>0</v>
-      </c>
-      <c r="P79">
-        <f t="shared" ref="P79:P81" si="16">D79+$P$1</f>
-        <v>237266.08760950161</v>
-      </c>
-      <c r="Q79">
-        <v>1127.2750356983499</v>
-      </c>
-      <c r="R79">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A80" t="s">
-        <v>22</v>
       </c>
       <c r="B80" t="s">
         <v>21</v>
@@ -4649,834 +4600,892 @@
       </c>
       <c r="D80">
         <f>J80+K80+L80+M80+N80</f>
+        <v>116706.4157905051</v>
+      </c>
+      <c r="E80">
+        <v>282179.671253876</v>
+      </c>
+      <c r="F80">
+        <v>0.84083338305413902</v>
+      </c>
+      <c r="G80" s="4">
+        <v>20578.5072164468</v>
+      </c>
+      <c r="H80">
+        <v>7102.5751506616798</v>
+      </c>
+      <c r="I80">
+        <v>2588.50529592865</v>
+      </c>
+      <c r="J80">
+        <v>30269.587663037099</v>
+      </c>
+      <c r="K80">
+        <v>50843.185173268197</v>
+      </c>
+      <c r="L80">
+        <v>15303.8015139912</v>
+      </c>
+      <c r="M80">
+        <v>19297.530732323299</v>
+      </c>
+      <c r="N80">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O80">
+        <v>0</v>
+      </c>
+      <c r="P80">
+        <f t="shared" ref="P80:P82" si="16">D80+$P$1</f>
+        <v>237266.08760950161</v>
+      </c>
+      <c r="Q80">
+        <v>1127.2750356983499</v>
+      </c>
+      <c r="R80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>22</v>
+      </c>
+      <c r="B81" t="s">
+        <v>21</v>
+      </c>
+      <c r="C81">
+        <v>4</v>
+      </c>
+      <c r="D81">
+        <f>J81+K81+L81+M81+N81</f>
         <v>121744.79706913032</v>
       </c>
-      <c r="E80">
+      <c r="E81">
         <v>282179.88376308198</v>
       </c>
-      <c r="F80">
+      <c r="F81">
         <v>0.85713546401894802</v>
       </c>
-      <c r="G80">
+      <c r="G81">
         <v>21291.5607898614</v>
       </c>
-      <c r="H80">
+      <c r="H81">
         <v>7432.3603175362596</v>
       </c>
-      <c r="I80">
+      <c r="I81">
         <v>5035.2758648834497</v>
       </c>
-      <c r="J80">
+      <c r="J81">
         <v>33759.196972281097</v>
       </c>
-      <c r="K80">
+      <c r="K81">
         <v>51128.3645002267</v>
       </c>
-      <c r="L80">
+      <c r="L81">
         <v>16070.129576240101</v>
       </c>
-      <c r="M80">
+      <c r="M81">
         <v>19356.7120304526</v>
       </c>
-      <c r="N80">
+      <c r="N81">
         <v>1430.39398992981</v>
       </c>
-      <c r="O80">
-        <v>0</v>
-      </c>
-      <c r="P80">
+      <c r="O81">
+        <v>0</v>
+      </c>
+      <c r="P81">
         <f t="shared" si="16"/>
         <v>242304.46888812684</v>
       </c>
-      <c r="Q80">
+      <c r="Q81">
         <v>1179.61640190856</v>
       </c>
-      <c r="R80">
+      <c r="R81">
         <v>13411.4010346792</v>
       </c>
-      <c r="S80">
+      <c r="S81">
         <v>478.97860838140201</v>
       </c>
-      <c r="T80">
+      <c r="T81">
         <v>0.22564405635506199</v>
       </c>
-      <c r="U80">
+      <c r="U81">
         <v>10550.3210016294</v>
       </c>
-      <c r="V80">
+      <c r="V81">
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="D81">
-        <f>D80-D74</f>
+    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="D82">
+        <f>D81-D75</f>
         <v>-4018.7603482047853</v>
       </c>
-      <c r="E81">
-        <f t="shared" ref="E81:N81" si="17">E80-E74</f>
+      <c r="E82">
+        <f t="shared" ref="E82:N82" si="17">E81-E75</f>
         <v>0.21251127298455685</v>
       </c>
-      <c r="F81">
+      <c r="F82">
         <f t="shared" si="17"/>
         <v>-1.5794992464996938E-2</v>
       </c>
-      <c r="G81">
+      <c r="G82">
         <f t="shared" si="17"/>
         <v>-1335.1371720950992</v>
       </c>
-      <c r="H81">
+      <c r="H82">
         <f t="shared" si="17"/>
         <v>329.78360458492989</v>
       </c>
-      <c r="I81">
+      <c r="I82">
         <f t="shared" si="17"/>
         <v>-4562.1832736040305</v>
       </c>
-      <c r="J81">
+      <c r="J82">
         <f t="shared" si="17"/>
         <v>-5567.5368411142044</v>
       </c>
-      <c r="K81">
+      <c r="K82">
         <f t="shared" si="17"/>
         <v>285.1804885383026</v>
       </c>
-      <c r="L81">
+      <c r="L82">
         <f t="shared" si="17"/>
         <v>766.33118310559985</v>
       </c>
-      <c r="M81">
+      <c r="M82">
         <f t="shared" si="17"/>
         <v>59.181539221001003</v>
       </c>
-      <c r="N81">
+      <c r="N82">
         <f t="shared" si="17"/>
         <v>438.08328204450595</v>
       </c>
-      <c r="P81">
+      <c r="P82">
         <f t="shared" si="16"/>
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A82" s="1" t="s">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A83" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G82" s="4"/>
-    </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A83" t="s">
-        <v>22</v>
-      </c>
-      <c r="B83" t="s">
-        <v>21</v>
-      </c>
-      <c r="C83">
-        <v>4</v>
-      </c>
-      <c r="D83">
-        <f>J83+K83+L83+M83+N83</f>
-        <v>147118.48206815872</v>
-      </c>
-      <c r="E83">
-        <v>355610.364944759</v>
-      </c>
-      <c r="F83">
-        <v>0.75267772890587503</v>
-      </c>
-      <c r="G83">
-        <v>25765.651662743599</v>
-      </c>
-      <c r="H83">
-        <v>7150.9042815892099</v>
-      </c>
-      <c r="I83">
-        <v>5144.3184852884797</v>
-      </c>
-      <c r="J83">
-        <v>38060.874429621297</v>
-      </c>
-      <c r="K83">
-        <v>64168.339029134899</v>
-      </c>
-      <c r="L83">
-        <v>19539.954214541001</v>
-      </c>
-      <c r="M83">
-        <v>24338.851661831999</v>
-      </c>
-      <c r="N83">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O83">
-        <v>0</v>
-      </c>
-      <c r="P83">
-        <f t="shared" ref="P83" si="18">D83+$P$1</f>
-        <v>267678.15388715523</v>
-      </c>
-      <c r="Q83">
-        <v>1597.68911089628</v>
-      </c>
-      <c r="R83">
-        <v>13084.0423994256</v>
-      </c>
-      <c r="S83">
-        <v>467.28722855091399</v>
-      </c>
-      <c r="T83">
-        <v>-0.25904927491985202</v>
-      </c>
-    </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="G83" s="4"/>
+    </row>
+    <row r="84" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>22</v>
       </c>
       <c r="B84" t="s">
+        <v>21</v>
+      </c>
+      <c r="C84">
+        <v>4</v>
+      </c>
+      <c r="D84">
+        <f>J84+K84+L84+M84+N84</f>
+        <v>147118.48206815872</v>
+      </c>
+      <c r="E84">
+        <v>355610.364944759</v>
+      </c>
+      <c r="F84">
+        <v>0.75267772890587503</v>
+      </c>
+      <c r="G84">
+        <v>25765.651662743599</v>
+      </c>
+      <c r="H84">
+        <v>7150.9042815892099</v>
+      </c>
+      <c r="I84">
+        <v>5144.3184852884797</v>
+      </c>
+      <c r="J84">
+        <v>38060.874429621297</v>
+      </c>
+      <c r="K84">
+        <v>64168.339029134899</v>
+      </c>
+      <c r="L84">
+        <v>19539.954214541001</v>
+      </c>
+      <c r="M84">
+        <v>24338.851661831999</v>
+      </c>
+      <c r="N84">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O84">
+        <v>0</v>
+      </c>
+      <c r="P84">
+        <f t="shared" ref="P84" si="18">D84+$P$1</f>
+        <v>267678.15388715523</v>
+      </c>
+      <c r="Q84">
+        <v>1597.68911089628</v>
+      </c>
+      <c r="R84">
+        <v>13084.0423994256</v>
+      </c>
+      <c r="S84">
+        <v>467.28722855091399</v>
+      </c>
+      <c r="T84">
+        <v>-0.25904927491985202</v>
+      </c>
+    </row>
+    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>22</v>
+      </c>
+      <c r="B85" t="s">
         <v>35</v>
       </c>
-      <c r="C84" t="s">
+      <c r="C85" t="s">
         <v>35</v>
       </c>
-      <c r="D84" t="s">
+      <c r="D85" t="s">
         <v>36</v>
       </c>
-      <c r="E84" t="s">
+      <c r="E85" t="s">
         <v>36</v>
       </c>
-      <c r="F84" t="s">
+      <c r="F85" t="s">
         <v>36</v>
       </c>
-      <c r="G84" s="4">
+      <c r="G85" s="4">
         <v>28838</v>
       </c>
-      <c r="H84">
+      <c r="H85">
         <v>7567.5</v>
       </c>
-      <c r="I84">
+      <c r="I85">
         <v>13764.1</v>
       </c>
-      <c r="J84">
+      <c r="J85">
         <v>50169.7</v>
       </c>
-      <c r="K84" t="s">
+      <c r="K85" t="s">
         <v>36</v>
       </c>
-      <c r="L84" t="s">
+      <c r="L85" t="s">
         <v>36</v>
       </c>
-      <c r="M84" t="s">
+      <c r="M85" t="s">
         <v>36</v>
       </c>
-      <c r="N84" t="s">
+      <c r="N85" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="86" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A86" s="1" t="s">
+    <row r="87" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A87" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G86" s="4"/>
-      <c r="P86" t="s">
+      <c r="G87" s="4"/>
+      <c r="P87" t="s">
         <v>15</v>
       </c>
-      <c r="Q86" t="s">
+      <c r="Q87" t="s">
         <v>16</v>
       </c>
-      <c r="R86" t="s">
+      <c r="R87" t="s">
         <v>17</v>
       </c>
-      <c r="S86" t="s">
+      <c r="S87" t="s">
         <v>18</v>
       </c>
-      <c r="T86" t="s">
+      <c r="T87" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="87" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A87" t="s">
-        <v>0</v>
-      </c>
-      <c r="B87" t="s">
+    <row r="88" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B88" t="s">
         <v>1</v>
       </c>
-      <c r="C87" t="s">
+      <c r="C88" t="s">
         <v>2</v>
       </c>
-      <c r="D87" t="s">
+      <c r="D88" t="s">
         <v>3</v>
       </c>
-      <c r="E87" t="s">
+      <c r="E88" t="s">
         <v>4</v>
       </c>
-      <c r="F87" t="s">
+      <c r="F88" t="s">
         <v>5</v>
       </c>
-      <c r="G87" s="4" t="s">
+      <c r="G88" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H87" t="s">
+      <c r="H88" t="s">
         <v>7</v>
       </c>
-      <c r="I87" t="s">
+      <c r="I88" t="s">
         <v>8</v>
       </c>
-      <c r="J87" t="s">
+      <c r="J88" t="s">
         <v>9</v>
       </c>
-      <c r="K87" t="s">
+      <c r="K88" t="s">
         <v>10</v>
       </c>
-      <c r="L87" t="s">
+      <c r="L88" t="s">
         <v>11</v>
       </c>
-      <c r="M87" t="s">
+      <c r="M88" t="s">
         <v>12</v>
       </c>
-      <c r="N87" t="s">
+      <c r="N88" t="s">
         <v>13</v>
       </c>
-      <c r="O87" t="s">
+      <c r="O88" t="s">
         <v>14</v>
       </c>
-      <c r="P87">
+      <c r="P88">
         <v>63734.6679</v>
       </c>
-      <c r="Q87">
+      <c r="Q88">
         <v>1078.4492829999999</v>
       </c>
-      <c r="R87">
+      <c r="R88">
         <v>624.70352849999995</v>
       </c>
-      <c r="S87">
+      <c r="S88">
         <v>13.014656840000001</v>
       </c>
-      <c r="T87">
+      <c r="T88">
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="88" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A88" s="2" t="s">
+    <row r="89" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A89" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B89" t="s">
         <v>21</v>
       </c>
-      <c r="C88">
+      <c r="C89">
         <v>4</v>
       </c>
-      <c r="D88">
+      <c r="D89">
         <v>29525.427309999999</v>
       </c>
-      <c r="E88">
+      <c r="E89">
         <v>80391.755990000005</v>
       </c>
-      <c r="F88">
+      <c r="F89">
         <v>0.79280104200000001</v>
       </c>
-      <c r="G88" s="4">
+      <c r="G89" s="4">
         <v>5050.6365619999997</v>
       </c>
-      <c r="H88">
+      <c r="H89">
         <v>4678.3390820000004</v>
       </c>
-      <c r="I88">
+      <c r="I89">
         <v>2508.6600360000002</v>
       </c>
-      <c r="J88">
+      <c r="J89">
         <v>12237.635679999999</v>
       </c>
-      <c r="K88">
+      <c r="K89">
         <v>13920</v>
       </c>
-      <c r="L88">
+      <c r="L89">
         <v>2841.544922</v>
       </c>
-      <c r="M88">
+      <c r="M89">
         <v>5380.5444360000001</v>
       </c>
-      <c r="N88">
+      <c r="N89">
         <v>279.27307350000001</v>
       </c>
-      <c r="O88">
-        <v>0</v>
-      </c>
-      <c r="P88">
+      <c r="O89">
+        <v>0</v>
+      </c>
+      <c r="P89">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q88">
+      <c r="Q89">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R88">
+      <c r="R89">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S88">
+      <c r="S89">
         <v>452.7322633</v>
       </c>
-      <c r="T88">
+      <c r="T89">
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A89" s="7" t="s">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A90" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A91" t="s">
+    <row r="92" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
         <v>32</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B92" t="s">
         <v>33</v>
       </c>
-      <c r="C91" t="s">
+      <c r="C92" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A92">
-        <v>20</v>
-      </c>
-      <c r="B92">
-        <v>60</v>
-      </c>
-      <c r="C92">
-        <v>2</v>
-      </c>
-      <c r="D92">
-        <f t="shared" ref="D92:D98" si="19">J92+K92+L92+M92+N92</f>
-        <v>120712.69088313227</v>
-      </c>
-      <c r="E92">
-        <v>282179.67123285501</v>
-      </c>
-      <c r="F92">
-        <v>0.854946898908852</v>
-      </c>
-      <c r="G92">
-        <v>18681.222424938602</v>
-      </c>
-      <c r="H92">
-        <v>5354.6114985546601</v>
-      </c>
-      <c r="I92">
-        <v>8156.08309050551</v>
-      </c>
-      <c r="J92">
-        <v>32191.917013998798</v>
-      </c>
-      <c r="K92">
-        <v>51372.124296964801</v>
-      </c>
-      <c r="L92">
-        <v>16725.325417965501</v>
-      </c>
-      <c r="M92">
-        <v>19407.285599838699</v>
-      </c>
-      <c r="N92">
-        <v>1016.03855436447</v>
-      </c>
-      <c r="O92">
-        <v>0</v>
-      </c>
-      <c r="P92">
-        <f t="shared" ref="P92:P98" si="20">D92+$P$1</f>
-        <v>241272.36270212877</v>
-      </c>
-      <c r="Q92">
-        <v>1192.7637589594799</v>
-      </c>
-      <c r="R92">
-        <v>19736.206339365101</v>
-      </c>
-      <c r="S92">
-        <v>481.37088632597801</v>
-      </c>
-      <c r="T92" s="6">
-        <v>0.12591688076390301</v>
-      </c>
-    </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>20</v>
       </c>
       <c r="B93">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C93">
         <v>2</v>
       </c>
       <c r="D93">
+        <f t="shared" ref="D93:D99" si="19">J93+K93+L93+M93+N93</f>
+        <v>120712.69088313227</v>
+      </c>
+      <c r="E93">
+        <v>282179.67123285501</v>
+      </c>
+      <c r="F93">
+        <v>0.854946898908852</v>
+      </c>
+      <c r="G93">
+        <v>18681.222424938602</v>
+      </c>
+      <c r="H93">
+        <v>5354.6114985546601</v>
+      </c>
+      <c r="I93">
+        <v>8156.08309050551</v>
+      </c>
+      <c r="J93">
+        <v>32191.917013998798</v>
+      </c>
+      <c r="K93">
+        <v>51372.124296964801</v>
+      </c>
+      <c r="L93">
+        <v>16725.325417965501</v>
+      </c>
+      <c r="M93">
+        <v>19407.285599838699</v>
+      </c>
+      <c r="N93">
+        <v>1016.03855436447</v>
+      </c>
+      <c r="O93">
+        <v>0</v>
+      </c>
+      <c r="P93">
+        <f t="shared" ref="P93:P99" si="20">D93+$P$1</f>
+        <v>241272.36270212877</v>
+      </c>
+      <c r="Q93">
+        <v>1192.7637589594799</v>
+      </c>
+      <c r="R93">
+        <v>19736.206339365101</v>
+      </c>
+      <c r="S93">
+        <v>481.37088632597801</v>
+      </c>
+      <c r="T93" s="6">
+        <v>0.12591688076390301</v>
+      </c>
+    </row>
+    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A94">
+        <v>20</v>
+      </c>
+      <c r="B94">
+        <v>50</v>
+      </c>
+      <c r="C94">
+        <v>2</v>
+      </c>
+      <c r="D94">
         <f t="shared" si="19"/>
         <v>119392.42354269064</v>
       </c>
-      <c r="E93">
+      <c r="E94">
         <v>282254.81855225202</v>
       </c>
-      <c r="F93">
+      <c r="F94">
         <v>0.85006146065890897</v>
       </c>
-      <c r="G93">
+      <c r="G94">
         <v>19407.840072768398</v>
       </c>
-      <c r="H93">
+      <c r="H94">
         <v>5891.8301217549197</v>
       </c>
-      <c r="I93">
+      <c r="I94">
         <v>6659.4942697455399</v>
       </c>
-      <c r="J93">
+      <c r="J94">
         <v>31959.164464268899</v>
       </c>
-      <c r="K93">
+      <c r="K94">
         <v>51102.045942938203</v>
       </c>
-      <c r="L93">
+      <c r="L94">
         <v>15967.176494174801</v>
       </c>
-      <c r="M93">
+      <c r="M94">
         <v>19353.573908279199</v>
       </c>
-      <c r="N93">
+      <c r="N94">
         <v>1010.46273302954</v>
       </c>
-      <c r="O93">
-        <v>0</v>
-      </c>
-      <c r="P93">
+      <c r="O94">
+        <v>0</v>
+      </c>
+      <c r="P94">
         <f t="shared" si="20"/>
         <v>239952.09536168716</v>
       </c>
-      <c r="Q93">
+      <c r="Q94">
         <v>1312.43161993582</v>
       </c>
-      <c r="R93">
+      <c r="R94">
         <v>18377.616631847999</v>
       </c>
-      <c r="S93">
+      <c r="S94">
         <v>459.4404157962</v>
       </c>
-      <c r="T93" s="6">
+      <c r="T94" s="6">
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A94">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A95">
         <v>20</v>
       </c>
-      <c r="B94">
+      <c r="B95">
         <v>40</v>
       </c>
-      <c r="C94">
+      <c r="C95">
         <v>2</v>
       </c>
-      <c r="D94">
+      <c r="D95">
         <f t="shared" si="19"/>
         <v>117777.02945340994</v>
       </c>
-      <c r="E94">
+      <c r="E95">
         <v>282179.67123287299</v>
       </c>
-      <c r="F94">
+      <c r="F95">
         <v>0.84456314023622803</v>
       </c>
-      <c r="G94">
+      <c r="G95">
         <v>19298.245593088301</v>
       </c>
-      <c r="H94">
+      <c r="H95">
         <v>5682.0016560700296</v>
       </c>
-      <c r="I94">
+      <c r="I95">
         <v>5350.3346939491703</v>
       </c>
-      <c r="J94">
+      <c r="J95">
         <v>30330.5819431075</v>
       </c>
-      <c r="K94">
+      <c r="K95">
         <v>51097.733915068202</v>
       </c>
-      <c r="L94">
+      <c r="L95">
         <v>15987.901266609</v>
       </c>
-      <c r="M94">
+      <c r="M95">
         <v>19350.349595595701</v>
       </c>
-      <c r="N94">
+      <c r="N95">
         <v>1010.46273302954</v>
       </c>
-      <c r="O94">
-        <v>0</v>
-      </c>
-      <c r="P94">
+      <c r="O95">
+        <v>0</v>
+      </c>
+      <c r="P95">
         <f t="shared" si="20"/>
         <v>238336.70127240644</v>
       </c>
-      <c r="Q94">
+      <c r="Q95">
         <v>1265.6913868611</v>
       </c>
-      <c r="R94">
+      <c r="R95">
         <v>17746.163883660702</v>
       </c>
-      <c r="S94">
+      <c r="S95">
         <v>507.03325381887902</v>
       </c>
-      <c r="T94" s="6">
+      <c r="T95" s="6">
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A95">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A96">
         <v>20</v>
       </c>
-      <c r="B95">
+      <c r="B96">
         <v>30</v>
       </c>
-      <c r="C95">
+      <c r="C96">
         <v>2</v>
       </c>
-      <c r="D95">
+      <c r="D96">
         <f t="shared" si="19"/>
         <v>116625.1695160947</v>
       </c>
-      <c r="E95">
+      <c r="E96">
         <v>282182.50548365602</v>
       </c>
-      <c r="F95">
+      <c r="F96">
         <v>0.84045954058697003</v>
       </c>
-      <c r="G95">
+      <c r="G96">
         <v>19302.752565837702</v>
       </c>
-      <c r="H95">
+      <c r="H96">
         <v>6226.5181629292701</v>
       </c>
-      <c r="I95">
+      <c r="I96">
         <v>3974.5318253822402</v>
       </c>
-      <c r="J95">
+      <c r="J96">
         <v>29503.802554149199</v>
       </c>
-      <c r="K95">
+      <c r="K96">
         <v>51013.610661725899</v>
       </c>
-      <c r="L95">
+      <c r="L96">
         <v>15760.601295416</v>
       </c>
-      <c r="M95">
+      <c r="M96">
         <v>19332.981882301501</v>
       </c>
-      <c r="N95">
+      <c r="N96">
         <v>1014.17312250211</v>
       </c>
-      <c r="O95">
-        <v>0</v>
-      </c>
-      <c r="P95">
+      <c r="O96">
+        <v>0</v>
+      </c>
+      <c r="P96">
         <f t="shared" si="20"/>
         <v>237184.84133509122</v>
       </c>
-      <c r="Q95">
+      <c r="Q96">
         <v>1386.9848841974899</v>
       </c>
-      <c r="R95">
+      <c r="R96">
         <v>18436.445202769701</v>
       </c>
-      <c r="S95">
+      <c r="S96">
         <v>209.50505912238299</v>
       </c>
-      <c r="T95" s="6">
+      <c r="T96" s="6">
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A96" s="3">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A97" s="3">
         <v>20</v>
       </c>
-      <c r="B96" s="3">
+      <c r="B97" s="3">
         <v>20</v>
       </c>
-      <c r="C96" s="3">
+      <c r="C97" s="3">
         <v>2</v>
       </c>
-      <c r="D96">
+      <c r="D97">
         <f t="shared" si="19"/>
         <v>115198.459983006</v>
       </c>
-      <c r="E96">
+      <c r="E97">
         <v>282179.67123297497</v>
       </c>
-      <c r="F96">
+      <c r="F97">
         <v>0.83541194997266699</v>
       </c>
-      <c r="G96">
+      <c r="G97">
         <v>19351.2255529412</v>
       </c>
-      <c r="H96">
+      <c r="H97">
         <v>6002.0469674603501</v>
       </c>
-      <c r="I96">
+      <c r="I97">
         <v>2645.4376652921501</v>
       </c>
-      <c r="J96">
+      <c r="J97">
         <v>27998.710185693701</v>
       </c>
-      <c r="K96">
+      <c r="K97">
         <v>51033.4442867088</v>
       </c>
-      <c r="L96">
+      <c r="L97">
         <v>15815.1228903871</v>
       </c>
-      <c r="M96">
+      <c r="M97">
         <v>19337.009497714302</v>
       </c>
-      <c r="N96">
+      <c r="N97">
         <v>1014.17312250211</v>
       </c>
-      <c r="O96">
-        <v>0</v>
-      </c>
-      <c r="P96">
+      <c r="O97">
+        <v>0</v>
+      </c>
+      <c r="P97">
         <f t="shared" si="20"/>
         <v>235758.13180200252</v>
       </c>
-      <c r="Q96">
+      <c r="Q97">
         <v>1336.98290493166</v>
       </c>
-      <c r="R96">
+      <c r="R97">
         <v>18577.307877855899</v>
       </c>
-      <c r="S96">
+      <c r="S97">
         <v>432.030415764091</v>
       </c>
-      <c r="T96" s="6">
+      <c r="T97" s="6">
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A97">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A98">
         <v>20</v>
       </c>
-      <c r="B97">
+      <c r="B98">
         <v>15</v>
       </c>
-      <c r="C97">
+      <c r="C98">
         <v>2</v>
       </c>
-      <c r="D97">
+      <c r="D98">
         <f t="shared" si="19"/>
         <v>114451.25872361983</v>
       </c>
-      <c r="E97">
+      <c r="E98">
         <v>282179.67123267101</v>
       </c>
-      <c r="F97">
+      <c r="F98">
         <v>0.83277713625127903</v>
       </c>
-      <c r="G97">
+      <c r="G98">
         <v>19390.977969205</v>
       </c>
-      <c r="H97">
+      <c r="H98">
         <v>5599.5405456203798</v>
       </c>
-      <c r="I97">
+      <c r="I98">
         <v>2128.1287863747102</v>
       </c>
-      <c r="J97">
+      <c r="J98">
         <v>27118.647301200101</v>
       </c>
-      <c r="K97">
+      <c r="K98">
         <v>51068.507704320902</v>
       </c>
-      <c r="L97">
+      <c r="L98">
         <v>15909.3558282099</v>
       </c>
-      <c r="M97">
+      <c r="M98">
         <v>19344.285156859401</v>
       </c>
-      <c r="N97">
+      <c r="N98">
         <v>1010.46273302954</v>
       </c>
-      <c r="O97">
-        <v>0</v>
-      </c>
-      <c r="P97">
+      <c r="O98">
+        <v>0</v>
+      </c>
+      <c r="P98">
         <f t="shared" si="20"/>
         <v>235010.93054261635</v>
       </c>
-      <c r="Q97">
+      <c r="Q98">
         <v>1247.3228025527501</v>
       </c>
-      <c r="R97">
+      <c r="R98">
         <v>16417.502561416801</v>
       </c>
-      <c r="S97">
+      <c r="S98">
         <v>469.07150175476602</v>
       </c>
-      <c r="T97" s="6">
+      <c r="T98" s="6">
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A98">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A99">
         <v>20</v>
       </c>
-      <c r="B98">
+      <c r="B99">
         <v>12</v>
       </c>
-      <c r="C98">
+      <c r="C99">
         <v>2</v>
       </c>
-      <c r="D98">
+      <c r="D99">
         <f t="shared" si="19"/>
         <v>114787.7594081375</v>
       </c>
-      <c r="E98">
+      <c r="E99">
         <v>282179.67123287602</v>
       </c>
-      <c r="F98">
+      <c r="F99">
         <v>0.83403396920434802</v>
       </c>
-      <c r="G98">
+      <c r="G99">
         <v>20436.472361711199</v>
       </c>
-      <c r="H98">
+      <c r="H99">
         <v>4946.5396722567002</v>
       </c>
-      <c r="I98">
+      <c r="I99">
         <v>2967.9237851293901</v>
       </c>
-      <c r="J98">
+      <c r="J99">
         <v>28350.9358190973</v>
       </c>
-      <c r="K98">
+      <c r="K99">
         <v>50843.184005923598</v>
       </c>
-      <c r="L98">
+      <c r="L99">
         <v>15303.798385783</v>
       </c>
-      <c r="M98">
+      <c r="M99">
         <v>19297.530489448302</v>
       </c>
-      <c r="N98">
+      <c r="N99">
         <v>992.31070788530405</v>
       </c>
-      <c r="O98">
-        <v>0</v>
-      </c>
-      <c r="P98">
+      <c r="O99">
+        <v>0</v>
+      </c>
+      <c r="P99">
         <f t="shared" si="20"/>
         <v>235347.43122713402</v>
       </c>
-      <c r="Q98">
+      <c r="Q99">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R98">
+      <c r="R99">
         <v>13.380488321454299</v>
       </c>
-      <c r="S98">
+      <c r="S99">
         <v>2.67609766429086</v>
       </c>
-      <c r="T98" s="6">
+      <c r="T99" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>

</xml_diff>

<commit_message>
testing result with only one forced shutdown
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E100DDC-5ADE-4EE0-A35A-79A2F83459B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2E049B6-A2C8-4593-8E7F-51E288AB2F85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="10680" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
+    <sheet name="Understanding DR Result" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -246,8 +247,113 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={D913FCAB-030D-49E3-A7A0-5803B7027754}</author>
+    <author>tc={59DFC78E-5F9D-4D05-9892-2664283F148D}</author>
+    <author>tc={5DA58C15-B5CA-4552-8F53-D4819003ECD4}</author>
+    <author>tc={2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}</author>
+    <author>tc={FFA36925-C069-4696-AC82-F35BD29C01EC}</author>
+    <author>tc={B28B570C-C764-4378-B61D-458DE4F990EC}</author>
+    <author>tc={FA61E68B-2D13-4D2E-B802-33BC32E35571}</author>
+    <author>tc={E1A102F6-1CF2-4D48-979A-0181ECF33C11}</author>
+    <author>tc={1B8056AB-E255-474B-8036-2D14416413FE}</author>
+  </authors>
+  <commentList>
+    <comment ref="J4" authorId="0" shapeId="0" xr:uid="{D913FCAB-030D-49E3-A7A0-5803B7027754}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    10 hrs = 133 m3/hr
+41 hrs = 267 m3/hr (4 trains @ 91.3% RR)
+Remainder = 222 m3/hr (3 trains @ 92.5%) 
+</t>
+      </text>
+    </comment>
+    <comment ref="A7" authorId="1" shapeId="0" xr:uid="{59DFC78E-5F9D-4D05-9892-2664283F148D}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Forced Five shutdowns</t>
+      </text>
+    </comment>
+    <comment ref="J7" authorId="2" shapeId="0" xr:uid="{5DA58C15-B5CA-4552-8F53-D4819003ECD4}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    25 hrs = 0 brine
+10 hours = 1083 m3/hr (from 2 Ro trains @ 520 + UF)
+133 hrs = 277 m3/hr (97 m3/hr from UF, remainer 45 m3/hr per train at 92.2% RR)</t>
+      </text>
+    </comment>
+    <comment ref="A10" authorId="3" shapeId="0" xr:uid="{2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Solution where there is a shutdown for all peak hours
+Reply:
+    I’d like to see numbers for only one shutdown</t>
+      </text>
+    </comment>
+    <comment ref="J10" authorId="4" shapeId="0" xr:uid="{FFA36925-C069-4696-AC82-F35BD29C01EC}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    25 hrs = 0 brine
+10 hours = 1083 m3/hr (from 2 Ro trains @ 520 + UF)
+133 hrs = 277 m3/hr (97 m3/hr from UF, remainer 45 m3/hr per train at 92.2% RR)</t>
+      </text>
+    </comment>
+    <comment ref="A13" authorId="5" shapeId="0" xr:uid="{B28B570C-C764-4378-B61D-458DE4F990EC}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Only one plant shutdown allowed</t>
+      </text>
+    </comment>
+    <comment ref="J13" authorId="6" shapeId="0" xr:uid="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    5 hrs = 0 brine
+2 hrs = 1083 m3/hr
+82 hrs = 270 m3/hr
+8 hrs = 133 m3/hr @ low RR
+Remaining = ~220 m3/hr
+Reply:
+    Low key this result is probs not the optimal version of one shutdown...</t>
+      </text>
+    </comment>
+    <comment ref="J17" authorId="7" shapeId="0" xr:uid="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    For one shutdown - there are significantly longer periods of operation at lower recovery. This occurs because there is more water to shift to off-peak hours, thus more time to be at the lower recovery value (minimizing the demand charge)</t>
+      </text>
+    </comment>
+    <comment ref="J19" authorId="8" shapeId="0" xr:uid="{1B8056AB-E255-474B-8036-2D14416413FE}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Slightly reduced recovery at 0.922 to get to 578 Feed flowrate. Plus the  start-up parts</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="57">
   <si>
     <t>Season</t>
   </si>
@@ -383,12 +489,48 @@
   <si>
     <t>1 shutdown - 5 shutdowns =</t>
   </si>
+  <si>
+    <t>No Shutdowns - 5 Shutdowns</t>
+  </si>
+  <si>
+    <t>DR, 1 SHUTDOWN</t>
+  </si>
+  <si>
+    <t>NO DR, NO SHUTDOWN</t>
+  </si>
+  <si>
+    <t>NO DR, 5 SHUTDOWN</t>
+  </si>
+  <si>
+    <t>DR, 5 SHUTDOWN</t>
+  </si>
+  <si>
+    <t>Same Solution</t>
+  </si>
+  <si>
+    <t>Differences</t>
+  </si>
+  <si>
+    <t>1 shutdown vs no shutdowns</t>
+  </si>
+  <si>
+    <t>1 shutdown vs 5 shutdowns</t>
+  </si>
+  <si>
+    <t>Op Cost (No DR)</t>
+  </si>
+  <si>
+    <t>5 shutdowns vs no shutdowns</t>
+  </si>
+  <si>
+    <t>Most difference is the start up periods (ofc)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -549,6 +691,18 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -892,7 +1046,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -908,6 +1062,9 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1369,23 +1526,72 @@
 </ThreadedComments>
 </file>
 
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="J4" dT="2026-07-31T00:16:36.52" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{D913FCAB-030D-49E3-A7A0-5803B7027754}">
+    <text xml:space="preserve">10 hrs = 133 m3/hr
+41 hrs = 267 m3/hr (4 trains @ 91.3% RR)
+Remainder = 222 m3/hr (3 trains @ 92.5%) 
+</text>
+  </threadedComment>
+  <threadedComment ref="A7" dT="2026-07-23T21:50:18.94" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{59DFC78E-5F9D-4D05-9892-2664283F148D}">
+    <text>Forced Five shutdowns</text>
+  </threadedComment>
+  <threadedComment ref="J7" dT="2026-07-30T23:48:23.68" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{5DA58C15-B5CA-4552-8F53-D4819003ECD4}">
+    <text>25 hrs = 0 brine
+10 hours = 1083 m3/hr (from 2 Ro trains @ 520 + UF)
+133 hrs = 277 m3/hr (97 m3/hr from UF, remainer 45 m3/hr per train at 92.2% RR)</text>
+  </threadedComment>
+  <threadedComment ref="A10" dT="2026-07-22T19:29:10.19" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}">
+    <text>Solution where there is a shutdown for all peak hours</text>
+  </threadedComment>
+  <threadedComment ref="A10" dT="2026-07-22T19:37:51.21" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{17E89EDA-58B7-4160-A587-C8F02064EE42}" parentId="{2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}">
+    <text>I’d like to see numbers for only one shutdown</text>
+  </threadedComment>
+  <threadedComment ref="J10" dT="2026-07-30T23:48:23.68" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FFA36925-C069-4696-AC82-F35BD29C01EC}">
+    <text>25 hrs = 0 brine
+10 hours = 1083 m3/hr (from 2 Ro trains @ 520 + UF)
+133 hrs = 277 m3/hr (97 m3/hr from UF, remainer 45 m3/hr per train at 92.2% RR)</text>
+  </threadedComment>
+  <threadedComment ref="A13" dT="2026-07-22T21:09:49.14" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B28B570C-C764-4378-B61D-458DE4F990EC}">
+    <text>Only one plant shutdown allowed</text>
+  </threadedComment>
+  <threadedComment ref="J13" dT="2026-07-31T00:30:46.97" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
+    <text>5 hrs = 0 brine
+2 hrs = 1083 m3/hr
+82 hrs = 270 m3/hr
+8 hrs = 133 m3/hr @ low RR
+Remaining = ~220 m3/hr</text>
+  </threadedComment>
+  <threadedComment ref="J13" dT="2026-07-31T00:31:51.36" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{53F1C0E0-DC73-4C54-B570-6E2EA35F43E0}" parentId="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
+    <text>Low key this result is probs not the optimal version of one shutdown...</text>
+  </threadedComment>
+  <threadedComment ref="J17" dT="2026-07-30T22:50:03.35" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
+    <text>For one shutdown - there are significantly longer periods of operation at lower recovery. This occurs because there is more water to shift to off-peak hours, thus more time to be at the lower recovery value (minimizing the demand charge)</text>
+  </threadedComment>
+  <threadedComment ref="J19" dT="2026-07-30T23:11:38.86" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{1B8056AB-E255-474B-8036-2D14416413FE}">
+    <text>Slightly reduced recovery at 0.922 to get to 578 Feed flowrate. Plus the  start-up parts</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:V99"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" customWidth="1"/>
-    <col min="3" max="3" width="11.453125" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" customWidth="1"/>
-    <col min="15" max="15" width="9.54296875" customWidth="1"/>
-    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.81640625" customWidth="1"/>
+    <col min="1" max="1" width="9.61328125" customWidth="1"/>
+    <col min="3" max="3" width="11.4609375" customWidth="1"/>
+    <col min="5" max="5" width="10.23046875" customWidth="1"/>
+    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.69140625" customWidth="1"/>
+    <col min="9" max="9" width="9.07421875" customWidth="1"/>
+    <col min="15" max="15" width="9.53515625" customWidth="1"/>
+    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1396,7 +1602,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1464,7 +1670,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1528,7 +1734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1592,10 +1798,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1659,7 +1865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -1723,10 +1929,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1790,7 +1996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -1854,10 +2060,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -1921,7 +2127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -1985,10 +2191,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2050,7 +2256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2106,10 +2312,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2173,7 +2379,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2237,7 +2443,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2246,7 +2452,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2257,7 +2463,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2321,10 +2527,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2388,7 +2594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2458,7 +2664,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="K26">
@@ -2466,7 +2672,7 @@
         <v>86355.755432219594</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2530,7 +2736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2594,10 +2800,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2661,7 +2867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -2731,7 +2937,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -2801,102 +3007,101 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A33" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B33" s="11"/>
+      <c r="C33" s="11"/>
       <c r="D33">
-        <f t="shared" ref="D33:V33" si="6">D32-D31</f>
-        <v>785.66289527932531</v>
+        <f>D31-D32</f>
+        <v>-785.66289527932531</v>
       </c>
       <c r="E33">
-        <f t="shared" si="6"/>
-        <v>2.4971086531877518E-8</v>
+        <f t="shared" ref="E33:N33" si="6">E31-E32</f>
+        <v>-2.4971086531877518E-8</v>
       </c>
       <c r="F33">
         <f t="shared" si="6"/>
-        <v>2.6907854028540568E-3</v>
+        <v>-2.6907854028540568E-3</v>
       </c>
       <c r="G33">
         <f t="shared" si="6"/>
-        <v>-221.42920834019969</v>
+        <v>221.42920834019969</v>
       </c>
       <c r="H33">
         <f t="shared" si="6"/>
-        <v>896.09976246881979</v>
+        <v>-896.09976246881979</v>
       </c>
       <c r="I33">
         <f t="shared" si="6"/>
-        <v>-4877.4899349639245</v>
+        <v>4877.4899349639245</v>
       </c>
       <c r="J33">
         <f t="shared" si="6"/>
-        <v>-4202.8193808354008</v>
+        <v>4202.8193808354008</v>
       </c>
       <c r="K33">
         <f t="shared" si="6"/>
-        <v>-87.19067491790338</v>
+        <v>87.19067491790338</v>
       </c>
       <c r="L33">
         <f t="shared" si="6"/>
-        <v>4424.0083944886992</v>
+        <v>-4424.0083944886992</v>
       </c>
       <c r="M33">
         <f t="shared" si="6"/>
-        <v>625.28660162189772</v>
+        <v>-625.28660162189772</v>
       </c>
       <c r="N33">
         <f t="shared" si="6"/>
-        <v>26.377954922030085</v>
+        <v>-26.377954922030085</v>
       </c>
       <c r="O33">
-        <f t="shared" si="6"/>
+        <f>O32-O31</f>
         <v>0</v>
       </c>
       <c r="P33">
-        <f t="shared" si="6"/>
+        <f>P32-P31</f>
         <v>785.66289527932531</v>
       </c>
       <c r="Q33">
-        <f t="shared" si="6"/>
+        <f>Q32-Q31</f>
         <v>200.21086642008004</v>
       </c>
       <c r="R33">
-        <f t="shared" si="6"/>
+        <f>R32-R31</f>
         <v>20835.930555410298</v>
       </c>
       <c r="S33">
-        <f t="shared" si="6"/>
+        <f>S32-S31</f>
         <v>397.33849572936299</v>
       </c>
       <c r="T33">
-        <f t="shared" si="6"/>
+        <f>T32-T31</f>
         <v>-0.1359304574304484</v>
       </c>
       <c r="U33">
-        <f t="shared" si="6"/>
+        <f>U32-U31</f>
         <v>25293.846976061999</v>
       </c>
       <c r="V33">
-        <f t="shared" si="6"/>
+        <f>V32-V31</f>
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
-      <c r="K34">
-        <f>K31+L31+M31</f>
-        <v>86355.755432219594</v>
-      </c>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -2960,7 +3165,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3024,12 +3229,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3096,7 +3301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3166,20 +3371,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3243,15 +3448,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3321,13 +3526,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
@@ -3391,7 +3596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
@@ -3455,11 +3660,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -3523,7 +3728,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -3587,10 +3792,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
@@ -3654,7 +3859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>22</v>
       </c>
@@ -3718,13 +3923,13 @@
         <v>0.51444695802960605</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -3788,7 +3993,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -3853,7 +4058,7 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A62" s="3" t="s">
         <v>22</v>
       </c>
@@ -3923,7 +4128,7 @@
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -3993,7 +4198,7 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A64" s="11" t="s">
         <v>44</v>
       </c>
@@ -4076,19 +4281,19 @@
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A66" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G66" s="4"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A67" s="3" t="s">
         <v>20</v>
       </c>
@@ -4100,7 +4305,7 @@
       </c>
       <c r="G67" s="4"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A68" t="s">
         <v>22</v>
       </c>
@@ -4164,13 +4369,13 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
       <c r="G69" s="4"/>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A70" s="3" t="s">
         <v>20</v>
       </c>
@@ -4182,7 +4387,7 @@
       </c>
       <c r="G70" s="4"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A71" t="s">
         <v>22</v>
       </c>
@@ -4250,7 +4455,7 @@
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A72" s="5"/>
       <c r="B72" s="5"/>
       <c r="D72">
@@ -4330,12 +4535,12 @@
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A73" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A74" s="3" t="s">
         <v>20</v>
       </c>
@@ -4399,7 +4604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A75" s="3" t="s">
         <v>22</v>
       </c>
@@ -4463,10 +4668,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A76" s="1"/>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A77" t="s">
         <v>20</v>
       </c>
@@ -4524,7 +4729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A78" s="2" t="s">
         <v>22</v>
       </c>
@@ -4588,7 +4793,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A80" t="s">
         <v>20</v>
       </c>
@@ -4646,7 +4851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A81" t="s">
         <v>22</v>
       </c>
@@ -4716,7 +4921,7 @@
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
       <c r="D82">
         <f>D81-D75</f>
         <v>-4018.7603482047853</v>
@@ -4766,13 +4971,13 @@
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A83" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G83" s="4"/>
     </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A84" t="s">
         <v>22</v>
       </c>
@@ -4836,7 +5041,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>22</v>
       </c>
@@ -4880,7 +5085,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="87" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A87" s="1" t="s">
         <v>26</v>
       </c>
@@ -4901,7 +5106,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="88" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A88" t="s">
         <v>0</v>
       </c>
@@ -4963,7 +5168,7 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="89" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A89" s="2" t="s">
         <v>20</v>
       </c>
@@ -5025,12 +5230,12 @@
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A90" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="92" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A92" t="s">
         <v>32</v>
       </c>
@@ -5041,7 +5246,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="93" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A93">
         <v>20</v>
       </c>
@@ -5105,7 +5310,7 @@
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A94">
         <v>20</v>
       </c>
@@ -5169,7 +5374,7 @@
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A95">
         <v>20</v>
       </c>
@@ -5233,7 +5438,7 @@
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A96">
         <v>20</v>
       </c>
@@ -5297,7 +5502,7 @@
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A97" s="3">
         <v>20</v>
       </c>
@@ -5361,7 +5566,7 @@
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A98">
         <v>20</v>
       </c>
@@ -5425,7 +5630,7 @@
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A99">
         <v>20</v>
       </c>
@@ -5490,12 +5695,441 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A64:C64"/>
+    <mergeCell ref="A33:C33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA993591-8C1F-4C7B-A75D-E9726DFB461B}">
+  <dimension ref="A2:P21"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="12.84375" customWidth="1"/>
+    <col min="3" max="3" width="11.3828125" customWidth="1"/>
+    <col min="4" max="4" width="15.53515625" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="17.07421875" customWidth="1"/>
+    <col min="7" max="7" width="15.23046875" customWidth="1"/>
+    <col min="8" max="8" width="13.3046875" customWidth="1"/>
+    <col min="9" max="11" width="11.3828125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P2" s="2"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4" s="10">
+        <f>H4+I4+J4+K4</f>
+        <v>116354.41551491321</v>
+      </c>
+      <c r="E4" s="10">
+        <v>19840.537050750401</v>
+      </c>
+      <c r="F4" s="10">
+        <v>5280.6330826172398</v>
+      </c>
+      <c r="G4" s="10">
+        <v>4877.4899493259099</v>
+      </c>
+      <c r="H4" s="10">
+        <v>29998.660082693601</v>
+      </c>
+      <c r="I4" s="10">
+        <v>51077.135880394701</v>
+      </c>
+      <c r="J4" s="10">
+        <v>15932.544048423801</v>
+      </c>
+      <c r="K4" s="10">
+        <v>19346.075503401102</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A6" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="M6" s="12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7" s="10">
+        <f>H7+I7+J7+K7</f>
+        <v>117113.7004552705</v>
+      </c>
+      <c r="E7" s="10">
+        <v>19619.107842410202</v>
+      </c>
+      <c r="F7" s="10">
+        <v>6176.7328450860596</v>
+      </c>
+      <c r="G7" s="10">
+        <v>1.43619850991576E-5</v>
+      </c>
+      <c r="H7" s="10">
+        <v>25795.8407018582</v>
+      </c>
+      <c r="I7" s="10">
+        <v>50989.945205476797</v>
+      </c>
+      <c r="J7" s="10">
+        <v>20356.5524429125</v>
+      </c>
+      <c r="K7" s="10">
+        <v>19971.362105022999</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7" s="12"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="M8" s="12"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="M9" s="12"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10">
+        <v>4</v>
+      </c>
+      <c r="D10" s="10">
+        <f>H10+I10+J10+K10</f>
+        <v>117112.9202243583</v>
+      </c>
+      <c r="E10" s="10">
+        <v>19617.269555424798</v>
+      </c>
+      <c r="F10" s="10">
+        <v>6177.79087142139</v>
+      </c>
+      <c r="G10" s="10">
+        <v>1.4897343661976701E-5</v>
+      </c>
+      <c r="H10" s="10">
+        <v>25795.060441743601</v>
+      </c>
+      <c r="I10" s="10">
+        <v>50989.945229661498</v>
+      </c>
+      <c r="J10" s="10">
+        <v>20356.5524429125</v>
+      </c>
+      <c r="K10" s="10">
+        <v>19971.3621100407</v>
+      </c>
+      <c r="L10">
+        <v>11020</v>
+      </c>
+      <c r="M10" s="12"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="M11" s="12"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A12" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+      <c r="D13" s="10">
+        <f>H13+I13+J13+K13</f>
+        <v>117626.33139463789</v>
+      </c>
+      <c r="E13" s="10">
+        <v>19403.054157778199</v>
+      </c>
+      <c r="F13" s="10">
+        <v>5553.2925107720503</v>
+      </c>
+      <c r="G13" s="10">
+        <v>4877.88612389215</v>
+      </c>
+      <c r="H13" s="10">
+        <v>29834.232792442399</v>
+      </c>
+      <c r="I13" s="10">
+        <v>51173.670096007401</v>
+      </c>
+      <c r="J13" s="10">
+        <v>17123.646419717399</v>
+      </c>
+      <c r="K13" s="10">
+        <v>19494.782086470699</v>
+      </c>
+      <c r="L13">
+        <v>11020</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>51</v>
+      </c>
+      <c r="J16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A17" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="10">
+        <f>D13-D4</f>
+        <v>1271.9158797246782</v>
+      </c>
+      <c r="E17" s="10">
+        <f t="shared" ref="E17:K17" si="0">E13-E4</f>
+        <v>-437.48289297220254</v>
+      </c>
+      <c r="F17" s="10">
+        <f t="shared" si="0"/>
+        <v>272.65942815481048</v>
+      </c>
+      <c r="G17" s="10">
+        <f t="shared" si="0"/>
+        <v>0.39617456624000624</v>
+      </c>
+      <c r="H17" s="10">
+        <f t="shared" si="0"/>
+        <v>-164.42729025120207</v>
+      </c>
+      <c r="I17" s="10">
+        <f t="shared" si="0"/>
+        <v>96.534215612700791</v>
+      </c>
+      <c r="J17" s="10">
+        <f t="shared" si="0"/>
+        <v>1191.1023712935985</v>
+      </c>
+      <c r="K17" s="10">
+        <f t="shared" si="0"/>
+        <v>148.7065830695974</v>
+      </c>
+      <c r="L17" s="10"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19" s="10">
+        <f>D7-D4</f>
+        <v>759.28494035729091</v>
+      </c>
+      <c r="E19" s="10">
+        <f>E7-E4</f>
+        <v>-221.42920834019969</v>
+      </c>
+      <c r="F19" s="10">
+        <f>F7-F4</f>
+        <v>896.09976246881979</v>
+      </c>
+      <c r="G19" s="10">
+        <f>G7-G4</f>
+        <v>-4877.4899349639245</v>
+      </c>
+      <c r="H19" s="10">
+        <f>H7-H4</f>
+        <v>-4202.8193808354008</v>
+      </c>
+      <c r="I19" s="10">
+        <f>I7-I4</f>
+        <v>-87.19067491790338</v>
+      </c>
+      <c r="J19" s="10">
+        <f>J7-J4</f>
+        <v>4424.0083944886992</v>
+      </c>
+      <c r="K19" s="10">
+        <f>K7-K4</f>
+        <v>625.28660162189772</v>
+      </c>
+      <c r="L19" s="10"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>53</v>
+      </c>
+      <c r="D21" s="10">
+        <f>D13-D10</f>
+        <v>513.41117027959262</v>
+      </c>
+      <c r="E21" s="10">
+        <f>E13-E10</f>
+        <v>-214.21539764659974</v>
+      </c>
+      <c r="F21" s="10">
+        <f>F13-F10</f>
+        <v>-624.4983606493397</v>
+      </c>
+      <c r="G21" s="10">
+        <f>G13-G10</f>
+        <v>4877.8861089948059</v>
+      </c>
+      <c r="H21" s="10">
+        <f>H13-H10</f>
+        <v>4039.1723506987983</v>
+      </c>
+      <c r="I21" s="10">
+        <f>I13-I10</f>
+        <v>183.72486634590314</v>
+      </c>
+      <c r="J21" s="10">
+        <f>J13-J10</f>
+        <v>-3232.9060231951007</v>
+      </c>
+      <c r="K21" s="10">
+        <f>K13-K10</f>
+        <v>-476.58002357000078</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="M6:M11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
redo RTP result with a delayed shutdown constraint
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2E049B6-A2C8-4593-8E7F-51E288AB2F85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8B7EE63-FD21-44E7-BB0C-0F6222E2FD58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -332,7 +332,7 @@
     Low key this result is probs not the optimal version of one shutdown...</t>
       </text>
     </comment>
-    <comment ref="J17" authorId="7" shapeId="0" xr:uid="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
+    <comment ref="J19" authorId="7" shapeId="0" xr:uid="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -340,7 +340,7 @@
     For one shutdown - there are significantly longer periods of operation at lower recovery. This occurs because there is more water to shift to off-peak hours, thus more time to be at the lower recovery value (minimizing the demand charge)</t>
       </text>
     </comment>
-    <comment ref="J19" authorId="8" shapeId="0" xr:uid="{1B8056AB-E255-474B-8036-2D14416413FE}">
+    <comment ref="J21" authorId="8" shapeId="0" xr:uid="{1B8056AB-E255-474B-8036-2D14416413FE}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -353,7 +353,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="60">
   <si>
     <t>Season</t>
   </si>
@@ -525,12 +525,21 @@
   <si>
     <t>Most difference is the start up periods (ofc)</t>
   </si>
+  <si>
+    <t>DR, 1 SHUTDOWN, 3 HR Startup</t>
+  </si>
+  <si>
+    <t>2 HR vs. 3 HR Shutdown</t>
+  </si>
+  <si>
+    <t>3 HR shutdown vs no shutdowns</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -691,18 +700,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1060,11 +1057,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1566,10 +1563,10 @@
   <threadedComment ref="J13" dT="2026-07-31T00:31:51.36" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{53F1C0E0-DC73-4C54-B570-6E2EA35F43E0}" parentId="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
     <text>Low key this result is probs not the optimal version of one shutdown...</text>
   </threadedComment>
-  <threadedComment ref="J17" dT="2026-07-30T22:50:03.35" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
+  <threadedComment ref="J19" dT="2026-07-30T22:50:03.35" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
     <text>For one shutdown - there are significantly longer periods of operation at lower recovery. This occurs because there is more water to shift to off-peak hours, thus more time to be at the lower recovery value (minimizing the demand charge)</text>
   </threadedComment>
-  <threadedComment ref="J19" dT="2026-07-30T23:11:38.86" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{1B8056AB-E255-474B-8036-2D14416413FE}">
+  <threadedComment ref="J21" dT="2026-07-30T23:11:38.86" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{1B8056AB-E255-474B-8036-2D14416413FE}">
     <text>Slightly reduced recovery at 0.922 to get to 578 Feed flowrate. Plus the  start-up parts</text>
   </threadedComment>
 </ThreadedComments>
@@ -1578,20 +1575,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:V99"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.61328125" customWidth="1"/>
-    <col min="3" max="3" width="11.4609375" customWidth="1"/>
-    <col min="5" max="5" width="10.23046875" customWidth="1"/>
-    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.69140625" customWidth="1"/>
-    <col min="9" max="9" width="9.07421875" customWidth="1"/>
-    <col min="15" max="15" width="9.53515625" customWidth="1"/>
-    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.84375" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" customWidth="1"/>
+    <col min="3" max="3" width="11.453125" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="11" max="11" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.54296875" customWidth="1"/>
+    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1602,7 +1600,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1670,7 +1668,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1734,7 +1732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1798,10 +1796,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G5" s="4"/>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="K5">
+        <f>K4+L4+M4</f>
+        <v>85444.512881154791</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1865,7 +1867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -1929,10 +1931,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1996,7 +1998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2060,10 +2062,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -2127,7 +2129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2191,10 +2193,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2256,7 +2258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2312,10 +2314,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2379,7 +2381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2443,7 +2445,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2452,7 +2454,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2463,7 +2465,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2527,10 +2529,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2594,7 +2596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2664,7 +2666,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="K26">
@@ -2672,7 +2674,7 @@
         <v>86355.755432219594</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2736,7 +2738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2800,10 +2802,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2867,7 +2869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -2937,7 +2939,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -3007,12 +3009,12 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A33" s="11" t="s">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A33" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
+      <c r="B33" s="12"/>
+      <c r="C33" s="12"/>
       <c r="D33">
         <f>D31-D32</f>
         <v>-785.66289527932531</v>
@@ -3058,50 +3060,50 @@
         <v>-26.377954922030085</v>
       </c>
       <c r="O33">
-        <f>O32-O31</f>
+        <f t="shared" ref="O33:V33" si="7">O32-O31</f>
         <v>0</v>
       </c>
       <c r="P33">
-        <f>P32-P31</f>
+        <f t="shared" si="7"/>
         <v>785.66289527932531</v>
       </c>
       <c r="Q33">
-        <f>Q32-Q31</f>
+        <f t="shared" si="7"/>
         <v>200.21086642008004</v>
       </c>
       <c r="R33">
-        <f>R32-R31</f>
+        <f t="shared" si="7"/>
         <v>20835.930555410298</v>
       </c>
       <c r="S33">
-        <f>S32-S31</f>
+        <f t="shared" si="7"/>
         <v>397.33849572936299</v>
       </c>
       <c r="T33">
-        <f>T32-T31</f>
+        <f t="shared" si="7"/>
         <v>-0.1359304574304484</v>
       </c>
       <c r="U33">
-        <f>U32-U31</f>
+        <f t="shared" si="7"/>
         <v>25293.846976061999</v>
       </c>
       <c r="V33">
-        <f>V32-V31</f>
+        <f t="shared" si="7"/>
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -3149,7 +3151,7 @@
         <v>0</v>
       </c>
       <c r="P36">
-        <f t="shared" ref="P36:P37" si="7">D36+$P$1</f>
+        <f t="shared" ref="P36:P37" si="8">D36+$P$1</f>
         <v>237552.9910647514</v>
       </c>
       <c r="Q36">
@@ -3165,7 +3167,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3213,7 +3215,7 @@
         <v>0</v>
       </c>
       <c r="P37">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>246460.49240879912</v>
       </c>
       <c r="Q37">
@@ -3229,12 +3231,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3282,7 +3284,7 @@
         <v>0</v>
       </c>
       <c r="P39">
-        <f t="shared" ref="P39:P40" si="8">D39+$P$1</f>
+        <f t="shared" ref="P39:P40" si="9">D39+$P$1</f>
         <v>237538.1865021491</v>
       </c>
       <c r="Q39">
@@ -3301,7 +3303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3349,7 +3351,7 @@
         <v>0</v>
       </c>
       <c r="P40">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>242769.60515337173</v>
       </c>
       <c r="Q40">
@@ -3371,20 +3373,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3432,7 +3434,7 @@
         <v>0</v>
       </c>
       <c r="P44">
-        <f t="shared" ref="P44" si="9">D44+$P$1</f>
+        <f t="shared" ref="P44" si="10">D44+$P$1</f>
         <v>246486.61307970091</v>
       </c>
       <c r="Q44">
@@ -3448,15 +3450,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3526,13 +3528,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
@@ -3580,7 +3582,7 @@
         <v>0</v>
       </c>
       <c r="P50">
-        <f t="shared" ref="P50:P57" si="10">D50+$P$1</f>
+        <f t="shared" ref="P50:P57" si="11">D50+$P$1</f>
         <v>238413.66244470741</v>
       </c>
       <c r="Q50">
@@ -3596,7 +3598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
@@ -3644,7 +3646,7 @@
         <v>0</v>
       </c>
       <c r="P51">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>308572.43924949365</v>
       </c>
       <c r="Q51">
@@ -3660,11 +3662,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -3712,7 +3714,7 @@
         <v>0</v>
       </c>
       <c r="P53">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>238584.40212047941</v>
       </c>
       <c r="Q53">
@@ -3728,7 +3730,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -3776,7 +3778,7 @@
         <v>0</v>
       </c>
       <c r="P54">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>293116.00381082937</v>
       </c>
       <c r="Q54">
@@ -3792,10 +3794,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
@@ -3843,7 +3845,7 @@
         <v>0</v>
       </c>
       <c r="P56">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>238385.73201352643</v>
       </c>
       <c r="Q56">
@@ -3859,7 +3861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>22</v>
       </c>
@@ -3907,7 +3909,7 @@
         <v>0</v>
       </c>
       <c r="P57">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>245994.13393950483</v>
       </c>
       <c r="Q57">
@@ -3923,13 +3925,13 @@
         <v>0.51444695802960605</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -3977,7 +3979,7 @@
         <v>3157.9970999842499</v>
       </c>
       <c r="P60">
-        <f t="shared" ref="P60:P63" si="11">D60+$P$1</f>
+        <f t="shared" ref="P60:P63" si="12">D60+$P$1</f>
         <v>237036.76680162852</v>
       </c>
       <c r="Q60">
@@ -3993,7 +3995,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -4042,7 +4044,7 @@
         <v>11020</v>
       </c>
       <c r="P61">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>230122.64709737207</v>
       </c>
       <c r="Q61">
@@ -4058,7 +4060,7 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
         <v>22</v>
       </c>
@@ -4106,7 +4108,7 @@
         <v>11020</v>
       </c>
       <c r="P62">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>228114.97006531907</v>
       </c>
       <c r="Q62">
@@ -4128,7 +4130,7 @@
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -4176,7 +4178,7 @@
         <v>11020</v>
       </c>
       <c r="P63">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>228601.63035230787</v>
       </c>
       <c r="Q63">
@@ -4198,102 +4200,102 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A64" s="11" t="s">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A64" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B64" s="11"/>
-      <c r="C64" s="11"/>
+      <c r="B64" s="12"/>
+      <c r="C64" s="12"/>
       <c r="D64" s="10">
         <f>D63-D62</f>
         <v>486.66028698880109</v>
       </c>
       <c r="E64">
-        <f t="shared" ref="E64:V64" si="12">E63-E62</f>
+        <f t="shared" ref="E64:V64" si="13">E63-E62</f>
         <v>-1.0599615052342415E-7</v>
       </c>
       <c r="F64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1.8194475210779881E-3</v>
       </c>
       <c r="G64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-214.21539764659974</v>
       </c>
       <c r="H64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-624.4983606493397</v>
       </c>
       <c r="I64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>4877.8861089948059</v>
       </c>
       <c r="J64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>4039.1723506987983</v>
       </c>
       <c r="K64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>183.72486634590314</v>
       </c>
       <c r="L64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-3232.9060902373021</v>
       </c>
       <c r="M64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-476.58002357000078</v>
       </c>
       <c r="N64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-26.750816248570118</v>
       </c>
       <c r="O64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="P64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>486.66028698880109</v>
       </c>
       <c r="Q64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-139.52840101139986</v>
       </c>
       <c r="R64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-16066.151948654198</v>
       </c>
       <c r="S64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-545.80690098968103</v>
       </c>
       <c r="T64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0.30386414961436203</v>
       </c>
       <c r="U64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-23556.497919273097</v>
       </c>
       <c r="V64">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G66" s="4"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
         <v>20</v>
       </c>
@@ -4305,7 +4307,7 @@
       </c>
       <c r="G67" s="4"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>22</v>
       </c>
@@ -4369,13 +4371,13 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
       <c r="G69" s="4"/>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A70" s="3" t="s">
         <v>20</v>
       </c>
@@ -4387,7 +4389,7 @@
       </c>
       <c r="G70" s="4"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>22</v>
       </c>
@@ -4455,7 +4457,7 @@
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A72" s="5"/>
       <c r="B72" s="5"/>
       <c r="D72">
@@ -4463,84 +4465,84 @@
         <v>-16260.494075352748</v>
       </c>
       <c r="E72">
-        <f t="shared" ref="E72:V72" si="13">E71-E68</f>
+        <f t="shared" ref="E72:V72" si="14">E71-E68</f>
         <v>-11.188766930019483</v>
       </c>
       <c r="F72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-5.2593913252494073E-2</v>
       </c>
       <c r="G72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-4474.9745192109003</v>
       </c>
       <c r="H72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1349.0083827482595</v>
       </c>
       <c r="I72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-9098.574812435656</v>
       </c>
       <c r="J72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-12224.540948898299</v>
       </c>
       <c r="K72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>99.745205475301191</v>
       </c>
       <c r="L72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>4931.2097430098001</v>
       </c>
       <c r="M72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>663.72894502789859</v>
       </c>
       <c r="N72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>52.540525326540092</v>
       </c>
       <c r="O72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>8320.7995903714655</v>
       </c>
       <c r="P72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-15268.183367467253</v>
       </c>
       <c r="Q72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>301.40187495156988</v>
       </c>
       <c r="R72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>34518.506961381201</v>
       </c>
       <c r="S72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>841.91480393612801</v>
       </c>
       <c r="T72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0.38784649209264499</v>
       </c>
       <c r="U72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>38249.060394551692</v>
       </c>
       <c r="V72">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
         <v>20</v>
       </c>
@@ -4588,7 +4590,7 @@
         <v>0</v>
       </c>
       <c r="P74">
-        <f t="shared" ref="P74:P75" si="14">D74+$P$1</f>
+        <f t="shared" ref="P74:P75" si="15">D74+$P$1</f>
         <v>236582.9608490612</v>
       </c>
       <c r="Q74">
@@ -4604,7 +4606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
         <v>22</v>
       </c>
@@ -4652,7 +4654,7 @@
         <v>0</v>
       </c>
       <c r="P75">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>246323.22923633162</v>
       </c>
       <c r="Q75">
@@ -4668,10 +4670,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A76" s="1"/>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>20</v>
       </c>
@@ -4719,7 +4721,7 @@
         <v>0</v>
       </c>
       <c r="P77">
-        <f t="shared" ref="P77:P78" si="15">D77+$P$1</f>
+        <f t="shared" ref="P77:P78" si="16">D77+$P$1</f>
         <v>237266.08760950522</v>
       </c>
       <c r="Q77">
@@ -4729,7 +4731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>22</v>
       </c>
@@ -4777,7 +4779,7 @@
         <v>0</v>
       </c>
       <c r="P78">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>242193.03042265025</v>
       </c>
       <c r="Q78">
@@ -4793,7 +4795,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>20</v>
       </c>
@@ -4841,7 +4843,7 @@
         <v>0</v>
       </c>
       <c r="P80">
-        <f t="shared" ref="P80:P82" si="16">D80+$P$1</f>
+        <f t="shared" ref="P80:P82" si="17">D80+$P$1</f>
         <v>237266.08760950161</v>
       </c>
       <c r="Q80">
@@ -4851,7 +4853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>22</v>
       </c>
@@ -4899,7 +4901,7 @@
         <v>0</v>
       </c>
       <c r="P81">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>242304.46888812684</v>
       </c>
       <c r="Q81">
@@ -4921,63 +4923,63 @@
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
       <c r="D82">
         <f>D81-D75</f>
         <v>-4018.7603482047853</v>
       </c>
       <c r="E82">
-        <f t="shared" ref="E82:N82" si="17">E81-E75</f>
+        <f t="shared" ref="E82:N82" si="18">E81-E75</f>
         <v>0.21251127298455685</v>
       </c>
       <c r="F82">
+        <f t="shared" si="18"/>
+        <v>-1.5794992464996938E-2</v>
+      </c>
+      <c r="G82">
+        <f t="shared" si="18"/>
+        <v>-1335.1371720950992</v>
+      </c>
+      <c r="H82">
+        <f t="shared" si="18"/>
+        <v>329.78360458492989</v>
+      </c>
+      <c r="I82">
+        <f t="shared" si="18"/>
+        <v>-4562.1832736040305</v>
+      </c>
+      <c r="J82">
+        <f t="shared" si="18"/>
+        <v>-5567.5368411142044</v>
+      </c>
+      <c r="K82">
+        <f t="shared" si="18"/>
+        <v>285.1804885383026</v>
+      </c>
+      <c r="L82">
+        <f t="shared" si="18"/>
+        <v>766.33118310559985</v>
+      </c>
+      <c r="M82">
+        <f t="shared" si="18"/>
+        <v>59.181539221001003</v>
+      </c>
+      <c r="N82">
+        <f t="shared" si="18"/>
+        <v>438.08328204450595</v>
+      </c>
+      <c r="P82">
         <f t="shared" si="17"/>
-        <v>-1.5794992464996938E-2</v>
-      </c>
-      <c r="G82">
-        <f t="shared" si="17"/>
-        <v>-1335.1371720950992</v>
-      </c>
-      <c r="H82">
-        <f t="shared" si="17"/>
-        <v>329.78360458492989</v>
-      </c>
-      <c r="I82">
-        <f t="shared" si="17"/>
-        <v>-4562.1832736040305</v>
-      </c>
-      <c r="J82">
-        <f t="shared" si="17"/>
-        <v>-5567.5368411142044</v>
-      </c>
-      <c r="K82">
-        <f t="shared" si="17"/>
-        <v>285.1804885383026</v>
-      </c>
-      <c r="L82">
-        <f t="shared" si="17"/>
-        <v>766.33118310559985</v>
-      </c>
-      <c r="M82">
-        <f t="shared" si="17"/>
-        <v>59.181539221001003</v>
-      </c>
-      <c r="N82">
-        <f t="shared" si="17"/>
-        <v>438.08328204450595</v>
-      </c>
-      <c r="P82">
-        <f t="shared" si="16"/>
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G83" s="4"/>
     </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>22</v>
       </c>
@@ -5025,7 +5027,7 @@
         <v>0</v>
       </c>
       <c r="P84">
-        <f t="shared" ref="P84" si="18">D84+$P$1</f>
+        <f t="shared" ref="P84" si="19">D84+$P$1</f>
         <v>267678.15388715523</v>
       </c>
       <c r="Q84">
@@ -5041,7 +5043,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>22</v>
       </c>
@@ -5085,7 +5087,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="87" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>26</v>
       </c>
@@ -5106,7 +5108,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="88" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>0</v>
       </c>
@@ -5168,7 +5170,7 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="89" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>20</v>
       </c>
@@ -5230,12 +5232,12 @@
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A90" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="92" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>32</v>
       </c>
@@ -5246,7 +5248,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="93" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>20</v>
       </c>
@@ -5257,7 +5259,7 @@
         <v>2</v>
       </c>
       <c r="D93">
-        <f t="shared" ref="D93:D99" si="19">J93+K93+L93+M93+N93</f>
+        <f t="shared" ref="D93:D99" si="20">J93+K93+L93+M93+N93</f>
         <v>120712.69088313227</v>
       </c>
       <c r="E93">
@@ -5294,7 +5296,7 @@
         <v>0</v>
       </c>
       <c r="P93">
-        <f t="shared" ref="P93:P99" si="20">D93+$P$1</f>
+        <f t="shared" ref="P93:P99" si="21">D93+$P$1</f>
         <v>241272.36270212877</v>
       </c>
       <c r="Q93">
@@ -5310,7 +5312,7 @@
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>20</v>
       </c>
@@ -5321,7 +5323,7 @@
         <v>2</v>
       </c>
       <c r="D94">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>119392.42354269064</v>
       </c>
       <c r="E94">
@@ -5358,7 +5360,7 @@
         <v>0</v>
       </c>
       <c r="P94">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>239952.09536168716</v>
       </c>
       <c r="Q94">
@@ -5374,7 +5376,7 @@
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>20</v>
       </c>
@@ -5385,7 +5387,7 @@
         <v>2</v>
       </c>
       <c r="D95">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>117777.02945340994</v>
       </c>
       <c r="E95">
@@ -5422,7 +5424,7 @@
         <v>0</v>
       </c>
       <c r="P95">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>238336.70127240644</v>
       </c>
       <c r="Q95">
@@ -5438,7 +5440,7 @@
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>20</v>
       </c>
@@ -5449,7 +5451,7 @@
         <v>2</v>
       </c>
       <c r="D96">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>116625.1695160947</v>
       </c>
       <c r="E96">
@@ -5486,7 +5488,7 @@
         <v>0</v>
       </c>
       <c r="P96">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>237184.84133509122</v>
       </c>
       <c r="Q96">
@@ -5502,7 +5504,7 @@
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A97" s="3">
         <v>20</v>
       </c>
@@ -5513,7 +5515,7 @@
         <v>2</v>
       </c>
       <c r="D97">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>115198.459983006</v>
       </c>
       <c r="E97">
@@ -5550,7 +5552,7 @@
         <v>0</v>
       </c>
       <c r="P97">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>235758.13180200252</v>
       </c>
       <c r="Q97">
@@ -5566,7 +5568,7 @@
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>20</v>
       </c>
@@ -5577,7 +5579,7 @@
         <v>2</v>
       </c>
       <c r="D98">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>114451.25872361983</v>
       </c>
       <c r="E98">
@@ -5614,7 +5616,7 @@
         <v>0</v>
       </c>
       <c r="P98">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>235010.93054261635</v>
       </c>
       <c r="Q98">
@@ -5630,7 +5632,7 @@
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>20</v>
       </c>
@@ -5641,7 +5643,7 @@
         <v>2</v>
       </c>
       <c r="D99">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>114787.7594081375</v>
       </c>
       <c r="E99">
@@ -5678,7 +5680,7 @@
         <v>0</v>
       </c>
       <c r="P99">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>235347.43122713402</v>
       </c>
       <c r="Q99">
@@ -5707,21 +5709,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA993591-8C1F-4C7B-A75D-E9726DFB461B}">
-  <dimension ref="A2:P21"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A2:P27"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="12.84375" customWidth="1"/>
-    <col min="3" max="3" width="11.3828125" customWidth="1"/>
-    <col min="4" max="4" width="15.53515625" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" customWidth="1"/>
+    <col min="3" max="3" width="11.36328125" customWidth="1"/>
+    <col min="4" max="4" width="15.54296875" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17.07421875" customWidth="1"/>
-    <col min="7" max="7" width="15.23046875" customWidth="1"/>
-    <col min="8" max="8" width="13.3046875" customWidth="1"/>
-    <col min="9" max="11" width="11.3828125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" customWidth="1"/>
+    <col min="7" max="7" width="15.26953125" customWidth="1"/>
+    <col min="8" max="8" width="13.26953125" customWidth="1"/>
+    <col min="9" max="11" width="11.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5760,12 +5762,12 @@
       </c>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -5804,7 +5806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="D5" s="10"/>
@@ -5816,7 +5818,7 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>48</v>
       </c>
@@ -5829,11 +5831,11 @@
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>
       <c r="K6" s="10"/>
-      <c r="M6" s="12" t="s">
+      <c r="M6" s="11" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:16" ht="14.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -5871,9 +5873,9 @@
       <c r="L7">
         <v>0</v>
       </c>
-      <c r="M7" s="12"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="M7" s="11"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -5882,9 +5884,9 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
       <c r="K8" s="10"/>
-      <c r="M8" s="12"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="M8" s="11"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>49</v>
       </c>
@@ -5896,9 +5898,9 @@
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
       <c r="K9" s="10"/>
-      <c r="M9" s="12"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="M9" s="11"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -5936,9 +5938,9 @@
       <c r="L10">
         <v>11020</v>
       </c>
-      <c r="M10" s="12"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="M10" s="11"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="D11" s="10"/>
@@ -5949,9 +5951,9 @@
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
       <c r="K11" s="10"/>
-      <c r="M11" s="12"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="M11" s="11"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>46</v>
       </c>
@@ -5964,7 +5966,7 @@
       <c r="J12" s="10"/>
       <c r="K12" s="10"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -6003,125 +6005,238 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A16" t="s">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15">
+        <v>4</v>
+      </c>
+      <c r="D15" s="10">
+        <f>H15+I15+J15+K15</f>
+        <v>118290.90224843152</v>
+      </c>
+      <c r="E15" s="10">
+        <v>19769.338187252601</v>
+      </c>
+      <c r="F15" s="10">
+        <v>6055.3448338257103</v>
+      </c>
+      <c r="G15" s="10">
+        <v>4869.7822488983002</v>
+      </c>
+      <c r="H15" s="10">
+        <v>30694.465269976601</v>
+      </c>
+      <c r="I15" s="10">
+        <v>50987.320205484903</v>
+      </c>
+      <c r="J15" s="10">
+        <v>17088.664422113401</v>
+      </c>
+      <c r="K15" s="10">
+        <v>19520.452350856602</v>
+      </c>
+      <c r="L15">
+        <v>11020</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>51</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J18" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A17" t="s">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>52</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D19" s="10">
         <f>D13-D4</f>
         <v>1271.9158797246782</v>
       </c>
-      <c r="E17" s="10">
-        <f t="shared" ref="E17:K17" si="0">E13-E4</f>
+      <c r="E19" s="10">
+        <f t="shared" ref="E19:K19" si="0">E13-E4</f>
         <v>-437.48289297220254</v>
       </c>
-      <c r="F17" s="10">
+      <c r="F19" s="10">
         <f t="shared" si="0"/>
         <v>272.65942815481048</v>
       </c>
-      <c r="G17" s="10">
+      <c r="G19" s="10">
         <f t="shared" si="0"/>
         <v>0.39617456624000624</v>
       </c>
-      <c r="H17" s="10">
+      <c r="H19" s="10">
         <f t="shared" si="0"/>
         <v>-164.42729025120207</v>
       </c>
-      <c r="I17" s="10">
+      <c r="I19" s="10">
         <f t="shared" si="0"/>
         <v>96.534215612700791</v>
       </c>
-      <c r="J17" s="10">
+      <c r="J19" s="10">
         <f t="shared" si="0"/>
         <v>1191.1023712935985</v>
       </c>
-      <c r="K17" s="10">
+      <c r="K19" s="10">
         <f t="shared" si="0"/>
         <v>148.7065830695974</v>
       </c>
-      <c r="L17" s="10"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A19" t="s">
+      <c r="L19" s="10"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="10">
-        <f>D7-D4</f>
+      <c r="D21" s="10">
+        <f t="shared" ref="D21:K21" si="1">D7-D4</f>
         <v>759.28494035729091</v>
       </c>
-      <c r="E19" s="10">
-        <f>E7-E4</f>
+      <c r="E21" s="10">
+        <f t="shared" si="1"/>
         <v>-221.42920834019969</v>
       </c>
-      <c r="F19" s="10">
-        <f>F7-F4</f>
+      <c r="F21" s="10">
+        <f t="shared" si="1"/>
         <v>896.09976246881979</v>
       </c>
-      <c r="G19" s="10">
-        <f>G7-G4</f>
+      <c r="G21" s="10">
+        <f t="shared" si="1"/>
         <v>-4877.4899349639245</v>
       </c>
-      <c r="H19" s="10">
-        <f>H7-H4</f>
+      <c r="H21" s="10">
+        <f t="shared" si="1"/>
         <v>-4202.8193808354008</v>
       </c>
-      <c r="I19" s="10">
-        <f>I7-I4</f>
+      <c r="I21" s="10">
+        <f t="shared" si="1"/>
         <v>-87.19067491790338</v>
       </c>
-      <c r="J19" s="10">
-        <f>J7-J4</f>
+      <c r="J21" s="10">
+        <f t="shared" si="1"/>
         <v>4424.0083944886992</v>
       </c>
-      <c r="K19" s="10">
-        <f>K7-K4</f>
+      <c r="K21" s="10">
+        <f t="shared" si="1"/>
         <v>625.28660162189772</v>
       </c>
-      <c r="L19" s="10"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A21" t="s">
+      <c r="L21" s="10"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>53</v>
       </c>
-      <c r="D21" s="10">
-        <f>D13-D10</f>
+      <c r="D23" s="10">
+        <f t="shared" ref="D23:K23" si="2">D13-D10</f>
         <v>513.41117027959262</v>
       </c>
-      <c r="E21" s="10">
-        <f>E13-E10</f>
+      <c r="E23" s="10">
+        <f t="shared" si="2"/>
         <v>-214.21539764659974</v>
       </c>
-      <c r="F21" s="10">
-        <f>F13-F10</f>
+      <c r="F23" s="10">
+        <f t="shared" si="2"/>
         <v>-624.4983606493397</v>
       </c>
-      <c r="G21" s="10">
-        <f>G13-G10</f>
+      <c r="G23" s="10">
+        <f t="shared" si="2"/>
         <v>4877.8861089948059</v>
       </c>
-      <c r="H21" s="10">
-        <f>H13-H10</f>
+      <c r="H23" s="10">
+        <f t="shared" si="2"/>
         <v>4039.1723506987983</v>
       </c>
-      <c r="I21" s="10">
-        <f>I13-I10</f>
+      <c r="I23" s="10">
+        <f t="shared" si="2"/>
         <v>183.72486634590314</v>
       </c>
-      <c r="J21" s="10">
-        <f>J13-J10</f>
+      <c r="J23" s="10">
+        <f t="shared" si="2"/>
         <v>-3232.9060231951007</v>
       </c>
-      <c r="K21" s="10">
-        <f>K13-K10</f>
+      <c r="K23" s="10">
+        <f t="shared" si="2"/>
         <v>-476.58002357000078</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>59</v>
+      </c>
+      <c r="D25" s="10">
+        <f>D15-D4</f>
+        <v>1936.486733518308</v>
+      </c>
+      <c r="E25" s="10">
+        <f t="shared" ref="E25:K25" si="3">E15-E4</f>
+        <v>-71.19886349780063</v>
+      </c>
+      <c r="F25" s="10">
+        <f t="shared" si="3"/>
+        <v>774.71175120847056</v>
+      </c>
+      <c r="G25" s="10">
+        <f t="shared" si="3"/>
+        <v>-7.7077004276097796</v>
+      </c>
+      <c r="H25" s="10">
+        <f t="shared" si="3"/>
+        <v>695.80518728300012</v>
+      </c>
+      <c r="I25" s="10">
+        <f t="shared" si="3"/>
+        <v>-89.815674909797963</v>
+      </c>
+      <c r="J25" s="10">
+        <f t="shared" si="3"/>
+        <v>1156.1203736896005</v>
+      </c>
+      <c r="K25" s="10">
+        <f t="shared" si="3"/>
+        <v>174.37684745549996</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>58</v>
+      </c>
+      <c r="D27" s="10">
+        <f>D13-D15</f>
+        <v>-664.57085379362979</v>
+      </c>
+      <c r="E27" s="10">
+        <f t="shared" ref="E27:K27" si="4">E13-E15</f>
+        <v>-366.2840294744019</v>
+      </c>
+      <c r="F27" s="10">
+        <f t="shared" si="4"/>
+        <v>-502.05232305366007</v>
+      </c>
+      <c r="G27" s="10">
+        <f t="shared" si="4"/>
+        <v>8.1038749938497858</v>
+      </c>
+      <c r="H27" s="10">
+        <f t="shared" si="4"/>
+        <v>-860.23247753420219</v>
+      </c>
+      <c r="I27" s="10">
+        <f t="shared" si="4"/>
+        <v>186.34989052249875</v>
+      </c>
+      <c r="J27" s="10">
+        <f t="shared" si="4"/>
+        <v>34.981997603998025</v>
+      </c>
+      <c r="K27" s="10">
+        <f t="shared" si="4"/>
+        <v>-25.670264385902556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Moving around RTP results files
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66918FA3-FAD5-4C54-A23C-85BD4344EEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67044EC2-E46D-4025-9632-FA041108B0BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,6 @@
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
     <author>tc={F9308CF0-AB74-4ABB-91B6-7382ECEADD39}</author>
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
-    <author>tc={7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}</author>
     <author>tc={B12FED98-6BE9-4BE2-A887-4CF314FA442B}</author>
     <author>tc={7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}</author>
     <author>tc={B7EDEAAD-67C9-4693-A0FC-570282E02182}</author>
@@ -170,15 +169,7 @@
     The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A57" authorId="13" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Result from the fast solve</t>
-      </text>
-    </comment>
-    <comment ref="A60" authorId="14" shapeId="0" xr:uid="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
+    <comment ref="A60" authorId="13" shapeId="0" xr:uid="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -186,7 +177,7 @@
     Wrong baseline power was used</t>
       </text>
     </comment>
-    <comment ref="A61" authorId="15" shapeId="0" xr:uid="{7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}">
+    <comment ref="A61" authorId="14" shapeId="0" xr:uid="{7E28AC63-C308-4B0A-97A5-B41EEB6DBCFB}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -194,7 +185,7 @@
     Old solution where there is only one plant shutdown.</t>
       </text>
     </comment>
-    <comment ref="A62" authorId="16" shapeId="0" xr:uid="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
+    <comment ref="A62" authorId="15" shapeId="0" xr:uid="{B7EDEAAD-67C9-4693-A0FC-570282E02182}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -202,7 +193,7 @@
     Solution where there is a shutdown for all peak hours</t>
       </text>
     </comment>
-    <comment ref="A63" authorId="17" shapeId="0" xr:uid="{0EBBD83F-AB64-4248-87E6-B99F88EE5F88}">
+    <comment ref="A63" authorId="16" shapeId="0" xr:uid="{0EBBD83F-AB64-4248-87E6-B99F88EE5F88}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -210,7 +201,7 @@
     Only one plant shutdown allowed</t>
       </text>
     </comment>
-    <comment ref="A68" authorId="18" shapeId="0" xr:uid="{8E704477-0437-40A7-B175-85F6EA0FB52A}">
+    <comment ref="A68" authorId="17" shapeId="0" xr:uid="{8E704477-0437-40A7-B175-85F6EA0FB52A}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -218,7 +209,7 @@
     Including this as the final result</t>
       </text>
     </comment>
-    <comment ref="L69" authorId="19" shapeId="0" xr:uid="{9BC5A461-E691-49A7-9AA5-314B7AD6B728}">
+    <comment ref="L69" authorId="18" shapeId="0" xr:uid="{9BC5A461-E691-49A7-9AA5-314B7AD6B728}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -226,7 +217,7 @@
     Just some random lower recovery periods</t>
       </text>
     </comment>
-    <comment ref="A76" authorId="20" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
+    <comment ref="A76" authorId="19" shapeId="0" xr:uid="{FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -235,7 +226,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="A83" authorId="21" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
+    <comment ref="A83" authorId="20" shapeId="0" xr:uid="{4644E393-F522-4E79-88BA-041770B595A7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -243,7 +234,7 @@
     Pretty sure this solution is wrong, but I don’t think I need this case for the paper</t>
       </text>
     </comment>
-    <comment ref="A89" authorId="22" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
+    <comment ref="A89" authorId="21" shapeId="0" xr:uid="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -251,7 +242,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T101" authorId="23" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T101" authorId="22" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -561,7 +552,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -722,12 +713,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1517,9 +1502,6 @@
   <threadedComment ref="T51" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>The baseline costs have to be updated in accordance with the demand structure type</text>
   </threadedComment>
-  <threadedComment ref="A57" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
-    <text>Result from the fast solve</text>
-  </threadedComment>
   <threadedComment ref="A60" dT="2026-07-21T19:50:00.59" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B12FED98-6BE9-4BE2-A887-4CF314FA442B}">
     <text>Wrong baseline power was used</text>
   </threadedComment>
@@ -3609,7 +3591,7 @@
         <v>0</v>
       </c>
       <c r="P50">
-        <f t="shared" ref="P50:P57" si="11">D50+$P$1</f>
+        <f t="shared" ref="P50:P58" si="11">D50+$P$1</f>
         <v>238413.66244470741</v>
       </c>
       <c r="Q50">
@@ -3889,10 +3871,10 @@
       </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
+      <c r="A57" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C57">
@@ -3900,56 +3882,68 @@
       </c>
       <c r="D57">
         <f>J57+K57+L57+M57+N57</f>
-        <v>125434.46212050831</v>
+        <v>123759.49613284627</v>
       </c>
       <c r="E57">
-        <v>282179.67123444699</v>
+        <v>282179.67123286799</v>
       </c>
       <c r="F57">
-        <v>0.87159189967643702</v>
-      </c>
-      <c r="G57" s="4">
-        <v>21072.189860718699</v>
+        <v>0.86412362052107095</v>
+      </c>
+      <c r="G57">
+        <v>22235.129466751401</v>
       </c>
       <c r="H57">
-        <v>9188.7245080883695</v>
+        <v>9205.4053509202495</v>
       </c>
       <c r="I57">
-        <v>2618.8827210474601</v>
+        <v>0</v>
       </c>
       <c r="J57">
-        <v>32879.797089854597</v>
+        <v>31440.534817671702</v>
       </c>
       <c r="K57">
-        <v>50904.118537438801</v>
+        <v>50868.697977035903</v>
       </c>
       <c r="L57">
-        <v>20591.7266090095</v>
+        <v>20030.700516482098</v>
       </c>
       <c r="M57">
-        <v>20017.890938119701</v>
+        <v>19946.203305120602</v>
       </c>
       <c r="N57">
-        <v>1040.9289460857101</v>
+        <v>1473.35951653596</v>
       </c>
       <c r="O57">
         <v>0</v>
       </c>
       <c r="P57">
-        <f t="shared" si="11"/>
-        <v>245994.13393950483</v>
+        <f>D57+$P$1</f>
+        <v>244319.16795184277</v>
       </c>
       <c r="Q57">
-        <v>1458.3752411216699</v>
+        <v>1461.0227171772699</v>
       </c>
       <c r="R57">
-        <v>35012.612233571497</v>
+        <v>37816.4634857485</v>
       </c>
       <c r="S57">
-        <v>875.31530583928895</v>
+        <v>822.09703229888203</v>
       </c>
       <c r="T57">
-        <v>0.51444695802960605</v>
+        <v>1.67282971584568</v>
+      </c>
+      <c r="U57">
+        <v>43765.040311224599</v>
+      </c>
+      <c r="V57">
+        <v>358.72983861659498</v>
+      </c>
+    </row>
+    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="K58">
+        <f>K57+L57+M57-K5</f>
+        <v>5401.088917483823</v>
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Create folder for sensitivity analysis on start up time
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67044EC2-E46D-4025-9632-FA041108B0BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7560A29D-97F0-4F54-A6E1-36BBAB920F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -264,6 +264,7 @@
     <author>tc={FFA36925-C069-4696-AC82-F35BD29C01EC}</author>
     <author>tc={B28B570C-C764-4378-B61D-458DE4F990EC}</author>
     <author>tc={FA61E68B-2D13-4D2E-B802-33BC32E35571}</author>
+    <author>tc={8E1FBD91-405E-4634-A247-E71AF8AA6758}</author>
     <author>tc={E1A102F6-1CF2-4D48-979A-0181ECF33C11}</author>
     <author>tc={1B8056AB-E255-474B-8036-2D14416413FE}</author>
   </authors>
@@ -339,7 +340,15 @@
     Low key this result is probs not the optimal version of one shutdown...</t>
       </text>
     </comment>
-    <comment ref="J19" authorId="7" shapeId="0" xr:uid="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
+    <comment ref="D14" authorId="7" shapeId="0" xr:uid="{8E1FBD91-405E-4634-A247-E71AF8AA6758}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Percent savings compared to baseline</t>
+      </text>
+    </comment>
+    <comment ref="J19" authorId="8" shapeId="0" xr:uid="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -347,7 +356,7 @@
     For one shutdown - there are significantly longer periods of operation at lower recovery. This occurs because there is more water to shift to off-peak hours, thus more time to be at the lower recovery value (minimizing the demand charge)</t>
       </text>
     </comment>
-    <comment ref="J21" authorId="8" shapeId="0" xr:uid="{1B8056AB-E255-474B-8036-2D14416413FE}">
+    <comment ref="J21" authorId="9" shapeId="0" xr:uid="{1B8056AB-E255-474B-8036-2D14416413FE}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -552,7 +561,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -713,6 +722,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1576,6 +1591,9 @@
   <threadedComment ref="J13" dT="2026-07-31T00:31:51.36" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{53F1C0E0-DC73-4C54-B570-6E2EA35F43E0}" parentId="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
     <text>Low key this result is probs not the optimal version of one shutdown...</text>
   </threadedComment>
+  <threadedComment ref="D14" dT="2026-08-06T01:53:20.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{8E1FBD91-405E-4634-A247-E71AF8AA6758}">
+    <text>Percent savings compared to baseline</text>
+  </threadedComment>
   <threadedComment ref="J19" dT="2026-07-30T22:50:03.35" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
     <text>For one shutdown - there are significantly longer periods of operation at lower recovery. This occurs because there is more water to shift to off-peak hours, thus more time to be at the lower recovery value (minimizing the demand charge)</text>
   </threadedComment>
@@ -1588,21 +1606,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:V104"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" customWidth="1"/>
-    <col min="3" max="3" width="11.453125" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" customWidth="1"/>
-    <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.54296875" customWidth="1"/>
-    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.81640625" customWidth="1"/>
+    <col min="1" max="1" width="9.61328125" customWidth="1"/>
+    <col min="3" max="3" width="11.4609375" customWidth="1"/>
+    <col min="5" max="5" width="10.23046875" customWidth="1"/>
+    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.69140625" customWidth="1"/>
+    <col min="9" max="9" width="9.07421875" customWidth="1"/>
+    <col min="11" max="11" width="10.84375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.53515625" customWidth="1"/>
+    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1613,7 +1631,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1681,7 +1699,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1745,7 +1763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1809,14 +1827,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G5" s="4"/>
       <c r="K5">
         <f>K4+L4+M4</f>
         <v>85444.512881154791</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1880,7 +1898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -1944,10 +1962,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2011,7 +2029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2075,10 +2093,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -2142,7 +2160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2206,10 +2224,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2271,7 +2289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2327,10 +2345,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2394,7 +2412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2458,7 +2476,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2467,7 +2485,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2478,7 +2496,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2542,10 +2560,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2609,7 +2627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2679,11 +2697,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2747,7 +2765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2811,10 +2829,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2878,7 +2896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -2948,7 +2966,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -3018,7 +3036,7 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A33" s="11" t="s">
         <v>45</v>
       </c>
@@ -3101,18 +3119,18 @@
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -3176,7 +3194,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3240,12 +3258,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3312,7 +3330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3382,20 +3400,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3459,15 +3477,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3537,13 +3555,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
@@ -3591,7 +3609,7 @@
         <v>0</v>
       </c>
       <c r="P50">
-        <f t="shared" ref="P50:P58" si="11">D50+$P$1</f>
+        <f t="shared" ref="P50:P56" si="11">D50+$P$1</f>
         <v>238413.66244470741</v>
       </c>
       <c r="Q50">
@@ -3607,7 +3625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
@@ -3671,11 +3689,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -3739,7 +3757,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -3803,10 +3821,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
@@ -3870,7 +3888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A57" s="5" t="s">
         <v>22</v>
       </c>
@@ -3940,19 +3958,19 @@
         <v>358.72983861659498</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.4">
       <c r="K58">
         <f>K57+L57+M57-K5</f>
         <v>5401.088917483823</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -4016,7 +4034,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -4081,7 +4099,7 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A62" s="3" t="s">
         <v>22</v>
       </c>
@@ -4151,7 +4169,7 @@
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -4221,7 +4239,7 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A64" s="11" t="s">
         <v>44</v>
       </c>
@@ -4304,19 +4322,19 @@
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
       <c r="D66" s="10"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A67" s="11" t="s">
         <v>60</v>
       </c>
@@ -4324,7 +4342,7 @@
       <c r="C67" s="9"/>
       <c r="D67" s="10"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A68" s="5" t="s">
         <v>22</v>
       </c>
@@ -4394,7 +4412,7 @@
         <v>350.36946039055402</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A69" s="11" t="s">
         <v>61</v>
       </c>
@@ -4453,7 +4471,7 @@
         <v>133.12347700700047</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -4474,13 +4492,13 @@
       <c r="O70" s="10"/>
       <c r="P70" s="10"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A71" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -4492,7 +4510,7 @@
       </c>
       <c r="G72" s="4"/>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
         <v>22</v>
       </c>
@@ -4556,13 +4574,13 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="G74" s="4"/>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A75" s="3" t="s">
         <v>20</v>
       </c>
@@ -4574,7 +4592,7 @@
       </c>
       <c r="G75" s="4"/>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -4643,7 +4661,7 @@
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="D77">
@@ -4723,12 +4741,12 @@
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A78" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A79" s="3" t="s">
         <v>20</v>
       </c>
@@ -4792,7 +4810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A80" s="3" t="s">
         <v>22</v>
       </c>
@@ -4856,10 +4874,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>20</v>
       </c>
@@ -4917,7 +4935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A83" s="2" t="s">
         <v>22</v>
       </c>
@@ -4981,7 +4999,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>20</v>
       </c>
@@ -5039,7 +5057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
         <v>22</v>
       </c>
@@ -5109,7 +5127,7 @@
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.4">
       <c r="D87">
         <f>D86-D80</f>
         <v>-4018.7603482047853</v>
@@ -5159,13 +5177,13 @@
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A88" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G88" s="4"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -5229,7 +5247,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -5273,8 +5291,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.4"/>
+    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A92" s="1" t="s">
         <v>26</v>
       </c>
@@ -5295,7 +5313,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
         <v>0</v>
       </c>
@@ -5357,7 +5375,7 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A94" s="2" t="s">
         <v>20</v>
       </c>
@@ -5419,12 +5437,12 @@
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A95" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A97" t="s">
         <v>32</v>
       </c>
@@ -5435,7 +5453,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A98">
         <v>20</v>
       </c>
@@ -5499,7 +5517,7 @@
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A99">
         <v>20</v>
       </c>
@@ -5563,7 +5581,7 @@
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A100">
         <v>20</v>
       </c>
@@ -5627,7 +5645,7 @@
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A101">
         <v>20</v>
       </c>
@@ -5691,7 +5709,7 @@
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A102" s="3">
         <v>20</v>
       </c>
@@ -5755,7 +5773,7 @@
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A103">
         <v>20</v>
       </c>
@@ -5819,7 +5837,7 @@
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A104">
         <v>20</v>
       </c>
@@ -5899,20 +5917,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA993591-8C1F-4C7B-A75D-E9726DFB461B}">
   <dimension ref="A2:P27"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="12.81640625" customWidth="1"/>
-    <col min="3" max="3" width="11.36328125" customWidth="1"/>
-    <col min="4" max="4" width="15.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.84375" customWidth="1"/>
+    <col min="3" max="3" width="11.3828125" customWidth="1"/>
+    <col min="4" max="4" width="15.53515625" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17.08984375" customWidth="1"/>
-    <col min="7" max="7" width="15.26953125" customWidth="1"/>
-    <col min="8" max="8" width="13.26953125" customWidth="1"/>
-    <col min="9" max="11" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.07421875" customWidth="1"/>
+    <col min="7" max="7" width="15.23046875" customWidth="1"/>
+    <col min="8" max="8" width="13.23046875" customWidth="1"/>
+    <col min="9" max="11" width="11.3828125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5951,12 +5969,12 @@
       </c>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -5995,7 +6013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="D5" s="10"/>
@@ -6007,7 +6025,7 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>48</v>
       </c>
@@ -6024,7 +6042,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="14.7" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -6064,7 +6082,7 @@
       </c>
       <c r="M7" s="12"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.4">
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -6075,7 +6093,7 @@
       <c r="K8" s="10"/>
       <c r="M8" s="12"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
         <v>49</v>
       </c>
@@ -6089,7 +6107,7 @@
       <c r="K9" s="10"/>
       <c r="M9" s="12"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -6129,7 +6147,7 @@
       </c>
       <c r="M10" s="12"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="D11" s="10"/>
@@ -6142,7 +6160,7 @@
       <c r="K11" s="10"/>
       <c r="M11" s="12"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>46</v>
       </c>
@@ -6155,7 +6173,7 @@
       <c r="J12" s="10"/>
       <c r="K12" s="10"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -6194,7 +6212,17 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="D14">
+        <f>(34653-H13-I14+wrd_pricetater_flex_type_summar!K5+L13)/34653</f>
+        <v>0.38932217950875497</v>
+      </c>
+      <c r="I14" s="10">
+        <f>I13+J13+K13</f>
+        <v>87792.098602195503</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>57</v>
       </c>
@@ -6233,7 +6261,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>51</v>
       </c>
@@ -6241,7 +6269,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>52</v>
       </c>
@@ -6279,7 +6307,7 @@
       </c>
       <c r="L19" s="10"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>55</v>
       </c>
@@ -6317,7 +6345,7 @@
       </c>
       <c r="L21" s="10"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>53</v>
       </c>
@@ -6354,7 +6382,7 @@
         <v>-476.58002357000078</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>59</v>
       </c>
@@ -6391,7 +6419,7 @@
         <v>174.37684745549996</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
testing 1 hr start-up with 5 shutdowns
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7560A29D-97F0-4F54-A6E1-36BBAB920F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7882DF40-535F-4A2F-B31F-3963AB7D704C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" activeTab="1" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -260,6 +260,7 @@
     <author>tc={D913FCAB-030D-49E3-A7A0-5803B7027754}</author>
     <author>tc={59DFC78E-5F9D-4D05-9892-2664283F148D}</author>
     <author>tc={5DA58C15-B5CA-4552-8F53-D4819003ECD4}</author>
+    <author>tc={DBFBEADE-D533-486A-B634-A22EF73696DB}</author>
     <author>tc={2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}</author>
     <author>tc={FFA36925-C069-4696-AC82-F35BD29C01EC}</author>
     <author>tc={B28B570C-C764-4378-B61D-458DE4F990EC}</author>
@@ -298,7 +299,15 @@
 133 hrs = 277 m3/hr (97 m3/hr from UF, remainer 45 m3/hr per train at 92.2% RR)</t>
       </text>
     </comment>
-    <comment ref="A10" authorId="3" shapeId="0" xr:uid="{2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}">
+    <comment ref="A9" authorId="3" shapeId="0" xr:uid="{DBFBEADE-D533-486A-B634-A22EF73696DB}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not optimal. The solution above has no shutdowns and is better</t>
+      </text>
+    </comment>
+    <comment ref="A13" authorId="4" shapeId="0" xr:uid="{2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -308,7 +317,7 @@
     I’d like to see numbers for only one shutdown</t>
       </text>
     </comment>
-    <comment ref="J10" authorId="4" shapeId="0" xr:uid="{FFA36925-C069-4696-AC82-F35BD29C01EC}">
+    <comment ref="J13" authorId="5" shapeId="0" xr:uid="{FFA36925-C069-4696-AC82-F35BD29C01EC}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -318,7 +327,7 @@
 133 hrs = 277 m3/hr (97 m3/hr from UF, remainer 45 m3/hr per train at 92.2% RR)</t>
       </text>
     </comment>
-    <comment ref="A13" authorId="5" shapeId="0" xr:uid="{B28B570C-C764-4378-B61D-458DE4F990EC}">
+    <comment ref="A16" authorId="6" shapeId="0" xr:uid="{B28B570C-C764-4378-B61D-458DE4F990EC}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -326,7 +335,7 @@
     Only one plant shutdown allowed</t>
       </text>
     </comment>
-    <comment ref="J13" authorId="6" shapeId="0" xr:uid="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
+    <comment ref="J16" authorId="7" shapeId="0" xr:uid="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -340,7 +349,7 @@
     Low key this result is probs not the optimal version of one shutdown...</t>
       </text>
     </comment>
-    <comment ref="D14" authorId="7" shapeId="0" xr:uid="{8E1FBD91-405E-4634-A247-E71AF8AA6758}">
+    <comment ref="D17" authorId="8" shapeId="0" xr:uid="{8E1FBD91-405E-4634-A247-E71AF8AA6758}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -348,7 +357,7 @@
     Percent savings compared to baseline</t>
       </text>
     </comment>
-    <comment ref="J19" authorId="8" shapeId="0" xr:uid="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
+    <comment ref="J23" authorId="9" shapeId="0" xr:uid="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -356,7 +365,7 @@
     For one shutdown - there are significantly longer periods of operation at lower recovery. This occurs because there is more water to shift to off-peak hours, thus more time to be at the lower recovery value (minimizing the demand charge)</t>
       </text>
     </comment>
-    <comment ref="J21" authorId="9" shapeId="0" xr:uid="{1B8056AB-E255-474B-8036-2D14416413FE}">
+    <comment ref="J25" authorId="10" shapeId="0" xr:uid="{1B8056AB-E255-474B-8036-2D14416413FE}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -369,7 +378,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="63">
   <si>
     <t>Season</t>
   </si>
@@ -555,6 +564,9 @@
   </si>
   <si>
     <t>Delayed Shutdowns vs. None</t>
+  </si>
+  <si>
+    <t>NO DR, 1 HR Start-Up, NO SHUTDOWN</t>
   </si>
 </sst>
 </file>
@@ -1089,7 +1101,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1567,37 +1579,40 @@
 10 hours = 1083 m3/hr (from 2 Ro trains @ 520 + UF)
 133 hrs = 277 m3/hr (97 m3/hr from UF, remainer 45 m3/hr per train at 92.2% RR)</text>
   </threadedComment>
-  <threadedComment ref="A10" dT="2026-07-22T19:29:10.19" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}">
+  <threadedComment ref="A9" dT="2026-08-06T15:32:55.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{DBFBEADE-D533-486A-B634-A22EF73696DB}">
+    <text>Not optimal. The solution above has no shutdowns and is better</text>
+  </threadedComment>
+  <threadedComment ref="A13" dT="2026-07-22T19:29:10.19" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}">
     <text>Solution where there is a shutdown for all peak hours</text>
   </threadedComment>
-  <threadedComment ref="A10" dT="2026-07-22T19:37:51.21" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{17E89EDA-58B7-4160-A587-C8F02064EE42}" parentId="{2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}">
+  <threadedComment ref="A13" dT="2026-07-22T19:37:51.21" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{17E89EDA-58B7-4160-A587-C8F02064EE42}" parentId="{2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}">
     <text>I’d like to see numbers for only one shutdown</text>
   </threadedComment>
-  <threadedComment ref="J10" dT="2026-07-30T23:48:23.68" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FFA36925-C069-4696-AC82-F35BD29C01EC}">
+  <threadedComment ref="J13" dT="2026-07-30T23:48:23.68" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FFA36925-C069-4696-AC82-F35BD29C01EC}">
     <text>25 hrs = 0 brine
 10 hours = 1083 m3/hr (from 2 Ro trains @ 520 + UF)
 133 hrs = 277 m3/hr (97 m3/hr from UF, remainer 45 m3/hr per train at 92.2% RR)</text>
   </threadedComment>
-  <threadedComment ref="A13" dT="2026-07-22T21:09:49.14" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B28B570C-C764-4378-B61D-458DE4F990EC}">
+  <threadedComment ref="A16" dT="2026-07-22T21:09:49.14" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B28B570C-C764-4378-B61D-458DE4F990EC}">
     <text>Only one plant shutdown allowed</text>
   </threadedComment>
-  <threadedComment ref="J13" dT="2026-07-31T00:30:46.97" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
+  <threadedComment ref="J16" dT="2026-07-31T00:30:46.97" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
     <text>5 hrs = 0 brine
 2 hrs = 1083 m3/hr
 82 hrs = 270 m3/hr
 8 hrs = 133 m3/hr @ low RR
 Remaining = ~220 m3/hr</text>
   </threadedComment>
-  <threadedComment ref="J13" dT="2026-07-31T00:31:51.36" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{53F1C0E0-DC73-4C54-B570-6E2EA35F43E0}" parentId="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
+  <threadedComment ref="J16" dT="2026-07-31T00:31:51.36" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{53F1C0E0-DC73-4C54-B570-6E2EA35F43E0}" parentId="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
     <text>Low key this result is probs not the optimal version of one shutdown...</text>
   </threadedComment>
-  <threadedComment ref="D14" dT="2026-08-06T01:53:20.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{8E1FBD91-405E-4634-A247-E71AF8AA6758}">
+  <threadedComment ref="D17" dT="2026-08-06T01:53:20.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{8E1FBD91-405E-4634-A247-E71AF8AA6758}">
     <text>Percent savings compared to baseline</text>
   </threadedComment>
-  <threadedComment ref="J19" dT="2026-07-30T22:50:03.35" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
+  <threadedComment ref="J23" dT="2026-07-30T22:50:03.35" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
     <text>For one shutdown - there are significantly longer periods of operation at lower recovery. This occurs because there is more water to shift to off-peak hours, thus more time to be at the lower recovery value (minimizing the demand charge)</text>
   </threadedComment>
-  <threadedComment ref="J21" dT="2026-07-30T23:11:38.86" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{1B8056AB-E255-474B-8036-2D14416413FE}">
+  <threadedComment ref="J25" dT="2026-07-30T23:11:38.86" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{1B8056AB-E255-474B-8036-2D14416413FE}">
     <text>Slightly reduced recovery at 0.922 to get to 578 Feed flowrate. Plus the  start-up parts</text>
   </threadedComment>
 </ThreadedComments>
@@ -1606,21 +1621,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:V104"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.61328125" customWidth="1"/>
-    <col min="3" max="3" width="11.4609375" customWidth="1"/>
-    <col min="5" max="5" width="10.23046875" customWidth="1"/>
-    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.69140625" customWidth="1"/>
-    <col min="9" max="9" width="9.07421875" customWidth="1"/>
-    <col min="11" max="11" width="10.84375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.53515625" customWidth="1"/>
-    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.84375" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" customWidth="1"/>
+    <col min="3" max="3" width="11.453125" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.54296875" customWidth="1"/>
+    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1631,7 +1646,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1699,7 +1714,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1763,7 +1778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1827,14 +1842,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G5" s="4"/>
       <c r="K5">
         <f>K4+L4+M4</f>
         <v>85444.512881154791</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1898,7 +1913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -1962,10 +1977,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2029,7 +2044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2093,10 +2108,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -2160,7 +2175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2224,10 +2239,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2289,7 +2304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2345,10 +2360,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2412,7 +2427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2476,7 +2491,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2485,7 +2500,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2496,7 +2511,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2560,10 +2575,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2627,7 +2642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2697,11 +2712,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2765,7 +2780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2829,10 +2844,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2896,7 +2911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -2966,7 +2981,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -3036,7 +3051,7 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A33" s="11" t="s">
         <v>45</v>
       </c>
@@ -3119,18 +3134,18 @@
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -3194,7 +3209,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3258,12 +3273,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3330,7 +3345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3400,20 +3415,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3477,15 +3492,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3555,13 +3570,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
@@ -3625,7 +3640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
@@ -3689,11 +3704,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -3757,7 +3772,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -3821,10 +3836,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
@@ -3888,7 +3903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>22</v>
       </c>
@@ -3958,19 +3973,19 @@
         <v>358.72983861659498</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
       <c r="K58">
         <f>K57+L57+M57-K5</f>
         <v>5401.088917483823</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -4034,7 +4049,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -4099,7 +4114,7 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
         <v>22</v>
       </c>
@@ -4169,7 +4184,7 @@
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -4239,7 +4254,7 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A64" s="11" t="s">
         <v>44</v>
       </c>
@@ -4322,19 +4337,19 @@
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
       <c r="D66" s="10"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A67" s="11" t="s">
         <v>60</v>
       </c>
@@ -4342,7 +4357,7 @@
       <c r="C67" s="9"/>
       <c r="D67" s="10"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
         <v>22</v>
       </c>
@@ -4412,7 +4427,7 @@
         <v>350.36946039055402</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A69" s="11" t="s">
         <v>61</v>
       </c>
@@ -4471,7 +4486,7 @@
         <v>133.12347700700047</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -4492,13 +4507,13 @@
       <c r="O70" s="10"/>
       <c r="P70" s="10"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -4510,7 +4525,7 @@
       </c>
       <c r="G72" s="4"/>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>22</v>
       </c>
@@ -4574,13 +4589,13 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="G74" s="4"/>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
         <v>20</v>
       </c>
@@ -4592,7 +4607,7 @@
       </c>
       <c r="G75" s="4"/>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -4661,7 +4676,7 @@
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="D77">
@@ -4741,12 +4756,12 @@
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
         <v>20</v>
       </c>
@@ -4810,7 +4825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
         <v>22</v>
       </c>
@@ -4874,10 +4889,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>20</v>
       </c>
@@ -4935,7 +4950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>22</v>
       </c>
@@ -4999,7 +5014,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>20</v>
       </c>
@@ -5057,7 +5072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>22</v>
       </c>
@@ -5127,7 +5142,7 @@
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.35">
       <c r="D87">
         <f>D86-D80</f>
         <v>-4018.7603482047853</v>
@@ -5177,13 +5192,13 @@
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G88" s="4"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -5247,7 +5262,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -5291,8 +5306,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.4"/>
-    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>26</v>
       </c>
@@ -5313,7 +5328,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>0</v>
       </c>
@@ -5375,7 +5390,7 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>20</v>
       </c>
@@ -5437,12 +5452,12 @@
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A95" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>32</v>
       </c>
@@ -5453,7 +5468,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>20</v>
       </c>
@@ -5517,7 +5532,7 @@
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>20</v>
       </c>
@@ -5581,7 +5596,7 @@
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>20</v>
       </c>
@@ -5645,7 +5660,7 @@
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>20</v>
       </c>
@@ -5709,7 +5724,7 @@
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A102" s="3">
         <v>20</v>
       </c>
@@ -5773,7 +5788,7 @@
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>20</v>
       </c>
@@ -5837,7 +5852,7 @@
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>20</v>
       </c>
@@ -5916,21 +5931,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA993591-8C1F-4C7B-A75D-E9726DFB461B}">
-  <dimension ref="A2:P27"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A2:P31"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="12.84375" customWidth="1"/>
-    <col min="3" max="3" width="11.3828125" customWidth="1"/>
-    <col min="4" max="4" width="15.53515625" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" customWidth="1"/>
+    <col min="3" max="3" width="11.36328125" customWidth="1"/>
+    <col min="4" max="4" width="15.54296875" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17.07421875" customWidth="1"/>
-    <col min="7" max="7" width="15.23046875" customWidth="1"/>
-    <col min="8" max="8" width="13.23046875" customWidth="1"/>
-    <col min="9" max="11" width="11.3828125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" customWidth="1"/>
+    <col min="7" max="7" width="15.26953125" customWidth="1"/>
+    <col min="8" max="8" width="13.26953125" customWidth="1"/>
+    <col min="9" max="11" width="11.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5969,12 +5984,12 @@
       </c>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -6013,7 +6028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="D5" s="10"/>
@@ -6025,7 +6040,7 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>48</v>
       </c>
@@ -6042,7 +6057,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.7" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -6082,7 +6097,7 @@
       </c>
       <c r="M7" s="12"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -6093,9 +6108,9 @@
       <c r="K8" s="10"/>
       <c r="M8" s="12"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A9" s="3" t="s">
-        <v>49</v>
+    <row r="9" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>62</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
@@ -6107,49 +6122,38 @@
       <c r="K9" s="10"/>
       <c r="M9" s="12"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A10" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10">
-        <v>4</v>
-      </c>
+    <row r="10" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D10" s="10">
         <f>H10+I10+J10+K10</f>
-        <v>117112.9202243583</v>
-      </c>
-      <c r="E10" s="10">
-        <v>19617.269555424798</v>
-      </c>
-      <c r="F10" s="10">
-        <v>6177.79087142139</v>
-      </c>
-      <c r="G10" s="10">
-        <v>1.4897343661976701E-5</v>
-      </c>
-      <c r="H10" s="10">
-        <v>25795.060441743601</v>
-      </c>
-      <c r="I10" s="10">
-        <v>50989.945229661498</v>
-      </c>
-      <c r="J10" s="10">
-        <v>20356.5524429125</v>
-      </c>
-      <c r="K10" s="10">
-        <v>19971.3621100407</v>
+        <v>116423.6512611575</v>
+      </c>
+      <c r="E10">
+        <v>19793.405782867099</v>
+      </c>
+      <c r="F10">
+        <v>5278.7073577880201</v>
+      </c>
+      <c r="G10">
+        <v>4906.1393788565601</v>
+      </c>
+      <c r="H10">
+        <v>29978.252519511701</v>
+      </c>
+      <c r="I10">
+        <v>51100.150850479702</v>
+      </c>
+      <c r="J10">
+        <v>15994.396781481701</v>
+      </c>
+      <c r="K10">
+        <v>19350.851109684401</v>
       </c>
       <c r="L10">
-        <v>11020</v>
+        <v>0</v>
       </c>
       <c r="M10" s="12"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -6160,9 +6164,9 @@
       <c r="K11" s="10"/>
       <c r="M11" s="12"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
@@ -6172,12 +6176,13 @@
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
       <c r="K12" s="10"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
+      <c r="M12" s="12"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C13">
@@ -6185,281 +6190,344 @@
       </c>
       <c r="D13" s="10">
         <f>H13+I13+J13+K13</f>
-        <v>117626.33139463789</v>
+        <v>117112.9202243583</v>
       </c>
       <c r="E13" s="10">
-        <v>19403.054157778199</v>
+        <v>19617.269555424798</v>
       </c>
       <c r="F13" s="10">
-        <v>5553.2925107720503</v>
+        <v>6177.79087142139</v>
       </c>
       <c r="G13" s="10">
-        <v>4877.88612389215</v>
+        <v>1.4897343661976701E-5</v>
       </c>
       <c r="H13" s="10">
-        <v>29834.232792442399</v>
+        <v>25795.060441743601</v>
       </c>
       <c r="I13" s="10">
-        <v>51173.670096007401</v>
+        <v>50989.945229661498</v>
       </c>
       <c r="J13" s="10">
-        <v>17123.646419717399</v>
+        <v>20356.5524429125</v>
       </c>
       <c r="K13" s="10">
-        <v>19494.782086470699</v>
+        <v>19971.3621100407</v>
       </c>
       <c r="L13">
         <v>11020</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="D14">
-        <f>(34653-H13-I14+wrd_pricetater_flex_type_summar!K5+L13)/34653</f>
+      <c r="M13" s="12"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="M14" s="12"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16">
+        <v>4</v>
+      </c>
+      <c r="D16" s="10">
+        <f>H16+I16+J16+K16</f>
+        <v>117626.33139463789</v>
+      </c>
+      <c r="E16" s="10">
+        <v>19403.054157778199</v>
+      </c>
+      <c r="F16" s="10">
+        <v>5553.2925107720503</v>
+      </c>
+      <c r="G16" s="10">
+        <v>4877.88612389215</v>
+      </c>
+      <c r="H16" s="10">
+        <v>29834.232792442399</v>
+      </c>
+      <c r="I16" s="10">
+        <v>51173.670096007401</v>
+      </c>
+      <c r="J16" s="10">
+        <v>17123.646419717399</v>
+      </c>
+      <c r="K16" s="10">
+        <v>19494.782086470699</v>
+      </c>
+      <c r="L16">
+        <v>11020</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="D17">
+        <f>(34653-H16-I17+wrd_pricetater_flex_type_summar!K5+L16)/34653</f>
         <v>0.38932217950875497</v>
       </c>
-      <c r="I14" s="10">
-        <f>I13+J13+K13</f>
+      <c r="I17" s="10">
+        <f>I16+J16+K16</f>
         <v>87792.098602195503</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A15" s="3" t="s">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A18" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B18" t="s">
         <v>21</v>
       </c>
-      <c r="C15">
+      <c r="C18">
         <v>4</v>
       </c>
-      <c r="D15" s="10">
-        <f>H15+I15+J15+K15</f>
+      <c r="D18" s="10">
+        <f>H18+I18+J18+K18</f>
         <v>118290.90224843152</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E18" s="10">
         <v>19769.338187252601</v>
       </c>
-      <c r="F15" s="10">
+      <c r="F18" s="10">
         <v>6055.3448338257103</v>
       </c>
-      <c r="G15" s="10">
+      <c r="G18" s="10">
         <v>4869.7822488983002</v>
       </c>
-      <c r="H15" s="10">
+      <c r="H18" s="10">
         <v>30694.465269976601</v>
       </c>
-      <c r="I15" s="10">
+      <c r="I18" s="10">
         <v>50987.320205484903</v>
       </c>
-      <c r="J15" s="10">
+      <c r="J18" s="10">
         <v>17088.664422113401</v>
       </c>
-      <c r="K15" s="10">
+      <c r="K18" s="10">
         <v>19520.452350856602</v>
       </c>
-      <c r="L15">
+      <c r="L18">
         <v>11020</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A18" t="s">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>51</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J22" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A19" t="s">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="10">
-        <f>D13-D4</f>
+      <c r="D23" s="10">
+        <f>D16-D4</f>
         <v>1271.9158797246782</v>
       </c>
-      <c r="E19" s="10">
-        <f t="shared" ref="E19:K19" si="0">E13-E4</f>
+      <c r="E23" s="10">
+        <f t="shared" ref="E23:K23" si="0">E16-E4</f>
         <v>-437.48289297220254</v>
       </c>
-      <c r="F19" s="10">
+      <c r="F23" s="10">
         <f t="shared" si="0"/>
         <v>272.65942815481048</v>
       </c>
-      <c r="G19" s="10">
+      <c r="G23" s="10">
         <f t="shared" si="0"/>
         <v>0.39617456624000624</v>
       </c>
-      <c r="H19" s="10">
+      <c r="H23" s="10">
         <f t="shared" si="0"/>
         <v>-164.42729025120207</v>
       </c>
-      <c r="I19" s="10">
+      <c r="I23" s="10">
         <f t="shared" si="0"/>
         <v>96.534215612700791</v>
       </c>
-      <c r="J19" s="10">
+      <c r="J23" s="10">
         <f t="shared" si="0"/>
         <v>1191.1023712935985</v>
       </c>
-      <c r="K19" s="10">
+      <c r="K23" s="10">
         <f t="shared" si="0"/>
         <v>148.7065830695974</v>
       </c>
-      <c r="L19" s="10"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A21" t="s">
+      <c r="L23" s="10"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>55</v>
       </c>
-      <c r="D21" s="10">
-        <f t="shared" ref="D21:K21" si="1">D7-D4</f>
+      <c r="D25" s="10">
+        <f t="shared" ref="D25:K25" si="1">D7-D4</f>
         <v>759.28494035729091</v>
       </c>
-      <c r="E21" s="10">
+      <c r="E25" s="10">
         <f t="shared" si="1"/>
         <v>-221.42920834019969</v>
       </c>
-      <c r="F21" s="10">
+      <c r="F25" s="10">
         <f t="shared" si="1"/>
         <v>896.09976246881979</v>
       </c>
-      <c r="G21" s="10">
+      <c r="G25" s="10">
         <f t="shared" si="1"/>
         <v>-4877.4899349639245</v>
       </c>
-      <c r="H21" s="10">
+      <c r="H25" s="10">
         <f t="shared" si="1"/>
         <v>-4202.8193808354008</v>
       </c>
-      <c r="I21" s="10">
+      <c r="I25" s="10">
         <f t="shared" si="1"/>
         <v>-87.19067491790338</v>
       </c>
-      <c r="J21" s="10">
+      <c r="J25" s="10">
         <f t="shared" si="1"/>
         <v>4424.0083944886992</v>
       </c>
-      <c r="K21" s="10">
+      <c r="K25" s="10">
         <f t="shared" si="1"/>
         <v>625.28660162189772</v>
       </c>
-      <c r="L21" s="10"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A23" t="s">
+      <c r="L25" s="10"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="10">
-        <f t="shared" ref="D23:K23" si="2">D13-D10</f>
+      <c r="D27" s="10">
+        <f t="shared" ref="D27:K27" si="2">D16-D13</f>
         <v>513.41117027959262</v>
       </c>
-      <c r="E23" s="10">
+      <c r="E27" s="10">
         <f t="shared" si="2"/>
         <v>-214.21539764659974</v>
       </c>
-      <c r="F23" s="10">
+      <c r="F27" s="10">
         <f t="shared" si="2"/>
         <v>-624.4983606493397</v>
       </c>
-      <c r="G23" s="10">
+      <c r="G27" s="10">
         <f t="shared" si="2"/>
         <v>4877.8861089948059</v>
       </c>
-      <c r="H23" s="10">
+      <c r="H27" s="10">
         <f t="shared" si="2"/>
         <v>4039.1723506987983</v>
       </c>
-      <c r="I23" s="10">
+      <c r="I27" s="10">
         <f t="shared" si="2"/>
         <v>183.72486634590314</v>
       </c>
-      <c r="J23" s="10">
+      <c r="J27" s="10">
         <f t="shared" si="2"/>
         <v>-3232.9060231951007</v>
       </c>
-      <c r="K23" s="10">
+      <c r="K27" s="10">
         <f t="shared" si="2"/>
         <v>-476.58002357000078</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A25" t="s">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>59</v>
       </c>
-      <c r="D25" s="10">
-        <f>D15-D4</f>
+      <c r="D29" s="10">
+        <f>D18-D4</f>
         <v>1936.486733518308</v>
       </c>
-      <c r="E25" s="10">
-        <f t="shared" ref="E25:K25" si="3">E15-E4</f>
+      <c r="E29" s="10">
+        <f t="shared" ref="E29:K29" si="3">E18-E4</f>
         <v>-71.19886349780063</v>
       </c>
-      <c r="F25" s="10">
+      <c r="F29" s="10">
         <f t="shared" si="3"/>
         <v>774.71175120847056</v>
       </c>
-      <c r="G25" s="10">
+      <c r="G29" s="10">
         <f t="shared" si="3"/>
         <v>-7.7077004276097796</v>
       </c>
-      <c r="H25" s="10">
+      <c r="H29" s="10">
         <f t="shared" si="3"/>
         <v>695.80518728300012</v>
       </c>
-      <c r="I25" s="10">
+      <c r="I29" s="10">
         <f t="shared" si="3"/>
         <v>-89.815674909797963</v>
       </c>
-      <c r="J25" s="10">
+      <c r="J29" s="10">
         <f t="shared" si="3"/>
         <v>1156.1203736896005</v>
       </c>
-      <c r="K25" s="10">
+      <c r="K29" s="10">
         <f t="shared" si="3"/>
         <v>174.37684745549996</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A27" t="s">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>58</v>
       </c>
-      <c r="D27" s="10">
-        <f>D13-D15</f>
+      <c r="D31" s="10">
+        <f>D16-D18</f>
         <v>-664.57085379362979</v>
       </c>
-      <c r="E27" s="10">
-        <f t="shared" ref="E27:K27" si="4">E13-E15</f>
+      <c r="E31" s="10">
+        <f t="shared" ref="E31:K31" si="4">E16-E18</f>
         <v>-366.2840294744019</v>
       </c>
-      <c r="F27" s="10">
+      <c r="F31" s="10">
         <f t="shared" si="4"/>
         <v>-502.05232305366007</v>
       </c>
-      <c r="G27" s="10">
+      <c r="G31" s="10">
         <f t="shared" si="4"/>
         <v>8.1038749938497858</v>
       </c>
-      <c r="H27" s="10">
+      <c r="H31" s="10">
         <f t="shared" si="4"/>
         <v>-860.23247753420219</v>
       </c>
-      <c r="I27" s="10">
+      <c r="I31" s="10">
         <f t="shared" si="4"/>
         <v>186.34989052249875</v>
       </c>
-      <c r="J27" s="10">
+      <c r="J31" s="10">
         <f t="shared" si="4"/>
         <v>34.981997603998025</v>
       </c>
-      <c r="K27" s="10">
+      <c r="K31" s="10">
         <f t="shared" si="4"/>
         <v>-25.670264385902556</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="M6:M11"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Cleaning up results files
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7882DF40-535F-4A2F-B31F-3963AB7D704C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D1FE8ED-83C4-44C2-B5FD-1D5D4D3EABAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" activeTab="1" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -58,6 +58,8 @@
     <author>tc={FD7ED5AD-FD5F-4506-A4A6-ADC8FF8FAC50}</author>
     <author>tc={4644E393-F522-4E79-88BA-041770B595A7}</author>
     <author>tc={9FF6B967-6104-43AC-8EED-15C48C9ACCA9}</author>
+    <author>tc={3B63C6BF-9DE1-4172-A721-F97EE0406603}</author>
+    <author>tc={FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}</author>
     <author>tc={86E634AB-9E52-4A6D-BE85-5D191C9227C6}</author>
   </authors>
   <commentList>
@@ -242,7 +244,23 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="T101" authorId="22" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="A98" authorId="22" shapeId="0" xr:uid="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    2.5x higher brine costs (1.08$/m3)</t>
+      </text>
+    </comment>
+    <comment ref="A101" authorId="23" shapeId="0" xr:uid="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    5x brine costs (2.15 $/m3)</t>
+      </text>
+    </comment>
+    <comment ref="T112" authorId="24" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -260,7 +278,8 @@
     <author>tc={D913FCAB-030D-49E3-A7A0-5803B7027754}</author>
     <author>tc={59DFC78E-5F9D-4D05-9892-2664283F148D}</author>
     <author>tc={5DA58C15-B5CA-4552-8F53-D4819003ECD4}</author>
-    <author>tc={DBFBEADE-D533-486A-B634-A22EF73696DB}</author>
+    <author>tc={A01F3DDE-54D6-40A4-B739-116C1106945C}</author>
+    <author>tc={430DB353-1291-4F52-9F24-0C56C9367687}</author>
     <author>tc={2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}</author>
     <author>tc={FFA36925-C069-4696-AC82-F35BD29C01EC}</author>
     <author>tc={B28B570C-C764-4378-B61D-458DE4F990EC}</author>
@@ -299,15 +318,23 @@
 133 hrs = 277 m3/hr (97 m3/hr from UF, remainer 45 m3/hr per train at 92.2% RR)</t>
       </text>
     </comment>
-    <comment ref="A9" authorId="3" shapeId="0" xr:uid="{DBFBEADE-D533-486A-B634-A22EF73696DB}">
+    <comment ref="A9" authorId="3" shapeId="0" xr:uid="{A01F3DDE-54D6-40A4-B739-116C1106945C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Not optimal. The solution above has no shutdowns and is better</t>
+    Has 5 shutdowns as expected</t>
       </text>
     </comment>
-    <comment ref="A13" authorId="4" shapeId="0" xr:uid="{2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}">
+    <comment ref="D11" authorId="4" shapeId="0" xr:uid="{430DB353-1291-4F52-9F24-0C56C9367687}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Percent savings compared to baseline</t>
+      </text>
+    </comment>
+    <comment ref="A13" authorId="5" shapeId="0" xr:uid="{2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -317,7 +344,7 @@
     I’d like to see numbers for only one shutdown</t>
       </text>
     </comment>
-    <comment ref="J13" authorId="5" shapeId="0" xr:uid="{FFA36925-C069-4696-AC82-F35BD29C01EC}">
+    <comment ref="J13" authorId="6" shapeId="0" xr:uid="{FFA36925-C069-4696-AC82-F35BD29C01EC}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -327,7 +354,7 @@
 133 hrs = 277 m3/hr (97 m3/hr from UF, remainer 45 m3/hr per train at 92.2% RR)</t>
       </text>
     </comment>
-    <comment ref="A16" authorId="6" shapeId="0" xr:uid="{B28B570C-C764-4378-B61D-458DE4F990EC}">
+    <comment ref="A16" authorId="7" shapeId="0" xr:uid="{B28B570C-C764-4378-B61D-458DE4F990EC}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -335,7 +362,7 @@
     Only one plant shutdown allowed</t>
       </text>
     </comment>
-    <comment ref="J16" authorId="7" shapeId="0" xr:uid="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
+    <comment ref="J16" authorId="8" shapeId="0" xr:uid="{FA61E68B-2D13-4D2E-B802-33BC32E35571}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -349,7 +376,7 @@
     Low key this result is probs not the optimal version of one shutdown...</t>
       </text>
     </comment>
-    <comment ref="D17" authorId="8" shapeId="0" xr:uid="{8E1FBD91-405E-4634-A247-E71AF8AA6758}">
+    <comment ref="D17" authorId="9" shapeId="0" xr:uid="{8E1FBD91-405E-4634-A247-E71AF8AA6758}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -357,7 +384,7 @@
     Percent savings compared to baseline</t>
       </text>
     </comment>
-    <comment ref="J23" authorId="9" shapeId="0" xr:uid="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
+    <comment ref="J23" authorId="10" shapeId="0" xr:uid="{E1A102F6-1CF2-4D48-979A-0181ECF33C11}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -365,7 +392,7 @@
     For one shutdown - there are significantly longer periods of operation at lower recovery. This occurs because there is more water to shift to off-peak hours, thus more time to be at the lower recovery value (minimizing the demand charge)</t>
       </text>
     </comment>
-    <comment ref="J25" authorId="10" shapeId="0" xr:uid="{1B8056AB-E255-474B-8036-2D14416413FE}">
+    <comment ref="J25" authorId="11" shapeId="0" xr:uid="{1B8056AB-E255-474B-8036-2D14416413FE}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -378,7 +405,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="64">
   <si>
     <t>Season</t>
   </si>
@@ -566,14 +593,21 @@
     <t>Delayed Shutdowns vs. None</t>
   </si>
   <si>
-    <t>NO DR, 1 HR Start-Up, NO SHUTDOWN</t>
+    <t>NO DR, 1 HR Start-Up</t>
+  </si>
+  <si>
+    <t>Higher Brine Costs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -734,12 +768,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1083,7 +1111,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1097,11 +1125,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1557,7 +1587,13 @@
   <threadedComment ref="A89" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
     <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
   </threadedComment>
-  <threadedComment ref="T101" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="A98" dT="2026-08-09T17:04:16.49" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
+    <text>2.5x higher brine costs (1.08$/m3)</text>
+  </threadedComment>
+  <threadedComment ref="A101" dT="2026-08-09T17:05:17.32" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
+    <text>5x brine costs (2.15 $/m3)</text>
+  </threadedComment>
+  <threadedComment ref="T112" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1579,8 +1615,11 @@
 10 hours = 1083 m3/hr (from 2 Ro trains @ 520 + UF)
 133 hrs = 277 m3/hr (97 m3/hr from UF, remainer 45 m3/hr per train at 92.2% RR)</text>
   </threadedComment>
-  <threadedComment ref="A9" dT="2026-08-06T15:32:55.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{DBFBEADE-D533-486A-B634-A22EF73696DB}">
-    <text>Not optimal. The solution above has no shutdowns and is better</text>
+  <threadedComment ref="A9" dT="2026-08-09T16:59:47.14" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{A01F3DDE-54D6-40A4-B739-116C1106945C}">
+    <text>Has 5 shutdowns as expected</text>
+  </threadedComment>
+  <threadedComment ref="D11" dT="2026-08-06T01:53:20.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{430DB353-1291-4F52-9F24-0C56C9367687}">
+    <text>Percent savings compared to baseline</text>
   </threadedComment>
   <threadedComment ref="A13" dT="2026-07-22T19:29:10.19" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{2A87BE78-C559-43AE-95E9-B9B1CDADA8AE}">
     <text>Solution where there is a shutdown for all peak hours</text>
@@ -1620,22 +1659,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:V104"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:V115"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" customWidth="1"/>
-    <col min="3" max="3" width="11.453125" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" customWidth="1"/>
-    <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.54296875" customWidth="1"/>
-    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.81640625" customWidth="1"/>
+    <col min="1" max="1" width="9.61328125" customWidth="1"/>
+    <col min="3" max="3" width="11.4609375" customWidth="1"/>
+    <col min="5" max="5" width="10.23046875" customWidth="1"/>
+    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.69140625" customWidth="1"/>
+    <col min="9" max="9" width="9.07421875" customWidth="1"/>
+    <col min="11" max="11" width="10.84375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.53515625" customWidth="1"/>
+    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1646,7 +1685,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1714,7 +1753,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1778,7 +1817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1842,14 +1881,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G5" s="4"/>
-      <c r="K5">
+      <c r="K5" s="10">
         <f>K4+L4+M4</f>
         <v>85444.512881154791</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1913,7 +1952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -1977,10 +2016,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2044,7 +2083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2108,10 +2147,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -2175,7 +2214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2239,10 +2278,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2304,7 +2343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2360,10 +2399,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2427,7 +2466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2491,7 +2530,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2500,7 +2539,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2511,7 +2550,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2575,10 +2614,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2642,7 +2681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2712,11 +2751,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2780,7 +2819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2844,10 +2883,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2911,7 +2950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -2981,7 +3020,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -3051,12 +3090,12 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A33" s="11" t="s">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A33" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
       <c r="D33">
         <f>D31-D32</f>
         <v>-785.66289527932531</v>
@@ -3134,18 +3173,19 @@
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="K34" s="10"/>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -3209,7 +3249,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3273,12 +3313,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3345,7 +3385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3415,20 +3455,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3492,15 +3532,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3570,13 +3610,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
@@ -3640,7 +3680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
@@ -3704,11 +3744,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -3772,7 +3812,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -3836,10 +3876,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
@@ -3903,7 +3943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A57" s="5" t="s">
         <v>22</v>
       </c>
@@ -3973,19 +4013,19 @@
         <v>358.72983861659498</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.4">
       <c r="K58">
         <f>K57+L57+M57-K5</f>
         <v>5401.088917483823</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -4049,7 +4089,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -4114,7 +4154,7 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A62" s="3" t="s">
         <v>22</v>
       </c>
@@ -4184,7 +4224,7 @@
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -4254,12 +4294,12 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A64" s="11" t="s">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A64" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B64" s="11"/>
-      <c r="C64" s="11"/>
+      <c r="B64" s="14"/>
+      <c r="C64" s="14"/>
       <c r="D64" s="10">
         <f>D63-D62</f>
         <v>486.66028698880109</v>
@@ -4337,27 +4377,27 @@
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
       <c r="D66" s="10"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A67" s="11" t="s">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A67" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="B67" s="11"/>
-      <c r="C67" s="9"/>
+      <c r="B67" s="14"/>
+      <c r="C67" s="14"/>
       <c r="D67" s="10"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A68" s="5" t="s">
         <v>22</v>
       </c>
@@ -4427,11 +4467,11 @@
         <v>350.36946039055402</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A69" s="11" t="s">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A69" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="B69" s="11"/>
+      <c r="B69" s="14"/>
       <c r="C69" s="9"/>
       <c r="D69" s="10">
         <f>D68-D62</f>
@@ -4486,7 +4526,7 @@
         <v>133.12347700700047</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -4507,13 +4547,13 @@
       <c r="O70" s="10"/>
       <c r="P70" s="10"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A71" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -4525,7 +4565,7 @@
       </c>
       <c r="G72" s="4"/>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
         <v>22</v>
       </c>
@@ -4589,13 +4629,13 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="G74" s="4"/>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A75" s="3" t="s">
         <v>20</v>
       </c>
@@ -4607,7 +4647,7 @@
       </c>
       <c r="G75" s="4"/>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -4676,7 +4716,7 @@
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="D77">
@@ -4756,12 +4796,12 @@
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A78" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A79" s="3" t="s">
         <v>20</v>
       </c>
@@ -4825,7 +4865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A80" s="3" t="s">
         <v>22</v>
       </c>
@@ -4889,10 +4929,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>20</v>
       </c>
@@ -4950,7 +4990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A83" s="2" t="s">
         <v>22</v>
       </c>
@@ -5014,7 +5054,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>20</v>
       </c>
@@ -5072,7 +5112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
         <v>22</v>
       </c>
@@ -5142,7 +5182,7 @@
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.4">
       <c r="D87">
         <f>D86-D80</f>
         <v>-4018.7603482047853</v>
@@ -5192,13 +5232,13 @@
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A88" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G88" s="4"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -5262,7 +5302,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -5306,8 +5346,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.4"/>
+    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A92" s="1" t="s">
         <v>26</v>
       </c>
@@ -5328,7 +5368,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
         <v>0</v>
       </c>
@@ -5390,7 +5430,7 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A94" s="2" t="s">
         <v>20</v>
       </c>
@@ -5401,7 +5441,8 @@
         <v>4</v>
       </c>
       <c r="D94">
-        <v>29525.427309999999</v>
+        <f>J94+K94+L94+M94+N94</f>
+        <v>34658.998111500005</v>
       </c>
       <c r="E94">
         <v>80391.755990000005</v>
@@ -5437,7 +5478,8 @@
         <v>0</v>
       </c>
       <c r="P94">
-        <v>64865.028310000002</v>
+        <f t="shared" ref="P94" si="22">D94+$P$1</f>
+        <v>155218.66993049652</v>
       </c>
       <c r="Q94">
         <v>1191.7509680000001</v>
@@ -5452,467 +5494,723 @@
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A95" s="7" t="s">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A96" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="97" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A97" t="s">
+        <v>22</v>
+      </c>
+      <c r="B97" t="s">
+        <v>23</v>
+      </c>
+      <c r="C97">
+        <v>0</v>
+      </c>
+      <c r="D97">
+        <f>J97+K97+L97+M97+N97</f>
+        <v>144641.57326653044</v>
+      </c>
+      <c r="E97">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F97">
+        <v>0.85636894399557495</v>
+      </c>
+      <c r="G97">
+        <v>20627.43117349</v>
+      </c>
+      <c r="H97">
+        <v>4930.8542128783001</v>
+      </c>
+      <c r="I97">
+        <v>9095.1262763121395</v>
+      </c>
+      <c r="J97">
+        <v>34653.411662680403</v>
+      </c>
+      <c r="K97">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L97">
+        <f>L4*(1.08/0.43)</f>
+        <v>38437.447108478234</v>
+      </c>
+      <c r="M97">
+        <v>19297.5304894482</v>
+      </c>
+      <c r="N97">
+        <v>1410</v>
+      </c>
+      <c r="O97">
+        <v>0</v>
+      </c>
+      <c r="P97">
+        <f t="shared" ref="P97" si="23">D97+$P$1</f>
+        <v>265201.24508552696</v>
+      </c>
+    </row>
+    <row r="98" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A98" t="s">
+        <v>22</v>
+      </c>
+      <c r="B98" t="s">
+        <v>21</v>
+      </c>
+      <c r="C98">
+        <v>4</v>
+      </c>
+      <c r="D98">
+        <f>J98+K98+L98+M98+N98</f>
+        <v>141686.61445013408</v>
+      </c>
+      <c r="E98">
+        <v>282179.70347192901</v>
+      </c>
+      <c r="F98">
+        <v>0.92782505226740197</v>
+      </c>
+      <c r="G98">
+        <v>19831.065688191899</v>
+      </c>
+      <c r="H98">
+        <v>6230.6791730567802</v>
+      </c>
+      <c r="I98">
+        <v>4871.4166947967997</v>
+      </c>
+      <c r="J98">
+        <v>30933.161556045401</v>
+      </c>
+      <c r="K98">
+        <v>50937.4505788346</v>
+      </c>
+      <c r="L98">
+        <v>39073.7116581429</v>
+      </c>
+      <c r="M98">
+        <v>19317.091802737999</v>
+      </c>
+      <c r="N98">
+        <v>1425.19885437316</v>
+      </c>
+      <c r="O98">
+        <v>0</v>
+      </c>
+      <c r="P98">
+        <f t="shared" ref="P98" si="24">D98+$P$1</f>
+        <v>262246.28626913059</v>
+      </c>
+      <c r="Q98">
+        <v>1392.0880151674601</v>
+      </c>
+      <c r="R98">
+        <v>14195.8581733913</v>
+      </c>
+      <c r="S98">
+        <v>112.66554105866101</v>
+      </c>
+      <c r="T98">
+        <v>-1.52076853589591</v>
+      </c>
+      <c r="U98">
+        <v>12183.2216733653</v>
+      </c>
+      <c r="V98">
+        <v>290.07670650869801</v>
+      </c>
+    </row>
+    <row r="99" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="K99">
+        <f>SUM(K97:M97)-SUM(K98:M98)</f>
+        <v>-750.09243586547382</v>
+      </c>
+    </row>
+    <row r="100" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A100" t="s">
+        <v>22</v>
+      </c>
+      <c r="B100" t="s">
+        <v>23</v>
+      </c>
+      <c r="C100">
+        <v>0</v>
+      </c>
+      <c r="D100">
+        <f>J100+K100+L100+M100+N100</f>
+        <v>182723.11808696718</v>
+      </c>
+      <c r="E100">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F100">
+        <v>0.85636894399557495</v>
+      </c>
+      <c r="G100">
+        <v>20627.43117349</v>
+      </c>
+      <c r="H100">
+        <v>4930.8542128783001</v>
+      </c>
+      <c r="I100">
+        <v>9095.1262763121395</v>
+      </c>
+      <c r="J100">
+        <v>34653.411662680403</v>
+      </c>
+      <c r="K100">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L100">
+        <f>L4*(2.15/0.43)</f>
+        <v>76518.991928914998</v>
+      </c>
+      <c r="M100">
+        <v>19297.5304894482</v>
+      </c>
+      <c r="N100">
+        <v>1410</v>
+      </c>
+    </row>
+    <row r="101" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A101" t="s">
+        <v>22</v>
+      </c>
+      <c r="B101" t="s">
+        <v>21</v>
+      </c>
+      <c r="C101">
+        <v>4</v>
+      </c>
+      <c r="D101" s="13">
+        <f>J101+K101+L101+M101+N101</f>
+        <v>180164.72653261331</v>
+      </c>
+      <c r="E101" s="13">
+        <v>282179.67123285698</v>
+      </c>
+      <c r="F101" s="12">
+        <v>1.0641670739695701</v>
+      </c>
+      <c r="G101" s="13">
+        <v>19863.1783561796</v>
+      </c>
+      <c r="H101" s="13">
+        <v>6506.5697069746102</v>
+      </c>
+      <c r="I101" s="13">
+        <v>4873.61028676154</v>
+      </c>
+      <c r="J101" s="13">
+        <v>31243.358349915699</v>
+      </c>
+      <c r="K101" s="13">
+        <v>50899.9452054371</v>
+      </c>
+      <c r="L101" s="13">
+        <v>77281.720548983998</v>
+      </c>
+      <c r="M101" s="13">
+        <v>19309.308438346699</v>
+      </c>
+      <c r="N101" s="13">
+        <v>1430.39398992981</v>
+      </c>
+      <c r="O101">
+        <v>0</v>
+      </c>
+      <c r="P101">
+        <f t="shared" ref="P101" si="25">D101+$P$1</f>
+        <v>300724.39835160982</v>
+      </c>
+      <c r="Q101" s="4">
+        <v>1453.7288077599201</v>
+      </c>
+      <c r="R101">
+        <v>14136.371585592</v>
+      </c>
+      <c r="S101" s="4">
+        <v>107.91123347780101</v>
+      </c>
+      <c r="T101" s="12">
+        <v>-4.2490908058638102</v>
+      </c>
+      <c r="U101">
+        <v>13013.5923280234</v>
+      </c>
+      <c r="V101" s="4">
+        <v>351.71871156820202</v>
+      </c>
+    </row>
+    <row r="102" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="K102" s="13">
+        <f>SUM(K100:M100)-SUM(K101:M101)</f>
+        <v>-831.26776848098962</v>
+      </c>
+    </row>
+    <row r="106" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A106" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
+    <row r="108" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A108" t="s">
         <v>32</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B108" t="s">
         <v>33</v>
       </c>
-      <c r="C97" t="s">
+      <c r="C108" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A98">
+    <row r="109" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A109">
         <v>20</v>
       </c>
-      <c r="B98">
+      <c r="B109">
         <v>60</v>
       </c>
-      <c r="C98">
+      <c r="C109">
         <v>2</v>
       </c>
-      <c r="D98">
-        <f t="shared" ref="D98:D104" si="22">J98+K98+L98+M98+N98</f>
+      <c r="D109">
+        <f t="shared" ref="D109:D115" si="26">J109+K109+L109+M109+N109</f>
         <v>120712.69088313227</v>
       </c>
-      <c r="E98">
+      <c r="E109">
         <v>282179.67123285501</v>
       </c>
-      <c r="F98">
+      <c r="F109">
         <v>0.854946898908852</v>
       </c>
-      <c r="G98">
+      <c r="G109">
         <v>18681.222424938602</v>
       </c>
-      <c r="H98">
+      <c r="H109">
         <v>5354.6114985546601</v>
       </c>
-      <c r="I98">
+      <c r="I109">
         <v>8156.08309050551</v>
       </c>
-      <c r="J98">
+      <c r="J109">
         <v>32191.917013998798</v>
       </c>
-      <c r="K98">
+      <c r="K109">
         <v>51372.124296964801</v>
       </c>
-      <c r="L98">
+      <c r="L109">
         <v>16725.325417965501</v>
       </c>
-      <c r="M98">
+      <c r="M109">
         <v>19407.285599838699</v>
       </c>
-      <c r="N98">
+      <c r="N109">
         <v>1016.03855436447</v>
       </c>
-      <c r="O98">
-        <v>0</v>
-      </c>
-      <c r="P98">
-        <f t="shared" ref="P98:P104" si="23">D98+$P$1</f>
+      <c r="O109">
+        <v>0</v>
+      </c>
+      <c r="P109">
+        <f t="shared" ref="P109:P115" si="27">D109+$P$1</f>
         <v>241272.36270212877</v>
       </c>
-      <c r="Q98">
+      <c r="Q109">
         <v>1192.7637589594799</v>
       </c>
-      <c r="R98">
+      <c r="R109">
         <v>19736.206339365101</v>
       </c>
-      <c r="S98">
+      <c r="S109">
         <v>481.37088632597801</v>
       </c>
-      <c r="T98" s="6">
+      <c r="T109" s="6">
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A99">
+    <row r="110" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A110">
         <v>20</v>
       </c>
-      <c r="B99">
+      <c r="B110">
         <v>50</v>
       </c>
-      <c r="C99">
+      <c r="C110">
         <v>2</v>
       </c>
-      <c r="D99">
-        <f t="shared" si="22"/>
+      <c r="D110">
+        <f t="shared" si="26"/>
         <v>119392.42354269064</v>
       </c>
-      <c r="E99">
+      <c r="E110">
         <v>282254.81855225202</v>
       </c>
-      <c r="F99">
+      <c r="F110">
         <v>0.85006146065890897</v>
       </c>
-      <c r="G99">
+      <c r="G110">
         <v>19407.840072768398</v>
       </c>
-      <c r="H99">
+      <c r="H110">
         <v>5891.8301217549197</v>
       </c>
-      <c r="I99">
+      <c r="I110">
         <v>6659.4942697455399</v>
       </c>
-      <c r="J99">
+      <c r="J110">
         <v>31959.164464268899</v>
       </c>
-      <c r="K99">
+      <c r="K110">
         <v>51102.045942938203</v>
       </c>
-      <c r="L99">
+      <c r="L110">
         <v>15967.176494174801</v>
       </c>
-      <c r="M99">
+      <c r="M110">
         <v>19353.573908279199</v>
       </c>
-      <c r="N99">
+      <c r="N110">
         <v>1010.46273302954</v>
       </c>
-      <c r="O99">
-        <v>0</v>
-      </c>
-      <c r="P99">
-        <f t="shared" si="23"/>
+      <c r="O110">
+        <v>0</v>
+      </c>
+      <c r="P110">
+        <f t="shared" si="27"/>
         <v>239952.09536168716</v>
       </c>
-      <c r="Q99">
+      <c r="Q110">
         <v>1312.43161993582</v>
       </c>
-      <c r="R99">
+      <c r="R110">
         <v>18377.616631847999</v>
       </c>
-      <c r="S99">
+      <c r="S110">
         <v>459.4404157962</v>
       </c>
-      <c r="T99" s="6">
+      <c r="T110" s="6">
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A100">
+    <row r="111" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A111">
         <v>20</v>
       </c>
-      <c r="B100">
+      <c r="B111">
         <v>40</v>
       </c>
-      <c r="C100">
+      <c r="C111">
         <v>2</v>
       </c>
-      <c r="D100">
-        <f t="shared" si="22"/>
+      <c r="D111">
+        <f t="shared" si="26"/>
         <v>117777.02945340994</v>
       </c>
-      <c r="E100">
+      <c r="E111">
         <v>282179.67123287299</v>
       </c>
-      <c r="F100">
+      <c r="F111">
         <v>0.84456314023622803</v>
       </c>
-      <c r="G100">
+      <c r="G111">
         <v>19298.245593088301</v>
       </c>
-      <c r="H100">
+      <c r="H111">
         <v>5682.0016560700296</v>
       </c>
-      <c r="I100">
+      <c r="I111">
         <v>5350.3346939491703</v>
       </c>
-      <c r="J100">
+      <c r="J111">
         <v>30330.5819431075</v>
       </c>
-      <c r="K100">
+      <c r="K111">
         <v>51097.733915068202</v>
       </c>
-      <c r="L100">
+      <c r="L111">
         <v>15987.901266609</v>
       </c>
-      <c r="M100">
+      <c r="M111">
         <v>19350.349595595701</v>
       </c>
-      <c r="N100">
+      <c r="N111">
         <v>1010.46273302954</v>
       </c>
-      <c r="O100">
-        <v>0</v>
-      </c>
-      <c r="P100">
-        <f t="shared" si="23"/>
+      <c r="O111">
+        <v>0</v>
+      </c>
+      <c r="P111">
+        <f t="shared" si="27"/>
         <v>238336.70127240644</v>
       </c>
-      <c r="Q100">
+      <c r="Q111">
         <v>1265.6913868611</v>
       </c>
-      <c r="R100">
+      <c r="R111">
         <v>17746.163883660702</v>
       </c>
-      <c r="S100">
+      <c r="S111">
         <v>507.03325381887902</v>
       </c>
-      <c r="T100" s="6">
+      <c r="T111" s="6">
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A101">
+    <row r="112" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A112">
         <v>20</v>
       </c>
-      <c r="B101">
+      <c r="B112">
         <v>30</v>
       </c>
-      <c r="C101">
+      <c r="C112">
         <v>2</v>
       </c>
-      <c r="D101">
-        <f t="shared" si="22"/>
+      <c r="D112">
+        <f t="shared" si="26"/>
         <v>116625.1695160947</v>
       </c>
-      <c r="E101">
+      <c r="E112">
         <v>282182.50548365602</v>
       </c>
-      <c r="F101">
+      <c r="F112">
         <v>0.84045954058697003</v>
       </c>
-      <c r="G101">
+      <c r="G112">
         <v>19302.752565837702</v>
       </c>
-      <c r="H101">
+      <c r="H112">
         <v>6226.5181629292701</v>
       </c>
-      <c r="I101">
+      <c r="I112">
         <v>3974.5318253822402</v>
       </c>
-      <c r="J101">
+      <c r="J112">
         <v>29503.802554149199</v>
       </c>
-      <c r="K101">
+      <c r="K112">
         <v>51013.610661725899</v>
       </c>
-      <c r="L101">
+      <c r="L112">
         <v>15760.601295416</v>
       </c>
-      <c r="M101">
+      <c r="M112">
         <v>19332.981882301501</v>
       </c>
-      <c r="N101">
+      <c r="N112">
         <v>1014.17312250211</v>
       </c>
-      <c r="O101">
-        <v>0</v>
-      </c>
-      <c r="P101">
-        <f t="shared" si="23"/>
+      <c r="O112">
+        <v>0</v>
+      </c>
+      <c r="P112">
+        <f t="shared" si="27"/>
         <v>237184.84133509122</v>
       </c>
-      <c r="Q101">
+      <c r="Q112">
         <v>1386.9848841974899</v>
       </c>
-      <c r="R101">
+      <c r="R112">
         <v>18436.445202769701</v>
       </c>
-      <c r="S101">
+      <c r="S112">
         <v>209.50505912238299</v>
       </c>
-      <c r="T101" s="6">
+      <c r="T112" s="6">
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A102" s="3">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A113" s="3">
         <v>20</v>
       </c>
-      <c r="B102" s="3">
+      <c r="B113" s="3">
         <v>20</v>
       </c>
-      <c r="C102" s="3">
+      <c r="C113" s="3">
         <v>2</v>
       </c>
-      <c r="D102">
-        <f t="shared" si="22"/>
+      <c r="D113">
+        <f t="shared" si="26"/>
         <v>115198.459983006</v>
       </c>
-      <c r="E102">
+      <c r="E113">
         <v>282179.67123297497</v>
       </c>
-      <c r="F102">
+      <c r="F113">
         <v>0.83541194997266699</v>
       </c>
-      <c r="G102">
+      <c r="G113">
         <v>19351.2255529412</v>
       </c>
-      <c r="H102">
+      <c r="H113">
         <v>6002.0469674603501</v>
       </c>
-      <c r="I102">
+      <c r="I113">
         <v>2645.4376652921501</v>
       </c>
-      <c r="J102">
+      <c r="J113">
         <v>27998.710185693701</v>
       </c>
-      <c r="K102">
+      <c r="K113">
         <v>51033.4442867088</v>
       </c>
-      <c r="L102">
+      <c r="L113">
         <v>15815.1228903871</v>
       </c>
-      <c r="M102">
+      <c r="M113">
         <v>19337.009497714302</v>
       </c>
-      <c r="N102">
+      <c r="N113">
         <v>1014.17312250211</v>
       </c>
-      <c r="O102">
-        <v>0</v>
-      </c>
-      <c r="P102">
-        <f t="shared" si="23"/>
+      <c r="O113">
+        <v>0</v>
+      </c>
+      <c r="P113">
+        <f t="shared" si="27"/>
         <v>235758.13180200252</v>
       </c>
-      <c r="Q102">
+      <c r="Q113">
         <v>1336.98290493166</v>
       </c>
-      <c r="R102">
+      <c r="R113">
         <v>18577.307877855899</v>
       </c>
-      <c r="S102">
+      <c r="S113">
         <v>432.030415764091</v>
       </c>
-      <c r="T102" s="6">
+      <c r="T113" s="6">
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A103">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A114">
         <v>20</v>
       </c>
-      <c r="B103">
+      <c r="B114">
         <v>15</v>
       </c>
-      <c r="C103">
+      <c r="C114">
         <v>2</v>
       </c>
-      <c r="D103">
-        <f t="shared" si="22"/>
+      <c r="D114">
+        <f t="shared" si="26"/>
         <v>114451.25872361983</v>
       </c>
-      <c r="E103">
+      <c r="E114">
         <v>282179.67123267101</v>
       </c>
-      <c r="F103">
+      <c r="F114">
         <v>0.83277713625127903</v>
       </c>
-      <c r="G103">
+      <c r="G114">
         <v>19390.977969205</v>
       </c>
-      <c r="H103">
+      <c r="H114">
         <v>5599.5405456203798</v>
       </c>
-      <c r="I103">
+      <c r="I114">
         <v>2128.1287863747102</v>
       </c>
-      <c r="J103">
+      <c r="J114">
         <v>27118.647301200101</v>
       </c>
-      <c r="K103">
+      <c r="K114">
         <v>51068.507704320902</v>
       </c>
-      <c r="L103">
+      <c r="L114">
         <v>15909.3558282099</v>
       </c>
-      <c r="M103">
+      <c r="M114">
         <v>19344.285156859401</v>
       </c>
-      <c r="N103">
+      <c r="N114">
         <v>1010.46273302954</v>
       </c>
-      <c r="O103">
-        <v>0</v>
-      </c>
-      <c r="P103">
-        <f t="shared" si="23"/>
+      <c r="O114">
+        <v>0</v>
+      </c>
+      <c r="P114">
+        <f t="shared" si="27"/>
         <v>235010.93054261635</v>
       </c>
-      <c r="Q103">
+      <c r="Q114">
         <v>1247.3228025527501</v>
       </c>
-      <c r="R103">
+      <c r="R114">
         <v>16417.502561416801</v>
       </c>
-      <c r="S103">
+      <c r="S114">
         <v>469.07150175476602</v>
       </c>
-      <c r="T103" s="6">
+      <c r="T114" s="6">
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A104">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A115">
         <v>20</v>
       </c>
-      <c r="B104">
+      <c r="B115">
         <v>12</v>
       </c>
-      <c r="C104">
+      <c r="C115">
         <v>2</v>
       </c>
-      <c r="D104">
-        <f t="shared" si="22"/>
+      <c r="D115">
+        <f t="shared" si="26"/>
         <v>114787.7594081375</v>
       </c>
-      <c r="E104">
+      <c r="E115">
         <v>282179.67123287602</v>
       </c>
-      <c r="F104">
+      <c r="F115">
         <v>0.83403396920434802</v>
       </c>
-      <c r="G104">
+      <c r="G115">
         <v>20436.472361711199</v>
       </c>
-      <c r="H104">
+      <c r="H115">
         <v>4946.5396722567002</v>
       </c>
-      <c r="I104">
+      <c r="I115">
         <v>2967.9237851293901</v>
       </c>
-      <c r="J104">
+      <c r="J115">
         <v>28350.9358190973</v>
       </c>
-      <c r="K104">
+      <c r="K115">
         <v>50843.184005923598</v>
       </c>
-      <c r="L104">
+      <c r="L115">
         <v>15303.798385783</v>
       </c>
-      <c r="M104">
+      <c r="M115">
         <v>19297.530489448302</v>
       </c>
-      <c r="N104">
+      <c r="N115">
         <v>992.31070788530405</v>
       </c>
-      <c r="O104">
-        <v>0</v>
-      </c>
-      <c r="P104">
-        <f t="shared" si="23"/>
+      <c r="O115">
+        <v>0</v>
+      </c>
+      <c r="P115">
+        <f t="shared" si="27"/>
         <v>235347.43122713402</v>
       </c>
-      <c r="Q104">
+      <c r="Q115">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R104">
+      <c r="R115">
         <v>13.380488321454299</v>
       </c>
-      <c r="S104">
+      <c r="S115">
         <v>2.67609766429086</v>
       </c>
-      <c r="T104" s="6">
+      <c r="T115" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>
@@ -5920,8 +6218,8 @@
   <mergeCells count="4">
     <mergeCell ref="A64:C64"/>
     <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A67:B67"/>
     <mergeCell ref="A69:B69"/>
+    <mergeCell ref="A67:C67"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5932,20 +6230,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA993591-8C1F-4C7B-A75D-E9726DFB461B}">
   <dimension ref="A2:P31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="12.81640625" customWidth="1"/>
-    <col min="3" max="3" width="11.36328125" customWidth="1"/>
-    <col min="4" max="4" width="15.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.84375" customWidth="1"/>
+    <col min="3" max="3" width="11.3828125" customWidth="1"/>
+    <col min="4" max="4" width="15.53515625" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17.08984375" customWidth="1"/>
-    <col min="7" max="7" width="15.26953125" customWidth="1"/>
-    <col min="8" max="8" width="13.26953125" customWidth="1"/>
-    <col min="9" max="11" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.07421875" customWidth="1"/>
+    <col min="7" max="7" width="15.23046875" customWidth="1"/>
+    <col min="8" max="8" width="13.23046875" customWidth="1"/>
+    <col min="9" max="11" width="11.3828125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5984,12 +6282,12 @@
       </c>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -6028,7 +6326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="D5" s="10"/>
@@ -6040,7 +6338,7 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>48</v>
       </c>
@@ -6053,11 +6351,11 @@
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>
       <c r="K6" s="10"/>
-      <c r="M6" s="12" t="s">
+      <c r="M6" s="11" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -6095,9 +6393,9 @@
       <c r="L7">
         <v>0</v>
       </c>
-      <c r="M7" s="12"/>
-    </row>
-    <row r="8" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="M7" s="11"/>
+    </row>
+    <row r="8" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -6106,9 +6404,9 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
       <c r="K8" s="10"/>
-      <c r="M8" s="12"/>
-    </row>
-    <row r="9" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="M8" s="11"/>
+    </row>
+    <row r="9" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -6120,51 +6418,62 @@
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
       <c r="K9" s="10"/>
-      <c r="M9" s="12"/>
-    </row>
-    <row r="10" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D10" s="10">
-        <f>H10+I10+J10+K10</f>
-        <v>116423.6512611575</v>
+      <c r="M9" s="11"/>
+    </row>
+    <row r="10" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10">
+        <v>4</v>
+      </c>
+      <c r="D10">
+        <v>114153.095713535</v>
       </c>
       <c r="E10">
-        <v>19793.405782867099</v>
+        <v>19390.3410434773</v>
       </c>
       <c r="F10">
-        <v>5278.7073577880201</v>
-      </c>
-      <c r="G10">
-        <v>4906.1393788565601</v>
+        <v>6212.6008869098296</v>
+      </c>
+      <c r="G10" s="8">
+        <v>1.21975885109732E-5</v>
       </c>
       <c r="H10">
-        <v>29978.252519511701</v>
+        <v>25602.941942584701</v>
       </c>
       <c r="I10">
-        <v>51100.150850479702</v>
+        <v>50959.945205482203</v>
       </c>
       <c r="J10">
-        <v>15994.396781481701</v>
+        <v>17946.760793761499</v>
       </c>
       <c r="K10">
-        <v>19350.851109684401</v>
+        <v>19643.4477717072</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
-      <c r="M10" s="12"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="D11" s="10"/>
+      <c r="M10" s="11"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="D11">
+        <f>(34653-H10-I11+wrd_pricetater_flex_type_summar!K5+L10)/34653</f>
+        <v>0.17154119896168271</v>
+      </c>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
       <c r="G11" s="10"/>
       <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
+      <c r="I11" s="10">
+        <f>SUM(I10:K10)</f>
+        <v>88550.153770950899</v>
+      </c>
       <c r="J11" s="10"/>
       <c r="K11" s="10"/>
-      <c r="M11" s="12"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="M11" s="11"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
@@ -6176,9 +6485,9 @@
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
       <c r="K12" s="10"/>
-      <c r="M12" s="12"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="M12" s="11"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
@@ -6216,9 +6525,9 @@
       <c r="L13">
         <v>11020</v>
       </c>
-      <c r="M13" s="12"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="M13" s="11"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="D14" s="10"/>
@@ -6229,9 +6538,9 @@
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
       <c r="K14" s="10"/>
-      <c r="M14" s="12"/>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="M14" s="11"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>46</v>
       </c>
@@ -6244,7 +6553,7 @@
       <c r="J15" s="10"/>
       <c r="K15" s="10"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -6283,7 +6592,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
       <c r="D17">
         <f>(34653-H16-I17+wrd_pricetater_flex_type_summar!K5+L16)/34653</f>
         <v>0.38932217950875497</v>
@@ -6293,7 +6602,7 @@
         <v>87792.098602195503</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
         <v>57</v>
       </c>
@@ -6332,7 +6641,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -6340,7 +6649,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -6378,7 +6687,7 @@
       </c>
       <c r="L23" s="10"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>55</v>
       </c>
@@ -6416,7 +6725,7 @@
       </c>
       <c r="L25" s="10"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -6453,7 +6762,7 @@
         <v>-476.58002357000078</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -6490,7 +6799,7 @@
         <v>174.37684745549996</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
Adding filename standardization for the results with different start up times
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D1FE8ED-83C4-44C2-B5FD-1D5D4D3EABAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A83C26BD-4FFD-40F8-BDDF-9112B52BF739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -244,7 +244,7 @@
     The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</t>
       </text>
     </comment>
-    <comment ref="A98" authorId="22" shapeId="0" xr:uid="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
+    <comment ref="A101" authorId="22" shapeId="0" xr:uid="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -252,7 +252,7 @@
     2.5x higher brine costs (1.08$/m3)</t>
       </text>
     </comment>
-    <comment ref="A101" authorId="23" shapeId="0" xr:uid="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
+    <comment ref="A104" authorId="23" shapeId="0" xr:uid="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -260,7 +260,7 @@
     5x brine costs (2.15 $/m3)</t>
       </text>
     </comment>
-    <comment ref="T112" authorId="24" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="T115" authorId="24" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -405,7 +405,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="65">
   <si>
     <t>Season</t>
   </si>
@@ -597,6 +597,9 @@
   </si>
   <si>
     <t>Higher Brine Costs</t>
+  </si>
+  <si>
+    <t>?</t>
   </si>
 </sst>
 </file>
@@ -1587,13 +1590,13 @@
   <threadedComment ref="A89" dT="2026-07-10T12:48:01.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9FF6B967-6104-43AC-8EED-15C48C9ACCA9}">
     <text>The flexibility metrics are all nonsense. Would have to run a baseline case for this to work.</text>
   </threadedComment>
-  <threadedComment ref="A98" dT="2026-08-09T17:04:16.49" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
+  <threadedComment ref="A101" dT="2026-08-09T17:04:16.49" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{3B63C6BF-9DE1-4172-A721-F97EE0406603}">
     <text>2.5x higher brine costs (1.08$/m3)</text>
   </threadedComment>
-  <threadedComment ref="A101" dT="2026-08-09T17:05:17.32" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
+  <threadedComment ref="A104" dT="2026-08-09T17:05:17.32" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
     <text>5x brine costs (2.15 $/m3)</text>
   </threadedComment>
-  <threadedComment ref="T112" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="T115" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1659,22 +1662,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:V115"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:V118"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.61328125" customWidth="1"/>
-    <col min="3" max="3" width="11.4609375" customWidth="1"/>
-    <col min="5" max="5" width="10.23046875" customWidth="1"/>
-    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.69140625" customWidth="1"/>
-    <col min="9" max="9" width="9.07421875" customWidth="1"/>
-    <col min="11" max="11" width="10.84375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.53515625" customWidth="1"/>
-    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.84375" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.54296875" customWidth="1"/>
+    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1685,7 +1688,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1753,7 +1756,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1817,7 +1820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1881,14 +1884,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G5" s="4"/>
       <c r="K5" s="10">
         <f>K4+L4+M4</f>
         <v>85444.512881154791</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1952,7 +1955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -2016,10 +2019,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2083,7 +2086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2147,10 +2150,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -2214,7 +2217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2278,10 +2281,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2343,7 +2346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2399,10 +2402,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2466,7 +2469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2530,7 +2533,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2539,7 +2542,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2550,7 +2553,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2614,10 +2617,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2681,7 +2684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2751,11 +2754,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2819,7 +2822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2883,10 +2886,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2950,7 +2953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -3020,7 +3023,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -3090,7 +3093,7 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A33" s="14" t="s">
         <v>45</v>
       </c>
@@ -3173,19 +3176,19 @@
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="K34" s="10"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -3249,7 +3252,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3313,12 +3316,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3385,7 +3388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3455,20 +3458,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3532,15 +3535,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3610,13 +3613,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
@@ -3680,7 +3683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
@@ -3744,11 +3747,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -3812,7 +3815,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -3876,10 +3879,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
@@ -3943,7 +3946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>22</v>
       </c>
@@ -4013,19 +4016,19 @@
         <v>358.72983861659498</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
       <c r="K58">
         <f>K57+L57+M57-K5</f>
         <v>5401.088917483823</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -4089,7 +4092,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -4154,77 +4157,75 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A62" s="3" t="s">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A62" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B62" s="3" t="s">
+      <c r="B62" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C62">
         <v>4</v>
       </c>
       <c r="D62" s="10">
-        <f>J62+K62+L62+M62+N62-O62</f>
-        <v>107555.29824632255</v>
+        <v>114153.095713535</v>
       </c>
       <c r="E62">
-        <v>282179.67123287602</v>
+        <v>282179.67123343103</v>
       </c>
       <c r="F62">
-        <v>0.80673743017586796</v>
+        <v>0.83530141349350295</v>
       </c>
       <c r="G62">
-        <v>19617.269555424798</v>
+        <v>19390.3410434773</v>
       </c>
       <c r="H62">
-        <v>6177.79087142139</v>
+        <v>6212.6008869098296</v>
       </c>
       <c r="I62" s="8">
-        <v>1.4897343661976701E-5</v>
+        <v>1.21975885109732E-5</v>
       </c>
       <c r="J62">
-        <v>25795.060441743601</v>
+        <v>25602.941942584701</v>
       </c>
       <c r="K62">
-        <v>50989.945229661498</v>
+        <v>50959.945205482203</v>
       </c>
       <c r="L62">
-        <v>20356.552509954701</v>
+        <v>17946.760793761499</v>
       </c>
       <c r="M62">
-        <v>19971.3621100407</v>
+        <v>19643.4477717072</v>
       </c>
       <c r="N62">
-        <v>1462.3779549220301</v>
+        <v>1459.6580951174601</v>
       </c>
       <c r="O62">
-        <v>11020</v>
+        <v>0</v>
       </c>
       <c r="P62">
-        <f t="shared" si="12"/>
-        <v>228114.97006531907</v>
+        <v>235705.078240417</v>
       </c>
       <c r="Q62">
-        <v>1380.27146414547</v>
+        <v>1388.04888293766</v>
       </c>
       <c r="R62">
-        <v>33980.634383525299</v>
+        <v>32406.8779181912</v>
       </c>
       <c r="S62">
-        <v>943.906510653483</v>
+        <v>611.45052675832505</v>
       </c>
       <c r="T62">
-        <v>0.36911323114551098</v>
+        <v>0.13840414379532001</v>
       </c>
       <c r="U62">
-        <v>36719.7300995962</v>
+        <v>32883.087260137101</v>
       </c>
       <c r="V62">
-        <v>278.17977348178903</v>
-      </c>
-    </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
+        <v>285.93988921858301</v>
+      </c>
+    </row>
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -4294,7 +4295,7 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A64" s="14" t="s">
         <v>44</v>
       </c>
@@ -4302,94 +4303,94 @@
       <c r="C64" s="14"/>
       <c r="D64" s="10">
         <f>D63-D62</f>
-        <v>486.66028698880109</v>
+        <v>-6111.1371802236536</v>
       </c>
       <c r="E64">
         <f t="shared" ref="E64:V64" si="13">E63-E62</f>
-        <v>-1.0599615052342415E-7</v>
+        <v>-6.6100619733333588E-7</v>
       </c>
       <c r="F64">
         <f t="shared" si="13"/>
-        <v>1.8194475210779881E-3</v>
+        <v>-2.6744535796557001E-2</v>
       </c>
       <c r="G64">
         <f t="shared" si="13"/>
-        <v>-214.21539764659974</v>
+        <v>12.713114300899178</v>
       </c>
       <c r="H64">
         <f t="shared" si="13"/>
-        <v>-624.4983606493397</v>
+        <v>-659.30837613777931</v>
       </c>
       <c r="I64">
         <f t="shared" si="13"/>
-        <v>4877.8861089948059</v>
+        <v>4877.8861116945618</v>
       </c>
       <c r="J64">
         <f t="shared" si="13"/>
-        <v>4039.1723506987983</v>
+        <v>4231.290849857698</v>
       </c>
       <c r="K64">
         <f t="shared" si="13"/>
-        <v>183.72486634590314</v>
+        <v>213.72489052519813</v>
       </c>
       <c r="L64">
         <f t="shared" si="13"/>
-        <v>-3232.9060902373021</v>
+        <v>-823.11437404410026</v>
       </c>
       <c r="M64">
         <f t="shared" si="13"/>
-        <v>-476.58002357000078</v>
+        <v>-148.6656852365013</v>
       </c>
       <c r="N64">
         <f t="shared" si="13"/>
-        <v>-26.750816248570118</v>
+        <v>-24.03095644400014</v>
       </c>
       <c r="O64">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>11020</v>
       </c>
       <c r="P64">
         <f t="shared" si="13"/>
-        <v>486.66028698880109</v>
+        <v>-7103.4478881091345</v>
       </c>
       <c r="Q64">
         <f t="shared" si="13"/>
-        <v>-139.52840101139986</v>
+        <v>-147.30581980358988</v>
       </c>
       <c r="R64">
         <f t="shared" si="13"/>
-        <v>-16066.151948654198</v>
+        <v>-14492.395483320099</v>
       </c>
       <c r="S64">
         <f t="shared" si="13"/>
-        <v>-545.80690098968103</v>
+        <v>-213.35091709452303</v>
       </c>
       <c r="T64">
         <f t="shared" si="13"/>
-        <v>0.30386414961436203</v>
+        <v>0.53457323696455306</v>
       </c>
       <c r="U64">
         <f t="shared" si="13"/>
-        <v>-23556.497919273097</v>
+        <v>-19719.855079813999</v>
       </c>
       <c r="V64">
         <f t="shared" si="13"/>
-        <v>-171.16162567428404</v>
-      </c>
-    </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
+        <v>-178.92174141107802</v>
+      </c>
+    </row>
+    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
       <c r="D66" s="10"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A67" s="14" t="s">
         <v>60</v>
       </c>
@@ -4397,7 +4398,7 @@
       <c r="C67" s="14"/>
       <c r="D67" s="10"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
         <v>22</v>
       </c>
@@ -4467,7 +4468,7 @@
         <v>350.36946039055402</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A69" s="14" t="s">
         <v>61</v>
       </c>
@@ -4475,58 +4476,58 @@
       <c r="C69" s="9"/>
       <c r="D69" s="10">
         <f>D68-D62</f>
-        <v>133.12347700698592</v>
+        <v>-6464.6739902054687</v>
       </c>
       <c r="E69" s="10">
         <f t="shared" ref="E69:P69" si="15">E68-E62</f>
-        <v>0</v>
+        <v>-5.5501004680991173E-7</v>
       </c>
       <c r="F69" s="10">
         <f t="shared" si="15"/>
-        <v>4.7176848858698772E-4</v>
+        <v>-2.8092214829048001E-2</v>
       </c>
       <c r="G69" s="10">
         <f t="shared" si="15"/>
-        <v>336.18543171020065</v>
+        <v>563.11394365769956</v>
       </c>
       <c r="H69" s="10">
         <f t="shared" si="15"/>
-        <v>322.76314238460964</v>
+        <v>287.95312689617003</v>
       </c>
       <c r="I69" s="10">
         <f t="shared" si="15"/>
-        <v>-8.5546091703980134E-7</v>
+        <v>1.844294233963699E-6</v>
       </c>
       <c r="J69" s="10">
         <f t="shared" si="15"/>
-        <v>658.94857323930046</v>
+        <v>851.06707239820025</v>
       </c>
       <c r="K69" s="10">
         <f t="shared" si="15"/>
-        <v>-135.00002418200165</v>
+        <v>-105.00000000270666</v>
       </c>
       <c r="L69" s="10">
         <f t="shared" si="15"/>
-        <v>-362.81256703230247</v>
+        <v>2046.9791491608994</v>
       </c>
       <c r="M69" s="10">
         <f t="shared" si="15"/>
-        <v>-28.012505017999501</v>
+        <v>299.90183331549997</v>
       </c>
       <c r="N69" s="10">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>2.7198598045699782</v>
       </c>
       <c r="O69" s="10">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>11020</v>
       </c>
       <c r="P69" s="10">
         <f t="shared" si="15"/>
-        <v>133.12347700700047</v>
-      </c>
-    </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
+        <v>-7456.9846980909351</v>
+      </c>
+    </row>
+    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -4547,13 +4548,13 @@
       <c r="O70" s="10"/>
       <c r="P70" s="10"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -4565,7 +4566,7 @@
       </c>
       <c r="G72" s="4"/>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>22</v>
       </c>
@@ -4629,13 +4630,13 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="G74" s="4"/>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
         <v>20</v>
       </c>
@@ -4647,7 +4648,7 @@
       </c>
       <c r="G75" s="4"/>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -4716,7 +4717,7 @@
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="D77">
@@ -4796,12 +4797,12 @@
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
         <v>20</v>
       </c>
@@ -4865,7 +4866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
         <v>22</v>
       </c>
@@ -4929,10 +4930,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>20</v>
       </c>
@@ -4990,7 +4991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>22</v>
       </c>
@@ -5054,7 +5055,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>20</v>
       </c>
@@ -5102,7 +5103,7 @@
         <v>0</v>
       </c>
       <c r="P85">
-        <f t="shared" ref="P85:P87" si="19">D85+$P$1</f>
+        <f t="shared" ref="P85:P89" si="19">D85+$P$1</f>
         <v>237266.08760950161</v>
       </c>
       <c r="Q85">
@@ -5112,7 +5113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>22</v>
       </c>
@@ -5182,7 +5183,7 @@
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.35">
       <c r="D87">
         <f>D86-D80</f>
         <v>-4018.7603482047853</v>
@@ -5232,13 +5233,13 @@
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G88" s="4"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -5286,7 +5287,7 @@
         <v>0</v>
       </c>
       <c r="P89">
-        <f t="shared" ref="P89" si="21">D89+$P$1</f>
+        <f t="shared" si="19"/>
         <v>267678.15388715523</v>
       </c>
       <c r="Q89">
@@ -5302,7 +5303,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -5334,20 +5335,20 @@
         <v>50169.7</v>
       </c>
       <c r="K90" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="L90" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="M90" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="N90" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.4"/>
-    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>26</v>
       </c>
@@ -5368,7 +5369,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>0</v>
       </c>
@@ -5430,702 +5431,560 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A94" s="2" t="s">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="G94" s="4"/>
+    </row>
+    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
         <v>20</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B95" t="s">
         <v>21</v>
       </c>
-      <c r="C94">
+      <c r="C95">
         <v>4</v>
       </c>
-      <c r="D94">
-        <f>J94+K94+L94+M94+N94</f>
-        <v>34658.998111500005</v>
-      </c>
-      <c r="E94">
-        <v>80391.755990000005</v>
-      </c>
-      <c r="F94">
-        <v>0.79280104200000001</v>
-      </c>
-      <c r="G94" s="4">
-        <v>5050.6365619999997</v>
-      </c>
-      <c r="H94">
-        <v>4678.3390820000004</v>
-      </c>
-      <c r="I94">
-        <v>2508.6600360000002</v>
-      </c>
-      <c r="J94">
-        <v>12237.635679999999</v>
-      </c>
-      <c r="K94">
-        <v>13920</v>
-      </c>
-      <c r="L94">
-        <v>2841.544922</v>
-      </c>
-      <c r="M94">
-        <v>5380.5444360000001</v>
-      </c>
-      <c r="N94">
-        <v>279.27307350000001</v>
-      </c>
-      <c r="O94">
-        <v>0</v>
-      </c>
-      <c r="P94">
-        <f t="shared" ref="P94" si="22">D94+$P$1</f>
-        <v>155218.66993049652</v>
-      </c>
-      <c r="Q94">
-        <v>1191.7509680000001</v>
-      </c>
-      <c r="R94">
-        <v>7243.7162129999997</v>
-      </c>
-      <c r="S94">
-        <v>452.7322633</v>
-      </c>
-      <c r="T94">
-        <v>5.8154128590000003</v>
-      </c>
-    </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A96" s="1" t="s">
+      <c r="D95">
+        <f>J95+K95+L95+M95+N95</f>
+        <v>121563.11893886774</v>
+      </c>
+      <c r="E95">
+        <v>306531.77686027403</v>
+      </c>
+      <c r="F95">
+        <v>0.78839751879627895</v>
+      </c>
+      <c r="G95">
+        <v>19075.241421310599</v>
+      </c>
+      <c r="H95">
+        <v>6261.96818995999</v>
+      </c>
+      <c r="I95">
+        <v>1707.4548259942601</v>
+      </c>
+      <c r="J95">
+        <v>27044.664437264801</v>
+      </c>
+      <c r="K95">
+        <v>55296.129476701703</v>
+      </c>
+      <c r="L95">
+        <v>16799.683918922601</v>
+      </c>
+      <c r="M95">
+        <v>20976.431949083999</v>
+      </c>
+      <c r="N95">
+        <v>1446.20915689464</v>
+      </c>
+      <c r="O95">
+        <v>0</v>
+      </c>
+      <c r="P95">
+        <f t="shared" ref="P95" si="21">D95+$P$1</f>
+        <v>242122.79075786425</v>
+      </c>
+      <c r="Q95">
+        <v>1421.8975872168901</v>
+      </c>
+      <c r="R95">
+        <v>16926.965777071098</v>
+      </c>
+      <c r="S95">
+        <v>248.92596730986901</v>
+      </c>
+      <c r="T95">
+        <v>-0.61547468554465901</v>
+      </c>
+      <c r="U95">
+        <v>31937.310450388199</v>
+      </c>
+      <c r="V95">
+        <v>319.37310450388202</v>
+      </c>
+    </row>
+    <row r="96" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A96" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B96" t="s">
+        <v>35</v>
+      </c>
+      <c r="C96" t="s">
+        <v>35</v>
+      </c>
+      <c r="D96" t="s">
+        <v>36</v>
+      </c>
+      <c r="E96" t="s">
+        <v>36</v>
+      </c>
+      <c r="F96" t="s">
+        <v>36</v>
+      </c>
+      <c r="G96" s="4"/>
+      <c r="K96" t="s">
+        <v>64</v>
+      </c>
+      <c r="L96" t="s">
+        <v>64</v>
+      </c>
+      <c r="M96" t="s">
+        <v>64</v>
+      </c>
+      <c r="N96" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="97" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A97" s="2"/>
+      <c r="G97" s="4"/>
+    </row>
+    <row r="99" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A99" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A97" t="s">
+    <row r="100" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
         <v>22</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B100" t="s">
         <v>23</v>
       </c>
-      <c r="C97">
-        <v>0</v>
-      </c>
-      <c r="D97">
-        <f>J97+K97+L97+M97+N97</f>
+      <c r="C100">
+        <v>0</v>
+      </c>
+      <c r="D100">
+        <f>J100+K100+L100+M100+N100</f>
         <v>144641.57326653044</v>
       </c>
-      <c r="E97">
+      <c r="E100">
         <v>282179.67123287602</v>
       </c>
-      <c r="F97">
+      <c r="F100">
         <v>0.85636894399557495</v>
       </c>
-      <c r="G97">
+      <c r="G100">
         <v>20627.43117349</v>
       </c>
-      <c r="H97">
+      <c r="H100">
         <v>4930.8542128783001</v>
       </c>
-      <c r="I97">
+      <c r="I100">
         <v>9095.1262763121395</v>
       </c>
-      <c r="J97">
+      <c r="J100">
         <v>34653.411662680403</v>
       </c>
-      <c r="K97">
+      <c r="K100">
         <v>50843.184005923598</v>
       </c>
-      <c r="L97">
+      <c r="L100">
         <f>L4*(1.08/0.43)</f>
         <v>38437.447108478234</v>
       </c>
-      <c r="M97">
+      <c r="M100">
         <v>19297.5304894482</v>
       </c>
-      <c r="N97">
+      <c r="N100">
         <v>1410</v>
       </c>
-      <c r="O97">
-        <v>0</v>
-      </c>
-      <c r="P97">
-        <f t="shared" ref="P97" si="23">D97+$P$1</f>
+      <c r="O100">
+        <v>0</v>
+      </c>
+      <c r="P100">
+        <f t="shared" ref="P100" si="22">D100+$P$1</f>
         <v>265201.24508552696</v>
       </c>
     </row>
-    <row r="98" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A98" t="s">
+    <row r="101" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
         <v>22</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B101" t="s">
         <v>21</v>
       </c>
-      <c r="C98">
+      <c r="C101">
         <v>4</v>
       </c>
-      <c r="D98">
-        <f>J98+K98+L98+M98+N98</f>
+      <c r="D101">
+        <f>J101+K101+L101+M101+N101</f>
         <v>141686.61445013408</v>
       </c>
-      <c r="E98">
+      <c r="E101">
         <v>282179.70347192901</v>
       </c>
-      <c r="F98">
+      <c r="F101">
         <v>0.92782505226740197</v>
       </c>
-      <c r="G98">
+      <c r="G101">
         <v>19831.065688191899</v>
       </c>
-      <c r="H98">
+      <c r="H101">
         <v>6230.6791730567802</v>
       </c>
-      <c r="I98">
+      <c r="I101">
         <v>4871.4166947967997</v>
       </c>
-      <c r="J98">
+      <c r="J101">
         <v>30933.161556045401</v>
       </c>
-      <c r="K98">
+      <c r="K101">
         <v>50937.4505788346</v>
       </c>
-      <c r="L98">
+      <c r="L101">
         <v>39073.7116581429</v>
       </c>
-      <c r="M98">
+      <c r="M101">
         <v>19317.091802737999</v>
       </c>
-      <c r="N98">
+      <c r="N101">
         <v>1425.19885437316</v>
       </c>
-      <c r="O98">
-        <v>0</v>
-      </c>
-      <c r="P98">
-        <f t="shared" ref="P98" si="24">D98+$P$1</f>
+      <c r="O101">
+        <v>0</v>
+      </c>
+      <c r="P101">
+        <f t="shared" ref="P101" si="23">D101+$P$1</f>
         <v>262246.28626913059</v>
       </c>
-      <c r="Q98">
+      <c r="Q101">
         <v>1392.0880151674601</v>
       </c>
-      <c r="R98">
+      <c r="R101">
         <v>14195.8581733913</v>
       </c>
-      <c r="S98">
+      <c r="S101">
         <v>112.66554105866101</v>
       </c>
-      <c r="T98">
+      <c r="T101">
         <v>-1.52076853589591</v>
       </c>
-      <c r="U98">
+      <c r="U101">
         <v>12183.2216733653</v>
       </c>
-      <c r="V98">
+      <c r="V101">
         <v>290.07670650869801</v>
       </c>
     </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="K99">
-        <f>SUM(K97:M97)-SUM(K98:M98)</f>
+    <row r="102" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="K102">
+        <f>SUM(K100:M100)-SUM(K101:M101)</f>
         <v>-750.09243586547382</v>
       </c>
     </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A100" t="s">
+    <row r="103" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
         <v>22</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B103" t="s">
         <v>23</v>
       </c>
-      <c r="C100">
-        <v>0</v>
-      </c>
-      <c r="D100">
-        <f>J100+K100+L100+M100+N100</f>
+      <c r="C103">
+        <v>0</v>
+      </c>
+      <c r="D103">
+        <f>J103+K103+L103+M103+N103</f>
         <v>182723.11808696718</v>
       </c>
-      <c r="E100">
+      <c r="E103">
         <v>282179.67123287602</v>
       </c>
-      <c r="F100">
+      <c r="F103">
         <v>0.85636894399557495</v>
       </c>
-      <c r="G100">
+      <c r="G103">
         <v>20627.43117349</v>
       </c>
-      <c r="H100">
+      <c r="H103">
         <v>4930.8542128783001</v>
       </c>
-      <c r="I100">
+      <c r="I103">
         <v>9095.1262763121395</v>
       </c>
-      <c r="J100">
+      <c r="J103">
         <v>34653.411662680403</v>
       </c>
-      <c r="K100">
+      <c r="K103">
         <v>50843.184005923598</v>
       </c>
-      <c r="L100">
+      <c r="L103">
         <f>L4*(2.15/0.43)</f>
         <v>76518.991928914998</v>
       </c>
-      <c r="M100">
+      <c r="M103">
         <v>19297.5304894482</v>
       </c>
-      <c r="N100">
+      <c r="N103">
         <v>1410</v>
       </c>
-    </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A101" t="s">
+      <c r="P103">
+        <f t="shared" ref="P103:P104" si="24">D103+$P$1</f>
+        <v>303282.7899059637</v>
+      </c>
+    </row>
+    <row r="104" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
         <v>22</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B104" t="s">
         <v>21</v>
       </c>
-      <c r="C101">
+      <c r="C104">
         <v>4</v>
       </c>
-      <c r="D101" s="13">
-        <f>J101+K101+L101+M101+N101</f>
+      <c r="D104" s="13">
+        <f>J104+K104+L104+M104+N104</f>
         <v>180164.72653261331</v>
       </c>
-      <c r="E101" s="13">
+      <c r="E104" s="13">
         <v>282179.67123285698</v>
       </c>
-      <c r="F101" s="12">
+      <c r="F104" s="12">
         <v>1.0641670739695701</v>
       </c>
-      <c r="G101" s="13">
+      <c r="G104" s="13">
         <v>19863.1783561796</v>
       </c>
-      <c r="H101" s="13">
+      <c r="H104" s="13">
         <v>6506.5697069746102</v>
       </c>
-      <c r="I101" s="13">
+      <c r="I104" s="13">
         <v>4873.61028676154</v>
       </c>
-      <c r="J101" s="13">
+      <c r="J104" s="13">
         <v>31243.358349915699</v>
       </c>
-      <c r="K101" s="13">
+      <c r="K104" s="13">
         <v>50899.9452054371</v>
       </c>
-      <c r="L101" s="13">
+      <c r="L104" s="13">
         <v>77281.720548983998</v>
       </c>
-      <c r="M101" s="13">
+      <c r="M104" s="13">
         <v>19309.308438346699</v>
       </c>
-      <c r="N101" s="13">
+      <c r="N104" s="13">
         <v>1430.39398992981</v>
       </c>
-      <c r="O101">
-        <v>0</v>
-      </c>
-      <c r="P101">
-        <f t="shared" ref="P101" si="25">D101+$P$1</f>
+      <c r="O104">
+        <v>0</v>
+      </c>
+      <c r="P104">
+        <f t="shared" si="24"/>
         <v>300724.39835160982</v>
       </c>
-      <c r="Q101" s="4">
+      <c r="Q104" s="4">
         <v>1453.7288077599201</v>
       </c>
-      <c r="R101">
+      <c r="R104">
         <v>14136.371585592</v>
       </c>
-      <c r="S101" s="4">
+      <c r="S104" s="4">
         <v>107.91123347780101</v>
       </c>
-      <c r="T101" s="12">
+      <c r="T104" s="12">
         <v>-4.2490908058638102</v>
       </c>
-      <c r="U101">
+      <c r="U104">
         <v>13013.5923280234</v>
       </c>
-      <c r="V101" s="4">
+      <c r="V104" s="4">
         <v>351.71871156820202</v>
       </c>
     </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="K102" s="13">
-        <f>SUM(K100:M100)-SUM(K101:M101)</f>
+    <row r="105" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="K105" s="13">
+        <f>SUM(K103:M103)-SUM(K104:M104)</f>
         <v>-831.26776848098962</v>
       </c>
     </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A106" s="7" t="s">
+    <row r="109" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A109" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A108" t="s">
+    <row r="111" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
         <v>32</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B111" t="s">
         <v>33</v>
       </c>
-      <c r="C108" t="s">
+      <c r="C111" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A109">
-        <v>20</v>
-      </c>
-      <c r="B109">
-        <v>60</v>
-      </c>
-      <c r="C109">
-        <v>2</v>
-      </c>
-      <c r="D109">
-        <f t="shared" ref="D109:D115" si="26">J109+K109+L109+M109+N109</f>
-        <v>120712.69088313227</v>
-      </c>
-      <c r="E109">
-        <v>282179.67123285501</v>
-      </c>
-      <c r="F109">
-        <v>0.854946898908852</v>
-      </c>
-      <c r="G109">
-        <v>18681.222424938602</v>
-      </c>
-      <c r="H109">
-        <v>5354.6114985546601</v>
-      </c>
-      <c r="I109">
-        <v>8156.08309050551</v>
-      </c>
-      <c r="J109">
-        <v>32191.917013998798</v>
-      </c>
-      <c r="K109">
-        <v>51372.124296964801</v>
-      </c>
-      <c r="L109">
-        <v>16725.325417965501</v>
-      </c>
-      <c r="M109">
-        <v>19407.285599838699</v>
-      </c>
-      <c r="N109">
-        <v>1016.03855436447</v>
-      </c>
-      <c r="O109">
-        <v>0</v>
-      </c>
-      <c r="P109">
-        <f t="shared" ref="P109:P115" si="27">D109+$P$1</f>
-        <v>241272.36270212877</v>
-      </c>
-      <c r="Q109">
-        <v>1192.7637589594799</v>
-      </c>
-      <c r="R109">
-        <v>19736.206339365101</v>
-      </c>
-      <c r="S109">
-        <v>481.37088632597801</v>
-      </c>
-      <c r="T109" s="6">
-        <v>0.12591688076390301</v>
-      </c>
-    </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A110">
-        <v>20</v>
-      </c>
-      <c r="B110">
-        <v>50</v>
-      </c>
-      <c r="C110">
-        <v>2</v>
-      </c>
-      <c r="D110">
-        <f t="shared" si="26"/>
-        <v>119392.42354269064</v>
-      </c>
-      <c r="E110">
-        <v>282254.81855225202</v>
-      </c>
-      <c r="F110">
-        <v>0.85006146065890897</v>
-      </c>
-      <c r="G110">
-        <v>19407.840072768398</v>
-      </c>
-      <c r="H110">
-        <v>5891.8301217549197</v>
-      </c>
-      <c r="I110">
-        <v>6659.4942697455399</v>
-      </c>
-      <c r="J110">
-        <v>31959.164464268899</v>
-      </c>
-      <c r="K110">
-        <v>51102.045942938203</v>
-      </c>
-      <c r="L110">
-        <v>15967.176494174801</v>
-      </c>
-      <c r="M110">
-        <v>19353.573908279199</v>
-      </c>
-      <c r="N110">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O110">
-        <v>0</v>
-      </c>
-      <c r="P110">
-        <f t="shared" si="27"/>
-        <v>239952.09536168716</v>
-      </c>
-      <c r="Q110">
-        <v>1312.43161993582</v>
-      </c>
-      <c r="R110">
-        <v>18377.616631847999</v>
-      </c>
-      <c r="S110">
-        <v>459.4404157962</v>
-      </c>
-      <c r="T110" s="6">
-        <v>0.14758705239613301</v>
-      </c>
-    </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A111">
-        <v>20</v>
-      </c>
-      <c r="B111">
-        <v>40</v>
-      </c>
-      <c r="C111">
-        <v>2</v>
-      </c>
-      <c r="D111">
-        <f t="shared" si="26"/>
-        <v>117777.02945340994</v>
-      </c>
-      <c r="E111">
-        <v>282179.67123287299</v>
-      </c>
-      <c r="F111">
-        <v>0.84456314023622803</v>
-      </c>
-      <c r="G111">
-        <v>19298.245593088301</v>
-      </c>
-      <c r="H111">
-        <v>5682.0016560700296</v>
-      </c>
-      <c r="I111">
-        <v>5350.3346939491703</v>
-      </c>
-      <c r="J111">
-        <v>30330.5819431075</v>
-      </c>
-      <c r="K111">
-        <v>51097.733915068202</v>
-      </c>
-      <c r="L111">
-        <v>15987.901266609</v>
-      </c>
-      <c r="M111">
-        <v>19350.349595595701</v>
-      </c>
-      <c r="N111">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O111">
-        <v>0</v>
-      </c>
-      <c r="P111">
-        <f t="shared" si="27"/>
-        <v>238336.70127240644</v>
-      </c>
-      <c r="Q111">
-        <v>1265.6913868611</v>
-      </c>
-      <c r="R111">
-        <v>17746.163883660702</v>
-      </c>
-      <c r="S111">
-        <v>507.03325381887902</v>
-      </c>
-      <c r="T111" s="6">
-        <v>-0.25983751983286502</v>
-      </c>
-    </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>20</v>
       </c>
       <c r="B112">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="C112">
         <v>2</v>
       </c>
       <c r="D112">
+        <f t="shared" ref="D112:D118" si="25">J112+K112+L112+M112+N112</f>
+        <v>120712.69088313227</v>
+      </c>
+      <c r="E112">
+        <v>282179.67123285501</v>
+      </c>
+      <c r="F112">
+        <v>0.854946898908852</v>
+      </c>
+      <c r="G112">
+        <v>18681.222424938602</v>
+      </c>
+      <c r="H112">
+        <v>5354.6114985546601</v>
+      </c>
+      <c r="I112">
+        <v>8156.08309050551</v>
+      </c>
+      <c r="J112">
+        <v>32191.917013998798</v>
+      </c>
+      <c r="K112">
+        <v>51372.124296964801</v>
+      </c>
+      <c r="L112">
+        <v>16725.325417965501</v>
+      </c>
+      <c r="M112">
+        <v>19407.285599838699</v>
+      </c>
+      <c r="N112">
+        <v>1016.03855436447</v>
+      </c>
+      <c r="O112">
+        <v>0</v>
+      </c>
+      <c r="P112">
+        <f t="shared" ref="P112:P118" si="26">D112+$P$1</f>
+        <v>241272.36270212877</v>
+      </c>
+      <c r="Q112">
+        <v>1192.7637589594799</v>
+      </c>
+      <c r="R112">
+        <v>19736.206339365101</v>
+      </c>
+      <c r="S112">
+        <v>481.37088632597801</v>
+      </c>
+      <c r="T112" s="6">
+        <v>0.12591688076390301</v>
+      </c>
+    </row>
+    <row r="113" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A113">
+        <v>20</v>
+      </c>
+      <c r="B113">
+        <v>50</v>
+      </c>
+      <c r="C113">
+        <v>2</v>
+      </c>
+      <c r="D113">
+        <f t="shared" si="25"/>
+        <v>119392.42354269064</v>
+      </c>
+      <c r="E113">
+        <v>282254.81855225202</v>
+      </c>
+      <c r="F113">
+        <v>0.85006146065890897</v>
+      </c>
+      <c r="G113">
+        <v>19407.840072768398</v>
+      </c>
+      <c r="H113">
+        <v>5891.8301217549197</v>
+      </c>
+      <c r="I113">
+        <v>6659.4942697455399</v>
+      </c>
+      <c r="J113">
+        <v>31959.164464268899</v>
+      </c>
+      <c r="K113">
+        <v>51102.045942938203</v>
+      </c>
+      <c r="L113">
+        <v>15967.176494174801</v>
+      </c>
+      <c r="M113">
+        <v>19353.573908279199</v>
+      </c>
+      <c r="N113">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O113">
+        <v>0</v>
+      </c>
+      <c r="P113">
         <f t="shared" si="26"/>
-        <v>116625.1695160947</v>
-      </c>
-      <c r="E112">
-        <v>282182.50548365602</v>
-      </c>
-      <c r="F112">
-        <v>0.84045954058697003</v>
-      </c>
-      <c r="G112">
-        <v>19302.752565837702</v>
-      </c>
-      <c r="H112">
-        <v>6226.5181629292701</v>
-      </c>
-      <c r="I112">
-        <v>3974.5318253822402</v>
-      </c>
-      <c r="J112">
-        <v>29503.802554149199</v>
-      </c>
-      <c r="K112">
-        <v>51013.610661725899</v>
-      </c>
-      <c r="L112">
-        <v>15760.601295416</v>
-      </c>
-      <c r="M112">
-        <v>19332.981882301501</v>
-      </c>
-      <c r="N112">
-        <v>1014.17312250211</v>
-      </c>
-      <c r="O112">
-        <v>0</v>
-      </c>
-      <c r="P112">
-        <f t="shared" si="27"/>
-        <v>237184.84133509122</v>
-      </c>
-      <c r="Q112">
-        <v>1386.9848841974899</v>
-      </c>
-      <c r="R112">
-        <v>18436.445202769701</v>
-      </c>
-      <c r="S112">
-        <v>209.50505912238299</v>
-      </c>
-      <c r="T112" s="6">
-        <v>0.28049716262959101</v>
-      </c>
-    </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A113" s="3">
-        <v>20</v>
-      </c>
-      <c r="B113" s="3">
-        <v>20</v>
-      </c>
-      <c r="C113" s="3">
-        <v>2</v>
-      </c>
-      <c r="D113">
-        <f t="shared" si="26"/>
-        <v>115198.459983006</v>
-      </c>
-      <c r="E113">
-        <v>282179.67123297497</v>
-      </c>
-      <c r="F113">
-        <v>0.83541194997266699</v>
-      </c>
-      <c r="G113">
-        <v>19351.2255529412</v>
-      </c>
-      <c r="H113">
-        <v>6002.0469674603501</v>
-      </c>
-      <c r="I113">
-        <v>2645.4376652921501</v>
-      </c>
-      <c r="J113">
-        <v>27998.710185693701</v>
-      </c>
-      <c r="K113">
-        <v>51033.4442867088</v>
-      </c>
-      <c r="L113">
-        <v>15815.1228903871</v>
-      </c>
-      <c r="M113">
-        <v>19337.009497714302</v>
-      </c>
-      <c r="N113">
-        <v>1014.17312250211</v>
-      </c>
-      <c r="O113">
-        <v>0</v>
-      </c>
-      <c r="P113">
-        <f t="shared" si="27"/>
-        <v>235758.13180200252</v>
+        <v>239952.09536168716</v>
       </c>
       <c r="Q113">
-        <v>1336.98290493166</v>
+        <v>1312.43161993582</v>
       </c>
       <c r="R113">
-        <v>18577.307877855899</v>
+        <v>18377.616631847999</v>
       </c>
       <c r="S113">
-        <v>432.030415764091</v>
+        <v>459.4404157962</v>
       </c>
       <c r="T113" s="6">
-        <v>-0.122490141098651</v>
-      </c>
-    </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.4">
+        <v>0.14758705239613301</v>
+      </c>
+    </row>
+    <row r="114" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>20</v>
       </c>
       <c r="B114">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="C114">
         <v>2</v>
       </c>
       <c r="D114">
-        <f t="shared" si="26"/>
-        <v>114451.25872361983</v>
+        <f t="shared" si="25"/>
+        <v>117777.02945340994</v>
       </c>
       <c r="E114">
-        <v>282179.67123267101</v>
+        <v>282179.67123287299</v>
       </c>
       <c r="F114">
-        <v>0.83277713625127903</v>
+        <v>0.84456314023622803</v>
       </c>
       <c r="G114">
-        <v>19390.977969205</v>
+        <v>19298.245593088301</v>
       </c>
       <c r="H114">
-        <v>5599.5405456203798</v>
+        <v>5682.0016560700296</v>
       </c>
       <c r="I114">
-        <v>2128.1287863747102</v>
+        <v>5350.3346939491703</v>
       </c>
       <c r="J114">
-        <v>27118.647301200101</v>
+        <v>30330.5819431075</v>
       </c>
       <c r="K114">
-        <v>51068.507704320902</v>
+        <v>51097.733915068202</v>
       </c>
       <c r="L114">
-        <v>15909.3558282099</v>
+        <v>15987.901266609</v>
       </c>
       <c r="M114">
-        <v>19344.285156859401</v>
+        <v>19350.349595595701</v>
       </c>
       <c r="N114">
         <v>1010.46273302954</v>
@@ -6134,83 +5993,275 @@
         <v>0</v>
       </c>
       <c r="P114">
-        <f t="shared" si="27"/>
-        <v>235010.93054261635</v>
+        <f t="shared" si="26"/>
+        <v>238336.70127240644</v>
       </c>
       <c r="Q114">
-        <v>1247.3228025527501</v>
+        <v>1265.6913868611</v>
       </c>
       <c r="R114">
-        <v>16417.502561416801</v>
+        <v>17746.163883660702</v>
       </c>
       <c r="S114">
-        <v>469.07150175476602</v>
+        <v>507.03325381887902</v>
       </c>
       <c r="T114" s="6">
-        <v>0.46004655114715598</v>
-      </c>
-    </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.4">
+        <v>-0.25983751983286502</v>
+      </c>
+    </row>
+    <row r="115" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>20</v>
       </c>
       <c r="B115">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="C115">
         <v>2</v>
       </c>
       <c r="D115">
+        <f t="shared" si="25"/>
+        <v>116625.1695160947</v>
+      </c>
+      <c r="E115">
+        <v>282182.50548365602</v>
+      </c>
+      <c r="F115">
+        <v>0.84045954058697003</v>
+      </c>
+      <c r="G115">
+        <v>19302.752565837702</v>
+      </c>
+      <c r="H115">
+        <v>6226.5181629292701</v>
+      </c>
+      <c r="I115">
+        <v>3974.5318253822402</v>
+      </c>
+      <c r="J115">
+        <v>29503.802554149199</v>
+      </c>
+      <c r="K115">
+        <v>51013.610661725899</v>
+      </c>
+      <c r="L115">
+        <v>15760.601295416</v>
+      </c>
+      <c r="M115">
+        <v>19332.981882301501</v>
+      </c>
+      <c r="N115">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O115">
+        <v>0</v>
+      </c>
+      <c r="P115">
         <f t="shared" si="26"/>
+        <v>237184.84133509122</v>
+      </c>
+      <c r="Q115">
+        <v>1386.9848841974899</v>
+      </c>
+      <c r="R115">
+        <v>18436.445202769701</v>
+      </c>
+      <c r="S115">
+        <v>209.50505912238299</v>
+      </c>
+      <c r="T115" s="6">
+        <v>0.28049716262959101</v>
+      </c>
+    </row>
+    <row r="116" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A116" s="3">
+        <v>20</v>
+      </c>
+      <c r="B116" s="3">
+        <v>20</v>
+      </c>
+      <c r="C116" s="3">
+        <v>2</v>
+      </c>
+      <c r="D116">
+        <f t="shared" si="25"/>
+        <v>115198.459983006</v>
+      </c>
+      <c r="E116">
+        <v>282179.67123297497</v>
+      </c>
+      <c r="F116">
+        <v>0.83541194997266699</v>
+      </c>
+      <c r="G116">
+        <v>19351.2255529412</v>
+      </c>
+      <c r="H116">
+        <v>6002.0469674603501</v>
+      </c>
+      <c r="I116">
+        <v>2645.4376652921501</v>
+      </c>
+      <c r="J116">
+        <v>27998.710185693701</v>
+      </c>
+      <c r="K116">
+        <v>51033.4442867088</v>
+      </c>
+      <c r="L116">
+        <v>15815.1228903871</v>
+      </c>
+      <c r="M116">
+        <v>19337.009497714302</v>
+      </c>
+      <c r="N116">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O116">
+        <v>0</v>
+      </c>
+      <c r="P116">
+        <f t="shared" si="26"/>
+        <v>235758.13180200252</v>
+      </c>
+      <c r="Q116">
+        <v>1336.98290493166</v>
+      </c>
+      <c r="R116">
+        <v>18577.307877855899</v>
+      </c>
+      <c r="S116">
+        <v>432.030415764091</v>
+      </c>
+      <c r="T116" s="6">
+        <v>-0.122490141098651</v>
+      </c>
+    </row>
+    <row r="117" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A117">
+        <v>20</v>
+      </c>
+      <c r="B117">
+        <v>15</v>
+      </c>
+      <c r="C117">
+        <v>2</v>
+      </c>
+      <c r="D117">
+        <f t="shared" si="25"/>
+        <v>114451.25872361983</v>
+      </c>
+      <c r="E117">
+        <v>282179.67123267101</v>
+      </c>
+      <c r="F117">
+        <v>0.83277713625127903</v>
+      </c>
+      <c r="G117">
+        <v>19390.977969205</v>
+      </c>
+      <c r="H117">
+        <v>5599.5405456203798</v>
+      </c>
+      <c r="I117">
+        <v>2128.1287863747102</v>
+      </c>
+      <c r="J117">
+        <v>27118.647301200101</v>
+      </c>
+      <c r="K117">
+        <v>51068.507704320902</v>
+      </c>
+      <c r="L117">
+        <v>15909.3558282099</v>
+      </c>
+      <c r="M117">
+        <v>19344.285156859401</v>
+      </c>
+      <c r="N117">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O117">
+        <v>0</v>
+      </c>
+      <c r="P117">
+        <f t="shared" si="26"/>
+        <v>235010.93054261635</v>
+      </c>
+      <c r="Q117">
+        <v>1247.3228025527501</v>
+      </c>
+      <c r="R117">
+        <v>16417.502561416801</v>
+      </c>
+      <c r="S117">
+        <v>469.07150175476602</v>
+      </c>
+      <c r="T117" s="6">
+        <v>0.46004655114715598</v>
+      </c>
+    </row>
+    <row r="118" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A118">
+        <v>20</v>
+      </c>
+      <c r="B118">
+        <v>12</v>
+      </c>
+      <c r="C118">
+        <v>2</v>
+      </c>
+      <c r="D118">
+        <f t="shared" si="25"/>
         <v>114787.7594081375</v>
       </c>
-      <c r="E115">
+      <c r="E118">
         <v>282179.67123287602</v>
       </c>
-      <c r="F115">
+      <c r="F118">
         <v>0.83403396920434802</v>
       </c>
-      <c r="G115">
+      <c r="G118">
         <v>20436.472361711199</v>
       </c>
-      <c r="H115">
+      <c r="H118">
         <v>4946.5396722567002</v>
       </c>
-      <c r="I115">
+      <c r="I118">
         <v>2967.9237851293901</v>
       </c>
-      <c r="J115">
+      <c r="J118">
         <v>28350.9358190973</v>
       </c>
-      <c r="K115">
+      <c r="K118">
         <v>50843.184005923598</v>
       </c>
-      <c r="L115">
+      <c r="L118">
         <v>15303.798385783</v>
       </c>
-      <c r="M115">
+      <c r="M118">
         <v>19297.530489448302</v>
       </c>
-      <c r="N115">
+      <c r="N118">
         <v>992.31070788530405</v>
       </c>
-      <c r="O115">
-        <v>0</v>
-      </c>
-      <c r="P115">
-        <f t="shared" si="27"/>
+      <c r="O118">
+        <v>0</v>
+      </c>
+      <c r="P118">
+        <f t="shared" si="26"/>
         <v>235347.43122713402</v>
       </c>
-      <c r="Q115">
+      <c r="Q118">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R115">
+      <c r="R118">
         <v>13.380488321454299</v>
       </c>
-      <c r="S115">
+      <c r="S118">
         <v>2.67609766429086</v>
       </c>
-      <c r="T115" s="6">
+      <c r="T118" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>
@@ -6230,20 +6281,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA993591-8C1F-4C7B-A75D-E9726DFB461B}">
   <dimension ref="A2:P31"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="12.84375" customWidth="1"/>
-    <col min="3" max="3" width="11.3828125" customWidth="1"/>
-    <col min="4" max="4" width="15.53515625" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" customWidth="1"/>
+    <col min="3" max="3" width="11.36328125" customWidth="1"/>
+    <col min="4" max="4" width="15.54296875" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17.07421875" customWidth="1"/>
-    <col min="7" max="7" width="15.23046875" customWidth="1"/>
-    <col min="8" max="8" width="13.23046875" customWidth="1"/>
-    <col min="9" max="11" width="11.3828125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" customWidth="1"/>
+    <col min="7" max="7" width="15.26953125" customWidth="1"/>
+    <col min="8" max="8" width="13.26953125" customWidth="1"/>
+    <col min="9" max="11" width="11.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6282,12 +6333,12 @@
       </c>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -6326,7 +6377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="D5" s="10"/>
@@ -6338,7 +6389,7 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>48</v>
       </c>
@@ -6355,7 +6406,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -6395,7 +6446,7 @@
       </c>
       <c r="M7" s="11"/>
     </row>
-    <row r="8" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -6406,7 +6457,7 @@
       <c r="K8" s="10"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -6420,7 +6471,7 @@
       <c r="K9" s="10"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>21</v>
       </c>
@@ -6456,7 +6507,7 @@
       </c>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="D11">
         <f>(34653-H10-I11+wrd_pricetater_flex_type_summar!K5+L10)/34653</f>
         <v>0.17154119896168271</v>
@@ -6473,7 +6524,7 @@
       <c r="K11" s="10"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
@@ -6487,7 +6538,7 @@
       <c r="K12" s="10"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
@@ -6527,7 +6578,7 @@
       </c>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="D14" s="10"/>
@@ -6540,7 +6591,7 @@
       <c r="K14" s="10"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>46</v>
       </c>
@@ -6553,7 +6604,7 @@
       <c r="J15" s="10"/>
       <c r="K15" s="10"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -6592,7 +6643,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="D17">
         <f>(34653-H16-I17+wrd_pricetater_flex_type_summar!K5+L16)/34653</f>
         <v>0.38932217950875497</v>
@@ -6602,7 +6653,7 @@
         <v>87792.098602195503</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>57</v>
       </c>
@@ -6641,7 +6692,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -6649,7 +6700,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -6687,7 +6738,7 @@
       </c>
       <c r="L23" s="10"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>55</v>
       </c>
@@ -6725,7 +6776,7 @@
       </c>
       <c r="L25" s="10"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -6762,7 +6813,7 @@
         <v>-476.58002357000078</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -6799,7 +6850,7 @@
         <v>174.37684745549996</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
Filling out all operation profiles for the start up time SA and added readme doc file
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A83C26BD-4FFD-40F8-BDDF-9112B52BF739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7F8078-85C9-4D50-AC78-CD6AC8E91A4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -4168,61 +4168,63 @@
         <v>4</v>
       </c>
       <c r="D62" s="10">
-        <v>114153.095713535</v>
+        <f>J62+K62+L62+M62+N62-O62</f>
+        <v>107555.29824632255</v>
       </c>
       <c r="E62">
-        <v>282179.67123343103</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F62">
-        <v>0.83530141349350295</v>
+        <v>0.80673743017586796</v>
       </c>
       <c r="G62">
-        <v>19390.3410434773</v>
+        <v>19617.269555424798</v>
       </c>
       <c r="H62">
-        <v>6212.6008869098296</v>
+        <v>6177.79087142139</v>
       </c>
       <c r="I62" s="8">
-        <v>1.21975885109732E-5</v>
+        <v>1.4897343661976701E-5</v>
       </c>
       <c r="J62">
-        <v>25602.941942584701</v>
+        <v>25795.060441743601</v>
       </c>
       <c r="K62">
-        <v>50959.945205482203</v>
+        <v>50989.945229661498</v>
       </c>
       <c r="L62">
-        <v>17946.760793761499</v>
+        <v>20356.552509954701</v>
       </c>
       <c r="M62">
-        <v>19643.4477717072</v>
+        <v>19971.3621100407</v>
       </c>
       <c r="N62">
-        <v>1459.6580951174601</v>
+        <v>1462.3779549220301</v>
       </c>
       <c r="O62">
-        <v>0</v>
+        <v>11020</v>
       </c>
       <c r="P62">
-        <v>235705.078240417</v>
+        <f t="shared" si="12"/>
+        <v>228114.97006531907</v>
       </c>
       <c r="Q62">
-        <v>1388.04888293766</v>
+        <v>1380.27146414547</v>
       </c>
       <c r="R62">
-        <v>32406.8779181912</v>
+        <v>33980.634383525299</v>
       </c>
       <c r="S62">
-        <v>611.45052675832505</v>
+        <v>943.906510653483</v>
       </c>
       <c r="T62">
-        <v>0.13840414379532001</v>
+        <v>0.36911323114551098</v>
       </c>
       <c r="U62">
-        <v>32883.087260137101</v>
+        <v>36719.7300995962</v>
       </c>
       <c r="V62">
-        <v>285.93988921858301</v>
+        <v>278.17977348178903</v>
       </c>
     </row>
     <row r="63" spans="1:22" x14ac:dyDescent="0.35">
@@ -4303,79 +4305,79 @@
       <c r="C64" s="14"/>
       <c r="D64" s="10">
         <f>D63-D62</f>
-        <v>-6111.1371802236536</v>
+        <v>486.66028698880109</v>
       </c>
       <c r="E64">
         <f t="shared" ref="E64:V64" si="13">E63-E62</f>
-        <v>-6.6100619733333588E-7</v>
+        <v>-1.0599615052342415E-7</v>
       </c>
       <c r="F64">
         <f t="shared" si="13"/>
-        <v>-2.6744535796557001E-2</v>
+        <v>1.8194475210779881E-3</v>
       </c>
       <c r="G64">
         <f t="shared" si="13"/>
-        <v>12.713114300899178</v>
+        <v>-214.21539764659974</v>
       </c>
       <c r="H64">
         <f t="shared" si="13"/>
-        <v>-659.30837613777931</v>
+        <v>-624.4983606493397</v>
       </c>
       <c r="I64">
         <f t="shared" si="13"/>
-        <v>4877.8861116945618</v>
+        <v>4877.8861089948059</v>
       </c>
       <c r="J64">
         <f t="shared" si="13"/>
-        <v>4231.290849857698</v>
+        <v>4039.1723506987983</v>
       </c>
       <c r="K64">
         <f t="shared" si="13"/>
-        <v>213.72489052519813</v>
+        <v>183.72486634590314</v>
       </c>
       <c r="L64">
         <f t="shared" si="13"/>
-        <v>-823.11437404410026</v>
+        <v>-3232.9060902373021</v>
       </c>
       <c r="M64">
         <f t="shared" si="13"/>
-        <v>-148.6656852365013</v>
+        <v>-476.58002357000078</v>
       </c>
       <c r="N64">
         <f t="shared" si="13"/>
-        <v>-24.03095644400014</v>
+        <v>-26.750816248570118</v>
       </c>
       <c r="O64">
         <f t="shared" si="13"/>
-        <v>11020</v>
+        <v>0</v>
       </c>
       <c r="P64">
         <f t="shared" si="13"/>
-        <v>-7103.4478881091345</v>
+        <v>486.66028698880109</v>
       </c>
       <c r="Q64">
         <f t="shared" si="13"/>
-        <v>-147.30581980358988</v>
+        <v>-139.52840101139986</v>
       </c>
       <c r="R64">
         <f t="shared" si="13"/>
-        <v>-14492.395483320099</v>
+        <v>-16066.151948654198</v>
       </c>
       <c r="S64">
         <f t="shared" si="13"/>
-        <v>-213.35091709452303</v>
+        <v>-545.80690098968103</v>
       </c>
       <c r="T64">
         <f t="shared" si="13"/>
-        <v>0.53457323696455306</v>
+        <v>0.30386414961436203</v>
       </c>
       <c r="U64">
         <f t="shared" si="13"/>
-        <v>-19719.855079813999</v>
+        <v>-23556.497919273097</v>
       </c>
       <c r="V64">
         <f t="shared" si="13"/>
-        <v>-178.92174141107802</v>
+        <v>-171.16162567428404</v>
       </c>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.35">
@@ -4476,55 +4478,55 @@
       <c r="C69" s="9"/>
       <c r="D69" s="10">
         <f>D68-D62</f>
-        <v>-6464.6739902054687</v>
+        <v>133.12347700698592</v>
       </c>
       <c r="E69" s="10">
         <f t="shared" ref="E69:P69" si="15">E68-E62</f>
-        <v>-5.5501004680991173E-7</v>
+        <v>0</v>
       </c>
       <c r="F69" s="10">
         <f t="shared" si="15"/>
-        <v>-2.8092214829048001E-2</v>
+        <v>4.7176848858698772E-4</v>
       </c>
       <c r="G69" s="10">
         <f t="shared" si="15"/>
-        <v>563.11394365769956</v>
+        <v>336.18543171020065</v>
       </c>
       <c r="H69" s="10">
         <f t="shared" si="15"/>
-        <v>287.95312689617003</v>
+        <v>322.76314238460964</v>
       </c>
       <c r="I69" s="10">
         <f t="shared" si="15"/>
-        <v>1.844294233963699E-6</v>
+        <v>-8.5546091703980134E-7</v>
       </c>
       <c r="J69" s="10">
         <f t="shared" si="15"/>
-        <v>851.06707239820025</v>
+        <v>658.94857323930046</v>
       </c>
       <c r="K69" s="10">
         <f t="shared" si="15"/>
-        <v>-105.00000000270666</v>
+        <v>-135.00002418200165</v>
       </c>
       <c r="L69" s="10">
         <f t="shared" si="15"/>
-        <v>2046.9791491608994</v>
+        <v>-362.81256703230247</v>
       </c>
       <c r="M69" s="10">
         <f t="shared" si="15"/>
-        <v>299.90183331549997</v>
+        <v>-28.012505017999501</v>
       </c>
       <c r="N69" s="10">
         <f t="shared" si="15"/>
-        <v>2.7198598045699782</v>
+        <v>0</v>
       </c>
       <c r="O69" s="10">
         <f t="shared" si="15"/>
-        <v>11020</v>
+        <v>0</v>
       </c>
       <c r="P69" s="10">
         <f t="shared" si="15"/>
-        <v>-7456.9846980909351</v>
+        <v>133.12347700700047</v>
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.35">
@@ -5523,7 +5525,19 @@
       <c r="F96" t="s">
         <v>36</v>
       </c>
-      <c r="G96" s="4"/>
+      <c r="G96" s="10">
+        <v>21558</v>
+      </c>
+      <c r="H96">
+        <v>7337</v>
+      </c>
+      <c r="I96">
+        <v>3883</v>
+      </c>
+      <c r="J96" s="10">
+        <f>G96+H96+I96</f>
+        <v>32778</v>
+      </c>
       <c r="K96" t="s">
         <v>64</v>
       </c>

</xml_diff>

<commit_message>
Adding initial results for working hours
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7F8078-85C9-4D50-AC78-CD6AC8E91A4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E9DD7CF-499C-4E10-93ED-BA1DA8494C03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -60,6 +60,7 @@
     <author>tc={9FF6B967-6104-43AC-8EED-15C48C9ACCA9}</author>
     <author>tc={3B63C6BF-9DE1-4172-A721-F97EE0406603}</author>
     <author>tc={FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}</author>
+    <author>tc={9D93D39A-4E12-4E91-8443-F39D5B5EA779}</author>
     <author>tc={86E634AB-9E52-4A6D-BE85-5D191C9227C6}</author>
   </authors>
   <commentList>
@@ -260,7 +261,15 @@
     5x brine costs (2.15 $/m3)</t>
       </text>
     </comment>
-    <comment ref="T115" authorId="24" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="A107" authorId="24" shapeId="0" xr:uid="{9D93D39A-4E12-4E91-8443-F39D5B5EA779}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Working Hours = 8 AM to 5 PM</t>
+      </text>
+    </comment>
+    <comment ref="T116" authorId="25" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -405,7 +414,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="66">
   <si>
     <t>Season</t>
   </si>
@@ -601,6 +610,9 @@
   <si>
     <t>?</t>
   </si>
+  <si>
+    <t>Working Hours</t>
+  </si>
 </sst>
 </file>
 
@@ -610,7 +622,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -771,6 +783,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1596,7 +1614,10 @@
   <threadedComment ref="A104" dT="2026-08-09T17:05:17.32" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}">
     <text>5x brine costs (2.15 $/m3)</text>
   </threadedComment>
-  <threadedComment ref="T115" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="A107" dT="2026-08-18T21:09:34.88" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9D93D39A-4E12-4E91-8443-F39D5B5EA779}">
+    <text>Working Hours = 8 AM to 5 PM</text>
+  </threadedComment>
+  <threadedComment ref="T116" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1662,22 +1683,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:V118"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:V119"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" customWidth="1"/>
-    <col min="3" max="3" width="10.81640625" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" customWidth="1"/>
-    <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.54296875" customWidth="1"/>
-    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.81640625" customWidth="1"/>
+    <col min="1" max="1" width="9.61328125" customWidth="1"/>
+    <col min="3" max="3" width="10.84375" customWidth="1"/>
+    <col min="5" max="5" width="10.23046875" customWidth="1"/>
+    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.69140625" customWidth="1"/>
+    <col min="9" max="9" width="9.07421875" customWidth="1"/>
+    <col min="11" max="11" width="10.84375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.53515625" customWidth="1"/>
+    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1688,7 +1709,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1756,7 +1777,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1820,7 +1841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1884,14 +1905,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G5" s="4"/>
       <c r="K5" s="10">
         <f>K4+L4+M4</f>
         <v>85444.512881154791</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1955,7 +1976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -2019,10 +2040,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2086,7 +2107,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2150,10 +2171,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -2217,7 +2238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2281,10 +2302,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2346,7 +2367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2402,10 +2423,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2469,7 +2490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2533,7 +2554,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2542,7 +2563,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2553,7 +2574,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2617,10 +2638,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2684,7 +2705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2754,11 +2775,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2822,7 +2843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2886,10 +2907,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2953,7 +2974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -3023,7 +3044,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -3093,7 +3114,7 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A33" s="14" t="s">
         <v>45</v>
       </c>
@@ -3176,19 +3197,19 @@
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="K34" s="10"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -3252,7 +3273,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3316,12 +3337,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3388,7 +3409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3458,20 +3479,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3535,15 +3556,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3613,13 +3634,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
@@ -3683,7 +3704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
@@ -3747,11 +3768,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -3815,7 +3836,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -3879,10 +3900,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
@@ -3946,7 +3967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A57" s="5" t="s">
         <v>22</v>
       </c>
@@ -4016,19 +4037,19 @@
         <v>358.72983861659498</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.4">
       <c r="K58">
         <f>K57+L57+M57-K5</f>
         <v>5401.088917483823</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -4092,7 +4113,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -4157,7 +4178,7 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A62" s="5" t="s">
         <v>22</v>
       </c>
@@ -4227,7 +4248,7 @@
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -4297,7 +4318,7 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A64" s="14" t="s">
         <v>44</v>
       </c>
@@ -4380,19 +4401,19 @@
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
       <c r="D66" s="10"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A67" s="14" t="s">
         <v>60</v>
       </c>
@@ -4400,7 +4421,7 @@
       <c r="C67" s="14"/>
       <c r="D67" s="10"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A68" s="5" t="s">
         <v>22</v>
       </c>
@@ -4470,7 +4491,7 @@
         <v>350.36946039055402</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A69" s="14" t="s">
         <v>61</v>
       </c>
@@ -4529,7 +4550,7 @@
         <v>133.12347700700047</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -4550,13 +4571,13 @@
       <c r="O70" s="10"/>
       <c r="P70" s="10"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A71" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -4568,7 +4589,7 @@
       </c>
       <c r="G72" s="4"/>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
         <v>22</v>
       </c>
@@ -4632,13 +4653,13 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="G74" s="4"/>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A75" s="3" t="s">
         <v>20</v>
       </c>
@@ -4650,7 +4671,7 @@
       </c>
       <c r="G75" s="4"/>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -4719,7 +4740,7 @@
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="D77">
@@ -4799,12 +4820,12 @@
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A78" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A79" s="3" t="s">
         <v>20</v>
       </c>
@@ -4868,7 +4889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A80" s="3" t="s">
         <v>22</v>
       </c>
@@ -4932,10 +4953,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>20</v>
       </c>
@@ -4993,7 +5014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A83" s="2" t="s">
         <v>22</v>
       </c>
@@ -5057,7 +5078,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>20</v>
       </c>
@@ -5115,7 +5136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
         <v>22</v>
       </c>
@@ -5185,7 +5206,7 @@
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.4">
       <c r="D87">
         <f>D86-D80</f>
         <v>-4018.7603482047853</v>
@@ -5235,13 +5256,13 @@
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A88" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G88" s="4"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -5305,7 +5326,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -5349,8 +5370,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.4"/>
+    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A92" s="1" t="s">
         <v>26</v>
       </c>
@@ -5371,7 +5392,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
         <v>0</v>
       </c>
@@ -5433,10 +5454,10 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G94" s="4"/>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
         <v>20</v>
       </c>
@@ -5506,7 +5527,7 @@
         <v>319.37310450388202</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A96" s="3" t="s">
         <v>20</v>
       </c>
@@ -5551,16 +5572,16 @@
         <v>36</v>
       </c>
     </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A97" s="2"/>
       <c r="G97" s="4"/>
     </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A99" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A100" t="s">
         <v>22</v>
       </c>
@@ -5613,7 +5634,7 @@
         <v>265201.24508552696</v>
       </c>
     </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
         <v>22</v>
       </c>
@@ -5683,13 +5704,13 @@
         <v>290.07670650869801</v>
       </c>
     </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:22" x14ac:dyDescent="0.4">
       <c r="K102">
         <f>SUM(K100:M100)-SUM(K101:M101)</f>
         <v>-750.09243586547382</v>
       </c>
     </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A103" t="s">
         <v>22</v>
       </c>
@@ -5739,7 +5760,7 @@
         <v>303282.7899059637</v>
       </c>
     </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A104" t="s">
         <v>22</v>
       </c>
@@ -5809,196 +5830,324 @@
         <v>351.71871156820202</v>
       </c>
     </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:22" x14ac:dyDescent="0.4">
       <c r="K105" s="13">
         <f>SUM(K103:M103)-SUM(K104:M104)</f>
         <v>-831.26776848098962</v>
       </c>
     </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A109" s="7" t="s">
+    <row r="106" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A106" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="K106" s="13"/>
+    </row>
+    <row r="107" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A107" t="s">
+        <v>22</v>
+      </c>
+      <c r="B107" t="s">
+        <v>23</v>
+      </c>
+      <c r="C107">
+        <v>4</v>
+      </c>
+      <c r="D107" s="13">
+        <f>J107+K107+L107+M107+N107</f>
+        <v>119726.39965297376</v>
+      </c>
+      <c r="E107">
+        <v>282179.83224964398</v>
+      </c>
+      <c r="F107">
+        <v>0.84996419881982699</v>
+      </c>
+      <c r="G107">
+        <v>20303.288104589901</v>
+      </c>
+      <c r="H107">
+        <v>6543.2205338351096</v>
+      </c>
+      <c r="I107">
+        <v>5999.24631325068</v>
+      </c>
+      <c r="J107">
+        <v>32845.754951675699</v>
+      </c>
+      <c r="K107">
+        <v>50843.330071946802</v>
+      </c>
+      <c r="L107">
+        <v>15304.121701009901</v>
+      </c>
+      <c r="M107">
+        <v>19297.5657896679</v>
+      </c>
+      <c r="N107">
+        <v>1435.62713867346</v>
+      </c>
+      <c r="O107">
+        <v>0</v>
+      </c>
+      <c r="P107">
+        <f t="shared" ref="P107:P108" si="25">D107+$P$1</f>
+        <v>240286.0714719703</v>
+      </c>
+      <c r="Q107">
+        <v>1461.9175121692599</v>
+      </c>
+      <c r="R107">
+        <v>30796.244401685999</v>
+      </c>
+      <c r="S107">
+        <v>375.56395611812201</v>
+      </c>
+      <c r="T107">
+        <v>1.20664176507714E-2</v>
+      </c>
+      <c r="U107">
+        <v>30890.848067330899</v>
+      </c>
+      <c r="V107">
+        <v>359.195907759661</v>
+      </c>
+    </row>
+    <row r="108" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A108" t="s">
+        <v>22</v>
+      </c>
+      <c r="B108" t="s">
+        <v>21</v>
+      </c>
+      <c r="C108">
+        <v>4</v>
+      </c>
+      <c r="D108" s="13">
+        <f>J108+K108+L108+M108+N108</f>
+        <v>118661.22865756074</v>
+      </c>
+      <c r="E108">
+        <v>282195.464864693</v>
+      </c>
+      <c r="F108">
+        <v>0.84615181718922305</v>
+      </c>
+      <c r="G108">
+        <v>20110.907995096401</v>
+      </c>
+      <c r="H108">
+        <v>6540.2066794450602</v>
+      </c>
+      <c r="I108">
+        <v>4890.2435679090904</v>
+      </c>
+      <c r="J108">
+        <v>31541.358242450598</v>
+      </c>
+      <c r="K108">
+        <v>50907.023134659299</v>
+      </c>
+      <c r="L108">
+        <v>15468.5747825788</v>
+      </c>
+      <c r="M108">
+        <v>19311.266711247299</v>
+      </c>
+      <c r="N108">
+        <v>1433.00578662475</v>
+      </c>
+      <c r="O108">
+        <v>0</v>
+      </c>
+      <c r="P108">
+        <f t="shared" si="25"/>
+        <v>239220.90047655726</v>
+      </c>
+      <c r="Q108">
+        <v>1461.2441424594499</v>
+      </c>
+      <c r="R108">
+        <v>30869.812631599802</v>
+      </c>
+      <c r="S108">
+        <v>411.59750175466399</v>
+      </c>
+      <c r="T108">
+        <v>4.6542923975130698E-2</v>
+      </c>
+      <c r="U108">
+        <v>30784.7301446001</v>
+      </c>
+      <c r="V108">
+        <v>331.01860370537798</v>
+      </c>
+    </row>
+    <row r="109" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="D109" s="13">
+        <f>D108-D31</f>
+        <v>870.81314264753019</v>
+      </c>
+      <c r="E109" s="13">
+        <f t="shared" ref="E109:N109" si="26">E108-E31</f>
+        <v>15.79363181698136</v>
+      </c>
+      <c r="F109" s="13">
+        <f t="shared" si="26"/>
+        <v>3.0492754563130609E-3</v>
+      </c>
+      <c r="G109" s="13">
+        <f t="shared" si="26"/>
+        <v>270.37094434599931</v>
+      </c>
+      <c r="H109" s="13">
+        <f t="shared" si="26"/>
+        <v>1259.5735968278204</v>
+      </c>
+      <c r="I109" s="13">
+        <f t="shared" si="26"/>
+        <v>12.753618583180469</v>
+      </c>
+      <c r="J109" s="13">
+        <f t="shared" si="26"/>
+        <v>1542.6981597569975</v>
+      </c>
+      <c r="K109" s="13">
+        <f t="shared" si="26"/>
+        <v>-170.1127457354014</v>
+      </c>
+      <c r="L109" s="13">
+        <f t="shared" si="26"/>
+        <v>-463.96926584500034</v>
+      </c>
+      <c r="M109" s="13">
+        <f t="shared" si="26"/>
+        <v>-34.808792153802642</v>
+      </c>
+      <c r="N109" s="13">
+        <f t="shared" si="26"/>
+        <v>-2.9942133752499558</v>
+      </c>
+    </row>
+    <row r="110" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A110" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A111" t="s">
+    <row r="112" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A112" t="s">
         <v>32</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B112" t="s">
         <v>33</v>
       </c>
-      <c r="C111" t="s">
+      <c r="C112" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A112">
-        <v>20</v>
-      </c>
-      <c r="B112">
-        <v>60</v>
-      </c>
-      <c r="C112">
-        <v>2</v>
-      </c>
-      <c r="D112">
-        <f t="shared" ref="D112:D118" si="25">J112+K112+L112+M112+N112</f>
-        <v>120712.69088313227</v>
-      </c>
-      <c r="E112">
-        <v>282179.67123285501</v>
-      </c>
-      <c r="F112">
-        <v>0.854946898908852</v>
-      </c>
-      <c r="G112">
-        <v>18681.222424938602</v>
-      </c>
-      <c r="H112">
-        <v>5354.6114985546601</v>
-      </c>
-      <c r="I112">
-        <v>8156.08309050551</v>
-      </c>
-      <c r="J112">
-        <v>32191.917013998798</v>
-      </c>
-      <c r="K112">
-        <v>51372.124296964801</v>
-      </c>
-      <c r="L112">
-        <v>16725.325417965501</v>
-      </c>
-      <c r="M112">
-        <v>19407.285599838699</v>
-      </c>
-      <c r="N112">
-        <v>1016.03855436447</v>
-      </c>
-      <c r="O112">
-        <v>0</v>
-      </c>
-      <c r="P112">
-        <f t="shared" ref="P112:P118" si="26">D112+$P$1</f>
-        <v>241272.36270212877</v>
-      </c>
-      <c r="Q112">
-        <v>1192.7637589594799</v>
-      </c>
-      <c r="R112">
-        <v>19736.206339365101</v>
-      </c>
-      <c r="S112">
-        <v>481.37088632597801</v>
-      </c>
-      <c r="T112" s="6">
-        <v>0.12591688076390301</v>
-      </c>
-    </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A113">
         <v>20</v>
       </c>
       <c r="B113">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C113">
         <v>2</v>
       </c>
       <c r="D113">
-        <f t="shared" si="25"/>
-        <v>119392.42354269064</v>
+        <f t="shared" ref="D113:D119" si="27">J113+K113+L113+M113+N113</f>
+        <v>120712.69088313227</v>
       </c>
       <c r="E113">
-        <v>282254.81855225202</v>
+        <v>282179.67123285501</v>
       </c>
       <c r="F113">
-        <v>0.85006146065890897</v>
+        <v>0.854946898908852</v>
       </c>
       <c r="G113">
-        <v>19407.840072768398</v>
+        <v>18681.222424938602</v>
       </c>
       <c r="H113">
-        <v>5891.8301217549197</v>
+        <v>5354.6114985546601</v>
       </c>
       <c r="I113">
-        <v>6659.4942697455399</v>
+        <v>8156.08309050551</v>
       </c>
       <c r="J113">
-        <v>31959.164464268899</v>
+        <v>32191.917013998798</v>
       </c>
       <c r="K113">
-        <v>51102.045942938203</v>
+        <v>51372.124296964801</v>
       </c>
       <c r="L113">
-        <v>15967.176494174801</v>
+        <v>16725.325417965501</v>
       </c>
       <c r="M113">
-        <v>19353.573908279199</v>
+        <v>19407.285599838699</v>
       </c>
       <c r="N113">
-        <v>1010.46273302954</v>
+        <v>1016.03855436447</v>
       </c>
       <c r="O113">
         <v>0</v>
       </c>
       <c r="P113">
-        <f t="shared" si="26"/>
-        <v>239952.09536168716</v>
+        <f t="shared" ref="P113:P119" si="28">D113+$P$1</f>
+        <v>241272.36270212877</v>
       </c>
       <c r="Q113">
-        <v>1312.43161993582</v>
+        <v>1192.7637589594799</v>
       </c>
       <c r="R113">
-        <v>18377.616631847999</v>
+        <v>19736.206339365101</v>
       </c>
       <c r="S113">
-        <v>459.4404157962</v>
+        <v>481.37088632597801</v>
       </c>
       <c r="T113" s="6">
-        <v>0.14758705239613301</v>
-      </c>
-    </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.35">
+        <v>0.12591688076390301</v>
+      </c>
+    </row>
+    <row r="114" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A114">
         <v>20</v>
       </c>
       <c r="B114">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C114">
         <v>2</v>
       </c>
       <c r="D114">
-        <f t="shared" si="25"/>
-        <v>117777.02945340994</v>
+        <f t="shared" si="27"/>
+        <v>119392.42354269064</v>
       </c>
       <c r="E114">
-        <v>282179.67123287299</v>
+        <v>282254.81855225202</v>
       </c>
       <c r="F114">
-        <v>0.84456314023622803</v>
+        <v>0.85006146065890897</v>
       </c>
       <c r="G114">
-        <v>19298.245593088301</v>
+        <v>19407.840072768398</v>
       </c>
       <c r="H114">
-        <v>5682.0016560700296</v>
+        <v>5891.8301217549197</v>
       </c>
       <c r="I114">
-        <v>5350.3346939491703</v>
+        <v>6659.4942697455399</v>
       </c>
       <c r="J114">
-        <v>30330.5819431075</v>
+        <v>31959.164464268899</v>
       </c>
       <c r="K114">
-        <v>51097.733915068202</v>
+        <v>51102.045942938203</v>
       </c>
       <c r="L114">
-        <v>15987.901266609</v>
+        <v>15967.176494174801</v>
       </c>
       <c r="M114">
-        <v>19350.349595595701</v>
+        <v>19353.573908279199</v>
       </c>
       <c r="N114">
         <v>1010.46273302954</v>
@@ -6007,126 +6156,126 @@
         <v>0</v>
       </c>
       <c r="P114">
-        <f t="shared" si="26"/>
-        <v>238336.70127240644</v>
+        <f t="shared" si="28"/>
+        <v>239952.09536168716</v>
       </c>
       <c r="Q114">
-        <v>1265.6913868611</v>
+        <v>1312.43161993582</v>
       </c>
       <c r="R114">
-        <v>17746.163883660702</v>
+        <v>18377.616631847999</v>
       </c>
       <c r="S114">
-        <v>507.03325381887902</v>
+        <v>459.4404157962</v>
       </c>
       <c r="T114" s="6">
-        <v>-0.25983751983286502</v>
-      </c>
-    </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.35">
+        <v>0.14758705239613301</v>
+      </c>
+    </row>
+    <row r="115" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A115">
         <v>20</v>
       </c>
       <c r="B115">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C115">
         <v>2</v>
       </c>
       <c r="D115">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
+        <v>117777.02945340994</v>
+      </c>
+      <c r="E115">
+        <v>282179.67123287299</v>
+      </c>
+      <c r="F115">
+        <v>0.84456314023622803</v>
+      </c>
+      <c r="G115">
+        <v>19298.245593088301</v>
+      </c>
+      <c r="H115">
+        <v>5682.0016560700296</v>
+      </c>
+      <c r="I115">
+        <v>5350.3346939491703</v>
+      </c>
+      <c r="J115">
+        <v>30330.5819431075</v>
+      </c>
+      <c r="K115">
+        <v>51097.733915068202</v>
+      </c>
+      <c r="L115">
+        <v>15987.901266609</v>
+      </c>
+      <c r="M115">
+        <v>19350.349595595701</v>
+      </c>
+      <c r="N115">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O115">
+        <v>0</v>
+      </c>
+      <c r="P115">
+        <f t="shared" si="28"/>
+        <v>238336.70127240644</v>
+      </c>
+      <c r="Q115">
+        <v>1265.6913868611</v>
+      </c>
+      <c r="R115">
+        <v>17746.163883660702</v>
+      </c>
+      <c r="S115">
+        <v>507.03325381887902</v>
+      </c>
+      <c r="T115" s="6">
+        <v>-0.25983751983286502</v>
+      </c>
+    </row>
+    <row r="116" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A116">
+        <v>20</v>
+      </c>
+      <c r="B116">
+        <v>30</v>
+      </c>
+      <c r="C116">
+        <v>2</v>
+      </c>
+      <c r="D116">
+        <f t="shared" si="27"/>
         <v>116625.1695160947</v>
       </c>
-      <c r="E115">
+      <c r="E116">
         <v>282182.50548365602</v>
       </c>
-      <c r="F115">
+      <c r="F116">
         <v>0.84045954058697003</v>
       </c>
-      <c r="G115">
+      <c r="G116">
         <v>19302.752565837702</v>
       </c>
-      <c r="H115">
+      <c r="H116">
         <v>6226.5181629292701</v>
       </c>
-      <c r="I115">
+      <c r="I116">
         <v>3974.5318253822402</v>
       </c>
-      <c r="J115">
+      <c r="J116">
         <v>29503.802554149199</v>
       </c>
-      <c r="K115">
+      <c r="K116">
         <v>51013.610661725899</v>
       </c>
-      <c r="L115">
+      <c r="L116">
         <v>15760.601295416</v>
       </c>
-      <c r="M115">
+      <c r="M116">
         <v>19332.981882301501</v>
-      </c>
-      <c r="N115">
-        <v>1014.17312250211</v>
-      </c>
-      <c r="O115">
-        <v>0</v>
-      </c>
-      <c r="P115">
-        <f t="shared" si="26"/>
-        <v>237184.84133509122</v>
-      </c>
-      <c r="Q115">
-        <v>1386.9848841974899</v>
-      </c>
-      <c r="R115">
-        <v>18436.445202769701</v>
-      </c>
-      <c r="S115">
-        <v>209.50505912238299</v>
-      </c>
-      <c r="T115" s="6">
-        <v>0.28049716262959101</v>
-      </c>
-    </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A116" s="3">
-        <v>20</v>
-      </c>
-      <c r="B116" s="3">
-        <v>20</v>
-      </c>
-      <c r="C116" s="3">
-        <v>2</v>
-      </c>
-      <c r="D116">
-        <f t="shared" si="25"/>
-        <v>115198.459983006</v>
-      </c>
-      <c r="E116">
-        <v>282179.67123297497</v>
-      </c>
-      <c r="F116">
-        <v>0.83541194997266699</v>
-      </c>
-      <c r="G116">
-        <v>19351.2255529412</v>
-      </c>
-      <c r="H116">
-        <v>6002.0469674603501</v>
-      </c>
-      <c r="I116">
-        <v>2645.4376652921501</v>
-      </c>
-      <c r="J116">
-        <v>27998.710185693701</v>
-      </c>
-      <c r="K116">
-        <v>51033.4442867088</v>
-      </c>
-      <c r="L116">
-        <v>15815.1228903871</v>
-      </c>
-      <c r="M116">
-        <v>19337.009497714302</v>
       </c>
       <c r="N116">
         <v>1014.17312250211</v>
@@ -6135,147 +6284,211 @@
         <v>0</v>
       </c>
       <c r="P116">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
+        <v>237184.84133509122</v>
+      </c>
+      <c r="Q116">
+        <v>1386.9848841974899</v>
+      </c>
+      <c r="R116">
+        <v>18436.445202769701</v>
+      </c>
+      <c r="S116">
+        <v>209.50505912238299</v>
+      </c>
+      <c r="T116" s="6">
+        <v>0.28049716262959101</v>
+      </c>
+    </row>
+    <row r="117" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A117" s="3">
+        <v>20</v>
+      </c>
+      <c r="B117" s="3">
+        <v>20</v>
+      </c>
+      <c r="C117" s="3">
+        <v>2</v>
+      </c>
+      <c r="D117">
+        <f t="shared" si="27"/>
+        <v>115198.459983006</v>
+      </c>
+      <c r="E117">
+        <v>282179.67123297497</v>
+      </c>
+      <c r="F117">
+        <v>0.83541194997266699</v>
+      </c>
+      <c r="G117">
+        <v>19351.2255529412</v>
+      </c>
+      <c r="H117">
+        <v>6002.0469674603501</v>
+      </c>
+      <c r="I117">
+        <v>2645.4376652921501</v>
+      </c>
+      <c r="J117">
+        <v>27998.710185693701</v>
+      </c>
+      <c r="K117">
+        <v>51033.4442867088</v>
+      </c>
+      <c r="L117">
+        <v>15815.1228903871</v>
+      </c>
+      <c r="M117">
+        <v>19337.009497714302</v>
+      </c>
+      <c r="N117">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O117">
+        <v>0</v>
+      </c>
+      <c r="P117">
+        <f t="shared" si="28"/>
         <v>235758.13180200252</v>
       </c>
-      <c r="Q116">
+      <c r="Q117">
         <v>1336.98290493166</v>
       </c>
-      <c r="R116">
+      <c r="R117">
         <v>18577.307877855899</v>
       </c>
-      <c r="S116">
+      <c r="S117">
         <v>432.030415764091</v>
       </c>
-      <c r="T116" s="6">
+      <c r="T117" s="6">
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A117">
-        <v>20</v>
-      </c>
-      <c r="B117">
-        <v>15</v>
-      </c>
-      <c r="C117">
-        <v>2</v>
-      </c>
-      <c r="D117">
-        <f t="shared" si="25"/>
-        <v>114451.25872361983</v>
-      </c>
-      <c r="E117">
-        <v>282179.67123267101</v>
-      </c>
-      <c r="F117">
-        <v>0.83277713625127903</v>
-      </c>
-      <c r="G117">
-        <v>19390.977969205</v>
-      </c>
-      <c r="H117">
-        <v>5599.5405456203798</v>
-      </c>
-      <c r="I117">
-        <v>2128.1287863747102</v>
-      </c>
-      <c r="J117">
-        <v>27118.647301200101</v>
-      </c>
-      <c r="K117">
-        <v>51068.507704320902</v>
-      </c>
-      <c r="L117">
-        <v>15909.3558282099</v>
-      </c>
-      <c r="M117">
-        <v>19344.285156859401</v>
-      </c>
-      <c r="N117">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O117">
-        <v>0</v>
-      </c>
-      <c r="P117">
-        <f t="shared" si="26"/>
-        <v>235010.93054261635</v>
-      </c>
-      <c r="Q117">
-        <v>1247.3228025527501</v>
-      </c>
-      <c r="R117">
-        <v>16417.502561416801</v>
-      </c>
-      <c r="S117">
-        <v>469.07150175476602</v>
-      </c>
-      <c r="T117" s="6">
-        <v>0.46004655114715598</v>
-      </c>
-    </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A118">
         <v>20</v>
       </c>
       <c r="B118">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C118">
         <v>2</v>
       </c>
       <c r="D118">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
+        <v>114451.25872361983</v>
+      </c>
+      <c r="E118">
+        <v>282179.67123267101</v>
+      </c>
+      <c r="F118">
+        <v>0.83277713625127903</v>
+      </c>
+      <c r="G118">
+        <v>19390.977969205</v>
+      </c>
+      <c r="H118">
+        <v>5599.5405456203798</v>
+      </c>
+      <c r="I118">
+        <v>2128.1287863747102</v>
+      </c>
+      <c r="J118">
+        <v>27118.647301200101</v>
+      </c>
+      <c r="K118">
+        <v>51068.507704320902</v>
+      </c>
+      <c r="L118">
+        <v>15909.3558282099</v>
+      </c>
+      <c r="M118">
+        <v>19344.285156859401</v>
+      </c>
+      <c r="N118">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O118">
+        <v>0</v>
+      </c>
+      <c r="P118">
+        <f t="shared" si="28"/>
+        <v>235010.93054261635</v>
+      </c>
+      <c r="Q118">
+        <v>1247.3228025527501</v>
+      </c>
+      <c r="R118">
+        <v>16417.502561416801</v>
+      </c>
+      <c r="S118">
+        <v>469.07150175476602</v>
+      </c>
+      <c r="T118" s="6">
+        <v>0.46004655114715598</v>
+      </c>
+    </row>
+    <row r="119" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A119">
+        <v>20</v>
+      </c>
+      <c r="B119">
+        <v>12</v>
+      </c>
+      <c r="C119">
+        <v>2</v>
+      </c>
+      <c r="D119">
+        <f t="shared" si="27"/>
         <v>114787.7594081375</v>
       </c>
-      <c r="E118">
+      <c r="E119">
         <v>282179.67123287602</v>
       </c>
-      <c r="F118">
+      <c r="F119">
         <v>0.83403396920434802</v>
       </c>
-      <c r="G118">
+      <c r="G119">
         <v>20436.472361711199</v>
       </c>
-      <c r="H118">
+      <c r="H119">
         <v>4946.5396722567002</v>
       </c>
-      <c r="I118">
+      <c r="I119">
         <v>2967.9237851293901</v>
       </c>
-      <c r="J118">
+      <c r="J119">
         <v>28350.9358190973</v>
       </c>
-      <c r="K118">
+      <c r="K119">
         <v>50843.184005923598</v>
       </c>
-      <c r="L118">
+      <c r="L119">
         <v>15303.798385783</v>
       </c>
-      <c r="M118">
+      <c r="M119">
         <v>19297.530489448302</v>
       </c>
-      <c r="N118">
+      <c r="N119">
         <v>992.31070788530405</v>
       </c>
-      <c r="O118">
-        <v>0</v>
-      </c>
-      <c r="P118">
-        <f t="shared" si="26"/>
+      <c r="O119">
+        <v>0</v>
+      </c>
+      <c r="P119">
+        <f t="shared" si="28"/>
         <v>235347.43122713402</v>
       </c>
-      <c r="Q118">
+      <c r="Q119">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R118">
+      <c r="R119">
         <v>13.380488321454299</v>
       </c>
-      <c r="S118">
+      <c r="S119">
         <v>2.67609766429086</v>
       </c>
-      <c r="T118" s="6">
+      <c r="T119" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>
@@ -6295,20 +6508,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA993591-8C1F-4C7B-A75D-E9726DFB461B}">
   <dimension ref="A2:P31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="12.81640625" customWidth="1"/>
-    <col min="3" max="3" width="11.36328125" customWidth="1"/>
-    <col min="4" max="4" width="15.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.84375" customWidth="1"/>
+    <col min="3" max="3" width="11.3828125" customWidth="1"/>
+    <col min="4" max="4" width="15.53515625" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17.08984375" customWidth="1"/>
-    <col min="7" max="7" width="15.26953125" customWidth="1"/>
-    <col min="8" max="8" width="13.26953125" customWidth="1"/>
-    <col min="9" max="11" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.07421875" customWidth="1"/>
+    <col min="7" max="7" width="15.23046875" customWidth="1"/>
+    <col min="8" max="8" width="13.23046875" customWidth="1"/>
+    <col min="9" max="11" width="11.3828125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6347,12 +6560,12 @@
       </c>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -6391,7 +6604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="D5" s="10"/>
@@ -6403,7 +6616,7 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>48</v>
       </c>
@@ -6420,7 +6633,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -6460,7 +6673,7 @@
       </c>
       <c r="M7" s="11"/>
     </row>
-    <row r="8" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -6471,7 +6684,7 @@
       <c r="K8" s="10"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -6485,7 +6698,7 @@
       <c r="K9" s="10"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B10" t="s">
         <v>21</v>
       </c>
@@ -6521,7 +6734,7 @@
       </c>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
       <c r="D11">
         <f>(34653-H10-I11+wrd_pricetater_flex_type_summar!K5+L10)/34653</f>
         <v>0.17154119896168271</v>
@@ -6538,7 +6751,7 @@
       <c r="K11" s="10"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
@@ -6552,7 +6765,7 @@
       <c r="K12" s="10"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
@@ -6592,7 +6805,7 @@
       </c>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="D14" s="10"/>
@@ -6605,7 +6818,7 @@
       <c r="K14" s="10"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>46</v>
       </c>
@@ -6618,7 +6831,7 @@
       <c r="J15" s="10"/>
       <c r="K15" s="10"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -6657,7 +6870,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
       <c r="D17">
         <f>(34653-H16-I17+wrd_pricetater_flex_type_summar!K5+L16)/34653</f>
         <v>0.38932217950875497</v>
@@ -6667,7 +6880,7 @@
         <v>87792.098602195503</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
         <v>57</v>
       </c>
@@ -6706,7 +6919,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -6714,7 +6927,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -6752,7 +6965,7 @@
       </c>
       <c r="L23" s="10"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>55</v>
       </c>
@@ -6790,7 +7003,7 @@
       </c>
       <c r="L25" s="10"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -6827,7 +7040,7 @@
         <v>-476.58002357000078</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -6864,7 +7077,7 @@
         <v>174.37684745549996</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
Renaming and moving files
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABF172F2-0314-48C3-A4B0-94AF47F3F4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B28D283B-92D7-4C23-AD96-27FA9C83007B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" firstSheet="1" activeTab="2" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
     <sheet name="Understanding DR Result" sheetId="2" r:id="rId2"/>
+    <sheet name="Sensitivity Analyses" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -61,6 +62,7 @@
     <author>tc={3B63C6BF-9DE1-4172-A721-F97EE0406603}</author>
     <author>tc={FE798470-8A4D-4C72-9935-5EF1B8A7CFB6}</author>
     <author>tc={9D93D39A-4E12-4E91-8443-F39D5B5EA779}</author>
+    <author>tc={9585276E-E9B8-4AFF-9F58-E3ADC73D024E}</author>
     <author>tc={86E634AB-9E52-4A6D-BE85-5D191C9227C6}</author>
   </authors>
   <commentList>
@@ -269,7 +271,15 @@
     Working Hours = 8 AM to 5 PM</t>
       </text>
     </comment>
-    <comment ref="T116" authorId="25" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <comment ref="A112" authorId="25" shapeId="0" xr:uid="{9585276E-E9B8-4AFF-9F58-E3ADC73D024E}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Five Shutdowns</t>
+      </text>
+    </comment>
+    <comment ref="T120" authorId="26" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -413,8 +423,53 @@
 </comments>
 </file>
 
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={91B01F22-295E-46BB-ACCB-2E4ED162A079}</author>
+    <author>tc={E817B344-0186-401A-AC52-C5615721C22C}</author>
+    <author>tc={338E2122-408B-451A-85D7-EF9A92A8E19E}</author>
+    <author>tc={82E3A100-DFFE-4CB2-B9B2-E28BF20128AB}</author>
+  </authors>
+  <commentList>
+    <comment ref="G2" authorId="0" shapeId="0" xr:uid="{91B01F22-295E-46BB-ACCB-2E4ED162A079}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This should be a formula</t>
+      </text>
+    </comment>
+    <comment ref="Q2" authorId="1" shapeId="0" xr:uid="{E817B344-0186-401A-AC52-C5615721C22C}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    By default, these numbers are incorrect. Only the green numbers are correct</t>
+      </text>
+    </comment>
+    <comment ref="V2" authorId="2" shapeId="0" xr:uid="{338E2122-408B-451A-85D7-EF9A92A8E19E}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This isn’t being calculated correctly...</t>
+      </text>
+    </comment>
+    <comment ref="A5" authorId="3" shapeId="0" xr:uid="{82E3A100-DFFE-4CB2-B9B2-E28BF20128AB}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Higher costs don’t change the solution because it avoids shutdowns</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="73">
   <si>
     <t>Season</t>
   </si>
@@ -613,6 +668,27 @@
   <si>
     <t>Working Hours</t>
   </si>
+  <si>
+    <t>No Brine Cost During Startup</t>
+  </si>
+  <si>
+    <t>BRINE COST DURING STARTUP</t>
+  </si>
+  <si>
+    <t>Rate Structure</t>
+  </si>
+  <si>
+    <t>TOU3</t>
+  </si>
+  <si>
+    <t>Shutdowns</t>
+  </si>
+  <si>
+    <t>TOU3 + DR</t>
+  </si>
+  <si>
+    <t>RTP</t>
+  </si>
 </sst>
 </file>
 
@@ -622,7 +698,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -783,6 +859,24 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1611,7 +1705,10 @@
   <threadedComment ref="A107" dT="2026-08-18T21:09:34.88" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9D93D39A-4E12-4E91-8443-F39D5B5EA779}">
     <text>Working Hours = 8 AM to 5 PM</text>
   </threadedComment>
-  <threadedComment ref="T116" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+  <threadedComment ref="A112" dT="2026-08-28T19:35:29.57" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9585276E-E9B8-4AFF-9F58-E3ADC73D024E}">
+    <text>Five Shutdowns</text>
+  </threadedComment>
+  <threadedComment ref="T120" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
     <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
@@ -1675,24 +1772,42 @@
 </ThreadedComments>
 </file>
 
+<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="G2" dT="2026-07-20T22:02:04.36" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{91B01F22-295E-46BB-ACCB-2E4ED162A079}">
+    <text>This should be a formula</text>
+  </threadedComment>
+  <threadedComment ref="Q2" dT="2026-07-15T21:03:49.32" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{E817B344-0186-401A-AC52-C5615721C22C}">
+    <text>By default, these numbers are incorrect. Only the green numbers are correct</text>
+  </threadedComment>
+  <threadedComment ref="V2" dT="2026-07-15T22:57:33.93" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{338E2122-408B-451A-85D7-EF9A92A8E19E}">
+    <text>This isn’t being calculated correctly...</text>
+  </threadedComment>
+  <threadedComment ref="A5" dT="2026-08-28T23:13:11.99" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{82E3A100-DFFE-4CB2-B9B2-E28BF20128AB}">
+    <text>Higher costs don’t change the solution because it avoids shutdowns</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:V119"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:V123"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.61328125" customWidth="1"/>
-    <col min="3" max="3" width="10.84375" customWidth="1"/>
-    <col min="5" max="5" width="10.23046875" customWidth="1"/>
-    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.69140625" customWidth="1"/>
-    <col min="9" max="9" width="9.07421875" customWidth="1"/>
-    <col min="11" max="11" width="10.84375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.53515625" customWidth="1"/>
-    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.84375" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" customWidth="1"/>
+    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.54296875" customWidth="1"/>
+    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1703,7 +1818,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1771,7 +1886,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1835,7 +1950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -1899,14 +2014,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G5" s="4"/>
       <c r="K5" s="10">
         <f>K4+L4+M4</f>
         <v>85444.512881154791</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1970,7 +2085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -2034,10 +2149,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2101,7 +2216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2165,10 +2280,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -2232,7 +2347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2296,10 +2411,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2361,7 +2476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2417,10 +2532,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2484,7 +2599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2548,7 +2663,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2557,7 +2672,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2568,7 +2683,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2632,10 +2747,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2699,7 +2814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2769,11 +2884,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2837,7 +2952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -2901,10 +3016,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2968,7 +3083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -3038,7 +3153,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -3108,7 +3223,7 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A33" s="14" t="s">
         <v>45</v>
       </c>
@@ -3191,19 +3306,19 @@
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="K34" s="10"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -3267,7 +3382,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3331,12 +3446,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3403,7 +3518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3473,20 +3588,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3550,15 +3665,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3628,13 +3743,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
@@ -3698,7 +3813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
@@ -3762,11 +3877,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -3830,7 +3945,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -3894,10 +4009,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
@@ -3961,7 +4076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>22</v>
       </c>
@@ -4031,19 +4146,19 @@
         <v>358.72983861659498</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
       <c r="K58">
         <f>K57+L57+M57-K5</f>
         <v>5401.088917483823</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -4107,7 +4222,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -4172,7 +4287,7 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
         <v>22</v>
       </c>
@@ -4242,7 +4357,7 @@
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -4312,7 +4427,7 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A64" s="14" t="s">
         <v>44</v>
       </c>
@@ -4395,19 +4510,19 @@
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
       <c r="D66" s="10"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A67" s="14" t="s">
         <v>60</v>
       </c>
@@ -4415,7 +4530,7 @@
       <c r="C67" s="14"/>
       <c r="D67" s="10"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
         <v>22</v>
       </c>
@@ -4485,7 +4600,7 @@
         <v>350.36946039055402</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A69" s="14" t="s">
         <v>61</v>
       </c>
@@ -4544,7 +4659,7 @@
         <v>133.12347700700047</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -4565,13 +4680,13 @@
       <c r="O70" s="10"/>
       <c r="P70" s="10"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -4583,7 +4698,7 @@
       </c>
       <c r="G72" s="4"/>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>22</v>
       </c>
@@ -4647,13 +4762,13 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="G74" s="4"/>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
         <v>20</v>
       </c>
@@ -4665,7 +4780,7 @@
       </c>
       <c r="G75" s="4"/>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -4734,7 +4849,7 @@
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="D77">
@@ -4814,12 +4929,12 @@
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
         <v>20</v>
       </c>
@@ -4883,7 +4998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
         <v>22</v>
       </c>
@@ -4947,10 +5062,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>20</v>
       </c>
@@ -5008,7 +5123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>22</v>
       </c>
@@ -5072,7 +5187,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>20</v>
       </c>
@@ -5130,7 +5245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>22</v>
       </c>
@@ -5200,7 +5315,7 @@
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.35">
       <c r="D87">
         <f>D86-D80</f>
         <v>-4018.7603482047853</v>
@@ -5250,13 +5365,13 @@
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G88" s="4"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -5320,7 +5435,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -5364,8 +5479,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.4"/>
-    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>26</v>
       </c>
@@ -5386,7 +5501,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>0</v>
       </c>
@@ -5448,10 +5563,10 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G94" s="4"/>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>20</v>
       </c>
@@ -5521,7 +5636,7 @@
         <v>319.37310450388202</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A96" s="3" t="s">
         <v>20</v>
       </c>
@@ -5566,16 +5681,16 @@
         <v>36</v>
       </c>
     </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A97" s="2"/>
       <c r="G97" s="4"/>
     </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>22</v>
       </c>
@@ -5628,7 +5743,7 @@
         <v>265201.24508552696</v>
       </c>
     </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>22</v>
       </c>
@@ -5698,13 +5813,13 @@
         <v>290.07670650869801</v>
       </c>
     </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:22" x14ac:dyDescent="0.35">
       <c r="K102">
         <f>SUM(K100:M100)-SUM(K101:M101)</f>
         <v>-750.09243586547382</v>
       </c>
     </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>22</v>
       </c>
@@ -5754,7 +5869,7 @@
         <v>303282.7899059637</v>
       </c>
     </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>22</v>
       </c>
@@ -5824,19 +5939,19 @@
         <v>351.71871156820202</v>
       </c>
     </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:22" x14ac:dyDescent="0.35">
       <c r="K105" s="13">
         <f>SUM(K103:M103)-SUM(K104:M104)</f>
         <v>-831.26776848098962</v>
       </c>
     </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="106" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>65</v>
       </c>
       <c r="K106" s="13"/>
     </row>
-    <row r="107" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="107" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>22</v>
       </c>
@@ -5906,7 +6021,7 @@
         <v>359.195907759661</v>
       </c>
     </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>22</v>
       </c>
@@ -5976,7 +6091,7 @@
         <v>331.01860370537798</v>
       </c>
     </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="109" spans="1:22" x14ac:dyDescent="0.35">
       <c r="D109" s="13">
         <f>D108-D31</f>
         <v>870.81314264753019</v>
@@ -6022,382 +6137,254 @@
         <v>-2.9942133752499558</v>
       </c>
     </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A110" s="7" t="s">
+    <row r="110" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="D110" s="13"/>
+      <c r="E110" s="13"/>
+      <c r="F110" s="13"/>
+      <c r="G110" s="13"/>
+      <c r="H110" s="13"/>
+      <c r="I110" s="13"/>
+      <c r="J110" s="13"/>
+      <c r="K110" s="13"/>
+      <c r="L110" s="13"/>
+      <c r="M110" s="13"/>
+      <c r="N110" s="13"/>
+    </row>
+    <row r="111" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A111" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D111" s="13"/>
+      <c r="E111" s="13"/>
+      <c r="F111" s="13"/>
+      <c r="G111" s="13"/>
+      <c r="H111" s="13"/>
+      <c r="I111" s="13"/>
+      <c r="J111" s="13"/>
+      <c r="K111" s="13"/>
+      <c r="L111" s="13"/>
+      <c r="M111" s="13"/>
+      <c r="N111" s="13"/>
+    </row>
+    <row r="112" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
+        <v>22</v>
+      </c>
+      <c r="B112" t="s">
+        <v>21</v>
+      </c>
+      <c r="C112">
+        <v>4</v>
+      </c>
+      <c r="D112" s="13">
+        <f>J112+K112+L112+M112+N112</f>
+        <v>113976.01616633293</v>
+      </c>
+      <c r="E112">
+        <v>282179.67123285797</v>
+      </c>
+      <c r="F112">
+        <v>0.82949143613233001</v>
+      </c>
+      <c r="G112">
+        <v>19739.4095985942</v>
+      </c>
+      <c r="H112">
+        <v>6280.2265894411403</v>
+      </c>
+      <c r="I112">
+        <v>0</v>
+      </c>
+      <c r="J112">
+        <v>26019.6361880353</v>
+      </c>
+      <c r="K112">
+        <v>50944.945205466604</v>
+      </c>
+      <c r="L112">
+        <v>15577.281609678699</v>
+      </c>
+      <c r="M112">
+        <v>19971.775208230301</v>
+      </c>
+      <c r="N112">
+        <v>1462.3779549220301</v>
+      </c>
+      <c r="O112">
+        <v>0</v>
+      </c>
+      <c r="P112">
+        <f t="shared" ref="P112" si="27">D112+$P$1</f>
+        <v>234535.68798532945</v>
+      </c>
+      <c r="Q112">
+        <v>1403.15815187257</v>
+      </c>
+      <c r="R112">
+        <v>34638.685534293101</v>
+      </c>
+      <c r="S112">
+        <v>865.96713835732805</v>
+      </c>
+      <c r="T112">
+        <v>0.1767383415172</v>
+      </c>
+      <c r="U112">
+        <v>38493.267558113897</v>
+      </c>
+      <c r="V112">
+        <v>300.72865279776499</v>
+      </c>
+    </row>
+    <row r="113" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="D113" s="12">
+        <f>(D112-D4)</f>
+        <v>-7531.9083775022591</v>
+      </c>
+      <c r="E113" s="13"/>
+      <c r="F113" s="13"/>
+      <c r="G113" s="13"/>
+      <c r="H113" s="13"/>
+      <c r="I113" s="13"/>
+      <c r="J113" s="13"/>
+      <c r="K113" s="13"/>
+      <c r="L113" s="13"/>
+      <c r="M113" s="13"/>
+      <c r="N113" s="13"/>
+    </row>
+    <row r="114" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="D114" s="13"/>
+      <c r="E114" s="13"/>
+      <c r="F114" s="13"/>
+      <c r="G114" s="13"/>
+      <c r="H114" s="13"/>
+      <c r="I114" s="13"/>
+      <c r="J114" s="13"/>
+      <c r="K114" s="13"/>
+      <c r="L114" s="13"/>
+      <c r="M114" s="13"/>
+      <c r="N114" s="13"/>
+    </row>
+    <row r="115" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A115" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A112" t="s">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
         <v>32</v>
       </c>
-      <c r="B112" t="s">
+      <c r="B116" t="s">
         <v>33</v>
       </c>
-      <c r="C112" t="s">
+      <c r="C116" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A113">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A117">
         <v>20</v>
       </c>
-      <c r="B113">
+      <c r="B117">
         <v>60</v>
       </c>
-      <c r="C113">
+      <c r="C117">
         <v>2</v>
       </c>
-      <c r="D113">
-        <f t="shared" ref="D113:D119" si="27">J113+K113+L113+M113+N113</f>
+      <c r="D117">
+        <f t="shared" ref="D117:D123" si="28">J117+K117+L117+M117+N117</f>
         <v>120712.69088313227</v>
       </c>
-      <c r="E113">
+      <c r="E117">
         <v>282179.67123285501</v>
       </c>
-      <c r="F113">
+      <c r="F117">
         <v>0.854946898908852</v>
       </c>
-      <c r="G113">
+      <c r="G117">
         <v>18681.222424938602</v>
       </c>
-      <c r="H113">
+      <c r="H117">
         <v>5354.6114985546601</v>
       </c>
-      <c r="I113">
+      <c r="I117">
         <v>8156.08309050551</v>
       </c>
-      <c r="J113">
+      <c r="J117">
         <v>32191.917013998798</v>
       </c>
-      <c r="K113">
+      <c r="K117">
         <v>51372.124296964801</v>
       </c>
-      <c r="L113">
+      <c r="L117">
         <v>16725.325417965501</v>
       </c>
-      <c r="M113">
+      <c r="M117">
         <v>19407.285599838699</v>
       </c>
-      <c r="N113">
+      <c r="N117">
         <v>1016.03855436447</v>
       </c>
-      <c r="O113">
-        <v>0</v>
-      </c>
-      <c r="P113">
-        <f t="shared" ref="P113:P119" si="28">D113+$P$1</f>
+      <c r="O117">
+        <v>0</v>
+      </c>
+      <c r="P117">
+        <f t="shared" ref="P117:P123" si="29">D117+$P$1</f>
         <v>241272.36270212877</v>
       </c>
-      <c r="Q113">
+      <c r="Q117">
         <v>1192.7637589594799</v>
       </c>
-      <c r="R113">
+      <c r="R117">
         <v>19736.206339365101</v>
       </c>
-      <c r="S113">
+      <c r="S117">
         <v>481.37088632597801</v>
       </c>
-      <c r="T113" s="6">
+      <c r="T117" s="6">
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A114">
-        <v>20</v>
-      </c>
-      <c r="B114">
-        <v>50</v>
-      </c>
-      <c r="C114">
-        <v>2</v>
-      </c>
-      <c r="D114">
-        <f t="shared" si="27"/>
-        <v>119392.42354269064</v>
-      </c>
-      <c r="E114">
-        <v>282254.81855225202</v>
-      </c>
-      <c r="F114">
-        <v>0.85006146065890897</v>
-      </c>
-      <c r="G114">
-        <v>19407.840072768398</v>
-      </c>
-      <c r="H114">
-        <v>5891.8301217549197</v>
-      </c>
-      <c r="I114">
-        <v>6659.4942697455399</v>
-      </c>
-      <c r="J114">
-        <v>31959.164464268899</v>
-      </c>
-      <c r="K114">
-        <v>51102.045942938203</v>
-      </c>
-      <c r="L114">
-        <v>15967.176494174801</v>
-      </c>
-      <c r="M114">
-        <v>19353.573908279199</v>
-      </c>
-      <c r="N114">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O114">
-        <v>0</v>
-      </c>
-      <c r="P114">
-        <f t="shared" si="28"/>
-        <v>239952.09536168716</v>
-      </c>
-      <c r="Q114">
-        <v>1312.43161993582</v>
-      </c>
-      <c r="R114">
-        <v>18377.616631847999</v>
-      </c>
-      <c r="S114">
-        <v>459.4404157962</v>
-      </c>
-      <c r="T114" s="6">
-        <v>0.14758705239613301</v>
-      </c>
-    </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A115">
-        <v>20</v>
-      </c>
-      <c r="B115">
-        <v>40</v>
-      </c>
-      <c r="C115">
-        <v>2</v>
-      </c>
-      <c r="D115">
-        <f t="shared" si="27"/>
-        <v>117777.02945340994</v>
-      </c>
-      <c r="E115">
-        <v>282179.67123287299</v>
-      </c>
-      <c r="F115">
-        <v>0.84456314023622803</v>
-      </c>
-      <c r="G115">
-        <v>19298.245593088301</v>
-      </c>
-      <c r="H115">
-        <v>5682.0016560700296</v>
-      </c>
-      <c r="I115">
-        <v>5350.3346939491703</v>
-      </c>
-      <c r="J115">
-        <v>30330.5819431075</v>
-      </c>
-      <c r="K115">
-        <v>51097.733915068202</v>
-      </c>
-      <c r="L115">
-        <v>15987.901266609</v>
-      </c>
-      <c r="M115">
-        <v>19350.349595595701</v>
-      </c>
-      <c r="N115">
-        <v>1010.46273302954</v>
-      </c>
-      <c r="O115">
-        <v>0</v>
-      </c>
-      <c r="P115">
-        <f t="shared" si="28"/>
-        <v>238336.70127240644</v>
-      </c>
-      <c r="Q115">
-        <v>1265.6913868611</v>
-      </c>
-      <c r="R115">
-        <v>17746.163883660702</v>
-      </c>
-      <c r="S115">
-        <v>507.03325381887902</v>
-      </c>
-      <c r="T115" s="6">
-        <v>-0.25983751983286502</v>
-      </c>
-    </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A116">
-        <v>20</v>
-      </c>
-      <c r="B116">
-        <v>30</v>
-      </c>
-      <c r="C116">
-        <v>2</v>
-      </c>
-      <c r="D116">
-        <f t="shared" si="27"/>
-        <v>116625.1695160947</v>
-      </c>
-      <c r="E116">
-        <v>282182.50548365602</v>
-      </c>
-      <c r="F116">
-        <v>0.84045954058697003</v>
-      </c>
-      <c r="G116">
-        <v>19302.752565837702</v>
-      </c>
-      <c r="H116">
-        <v>6226.5181629292701</v>
-      </c>
-      <c r="I116">
-        <v>3974.5318253822402</v>
-      </c>
-      <c r="J116">
-        <v>29503.802554149199</v>
-      </c>
-      <c r="K116">
-        <v>51013.610661725899</v>
-      </c>
-      <c r="L116">
-        <v>15760.601295416</v>
-      </c>
-      <c r="M116">
-        <v>19332.981882301501</v>
-      </c>
-      <c r="N116">
-        <v>1014.17312250211</v>
-      </c>
-      <c r="O116">
-        <v>0</v>
-      </c>
-      <c r="P116">
-        <f t="shared" si="28"/>
-        <v>237184.84133509122</v>
-      </c>
-      <c r="Q116">
-        <v>1386.9848841974899</v>
-      </c>
-      <c r="R116">
-        <v>18436.445202769701</v>
-      </c>
-      <c r="S116">
-        <v>209.50505912238299</v>
-      </c>
-      <c r="T116" s="6">
-        <v>0.28049716262959101</v>
-      </c>
-    </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A117" s="3">
-        <v>20</v>
-      </c>
-      <c r="B117" s="3">
-        <v>20</v>
-      </c>
-      <c r="C117" s="3">
-        <v>2</v>
-      </c>
-      <c r="D117">
-        <f t="shared" si="27"/>
-        <v>115198.459983006</v>
-      </c>
-      <c r="E117">
-        <v>282179.67123297497</v>
-      </c>
-      <c r="F117">
-        <v>0.83541194997266699</v>
-      </c>
-      <c r="G117">
-        <v>19351.2255529412</v>
-      </c>
-      <c r="H117">
-        <v>6002.0469674603501</v>
-      </c>
-      <c r="I117">
-        <v>2645.4376652921501</v>
-      </c>
-      <c r="J117">
-        <v>27998.710185693701</v>
-      </c>
-      <c r="K117">
-        <v>51033.4442867088</v>
-      </c>
-      <c r="L117">
-        <v>15815.1228903871</v>
-      </c>
-      <c r="M117">
-        <v>19337.009497714302</v>
-      </c>
-      <c r="N117">
-        <v>1014.17312250211</v>
-      </c>
-      <c r="O117">
-        <v>0</v>
-      </c>
-      <c r="P117">
-        <f t="shared" si="28"/>
-        <v>235758.13180200252</v>
-      </c>
-      <c r="Q117">
-        <v>1336.98290493166</v>
-      </c>
-      <c r="R117">
-        <v>18577.307877855899</v>
-      </c>
-      <c r="S117">
-        <v>432.030415764091</v>
-      </c>
-      <c r="T117" s="6">
-        <v>-0.122490141098651</v>
-      </c>
-    </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>20</v>
       </c>
       <c r="B118">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C118">
         <v>2</v>
       </c>
       <c r="D118">
-        <f t="shared" si="27"/>
-        <v>114451.25872361983</v>
+        <f t="shared" si="28"/>
+        <v>119392.42354269064</v>
       </c>
       <c r="E118">
-        <v>282179.67123267101</v>
+        <v>282254.81855225202</v>
       </c>
       <c r="F118">
-        <v>0.83277713625127903</v>
+        <v>0.85006146065890897</v>
       </c>
       <c r="G118">
-        <v>19390.977969205</v>
+        <v>19407.840072768398</v>
       </c>
       <c r="H118">
-        <v>5599.5405456203798</v>
+        <v>5891.8301217549197</v>
       </c>
       <c r="I118">
-        <v>2128.1287863747102</v>
+        <v>6659.4942697455399</v>
       </c>
       <c r="J118">
-        <v>27118.647301200101</v>
+        <v>31959.164464268899</v>
       </c>
       <c r="K118">
-        <v>51068.507704320902</v>
+        <v>51102.045942938203</v>
       </c>
       <c r="L118">
-        <v>15909.3558282099</v>
+        <v>15967.176494174801</v>
       </c>
       <c r="M118">
-        <v>19344.285156859401</v>
+        <v>19353.573908279199</v>
       </c>
       <c r="N118">
         <v>1010.46273302954</v>
@@ -6406,83 +6393,339 @@
         <v>0</v>
       </c>
       <c r="P118">
-        <f t="shared" si="28"/>
-        <v>235010.93054261635</v>
+        <f t="shared" si="29"/>
+        <v>239952.09536168716</v>
       </c>
       <c r="Q118">
-        <v>1247.3228025527501</v>
+        <v>1312.43161993582</v>
       </c>
       <c r="R118">
-        <v>16417.502561416801</v>
+        <v>18377.616631847999</v>
       </c>
       <c r="S118">
-        <v>469.07150175476602</v>
+        <v>459.4404157962</v>
       </c>
       <c r="T118" s="6">
-        <v>0.46004655114715598</v>
-      </c>
-    </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.4">
+        <v>0.14758705239613301</v>
+      </c>
+    </row>
+    <row r="119" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>20</v>
       </c>
       <c r="B119">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C119">
         <v>2</v>
       </c>
       <c r="D119">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
+        <v>117777.02945340994</v>
+      </c>
+      <c r="E119">
+        <v>282179.67123287299</v>
+      </c>
+      <c r="F119">
+        <v>0.84456314023622803</v>
+      </c>
+      <c r="G119">
+        <v>19298.245593088301</v>
+      </c>
+      <c r="H119">
+        <v>5682.0016560700296</v>
+      </c>
+      <c r="I119">
+        <v>5350.3346939491703</v>
+      </c>
+      <c r="J119">
+        <v>30330.5819431075</v>
+      </c>
+      <c r="K119">
+        <v>51097.733915068202</v>
+      </c>
+      <c r="L119">
+        <v>15987.901266609</v>
+      </c>
+      <c r="M119">
+        <v>19350.349595595701</v>
+      </c>
+      <c r="N119">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O119">
+        <v>0</v>
+      </c>
+      <c r="P119">
+        <f t="shared" si="29"/>
+        <v>238336.70127240644</v>
+      </c>
+      <c r="Q119">
+        <v>1265.6913868611</v>
+      </c>
+      <c r="R119">
+        <v>17746.163883660702</v>
+      </c>
+      <c r="S119">
+        <v>507.03325381887902</v>
+      </c>
+      <c r="T119" s="6">
+        <v>-0.25983751983286502</v>
+      </c>
+    </row>
+    <row r="120" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A120">
+        <v>20</v>
+      </c>
+      <c r="B120">
+        <v>30</v>
+      </c>
+      <c r="C120">
+        <v>2</v>
+      </c>
+      <c r="D120">
+        <f t="shared" si="28"/>
+        <v>116625.1695160947</v>
+      </c>
+      <c r="E120">
+        <v>282182.50548365602</v>
+      </c>
+      <c r="F120">
+        <v>0.84045954058697003</v>
+      </c>
+      <c r="G120">
+        <v>19302.752565837702</v>
+      </c>
+      <c r="H120">
+        <v>6226.5181629292701</v>
+      </c>
+      <c r="I120">
+        <v>3974.5318253822402</v>
+      </c>
+      <c r="J120">
+        <v>29503.802554149199</v>
+      </c>
+      <c r="K120">
+        <v>51013.610661725899</v>
+      </c>
+      <c r="L120">
+        <v>15760.601295416</v>
+      </c>
+      <c r="M120">
+        <v>19332.981882301501</v>
+      </c>
+      <c r="N120">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O120">
+        <v>0</v>
+      </c>
+      <c r="P120">
+        <f t="shared" si="29"/>
+        <v>237184.84133509122</v>
+      </c>
+      <c r="Q120">
+        <v>1386.9848841974899</v>
+      </c>
+      <c r="R120">
+        <v>18436.445202769701</v>
+      </c>
+      <c r="S120">
+        <v>209.50505912238299</v>
+      </c>
+      <c r="T120" s="6">
+        <v>0.28049716262959101</v>
+      </c>
+    </row>
+    <row r="121" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A121" s="3">
+        <v>20</v>
+      </c>
+      <c r="B121" s="3">
+        <v>20</v>
+      </c>
+      <c r="C121" s="3">
+        <v>2</v>
+      </c>
+      <c r="D121">
+        <f t="shared" si="28"/>
+        <v>115198.459983006</v>
+      </c>
+      <c r="E121">
+        <v>282179.67123297497</v>
+      </c>
+      <c r="F121">
+        <v>0.83541194997266699</v>
+      </c>
+      <c r="G121">
+        <v>19351.2255529412</v>
+      </c>
+      <c r="H121">
+        <v>6002.0469674603501</v>
+      </c>
+      <c r="I121">
+        <v>2645.4376652921501</v>
+      </c>
+      <c r="J121">
+        <v>27998.710185693701</v>
+      </c>
+      <c r="K121">
+        <v>51033.4442867088</v>
+      </c>
+      <c r="L121">
+        <v>15815.1228903871</v>
+      </c>
+      <c r="M121">
+        <v>19337.009497714302</v>
+      </c>
+      <c r="N121">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O121">
+        <v>0</v>
+      </c>
+      <c r="P121">
+        <f t="shared" si="29"/>
+        <v>235758.13180200252</v>
+      </c>
+      <c r="Q121">
+        <v>1336.98290493166</v>
+      </c>
+      <c r="R121">
+        <v>18577.307877855899</v>
+      </c>
+      <c r="S121">
+        <v>432.030415764091</v>
+      </c>
+      <c r="T121" s="6">
+        <v>-0.122490141098651</v>
+      </c>
+    </row>
+    <row r="122" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A122">
+        <v>20</v>
+      </c>
+      <c r="B122">
+        <v>15</v>
+      </c>
+      <c r="C122">
+        <v>2</v>
+      </c>
+      <c r="D122">
+        <f t="shared" si="28"/>
+        <v>114451.25872361983</v>
+      </c>
+      <c r="E122">
+        <v>282179.67123267101</v>
+      </c>
+      <c r="F122">
+        <v>0.83277713625127903</v>
+      </c>
+      <c r="G122">
+        <v>19390.977969205</v>
+      </c>
+      <c r="H122">
+        <v>5599.5405456203798</v>
+      </c>
+      <c r="I122">
+        <v>2128.1287863747102</v>
+      </c>
+      <c r="J122">
+        <v>27118.647301200101</v>
+      </c>
+      <c r="K122">
+        <v>51068.507704320902</v>
+      </c>
+      <c r="L122">
+        <v>15909.3558282099</v>
+      </c>
+      <c r="M122">
+        <v>19344.285156859401</v>
+      </c>
+      <c r="N122">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O122">
+        <v>0</v>
+      </c>
+      <c r="P122">
+        <f t="shared" si="29"/>
+        <v>235010.93054261635</v>
+      </c>
+      <c r="Q122">
+        <v>1247.3228025527501</v>
+      </c>
+      <c r="R122">
+        <v>16417.502561416801</v>
+      </c>
+      <c r="S122">
+        <v>469.07150175476602</v>
+      </c>
+      <c r="T122" s="6">
+        <v>0.46004655114715598</v>
+      </c>
+    </row>
+    <row r="123" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A123">
+        <v>20</v>
+      </c>
+      <c r="B123">
+        <v>12</v>
+      </c>
+      <c r="C123">
+        <v>2</v>
+      </c>
+      <c r="D123">
+        <f t="shared" si="28"/>
         <v>114787.7594081375</v>
       </c>
-      <c r="E119">
+      <c r="E123">
         <v>282179.67123287602</v>
       </c>
-      <c r="F119">
+      <c r="F123">
         <v>0.83403396920434802</v>
       </c>
-      <c r="G119">
+      <c r="G123">
         <v>20436.472361711199</v>
       </c>
-      <c r="H119">
+      <c r="H123">
         <v>4946.5396722567002</v>
       </c>
-      <c r="I119">
+      <c r="I123">
         <v>2967.9237851293901</v>
       </c>
-      <c r="J119">
+      <c r="J123">
         <v>28350.9358190973</v>
       </c>
-      <c r="K119">
+      <c r="K123">
         <v>50843.184005923598</v>
       </c>
-      <c r="L119">
+      <c r="L123">
         <v>15303.798385783</v>
       </c>
-      <c r="M119">
+      <c r="M123">
         <v>19297.530489448302</v>
       </c>
-      <c r="N119">
+      <c r="N123">
         <v>992.31070788530405</v>
       </c>
-      <c r="O119">
-        <v>0</v>
-      </c>
-      <c r="P119">
-        <f t="shared" si="28"/>
+      <c r="O123">
+        <v>0</v>
+      </c>
+      <c r="P123">
+        <f t="shared" si="29"/>
         <v>235347.43122713402</v>
       </c>
-      <c r="Q119">
+      <c r="Q123">
         <v>1101.8639118583401</v>
       </c>
-      <c r="R119">
+      <c r="R123">
         <v>13.380488321454299</v>
       </c>
-      <c r="S119">
+      <c r="S123">
         <v>2.67609766429086</v>
       </c>
-      <c r="T119" s="6">
+      <c r="T123" s="6">
         <v>-198.021555533488</v>
       </c>
     </row>
@@ -6502,20 +6745,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA993591-8C1F-4C7B-A75D-E9726DFB461B}">
   <dimension ref="A2:P31"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="12.84375" customWidth="1"/>
-    <col min="3" max="3" width="11.3828125" customWidth="1"/>
-    <col min="4" max="4" width="15.53515625" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" customWidth="1"/>
+    <col min="3" max="3" width="11.36328125" customWidth="1"/>
+    <col min="4" max="4" width="15.54296875" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17.07421875" customWidth="1"/>
-    <col min="7" max="7" width="15.23046875" customWidth="1"/>
-    <col min="8" max="8" width="13.23046875" customWidth="1"/>
-    <col min="9" max="11" width="11.3828125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" customWidth="1"/>
+    <col min="7" max="7" width="15.26953125" customWidth="1"/>
+    <col min="8" max="8" width="13.26953125" customWidth="1"/>
+    <col min="9" max="11" width="11.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6554,12 +6797,12 @@
       </c>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -6598,7 +6841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="D5" s="10"/>
@@ -6610,7 +6853,7 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>48</v>
       </c>
@@ -6627,7 +6870,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -6667,18 +6910,42 @@
       </c>
       <c r="M7" s="11"/>
     </row>
-    <row r="8" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
+    <row r="8" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D8" s="10">
+        <f>D7-D4</f>
+        <v>759.28494035729091</v>
+      </c>
+      <c r="E8" s="10">
+        <f>E7-E4</f>
+        <v>-221.42920834019969</v>
+      </c>
+      <c r="F8" s="10">
+        <f>F7-F4</f>
+        <v>896.09976246881979</v>
+      </c>
+      <c r="G8" s="10">
+        <f>G7-G4</f>
+        <v>-4877.4899349639245</v>
+      </c>
+      <c r="H8" s="10">
+        <f>H7-H4</f>
+        <v>-4202.8193808354008</v>
+      </c>
+      <c r="I8" s="10">
+        <f>I7-I4</f>
+        <v>-87.19067491790338</v>
+      </c>
+      <c r="J8" s="10">
+        <f>J7-J4</f>
+        <v>4424.0083944886992</v>
+      </c>
+      <c r="K8" s="10">
+        <f>K7-K4</f>
+        <v>625.28660162189772</v>
+      </c>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -6692,7 +6959,7 @@
       <c r="K9" s="10"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>21</v>
       </c>
@@ -6728,7 +6995,7 @@
       </c>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="D11">
         <f>(34653-H10-I11+wrd_pricetater_flex_type_summar!K5+L10)/34653</f>
         <v>0.17154119896168271</v>
@@ -6745,7 +7012,7 @@
       <c r="K11" s="10"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
@@ -6759,7 +7026,7 @@
       <c r="K12" s="10"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
@@ -6799,7 +7066,7 @@
       </c>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="D14" s="10"/>
@@ -6812,7 +7079,7 @@
       <c r="K14" s="10"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>46</v>
       </c>
@@ -6825,7 +7092,7 @@
       <c r="J15" s="10"/>
       <c r="K15" s="10"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -6864,7 +7131,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="D17">
         <f>(34653-H16-I17+wrd_pricetater_flex_type_summar!K5+L16)/34653</f>
         <v>0.38932217950875497</v>
@@ -6874,7 +7141,7 @@
         <v>87792.098602195503</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>57</v>
       </c>
@@ -6913,7 +7180,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -6921,7 +7188,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -6959,7 +7226,7 @@
       </c>
       <c r="L23" s="10"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>55</v>
       </c>
@@ -6997,7 +7264,7 @@
       </c>
       <c r="L25" s="10"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -7034,7 +7301,7 @@
         <v>-476.58002357000078</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -7071,7 +7338,7 @@
         <v>174.37684745549996</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>58</v>
       </c>
@@ -7109,6 +7376,573 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BC34AED-31C3-47D6-9398-9693457BF528}">
+  <dimension ref="A2:Y17"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="27.6328125" customWidth="1"/>
+    <col min="2" max="2" width="15.90625" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" customWidth="1"/>
+    <col min="4" max="4" width="12.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" t="s">
+        <v>7</v>
+      </c>
+      <c r="L2" t="s">
+        <v>8</v>
+      </c>
+      <c r="M2" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" t="s">
+        <v>10</v>
+      </c>
+      <c r="O2" t="s">
+        <v>11</v>
+      </c>
+      <c r="P2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="R2" t="s">
+        <v>14</v>
+      </c>
+      <c r="S2" t="s">
+        <v>15</v>
+      </c>
+      <c r="T2" t="s">
+        <v>29</v>
+      </c>
+      <c r="U2" t="s">
+        <v>17</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="W2" t="s">
+        <v>19</v>
+      </c>
+      <c r="X2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <f>M3+N3+O3+P3+Q3</f>
+        <v>113976.01616633293</v>
+      </c>
+      <c r="H3">
+        <v>282179.67123285797</v>
+      </c>
+      <c r="I3">
+        <v>0.82949143613233001</v>
+      </c>
+      <c r="J3">
+        <v>19739.4095985942</v>
+      </c>
+      <c r="K3">
+        <v>6280.2265894411403</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>26019.6361880353</v>
+      </c>
+      <c r="N3">
+        <v>50944.945205466604</v>
+      </c>
+      <c r="O3">
+        <v>15577.281609678699</v>
+      </c>
+      <c r="P3">
+        <v>19971.775208230301</v>
+      </c>
+      <c r="Q3">
+        <v>1462.3779549220301</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>234065.620738292</v>
+      </c>
+      <c r="T3">
+        <v>1403.15815187257</v>
+      </c>
+      <c r="U3">
+        <v>34638.685534293101</v>
+      </c>
+      <c r="V3">
+        <v>865.96713835732805</v>
+      </c>
+      <c r="W3">
+        <v>0.1767383415172</v>
+      </c>
+      <c r="X3">
+        <v>38493.267558113897</v>
+      </c>
+      <c r="Y3">
+        <v>300.72865279776499</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>0.215</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>114954.996549677</v>
+      </c>
+      <c r="H4">
+        <v>282189.04894895799</v>
+      </c>
+      <c r="I4">
+        <v>0.83811536966956601</v>
+      </c>
+      <c r="J4">
+        <v>19873.444109634402</v>
+      </c>
+      <c r="K4">
+        <v>6410.9423067498801</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>26284.386416384299</v>
+      </c>
+      <c r="N4">
+        <v>50909.2414199216</v>
+      </c>
+      <c r="O4">
+        <v>17806.461934653598</v>
+      </c>
+      <c r="P4">
+        <v>19954.906778718101</v>
+      </c>
+      <c r="Q4">
+        <v>1467.84819664867</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>236506.97907655899</v>
+      </c>
+      <c r="T4">
+        <v>1432.36328032659</v>
+      </c>
+      <c r="U4">
+        <v>34730.692350556303</v>
+      </c>
+      <c r="V4">
+        <v>847.09005733064203</v>
+      </c>
+      <c r="W4">
+        <v>0.10581865793454701</v>
+      </c>
+      <c r="X4">
+        <v>39803.051493393003</v>
+      </c>
+      <c r="Y4">
+        <v>313.40985427868497</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>0.43</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <f>M5+N5+O5+P5+Q5</f>
+        <v>117790.41551491321</v>
+      </c>
+      <c r="H5">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="I5">
+        <v>0.84310254173290999</v>
+      </c>
+      <c r="J5">
+        <v>19840.537050750401</v>
+      </c>
+      <c r="K5">
+        <v>5280.6330826172398</v>
+      </c>
+      <c r="L5">
+        <v>4877.4899493259099</v>
+      </c>
+      <c r="M5">
+        <v>29998.660082693601</v>
+      </c>
+      <c r="N5">
+        <v>51077.135880394701</v>
+      </c>
+      <c r="O5">
+        <v>15932.544048423801</v>
+      </c>
+      <c r="P5">
+        <v>19346.075503401102</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>1436</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <f t="shared" ref="S5:S7" si="0">G5+$P$1</f>
+        <v>117790.41551491321</v>
+      </c>
+      <c r="T5">
+        <v>1179.82420335646</v>
+      </c>
+      <c r="U5">
+        <v>12780.012944633199</v>
+      </c>
+      <c r="V5">
+        <v>511.20051778532797</v>
+      </c>
+      <c r="W5">
+        <v>0.18120426001776399</v>
+      </c>
+      <c r="X5">
+        <v>11081.318719635499</v>
+      </c>
+      <c r="Y5">
+        <v>77.491739298150407</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>0.86</v>
+      </c>
+      <c r="B6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6">
+        <f>M6+N6+O6+P6+Q6</f>
+        <v>117790.41551491321</v>
+      </c>
+      <c r="H6">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="I6">
+        <v>0.84310254173290999</v>
+      </c>
+      <c r="J6">
+        <v>19840.537050750401</v>
+      </c>
+      <c r="K6">
+        <v>5280.6330826172398</v>
+      </c>
+      <c r="L6">
+        <v>4877.4899493259099</v>
+      </c>
+      <c r="M6">
+        <v>29998.660082693601</v>
+      </c>
+      <c r="N6">
+        <v>51077.135880394701</v>
+      </c>
+      <c r="O6">
+        <v>15932.544048423801</v>
+      </c>
+      <c r="P6">
+        <v>19346.075503401102</v>
+      </c>
+      <c r="Q6" s="5">
+        <v>1436</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <f t="shared" si="0"/>
+        <v>117790.41551491321</v>
+      </c>
+      <c r="T6">
+        <v>1179.82420335646</v>
+      </c>
+      <c r="U6">
+        <v>12780.012944633199</v>
+      </c>
+      <c r="V6">
+        <v>511.20051778532797</v>
+      </c>
+      <c r="W6">
+        <v>0.18120426001776399</v>
+      </c>
+      <c r="X6">
+        <v>11081.318719635499</v>
+      </c>
+      <c r="Y6">
+        <v>77.491739298150407</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1.29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <f>M7+N7+O7+P7+Q7</f>
+        <v>117790.41551491321</v>
+      </c>
+      <c r="H7">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="I7">
+        <v>0.84310254173290999</v>
+      </c>
+      <c r="J7">
+        <v>19840.537050750401</v>
+      </c>
+      <c r="K7">
+        <v>5280.6330826172398</v>
+      </c>
+      <c r="L7">
+        <v>4877.4899493259099</v>
+      </c>
+      <c r="M7">
+        <v>29998.660082693601</v>
+      </c>
+      <c r="N7">
+        <v>51077.135880394701</v>
+      </c>
+      <c r="O7">
+        <v>15932.544048423801</v>
+      </c>
+      <c r="P7">
+        <v>19346.075503401102</v>
+      </c>
+      <c r="Q7" s="5">
+        <v>1436</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <f t="shared" si="0"/>
+        <v>117790.41551491321</v>
+      </c>
+      <c r="T7">
+        <v>1179.82420335646</v>
+      </c>
+      <c r="U7">
+        <v>12780.012944633199</v>
+      </c>
+      <c r="V7">
+        <v>511.20051778532797</v>
+      </c>
+      <c r="W7">
+        <v>0.18120426001776399</v>
+      </c>
+      <c r="X7">
+        <v>11081.318719635499</v>
+      </c>
+      <c r="Y7">
+        <v>77.491739298150407</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>0</v>
+      </c>
+      <c r="B8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>0.215</v>
+      </c>
+      <c r="B9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>0.43</v>
+      </c>
+      <c r="B10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>0.86</v>
+      </c>
+      <c r="B11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>1.29</v>
+      </c>
+      <c r="B12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>0</v>
+      </c>
+      <c r="B13" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>0.215</v>
+      </c>
+      <c r="B14" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>0.43</v>
+      </c>
+      <c r="B15" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>0.86</v>
+      </c>
+      <c r="B16" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>1.29</v>
+      </c>
+      <c r="B17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="23" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Double startup brine cost for DR results
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B28D283B-92D7-4C23-AD96-27FA9C83007B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6A7FB53-8F56-4F84-870E-0A51C6DF722D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" firstSheet="1" activeTab="2" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -430,6 +430,7 @@
     <author>tc={E817B344-0186-401A-AC52-C5615721C22C}</author>
     <author>tc={338E2122-408B-451A-85D7-EF9A92A8E19E}</author>
     <author>tc={82E3A100-DFFE-4CB2-B9B2-E28BF20128AB}</author>
+    <author>tc={30E6622D-E007-41AB-B0B0-A6FA07445B38}</author>
   </authors>
   <commentList>
     <comment ref="G2" authorId="0" shapeId="0" xr:uid="{91B01F22-295E-46BB-ACCB-2E4ED162A079}">
@@ -464,12 +465,20 @@
     Higher costs don’t change the solution because it avoids shutdowns</t>
       </text>
     </comment>
+    <comment ref="D8" authorId="4" shapeId="0" xr:uid="{30E6622D-E007-41AB-B0B0-A6FA07445B38}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Total Cost will change</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="73">
   <si>
     <t>Season</t>
   </si>
@@ -698,7 +707,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -859,12 +868,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -1786,28 +1789,31 @@
   <threadedComment ref="A5" dT="2026-08-28T23:13:11.99" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{82E3A100-DFFE-4CB2-B9B2-E28BF20128AB}">
     <text>Higher costs don’t change the solution because it avoids shutdowns</text>
   </threadedComment>
+  <threadedComment ref="D8" dT="2026-08-31T16:54:44.56" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{30E6622D-E007-41AB-B0B0-A6FA07445B38}">
+    <text>Total Cost will change</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:V123"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" customWidth="1"/>
-    <col min="3" max="3" width="10.81640625" customWidth="1"/>
+    <col min="1" max="1" width="9.61328125" customWidth="1"/>
+    <col min="3" max="3" width="10.84375" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" customWidth="1"/>
-    <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.54296875" customWidth="1"/>
-    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.81640625" customWidth="1"/>
+    <col min="5" max="5" width="10.23046875" customWidth="1"/>
+    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.69140625" customWidth="1"/>
+    <col min="9" max="9" width="9.07421875" customWidth="1"/>
+    <col min="11" max="11" width="10.84375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.53515625" customWidth="1"/>
+    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1818,7 +1824,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1886,7 +1892,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1950,7 +1956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -2014,14 +2020,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G5" s="4"/>
       <c r="K5" s="10">
         <f>K4+L4+M4</f>
         <v>85444.512881154791</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -2085,7 +2091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -2149,10 +2155,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2216,7 +2222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2280,10 +2286,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -2347,7 +2353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2411,10 +2417,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2476,7 +2482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2532,10 +2538,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2599,7 +2605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2663,7 +2669,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2672,7 +2678,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2683,7 +2689,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2747,10 +2753,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2814,7 +2820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -2884,11 +2890,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -2952,7 +2958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -3016,10 +3022,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -3083,7 +3089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -3153,7 +3159,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -3223,7 +3229,7 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A33" s="14" t="s">
         <v>45</v>
       </c>
@@ -3306,19 +3312,19 @@
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="K34" s="10"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -3382,7 +3388,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3446,12 +3452,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3518,7 +3524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3588,20 +3594,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3665,15 +3671,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3743,13 +3749,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
@@ -3813,7 +3819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
@@ -3877,11 +3883,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -3945,7 +3951,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -4009,10 +4015,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
@@ -4076,7 +4082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A57" s="5" t="s">
         <v>22</v>
       </c>
@@ -4146,19 +4152,19 @@
         <v>358.72983861659498</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.4">
       <c r="K58">
         <f>K57+L57+M57-K5</f>
         <v>5401.088917483823</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -4222,7 +4228,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -4287,7 +4293,7 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A62" s="5" t="s">
         <v>22</v>
       </c>
@@ -4357,7 +4363,7 @@
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -4427,7 +4433,7 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A64" s="14" t="s">
         <v>44</v>
       </c>
@@ -4510,19 +4516,19 @@
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
       <c r="D66" s="10"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A67" s="14" t="s">
         <v>60</v>
       </c>
@@ -4530,7 +4536,7 @@
       <c r="C67" s="14"/>
       <c r="D67" s="10"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A68" s="5" t="s">
         <v>22</v>
       </c>
@@ -4600,7 +4606,7 @@
         <v>350.36946039055402</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A69" s="14" t="s">
         <v>61</v>
       </c>
@@ -4659,7 +4665,7 @@
         <v>133.12347700700047</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -4680,13 +4686,13 @@
       <c r="O70" s="10"/>
       <c r="P70" s="10"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A71" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -4698,7 +4704,7 @@
       </c>
       <c r="G72" s="4"/>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
         <v>22</v>
       </c>
@@ -4762,13 +4768,13 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="G74" s="4"/>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A75" s="3" t="s">
         <v>20</v>
       </c>
@@ -4780,7 +4786,7 @@
       </c>
       <c r="G75" s="4"/>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -4849,7 +4855,7 @@
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="D77">
@@ -4929,12 +4935,12 @@
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A78" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A79" s="3" t="s">
         <v>20</v>
       </c>
@@ -4998,7 +5004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A80" s="3" t="s">
         <v>22</v>
       </c>
@@ -5062,10 +5068,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>20</v>
       </c>
@@ -5123,7 +5129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A83" s="2" t="s">
         <v>22</v>
       </c>
@@ -5187,7 +5193,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>20</v>
       </c>
@@ -5245,7 +5251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
         <v>22</v>
       </c>
@@ -5315,7 +5321,7 @@
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.4">
       <c r="D87">
         <f>D86-D80</f>
         <v>-4018.7603482047853</v>
@@ -5365,13 +5371,13 @@
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A88" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G88" s="4"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -5435,7 +5441,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -5479,8 +5485,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.4"/>
+    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A92" s="1" t="s">
         <v>26</v>
       </c>
@@ -5501,7 +5507,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
         <v>0</v>
       </c>
@@ -5563,10 +5569,10 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
       <c r="G94" s="4"/>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
         <v>20</v>
       </c>
@@ -5636,7 +5642,7 @@
         <v>319.37310450388202</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A96" s="3" t="s">
         <v>20</v>
       </c>
@@ -5681,16 +5687,16 @@
         <v>36</v>
       </c>
     </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A97" s="2"/>
       <c r="G97" s="4"/>
     </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A99" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A100" t="s">
         <v>22</v>
       </c>
@@ -5743,7 +5749,7 @@
         <v>265201.24508552696</v>
       </c>
     </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
         <v>22</v>
       </c>
@@ -5813,13 +5819,13 @@
         <v>290.07670650869801</v>
       </c>
     </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:22" x14ac:dyDescent="0.4">
       <c r="K102">
         <f>SUM(K100:M100)-SUM(K101:M101)</f>
         <v>-750.09243586547382</v>
       </c>
     </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A103" t="s">
         <v>22</v>
       </c>
@@ -5869,7 +5875,7 @@
         <v>303282.7899059637</v>
       </c>
     </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A104" t="s">
         <v>22</v>
       </c>
@@ -5939,19 +5945,19 @@
         <v>351.71871156820202</v>
       </c>
     </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:22" x14ac:dyDescent="0.4">
       <c r="K105" s="13">
         <f>SUM(K103:M103)-SUM(K104:M104)</f>
         <v>-831.26776848098962</v>
       </c>
     </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A106" s="1" t="s">
         <v>65</v>
       </c>
       <c r="K106" s="13"/>
     </row>
-    <row r="107" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A107" t="s">
         <v>22</v>
       </c>
@@ -6021,7 +6027,7 @@
         <v>359.195907759661</v>
       </c>
     </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A108" t="s">
         <v>22</v>
       </c>
@@ -6091,7 +6097,7 @@
         <v>331.01860370537798</v>
       </c>
     </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:22" x14ac:dyDescent="0.4">
       <c r="D109" s="13">
         <f>D108-D31</f>
         <v>870.81314264753019</v>
@@ -6137,7 +6143,7 @@
         <v>-2.9942133752499558</v>
       </c>
     </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:22" x14ac:dyDescent="0.4">
       <c r="D110" s="13"/>
       <c r="E110" s="13"/>
       <c r="F110" s="13"/>
@@ -6150,7 +6156,7 @@
       <c r="M110" s="13"/>
       <c r="N110" s="13"/>
     </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A111" s="1" t="s">
         <v>66</v>
       </c>
@@ -6166,7 +6172,7 @@
       <c r="M111" s="13"/>
       <c r="N111" s="13"/>
     </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A112" t="s">
         <v>22</v>
       </c>
@@ -6236,7 +6242,7 @@
         <v>300.72865279776499</v>
       </c>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.4">
       <c r="D113" s="12">
         <f>(D112-D4)</f>
         <v>-7531.9083775022591</v>
@@ -6252,7 +6258,7 @@
       <c r="M113" s="13"/>
       <c r="N113" s="13"/>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.4">
       <c r="D114" s="13"/>
       <c r="E114" s="13"/>
       <c r="F114" s="13"/>
@@ -6265,12 +6271,12 @@
       <c r="M114" s="13"/>
       <c r="N114" s="13"/>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A115" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A116" t="s">
         <v>32</v>
       </c>
@@ -6281,7 +6287,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A117">
         <v>20</v>
       </c>
@@ -6345,7 +6351,7 @@
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A118">
         <v>20</v>
       </c>
@@ -6409,7 +6415,7 @@
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A119">
         <v>20</v>
       </c>
@@ -6473,7 +6479,7 @@
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A120">
         <v>20</v>
       </c>
@@ -6537,7 +6543,7 @@
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A121" s="3">
         <v>20</v>
       </c>
@@ -6601,7 +6607,7 @@
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A122">
         <v>20</v>
       </c>
@@ -6665,7 +6671,7 @@
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A123">
         <v>20</v>
       </c>
@@ -6745,20 +6751,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA993591-8C1F-4C7B-A75D-E9726DFB461B}">
   <dimension ref="A2:P31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="12.81640625" customWidth="1"/>
-    <col min="3" max="3" width="11.36328125" customWidth="1"/>
-    <col min="4" max="4" width="15.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.84375" customWidth="1"/>
+    <col min="3" max="3" width="11.3828125" customWidth="1"/>
+    <col min="4" max="4" width="15.53515625" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17.08984375" customWidth="1"/>
-    <col min="7" max="7" width="15.26953125" customWidth="1"/>
-    <col min="8" max="8" width="13.26953125" customWidth="1"/>
-    <col min="9" max="11" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.07421875" customWidth="1"/>
+    <col min="7" max="7" width="15.23046875" customWidth="1"/>
+    <col min="8" max="8" width="13.23046875" customWidth="1"/>
+    <col min="9" max="11" width="11.3828125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6797,12 +6803,12 @@
       </c>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -6841,7 +6847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="D5" s="10"/>
@@ -6853,7 +6859,7 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>48</v>
       </c>
@@ -6870,7 +6876,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -6910,42 +6916,42 @@
       </c>
       <c r="M7" s="11"/>
     </row>
-    <row r="8" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D8" s="10">
-        <f>D7-D4</f>
+        <f t="shared" ref="D8:K8" si="0">D7-D4</f>
         <v>759.28494035729091</v>
       </c>
       <c r="E8" s="10">
-        <f>E7-E4</f>
+        <f t="shared" si="0"/>
         <v>-221.42920834019969</v>
       </c>
       <c r="F8" s="10">
-        <f>F7-F4</f>
+        <f t="shared" si="0"/>
         <v>896.09976246881979</v>
       </c>
       <c r="G8" s="10">
-        <f>G7-G4</f>
+        <f t="shared" si="0"/>
         <v>-4877.4899349639245</v>
       </c>
       <c r="H8" s="10">
-        <f>H7-H4</f>
+        <f t="shared" si="0"/>
         <v>-4202.8193808354008</v>
       </c>
       <c r="I8" s="10">
-        <f>I7-I4</f>
+        <f t="shared" si="0"/>
         <v>-87.19067491790338</v>
       </c>
       <c r="J8" s="10">
-        <f>J7-J4</f>
+        <f t="shared" si="0"/>
         <v>4424.0083944886992</v>
       </c>
       <c r="K8" s="10">
-        <f>K7-K4</f>
+        <f t="shared" si="0"/>
         <v>625.28660162189772</v>
       </c>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -6959,7 +6965,7 @@
       <c r="K9" s="10"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B10" t="s">
         <v>21</v>
       </c>
@@ -6995,7 +7001,7 @@
       </c>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
       <c r="D11">
         <f>(34653-H10-I11+wrd_pricetater_flex_type_summar!K5+L10)/34653</f>
         <v>0.17154119896168271</v>
@@ -7012,7 +7018,7 @@
       <c r="K11" s="10"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
@@ -7026,7 +7032,7 @@
       <c r="K12" s="10"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
@@ -7066,7 +7072,7 @@
       </c>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="D14" s="10"/>
@@ -7079,7 +7085,7 @@
       <c r="K14" s="10"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>46</v>
       </c>
@@ -7092,7 +7098,7 @@
       <c r="J15" s="10"/>
       <c r="K15" s="10"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -7131,7 +7137,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
       <c r="D17">
         <f>(34653-H16-I17+wrd_pricetater_flex_type_summar!K5+L16)/34653</f>
         <v>0.38932217950875497</v>
@@ -7141,7 +7147,7 @@
         <v>87792.098602195503</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
         <v>57</v>
       </c>
@@ -7180,7 +7186,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -7188,7 +7194,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -7197,111 +7203,111 @@
         <v>1271.9158797246782</v>
       </c>
       <c r="E23" s="10">
-        <f t="shared" ref="E23:K23" si="0">E16-E4</f>
+        <f t="shared" ref="E23:K23" si="1">E16-E4</f>
         <v>-437.48289297220254</v>
       </c>
       <c r="F23" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>272.65942815481048</v>
       </c>
       <c r="G23" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.39617456624000624</v>
       </c>
       <c r="H23" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-164.42729025120207</v>
       </c>
       <c r="I23" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>96.534215612700791</v>
       </c>
       <c r="J23" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1191.1023712935985</v>
       </c>
       <c r="K23" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>148.7065830695974</v>
       </c>
       <c r="L23" s="10"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>55</v>
       </c>
       <c r="D25" s="10">
-        <f t="shared" ref="D25:K25" si="1">D7-D4</f>
+        <f t="shared" ref="D25:K25" si="2">D7-D4</f>
         <v>759.28494035729091</v>
       </c>
       <c r="E25" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-221.42920834019969</v>
       </c>
       <c r="F25" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>896.09976246881979</v>
       </c>
       <c r="G25" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-4877.4899349639245</v>
       </c>
       <c r="H25" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-4202.8193808354008</v>
       </c>
       <c r="I25" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-87.19067491790338</v>
       </c>
       <c r="J25" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4424.0083944886992</v>
       </c>
       <c r="K25" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>625.28660162189772</v>
       </c>
       <c r="L25" s="10"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>53</v>
       </c>
       <c r="D27" s="10">
-        <f t="shared" ref="D27:K27" si="2">D16-D13</f>
+        <f t="shared" ref="D27:K27" si="3">D16-D13</f>
         <v>513.41117027959262</v>
       </c>
       <c r="E27" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-214.21539764659974</v>
       </c>
       <c r="F27" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-624.4983606493397</v>
       </c>
       <c r="G27" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4877.8861089948059</v>
       </c>
       <c r="H27" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4039.1723506987983</v>
       </c>
       <c r="I27" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>183.72486634590314</v>
       </c>
       <c r="J27" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-3232.9060231951007</v>
       </c>
       <c r="K27" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-476.58002357000078</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -7310,35 +7316,35 @@
         <v>1936.486733518308</v>
       </c>
       <c r="E29" s="10">
-        <f t="shared" ref="E29:K29" si="3">E18-E4</f>
+        <f t="shared" ref="E29:K29" si="4">E18-E4</f>
         <v>-71.19886349780063</v>
       </c>
       <c r="F29" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>774.71175120847056</v>
       </c>
       <c r="G29" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-7.7077004276097796</v>
       </c>
       <c r="H29" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>695.80518728300012</v>
       </c>
       <c r="I29" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>-89.815674909797963</v>
       </c>
       <c r="J29" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1156.1203736896005</v>
       </c>
       <c r="K29" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>174.37684745549996</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>58</v>
       </c>
@@ -7347,31 +7353,31 @@
         <v>-664.57085379362979</v>
       </c>
       <c r="E31" s="10">
-        <f t="shared" ref="E31:K31" si="4">E16-E18</f>
+        <f t="shared" ref="E31:K31" si="5">E16-E18</f>
         <v>-366.2840294744019</v>
       </c>
       <c r="F31" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-502.05232305366007</v>
       </c>
       <c r="G31" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>8.1038749938497858</v>
       </c>
       <c r="H31" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-860.23247753420219</v>
       </c>
       <c r="I31" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>186.34989052249875</v>
       </c>
       <c r="J31" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>34.981997603998025</v>
       </c>
       <c r="K31" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-25.670264385902556</v>
       </c>
     </row>
@@ -7384,15 +7390,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BC34AED-31C3-47D6-9398-9693457BF528}">
   <dimension ref="A2:Y17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="27.6328125" customWidth="1"/>
-    <col min="2" max="2" width="15.90625" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" customWidth="1"/>
-    <col min="4" max="4" width="12.08984375" customWidth="1"/>
+    <col min="1" max="1" width="27.61328125" customWidth="1"/>
+    <col min="2" max="2" width="15.921875" customWidth="1"/>
+    <col min="3" max="3" width="13.15234375" customWidth="1"/>
+    <col min="4" max="4" width="12.07421875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>67</v>
       </c>
@@ -7469,7 +7475,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>0</v>
       </c>
@@ -7547,7 +7553,7 @@
         <v>300.72865279776499</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>0.215</v>
       </c>
@@ -7567,64 +7573,65 @@
         <v>4</v>
       </c>
       <c r="G4">
-        <v>114954.996549677</v>
+        <f>M4+N4+O4+P4+Q4</f>
+        <v>116312.83602496333</v>
       </c>
       <c r="H4">
-        <v>282189.04894895799</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="I4">
-        <v>0.83811536966956601</v>
+        <v>0.83777275508208204</v>
       </c>
       <c r="J4">
-        <v>19873.444109634402</v>
+        <v>19752.187448396198</v>
       </c>
       <c r="K4">
-        <v>6410.9423067498801</v>
+        <v>6300.5639513368096</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4">
-        <v>26284.386416384299</v>
+        <v>26052.751399732999</v>
       </c>
       <c r="N4">
-        <v>50909.2414199216</v>
+        <v>50940.911465697704</v>
       </c>
       <c r="O4">
-        <v>17806.461934653598</v>
+        <v>17895.607600592499</v>
       </c>
       <c r="P4">
-        <v>19954.906778718101</v>
+        <v>19961.187604018101</v>
       </c>
       <c r="Q4">
-        <v>1467.84819664867</v>
+        <v>1462.3779549220301</v>
       </c>
       <c r="R4">
         <v>0</v>
       </c>
       <c r="S4">
-        <v>236506.97907655899</v>
+        <v>236402.440596923</v>
       </c>
       <c r="T4">
-        <v>1432.36328032659</v>
+        <v>1407.70202217271</v>
       </c>
       <c r="U4">
-        <v>34730.692350556303</v>
+        <v>34730.9523834672</v>
       </c>
       <c r="V4">
-        <v>847.09005733064203</v>
+        <v>847.09639959676201</v>
       </c>
       <c r="W4">
-        <v>0.10581865793454701</v>
+        <v>0.108985320449728</v>
       </c>
       <c r="X4">
-        <v>39803.051493393003</v>
+        <v>38694.883606707001</v>
       </c>
       <c r="Y4">
-        <v>313.40985427868497</v>
-      </c>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.35">
+        <v>304.684122887456</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>0.43</v>
       </c>
@@ -7681,7 +7688,7 @@
         <v>0</v>
       </c>
       <c r="S5">
-        <f t="shared" ref="S5:S7" si="0">G5+$P$1</f>
+        <f t="shared" ref="S5:S8" si="0">G5+$P$1</f>
         <v>117790.41551491321</v>
       </c>
       <c r="T5">
@@ -7703,7 +7710,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>0.86</v>
       </c>
@@ -7782,7 +7789,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>1.29</v>
       </c>
@@ -7861,71 +7868,178 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>0</v>
       </c>
       <c r="B8" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>0.215</v>
       </c>
       <c r="B9" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="C9">
+        <v>5</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>0.43</v>
       </c>
       <c r="B10" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10">
+        <v>4</v>
+      </c>
+      <c r="G10">
+        <f>M10+N10+O10+P10+Q10</f>
+        <v>118575.29824632255</v>
+      </c>
+      <c r="H10">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="I10">
+        <v>0.80673743017586796</v>
+      </c>
+      <c r="J10">
+        <v>19617.269555424798</v>
+      </c>
+      <c r="K10">
+        <v>6177.79087142139</v>
+      </c>
+      <c r="L10" s="8">
+        <v>1.4897343661976701E-5</v>
+      </c>
+      <c r="M10">
+        <v>25795.060441743601</v>
+      </c>
+      <c r="N10">
+        <v>50989.945229661498</v>
+      </c>
+      <c r="O10">
+        <v>20356.552509954701</v>
+      </c>
+      <c r="P10">
+        <v>19971.3621100407</v>
+      </c>
+      <c r="Q10">
+        <v>1462.3779549220301</v>
+      </c>
+      <c r="R10">
+        <v>11020</v>
+      </c>
+      <c r="S10">
+        <f>G10+$P$1</f>
+        <v>118575.29824632255</v>
+      </c>
+      <c r="T10">
+        <v>1380.27146414547</v>
+      </c>
+      <c r="U10">
+        <v>33980.634383525299</v>
+      </c>
+      <c r="V10">
+        <v>943.906510653483</v>
+      </c>
+      <c r="W10">
+        <v>0.36911323114551098</v>
+      </c>
+      <c r="X10">
+        <v>36719.7300995962</v>
+      </c>
+      <c r="Y10">
+        <v>278.17977348178903</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>0.86</v>
       </c>
       <c r="B11" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="C11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>1.29</v>
       </c>
       <c r="B12" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>0</v>
       </c>
       <c r="B13" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>0.215</v>
       </c>
       <c r="B14" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>0.43</v>
       </c>
       <c r="B15" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>0.86</v>
       </c>
@@ -7933,7 +8047,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>1.29</v>
       </c>
@@ -7942,7 +8056,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="23" type="noConversion"/>
+  <phoneticPr fontId="22" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
trying RTP with tripled start-up costs
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D57D54-1693-4C94-BD15-646F207F937D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E20BBE6-975C-4056-87A6-9DD93EF0E7E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" activeTab="2" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -501,7 +501,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="103">
   <si>
     <t>Season</t>
   </si>
@@ -821,7 +821,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -988,12 +988,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="35">
@@ -1373,7 +1367,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1398,16 +1392,15 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1973,22 +1966,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:V123"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.61328125" customWidth="1"/>
-    <col min="3" max="3" width="10.84375" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.23046875" customWidth="1"/>
-    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.69140625" customWidth="1"/>
-    <col min="9" max="9" width="9.07421875" customWidth="1"/>
-    <col min="11" max="11" width="10.84375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.53515625" customWidth="1"/>
-    <col min="16" max="16" width="9.84375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.84375" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.54296875" customWidth="1"/>
+    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -1999,7 +1992,7 @@
         <v>120559.67181899652</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2067,7 +2060,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -2131,7 +2124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -2195,14 +2188,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G5" s="4"/>
       <c r="K5" s="10">
         <f>K4+L4+M4</f>
         <v>85444.512881154791</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -2266,7 +2259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -2330,10 +2323,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2397,7 +2390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -2461,10 +2454,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
@@ -2528,7 +2521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -2592,10 +2585,10 @@
         <v>0.33425013552507798</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2657,7 +2650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2713,10 +2706,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -2780,7 +2773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -2844,7 +2837,7 @@
         <v>0.12159211918729</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="K20">
@@ -2853,7 +2846,7 @@
       </c>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2864,7 +2857,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2928,10 +2921,10 @@
         <v>0.116169937532689</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>20</v>
       </c>
@@ -2995,7 +2988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
@@ -3065,11 +3058,11 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
@@ -3133,7 +3126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
@@ -3197,10 +3190,10 @@
         <v>0.105527046108572</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -3264,7 +3257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>22</v>
       </c>
@@ -3334,7 +3327,7 @@
         <v>77.491739298150407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -3404,12 +3397,12 @@
         <v>277.67302057784298</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A33" s="20" t="s">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A33" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
+      <c r="B33" s="26"/>
+      <c r="C33" s="26"/>
       <c r="D33">
         <f>D31-D32</f>
         <v>-785.66289527932531</v>
@@ -3487,19 +3480,19 @@
         <v>200.18128127969257</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="K34" s="10"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -3563,7 +3556,7 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3627,12 +3620,12 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38" s="7"/>
       <c r="B38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>20</v>
       </c>
@@ -3699,7 +3692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>22</v>
       </c>
@@ -3769,20 +3762,20 @@
         <v>69.034824646017199</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3846,15 +3839,15 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -3924,13 +3917,13 @@
         <v>51.1914660847183</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>20</v>
       </c>
@@ -3994,7 +3987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>22</v>
       </c>
@@ -4058,11 +4051,11 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A52" s="3"/>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>20</v>
       </c>
@@ -4126,7 +4119,7 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -4190,10 +4183,10 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>20</v>
       </c>
@@ -4257,7 +4250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>22</v>
       </c>
@@ -4327,19 +4320,19 @@
         <v>358.72983861659498</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
       <c r="K58">
         <f>K57+L57+M57-K5</f>
         <v>5401.088917483823</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>22</v>
       </c>
@@ -4403,7 +4396,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>22</v>
       </c>
@@ -4468,7 +4461,7 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
         <v>22</v>
       </c>
@@ -4538,7 +4531,7 @@
         <v>278.17977348178903</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -4608,12 +4601,12 @@
         <v>107.018147807505</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A64" s="20" t="s">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A64" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="B64" s="20"/>
-      <c r="C64" s="20"/>
+      <c r="B64" s="26"/>
+      <c r="C64" s="26"/>
       <c r="D64" s="10">
         <f>D63-D62</f>
         <v>486.66028698880109</v>
@@ -4691,27 +4684,27 @@
         <v>-171.16162567428404</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A66" s="9"/>
       <c r="B66" s="9"/>
       <c r="C66" s="9"/>
       <c r="D66" s="13"/>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A67" s="20" t="s">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A67" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="B67" s="20"/>
-      <c r="C67" s="20"/>
+      <c r="B67" s="26"/>
+      <c r="C67" s="26"/>
       <c r="D67" s="10"/>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
         <v>22</v>
       </c>
@@ -4781,11 +4774,11 @@
         <v>350.36946039055402</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A69" s="20" t="s">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A69" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="B69" s="20"/>
+      <c r="B69" s="26"/>
       <c r="C69" s="9"/>
       <c r="D69" s="10">
         <f>D68-D62</f>
@@ -4840,7 +4833,7 @@
         <v>133.12347700700047</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
       <c r="C70" s="9"/>
@@ -4861,13 +4854,13 @@
       <c r="O70" s="10"/>
       <c r="P70" s="10"/>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>42</v>
       </c>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -4879,7 +4872,7 @@
       </c>
       <c r="G72" s="4"/>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>22</v>
       </c>
@@ -4943,13 +4936,13 @@
         <v>9.2660976353045002E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
       <c r="G74" s="4"/>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
         <v>20</v>
       </c>
@@ -4961,7 +4954,7 @@
       </c>
       <c r="G75" s="4"/>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -5030,7 +5023,7 @@
         <v>301.29627904392902</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="D77">
@@ -5110,12 +5103,12 @@
         <v>301.20361806757597</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
         <v>20</v>
       </c>
@@ -5179,7 +5172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
         <v>22</v>
       </c>
@@ -5243,10 +5236,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>20</v>
       </c>
@@ -5304,7 +5297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>22</v>
       </c>
@@ -5368,7 +5361,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>20</v>
       </c>
@@ -5426,7 +5419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>22</v>
       </c>
@@ -5496,7 +5489,7 @@
         <v>75.359435725924598</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.35">
       <c r="D87">
         <f>D86-D80</f>
         <v>-4018.7603482047853</v>
@@ -5546,13 +5539,13 @@
         <v>116540.91147079173</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G88" s="4"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -5616,7 +5609,7 @@
         <v>-0.25904927491985202</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -5660,8 +5653,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.4"/>
-    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>26</v>
       </c>
@@ -5682,7 +5675,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>0</v>
       </c>
@@ -5744,10 +5737,10 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
       <c r="G94" s="4"/>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>20</v>
       </c>
@@ -5817,7 +5810,7 @@
         <v>319.37310450388202</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A96" s="3" t="s">
         <v>20</v>
       </c>
@@ -5862,16 +5855,16 @@
         <v>36</v>
       </c>
     </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A97" s="2"/>
       <c r="G97" s="4"/>
     </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>22</v>
       </c>
@@ -5924,7 +5917,7 @@
         <v>265201.24508552696</v>
       </c>
     </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>22</v>
       </c>
@@ -5994,13 +5987,13 @@
         <v>290.07670650869801</v>
       </c>
     </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:22" x14ac:dyDescent="0.35">
       <c r="K102">
         <f>SUM(K100:M100)-SUM(K101:M101)</f>
         <v>-750.09243586547382</v>
       </c>
     </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>22</v>
       </c>
@@ -6050,7 +6043,7 @@
         <v>303282.7899059637</v>
       </c>
     </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>22</v>
       </c>
@@ -6120,19 +6113,19 @@
         <v>351.71871156820202</v>
       </c>
     </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:22" x14ac:dyDescent="0.35">
       <c r="K105" s="13">
         <f>SUM(K103:M103)-SUM(K104:M104)</f>
         <v>-831.26776848098962</v>
       </c>
     </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="106" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>65</v>
       </c>
       <c r="K106" s="13"/>
     </row>
-    <row r="107" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="107" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>22</v>
       </c>
@@ -6202,7 +6195,7 @@
         <v>359.195907759661</v>
       </c>
     </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>22</v>
       </c>
@@ -6272,7 +6265,7 @@
         <v>331.01860370537798</v>
       </c>
     </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="109" spans="1:22" x14ac:dyDescent="0.35">
       <c r="D109" s="13">
         <f>D108-D31</f>
         <v>870.81314264753019</v>
@@ -6318,7 +6311,7 @@
         <v>-2.9942133752499558</v>
       </c>
     </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="110" spans="1:22" x14ac:dyDescent="0.35">
       <c r="D110" s="13"/>
       <c r="E110" s="13"/>
       <c r="F110" s="13"/>
@@ -6331,7 +6324,7 @@
       <c r="M110" s="13"/>
       <c r="N110" s="13"/>
     </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>66</v>
       </c>
@@ -6347,7 +6340,7 @@
       <c r="M111" s="13"/>
       <c r="N111" s="13"/>
     </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>22</v>
       </c>
@@ -6417,7 +6410,7 @@
         <v>300.72865279776499</v>
       </c>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.35">
       <c r="D113" s="12">
         <f>(D112-D4)</f>
         <v>-7531.9083775022591</v>
@@ -6433,7 +6426,7 @@
       <c r="M113" s="13"/>
       <c r="N113" s="13"/>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.35">
       <c r="D114" s="13"/>
       <c r="E114" s="13"/>
       <c r="F114" s="13"/>
@@ -6446,12 +6439,12 @@
       <c r="M114" s="13"/>
       <c r="N114" s="13"/>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A115" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>32</v>
       </c>
@@ -6462,7 +6455,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>20</v>
       </c>
@@ -6526,7 +6519,7 @@
         <v>0.12591688076390301</v>
       </c>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>20</v>
       </c>
@@ -6590,7 +6583,7 @@
         <v>0.14758705239613301</v>
       </c>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>20</v>
       </c>
@@ -6654,7 +6647,7 @@
         <v>-0.25983751983286502</v>
       </c>
     </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="120" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>20</v>
       </c>
@@ -6718,7 +6711,7 @@
         <v>0.28049716262959101</v>
       </c>
     </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="121" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A121" s="3">
         <v>20</v>
       </c>
@@ -6782,7 +6775,7 @@
         <v>-0.122490141098651</v>
       </c>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>20</v>
       </c>
@@ -6846,7 +6839,7 @@
         <v>0.46004655114715598</v>
       </c>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>20</v>
       </c>
@@ -6926,20 +6919,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA993591-8C1F-4C7B-A75D-E9726DFB461B}">
   <dimension ref="A2:P31"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="12.84375" customWidth="1"/>
-    <col min="3" max="3" width="11.3828125" customWidth="1"/>
-    <col min="4" max="4" width="15.53515625" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" customWidth="1"/>
+    <col min="3" max="3" width="11.36328125" customWidth="1"/>
+    <col min="4" max="4" width="15.54296875" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="17.07421875" customWidth="1"/>
-    <col min="7" max="7" width="15.23046875" customWidth="1"/>
-    <col min="8" max="8" width="13.23046875" customWidth="1"/>
-    <col min="9" max="11" width="11.3828125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" customWidth="1"/>
+    <col min="7" max="7" width="15.26953125" customWidth="1"/>
+    <col min="8" max="8" width="13.26953125" customWidth="1"/>
+    <col min="9" max="11" width="11.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6978,12 +6971,12 @@
       </c>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -7022,7 +7015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="D5" s="10"/>
@@ -7034,7 +7027,7 @@
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>48</v>
       </c>
@@ -7051,7 +7044,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -7091,7 +7084,7 @@
       </c>
       <c r="M7" s="11"/>
     </row>
-    <row r="8" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="D8" s="10">
         <f t="shared" ref="D8:K8" si="0">D7-D4</f>
         <v>759.28494035729091</v>
@@ -7126,7 +7119,7 @@
       </c>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -7140,7 +7133,7 @@
       <c r="K9" s="10"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="1:16" ht="14.8" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:16" ht="14.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>21</v>
       </c>
@@ -7176,7 +7169,7 @@
       </c>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="D11">
         <f>(34653-H10-I11+wrd_pricetater_flex_type_summar!K5+L10)/34653</f>
         <v>0.17154119896168271</v>
@@ -7193,7 +7186,7 @@
       <c r="K11" s="10"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
@@ -7207,7 +7200,7 @@
       <c r="K12" s="10"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
@@ -7247,7 +7240,7 @@
       </c>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="D14" s="10"/>
@@ -7260,7 +7253,7 @@
       <c r="K14" s="10"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>46</v>
       </c>
@@ -7273,7 +7266,7 @@
       <c r="J15" s="10"/>
       <c r="K15" s="10"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -7312,7 +7305,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="D17">
         <f>(34653-H16-I17+wrd_pricetater_flex_type_summar!K5+L16)/34653</f>
         <v>0.38932217950875497</v>
@@ -7322,7 +7315,7 @@
         <v>87792.098602195503</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>57</v>
       </c>
@@ -7361,7 +7354,7 @@
         <v>11020</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -7369,7 +7362,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -7407,7 +7400,7 @@
       </c>
       <c r="L23" s="10"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>55</v>
       </c>
@@ -7445,7 +7438,7 @@
       </c>
       <c r="L25" s="10"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -7482,7 +7475,7 @@
         <v>-476.58002357000078</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -7519,7 +7512,7 @@
         <v>174.37684745549996</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>58</v>
       </c>
@@ -7565,25 +7558,25 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BC34AED-31C3-47D6-9398-9693457BF528}">
   <dimension ref="A1:AB19"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.921875" customWidth="1"/>
-    <col min="2" max="2" width="14.69140625" customWidth="1"/>
-    <col min="3" max="3" width="12.07421875" customWidth="1"/>
+    <col min="1" max="1" width="26.90625" customWidth="1"/>
+    <col min="2" max="2" width="14.7265625" customWidth="1"/>
+    <col min="3" max="3" width="12.08984375" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="8.53515625" customWidth="1"/>
-    <col min="6" max="6" width="11.3828125" customWidth="1"/>
-    <col min="7" max="7" width="15.07421875" customWidth="1"/>
-    <col min="8" max="8" width="10.15234375" customWidth="1"/>
-    <col min="9" max="9" width="11.3828125" customWidth="1"/>
+    <col min="5" max="5" width="8.54296875" customWidth="1"/>
+    <col min="6" max="6" width="11.36328125" customWidth="1"/>
+    <col min="7" max="7" width="15.08984375" customWidth="1"/>
+    <col min="8" max="8" width="10.1796875" customWidth="1"/>
+    <col min="9" max="9" width="11.36328125" customWidth="1"/>
     <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.921875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.765625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.69140625" customWidth="1"/>
-    <col min="28" max="28" width="13.84375" customWidth="1"/>
+    <col min="11" max="11" width="16.90625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.7265625" customWidth="1"/>
+    <col min="28" max="28" width="13.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
       <c r="G1">
         <v>121507.92454383519</v>
       </c>
@@ -7591,7 +7584,7 @@
         <v>34653.411662680403</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>67</v>
       </c>
@@ -7677,7 +7670,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>0</v>
       </c>
@@ -7767,7 +7760,7 @@
         <v>0.21734969274652002</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>0.215</v>
       </c>
@@ -7857,7 +7850,7 @@
         <v>0.14991564378830438</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>0.43</v>
       </c>
@@ -7948,7 +7941,7 @@
         <v>0.1072768553096176</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>0.86</v>
       </c>
@@ -8039,7 +8032,7 @@
         <v>0.1072768553096176</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1.29</v>
       </c>
@@ -8130,14 +8123,14 @@
         <v>0.1072768553096176</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="23" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="Q8" s="25"/>
-      <c r="AA8" s="26"/>
-      <c r="AB8" s="27"/>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:28" s="21" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="Q8" s="23"/>
+      <c r="AA8" s="24"/>
+      <c r="AB8" s="25"/>
+    </row>
+    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>0</v>
       </c>
@@ -8161,74 +8154,74 @@
         <v>102956.01616633293</v>
       </c>
       <c r="H9">
-        <f>H3</f>
+        <f t="shared" ref="H9:Q9" si="5">H3</f>
         <v>282179.67123285797</v>
       </c>
       <c r="I9">
-        <f>I3</f>
+        <f t="shared" si="5"/>
         <v>0.82949143613233001</v>
       </c>
       <c r="J9">
-        <f>J3</f>
+        <f t="shared" si="5"/>
         <v>19739.4095985942</v>
       </c>
       <c r="K9">
-        <f>K3</f>
+        <f t="shared" si="5"/>
         <v>6280.2265894411403</v>
       </c>
       <c r="L9">
-        <f>L3</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="M9">
-        <f>M3</f>
+        <f t="shared" si="5"/>
         <v>26019.6361880353</v>
       </c>
       <c r="N9">
-        <f>N3</f>
+        <f t="shared" si="5"/>
         <v>50944.945205466604</v>
       </c>
       <c r="O9">
-        <f>O3</f>
+        <f t="shared" si="5"/>
         <v>15577.281609678699</v>
       </c>
       <c r="P9">
-        <f>P3</f>
+        <f t="shared" si="5"/>
         <v>19971.775208230301</v>
       </c>
       <c r="Q9">
-        <f>Q3</f>
+        <f t="shared" si="5"/>
         <v>1462.3779549220301</v>
       </c>
       <c r="R9">
         <v>11020</v>
       </c>
       <c r="S9">
-        <f>S3</f>
+        <f t="shared" ref="S9:Y10" si="6">S3</f>
         <v>234065.620738292</v>
       </c>
       <c r="T9">
-        <f>T3</f>
+        <f t="shared" si="6"/>
         <v>1403.15815187257</v>
       </c>
       <c r="U9">
-        <f>U3</f>
+        <f t="shared" si="6"/>
         <v>34638.685534293101</v>
       </c>
       <c r="V9">
-        <f>V3</f>
+        <f t="shared" si="6"/>
         <v>865.96713835732805</v>
       </c>
       <c r="W9">
-        <f>W3</f>
+        <f t="shared" si="6"/>
         <v>0.1767383415172</v>
       </c>
       <c r="X9">
-        <f>X3</f>
+        <f t="shared" si="6"/>
         <v>38493.267558113897</v>
       </c>
       <c r="Y9">
-        <f>Y3</f>
+        <f t="shared" si="6"/>
         <v>300.72865279776499</v>
       </c>
       <c r="Z9">
@@ -8244,7 +8237,7 @@
         <v>0.53535589967557295</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>0.215</v>
       </c>
@@ -8268,74 +8261,74 @@
         <v>105292.83602496333</v>
       </c>
       <c r="H10">
-        <f>H4</f>
+        <f t="shared" ref="H10:Q10" si="7">H4</f>
         <v>282179.67123287602</v>
       </c>
       <c r="I10">
-        <f>I4</f>
+        <f t="shared" si="7"/>
         <v>0.83777275508208204</v>
       </c>
       <c r="J10">
-        <f>J4</f>
+        <f t="shared" si="7"/>
         <v>19752.187448396198</v>
       </c>
       <c r="K10">
-        <f>K4</f>
+        <f t="shared" si="7"/>
         <v>6300.5639513368096</v>
       </c>
       <c r="L10">
-        <f>L4</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="M10">
-        <f>M4</f>
+        <f t="shared" si="7"/>
         <v>26052.751399732999</v>
       </c>
       <c r="N10">
-        <f>N4</f>
+        <f t="shared" si="7"/>
         <v>50940.911465697704</v>
       </c>
       <c r="O10">
-        <f>O4</f>
+        <f t="shared" si="7"/>
         <v>17895.607600592499</v>
       </c>
       <c r="P10">
-        <f>P4</f>
+        <f t="shared" si="7"/>
         <v>19961.187604018101</v>
       </c>
       <c r="Q10">
-        <f>Q4</f>
+        <f t="shared" si="7"/>
         <v>1462.3779549220301</v>
       </c>
       <c r="R10">
         <v>11020</v>
       </c>
       <c r="S10">
-        <f>S4</f>
+        <f t="shared" si="6"/>
         <v>236402.440596923</v>
       </c>
       <c r="T10">
-        <f>T4</f>
+        <f t="shared" si="6"/>
         <v>1407.70202217271</v>
       </c>
       <c r="U10">
-        <f>U4</f>
+        <f t="shared" si="6"/>
         <v>34730.9523834672</v>
       </c>
       <c r="V10">
-        <f>V4</f>
+        <f t="shared" si="6"/>
         <v>847.09639959676201</v>
       </c>
       <c r="W10">
-        <f>W4</f>
+        <f t="shared" si="6"/>
         <v>0.108985320449728</v>
       </c>
       <c r="X10">
-        <f>X4</f>
+        <f t="shared" si="6"/>
         <v>38694.883606707001</v>
       </c>
       <c r="Y10">
-        <f>Y4</f>
+        <f t="shared" si="6"/>
         <v>304.684122887456</v>
       </c>
       <c r="Z10">
@@ -8343,7 +8336,7 @@
         <v>2327.5</v>
       </c>
       <c r="AA10" s="10">
-        <f t="shared" ref="AA10" si="5">O10-Z10</f>
+        <f t="shared" ref="AA10" si="8">O10-Z10</f>
         <v>15568.107600592499</v>
       </c>
       <c r="AB10" s="12">
@@ -8351,7 +8344,7 @@
         <v>0.46792185071735731</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>0.43</v>
       </c>
@@ -8434,7 +8427,7 @@
         <v>4655</v>
       </c>
       <c r="AA11" s="10">
-        <f t="shared" ref="AA11:AA12" si="6">O11-Z11</f>
+        <f t="shared" ref="AA11:AA12" si="9">O11-Z11</f>
         <v>15701.552509954701</v>
       </c>
       <c r="AB11" s="12">
@@ -8442,7 +8435,7 @@
         <v>0.40263355404451467</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>0.86</v>
       </c>
@@ -8524,7 +8517,7 @@
         <v>1862</v>
       </c>
       <c r="AA12" s="10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>15923.318787562501</v>
       </c>
       <c r="AB12" s="12">
@@ -8532,7 +8525,7 @@
         <v>0.36082050708979968</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1.29</v>
       </c>
@@ -8623,11 +8616,11 @@
         <v>0.33396366478241479</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="23" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="AA14" s="26"/>
-      <c r="AB14" s="27"/>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:28" s="21" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="AA14" s="24"/>
+      <c r="AB14" s="25"/>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>0</v>
       </c>
@@ -8637,7 +8630,7 @@
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>0.215</v>
       </c>
@@ -8647,7 +8640,7 @@
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>0.43</v>
       </c>
@@ -8667,7 +8660,7 @@
         <v>4</v>
       </c>
       <c r="G17">
-        <f t="shared" ref="G17" si="7">M17+N17+O17+P17+Q17-R17</f>
+        <f t="shared" ref="G17" si="10">M17+N17+O17+P17+Q17-R17</f>
         <v>188012.7674304971</v>
       </c>
       <c r="H17">
@@ -8704,7 +8697,7 @@
         <v>0</v>
       </c>
       <c r="S17">
-        <f t="shared" ref="S17" si="8">G17+$P$1</f>
+        <f t="shared" ref="S17" si="11">G17+$P$1</f>
         <v>188012.7674304971</v>
       </c>
       <c r="T17">
@@ -8728,15 +8721,92 @@
         <v>10648.798385783</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>0.86</v>
       </c>
       <c r="B18" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="C18">
+        <v>5</v>
+      </c>
+      <c r="D18" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18">
+        <v>4</v>
+      </c>
+      <c r="G18">
+        <v>127037.185869735</v>
+      </c>
+      <c r="H18">
+        <v>282179.67123288399</v>
+      </c>
+      <c r="I18">
+        <v>0.88096058553932999</v>
+      </c>
+      <c r="J18">
+        <v>22250.673834736099</v>
+      </c>
+      <c r="K18">
+        <v>9244.6813880767095</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>31495.355222812799</v>
+      </c>
+      <c r="N18">
+        <v>50878.4272491683</v>
+      </c>
+      <c r="O18">
+        <v>24715.181268666001</v>
+      </c>
+      <c r="P18">
+        <v>19948.222129088499</v>
+      </c>
+      <c r="Q18">
+        <v>1473.35951653596</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18">
+        <v>248589.16839661699</v>
+      </c>
+      <c r="T18">
+        <v>1467.25635714281</v>
+      </c>
+      <c r="U18">
+        <v>37808.968336081402</v>
+      </c>
+      <c r="V18">
+        <v>821.934094262641</v>
+      </c>
+      <c r="W18">
+        <v>1.54750201311078</v>
+      </c>
+      <c r="X18">
+        <v>43921.314308243796</v>
+      </c>
+      <c r="Y18">
+        <v>360.010773018392</v>
+      </c>
+      <c r="Z18">
+        <f>IF(A18=0,0,C18*931*(A18/0.43))</f>
+        <v>9310</v>
+      </c>
+      <c r="AA18" s="10">
+        <f>O18-Z18</f>
+        <v>15405.181268666001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1.29</v>
       </c>
@@ -8754,24 +8824,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FD55A87-71DC-49C4-874A-7F05794F4461}">
   <dimension ref="A3:P22"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="12.61328125" customWidth="1"/>
-    <col min="3" max="3" width="9.765625" customWidth="1"/>
-    <col min="4" max="4" width="12.4609375" customWidth="1"/>
+    <col min="2" max="2" width="12.6328125" customWidth="1"/>
+    <col min="3" max="3" width="9.7265625" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="20.921875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.3046875" customWidth="1"/>
-    <col min="8" max="8" width="18.53515625" customWidth="1"/>
-    <col min="9" max="9" width="20.15234375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.07421875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.3828125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.23046875" customWidth="1"/>
-    <col min="13" max="13" width="9.3828125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.15234375" customWidth="1"/>
+    <col min="6" max="6" width="20.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.26953125" customWidth="1"/>
+    <col min="8" max="8" width="18.54296875" customWidth="1"/>
+    <col min="9" max="9" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.26953125" customWidth="1"/>
+    <col min="13" max="13" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
         <v>76</v>
       </c>
@@ -8794,7 +8864,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>101</v>
       </c>
@@ -8811,7 +8881,7 @@
       <c r="F4" s="10">
         <v>23102.276630754801</v>
       </c>
-      <c r="G4" s="22">
+      <c r="G4" s="10">
         <v>21941.326830000002</v>
       </c>
       <c r="H4" s="10">
@@ -8823,7 +8893,7 @@
         <v>-4.0410044714229976</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C5">
         <v>10000</v>
       </c>
@@ -8837,7 +8907,7 @@
       <c r="F5" s="10">
         <v>34228.405091644003</v>
       </c>
-      <c r="G5" s="22">
+      <c r="G5" s="10">
         <v>25825.974624668099</v>
       </c>
       <c r="H5" s="10">
@@ -8845,7 +8915,7 @@
         <v>-12815.109372157822</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C6">
         <v>12000</v>
       </c>
@@ -8859,11 +8929,11 @@
       <c r="F6" s="10">
         <v>34654.757319050303</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="10">
         <v>29978.252519511701</v>
       </c>
       <c r="H6" s="10">
-        <f t="shared" ref="H5:H8" si="0">(J15+K15+L15)-(J20+K20+L20)</f>
+        <f t="shared" ref="H6:H8" si="0">(J15+K15+L15)-(J20+K20+L20)</f>
         <v>1000.8858604910201</v>
       </c>
       <c r="I6" s="13">
@@ -8871,7 +8941,7 @@
         <v>-10.60639064705564</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C7">
         <v>14000</v>
       </c>
@@ -8885,7 +8955,7 @@
       <c r="F7" s="10">
         <v>45897.885924687798</v>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="10">
         <v>34616.141121013003</v>
       </c>
       <c r="H7" s="10">
@@ -8893,7 +8963,7 @@
         <v>-13034.940154857992</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>102</v>
       </c>
@@ -8910,7 +8980,7 @@
       <c r="F8" s="10">
         <v>46518.361670285398</v>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="10">
         <v>43908.345722562502</v>
       </c>
       <c r="H8" s="10">
@@ -8922,7 +8992,7 @@
         <v>-5.2757114382118635</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>78</v>
       </c>
@@ -8930,12 +9000,12 @@
         <v>394716</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="18" t="s">
         <v>0</v>
       </c>
@@ -8985,7 +9055,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="15" t="s">
         <v>84</v>
       </c>
@@ -9002,31 +9072,31 @@
       <c r="E13" s="16">
         <v>10</v>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="20">
         <v>188119.78330000001</v>
       </c>
-      <c r="G13" s="21">
+      <c r="G13" s="20">
         <v>200683.70370000001</v>
       </c>
-      <c r="H13" s="21">
+      <c r="H13" s="20">
         <v>13644.59908</v>
       </c>
-      <c r="I13" s="21">
+      <c r="I13" s="20">
         <v>8296.7277529999992</v>
       </c>
-      <c r="J13" s="21">
+      <c r="J13" s="20">
         <v>33953.835149999999</v>
       </c>
-      <c r="K13" s="21">
+      <c r="K13" s="20">
         <v>10359.425139999999</v>
       </c>
-      <c r="L13" s="21">
+      <c r="L13" s="20">
         <v>12877.13408</v>
       </c>
-      <c r="M13" s="21">
+      <c r="M13" s="20">
         <v>21941.326830000002</v>
       </c>
-      <c r="N13" s="21">
+      <c r="N13" s="20">
         <v>1409.83743</v>
       </c>
       <c r="O13" s="16">
@@ -9036,7 +9106,7 @@
         <v>1.0667868110000001</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="15" t="s">
         <v>84</v>
       </c>
@@ -9053,31 +9123,31 @@
       <c r="E14" s="16">
         <v>10</v>
       </c>
-      <c r="F14" s="21">
+      <c r="F14" s="20">
         <v>235149.72602739499</v>
       </c>
-      <c r="G14" s="21">
+      <c r="G14" s="20">
         <v>219262.567779392</v>
       </c>
-      <c r="H14" s="21">
+      <c r="H14" s="20">
         <v>16362.727098568001</v>
       </c>
-      <c r="I14" s="21">
+      <c r="I14" s="20">
         <v>9463.2475261001691</v>
       </c>
-      <c r="J14" s="21">
+      <c r="J14" s="20">
         <v>42544.121004540699</v>
       </c>
-      <c r="K14" s="21">
+      <c r="K14" s="20">
         <v>13222.943008009999</v>
       </c>
-      <c r="L14" s="21">
+      <c r="L14" s="20">
         <v>16117.5466152914</v>
       </c>
-      <c r="M14" s="21">
+      <c r="M14" s="20">
         <v>25825.974624668099</v>
       </c>
-      <c r="N14" s="21">
+      <c r="N14" s="20">
         <v>1425.19885437316</v>
       </c>
       <c r="O14" s="16">
@@ -9087,7 +9157,7 @@
         <v>0.93243811712477798</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
         <v>84</v>
       </c>
@@ -9104,31 +9174,31 @@
       <c r="E15" s="16">
         <v>10</v>
       </c>
-      <c r="F15" s="21">
+      <c r="F15" s="20">
         <v>282179.67123257701</v>
       </c>
-      <c r="G15" s="21">
+      <c r="G15" s="20">
         <v>237975.63378803901</v>
       </c>
-      <c r="H15" s="21">
+      <c r="H15" s="20">
         <v>19793.405782867099</v>
       </c>
-      <c r="I15" s="21">
+      <c r="I15" s="20">
         <v>10184.8467366445</v>
       </c>
-      <c r="J15" s="21">
+      <c r="J15" s="20">
         <v>51100.150850479702</v>
       </c>
-      <c r="K15" s="21">
+      <c r="K15" s="20">
         <v>15994.396781481701</v>
       </c>
-      <c r="L15" s="21">
+      <c r="L15" s="20">
         <v>19350.851109684401</v>
       </c>
-      <c r="M15" s="21">
+      <c r="M15" s="20">
         <v>29978.252519511701</v>
       </c>
-      <c r="N15" s="21">
+      <c r="N15" s="20">
         <v>1433.00578662475</v>
       </c>
       <c r="O15" s="16">
@@ -9138,7 +9208,7 @@
         <v>0.84334790223742195</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="15" t="s">
         <v>84</v>
       </c>
@@ -9155,31 +9225,31 @@
       <c r="E16" s="16">
         <v>10</v>
       </c>
-      <c r="F16" s="21">
+      <c r="F16" s="20">
         <v>329210.46374056302</v>
       </c>
-      <c r="G16" s="21">
+      <c r="G16" s="20">
         <v>256066.1476925</v>
       </c>
-      <c r="H16" s="21">
+      <c r="H16" s="20">
         <v>23209.551664587099</v>
       </c>
-      <c r="I16" s="21">
+      <c r="I16" s="20">
         <v>11406.5894564259</v>
       </c>
-      <c r="J16" s="21">
+      <c r="J16" s="20">
         <v>59371.758428007903</v>
       </c>
-      <c r="K16" s="21">
+      <c r="K16" s="20">
         <v>18001.101366829</v>
       </c>
-      <c r="L16" s="21">
+      <c r="L16" s="20">
         <v>22525.164249769001</v>
       </c>
-      <c r="M16" s="21">
+      <c r="M16" s="20">
         <v>34616.141121013003</v>
       </c>
-      <c r="N16" s="21">
+      <c r="N16" s="20">
         <v>1433.00578662475</v>
       </c>
       <c r="O16" s="16">
@@ -9189,7 +9259,7 @@
         <v>0.77781898176327602</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" s="15" t="s">
         <v>84</v>
       </c>
@@ -9206,31 +9276,31 @@
       <c r="E17" s="16">
         <v>10</v>
       </c>
-      <c r="F17" s="21">
+      <c r="F17" s="20">
         <v>376239.56164383498</v>
       </c>
-      <c r="G17" s="21">
+      <c r="G17" s="20">
         <v>279542.18685761699</v>
       </c>
-      <c r="H17" s="21">
+      <c r="H17" s="20">
         <v>27786.2889118024</v>
       </c>
-      <c r="I17" s="21">
+      <c r="I17" s="20">
         <v>16122.056810759999</v>
       </c>
-      <c r="J17" s="21">
+      <c r="J17" s="20">
         <v>67830.922645459694</v>
       </c>
-      <c r="K17" s="21">
+      <c r="K17" s="20">
         <v>20512.593102821898</v>
       </c>
-      <c r="L17" s="21">
+      <c r="L17" s="20">
         <v>25738.3428598918</v>
       </c>
-      <c r="M17" s="21">
+      <c r="M17" s="20">
         <v>43908.345722562502</v>
       </c>
-      <c r="N17" s="21">
+      <c r="N17" s="20">
         <v>1422.6154123410699</v>
       </c>
       <c r="O17" s="16">
@@ -9240,7 +9310,7 @@
         <v>0.74298988026741397</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A18" s="15" t="s">
         <v>84</v>
       </c>
@@ -9291,7 +9361,7 @@
         <v>1.0717494293005001</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19" s="15" t="s">
         <v>84</v>
       </c>
@@ -9342,7 +9412,7 @@
         <v>0.85971724445347397</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A20" s="15" t="s">
         <v>84</v>
       </c>
@@ -9393,7 +9463,7 @@
         <v>0.85637371278832397</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21" s="15" t="s">
         <v>84</v>
       </c>
@@ -9444,7 +9514,7 @@
         <v>0.75177719391388198</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22" s="15" t="s">
         <v>84</v>
       </c>

</xml_diff>

<commit_message>
no start-up cost RTP
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E20BBE6-975C-4056-87A6-9DD93EF0E7E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169DF754-40E9-412C-870E-BBCC602FB4C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" activeTab="2" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -433,7 +433,6 @@
     <author>tc={30E6622D-E007-41AB-B0B0-A6FA07445B38}</author>
     <author>tc={CC2FED43-9317-4942-84AB-D91CBD6CC0A1}</author>
     <author>tc={964F0726-9326-406D-BF37-7999B0A6D102}</author>
-    <author>tc={CD9B9187-2B2A-46AC-8788-C7718BA1D062}</author>
   </authors>
   <commentList>
     <comment ref="G2" authorId="0" shapeId="0" xr:uid="{91B01F22-295E-46BB-ACCB-2E4ED162A079}">
@@ -486,22 +485,12 @@
     Calculated by manually adding in the cost of startup</t>
       </text>
     </comment>
-    <comment ref="W17" authorId="6" shapeId="0" xr:uid="{CD9B9187-2B2A-46AC-8788-C7718BA1D062}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure
-Reply:
-    The baseline costs have to be updated in accordance with the demand structure type</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="103">
   <si>
     <t>Season</t>
   </si>
@@ -1954,12 +1943,6 @@
   <threadedComment ref="O13" dT="2026-08-31T20:52:23.61" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{964F0726-9326-406D-BF37-7999B0A6D102}">
     <text>Calculated by manually adding in the cost of startup</text>
   </threadedComment>
-  <threadedComment ref="W17" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{CD9B9187-2B2A-46AC-8788-C7718BA1D062}">
-    <text>Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure</text>
-  </threadedComment>
-  <threadedComment ref="W17" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{67FDA27F-4BC3-4CAF-AEC3-31D297C583F8}" parentId="{CD9B9187-2B2A-46AC-8788-C7718BA1D062}">
-    <text>The baseline costs have to be updated in accordance with the demand structure type</text>
-  </threadedComment>
 </ThreadedComments>
 </file>
 
@@ -8637,8 +8620,84 @@
       <c r="B16" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
+      <c r="C16">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16">
+        <v>4</v>
+      </c>
+      <c r="G16">
+        <f t="shared" ref="G16:G17" si="10">M16+N16+O16+P16+Q16-R16</f>
+        <v>122207.43848874117</v>
+      </c>
+      <c r="H16">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="I16">
+        <v>0.85862337439302705</v>
+      </c>
+      <c r="J16">
+        <v>22422.4091975925</v>
+      </c>
+      <c r="K16">
+        <v>9246.5948656492601</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>31669.0040632417</v>
+      </c>
+      <c r="N16">
+        <v>50981.234041832096</v>
+      </c>
+      <c r="O16">
+        <v>18099.530680245101</v>
+      </c>
+      <c r="P16">
+        <v>19984.310186886301</v>
+      </c>
+      <c r="Q16">
+        <v>1473.35951653596</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16">
+        <v>242286.06149908699</v>
+      </c>
+      <c r="T16">
+        <v>1467.5600519750701</v>
+      </c>
+      <c r="U16">
+        <v>37047.600328837303</v>
+      </c>
+      <c r="V16">
+        <v>823.280007307495</v>
+      </c>
+      <c r="W16">
+        <v>1.74944020492494</v>
+      </c>
+      <c r="X16">
+        <v>43335.021637601203</v>
+      </c>
+      <c r="Y16">
+        <v>352.31724908618901</v>
+      </c>
+      <c r="Z16">
+        <f>IF(A16=0,0,C16*931*(A16/0.43))</f>
+        <v>2327.5</v>
+      </c>
+      <c r="AA16" s="10">
+        <f>O16-Z16</f>
+        <v>15772.030680245101</v>
+      </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A17">
@@ -8660,57 +8719,63 @@
         <v>4</v>
       </c>
       <c r="G17">
-        <f t="shared" ref="G17" si="10">M17+N17+O17+P17+Q17-R17</f>
-        <v>188012.7674304971</v>
+        <f t="shared" si="10"/>
+        <v>123759.49613284627</v>
       </c>
       <c r="H17">
-        <v>282179.67123287602</v>
+        <v>282179.67123286799</v>
       </c>
       <c r="I17">
-        <v>1.09353178385</v>
+        <v>0.86412362052107095</v>
       </c>
       <c r="J17">
-        <v>89520.694507565597</v>
+        <v>22235.129466751401</v>
       </c>
       <c r="K17">
-        <v>6971.3813103080802</v>
+        <v>9205.4053509202495</v>
       </c>
       <c r="L17">
-        <v>5083.8680235841202</v>
+        <v>0</v>
       </c>
       <c r="M17">
-        <v>101575.943841457</v>
+        <v>31440.534817671702</v>
       </c>
       <c r="N17">
-        <v>50843.184005923598</v>
+        <v>50868.697977035903</v>
       </c>
       <c r="O17">
-        <v>15303.798385783</v>
+        <v>20030.700516482098</v>
       </c>
       <c r="P17">
-        <v>19297.5304894482</v>
+        <v>19946.203305120602</v>
       </c>
       <c r="Q17">
-        <v>992.31070788530405</v>
+        <v>1473.35951653596</v>
       </c>
       <c r="R17">
         <v>0</v>
       </c>
       <c r="S17">
-        <f t="shared" ref="S17" si="11">G17+$P$1</f>
-        <v>188012.7674304971</v>
+        <f>G17+$P$1</f>
+        <v>123759.49613284627</v>
       </c>
       <c r="T17">
-        <v>1106.4527933521999</v>
+        <v>1461.0227171772699</v>
       </c>
       <c r="U17">
-        <v>3451.9307168288801</v>
+        <v>37816.4634857485</v>
       </c>
       <c r="V17">
-        <v>20.547206647791</v>
+        <v>822.09703229888203</v>
       </c>
       <c r="W17">
-        <v>-14.696886263168601</v>
+        <v>1.67282971584568</v>
+      </c>
+      <c r="X17">
+        <v>43765.040311224599</v>
+      </c>
+      <c r="Y17">
+        <v>358.72983861659498</v>
       </c>
       <c r="Z17">
         <f>IF(A17=0,0,C17*931*(A17/0.43))</f>
@@ -8718,7 +8783,7 @@
       </c>
       <c r="AA17" s="10">
         <f>O17-Z17</f>
-        <v>10648.798385783</v>
+        <v>15375.700516482098</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.35">
@@ -8741,7 +8806,8 @@
         <v>4</v>
       </c>
       <c r="G18">
-        <v>127037.185869735</v>
+        <f t="shared" ref="G17:G19" si="11">M18+N18+O18+P18+Q18-R18</f>
+        <v>128510.54538627157</v>
       </c>
       <c r="H18">
         <v>282179.67123288399</v>
@@ -8812,6 +8878,84 @@
       </c>
       <c r="B19" t="s">
         <v>72</v>
+      </c>
+      <c r="C19">
+        <v>5</v>
+      </c>
+      <c r="D19" t="s">
+        <v>22</v>
+      </c>
+      <c r="E19" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19">
+        <v>4</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="11"/>
+        <v>133101.99841632816</v>
+      </c>
+      <c r="H19">
+        <v>282179.67123286898</v>
+      </c>
+      <c r="I19">
+        <v>0.89723196685467799</v>
+      </c>
+      <c r="J19">
+        <v>22239.845837604698</v>
+      </c>
+      <c r="K19">
+        <v>9215.99935297312</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>31455.845190577798</v>
+      </c>
+      <c r="N19">
+        <v>50871.400221928801</v>
+      </c>
+      <c r="O19">
+        <v>29354.629466349801</v>
+      </c>
+      <c r="P19">
+        <v>19946.7640209358</v>
+      </c>
+      <c r="Q19">
+        <v>1473.35951653596</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>253180.62142667401</v>
+      </c>
+      <c r="T19">
+        <v>1462.70412903026</v>
+      </c>
+      <c r="U19">
+        <v>37658.737638395498</v>
+      </c>
+      <c r="V19">
+        <v>818.66820953033698</v>
+      </c>
+      <c r="W19">
+        <v>1.43175276084397</v>
+      </c>
+      <c r="X19">
+        <v>43571.5293994557</v>
+      </c>
+      <c r="Y19">
+        <v>357.14368360209602</v>
+      </c>
+      <c r="Z19">
+        <f>IF(A19=0,0,C19*931*(A19/0.43))</f>
+        <v>13965</v>
+      </c>
+      <c r="AA19" s="10">
+        <f>O19-Z19</f>
+        <v>15389.629466349801</v>
       </c>
     </row>
   </sheetData>

</xml_diff>